<commit_message>
Atualiza planilha 02/10/2026 15:43
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2081" uniqueCount="842">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2082" uniqueCount="842">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2799,8 +2799,7 @@
         <name val="Calibri"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2814,7 +2813,8 @@
         <name val="Calibri"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -3067,10 +3067,10 @@
     <tableColumn id="3" name="Quantidade" dataDxfId="4" dataCellStyle="Normal"/>
     <tableColumn id="4" name="Unidade" dataDxfId="3" dataCellStyle="Normal"/>
     <tableColumn id="5" name="Preço Unitário" dataDxfId="2" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="0" dataCellStyle="Moeda">
+    <tableColumn id="6" name="Preço Total" dataDxfId="1" dataCellStyle="Moeda">
       <calculatedColumnFormula>G4*E4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="1" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="0" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12652,7 +12652,7 @@
       </c>
       <c r="J7" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Fechamento Lateral",Tabela2[Preço Total])</f>
-        <v>0</v>
+        <v>18900</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
@@ -13172,12 +13172,18 @@
       <c r="C31" s="25" t="s">
         <v>783</v>
       </c>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="26"/>
+      <c r="D31" s="24">
+        <v>540</v>
+      </c>
+      <c r="E31" s="24" t="s">
+        <v>761</v>
+      </c>
+      <c r="F31" s="26">
+        <v>35</v>
+      </c>
       <c r="G31" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18900</v>
       </c>
       <c r="H31" s="24" t="s">
         <v>776</v>
@@ -13434,7 +13440,7 @@
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G46" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>1875005.0538461539</v>
+        <v>1893905.0538461539</v>
       </c>
     </row>
   </sheetData>
@@ -13581,7 +13587,7 @@
         <v>968004</v>
       </c>
       <c r="P5" s="44">
-        <f>O5/$O$18</f>
+        <f t="shared" ref="P5:P16" si="1">O5/$O$18</f>
         <v>0.35024144543236768</v>
       </c>
       <c r="Q5" s="46">
@@ -13627,7 +13633,7 @@
         <v>791792.51</v>
       </c>
       <c r="P6" s="44">
-        <f>O6/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0.28648492484010651</v>
       </c>
       <c r="Q6" s="46">
@@ -13672,7 +13678,7 @@
         <v>645545.6</v>
       </c>
       <c r="P7" s="44">
-        <f>O7/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0.2335701340454224</v>
       </c>
     </row>
@@ -13714,7 +13720,7 @@
         <v>358477</v>
       </c>
       <c r="P8" s="44">
-        <f>O8/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0.12970349568210346</v>
       </c>
     </row>
@@ -13755,7 +13761,7 @@
         <v>0</v>
       </c>
       <c r="P9" s="44">
-        <f>O9/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13787,7 +13793,7 @@
         <v>0</v>
       </c>
       <c r="P10" s="44">
-        <f>O10/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13819,7 +13825,7 @@
         <v>0</v>
       </c>
       <c r="P11" s="44">
-        <f>O11/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13851,7 +13857,7 @@
         <v>0</v>
       </c>
       <c r="P12" s="44">
-        <f>O12/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13889,7 +13895,7 @@
         <v>0</v>
       </c>
       <c r="P13" s="44">
-        <f>O13/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13921,7 +13927,7 @@
         <v>0</v>
       </c>
       <c r="P14" s="44">
-        <f>O14/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13953,7 +13959,7 @@
         <v>0</v>
       </c>
       <c r="P15" s="44">
-        <f>O15/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13985,7 +13991,7 @@
         <v>0</v>
       </c>
       <c r="P16" s="44">
-        <f>O16/$O$18</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -14448,7 +14454,7 @@
         <v>46600</v>
       </c>
       <c r="H37" s="26">
-        <f t="shared" ref="H37:H40" si="1">G37*E37</f>
+        <f t="shared" ref="H37:H40" si="2">G37*E37</f>
         <v>46600</v>
       </c>
       <c r="I37" s="24" t="s">
@@ -14529,7 +14535,7 @@
         <v>298777</v>
       </c>
       <c r="H40" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>298777</v>
       </c>
       <c r="I40" s="24" t="s">
@@ -14582,7 +14588,7 @@
         <v>670</v>
       </c>
       <c r="H42" s="26">
-        <f t="shared" ref="H42:H43" si="2">G42*E42</f>
+        <f t="shared" ref="H42:H43" si="3">G42*E42</f>
         <v>188256.59999999998</v>
       </c>
       <c r="I42" s="24" t="s">
@@ -14610,7 +14616,7 @@
         <v>220.5</v>
       </c>
       <c r="H43" s="26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>30259.384615384613</v>
       </c>
       <c r="I43" s="24" t="s">

</xml_diff>

<commit_message>
Atualiza planilha 02/10/2026 15:45
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2082" uniqueCount="842">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2081" uniqueCount="842">
   <si>
     <t>Código EAP</t>
   </si>
@@ -12652,7 +12652,7 @@
       </c>
       <c r="J7" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Fechamento Lateral",Tabela2[Preço Total])</f>
-        <v>18900</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
@@ -13172,18 +13172,12 @@
       <c r="C31" s="25" t="s">
         <v>783</v>
       </c>
-      <c r="D31" s="24">
-        <v>540</v>
-      </c>
-      <c r="E31" s="24" t="s">
-        <v>761</v>
-      </c>
-      <c r="F31" s="26">
-        <v>35</v>
-      </c>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="26"/>
       <c r="G31" s="26">
         <f t="shared" si="2"/>
-        <v>18900</v>
+        <v>0</v>
       </c>
       <c r="H31" s="24" t="s">
         <v>776</v>
@@ -13440,7 +13434,7 @@
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G46" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>1893905.0538461539</v>
+        <v>1875005.0538461539</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 05/10/2026 11:29
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2081" uniqueCount="842">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2087" uniqueCount="843">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2466,9 +2466,6 @@
     <t>Diária bomba de concreto - valor por metro bombeado</t>
   </si>
   <si>
-    <t>Arrasamento das estacas e Locação dos cálices</t>
-  </si>
-  <si>
     <t>Poço Artesiano para alimentação do alojamento</t>
   </si>
   <si>
@@ -2551,6 +2548,12 @@
   </si>
   <si>
     <t>C&gt;90%</t>
+  </si>
+  <si>
+    <t>Arrasamento das estacas, Locação dos cálices e concretagem</t>
+  </si>
+  <si>
+    <t>Arrasamento das estacas, locação dos blocos e concretagem dos cálices</t>
   </si>
 </sst>
 </file>
@@ -3041,7 +3044,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H43" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:H43"/>
+  <autoFilter ref="B3:H43">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Arrasamento das estacas e Locação dos cálices"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="7">
     <tableColumn id="1" name="Item" dataDxfId="15" dataCellStyle="Normal"/>
     <tableColumn id="2" name="Descrição" dataDxfId="14" dataCellStyle="Normal"/>
@@ -3058,8 +3067,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I44" totalsRowShown="0" dataDxfId="8">
-  <autoFilter ref="B3:I44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I45" totalsRowShown="0" dataDxfId="8">
+  <autoFilter ref="B3:I45"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Item" dataDxfId="7" dataCellStyle="Normal"/>
     <tableColumn id="8" name="Local" dataDxfId="6"/>
@@ -12538,10 +12547,10 @@
         <v>767</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>833</v>
-      </c>
-    </row>
-    <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" s="14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B4" s="27">
         <v>1</v>
       </c>
@@ -12566,10 +12575,10 @@
       </c>
       <c r="J4" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
-        <v>6000</v>
-      </c>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+        <v>186000</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B5" s="27">
         <v>2</v>
       </c>
@@ -12598,7 +12607,7 @@
         <v>361131.5538461539</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B6" s="27">
         <v>3</v>
       </c>
@@ -12627,7 +12636,7 @@
         <v>1267174</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B7" s="27">
         <v>4</v>
       </c>
@@ -12638,7 +12647,7 @@
         <v>167</v>
       </c>
       <c r="E7" s="27" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="F7" s="32">
         <v>56.2</v>
@@ -12655,7 +12664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B8" s="27">
         <v>5</v>
       </c>
@@ -12683,7 +12692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" s="27">
         <v>6</v>
       </c>
@@ -12711,7 +12720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B10" s="27">
         <v>7</v>
       </c>
@@ -12739,7 +12748,7 @@
         <v>157963.5</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" s="27">
         <v>8</v>
       </c>
@@ -12761,7 +12770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B12" s="27">
         <v>9</v>
       </c>
@@ -12783,7 +12792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B13" s="27">
         <v>10</v>
       </c>
@@ -12805,7 +12814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B14" s="27">
         <v>11</v>
       </c>
@@ -12838,22 +12847,30 @@
         <v>12</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>813</v>
-      </c>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="20"/>
+        <v>841</v>
+      </c>
+      <c r="D15" s="17">
+        <v>1</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="F15" s="20">
+        <v>180000</v>
+      </c>
       <c r="G15" s="20">
         <f>F15*D15</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="17"/>
+        <v>180000</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>771</v>
+      </c>
       <c r="J15" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Serviço Prévio",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" s="27">
         <v>13</v>
       </c>
@@ -12871,7 +12888,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" s="27">
         <v>14</v>
       </c>
@@ -12889,7 +12906,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B18" s="27">
         <v>15</v>
       </c>
@@ -12907,7 +12924,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" s="27">
         <v>16</v>
       </c>
@@ -12931,7 +12948,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B20" s="27">
         <v>17</v>
       </c>
@@ -12955,7 +12972,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B21" s="27">
         <v>18</v>
       </c>
@@ -12979,7 +12996,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B22" s="27">
         <v>19</v>
       </c>
@@ -13003,7 +13020,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B23" s="27">
         <v>20</v>
       </c>
@@ -13027,7 +13044,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B24" s="27">
         <v>21</v>
       </c>
@@ -13045,7 +13062,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B25" s="27">
         <v>22</v>
       </c>
@@ -13066,7 +13083,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B26" s="27">
         <v>23</v>
       </c>
@@ -13084,7 +13101,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B27" s="27">
         <v>24</v>
       </c>
@@ -13111,7 +13128,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B28" s="27">
         <v>25</v>
       </c>
@@ -13129,7 +13146,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B29" s="27">
         <v>26</v>
       </c>
@@ -13147,7 +13164,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B30" s="27">
         <v>27</v>
       </c>
@@ -13165,7 +13182,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B31" s="27">
         <v>28</v>
       </c>
@@ -13183,7 +13200,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B32" s="27">
         <v>29</v>
       </c>
@@ -13201,7 +13218,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" s="27">
         <v>30</v>
       </c>
@@ -13219,7 +13236,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B34" s="27">
         <v>31</v>
       </c>
@@ -13237,7 +13254,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B35" s="27">
         <v>32</v>
       </c>
@@ -13259,7 +13276,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B36" s="27">
         <v>33</v>
       </c>
@@ -13281,7 +13298,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B37" s="27">
         <v>34</v>
       </c>
@@ -13299,7 +13316,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B38" s="27">
         <v>35</v>
       </c>
@@ -13317,7 +13334,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B39" s="27">
         <v>36</v>
       </c>
@@ -13335,7 +13352,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B40" s="27">
         <v>37</v>
       </c>
@@ -13353,7 +13370,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B41" s="27">
         <v>38</v>
       </c>
@@ -13371,12 +13388,12 @@
         <v>803</v>
       </c>
     </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B42" s="27">
         <v>39</v>
       </c>
       <c r="C42" s="25" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D42" s="24">
         <v>1</v>
@@ -13390,13 +13407,13 @@
         <v>0</v>
       </c>
       <c r="H42" s="24" t="s">
-        <v>816</v>
-      </c>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B43" s="24"/>
       <c r="C43" s="25" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D43" s="24">
         <v>1</v>
@@ -13410,7 +13427,7 @@
         <v>0</v>
       </c>
       <c r="H43" s="24" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
@@ -13434,7 +13451,7 @@
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G46" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>1875005.0538461539</v>
+        <v>2055005.0538461539</v>
       </c>
     </row>
   </sheetData>
@@ -13448,7 +13465,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R47"/>
+  <dimension ref="B1:R48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -13469,12 +13486,12 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P1" s="14" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P2" s="14" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="3" spans="2:18" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -13482,7 +13499,7 @@
         <v>753</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="D3" t="s">
         <v>754</v>
@@ -13503,7 +13520,7 @@
         <v>767</v>
       </c>
       <c r="P3" s="14" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
@@ -13511,7 +13528,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>757</v>
@@ -13534,16 +13551,16 @@
         <v>635</v>
       </c>
       <c r="O4" s="14" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="P4" s="14" t="s">
+        <v>834</v>
+      </c>
+      <c r="Q4" s="14" t="s">
         <v>835</v>
       </c>
-      <c r="Q4" s="14" t="s">
+      <c r="R4" s="14" t="s">
         <v>836</v>
-      </c>
-      <c r="R4" s="14" t="s">
-        <v>837</v>
       </c>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
@@ -13551,7 +13568,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>778</v>
@@ -13567,7 +13584,7 @@
         <v>220.5</v>
       </c>
       <c r="H5" s="20">
-        <f t="shared" ref="H5:H35" si="0">G5*E5</f>
+        <f t="shared" ref="H5:H36" si="0">G5*E5</f>
         <v>72934.61538461539</v>
       </c>
       <c r="I5" s="17" t="s">
@@ -13581,15 +13598,15 @@
         <v>968004</v>
       </c>
       <c r="P5" s="44">
-        <f t="shared" ref="P5:P16" si="1">O5/$O$18</f>
-        <v>0.35024144543236768</v>
+        <f t="shared" ref="P5:P17" si="1">O5/$O$19</f>
+        <v>0.33062288469044115</v>
       </c>
       <c r="Q5" s="46">
         <f>P5</f>
-        <v>0.35024144543236768</v>
+        <v>0.33062288469044115</v>
       </c>
       <c r="R5" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.25">
@@ -13597,7 +13614,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D6" s="18" t="s">
         <v>758</v>
@@ -13628,14 +13645,14 @@
       </c>
       <c r="P6" s="44">
         <f t="shared" si="1"/>
-        <v>0.28648492484010651</v>
+        <v>0.27043764667551473</v>
       </c>
       <c r="Q6" s="46">
         <f>P6+Q5</f>
-        <v>0.63672637027247414</v>
+        <v>0.60106053136595583</v>
       </c>
       <c r="R6" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
@@ -13643,7 +13660,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D7" s="18" t="s">
         <v>762</v>
@@ -13673,7 +13690,7 @@
       </c>
       <c r="P7" s="44">
         <f t="shared" si="1"/>
-        <v>0.2335701340454224</v>
+        <v>0.22048684558247864</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
@@ -13681,10 +13698,10 @@
         <v>5</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="E8" s="23">
         <f>E4</f>
@@ -13704,10 +13721,10 @@
         <v>635</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="N8" s="45" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="O8" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
@@ -13715,7 +13732,7 @@
       </c>
       <c r="P8" s="44">
         <f t="shared" si="1"/>
-        <v>0.12970349568210346</v>
+        <v>0.12243823355603414</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
@@ -13723,7 +13740,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D9" s="18" t="s">
         <v>768</v>
@@ -13745,18 +13762,18 @@
         <v>635</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="N9" s="42" t="s">
         <v>771</v>
       </c>
       <c r="O9" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Fundação",Tabela24[Preço Total])</f>
-        <v>0</v>
+        <v>164000</v>
       </c>
       <c r="P9" s="44">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5.6014389495531371E-2</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
@@ -13764,7 +13781,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D10" s="18" t="s">
         <v>801</v>
@@ -13796,7 +13813,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D11" s="18" t="s">
         <v>769</v>
@@ -13828,7 +13845,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D12" s="18" t="s">
         <v>770</v>
@@ -13856,14 +13873,12 @@
       </c>
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B13" s="17">
-        <v>10</v>
-      </c>
+      <c r="B13" s="17"/>
       <c r="C13" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>773</v>
+        <v>842</v>
       </c>
       <c r="E13" s="17">
         <v>1</v>
@@ -13872,52 +13887,50 @@
         <v>760</v>
       </c>
       <c r="G13" s="20">
+        <v>164000</v>
+      </c>
+      <c r="H13" s="20">
+        <f>G13*E13</f>
+        <v>164000</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="N13" s="41"/>
+      <c r="O13" s="40"/>
+      <c r="P13" s="44"/>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B14" s="17">
+        <v>10</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>818</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="E14" s="17">
+        <v>1</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G14" s="20">
         <v>968004</v>
       </c>
-      <c r="H13" s="20">
+      <c r="H14" s="20">
         <f t="shared" si="0"/>
         <v>968004</v>
       </c>
-      <c r="I13" s="17" t="s">
+      <c r="I14" s="17" t="s">
         <v>772</v>
       </c>
-      <c r="N13" s="41" t="s">
+      <c r="N14" s="41" t="s">
         <v>776</v>
       </c>
-      <c r="O13" s="40">
+      <c r="O14" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
-        <v>0</v>
-      </c>
-      <c r="P13" s="44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B14" s="17">
-        <v>11</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>819</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>774</v>
-      </c>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I14" s="17" t="s">
-        <v>771</v>
-      </c>
-      <c r="N14" s="41" t="s">
-        <v>643</v>
-      </c>
-      <c r="O14" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Elétrica",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
       <c r="P14" s="44">
@@ -13927,13 +13940,13 @@
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B15" s="17">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="E15" s="17"/>
       <c r="F15" s="17"/>
@@ -13946,10 +13959,10 @@
         <v>771</v>
       </c>
       <c r="N15" s="41" t="s">
-        <v>576</v>
+        <v>643</v>
       </c>
       <c r="O15" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Pintura",Tabela24[Preço Total])</f>
+        <f>SUMIF(Tabela24[Aplicação],"Elétrica",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
       <c r="P15" s="44">
@@ -13959,29 +13972,29 @@
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B16" s="17">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>819</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>798</v>
-      </c>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19">
+        <v>818</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>775</v>
+      </c>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I16" s="22" t="s">
-        <v>776</v>
+      <c r="I16" s="17" t="s">
+        <v>771</v>
       </c>
       <c r="N16" s="41" t="s">
-        <v>827</v>
+        <v>576</v>
       </c>
       <c r="O16" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
+        <f>SUMIF(Tabela24[Aplicação],"Pintura",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
       <c r="P16" s="44">
@@ -13989,64 +14002,68 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" s="17">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="E17" s="22"/>
       <c r="F17" s="22"/>
       <c r="G17" s="19"/>
       <c r="H17" s="19">
-        <f>G17*E17</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I17" s="17" t="s">
-        <v>772</v>
-      </c>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="I17" s="22" t="s">
+        <v>776</v>
+      </c>
+      <c r="N17" s="41" t="s">
+        <v>826</v>
+      </c>
+      <c r="O17" s="40">
+        <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
+        <v>0</v>
+      </c>
+      <c r="P17" s="44">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" s="17">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="E18" s="22"/>
       <c r="F18" s="22"/>
       <c r="G18" s="19"/>
       <c r="H18" s="19">
-        <f t="shared" si="0"/>
+        <f>G18*E18</f>
         <v>0</v>
       </c>
-      <c r="I18" s="22" t="s">
-        <v>776</v>
-      </c>
-      <c r="N18" s="41" t="s">
-        <v>834</v>
-      </c>
-      <c r="O18" s="43">
-        <f>SUM(O5:O16)</f>
-        <v>2763819.11</v>
-      </c>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="I18" s="17" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B19" s="17">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
@@ -14056,18 +14073,25 @@
         <v>0</v>
       </c>
       <c r="I19" s="22" t="s">
-        <v>787</v>
-      </c>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+        <v>776</v>
+      </c>
+      <c r="N19" s="41" t="s">
+        <v>833</v>
+      </c>
+      <c r="O19" s="43">
+        <f>SUM(O5:O17)</f>
+        <v>2927819.11</v>
+      </c>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="17">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>797</v>
+        <v>779</v>
       </c>
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
@@ -14077,66 +14101,66 @@
         <v>0</v>
       </c>
       <c r="I20" s="22" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B21" s="17">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>789</v>
-      </c>
-      <c r="E21" s="22">
-        <v>1</v>
-      </c>
-      <c r="F21" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G21" s="19">
-        <v>791792.51</v>
-      </c>
+        <v>797</v>
+      </c>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="19"/>
       <c r="H21" s="19">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I21" s="22" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B22" s="17">
+        <v>18</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>818</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>789</v>
+      </c>
+      <c r="E22" s="22">
+        <v>1</v>
+      </c>
+      <c r="F22" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G22" s="19">
         <v>791792.51</v>
       </c>
-      <c r="I21" s="22" t="s">
-        <v>788</v>
-      </c>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B22" s="17">
-        <v>19</v>
-      </c>
-      <c r="C22" s="17" t="s">
-        <v>819</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>780</v>
-      </c>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="19"/>
       <c r="H22" s="19">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>791792.51</v>
       </c>
       <c r="I22" s="22" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B23" s="17">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="E23" s="22"/>
       <c r="F23" s="22"/>
@@ -14146,18 +14170,18 @@
         <v>0</v>
       </c>
       <c r="I23" s="22" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B24" s="17">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E24" s="22"/>
       <c r="F24" s="22"/>
@@ -14170,36 +14194,36 @@
         <v>449</v>
       </c>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B25" s="17">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>819</v>
-      </c>
-      <c r="D25" s="25" t="s">
-        <v>783</v>
-      </c>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26">
+        <v>818</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>782</v>
+      </c>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I25" s="24" t="s">
-        <v>776</v>
-      </c>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="I25" s="22" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B26" s="17">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D26" s="25" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E26" s="24"/>
       <c r="F26" s="24"/>
@@ -14212,15 +14236,15 @@
         <v>776</v>
       </c>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B27" s="17">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="E27" s="24"/>
       <c r="F27" s="24"/>
@@ -14233,19 +14257,17 @@
         <v>776</v>
       </c>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B28" s="17">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D28" s="25" t="s">
-        <v>831</v>
-      </c>
-      <c r="E28" s="24">
-        <v>1</v>
-      </c>
+        <v>785</v>
+      </c>
+      <c r="E28" s="24"/>
       <c r="F28" s="24"/>
       <c r="G28" s="26"/>
       <c r="H28" s="26">
@@ -14256,18 +14278,18 @@
         <v>776</v>
       </c>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B29" s="17">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>795</v>
+        <v>830</v>
       </c>
       <c r="E29" s="24">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F29" s="24"/>
       <c r="G29" s="26"/>
@@ -14276,25 +14298,23 @@
         <v>0</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B30" s="17">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D30" s="25" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E30" s="24">
-        <v>500</v>
-      </c>
-      <c r="F30" s="24" t="s">
-        <v>761</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F30" s="24"/>
       <c r="G30" s="26"/>
       <c r="H30" s="26">
         <f t="shared" si="0"/>
@@ -14304,55 +14324,59 @@
         <v>643</v>
       </c>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B31" s="17"/>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B31" s="17">
+        <v>27</v>
+      </c>
       <c r="C31" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D31" s="25" t="s">
-        <v>826</v>
-      </c>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
+        <v>796</v>
+      </c>
+      <c r="E31" s="24">
+        <v>500</v>
+      </c>
+      <c r="F31" s="24" t="s">
+        <v>761</v>
+      </c>
       <c r="G31" s="26"/>
       <c r="H31" s="26">
-        <f>G31*E31</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I31" s="24" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B32" s="17">
-        <v>28</v>
-      </c>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B32" s="17"/>
       <c r="C32" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D32" s="25" t="s">
-        <v>790</v>
+        <v>825</v>
       </c>
       <c r="E32" s="24"/>
       <c r="F32" s="24"/>
       <c r="G32" s="26"/>
       <c r="H32" s="26">
-        <f t="shared" si="0"/>
+        <f>G32*E32</f>
         <v>0</v>
       </c>
       <c r="I32" s="24" t="s">
-        <v>576</v>
+        <v>643</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" s="17">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D33" s="25" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="E33" s="24"/>
       <c r="F33" s="24"/>
@@ -14367,13 +14391,13 @@
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" s="17">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D34" s="25" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="E34" s="24"/>
       <c r="F34" s="24"/>
@@ -14388,13 +14412,13 @@
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" s="17">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D35" s="25" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="E35" s="24"/>
       <c r="F35" s="24"/>
@@ -14409,61 +14433,55 @@
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" s="17">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="D36" s="25" t="s">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="E36" s="24"/>
       <c r="F36" s="24"/>
       <c r="G36" s="26"/>
       <c r="H36" s="26">
-        <f>G36*E36</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>827</v>
+        <v>576</v>
       </c>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B37" s="17">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C37" s="17" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="D37" s="25" t="s">
-        <v>814</v>
-      </c>
-      <c r="E37" s="24">
-        <v>1</v>
-      </c>
-      <c r="F37" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G37" s="26">
-        <v>46600</v>
-      </c>
+        <v>800</v>
+      </c>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="26"/>
       <c r="H37" s="26">
-        <f t="shared" ref="H37:H40" si="2">G37*E37</f>
-        <v>46600</v>
+        <f>G37*E37</f>
+        <v>0</v>
       </c>
       <c r="I37" s="24" t="s">
-        <v>816</v>
+        <v>826</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B38" s="17">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C38" s="17" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="D38" s="25" t="s">
-        <v>817</v>
+        <v>813</v>
       </c>
       <c r="E38" s="24">
         <v>1</v>
@@ -14472,25 +14490,25 @@
         <v>760</v>
       </c>
       <c r="G38" s="26">
-        <v>8100</v>
+        <v>46600</v>
       </c>
       <c r="H38" s="26">
-        <f>G38*E38</f>
-        <v>8100</v>
+        <f t="shared" ref="H38:H41" si="2">G38*E38</f>
+        <v>46600</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B39" s="17">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C39" s="17" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="D39" s="25" t="s">
-        <v>832</v>
+        <v>816</v>
       </c>
       <c r="E39" s="24">
         <v>1</v>
@@ -14499,25 +14517,25 @@
         <v>760</v>
       </c>
       <c r="G39" s="26">
-        <v>5000</v>
+        <v>8100</v>
       </c>
       <c r="H39" s="26">
         <f>G39*E39</f>
-        <v>5000</v>
+        <v>8100</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B40" s="17">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C40" s="17" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="D40" s="25" t="s">
-        <v>821</v>
+        <v>831</v>
       </c>
       <c r="E40" s="24">
         <v>1</v>
@@ -14526,138 +14544,155 @@
         <v>760</v>
       </c>
       <c r="G40" s="26">
+        <v>5000</v>
+      </c>
+      <c r="H40" s="26">
+        <f>G40*E40</f>
+        <v>5000</v>
+      </c>
+      <c r="I40" s="24" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B41" s="17">
+        <v>36</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>819</v>
+      </c>
+      <c r="D41" s="25" t="s">
+        <v>820</v>
+      </c>
+      <c r="E41" s="24">
+        <v>1</v>
+      </c>
+      <c r="F41" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G41" s="26">
         <v>298777</v>
       </c>
-      <c r="H40" s="26">
+      <c r="H41" s="26">
         <f t="shared" si="2"/>
         <v>298777</v>
       </c>
-      <c r="I40" s="24" t="s">
-        <v>816</v>
-      </c>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="17">
-        <v>37</v>
-      </c>
-      <c r="C41" s="34" t="s">
-        <v>820</v>
-      </c>
-      <c r="D41" s="25" t="s">
-        <v>830</v>
-      </c>
-      <c r="E41" s="24">
-        <v>110</v>
-      </c>
-      <c r="F41" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G41" s="26"/>
-      <c r="H41" s="26">
-        <f>G41*E41</f>
-        <v>0</v>
-      </c>
       <c r="I41" s="24" t="s">
-        <v>635</v>
+        <v>815</v>
       </c>
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B42" s="17">
+        <v>37</v>
+      </c>
+      <c r="C42" s="34" t="s">
+        <v>819</v>
+      </c>
+      <c r="D42" s="25" t="s">
+        <v>829</v>
+      </c>
+      <c r="E42" s="24">
+        <v>110</v>
+      </c>
+      <c r="F42" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G42" s="26"/>
+      <c r="H42" s="26">
+        <f>G42*E42</f>
+        <v>0</v>
+      </c>
+      <c r="I42" s="24" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B43" s="17">
         <v>38</v>
       </c>
-      <c r="C42" s="34" t="s">
-        <v>820</v>
-      </c>
-      <c r="D42" s="25" t="s">
+      <c r="C43" s="34" t="s">
+        <v>819</v>
+      </c>
+      <c r="D43" s="25" t="s">
         <v>757</v>
       </c>
-      <c r="E42" s="35">
+      <c r="E43" s="35">
         <f>(1784*0.15)*1.05</f>
         <v>280.97999999999996</v>
       </c>
-      <c r="F42" s="24" t="s">
+      <c r="F43" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="G42" s="26">
+      <c r="G43" s="26">
         <v>670</v>
       </c>
-      <c r="H42" s="26">
-        <f t="shared" ref="H42:H43" si="3">G42*E42</f>
+      <c r="H43" s="26">
+        <f t="shared" ref="H43:H44" si="3">G43*E43</f>
         <v>188256.59999999998</v>
       </c>
-      <c r="I42" s="24" t="s">
+      <c r="I43" s="24" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B43" s="17">
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B44" s="17">
         <v>40</v>
       </c>
-      <c r="C43" s="34" t="s">
-        <v>820</v>
-      </c>
-      <c r="D43" s="18" t="s">
+      <c r="C44" s="34" t="s">
+        <v>819</v>
+      </c>
+      <c r="D44" s="18" t="s">
         <v>778</v>
       </c>
-      <c r="E43" s="35">
+      <c r="E44" s="35">
         <f>1784/13</f>
         <v>137.23076923076923</v>
       </c>
-      <c r="F43" s="24" t="s">
+      <c r="F44" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G43" s="26">
+      <c r="G44" s="26">
         <v>220.5</v>
       </c>
-      <c r="H43" s="26">
+      <c r="H44" s="26">
         <f t="shared" si="3"/>
         <v>30259.384615384613</v>
       </c>
-      <c r="I43" s="24" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B44" s="17">
-        <v>41</v>
-      </c>
-      <c r="C44" s="34" t="s">
-        <v>820</v>
-      </c>
-      <c r="D44" s="25" t="s">
-        <v>829</v>
-      </c>
-      <c r="E44" s="24">
-        <v>1</v>
-      </c>
-      <c r="F44" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G44" s="26">
-        <v>43350</v>
-      </c>
-      <c r="H44" s="26">
-        <f>G44*E44</f>
-        <v>43350</v>
-      </c>
       <c r="I44" s="24" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B45" s="24"/>
-      <c r="C45" s="34"/>
-      <c r="D45" s="25"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="26"/>
-      <c r="I45" s="25"/>
+      <c r="B45" s="17">
+        <v>41</v>
+      </c>
+      <c r="C45" s="34" t="s">
+        <v>819</v>
+      </c>
+      <c r="D45" s="25" t="s">
+        <v>828</v>
+      </c>
+      <c r="E45" s="24">
+        <v>1</v>
+      </c>
+      <c r="F45" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G45" s="26">
+        <v>43350</v>
+      </c>
+      <c r="H45" s="26">
+        <f>G45*E45</f>
+        <v>43350</v>
+      </c>
+      <c r="I45" s="24" t="s">
+        <v>635</v>
+      </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B46" s="24"/>
       <c r="C46" s="34"/>
-      <c r="D46" s="39"/>
+      <c r="D46" s="25"/>
       <c r="E46" s="24"/>
       <c r="F46" s="24"/>
       <c r="G46" s="26"/>
@@ -14665,10 +14700,20 @@
       <c r="I46" s="25"/>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D47" s="38"/>
-      <c r="H47" s="16">
+      <c r="B47" s="24"/>
+      <c r="C47" s="34"/>
+      <c r="D47" s="39"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24"/>
+      <c r="G47" s="26"/>
+      <c r="H47" s="26"/>
+      <c r="I47" s="25"/>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D48" s="38"/>
+      <c r="H48" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>2763819.1100000003</v>
+        <v>2927819.1100000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 05/10/2026 12:13
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -3044,13 +3044,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H43" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:H43">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Arrasamento das estacas e Locação dos cálices"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B3:H43"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Item" dataDxfId="15" dataCellStyle="Normal"/>
     <tableColumn id="2" name="Descrição" dataDxfId="14" dataCellStyle="Normal"/>
@@ -12550,7 +12544,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="4" spans="2:10" s="14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="27">
         <v>1</v>
       </c>
@@ -12578,7 +12572,7 @@
         <v>186000</v>
       </c>
     </row>
-    <row r="5" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="27">
         <v>2</v>
       </c>
@@ -12607,7 +12601,7 @@
         <v>361131.5538461539</v>
       </c>
     </row>
-    <row r="6" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="27">
         <v>3</v>
       </c>
@@ -12636,7 +12630,7 @@
         <v>1267174</v>
       </c>
     </row>
-    <row r="7" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="27">
         <v>4</v>
       </c>
@@ -12664,7 +12658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" s="27">
         <v>5</v>
       </c>
@@ -12692,7 +12686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="27">
         <v>6</v>
       </c>
@@ -12720,7 +12714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="27">
         <v>7</v>
       </c>
@@ -12748,7 +12742,7 @@
         <v>157963.5</v>
       </c>
     </row>
-    <row r="11" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="27">
         <v>8</v>
       </c>
@@ -12770,7 +12764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="27">
         <v>9</v>
       </c>
@@ -12792,7 +12786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="27">
         <v>10</v>
       </c>
@@ -12814,7 +12808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="27">
         <v>11</v>
       </c>
@@ -12870,7 +12864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="27">
         <v>13</v>
       </c>
@@ -12888,7 +12882,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="17" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="27">
         <v>14</v>
       </c>
@@ -12906,7 +12900,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="18" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="27">
         <v>15</v>
       </c>
@@ -12924,7 +12918,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="19" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="27">
         <v>16</v>
       </c>
@@ -12948,7 +12942,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="20" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="27">
         <v>17</v>
       </c>
@@ -12972,7 +12966,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="21" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="27">
         <v>18</v>
       </c>
@@ -12996,7 +12990,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="22" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" s="27">
         <v>19</v>
       </c>
@@ -13020,7 +13014,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="23" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" s="27">
         <v>20</v>
       </c>
@@ -13044,7 +13038,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="24" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="27">
         <v>21</v>
       </c>
@@ -13062,7 +13056,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="25" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="27">
         <v>22</v>
       </c>
@@ -13083,7 +13077,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="26" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="27">
         <v>23</v>
       </c>
@@ -13101,7 +13095,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="27" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" s="27">
         <v>24</v>
       </c>
@@ -13128,7 +13122,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="28" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" s="27">
         <v>25</v>
       </c>
@@ -13146,7 +13140,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="29" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" s="27">
         <v>26</v>
       </c>
@@ -13164,7 +13158,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="30" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" s="27">
         <v>27</v>
       </c>
@@ -13182,7 +13176,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="31" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" s="27">
         <v>28</v>
       </c>
@@ -13200,7 +13194,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="32" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="27">
         <v>29</v>
       </c>
@@ -13218,7 +13212,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="33" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="27">
         <v>30</v>
       </c>
@@ -13236,7 +13230,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="34" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="27">
         <v>31</v>
       </c>
@@ -13254,7 +13248,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="35" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="27">
         <v>32</v>
       </c>
@@ -13276,7 +13270,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="36" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="27">
         <v>33</v>
       </c>
@@ -13298,7 +13292,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="37" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" s="27">
         <v>34</v>
       </c>
@@ -13316,7 +13310,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="38" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" s="27">
         <v>35</v>
       </c>
@@ -13334,7 +13328,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="39" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="27">
         <v>36</v>
       </c>
@@ -13352,7 +13346,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="40" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" s="27">
         <v>37</v>
       </c>
@@ -13370,7 +13364,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="41" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" s="27">
         <v>38</v>
       </c>
@@ -13388,7 +13382,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="42" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" s="27">
         <v>39</v>
       </c>
@@ -13410,7 +13404,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="43" spans="2:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" s="24"/>
       <c r="C43" s="25" t="s">
         <v>827</v>

</xml_diff>

<commit_message>
Atualiza planilha 06/10/2026 16:45
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2087" uniqueCount="843">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2103" uniqueCount="846">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2358,9 +2358,6 @@
     <t>Fechamento Lateral</t>
   </si>
   <si>
-    <t xml:space="preserve">Perfil Enrijecido </t>
-  </si>
-  <si>
     <t>Tela POP 10x10 Fio 4.2mm EQ138 2,45 x 6,00m</t>
   </si>
   <si>
@@ -2421,9 +2418,6 @@
     <t>SPDA do galpão completo</t>
   </si>
   <si>
-    <t>Telha Trapeizodal TP40 Fechamento Lateral</t>
-  </si>
-  <si>
     <t>Telha Trapeizodal TP40 Fechamento Telhado</t>
   </si>
   <si>
@@ -2554,6 +2548,21 @@
   </si>
   <si>
     <t>Arrasamento das estacas, locação dos blocos e concretagem dos cálices</t>
+  </si>
+  <si>
+    <t>Perfil Enrijecido A/C 150x50x20mm</t>
+  </si>
+  <si>
+    <t>Telha Trapeizodal TP40 6100mm #0,50mm</t>
+  </si>
+  <si>
+    <t>Fechamento Frontal</t>
+  </si>
+  <si>
+    <t>Telha Trapeizodal TP40 3000mm #0,50mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tubulação de drenagem pluvial </t>
   </si>
 </sst>
 </file>
@@ -2661,7 +2670,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2783,6 +2792,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -3061,8 +3073,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I45" totalsRowShown="0" dataDxfId="8">
-  <autoFilter ref="B3:I45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I48" totalsRowShown="0" dataDxfId="8">
+  <autoFilter ref="B3:I48"/>
+  <sortState ref="B4:I48">
+    <sortCondition ref="I3:I48"/>
+  </sortState>
   <tableColumns count="8">
     <tableColumn id="1" name="Item" dataDxfId="7" dataCellStyle="Normal"/>
     <tableColumn id="8" name="Local" dataDxfId="6"/>
@@ -12541,7 +12556,7 @@
         <v>767</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
     </row>
     <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -12549,7 +12564,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="D4" s="29">
         <v>4</v>
@@ -12606,7 +12621,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="D6" s="33">
         <f>2000/13*2</f>
@@ -12641,7 +12656,7 @@
         <v>167</v>
       </c>
       <c r="E7" s="27" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
       <c r="F7" s="32">
         <v>56.2</v>
@@ -12691,7 +12706,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="D9" s="27">
         <v>315</v>
@@ -12747,7 +12762,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="D11" s="17"/>
       <c r="E11" s="17"/>
@@ -12841,7 +12856,7 @@
         <v>12</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="D15" s="17">
         <v>1</v>
@@ -12905,7 +12920,7 @@
         <v>15</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="D18" s="22"/>
       <c r="E18" s="22"/>
@@ -12923,7 +12938,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="D19" s="27">
         <v>252</v>
@@ -12939,7 +12954,7 @@
         <v>67914</v>
       </c>
       <c r="H19" s="27" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
@@ -12947,7 +12962,7 @@
         <v>17</v>
       </c>
       <c r="C20" s="31" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="D20" s="27">
         <v>84</v>
@@ -12963,7 +12978,7 @@
         <v>9702</v>
       </c>
       <c r="H20" s="27" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
@@ -12971,7 +12986,7 @@
         <v>18</v>
       </c>
       <c r="C21" s="31" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D21" s="27">
         <v>42</v>
@@ -12987,7 +13002,7 @@
         <v>1470</v>
       </c>
       <c r="H21" s="27" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
@@ -12995,7 +13010,7 @@
         <v>19</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="D22" s="27">
         <v>4200</v>
@@ -13011,7 +13026,7 @@
         <v>2100</v>
       </c>
       <c r="H22" s="27" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
@@ -13019,7 +13034,7 @@
         <v>20</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="D23" s="27">
         <v>3100</v>
@@ -13035,7 +13050,7 @@
         <v>1550</v>
       </c>
       <c r="H23" s="27" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
@@ -13043,7 +13058,7 @@
         <v>21</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="D24" s="22"/>
       <c r="E24" s="22"/>
@@ -13061,7 +13076,7 @@
         <v>22</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
@@ -13071,10 +13086,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="22" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
@@ -13082,7 +13097,7 @@
         <v>23</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="D26" s="22"/>
       <c r="E26" s="22"/>
@@ -13100,7 +13115,7 @@
         <v>24</v>
       </c>
       <c r="C27" s="31" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="D27" s="27">
         <v>1</v>
@@ -13116,10 +13131,10 @@
         <v>157963.5</v>
       </c>
       <c r="H27" s="27" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
@@ -13127,7 +13142,7 @@
         <v>25</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="D28" s="22"/>
       <c r="E28" s="22"/>
@@ -13145,7 +13160,7 @@
         <v>26</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="D29" s="22"/>
       <c r="E29" s="22"/>
@@ -13163,7 +13178,7 @@
         <v>27</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="D30" s="22"/>
       <c r="E30" s="22"/>
@@ -13181,7 +13196,7 @@
         <v>28</v>
       </c>
       <c r="C31" s="25" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="D31" s="24"/>
       <c r="E31" s="24"/>
@@ -13199,7 +13214,7 @@
         <v>29</v>
       </c>
       <c r="C32" s="25" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="D32" s="24"/>
       <c r="E32" s="24"/>
@@ -13217,7 +13232,7 @@
         <v>30</v>
       </c>
       <c r="C33" s="25" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="D33" s="24"/>
       <c r="E33" s="24"/>
@@ -13235,7 +13250,7 @@
         <v>31</v>
       </c>
       <c r="C34" s="25" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="D34" s="24"/>
       <c r="E34" s="24"/>
@@ -13253,7 +13268,7 @@
         <v>32</v>
       </c>
       <c r="C35" s="25" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="D35" s="24">
         <v>10</v>
@@ -13275,7 +13290,7 @@
         <v>33</v>
       </c>
       <c r="C36" s="25" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D36" s="24">
         <v>500</v>
@@ -13297,7 +13312,7 @@
         <v>34</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="D37" s="24"/>
       <c r="E37" s="24"/>
@@ -13315,7 +13330,7 @@
         <v>35</v>
       </c>
       <c r="C38" s="25" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="D38" s="24"/>
       <c r="E38" s="24"/>
@@ -13333,7 +13348,7 @@
         <v>36</v>
       </c>
       <c r="C39" s="25" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="D39" s="24"/>
       <c r="E39" s="24"/>
@@ -13351,7 +13366,7 @@
         <v>37</v>
       </c>
       <c r="C40" s="25" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="D40" s="24"/>
       <c r="E40" s="24"/>
@@ -13369,7 +13384,7 @@
         <v>38</v>
       </c>
       <c r="C41" s="25" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="D41" s="24"/>
       <c r="E41" s="24"/>
@@ -13379,7 +13394,7 @@
         <v>0</v>
       </c>
       <c r="H41" s="24" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
@@ -13387,7 +13402,7 @@
         <v>39</v>
       </c>
       <c r="C42" s="25" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="D42" s="24">
         <v>1</v>
@@ -13401,13 +13416,13 @@
         <v>0</v>
       </c>
       <c r="H42" s="24" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" s="24"/>
       <c r="C43" s="25" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="D43" s="24">
         <v>1</v>
@@ -13421,7 +13436,7 @@
         <v>0</v>
       </c>
       <c r="H43" s="24" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
@@ -13459,17 +13474,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R48"/>
+  <dimension ref="B1:R51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
-    <col min="3" max="3" width="20" style="14" customWidth="1"/>
+    <col min="3" max="3" width="20" style="14" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="63.85546875" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" style="14" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" style="14" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" style="15" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="14" customWidth="1"/>
+    <col min="9" max="9" width="23.85546875" style="14" customWidth="1"/>
     <col min="10" max="13" width="16" style="14" customWidth="1"/>
     <col min="14" max="14" width="18.42578125" customWidth="1"/>
     <col min="15" max="15" width="25" customWidth="1"/>
@@ -13480,12 +13495,12 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P1" s="14" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P2" s="14" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
     </row>
     <row r="3" spans="2:18" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -13493,7 +13508,7 @@
         <v>753</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="D3" t="s">
         <v>754</v>
@@ -13514,7 +13529,7 @@
         <v>767</v>
       </c>
       <c r="P3" s="14" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
@@ -13522,39 +13537,32 @@
         <v>1</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>757</v>
-      </c>
-      <c r="E4" s="23">
-        <f>(2150*1.05)*0.15</f>
-        <v>338.625</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>759</v>
-      </c>
-      <c r="G4" s="20">
-        <v>670</v>
-      </c>
-      <c r="H4" s="20">
+        <v>816</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>798</v>
+      </c>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26">
         <f>G4*E4</f>
-        <v>226878.75</v>
-      </c>
-      <c r="I4" s="17" t="s">
-        <v>635</v>
+        <v>0</v>
+      </c>
+      <c r="I4" s="24" t="s">
+        <v>824</v>
       </c>
       <c r="O4" s="14" t="s">
+        <v>830</v>
+      </c>
+      <c r="P4" s="14" t="s">
         <v>832</v>
       </c>
-      <c r="P4" s="14" t="s">
+      <c r="Q4" s="14" t="s">
+        <v>833</v>
+      </c>
+      <c r="R4" s="14" t="s">
         <v>834</v>
-      </c>
-      <c r="Q4" s="14" t="s">
-        <v>835</v>
-      </c>
-      <c r="R4" s="14" t="s">
-        <v>836</v>
       </c>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
@@ -13562,27 +13570,20 @@
         <v>2</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D5" s="18" t="s">
+        <v>816</v>
+      </c>
+      <c r="D5" s="21" t="s">
         <v>778</v>
       </c>
-      <c r="E5" s="23">
-        <f>(2150/13)*2</f>
-        <v>330.76923076923077</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="G5" s="20">
-        <v>220.5</v>
-      </c>
-      <c r="H5" s="20">
-        <f t="shared" ref="H5:H36" si="0">G5*E5</f>
-        <v>72934.61538461539</v>
-      </c>
-      <c r="I5" s="17" t="s">
-        <v>635</v>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19">
+        <f>G5*E5</f>
+        <v>0</v>
+      </c>
+      <c r="I5" s="22" t="s">
+        <v>786</v>
       </c>
       <c r="N5" s="37" t="s">
         <v>772</v>
@@ -13592,7 +13593,7 @@
         <v>968004</v>
       </c>
       <c r="P5" s="44">
-        <f t="shared" ref="P5:P17" si="1">O5/$O$19</f>
+        <f t="shared" ref="P5:P17" si="0">O5/$O$21</f>
         <v>0.33062288469044115</v>
       </c>
       <c r="Q5" s="46">
@@ -13600,7 +13601,7 @@
         <v>0.33062288469044115</v>
       </c>
       <c r="R5" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.25">
@@ -13608,37 +13609,30 @@
         <v>3</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>758</v>
-      </c>
-      <c r="E6" s="17">
-        <f>2100/12</f>
-        <v>175</v>
-      </c>
-      <c r="F6" s="17" t="s">
-        <v>761</v>
-      </c>
-      <c r="G6" s="20">
-        <v>56.2</v>
-      </c>
-      <c r="H6" s="20">
-        <f t="shared" si="0"/>
-        <v>9835</v>
-      </c>
-      <c r="I6" s="17" t="s">
-        <v>635</v>
+        <v>816</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>780</v>
+      </c>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19">
+        <f>G6*E6</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="22" t="s">
+        <v>449</v>
       </c>
       <c r="N6" s="45" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="O6" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Terraplanagem",Tabela24[Preço Total])</f>
         <v>791792.51</v>
       </c>
       <c r="P6" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.27043764667551473</v>
       </c>
       <c r="Q6" s="46">
@@ -13646,7 +13640,7 @@
         <v>0.60106053136595583</v>
       </c>
       <c r="R6" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
@@ -13654,26 +13648,20 @@
         <v>4</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>762</v>
-      </c>
-      <c r="E7" s="17">
-        <v>1000</v>
-      </c>
-      <c r="F7" s="17" t="s">
-        <v>763</v>
-      </c>
-      <c r="G7" s="20">
-        <v>7.3</v>
-      </c>
-      <c r="H7" s="20">
-        <f t="shared" si="0"/>
-        <v>7300</v>
-      </c>
-      <c r="I7" s="17" t="s">
-        <v>635</v>
+        <v>816</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>845</v>
+      </c>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19">
+        <f>G7*E7</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="22" t="s">
+        <v>449</v>
       </c>
       <c r="N7" s="37" t="s">
         <v>635</v>
@@ -13683,7 +13671,7 @@
         <v>645545.6</v>
       </c>
       <c r="P7" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.22048684558247864</v>
       </c>
     </row>
@@ -13692,40 +13680,37 @@
         <v>5</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>824</v>
-      </c>
-      <c r="E8" s="23">
-        <f>E4</f>
-        <v>338.625</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>766</v>
-      </c>
-      <c r="G8" s="20">
-        <v>50</v>
-      </c>
-      <c r="H8" s="20">
-        <f t="shared" si="0"/>
-        <v>16931.25</v>
-      </c>
-      <c r="I8" s="17" t="s">
-        <v>635</v>
+        <v>816</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>794</v>
+      </c>
+      <c r="E8" s="24">
+        <v>26</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26">
+        <f>G8*E8</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="24" t="s">
+        <v>643</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="N8" s="45" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="O8" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
         <v>358477</v>
       </c>
       <c r="P8" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.12243823355603414</v>
       </c>
     </row>
@@ -13734,29 +13719,27 @@
         <v>6</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>768</v>
-      </c>
-      <c r="E9" s="17">
-        <v>1</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="G9" s="20">
-        <v>49800</v>
-      </c>
-      <c r="H9" s="20">
-        <f t="shared" si="0"/>
-        <v>49800</v>
-      </c>
-      <c r="I9" s="17" t="s">
-        <v>635</v>
+        <v>816</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>795</v>
+      </c>
+      <c r="E9" s="24">
+        <v>500</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>761</v>
+      </c>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26">
+        <f>G9*E9</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="24" t="s">
+        <v>643</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="N9" s="42" t="s">
         <v>771</v>
@@ -13766,7 +13749,7 @@
         <v>164000</v>
       </c>
       <c r="P9" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5.6014389495531371E-2</v>
       </c>
     </row>
@@ -13775,20 +13758,20 @@
         <v>7</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>801</v>
-      </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20">
+        <v>816</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>823</v>
+      </c>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26">
         <f>G10*E10</f>
         <v>0</v>
       </c>
-      <c r="I10" s="17" t="s">
-        <v>771</v>
+      <c r="I10" s="24" t="s">
+        <v>643</v>
       </c>
       <c r="N10" s="42" t="s">
         <v>776</v>
@@ -13798,7 +13781,7 @@
         <v>0</v>
       </c>
       <c r="P10" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -13807,30 +13790,34 @@
         <v>8</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>769</v>
-      </c>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20">
-        <f t="shared" si="0"/>
+        <v>816</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>842</v>
+      </c>
+      <c r="E11" s="22">
+        <v>54</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19">
+        <f>G11*E11</f>
         <v>0</v>
       </c>
-      <c r="I11" s="17" t="s">
-        <v>771</v>
+      <c r="I11" s="22" t="s">
+        <v>843</v>
       </c>
       <c r="N11" s="41" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="O11" s="40">
         <f>SUMIF(Tabela24[Aplicação],"AVCB",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
       <c r="P11" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -13839,20 +13826,24 @@
         <v>9</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>770</v>
-      </c>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20">
-        <f t="shared" si="0"/>
+        <v>816</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>844</v>
+      </c>
+      <c r="E12" s="22">
+        <v>30</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19">
+        <f>G12*E12</f>
         <v>0</v>
       </c>
-      <c r="I12" s="17" t="s">
-        <v>771</v>
+      <c r="I12" s="22" t="s">
+        <v>843</v>
       </c>
       <c r="N12" s="41" t="s">
         <v>449</v>
@@ -13862,33 +13853,33 @@
         <v>0</v>
       </c>
       <c r="P12" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B13" s="17"/>
+      <c r="B13" s="17">
+        <v>10</v>
+      </c>
       <c r="C13" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>842</v>
-      </c>
-      <c r="E13" s="17">
-        <v>1</v>
-      </c>
-      <c r="F13" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="G13" s="20">
-        <v>164000</v>
-      </c>
-      <c r="H13" s="20">
+        <v>816</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>841</v>
+      </c>
+      <c r="E13" s="24">
+        <v>390</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>761</v>
+      </c>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19">
         <f>G13*E13</f>
-        <v>164000</v>
-      </c>
-      <c r="I13" s="17" t="s">
-        <v>771</v>
+        <v>0</v>
+      </c>
+      <c r="I13" s="22" t="s">
+        <v>843</v>
       </c>
       <c r="N13" s="41"/>
       <c r="O13" s="40"/>
@@ -13896,29 +13887,28 @@
     </row>
     <row r="14" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B14" s="17">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>773</v>
-      </c>
-      <c r="E14" s="17">
-        <v>1</v>
-      </c>
-      <c r="F14" s="17" t="s">
+        <v>816</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>842</v>
+      </c>
+      <c r="E14" s="47">
+        <f>(84*1.02)*2*1.02</f>
+        <v>174.78720000000001</v>
+      </c>
+      <c r="F14" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="G14" s="20">
-        <v>968004</v>
-      </c>
-      <c r="H14" s="20">
-        <f t="shared" si="0"/>
-        <v>968004</v>
-      </c>
-      <c r="I14" s="17" t="s">
-        <v>772</v>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19">
+        <f>G14*E14</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="22" t="s">
+        <v>776</v>
       </c>
       <c r="N14" s="41" t="s">
         <v>776</v>
@@ -13928,29 +13918,34 @@
         <v>0</v>
       </c>
       <c r="P14" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B15" s="17">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>774</v>
-      </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20">
-        <f t="shared" si="0"/>
+        <v>816</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>841</v>
+      </c>
+      <c r="E15" s="22">
+        <f>84*7</f>
+        <v>588</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>761</v>
+      </c>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19">
+        <f>G15*E15</f>
         <v>0</v>
       </c>
-      <c r="I15" s="17" t="s">
-        <v>771</v>
+      <c r="I15" s="22" t="s">
+        <v>776</v>
       </c>
       <c r="N15" s="41" t="s">
         <v>643</v>
@@ -13960,29 +13955,31 @@
         <v>0</v>
       </c>
       <c r="P15" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B16" s="17">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>775</v>
-      </c>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20">
-        <f t="shared" si="0"/>
+        <v>816</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>782</v>
+      </c>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24" t="s">
+        <v>761</v>
+      </c>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26">
+        <f>G16*E16</f>
         <v>0</v>
       </c>
-      <c r="I16" s="17" t="s">
-        <v>771</v>
+      <c r="I16" s="24" t="s">
+        <v>776</v>
       </c>
       <c r="N16" s="41" t="s">
         <v>576</v>
@@ -13992,544 +13989,594 @@
         <v>0</v>
       </c>
       <c r="P16" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" s="17">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D17" s="21" t="s">
-        <v>798</v>
-      </c>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19">
-        <f t="shared" si="0"/>
+        <v>816</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>783</v>
+      </c>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26">
+        <f>G17*E17</f>
         <v>0</v>
       </c>
-      <c r="I17" s="22" t="s">
+      <c r="I17" s="24" t="s">
         <v>776</v>
       </c>
       <c r="N17" s="41" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="O17" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
       <c r="P17" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" s="17">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>799</v>
-      </c>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19">
+        <v>816</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>784</v>
+      </c>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26">
         <f>G18*E18</f>
         <v>0</v>
       </c>
-      <c r="I18" s="17" t="s">
-        <v>772</v>
-      </c>
+      <c r="I18" s="24" t="s">
+        <v>776</v>
+      </c>
+      <c r="N18" s="41"/>
+      <c r="O18" s="40"/>
+      <c r="P18" s="44"/>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B19" s="17">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>777</v>
-      </c>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19">
-        <f t="shared" si="0"/>
+        <v>816</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>828</v>
+      </c>
+      <c r="E19" s="24">
+        <v>1</v>
+      </c>
+      <c r="F19" s="24"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26">
+        <f>G19*E19</f>
         <v>0</v>
       </c>
-      <c r="I19" s="22" t="s">
+      <c r="I19" s="24" t="s">
         <v>776</v>
       </c>
-      <c r="N19" s="41" t="s">
-        <v>833</v>
-      </c>
-      <c r="O19" s="43">
+      <c r="N19" s="41"/>
+      <c r="O19" s="40"/>
+      <c r="P19" s="44"/>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B20" s="17">
+        <v>17</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>816</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>799</v>
+      </c>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20">
+        <f>G20*E20</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="17" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B21" s="17">
+        <v>18</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>816</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>769</v>
+      </c>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20">
+        <f>G21*E21</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="N21" s="41" t="s">
+        <v>831</v>
+      </c>
+      <c r="O21" s="43">
         <f>SUM(O5:O17)</f>
         <v>2927819.11</v>
       </c>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B20" s="17">
-        <v>16</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>779</v>
-      </c>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I20" s="22" t="s">
-        <v>787</v>
-      </c>
-    </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B21" s="17">
-        <v>17</v>
-      </c>
-      <c r="C21" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>797</v>
-      </c>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I21" s="22" t="s">
-        <v>419</v>
-      </c>
-    </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B22" s="17">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>789</v>
-      </c>
-      <c r="E22" s="22">
-        <v>1</v>
-      </c>
-      <c r="F22" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G22" s="19">
-        <v>791792.51</v>
-      </c>
-      <c r="H22" s="19">
-        <f t="shared" si="0"/>
-        <v>791792.51</v>
-      </c>
-      <c r="I22" s="22" t="s">
-        <v>788</v>
-      </c>
+        <v>816</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>770</v>
+      </c>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20">
+        <f>G22*E22</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="N22" s="41"/>
+      <c r="O22" s="43"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B23" s="17">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>780</v>
-      </c>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I23" s="22" t="s">
+        <v>816</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>840</v>
+      </c>
+      <c r="E23" s="17">
+        <v>1</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G23" s="20">
+        <v>164000</v>
+      </c>
+      <c r="H23" s="20">
+        <f>G23*E23</f>
+        <v>164000</v>
+      </c>
+      <c r="I23" s="17" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B24" s="17">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>781</v>
-      </c>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="19">
-        <f t="shared" si="0"/>
+        <v>816</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>774</v>
+      </c>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="20">
+        <f>G24*E24</f>
         <v>0</v>
       </c>
-      <c r="I24" s="22" t="s">
-        <v>449</v>
+      <c r="I24" s="17" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B25" s="17">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>782</v>
-      </c>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19">
-        <f t="shared" si="0"/>
+        <v>816</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>775</v>
+      </c>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20">
+        <f>G25*E25</f>
         <v>0</v>
       </c>
-      <c r="I25" s="22" t="s">
-        <v>449</v>
+      <c r="I25" s="17" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B26" s="17">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D26" s="25" t="s">
-        <v>783</v>
-      </c>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="26">
-        <f t="shared" si="0"/>
+        <v>816</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>779</v>
+      </c>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19">
+        <f>G26*E26</f>
         <v>0</v>
       </c>
-      <c r="I26" s="24" t="s">
-        <v>776</v>
+      <c r="I26" s="22" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B27" s="17">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>784</v>
+        <v>789</v>
       </c>
       <c r="E27" s="24"/>
       <c r="F27" s="24"/>
       <c r="G27" s="26"/>
       <c r="H27" s="26">
-        <f t="shared" si="0"/>
+        <f>G27*E27</f>
         <v>0</v>
       </c>
       <c r="I27" s="24" t="s">
-        <v>776</v>
+        <v>576</v>
       </c>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B28" s="17">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="D28" s="25" t="s">
-        <v>785</v>
+        <v>790</v>
       </c>
       <c r="E28" s="24"/>
       <c r="F28" s="24"/>
       <c r="G28" s="26"/>
       <c r="H28" s="26">
-        <f t="shared" si="0"/>
+        <f>G28*E28</f>
         <v>0</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>776</v>
+        <v>576</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B29" s="17">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>830</v>
-      </c>
-      <c r="E29" s="24">
-        <v>1</v>
-      </c>
+        <v>791</v>
+      </c>
+      <c r="E29" s="24"/>
       <c r="F29" s="24"/>
       <c r="G29" s="26"/>
       <c r="H29" s="26">
-        <f t="shared" si="0"/>
+        <f>G29*E29</f>
         <v>0</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>776</v>
+        <v>576</v>
       </c>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B30" s="17">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="D30" s="25" t="s">
-        <v>795</v>
-      </c>
-      <c r="E30" s="24">
-        <v>10</v>
-      </c>
+        <v>792</v>
+      </c>
+      <c r="E30" s="24"/>
       <c r="F30" s="24"/>
       <c r="G30" s="26"/>
       <c r="H30" s="26">
-        <f t="shared" si="0"/>
+        <f>G30*E30</f>
         <v>0</v>
       </c>
       <c r="I30" s="24" t="s">
-        <v>643</v>
+        <v>576</v>
       </c>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B31" s="17">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D31" s="25" t="s">
-        <v>796</v>
-      </c>
-      <c r="E31" s="24">
-        <v>500</v>
-      </c>
-      <c r="F31" s="24" t="s">
-        <v>761</v>
-      </c>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I31" s="24" t="s">
-        <v>643</v>
+        <v>816</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>757</v>
+      </c>
+      <c r="E31" s="23">
+        <f>(2150*1.05)*0.15</f>
+        <v>338.625</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>759</v>
+      </c>
+      <c r="G31" s="20">
+        <v>670</v>
+      </c>
+      <c r="H31" s="20">
+        <f>G31*E31</f>
+        <v>226878.75</v>
+      </c>
+      <c r="I31" s="17" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B32" s="17"/>
+      <c r="B32" s="17">
+        <v>29</v>
+      </c>
       <c r="C32" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D32" s="25" t="s">
-        <v>825</v>
-      </c>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26">
+        <v>816</v>
+      </c>
+      <c r="D32" s="18" t="s">
+        <v>777</v>
+      </c>
+      <c r="E32" s="23">
+        <f>(2150/13)*2</f>
+        <v>330.76923076923077</v>
+      </c>
+      <c r="F32" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G32" s="20">
+        <v>220.5</v>
+      </c>
+      <c r="H32" s="20">
         <f>G32*E32</f>
-        <v>0</v>
-      </c>
-      <c r="I32" s="24" t="s">
-        <v>643</v>
+        <v>72934.61538461539</v>
+      </c>
+      <c r="I32" s="17" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" s="17">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D33" s="25" t="s">
-        <v>790</v>
-      </c>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I33" s="24" t="s">
-        <v>576</v>
+        <v>816</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>758</v>
+      </c>
+      <c r="E33" s="17">
+        <f>2100/12</f>
+        <v>175</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>761</v>
+      </c>
+      <c r="G33" s="20">
+        <v>56.2</v>
+      </c>
+      <c r="H33" s="20">
+        <f>G33*E33</f>
+        <v>9835</v>
+      </c>
+      <c r="I33" s="17" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" s="17">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D34" s="25" t="s">
-        <v>791</v>
-      </c>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I34" s="24" t="s">
-        <v>576</v>
+        <v>816</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>762</v>
+      </c>
+      <c r="E34" s="17">
+        <v>1000</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>763</v>
+      </c>
+      <c r="G34" s="20">
+        <v>7.3</v>
+      </c>
+      <c r="H34" s="20">
+        <f>G34*E34</f>
+        <v>7300</v>
+      </c>
+      <c r="I34" s="17" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" s="17">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D35" s="25" t="s">
-        <v>792</v>
-      </c>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I35" s="24" t="s">
-        <v>576</v>
+        <v>816</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>822</v>
+      </c>
+      <c r="E35" s="23">
+        <f>E31</f>
+        <v>338.625</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>766</v>
+      </c>
+      <c r="G35" s="20">
+        <v>50</v>
+      </c>
+      <c r="H35" s="20">
+        <f>G35*E35</f>
+        <v>16931.25</v>
+      </c>
+      <c r="I35" s="17" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" s="17">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>818</v>
-      </c>
-      <c r="D36" s="25" t="s">
-        <v>793</v>
-      </c>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I36" s="24" t="s">
-        <v>576</v>
+        <v>816</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>768</v>
+      </c>
+      <c r="E36" s="17">
+        <v>1</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G36" s="20">
+        <v>49800</v>
+      </c>
+      <c r="H36" s="20">
+        <f>G36*E36</f>
+        <v>49800</v>
+      </c>
+      <c r="I36" s="17" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B37" s="17">
-        <v>32</v>
-      </c>
-      <c r="C37" s="17" t="s">
-        <v>818</v>
+        <v>34</v>
+      </c>
+      <c r="C37" s="34" t="s">
+        <v>817</v>
       </c>
       <c r="D37" s="25" t="s">
-        <v>800</v>
-      </c>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
+        <v>827</v>
+      </c>
+      <c r="E37" s="24">
+        <v>110</v>
+      </c>
+      <c r="F37" s="24" t="s">
+        <v>760</v>
+      </c>
       <c r="G37" s="26"/>
       <c r="H37" s="26">
         <f>G37*E37</f>
         <v>0</v>
       </c>
       <c r="I37" s="24" t="s">
-        <v>826</v>
+        <v>635</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B38" s="17">
-        <v>33</v>
-      </c>
-      <c r="C38" s="17" t="s">
-        <v>819</v>
+        <v>35</v>
+      </c>
+      <c r="C38" s="34" t="s">
+        <v>817</v>
       </c>
       <c r="D38" s="25" t="s">
-        <v>813</v>
-      </c>
-      <c r="E38" s="24">
-        <v>1</v>
+        <v>757</v>
+      </c>
+      <c r="E38" s="35">
+        <f>(1784*0.15)*1.05</f>
+        <v>280.97999999999996</v>
       </c>
       <c r="F38" s="24" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G38" s="26">
-        <v>46600</v>
+        <v>670</v>
       </c>
       <c r="H38" s="26">
-        <f t="shared" ref="H38:H41" si="2">G38*E38</f>
-        <v>46600</v>
+        <f>G38*E38</f>
+        <v>188256.59999999998</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>815</v>
+        <v>635</v>
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B39" s="17">
-        <v>34</v>
-      </c>
-      <c r="C39" s="17" t="s">
-        <v>819</v>
-      </c>
-      <c r="D39" s="25" t="s">
-        <v>816</v>
-      </c>
-      <c r="E39" s="24">
-        <v>1</v>
+        <v>36</v>
+      </c>
+      <c r="C39" s="34" t="s">
+        <v>817</v>
+      </c>
+      <c r="D39" s="18" t="s">
+        <v>777</v>
+      </c>
+      <c r="E39" s="35">
+        <f>1784/13</f>
+        <v>137.23076923076923</v>
       </c>
       <c r="F39" s="24" t="s">
         <v>760</v>
       </c>
       <c r="G39" s="26">
-        <v>8100</v>
+        <v>220.5</v>
       </c>
       <c r="H39" s="26">
         <f>G39*E39</f>
-        <v>8100</v>
+        <v>30259.384615384613</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>815</v>
+        <v>635</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B40" s="17">
-        <v>35</v>
-      </c>
-      <c r="C40" s="17" t="s">
-        <v>819</v>
+        <v>37</v>
+      </c>
+      <c r="C40" s="34" t="s">
+        <v>817</v>
       </c>
       <c r="D40" s="25" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
       <c r="E40" s="24">
         <v>1</v>
@@ -14538,133 +14585,127 @@
         <v>760</v>
       </c>
       <c r="G40" s="26">
-        <v>5000</v>
+        <v>43350</v>
       </c>
       <c r="H40" s="26">
         <f>G40*E40</f>
-        <v>5000</v>
+        <v>43350</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>815</v>
+        <v>635</v>
       </c>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B41" s="17">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C41" s="17" t="s">
-        <v>819</v>
-      </c>
-      <c r="D41" s="25" t="s">
-        <v>820</v>
-      </c>
-      <c r="E41" s="24">
-        <v>1</v>
-      </c>
-      <c r="F41" s="24" t="s">
+        <v>816</v>
+      </c>
+      <c r="D41" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="E41" s="17">
+        <v>1</v>
+      </c>
+      <c r="F41" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G41" s="26">
-        <v>298777</v>
-      </c>
-      <c r="H41" s="26">
-        <f t="shared" si="2"/>
-        <v>298777</v>
-      </c>
-      <c r="I41" s="24" t="s">
-        <v>815</v>
+      <c r="G41" s="20">
+        <v>968004</v>
+      </c>
+      <c r="H41" s="20">
+        <f>G41*E41</f>
+        <v>968004</v>
+      </c>
+      <c r="I41" s="17" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B42" s="17">
-        <v>37</v>
-      </c>
-      <c r="C42" s="34" t="s">
-        <v>819</v>
-      </c>
-      <c r="D42" s="25" t="s">
-        <v>829</v>
-      </c>
-      <c r="E42" s="24">
-        <v>110</v>
-      </c>
-      <c r="F42" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G42" s="26"/>
-      <c r="H42" s="26">
+        <v>39</v>
+      </c>
+      <c r="C42" s="17" t="s">
+        <v>816</v>
+      </c>
+      <c r="D42" s="21" t="s">
+        <v>797</v>
+      </c>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="19"/>
+      <c r="H42" s="19">
         <f>G42*E42</f>
         <v>0</v>
       </c>
-      <c r="I42" s="24" t="s">
-        <v>635</v>
+      <c r="I42" s="17" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B43" s="17">
-        <v>38</v>
-      </c>
-      <c r="C43" s="34" t="s">
-        <v>819</v>
+        <v>40</v>
+      </c>
+      <c r="C43" s="17" t="s">
+        <v>817</v>
       </c>
       <c r="D43" s="25" t="s">
-        <v>757</v>
-      </c>
-      <c r="E43" s="35">
-        <f>(1784*0.15)*1.05</f>
-        <v>280.97999999999996</v>
+        <v>811</v>
+      </c>
+      <c r="E43" s="24">
+        <v>1</v>
       </c>
       <c r="F43" s="24" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="G43" s="26">
-        <v>670</v>
+        <v>46600</v>
       </c>
       <c r="H43" s="26">
-        <f t="shared" ref="H43:H44" si="3">G43*E43</f>
-        <v>188256.59999999998</v>
+        <f>G43*E43</f>
+        <v>46600</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>635</v>
+        <v>813</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B44" s="17">
-        <v>40</v>
-      </c>
-      <c r="C44" s="34" t="s">
-        <v>819</v>
-      </c>
-      <c r="D44" s="18" t="s">
-        <v>778</v>
-      </c>
-      <c r="E44" s="35">
-        <f>1784/13</f>
-        <v>137.23076923076923</v>
+        <v>41</v>
+      </c>
+      <c r="C44" s="17" t="s">
+        <v>817</v>
+      </c>
+      <c r="D44" s="25" t="s">
+        <v>814</v>
+      </c>
+      <c r="E44" s="24">
+        <v>1</v>
       </c>
       <c r="F44" s="24" t="s">
         <v>760</v>
       </c>
       <c r="G44" s="26">
-        <v>220.5</v>
+        <v>8100</v>
       </c>
       <c r="H44" s="26">
-        <f t="shared" si="3"/>
-        <v>30259.384615384613</v>
+        <f>G44*E44</f>
+        <v>8100</v>
       </c>
       <c r="I44" s="24" t="s">
-        <v>635</v>
+        <v>813</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B45" s="17">
-        <v>41</v>
-      </c>
-      <c r="C45" s="34" t="s">
-        <v>819</v>
+        <v>42</v>
+      </c>
+      <c r="C45" s="17" t="s">
+        <v>817</v>
       </c>
       <c r="D45" s="25" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="E45" s="24">
         <v>1</v>
@@ -14673,39 +14714,114 @@
         <v>760</v>
       </c>
       <c r="G45" s="26">
-        <v>43350</v>
+        <v>5000</v>
       </c>
       <c r="H45" s="26">
         <f>G45*E45</f>
-        <v>43350</v>
+        <v>5000</v>
       </c>
       <c r="I45" s="24" t="s">
-        <v>635</v>
+        <v>813</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B46" s="24"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="25"/>
-      <c r="E46" s="24"/>
-      <c r="F46" s="24"/>
-      <c r="G46" s="26"/>
-      <c r="H46" s="26"/>
-      <c r="I46" s="25"/>
+      <c r="B46" s="17">
+        <v>43</v>
+      </c>
+      <c r="C46" s="17" t="s">
+        <v>817</v>
+      </c>
+      <c r="D46" s="25" t="s">
+        <v>818</v>
+      </c>
+      <c r="E46" s="24">
+        <v>1</v>
+      </c>
+      <c r="F46" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G46" s="26">
+        <v>298777</v>
+      </c>
+      <c r="H46" s="26">
+        <f>G46*E46</f>
+        <v>298777</v>
+      </c>
+      <c r="I46" s="24" t="s">
+        <v>813</v>
+      </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="24"/>
-      <c r="C47" s="34"/>
-      <c r="D47" s="39"/>
-      <c r="E47" s="24"/>
-      <c r="F47" s="24"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="26"/>
-      <c r="I47" s="25"/>
+      <c r="B47" s="17">
+        <v>44</v>
+      </c>
+      <c r="C47" s="17" t="s">
+        <v>816</v>
+      </c>
+      <c r="D47" s="21" t="s">
+        <v>796</v>
+      </c>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="19"/>
+      <c r="H47" s="19">
+        <f>G47*E47</f>
+        <v>0</v>
+      </c>
+      <c r="I47" s="22" t="s">
+        <v>419</v>
+      </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D48" s="38"/>
-      <c r="H48" s="16">
+      <c r="B48" s="17">
+        <v>45</v>
+      </c>
+      <c r="C48" s="17" t="s">
+        <v>816</v>
+      </c>
+      <c r="D48" s="21" t="s">
+        <v>788</v>
+      </c>
+      <c r="E48" s="22">
+        <v>1</v>
+      </c>
+      <c r="F48" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G48" s="19">
+        <v>791792.51</v>
+      </c>
+      <c r="H48" s="19">
+        <f>G48*E48</f>
+        <v>791792.51</v>
+      </c>
+      <c r="I48" s="22" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B49" s="24"/>
+      <c r="C49" s="34"/>
+      <c r="D49" s="25"/>
+      <c r="E49" s="24"/>
+      <c r="F49" s="24"/>
+      <c r="G49" s="26"/>
+      <c r="H49" s="26"/>
+      <c r="I49" s="25"/>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B50" s="24"/>
+      <c r="C50" s="34"/>
+      <c r="D50" s="39"/>
+      <c r="E50" s="24"/>
+      <c r="F50" s="24"/>
+      <c r="G50" s="26"/>
+      <c r="H50" s="26"/>
+      <c r="I50" s="25"/>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D51" s="38"/>
+      <c r="H51" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
         <v>2927819.1100000003</v>
       </c>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 08:45
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2103" uniqueCount="846">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="849">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2563,6 +2563,15 @@
   </si>
   <si>
     <t xml:space="preserve">Tubulação de drenagem pluvial </t>
+  </si>
+  <si>
+    <t>Execução da fundação profunda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concreto FCK 30 Brita 0 Slump 20±2 fundação profunda </t>
+  </si>
+  <si>
+    <t>Concreto FCK 30 Brita 0 Slump 10±2 cálices e blocos</t>
   </si>
 </sst>
 </file>
@@ -3055,8 +3064,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H43" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:H43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H45" totalsRowShown="0" dataDxfId="16">
+  <autoFilter ref="B3:H45"/>
+  <sortState ref="B4:H43">
+    <sortCondition ref="H3:H43"/>
+  </sortState>
   <tableColumns count="7">
     <tableColumn id="1" name="Item" dataDxfId="15" dataCellStyle="Normal"/>
     <tableColumn id="2" name="Descrição" dataDxfId="14" dataCellStyle="Normal"/>
@@ -12519,7 +12531,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:J46"/>
+  <dimension ref="B3:J48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -12563,53 +12575,40 @@
       <c r="B4" s="27">
         <v>1</v>
       </c>
-      <c r="C4" s="28" t="s">
-        <v>802</v>
-      </c>
-      <c r="D4" s="29">
-        <v>4</v>
-      </c>
-      <c r="E4" s="29" t="s">
-        <v>760</v>
-      </c>
-      <c r="F4" s="30">
-        <v>1500</v>
-      </c>
-      <c r="G4" s="30">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>6000</v>
-      </c>
-      <c r="H4" s="29" t="s">
-        <v>771</v>
+      <c r="C4" s="21" t="s">
+        <v>778</v>
+      </c>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19">
+        <f>F4*D4</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="22" t="s">
+        <v>786</v>
       </c>
       <c r="J4" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
-        <v>186000</v>
+        <v>298280</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="27">
         <v>2</v>
       </c>
-      <c r="C5" s="31" t="s">
-        <v>757</v>
-      </c>
-      <c r="D5" s="27">
-        <f>(2000*1.05)*0.15</f>
-        <v>315</v>
-      </c>
-      <c r="E5" s="27" t="s">
-        <v>759</v>
-      </c>
-      <c r="F5" s="32">
-        <v>670</v>
-      </c>
-      <c r="G5" s="32">
+      <c r="C5" s="21" t="s">
+        <v>780</v>
+      </c>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19">
         <f>F5*D5</f>
-        <v>211050</v>
-      </c>
-      <c r="H5" s="27" t="s">
-        <v>635</v>
+        <v>0</v>
+      </c>
+      <c r="H5" s="22" t="s">
+        <v>449</v>
       </c>
       <c r="J5" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Piso",Tabela2[Preço Total])</f>
@@ -12620,25 +12619,18 @@
       <c r="B6" s="27">
         <v>3</v>
       </c>
-      <c r="C6" s="31" t="s">
-        <v>777</v>
-      </c>
-      <c r="D6" s="33">
-        <f>2000/13*2</f>
-        <v>307.69230769230768</v>
-      </c>
-      <c r="E6" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="F6" s="32">
-        <v>220.5</v>
-      </c>
-      <c r="G6" s="32">
-        <f t="shared" ref="G6:G17" si="0">F6*D6</f>
-        <v>67846.153846153844</v>
-      </c>
-      <c r="H6" s="27" t="s">
-        <v>635</v>
+      <c r="C6" s="21" t="s">
+        <v>781</v>
+      </c>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19">
+        <f>F6*D6</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="22" t="s">
+        <v>449</v>
       </c>
       <c r="J6" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Pré Moldado",Tabela2[Preço Total])</f>
@@ -12649,24 +12641,22 @@
       <c r="B7" s="27">
         <v>4</v>
       </c>
-      <c r="C7" s="31" t="s">
-        <v>758</v>
-      </c>
-      <c r="D7" s="27">
-        <v>167</v>
-      </c>
-      <c r="E7" s="27" t="s">
-        <v>820</v>
-      </c>
-      <c r="F7" s="32">
-        <v>56.2</v>
-      </c>
-      <c r="G7" s="32">
-        <f t="shared" si="0"/>
-        <v>9385.4</v>
-      </c>
-      <c r="H7" s="27" t="s">
-        <v>635</v>
+      <c r="C7" s="25" t="s">
+        <v>794</v>
+      </c>
+      <c r="D7" s="24">
+        <v>10</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26">
+        <f>F7*D7</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>643</v>
       </c>
       <c r="J7" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Fechamento Lateral",Tabela2[Preço Total])</f>
@@ -12677,24 +12667,22 @@
       <c r="B8" s="27">
         <v>5</v>
       </c>
-      <c r="C8" s="31" t="s">
-        <v>762</v>
-      </c>
-      <c r="D8" s="27">
-        <v>1000</v>
-      </c>
-      <c r="E8" s="27" t="s">
-        <v>763</v>
-      </c>
-      <c r="F8" s="32">
-        <v>7.3</v>
-      </c>
-      <c r="G8" s="32">
-        <f t="shared" si="0"/>
-        <v>7300</v>
-      </c>
-      <c r="H8" s="27" t="s">
-        <v>635</v>
+      <c r="C8" s="25" t="s">
+        <v>795</v>
+      </c>
+      <c r="D8" s="24">
+        <v>500</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>761</v>
+      </c>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26">
+        <f>F8*D8</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="24" t="s">
+        <v>643</v>
       </c>
       <c r="J8" s="40">
         <f>SUMIF(Tabela2[Aplicação],"AVCB",Tabela2[Preço Total])</f>
@@ -12705,24 +12693,18 @@
       <c r="B9" s="27">
         <v>6</v>
       </c>
-      <c r="C9" s="31" t="s">
-        <v>810</v>
-      </c>
-      <c r="D9" s="27">
-        <v>315</v>
-      </c>
-      <c r="E9" s="27" t="s">
-        <v>759</v>
-      </c>
-      <c r="F9" s="32">
-        <v>50</v>
-      </c>
-      <c r="G9" s="32">
-        <f t="shared" si="0"/>
-        <v>15750</v>
-      </c>
-      <c r="H9" s="27" t="s">
-        <v>635</v>
+      <c r="C9" s="25" t="s">
+        <v>798</v>
+      </c>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26">
+        <f>F9*D9</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="24" t="s">
+        <v>801</v>
       </c>
       <c r="J9" s="40">
         <f>SUMIF(Tabela2[Aplicação],"SPDA",Tabela2[Preço Total])</f>
@@ -12733,24 +12715,18 @@
       <c r="B10" s="27">
         <v>7</v>
       </c>
-      <c r="C10" s="31" t="s">
-        <v>768</v>
-      </c>
-      <c r="D10" s="27">
-        <v>1</v>
-      </c>
-      <c r="E10" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="F10" s="32">
-        <v>49800</v>
-      </c>
-      <c r="G10" s="32">
-        <f t="shared" si="0"/>
-        <v>49800</v>
-      </c>
-      <c r="H10" s="27" t="s">
-        <v>635</v>
+      <c r="C10" s="21" t="s">
+        <v>805</v>
+      </c>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19">
+        <f>F10*D10</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="22" t="s">
+        <v>776</v>
       </c>
       <c r="J10" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Terraplanagem",Tabela2[Preço Total])</f>
@@ -12761,18 +12737,18 @@
       <c r="B11" s="27">
         <v>8</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>800</v>
-      </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20">
+      <c r="C11" s="21" t="s">
+        <v>803</v>
+      </c>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19">
         <f>F11*D11</f>
         <v>0</v>
       </c>
-      <c r="H11" s="17" t="s">
-        <v>771</v>
+      <c r="H11" s="22" t="s">
+        <v>776</v>
       </c>
       <c r="J11" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Drenagem",Tabela2[Preço Total])</f>
@@ -12783,18 +12759,18 @@
       <c r="B12" s="27">
         <v>9</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>769</v>
-      </c>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20">
-        <f t="shared" si="0"/>
+      <c r="C12" s="25" t="s">
+        <v>782</v>
+      </c>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26">
+        <f>F12*D12</f>
         <v>0</v>
       </c>
-      <c r="H12" s="17" t="s">
-        <v>771</v>
+      <c r="H12" s="24" t="s">
+        <v>776</v>
       </c>
       <c r="J12" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Elétrica",Tabela2[Preço Total])</f>
@@ -12805,18 +12781,18 @@
       <c r="B13" s="27">
         <v>10</v>
       </c>
-      <c r="C13" s="18" t="s">
-        <v>770</v>
-      </c>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20">
-        <f t="shared" si="0"/>
+      <c r="C13" s="25" t="s">
+        <v>783</v>
+      </c>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26">
+        <f>F13*D13</f>
         <v>0</v>
       </c>
-      <c r="H13" s="17" t="s">
-        <v>771</v>
+      <c r="H13" s="24" t="s">
+        <v>776</v>
       </c>
       <c r="J13" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Pintura",Tabela2[Preço Total])</f>
@@ -12827,24 +12803,18 @@
       <c r="B14" s="27">
         <v>11</v>
       </c>
-      <c r="C14" s="31" t="s">
-        <v>773</v>
-      </c>
-      <c r="D14" s="27">
-        <v>1</v>
-      </c>
-      <c r="E14" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="F14" s="32">
-        <v>1267174</v>
-      </c>
-      <c r="G14" s="32">
-        <f t="shared" si="0"/>
-        <v>1267174</v>
-      </c>
-      <c r="H14" s="27" t="s">
-        <v>772</v>
+      <c r="C14" s="25" t="s">
+        <v>784</v>
+      </c>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26">
+        <f>F14*D14</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="24" t="s">
+        <v>776</v>
       </c>
       <c r="J14" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Estrura Armazenamento",Tabela2[Preço Total])</f>
@@ -12855,24 +12825,18 @@
       <c r="B15" s="27">
         <v>12</v>
       </c>
-      <c r="C15" s="18" t="s">
-        <v>839</v>
-      </c>
-      <c r="D15" s="17">
-        <v>1</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="F15" s="20">
-        <v>180000</v>
-      </c>
-      <c r="G15" s="20">
+      <c r="C15" s="25" t="s">
+        <v>785</v>
+      </c>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26">
         <f>F15*D15</f>
-        <v>180000</v>
-      </c>
-      <c r="H15" s="17" t="s">
-        <v>771</v>
+        <v>0</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>776</v>
       </c>
       <c r="J15" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Serviço Prévio",Tabela2[Preço Total])</f>
@@ -12883,17 +12847,23 @@
       <c r="B16" s="27">
         <v>13</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>774</v>
-      </c>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H16" s="17" t="s">
+      <c r="C16" s="28" t="s">
+        <v>802</v>
+      </c>
+      <c r="D16" s="29">
+        <v>4</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>760</v>
+      </c>
+      <c r="F16" s="30">
+        <v>1500</v>
+      </c>
+      <c r="G16" s="30">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>6000</v>
+      </c>
+      <c r="H16" s="29" t="s">
         <v>771</v>
       </c>
     </row>
@@ -12902,14 +12872,20 @@
         <v>14</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>775</v>
-      </c>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="20"/>
+        <v>800</v>
+      </c>
+      <c r="D17" s="17">
+        <v>1</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="F17" s="20">
+        <v>4500</v>
+      </c>
       <c r="G17" s="20">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>F17*D17</f>
+        <v>4500</v>
       </c>
       <c r="H17" s="17" t="s">
         <v>771</v>
@@ -12919,156 +12895,150 @@
       <c r="B18" s="27">
         <v>15</v>
       </c>
-      <c r="C18" s="21" t="s">
-        <v>805</v>
-      </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19">
-        <f t="shared" ref="G18:G28" si="1">F18*D18</f>
+      <c r="C18" s="18" t="s">
+        <v>769</v>
+      </c>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20">
+        <f>F18*D18</f>
         <v>0</v>
       </c>
-      <c r="H18" s="22" t="s">
-        <v>776</v>
+      <c r="H18" s="17" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="27">
         <v>16</v>
       </c>
-      <c r="C19" s="31" t="s">
-        <v>806</v>
-      </c>
-      <c r="D19" s="27">
-        <v>252</v>
-      </c>
-      <c r="E19" s="27" t="s">
-        <v>761</v>
-      </c>
-      <c r="F19" s="36">
-        <v>269.5</v>
-      </c>
-      <c r="G19" s="36">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>67914</v>
-      </c>
-      <c r="H19" s="27" t="s">
-        <v>804</v>
+      <c r="C19" s="18" t="s">
+        <v>770</v>
+      </c>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20">
+        <f>F19*D19</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="17" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="27">
         <v>17</v>
       </c>
-      <c r="C20" s="31" t="s">
-        <v>806</v>
-      </c>
-      <c r="D20" s="27">
-        <v>84</v>
-      </c>
-      <c r="E20" s="27" t="s">
-        <v>761</v>
-      </c>
-      <c r="F20" s="36">
-        <v>115.5</v>
-      </c>
-      <c r="G20" s="36">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>9702</v>
-      </c>
-      <c r="H20" s="27" t="s">
-        <v>804</v>
+      <c r="C20" s="18" t="s">
+        <v>846</v>
+      </c>
+      <c r="D20" s="17">
+        <v>1</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="F20" s="20">
+        <v>51500</v>
+      </c>
+      <c r="G20" s="20">
+        <f>F20*D20</f>
+        <v>51500</v>
+      </c>
+      <c r="H20" s="17" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="27">
         <v>18</v>
       </c>
-      <c r="C21" s="31" t="s">
-        <v>807</v>
-      </c>
-      <c r="D21" s="27">
-        <v>42</v>
-      </c>
-      <c r="E21" s="27" t="s">
-        <v>761</v>
-      </c>
-      <c r="F21" s="36">
-        <v>35</v>
-      </c>
-      <c r="G21" s="36">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>1470</v>
-      </c>
-      <c r="H21" s="27" t="s">
-        <v>804</v>
+      <c r="C21" s="18" t="s">
+        <v>839</v>
+      </c>
+      <c r="D21" s="17">
+        <v>1</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="F21" s="20">
+        <v>180000</v>
+      </c>
+      <c r="G21" s="20">
+        <f>F21*D21</f>
+        <v>180000</v>
+      </c>
+      <c r="H21" s="17" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" s="27">
         <v>19</v>
       </c>
-      <c r="C22" s="31" t="s">
-        <v>808</v>
-      </c>
-      <c r="D22" s="27">
-        <v>4200</v>
-      </c>
-      <c r="E22" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="F22" s="36">
-        <v>0.5</v>
-      </c>
-      <c r="G22" s="36">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>2100</v>
-      </c>
-      <c r="H22" s="27" t="s">
-        <v>804</v>
+      <c r="C22" s="18" t="s">
+        <v>847</v>
+      </c>
+      <c r="D22" s="23">
+        <v>46.8</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>759</v>
+      </c>
+      <c r="F22" s="20">
+        <v>670</v>
+      </c>
+      <c r="G22" s="20">
+        <f>F22*D22</f>
+        <v>31355.999999999996</v>
+      </c>
+      <c r="H22" s="17" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" s="27">
         <v>20</v>
       </c>
-      <c r="C23" s="31" t="s">
-        <v>809</v>
-      </c>
-      <c r="D23" s="27">
-        <v>3100</v>
-      </c>
-      <c r="E23" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="F23" s="36">
-        <v>0.5</v>
-      </c>
-      <c r="G23" s="36">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>1550</v>
-      </c>
-      <c r="H23" s="27" t="s">
-        <v>804</v>
+      <c r="C23" s="18" t="s">
+        <v>848</v>
+      </c>
+      <c r="D23" s="23">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>759</v>
+      </c>
+      <c r="F23" s="20">
+        <v>670</v>
+      </c>
+      <c r="G23" s="20">
+        <f>F23*D23</f>
+        <v>24924.000000000004</v>
+      </c>
+      <c r="H23" s="17" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="27">
         <v>21</v>
       </c>
-      <c r="C24" s="21" t="s">
-        <v>803</v>
-      </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19">
-        <f t="shared" si="1"/>
+      <c r="C24" s="18" t="s">
+        <v>775</v>
+      </c>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20">
+        <f>F24*D24</f>
         <v>0</v>
       </c>
-      <c r="H24" s="22" t="s">
-        <v>776</v>
+      <c r="H24" s="17" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
@@ -13076,62 +13046,53 @@
         <v>22</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
       <c r="F25" s="19"/>
       <c r="G25" s="19">
-        <f t="shared" si="1"/>
+        <f>F25*D25</f>
         <v>0</v>
       </c>
       <c r="H25" s="22" t="s">
-        <v>786</v>
-      </c>
-      <c r="I25" s="14" t="s">
-        <v>793</v>
+        <v>771</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="27">
         <v>23</v>
       </c>
-      <c r="C26" s="21" t="s">
-        <v>796</v>
-      </c>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19">
-        <f t="shared" si="1"/>
+      <c r="C26" s="25" t="s">
+        <v>789</v>
+      </c>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="26">
+        <f>F26*D26</f>
         <v>0</v>
       </c>
-      <c r="H26" s="22" t="s">
-        <v>419</v>
+      <c r="H26" s="24" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" s="27">
         <v>24</v>
       </c>
-      <c r="C27" s="31" t="s">
-        <v>788</v>
-      </c>
-      <c r="D27" s="27">
-        <v>1</v>
-      </c>
-      <c r="E27" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="F27" s="36">
-        <v>157963.5</v>
-      </c>
-      <c r="G27" s="36">
-        <f t="shared" si="1"/>
-        <v>157963.5</v>
-      </c>
-      <c r="H27" s="27" t="s">
-        <v>787</v>
+      <c r="C27" s="25" t="s">
+        <v>790</v>
+      </c>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26">
+        <f>F27*D27</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="24" t="s">
+        <v>576</v>
       </c>
       <c r="I27" s="14" t="s">
         <v>793</v>
@@ -13141,170 +13102,209 @@
       <c r="B28" s="27">
         <v>25</v>
       </c>
-      <c r="C28" s="21" t="s">
-        <v>779</v>
-      </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19">
-        <f t="shared" si="1"/>
+      <c r="C28" s="25" t="s">
+        <v>791</v>
+      </c>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26">
+        <f>F28*D28</f>
         <v>0</v>
       </c>
-      <c r="H28" s="22" t="s">
-        <v>771</v>
+      <c r="H28" s="24" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" s="27">
         <v>26</v>
       </c>
-      <c r="C29" s="21" t="s">
-        <v>780</v>
-      </c>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19">
-        <f t="shared" ref="G29:G40" si="2">F29*D29</f>
+      <c r="C29" s="25" t="s">
+        <v>792</v>
+      </c>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26">
+        <f>F29*D29</f>
         <v>0</v>
       </c>
-      <c r="H29" s="22" t="s">
-        <v>449</v>
+      <c r="H29" s="24" t="s">
+        <v>576</v>
+      </c>
+      <c r="I29" s="14" t="s">
+        <v>793</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" s="27">
         <v>27</v>
       </c>
-      <c r="C30" s="21" t="s">
-        <v>781</v>
-      </c>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H30" s="22" t="s">
-        <v>449</v>
+      <c r="C30" s="31" t="s">
+        <v>757</v>
+      </c>
+      <c r="D30" s="27">
+        <f>(2000*1.05)*0.15</f>
+        <v>315</v>
+      </c>
+      <c r="E30" s="27" t="s">
+        <v>759</v>
+      </c>
+      <c r="F30" s="32">
+        <v>670</v>
+      </c>
+      <c r="G30" s="32">
+        <f>F30*D30</f>
+        <v>211050</v>
+      </c>
+      <c r="H30" s="27" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" s="27">
         <v>28</v>
       </c>
-      <c r="C31" s="25" t="s">
-        <v>782</v>
-      </c>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H31" s="24" t="s">
-        <v>776</v>
+      <c r="C31" s="31" t="s">
+        <v>777</v>
+      </c>
+      <c r="D31" s="33">
+        <f>2000/13*2</f>
+        <v>307.69230769230768</v>
+      </c>
+      <c r="E31" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="F31" s="32">
+        <v>220.5</v>
+      </c>
+      <c r="G31" s="32">
+        <f>F31*D31</f>
+        <v>67846.153846153844</v>
+      </c>
+      <c r="H31" s="27" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="27">
         <v>29</v>
       </c>
-      <c r="C32" s="25" t="s">
-        <v>783</v>
-      </c>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H32" s="24" t="s">
-        <v>776</v>
+      <c r="C32" s="31" t="s">
+        <v>758</v>
+      </c>
+      <c r="D32" s="27">
+        <v>167</v>
+      </c>
+      <c r="E32" s="27" t="s">
+        <v>820</v>
+      </c>
+      <c r="F32" s="32">
+        <v>56.2</v>
+      </c>
+      <c r="G32" s="32">
+        <f>F32*D32</f>
+        <v>9385.4</v>
+      </c>
+      <c r="H32" s="27" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="27">
         <v>30</v>
       </c>
-      <c r="C33" s="25" t="s">
-        <v>784</v>
-      </c>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H33" s="24" t="s">
-        <v>776</v>
+      <c r="C33" s="31" t="s">
+        <v>762</v>
+      </c>
+      <c r="D33" s="27">
+        <v>1000</v>
+      </c>
+      <c r="E33" s="27" t="s">
+        <v>763</v>
+      </c>
+      <c r="F33" s="32">
+        <v>7.3</v>
+      </c>
+      <c r="G33" s="32">
+        <f>F33*D33</f>
+        <v>7300</v>
+      </c>
+      <c r="H33" s="27" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="27">
         <v>31</v>
       </c>
-      <c r="C34" s="25" t="s">
-        <v>785</v>
-      </c>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H34" s="24" t="s">
-        <v>776</v>
+      <c r="C34" s="31" t="s">
+        <v>810</v>
+      </c>
+      <c r="D34" s="27">
+        <v>315</v>
+      </c>
+      <c r="E34" s="27" t="s">
+        <v>759</v>
+      </c>
+      <c r="F34" s="32">
+        <v>50</v>
+      </c>
+      <c r="G34" s="32">
+        <f>F34*D34</f>
+        <v>15750</v>
+      </c>
+      <c r="H34" s="27" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="27">
         <v>32</v>
       </c>
-      <c r="C35" s="25" t="s">
-        <v>794</v>
-      </c>
-      <c r="D35" s="24">
-        <v>10</v>
-      </c>
-      <c r="E35" s="24" t="s">
+      <c r="C35" s="31" t="s">
+        <v>768</v>
+      </c>
+      <c r="D35" s="27">
+        <v>1</v>
+      </c>
+      <c r="E35" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H35" s="24" t="s">
-        <v>643</v>
+      <c r="F35" s="32">
+        <v>49800</v>
+      </c>
+      <c r="G35" s="32">
+        <f>F35*D35</f>
+        <v>49800</v>
+      </c>
+      <c r="H35" s="27" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="27">
         <v>33</v>
       </c>
-      <c r="C36" s="25" t="s">
-        <v>795</v>
-      </c>
-      <c r="D36" s="24">
-        <v>500</v>
-      </c>
-      <c r="E36" s="24" t="s">
-        <v>761</v>
-      </c>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H36" s="24" t="s">
-        <v>643</v>
+      <c r="C36" s="31" t="s">
+        <v>773</v>
+      </c>
+      <c r="D36" s="27">
+        <v>1</v>
+      </c>
+      <c r="E36" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="F36" s="32">
+        <v>1267174</v>
+      </c>
+      <c r="G36" s="32">
+        <f>F36*D36</f>
+        <v>1267174</v>
+      </c>
+      <c r="H36" s="27" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
@@ -13312,17 +13312,21 @@
         <v>34</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>789</v>
-      </c>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
+        <v>812</v>
+      </c>
+      <c r="D37" s="24">
+        <v>1</v>
+      </c>
+      <c r="E37" s="24" t="s">
+        <v>760</v>
+      </c>
       <c r="F37" s="26"/>
       <c r="G37" s="26">
-        <f t="shared" si="2"/>
+        <f>F37*D37</f>
         <v>0</v>
       </c>
       <c r="H37" s="24" t="s">
-        <v>576</v>
+        <v>813</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
@@ -13330,137 +13334,207 @@
         <v>35</v>
       </c>
       <c r="C38" s="25" t="s">
-        <v>790</v>
-      </c>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
+        <v>825</v>
+      </c>
+      <c r="D38" s="24">
+        <v>1</v>
+      </c>
+      <c r="E38" s="24" t="s">
+        <v>760</v>
+      </c>
       <c r="F38" s="26"/>
       <c r="G38" s="26">
-        <f t="shared" si="2"/>
+        <f>F38*D38</f>
         <v>0</v>
       </c>
       <c r="H38" s="24" t="s">
-        <v>576</v>
+        <v>813</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="27">
         <v>36</v>
       </c>
-      <c r="C39" s="25" t="s">
-        <v>791</v>
-      </c>
-      <c r="D39" s="24"/>
-      <c r="E39" s="24"/>
-      <c r="F39" s="26"/>
-      <c r="G39" s="26">
-        <f t="shared" si="2"/>
+      <c r="C39" s="21" t="s">
+        <v>796</v>
+      </c>
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="19">
+        <f>F39*D39</f>
         <v>0</v>
       </c>
-      <c r="H39" s="24" t="s">
-        <v>576</v>
+      <c r="H39" s="22" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" s="27">
         <v>37</v>
       </c>
-      <c r="C40" s="25" t="s">
-        <v>792</v>
-      </c>
-      <c r="D40" s="24"/>
-      <c r="E40" s="24"/>
-      <c r="F40" s="26"/>
-      <c r="G40" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H40" s="24" t="s">
-        <v>576</v>
+      <c r="C40" s="31" t="s">
+        <v>806</v>
+      </c>
+      <c r="D40" s="27">
+        <v>252</v>
+      </c>
+      <c r="E40" s="27" t="s">
+        <v>761</v>
+      </c>
+      <c r="F40" s="36">
+        <v>269.5</v>
+      </c>
+      <c r="G40" s="36">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>67914</v>
+      </c>
+      <c r="H40" s="27" t="s">
+        <v>804</v>
       </c>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" s="27">
         <v>38</v>
       </c>
-      <c r="C41" s="25" t="s">
-        <v>798</v>
-      </c>
-      <c r="D41" s="24"/>
-      <c r="E41" s="24"/>
-      <c r="F41" s="26"/>
-      <c r="G41" s="26">
-        <f>F41*D41</f>
-        <v>0</v>
-      </c>
-      <c r="H41" s="24" t="s">
-        <v>801</v>
+      <c r="C41" s="31" t="s">
+        <v>806</v>
+      </c>
+      <c r="D41" s="27">
+        <v>84</v>
+      </c>
+      <c r="E41" s="27" t="s">
+        <v>761</v>
+      </c>
+      <c r="F41" s="36">
+        <v>115.5</v>
+      </c>
+      <c r="G41" s="36">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>9702</v>
+      </c>
+      <c r="H41" s="27" t="s">
+        <v>804</v>
       </c>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" s="27">
         <v>39</v>
       </c>
-      <c r="C42" s="25" t="s">
-        <v>812</v>
-      </c>
-      <c r="D42" s="24">
-        <v>1</v>
-      </c>
-      <c r="E42" s="24" t="s">
+      <c r="C42" s="31" t="s">
+        <v>807</v>
+      </c>
+      <c r="D42" s="27">
+        <v>42</v>
+      </c>
+      <c r="E42" s="27" t="s">
+        <v>761</v>
+      </c>
+      <c r="F42" s="36">
+        <v>35</v>
+      </c>
+      <c r="G42" s="36">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>1470</v>
+      </c>
+      <c r="H42" s="27" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B43" s="27">
+        <v>40</v>
+      </c>
+      <c r="C43" s="31" t="s">
+        <v>808</v>
+      </c>
+      <c r="D43" s="27">
+        <v>4200</v>
+      </c>
+      <c r="E43" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F42" s="26"/>
-      <c r="G42" s="26">
-        <f>F42*D42</f>
-        <v>0</v>
-      </c>
-      <c r="H42" s="24" t="s">
-        <v>813</v>
-      </c>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B43" s="24"/>
-      <c r="C43" s="25" t="s">
-        <v>825</v>
-      </c>
-      <c r="D43" s="24">
-        <v>1</v>
-      </c>
-      <c r="E43" s="24" t="s">
+      <c r="F43" s="36">
+        <v>0.5</v>
+      </c>
+      <c r="G43" s="36">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>2100</v>
+      </c>
+      <c r="H43" s="27" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B44" s="27">
+        <v>41</v>
+      </c>
+      <c r="C44" s="31" t="s">
+        <v>809</v>
+      </c>
+      <c r="D44" s="27">
+        <v>3100</v>
+      </c>
+      <c r="E44" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F43" s="26"/>
-      <c r="G43" s="26">
-        <f>F43*D43</f>
-        <v>0</v>
-      </c>
-      <c r="H43" s="24" t="s">
-        <v>813</v>
-      </c>
-    </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B44" s="24"/>
-      <c r="C44" s="25"/>
-      <c r="D44" s="24"/>
-      <c r="E44" s="24"/>
-      <c r="F44" s="26"/>
-      <c r="G44" s="26"/>
-      <c r="H44" s="24"/>
+      <c r="F44" s="36">
+        <v>0.5</v>
+      </c>
+      <c r="G44" s="36">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>1550</v>
+      </c>
+      <c r="H44" s="27" t="s">
+        <v>804</v>
+      </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B45" s="24"/>
-      <c r="C45" s="25"/>
-      <c r="D45" s="24"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="24"/>
+      <c r="B45" s="27">
+        <v>42</v>
+      </c>
+      <c r="C45" s="31" t="s">
+        <v>788</v>
+      </c>
+      <c r="D45" s="27">
+        <v>1</v>
+      </c>
+      <c r="E45" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="F45" s="36">
+        <v>157963.5</v>
+      </c>
+      <c r="G45" s="36">
+        <f>F45*D45</f>
+        <v>157963.5</v>
+      </c>
+      <c r="H45" s="27" t="s">
+        <v>787</v>
+      </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="G46" s="16">
+      <c r="B46" s="24"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="24"/>
+      <c r="E46" s="24"/>
+      <c r="F46" s="26"/>
+      <c r="G46" s="26"/>
+      <c r="H46" s="24"/>
+    </row>
+    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B47" s="24"/>
+      <c r="C47" s="25"/>
+      <c r="D47" s="24"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="26"/>
+      <c r="G47" s="26"/>
+      <c r="H47" s="24"/>
+    </row>
+    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G48" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>2055005.0538461539</v>
+        <v>2167285.0538461539</v>
       </c>
     </row>
   </sheetData>
@@ -13546,7 +13620,7 @@
       <c r="F4" s="24"/>
       <c r="G4" s="26"/>
       <c r="H4" s="26">
-        <f>G4*E4</f>
+        <f t="shared" ref="H4:H48" si="0">G4*E4</f>
         <v>0</v>
       </c>
       <c r="I4" s="24" t="s">
@@ -13579,7 +13653,7 @@
       <c r="F5" s="22"/>
       <c r="G5" s="19"/>
       <c r="H5" s="19">
-        <f>G5*E5</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I5" s="22" t="s">
@@ -13593,7 +13667,7 @@
         <v>968004</v>
       </c>
       <c r="P5" s="44">
-        <f t="shared" ref="P5:P17" si="0">O5/$O$21</f>
+        <f t="shared" ref="P5:P17" si="1">O5/$O$21</f>
         <v>0.33062288469044115</v>
       </c>
       <c r="Q5" s="46">
@@ -13618,7 +13692,7 @@
       <c r="F6" s="22"/>
       <c r="G6" s="19"/>
       <c r="H6" s="19">
-        <f>G6*E6</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I6" s="22" t="s">
@@ -13632,7 +13706,7 @@
         <v>791792.51</v>
       </c>
       <c r="P6" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.27043764667551473</v>
       </c>
       <c r="Q6" s="46">
@@ -13657,7 +13731,7 @@
       <c r="F7" s="22"/>
       <c r="G7" s="19"/>
       <c r="H7" s="19">
-        <f>G7*E7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I7" s="22" t="s">
@@ -13671,7 +13745,7 @@
         <v>645545.6</v>
       </c>
       <c r="P7" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.22048684558247864</v>
       </c>
     </row>
@@ -13693,7 +13767,7 @@
       </c>
       <c r="G8" s="26"/>
       <c r="H8" s="26">
-        <f>G8*E8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I8" s="24" t="s">
@@ -13710,7 +13784,7 @@
         <v>358477</v>
       </c>
       <c r="P8" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.12243823355603414</v>
       </c>
     </row>
@@ -13732,7 +13806,7 @@
       </c>
       <c r="G9" s="26"/>
       <c r="H9" s="26">
-        <f>G9*E9</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I9" s="24" t="s">
@@ -13749,7 +13823,7 @@
         <v>164000</v>
       </c>
       <c r="P9" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5.6014389495531371E-2</v>
       </c>
     </row>
@@ -13767,7 +13841,7 @@
       <c r="F10" s="24"/>
       <c r="G10" s="26"/>
       <c r="H10" s="26">
-        <f>G10*E10</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I10" s="24" t="s">
@@ -13781,7 +13855,7 @@
         <v>0</v>
       </c>
       <c r="P10" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13803,7 +13877,7 @@
       </c>
       <c r="G11" s="19"/>
       <c r="H11" s="19">
-        <f>G11*E11</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I11" s="22" t="s">
@@ -13817,7 +13891,7 @@
         <v>0</v>
       </c>
       <c r="P11" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13839,7 +13913,7 @@
       </c>
       <c r="G12" s="19"/>
       <c r="H12" s="19">
-        <f>G12*E12</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I12" s="22" t="s">
@@ -13853,7 +13927,7 @@
         <v>0</v>
       </c>
       <c r="P12" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13875,7 +13949,7 @@
       </c>
       <c r="G13" s="19"/>
       <c r="H13" s="19">
-        <f>G13*E13</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I13" s="22" t="s">
@@ -13904,7 +13978,7 @@
       </c>
       <c r="G14" s="19"/>
       <c r="H14" s="19">
-        <f>G14*E14</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I14" s="22" t="s">
@@ -13918,7 +13992,7 @@
         <v>0</v>
       </c>
       <c r="P14" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13941,7 +14015,7 @@
       </c>
       <c r="G15" s="19"/>
       <c r="H15" s="19">
-        <f>G15*E15</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I15" s="22" t="s">
@@ -13955,7 +14029,7 @@
         <v>0</v>
       </c>
       <c r="P15" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13975,7 +14049,7 @@
       </c>
       <c r="G16" s="26"/>
       <c r="H16" s="26">
-        <f>G16*E16</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I16" s="24" t="s">
@@ -13989,7 +14063,7 @@
         <v>0</v>
       </c>
       <c r="P16" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -14007,7 +14081,7 @@
       <c r="F17" s="24"/>
       <c r="G17" s="26"/>
       <c r="H17" s="26">
-        <f>G17*E17</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I17" s="24" t="s">
@@ -14021,7 +14095,7 @@
         <v>0</v>
       </c>
       <c r="P17" s="44">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -14039,7 +14113,7 @@
       <c r="F18" s="24"/>
       <c r="G18" s="26"/>
       <c r="H18" s="26">
-        <f>G18*E18</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I18" s="24" t="s">
@@ -14065,7 +14139,7 @@
       <c r="F19" s="24"/>
       <c r="G19" s="26"/>
       <c r="H19" s="26">
-        <f>G19*E19</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I19" s="24" t="s">
@@ -14089,7 +14163,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="20"/>
       <c r="H20" s="20">
-        <f>G20*E20</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I20" s="17" t="s">
@@ -14110,7 +14184,7 @@
       <c r="F21" s="17"/>
       <c r="G21" s="20"/>
       <c r="H21" s="20">
-        <f>G21*E21</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I21" s="17" t="s">
@@ -14138,7 +14212,7 @@
       <c r="F22" s="17"/>
       <c r="G22" s="20"/>
       <c r="H22" s="20">
-        <f>G22*E22</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I22" s="17" t="s">
@@ -14167,7 +14241,7 @@
         <v>164000</v>
       </c>
       <c r="H23" s="20">
-        <f>G23*E23</f>
+        <f t="shared" si="0"/>
         <v>164000</v>
       </c>
       <c r="I23" s="17" t="s">
@@ -14188,7 +14262,7 @@
       <c r="F24" s="17"/>
       <c r="G24" s="20"/>
       <c r="H24" s="20">
-        <f>G24*E24</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I24" s="17" t="s">
@@ -14209,7 +14283,7 @@
       <c r="F25" s="17"/>
       <c r="G25" s="20"/>
       <c r="H25" s="20">
-        <f>G25*E25</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I25" s="17" t="s">
@@ -14230,7 +14304,7 @@
       <c r="F26" s="22"/>
       <c r="G26" s="19"/>
       <c r="H26" s="19">
-        <f>G26*E26</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I26" s="22" t="s">
@@ -14251,7 +14325,7 @@
       <c r="F27" s="24"/>
       <c r="G27" s="26"/>
       <c r="H27" s="26">
-        <f>G27*E27</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I27" s="24" t="s">
@@ -14272,7 +14346,7 @@
       <c r="F28" s="24"/>
       <c r="G28" s="26"/>
       <c r="H28" s="26">
-        <f>G28*E28</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I28" s="24" t="s">
@@ -14293,7 +14367,7 @@
       <c r="F29" s="24"/>
       <c r="G29" s="26"/>
       <c r="H29" s="26">
-        <f>G29*E29</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I29" s="24" t="s">
@@ -14314,7 +14388,7 @@
       <c r="F30" s="24"/>
       <c r="G30" s="26"/>
       <c r="H30" s="26">
-        <f>G30*E30</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I30" s="24" t="s">
@@ -14342,7 +14416,7 @@
         <v>670</v>
       </c>
       <c r="H31" s="20">
-        <f>G31*E31</f>
+        <f t="shared" si="0"/>
         <v>226878.75</v>
       </c>
       <c r="I31" s="17" t="s">
@@ -14370,7 +14444,7 @@
         <v>220.5</v>
       </c>
       <c r="H32" s="20">
-        <f>G32*E32</f>
+        <f t="shared" si="0"/>
         <v>72934.61538461539</v>
       </c>
       <c r="I32" s="17" t="s">
@@ -14398,7 +14472,7 @@
         <v>56.2</v>
       </c>
       <c r="H33" s="20">
-        <f>G33*E33</f>
+        <f t="shared" si="0"/>
         <v>9835</v>
       </c>
       <c r="I33" s="17" t="s">
@@ -14425,7 +14499,7 @@
         <v>7.3</v>
       </c>
       <c r="H34" s="20">
-        <f>G34*E34</f>
+        <f t="shared" si="0"/>
         <v>7300</v>
       </c>
       <c r="I34" s="17" t="s">
@@ -14453,7 +14527,7 @@
         <v>50</v>
       </c>
       <c r="H35" s="20">
-        <f>G35*E35</f>
+        <f t="shared" si="0"/>
         <v>16931.25</v>
       </c>
       <c r="I35" s="17" t="s">
@@ -14480,7 +14554,7 @@
         <v>49800</v>
       </c>
       <c r="H36" s="20">
-        <f>G36*E36</f>
+        <f t="shared" si="0"/>
         <v>49800</v>
       </c>
       <c r="I36" s="17" t="s">
@@ -14505,7 +14579,7 @@
       </c>
       <c r="G37" s="26"/>
       <c r="H37" s="26">
-        <f>G37*E37</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I37" s="24" t="s">
@@ -14533,7 +14607,7 @@
         <v>670</v>
       </c>
       <c r="H38" s="26">
-        <f>G38*E38</f>
+        <f t="shared" si="0"/>
         <v>188256.59999999998</v>
       </c>
       <c r="I38" s="24" t="s">
@@ -14561,7 +14635,7 @@
         <v>220.5</v>
       </c>
       <c r="H39" s="26">
-        <f>G39*E39</f>
+        <f t="shared" si="0"/>
         <v>30259.384615384613</v>
       </c>
       <c r="I39" s="24" t="s">
@@ -14588,7 +14662,7 @@
         <v>43350</v>
       </c>
       <c r="H40" s="26">
-        <f>G40*E40</f>
+        <f t="shared" si="0"/>
         <v>43350</v>
       </c>
       <c r="I40" s="24" t="s">
@@ -14615,7 +14689,7 @@
         <v>968004</v>
       </c>
       <c r="H41" s="20">
-        <f>G41*E41</f>
+        <f t="shared" si="0"/>
         <v>968004</v>
       </c>
       <c r="I41" s="17" t="s">
@@ -14636,7 +14710,7 @@
       <c r="F42" s="22"/>
       <c r="G42" s="19"/>
       <c r="H42" s="19">
-        <f>G42*E42</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I42" s="17" t="s">
@@ -14663,7 +14737,7 @@
         <v>46600</v>
       </c>
       <c r="H43" s="26">
-        <f>G43*E43</f>
+        <f t="shared" si="0"/>
         <v>46600</v>
       </c>
       <c r="I43" s="24" t="s">
@@ -14690,7 +14764,7 @@
         <v>8100</v>
       </c>
       <c r="H44" s="26">
-        <f>G44*E44</f>
+        <f t="shared" si="0"/>
         <v>8100</v>
       </c>
       <c r="I44" s="24" t="s">
@@ -14717,7 +14791,7 @@
         <v>5000</v>
       </c>
       <c r="H45" s="26">
-        <f>G45*E45</f>
+        <f t="shared" si="0"/>
         <v>5000</v>
       </c>
       <c r="I45" s="24" t="s">
@@ -14744,7 +14818,7 @@
         <v>298777</v>
       </c>
       <c r="H46" s="26">
-        <f>G46*E46</f>
+        <f t="shared" si="0"/>
         <v>298777</v>
       </c>
       <c r="I46" s="24" t="s">
@@ -14765,7 +14839,7 @@
       <c r="F47" s="22"/>
       <c r="G47" s="19"/>
       <c r="H47" s="19">
-        <f>G47*E47</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I47" s="22" t="s">
@@ -14792,7 +14866,7 @@
         <v>791792.51</v>
       </c>
       <c r="H48" s="19">
-        <f>G48*E48</f>
+        <f t="shared" si="0"/>
         <v>791792.51</v>
       </c>
       <c r="I48" s="22" t="s">

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 08:48
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2109" uniqueCount="848">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="850">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2569,6 +2569,12 @@
   </si>
   <si>
     <t>Concreto FCK 30 Brita 0 Slump 10±2 cálices e blocos</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>Valor Estimado - Será fechado somente após detalhamento do projeto</t>
   </si>
 </sst>
 </file>
@@ -2834,6 +2840,116 @@
         <name val="Calibri"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
       <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2937,116 +3053,6 @@
         <scheme val="none"/>
       </font>
     </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3061,43 +3067,43 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H45" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:H45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H44" totalsRowShown="0" dataDxfId="7">
+  <autoFilter ref="B3:H44"/>
   <sortState ref="B4:H43">
     <sortCondition ref="H3:H43"/>
   </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" name="Item" dataDxfId="15" dataCellStyle="Normal"/>
-    <tableColumn id="2" name="Descrição" dataDxfId="14" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="13" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="12" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="11" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="10" dataCellStyle="Moeda">
+    <tableColumn id="1" name="Item" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="2" name="Descrição" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="2" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="1" dataCellStyle="Moeda">
       <calculatedColumnFormula>F4*D4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="9" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="0" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I48" totalsRowShown="0" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I48" totalsRowShown="0" dataDxfId="16">
   <autoFilter ref="B3:I48"/>
   <sortState ref="B4:I48">
     <sortCondition ref="I3:I48"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" name="Item" dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="8" name="Local" dataDxfId="6"/>
-    <tableColumn id="2" name="Descrição" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="2" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="1" dataCellStyle="Moeda">
+    <tableColumn id="1" name="Item" dataDxfId="15" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Local" dataDxfId="14"/>
+    <tableColumn id="2" name="Descrição" dataDxfId="13" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="12" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="11" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="10" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="9" dataCellStyle="Moeda">
       <calculatedColumnFormula>G4*E4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="0" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="8" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12528,7 +12534,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:J48"/>
+  <dimension ref="B3:J47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -12538,7 +12544,7 @@
     <col min="6" max="6" width="15.85546875" style="15" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" style="15" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="27.42578125" style="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.85546875" style="14" customWidth="1"/>
+    <col min="9" max="9" width="64.7109375" style="14" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -12864,7 +12870,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="27">
         <v>14</v>
       </c>
@@ -12888,15 +12894,19 @@
         <v>771</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="27">
         <v>15</v>
       </c>
       <c r="C18" s="18" t="s">
         <v>769</v>
       </c>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
+      <c r="D18" s="17">
+        <v>2100</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>848</v>
+      </c>
       <c r="F18" s="20"/>
       <c r="G18" s="20">
         <f>F18*D18</f>
@@ -12905,16 +12915,23 @@
       <c r="H18" s="17" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I18" s="14" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="27">
         <v>16</v>
       </c>
       <c r="C19" s="18" t="s">
         <v>770</v>
       </c>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
+      <c r="D19" s="17">
+        <v>2300</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>848</v>
+      </c>
       <c r="F19" s="20"/>
       <c r="G19" s="20">
         <f>F19*D19</f>
@@ -12923,8 +12940,11 @@
       <c r="H19" s="17" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I19" s="14" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="27">
         <v>17</v>
       </c>
@@ -12948,7 +12968,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="27">
         <v>18</v>
       </c>
@@ -12972,7 +12992,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" s="27">
         <v>19</v>
       </c>
@@ -12996,7 +13016,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" s="27">
         <v>20</v>
       </c>
@@ -13020,48 +13040,48 @@
         <v>771</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="27">
-        <v>21</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>775</v>
-      </c>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="20">
+        <v>22</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>779</v>
+      </c>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19">
         <f>F24*D24</f>
         <v>0</v>
       </c>
-      <c r="H24" s="17" t="s">
+      <c r="H24" s="22" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="27">
-        <v>22</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>779</v>
-      </c>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19">
+        <v>23</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>789</v>
+      </c>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="26">
         <f>F25*D25</f>
         <v>0</v>
       </c>
-      <c r="H25" s="22" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="H25" s="24" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="27">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C26" s="25" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="D26" s="24"/>
       <c r="E26" s="24"/>
@@ -13074,12 +13094,12 @@
         <v>576</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" s="27">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="24"/>
@@ -13092,12 +13112,12 @@
         <v>576</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" s="27">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C28" s="25" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="D28" s="24"/>
       <c r="E28" s="24"/>
@@ -13110,93 +13130,99 @@
         <v>576</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" s="27">
-        <v>26</v>
-      </c>
-      <c r="C29" s="25" t="s">
-        <v>792</v>
-      </c>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26">
-        <f>F29*D29</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="24" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B30" s="27">
         <v>27</v>
       </c>
-      <c r="C30" s="31" t="s">
+      <c r="C29" s="31" t="s">
         <v>757</v>
       </c>
-      <c r="D30" s="27">
+      <c r="D29" s="27">
         <f>(2000*1.05)*0.15</f>
         <v>315</v>
       </c>
+      <c r="E29" s="27" t="s">
+        <v>759</v>
+      </c>
+      <c r="F29" s="32">
+        <v>670</v>
+      </c>
+      <c r="G29" s="32">
+        <f>F29*D29</f>
+        <v>211050</v>
+      </c>
+      <c r="H29" s="27" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B30" s="27">
+        <v>28</v>
+      </c>
+      <c r="C30" s="31" t="s">
+        <v>777</v>
+      </c>
+      <c r="D30" s="33">
+        <f>2000/13*2</f>
+        <v>307.69230769230768</v>
+      </c>
       <c r="E30" s="27" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="F30" s="32">
-        <v>670</v>
+        <v>220.5</v>
       </c>
       <c r="G30" s="32">
         <f>F30*D30</f>
-        <v>211050</v>
+        <v>67846.153846153844</v>
       </c>
       <c r="H30" s="27" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" s="27">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>777</v>
-      </c>
-      <c r="D31" s="33">
-        <f>2000/13*2</f>
-        <v>307.69230769230768</v>
+        <v>758</v>
+      </c>
+      <c r="D31" s="27">
+        <v>167</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>760</v>
+        <v>819</v>
       </c>
       <c r="F31" s="32">
-        <v>220.5</v>
+        <v>56.2</v>
       </c>
       <c r="G31" s="32">
         <f>F31*D31</f>
-        <v>67846.153846153844</v>
+        <v>9385.4</v>
       </c>
       <c r="H31" s="27" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="27">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="D32" s="27">
-        <v>167</v>
+        <v>1000</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>819</v>
+        <v>763</v>
       </c>
       <c r="F32" s="32">
-        <v>56.2</v>
+        <v>7.3</v>
       </c>
       <c r="G32" s="32">
         <f>F32*D32</f>
-        <v>9385.4</v>
+        <v>7300</v>
       </c>
       <c r="H32" s="27" t="s">
         <v>635</v>
@@ -13204,23 +13230,23 @@
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="27">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>762</v>
+        <v>809</v>
       </c>
       <c r="D33" s="27">
-        <v>1000</v>
+        <v>315</v>
       </c>
       <c r="E33" s="27" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="F33" s="32">
-        <v>7.3</v>
+        <v>50</v>
       </c>
       <c r="G33" s="32">
         <f>F33*D33</f>
-        <v>7300</v>
+        <v>15750</v>
       </c>
       <c r="H33" s="27" t="s">
         <v>635</v>
@@ -13228,23 +13254,23 @@
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="27">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>809</v>
+        <v>768</v>
       </c>
       <c r="D34" s="27">
-        <v>315</v>
+        <v>1</v>
       </c>
       <c r="E34" s="27" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="F34" s="32">
-        <v>50</v>
+        <v>49800</v>
       </c>
       <c r="G34" s="32">
         <f>F34*D34</f>
-        <v>15750</v>
+        <v>49800</v>
       </c>
       <c r="H34" s="27" t="s">
         <v>635</v>
@@ -13252,10 +13278,10 @@
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="27">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C35" s="31" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="D35" s="27">
         <v>1</v>
@@ -13264,46 +13290,44 @@
         <v>760</v>
       </c>
       <c r="F35" s="32">
-        <v>49800</v>
+        <v>1267174</v>
       </c>
       <c r="G35" s="32">
         <f>F35*D35</f>
-        <v>49800</v>
+        <v>1267174</v>
       </c>
       <c r="H35" s="27" t="s">
-        <v>635</v>
+        <v>772</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="27">
-        <v>33</v>
-      </c>
-      <c r="C36" s="31" t="s">
-        <v>773</v>
-      </c>
-      <c r="D36" s="27">
-        <v>1</v>
-      </c>
-      <c r="E36" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="C36" s="25" t="s">
+        <v>811</v>
+      </c>
+      <c r="D36" s="24">
+        <v>1</v>
+      </c>
+      <c r="E36" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F36" s="32">
-        <v>1267174</v>
-      </c>
-      <c r="G36" s="32">
+      <c r="F36" s="26"/>
+      <c r="G36" s="26">
         <f>F36*D36</f>
-        <v>1267174</v>
-      </c>
-      <c r="H36" s="27" t="s">
-        <v>772</v>
+        <v>0</v>
+      </c>
+      <c r="H36" s="24" t="s">
+        <v>812</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" s="27">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>811</v>
+        <v>824</v>
       </c>
       <c r="D37" s="24">
         <v>1</v>
@@ -13322,63 +13346,65 @@
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" s="27">
-        <v>35</v>
-      </c>
-      <c r="C38" s="25" t="s">
-        <v>824</v>
-      </c>
-      <c r="D38" s="24">
-        <v>1</v>
-      </c>
-      <c r="E38" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="F38" s="26"/>
-      <c r="G38" s="26">
+        <v>36</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>795</v>
+      </c>
+      <c r="D38" s="22"/>
+      <c r="E38" s="22"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19">
         <f>F38*D38</f>
         <v>0</v>
       </c>
-      <c r="H38" s="24" t="s">
-        <v>812</v>
+      <c r="H38" s="22" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="27">
-        <v>36</v>
-      </c>
-      <c r="C39" s="21" t="s">
-        <v>795</v>
-      </c>
-      <c r="D39" s="22"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19">
-        <f>F39*D39</f>
-        <v>0</v>
-      </c>
-      <c r="H39" s="22" t="s">
-        <v>419</v>
+        <v>37</v>
+      </c>
+      <c r="C39" s="31" t="s">
+        <v>805</v>
+      </c>
+      <c r="D39" s="27">
+        <v>252</v>
+      </c>
+      <c r="E39" s="27" t="s">
+        <v>761</v>
+      </c>
+      <c r="F39" s="36">
+        <v>269.5</v>
+      </c>
+      <c r="G39" s="36">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>67914</v>
+      </c>
+      <c r="H39" s="27" t="s">
+        <v>803</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" s="27">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C40" s="31" t="s">
         <v>805</v>
       </c>
       <c r="D40" s="27">
-        <v>252</v>
+        <v>84</v>
       </c>
       <c r="E40" s="27" t="s">
         <v>761</v>
       </c>
       <c r="F40" s="36">
-        <v>269.5</v>
+        <v>115.5</v>
       </c>
       <c r="G40" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>67914</v>
+        <v>9702</v>
       </c>
       <c r="H40" s="27" t="s">
         <v>803</v>
@@ -13386,23 +13412,23 @@
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" s="27">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C41" s="31" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="D41" s="27">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="E41" s="27" t="s">
         <v>761</v>
       </c>
       <c r="F41" s="36">
-        <v>115.5</v>
+        <v>35</v>
       </c>
       <c r="G41" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>9702</v>
+        <v>1470</v>
       </c>
       <c r="H41" s="27" t="s">
         <v>803</v>
@@ -13410,23 +13436,23 @@
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" s="27">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C42" s="31" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="D42" s="27">
-        <v>42</v>
+        <v>4200</v>
       </c>
       <c r="E42" s="27" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="F42" s="36">
-        <v>35</v>
+        <v>0.5</v>
       </c>
       <c r="G42" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>1470</v>
+        <v>2100</v>
       </c>
       <c r="H42" s="27" t="s">
         <v>803</v>
@@ -13434,13 +13460,13 @@
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" s="27">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C43" s="31" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="D43" s="27">
-        <v>4200</v>
+        <v>3100</v>
       </c>
       <c r="E43" s="27" t="s">
         <v>760</v>
@@ -13450,7 +13476,7 @@
       </c>
       <c r="G43" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>2100</v>
+        <v>1550</v>
       </c>
       <c r="H43" s="27" t="s">
         <v>803</v>
@@ -13458,51 +13484,36 @@
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B44" s="27">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C44" s="31" t="s">
-        <v>808</v>
+        <v>788</v>
       </c>
       <c r="D44" s="27">
-        <v>3100</v>
+        <v>1</v>
       </c>
       <c r="E44" s="27" t="s">
         <v>760</v>
       </c>
       <c r="F44" s="36">
-        <v>0.5</v>
+        <v>157963.5</v>
       </c>
       <c r="G44" s="36">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>1550</v>
+        <f>F44*D44</f>
+        <v>157963.5</v>
       </c>
       <c r="H44" s="27" t="s">
-        <v>803</v>
+        <v>787</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B45" s="27">
-        <v>42</v>
-      </c>
-      <c r="C45" s="31" t="s">
-        <v>788</v>
-      </c>
-      <c r="D45" s="27">
-        <v>1</v>
-      </c>
-      <c r="E45" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="F45" s="36">
-        <v>157963.5</v>
-      </c>
-      <c r="G45" s="36">
-        <f>F45*D45</f>
-        <v>157963.5</v>
-      </c>
-      <c r="H45" s="27" t="s">
-        <v>787</v>
-      </c>
+      <c r="B45" s="24"/>
+      <c r="C45" s="25"/>
+      <c r="D45" s="24"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="26"/>
+      <c r="G45" s="26"/>
+      <c r="H45" s="24"/>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" s="24"/>
@@ -13514,16 +13525,7 @@
       <c r="H46" s="24"/>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B47" s="24"/>
-      <c r="C47" s="25"/>
-      <c r="D47" s="24"/>
-      <c r="E47" s="24"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="24"/>
-    </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="G48" s="16">
+      <c r="G47" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
         <v>2167285.0538461539</v>
       </c>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 08:57
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="850">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2113" uniqueCount="851">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2382,9 +2382,6 @@
     <t xml:space="preserve">Mão de obra para montagem e cobertura </t>
   </si>
   <si>
-    <t>Fechamento em Alvenaria</t>
-  </si>
-  <si>
     <t>AVCB</t>
   </si>
   <si>
@@ -2575,6 +2572,12 @@
   </si>
   <si>
     <t>Valor Estimado - Será fechado somente após detalhamento do projeto</t>
+  </si>
+  <si>
+    <t>Fechamento em Alvenaria - Mão de Obra</t>
+  </si>
+  <si>
+    <t>Telha Termoacústica para cobertura do telhado</t>
   </si>
 </sst>
 </file>
@@ -3067,8 +3070,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H44" totalsRowShown="0" dataDxfId="7">
-  <autoFilter ref="B3:H44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H45" totalsRowShown="0" dataDxfId="7">
+  <autoFilter ref="B3:H45"/>
   <sortState ref="B4:H43">
     <sortCondition ref="H3:H43"/>
   </sortState>
@@ -12534,7 +12537,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:J47"/>
+  <dimension ref="B3:J48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -12571,7 +12574,7 @@
         <v>767</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -12589,7 +12592,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="22" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="J4" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
@@ -12645,7 +12648,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="D7" s="24">
         <v>10</v>
@@ -12671,7 +12674,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="D8" s="24">
         <v>500</v>
@@ -12679,10 +12682,12 @@
       <c r="E8" s="24" t="s">
         <v>761</v>
       </c>
-      <c r="F8" s="26"/>
+      <c r="F8" s="26">
+        <v>2.35</v>
+      </c>
       <c r="G8" s="26">
         <f>F8*D8</f>
-        <v>0</v>
+        <v>1175</v>
       </c>
       <c r="H8" s="24" t="s">
         <v>643</v>
@@ -12697,7 +12702,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="D9" s="24"/>
       <c r="E9" s="24"/>
@@ -12707,7 +12712,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="24" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="J9" s="40">
         <f>SUMIF(Tabela2[Aplicação],"SPDA",Tabela2[Preço Total])</f>
@@ -12719,7 +12724,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="D10" s="22"/>
       <c r="E10" s="22"/>
@@ -12741,7 +12746,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="D11" s="22"/>
       <c r="E11" s="22"/>
@@ -12777,7 +12782,7 @@
       </c>
       <c r="J12" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Elétrica",Tabela2[Preço Total])</f>
-        <v>0</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
@@ -12829,7 +12834,7 @@
         <v>12</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>785</v>
+        <v>849</v>
       </c>
       <c r="D15" s="24"/>
       <c r="E15" s="24"/>
@@ -12847,90 +12852,82 @@
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="27">
+      <c r="B16" s="27"/>
+      <c r="C16" s="25" t="s">
+        <v>850</v>
+      </c>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26">
+        <f>F16*D16</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>802</v>
+      </c>
+      <c r="J16" s="40"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="27">
         <v>13</v>
       </c>
-      <c r="C16" s="28" t="s">
-        <v>801</v>
-      </c>
-      <c r="D16" s="29">
+      <c r="C17" s="28" t="s">
+        <v>800</v>
+      </c>
+      <c r="D17" s="29">
         <v>4</v>
       </c>
-      <c r="E16" s="29" t="s">
+      <c r="E17" s="29" t="s">
         <v>760</v>
       </c>
-      <c r="F16" s="30">
+      <c r="F17" s="30">
         <v>1500</v>
       </c>
-      <c r="G16" s="30">
+      <c r="G17" s="30">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>6000</v>
       </c>
-      <c r="H16" s="29" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="27">
-        <v>14</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>799</v>
-      </c>
-      <c r="D17" s="17">
-        <v>1</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="F17" s="20">
-        <v>4500</v>
-      </c>
-      <c r="G17" s="20">
-        <f>F17*D17</f>
-        <v>4500</v>
-      </c>
-      <c r="H17" s="17" t="s">
+      <c r="H17" s="29" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="27">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>769</v>
+        <v>798</v>
       </c>
       <c r="D18" s="17">
-        <v>2100</v>
+        <v>1</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>848</v>
-      </c>
-      <c r="F18" s="20"/>
+        <v>760</v>
+      </c>
+      <c r="F18" s="20">
+        <v>4500</v>
+      </c>
       <c r="G18" s="20">
         <f>F18*D18</f>
-        <v>0</v>
+        <v>4500</v>
       </c>
       <c r="H18" s="17" t="s">
         <v>771</v>
       </c>
-      <c r="I18" s="14" t="s">
-        <v>849</v>
-      </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="27">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="D19" s="17">
-        <v>2300</v>
+        <v>2100</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="F19" s="20"/>
       <c r="G19" s="20">
@@ -12941,39 +12938,40 @@
         <v>771</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="27">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>845</v>
+        <v>770</v>
       </c>
       <c r="D20" s="17">
-        <v>1</v>
+        <v>2300</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="F20" s="20">
-        <v>51500</v>
-      </c>
+        <v>847</v>
+      </c>
+      <c r="F20" s="20"/>
       <c r="G20" s="20">
         <f>F20*D20</f>
-        <v>51500</v>
+        <v>0</v>
       </c>
       <c r="H20" s="17" t="s">
         <v>771</v>
       </c>
+      <c r="I20" s="14" t="s">
+        <v>848</v>
+      </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="27">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>838</v>
+        <v>844</v>
       </c>
       <c r="D21" s="17">
         <v>1</v>
@@ -12982,11 +12980,11 @@
         <v>760</v>
       </c>
       <c r="F21" s="20">
-        <v>180000</v>
+        <v>51500</v>
       </c>
       <c r="G21" s="20">
         <f>F21*D21</f>
-        <v>180000</v>
+        <v>51500</v>
       </c>
       <c r="H21" s="17" t="s">
         <v>771</v>
@@ -12994,23 +12992,23 @@
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" s="27">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>846</v>
-      </c>
-      <c r="D22" s="23">
-        <v>46.8</v>
+        <v>837</v>
+      </c>
+      <c r="D22" s="17">
+        <v>1</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="F22" s="20">
-        <v>670</v>
+        <v>180000</v>
       </c>
       <c r="G22" s="20">
         <f>F22*D22</f>
-        <v>31355.999999999996</v>
+        <v>180000</v>
       </c>
       <c r="H22" s="17" t="s">
         <v>771</v>
@@ -13018,13 +13016,13 @@
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" s="27">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="D23" s="23">
-        <v>37.200000000000003</v>
+        <v>46.8</v>
       </c>
       <c r="E23" s="17" t="s">
         <v>759</v>
@@ -13034,7 +13032,7 @@
       </c>
       <c r="G23" s="20">
         <f>F23*D23</f>
-        <v>24924.000000000004</v>
+        <v>31355.999999999996</v>
       </c>
       <c r="H23" s="17" t="s">
         <v>771</v>
@@ -13042,46 +13040,52 @@
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="27">
-        <v>22</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>779</v>
-      </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19">
+        <v>20</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>846</v>
+      </c>
+      <c r="D24" s="23">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>759</v>
+      </c>
+      <c r="F24" s="20">
+        <v>670</v>
+      </c>
+      <c r="G24" s="20">
         <f>F24*D24</f>
-        <v>0</v>
-      </c>
-      <c r="H24" s="22" t="s">
+        <v>24924.000000000004</v>
+      </c>
+      <c r="H24" s="17" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="27">
-        <v>23</v>
-      </c>
-      <c r="C25" s="25" t="s">
-        <v>789</v>
-      </c>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26">
+        <v>22</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>779</v>
+      </c>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19">
         <f>F25*D25</f>
         <v>0</v>
       </c>
-      <c r="H25" s="24" t="s">
-        <v>576</v>
+      <c r="H25" s="22" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="27">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C26" s="25" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="D26" s="24"/>
       <c r="E26" s="24"/>
@@ -13096,10 +13100,10 @@
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" s="27">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="24"/>
@@ -13114,10 +13118,10 @@
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" s="27">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C28" s="25" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="D28" s="24"/>
       <c r="E28" s="24"/>
@@ -13132,73 +13136,67 @@
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" s="27">
+        <v>26</v>
+      </c>
+      <c r="C29" s="25" t="s">
+        <v>791</v>
+      </c>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26">
+        <f>F29*D29</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="24" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B30" s="27">
         <v>27</v>
       </c>
-      <c r="C29" s="31" t="s">
+      <c r="C30" s="31" t="s">
         <v>757</v>
       </c>
-      <c r="D29" s="27">
+      <c r="D30" s="27">
         <f>(2000*1.05)*0.15</f>
         <v>315</v>
       </c>
-      <c r="E29" s="27" t="s">
+      <c r="E30" s="27" t="s">
         <v>759</v>
       </c>
-      <c r="F29" s="32">
+      <c r="F30" s="32">
         <v>670</v>
       </c>
-      <c r="G29" s="32">
-        <f>F29*D29</f>
+      <c r="G30" s="32">
+        <f>F30*D30</f>
         <v>211050</v>
       </c>
-      <c r="H29" s="27" t="s">
+      <c r="H30" s="27" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B30" s="27">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B31" s="27">
         <v>28</v>
       </c>
-      <c r="C30" s="31" t="s">
+      <c r="C31" s="31" t="s">
         <v>777</v>
       </c>
-      <c r="D30" s="33">
+      <c r="D31" s="33">
         <f>2000/13*2</f>
         <v>307.69230769230768</v>
       </c>
-      <c r="E30" s="27" t="s">
+      <c r="E31" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F30" s="32">
+      <c r="F31" s="32">
         <v>220.5</v>
-      </c>
-      <c r="G30" s="32">
-        <f>F30*D30</f>
-        <v>67846.153846153844</v>
-      </c>
-      <c r="H30" s="27" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B31" s="27">
-        <v>29</v>
-      </c>
-      <c r="C31" s="31" t="s">
-        <v>758</v>
-      </c>
-      <c r="D31" s="27">
-        <v>167</v>
-      </c>
-      <c r="E31" s="27" t="s">
-        <v>819</v>
-      </c>
-      <c r="F31" s="32">
-        <v>56.2</v>
       </c>
       <c r="G31" s="32">
         <f>F31*D31</f>
-        <v>9385.4</v>
+        <v>67846.153846153844</v>
       </c>
       <c r="H31" s="27" t="s">
         <v>635</v>
@@ -13206,23 +13204,23 @@
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="27">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="D32" s="27">
-        <v>1000</v>
+        <v>167</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>763</v>
+        <v>818</v>
       </c>
       <c r="F32" s="32">
-        <v>7.3</v>
+        <v>56.2</v>
       </c>
       <c r="G32" s="32">
         <f>F32*D32</f>
-        <v>7300</v>
+        <v>9385.4</v>
       </c>
       <c r="H32" s="27" t="s">
         <v>635</v>
@@ -13230,23 +13228,23 @@
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="27">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>809</v>
+        <v>762</v>
       </c>
       <c r="D33" s="27">
-        <v>315</v>
+        <v>1000</v>
       </c>
       <c r="E33" s="27" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="F33" s="32">
-        <v>50</v>
+        <v>7.3</v>
       </c>
       <c r="G33" s="32">
         <f>F33*D33</f>
-        <v>15750</v>
+        <v>7300</v>
       </c>
       <c r="H33" s="27" t="s">
         <v>635</v>
@@ -13254,23 +13252,23 @@
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="27">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>768</v>
+        <v>808</v>
       </c>
       <c r="D34" s="27">
-        <v>1</v>
+        <v>315</v>
       </c>
       <c r="E34" s="27" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="F34" s="32">
-        <v>49800</v>
+        <v>50</v>
       </c>
       <c r="G34" s="32">
         <f>F34*D34</f>
-        <v>49800</v>
+        <v>15750</v>
       </c>
       <c r="H34" s="27" t="s">
         <v>635</v>
@@ -13278,10 +13276,10 @@
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="27">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C35" s="31" t="s">
-        <v>773</v>
+        <v>768</v>
       </c>
       <c r="D35" s="27">
         <v>1</v>
@@ -13290,44 +13288,46 @@
         <v>760</v>
       </c>
       <c r="F35" s="32">
-        <v>1267174</v>
+        <v>49800</v>
       </c>
       <c r="G35" s="32">
         <f>F35*D35</f>
-        <v>1267174</v>
+        <v>49800</v>
       </c>
       <c r="H35" s="27" t="s">
-        <v>772</v>
+        <v>635</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="27">
-        <v>34</v>
-      </c>
-      <c r="C36" s="25" t="s">
-        <v>811</v>
-      </c>
-      <c r="D36" s="24">
-        <v>1</v>
-      </c>
-      <c r="E36" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="31" t="s">
+        <v>773</v>
+      </c>
+      <c r="D36" s="27">
+        <v>1</v>
+      </c>
+      <c r="E36" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26">
+      <c r="F36" s="32">
+        <v>1267174</v>
+      </c>
+      <c r="G36" s="32">
         <f>F36*D36</f>
-        <v>0</v>
-      </c>
-      <c r="H36" s="24" t="s">
-        <v>812</v>
+        <v>1267174</v>
+      </c>
+      <c r="H36" s="27" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" s="27">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>824</v>
+        <v>810</v>
       </c>
       <c r="D37" s="24">
         <v>1</v>
@@ -13341,179 +13341,192 @@
         <v>0</v>
       </c>
       <c r="H37" s="24" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" s="27">
-        <v>36</v>
-      </c>
-      <c r="C38" s="21" t="s">
-        <v>795</v>
-      </c>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19">
+        <v>35</v>
+      </c>
+      <c r="C38" s="25" t="s">
+        <v>823</v>
+      </c>
+      <c r="D38" s="24">
+        <v>1</v>
+      </c>
+      <c r="E38" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="F38" s="26"/>
+      <c r="G38" s="26">
         <f>F38*D38</f>
         <v>0</v>
       </c>
-      <c r="H38" s="22" t="s">
-        <v>419</v>
+      <c r="H38" s="24" t="s">
+        <v>811</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="27">
+        <v>36</v>
+      </c>
+      <c r="C39" s="21" t="s">
+        <v>794</v>
+      </c>
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="19">
+        <f>F39*D39</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="22" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B40" s="27">
         <v>37</v>
       </c>
-      <c r="C39" s="31" t="s">
-        <v>805</v>
-      </c>
-      <c r="D39" s="27">
+      <c r="C40" s="31" t="s">
+        <v>804</v>
+      </c>
+      <c r="D40" s="27">
         <v>252</v>
       </c>
-      <c r="E39" s="27" t="s">
+      <c r="E40" s="27" t="s">
         <v>761</v>
       </c>
-      <c r="F39" s="36">
+      <c r="F40" s="36">
         <v>269.5</v>
       </c>
-      <c r="G39" s="36">
+      <c r="G40" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>67914</v>
       </c>
-      <c r="H39" s="27" t="s">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B40" s="27">
+      <c r="H40" s="27" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B41" s="27">
         <v>38</v>
       </c>
-      <c r="C40" s="31" t="s">
-        <v>805</v>
-      </c>
-      <c r="D40" s="27">
+      <c r="C41" s="31" t="s">
+        <v>804</v>
+      </c>
+      <c r="D41" s="27">
         <v>84</v>
       </c>
-      <c r="E40" s="27" t="s">
+      <c r="E41" s="27" t="s">
         <v>761</v>
       </c>
-      <c r="F40" s="36">
+      <c r="F41" s="36">
         <v>115.5</v>
       </c>
-      <c r="G40" s="36">
+      <c r="G41" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>9702</v>
       </c>
-      <c r="H40" s="27" t="s">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B41" s="27">
+      <c r="H41" s="27" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B42" s="27">
         <v>39</v>
       </c>
-      <c r="C41" s="31" t="s">
-        <v>806</v>
-      </c>
-      <c r="D41" s="27">
+      <c r="C42" s="31" t="s">
+        <v>805</v>
+      </c>
+      <c r="D42" s="27">
         <v>42</v>
       </c>
-      <c r="E41" s="27" t="s">
+      <c r="E42" s="27" t="s">
         <v>761</v>
       </c>
-      <c r="F41" s="36">
+      <c r="F42" s="36">
         <v>35</v>
       </c>
-      <c r="G41" s="36">
+      <c r="G42" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>1470</v>
       </c>
-      <c r="H41" s="27" t="s">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B42" s="27">
+      <c r="H42" s="27" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B43" s="27">
         <v>40</v>
       </c>
-      <c r="C42" s="31" t="s">
-        <v>807</v>
-      </c>
-      <c r="D42" s="27">
+      <c r="C43" s="31" t="s">
+        <v>806</v>
+      </c>
+      <c r="D43" s="27">
         <v>4200</v>
       </c>
-      <c r="E42" s="27" t="s">
+      <c r="E43" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F42" s="36">
+      <c r="F43" s="36">
         <v>0.5</v>
       </c>
-      <c r="G42" s="36">
+      <c r="G43" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>2100</v>
       </c>
-      <c r="H42" s="27" t="s">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B43" s="27">
+      <c r="H43" s="27" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B44" s="27">
         <v>41</v>
       </c>
-      <c r="C43" s="31" t="s">
-        <v>808</v>
-      </c>
-      <c r="D43" s="27">
+      <c r="C44" s="31" t="s">
+        <v>807</v>
+      </c>
+      <c r="D44" s="27">
         <v>3100</v>
       </c>
-      <c r="E43" s="27" t="s">
+      <c r="E44" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F43" s="36">
+      <c r="F44" s="36">
         <v>0.5</v>
       </c>
-      <c r="G43" s="36">
+      <c r="G44" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>1550</v>
       </c>
-      <c r="H43" s="27" t="s">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B44" s="27">
+      <c r="H44" s="27" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B45" s="27">
         <v>42</v>
       </c>
-      <c r="C44" s="31" t="s">
-        <v>788</v>
-      </c>
-      <c r="D44" s="27">
-        <v>1</v>
-      </c>
-      <c r="E44" s="27" t="s">
+      <c r="C45" s="31" t="s">
+        <v>787</v>
+      </c>
+      <c r="D45" s="27">
+        <v>1</v>
+      </c>
+      <c r="E45" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F44" s="36">
+      <c r="F45" s="36">
         <v>157963.5</v>
       </c>
-      <c r="G44" s="36">
-        <f>F44*D44</f>
+      <c r="G45" s="36">
+        <f>F45*D45</f>
         <v>157963.5</v>
       </c>
-      <c r="H44" s="27" t="s">
-        <v>787</v>
-      </c>
-    </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B45" s="24"/>
-      <c r="C45" s="25"/>
-      <c r="D45" s="24"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="24"/>
+      <c r="H45" s="27" t="s">
+        <v>786</v>
+      </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" s="24"/>
@@ -13525,9 +13538,18 @@
       <c r="H46" s="24"/>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="G47" s="16">
+      <c r="B47" s="24"/>
+      <c r="C47" s="25"/>
+      <c r="D47" s="24"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="26"/>
+      <c r="G47" s="26"/>
+      <c r="H47" s="24"/>
+    </row>
+    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G48" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>2167285.0538461539</v>
+        <v>2168460.0538461539</v>
       </c>
     </row>
   </sheetData>
@@ -13562,12 +13584,12 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P1" s="14" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P2" s="14" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="3" spans="2:18" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -13575,7 +13597,7 @@
         <v>753</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="D3" t="s">
         <v>754</v>
@@ -13596,7 +13618,7 @@
         <v>767</v>
       </c>
       <c r="P3" s="14" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
@@ -13604,10 +13626,10 @@
         <v>1</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="E4" s="24"/>
       <c r="F4" s="24"/>
@@ -13617,19 +13639,19 @@
         <v>0</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="O4" s="14" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="P4" s="14" t="s">
+        <v>830</v>
+      </c>
+      <c r="Q4" s="14" t="s">
         <v>831</v>
       </c>
-      <c r="Q4" s="14" t="s">
+      <c r="R4" s="14" t="s">
         <v>832</v>
-      </c>
-      <c r="R4" s="14" t="s">
-        <v>833</v>
       </c>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
@@ -13637,7 +13659,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D5" s="21" t="s">
         <v>778</v>
@@ -13650,7 +13672,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="22" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="N5" s="37" t="s">
         <v>772</v>
@@ -13668,7 +13690,7 @@
         <v>0.33062288469044115</v>
       </c>
       <c r="R5" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.25">
@@ -13676,7 +13698,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>780</v>
@@ -13692,7 +13714,7 @@
         <v>449</v>
       </c>
       <c r="N6" s="45" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="O6" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Terraplanagem",Tabela24[Preço Total])</f>
@@ -13707,7 +13729,7 @@
         <v>0.60106053136595583</v>
       </c>
       <c r="R6" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
@@ -13715,10 +13737,10 @@
         <v>4</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="E7" s="22"/>
       <c r="F7" s="22"/>
@@ -13747,10 +13769,10 @@
         <v>5</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="E8" s="24">
         <v>26</v>
@@ -13767,10 +13789,10 @@
         <v>643</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="N8" s="45" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="O8" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
@@ -13786,10 +13808,10 @@
         <v>6</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E9" s="24">
         <v>500</v>
@@ -13806,7 +13828,7 @@
         <v>643</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="N9" s="42" t="s">
         <v>771</v>
@@ -13825,10 +13847,10 @@
         <v>7</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="E10" s="24"/>
       <c r="F10" s="24"/>
@@ -13857,10 +13879,10 @@
         <v>8</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E11" s="22">
         <v>54</v>
@@ -13874,10 +13896,10 @@
         <v>0</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="N11" s="41" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="O11" s="40">
         <f>SUMIF(Tabela24[Aplicação],"AVCB",Tabela24[Preço Total])</f>
@@ -13893,10 +13915,10 @@
         <v>9</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="E12" s="22">
         <v>30</v>
@@ -13910,7 +13932,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="22" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="N12" s="41" t="s">
         <v>449</v>
@@ -13929,10 +13951,10 @@
         <v>10</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="E13" s="24">
         <v>390</v>
@@ -13946,7 +13968,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="22" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="N13" s="41"/>
       <c r="O13" s="40"/>
@@ -13957,10 +13979,10 @@
         <v>11</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E14" s="47">
         <f>(84*1.02)*2*1.02</f>
@@ -13994,10 +14016,10 @@
         <v>12</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="E15" s="22">
         <f>84*7</f>
@@ -14031,7 +14053,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D16" s="25" t="s">
         <v>782</v>
@@ -14065,7 +14087,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D17" s="25" t="s">
         <v>783</v>
@@ -14081,7 +14103,7 @@
         <v>776</v>
       </c>
       <c r="N17" s="41" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="O17" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
@@ -14097,7 +14119,7 @@
         <v>15</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D18" s="25" t="s">
         <v>784</v>
@@ -14121,10 +14143,10 @@
         <v>16</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="E19" s="24">
         <v>1</v>
@@ -14147,10 +14169,10 @@
         <v>17</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="E20" s="17"/>
       <c r="F20" s="17"/>
@@ -14168,7 +14190,7 @@
         <v>18</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D21" s="18" t="s">
         <v>769</v>
@@ -14184,7 +14206,7 @@
         <v>771</v>
       </c>
       <c r="N21" s="41" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="O21" s="43">
         <f>SUM(O5:O17)</f>
@@ -14196,7 +14218,7 @@
         <v>19</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D22" s="18" t="s">
         <v>770</v>
@@ -14219,10 +14241,10 @@
         <v>20</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="E23" s="17">
         <v>1</v>
@@ -14246,7 +14268,7 @@
         <v>21</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D24" s="18" t="s">
         <v>774</v>
@@ -14267,7 +14289,7 @@
         <v>22</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D25" s="18" t="s">
         <v>775</v>
@@ -14288,7 +14310,7 @@
         <v>23</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D26" s="21" t="s">
         <v>779</v>
@@ -14309,10 +14331,10 @@
         <v>24</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="E27" s="24"/>
       <c r="F27" s="24"/>
@@ -14330,10 +14352,10 @@
         <v>25</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D28" s="25" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="E28" s="24"/>
       <c r="F28" s="24"/>
@@ -14351,10 +14373,10 @@
         <v>26</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="E29" s="24"/>
       <c r="F29" s="24"/>
@@ -14372,10 +14394,10 @@
         <v>27</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D30" s="25" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="E30" s="24"/>
       <c r="F30" s="24"/>
@@ -14393,7 +14415,7 @@
         <v>28</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D31" s="18" t="s">
         <v>757</v>
@@ -14421,7 +14443,7 @@
         <v>29</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D32" s="18" t="s">
         <v>777</v>
@@ -14449,7 +14471,7 @@
         <v>30</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D33" s="18" t="s">
         <v>758</v>
@@ -14477,7 +14499,7 @@
         <v>31</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D34" s="18" t="s">
         <v>762</v>
@@ -14504,10 +14526,10 @@
         <v>32</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="E35" s="23">
         <f>E31</f>
@@ -14532,7 +14554,7 @@
         <v>33</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D36" s="18" t="s">
         <v>768</v>
@@ -14559,10 +14581,10 @@
         <v>34</v>
       </c>
       <c r="C37" s="34" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="D37" s="25" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="E37" s="24">
         <v>110</v>
@@ -14584,7 +14606,7 @@
         <v>35</v>
       </c>
       <c r="C38" s="34" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="D38" s="25" t="s">
         <v>757</v>
@@ -14612,7 +14634,7 @@
         <v>36</v>
       </c>
       <c r="C39" s="34" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="D39" s="18" t="s">
         <v>777</v>
@@ -14640,10 +14662,10 @@
         <v>37</v>
       </c>
       <c r="C40" s="34" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="D40" s="25" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="E40" s="24">
         <v>1</v>
@@ -14667,7 +14689,7 @@
         <v>38</v>
       </c>
       <c r="C41" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D41" s="18" t="s">
         <v>773</v>
@@ -14694,10 +14716,10 @@
         <v>39</v>
       </c>
       <c r="C42" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D42" s="21" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E42" s="22"/>
       <c r="F42" s="22"/>
@@ -14715,10 +14737,10 @@
         <v>40</v>
       </c>
       <c r="C43" s="17" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="D43" s="25" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="E43" s="24">
         <v>1</v>
@@ -14734,7 +14756,7 @@
         <v>46600</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.25">
@@ -14742,10 +14764,10 @@
         <v>41</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="D44" s="25" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="E44" s="24">
         <v>1</v>
@@ -14761,7 +14783,7 @@
         <v>8100</v>
       </c>
       <c r="I44" s="24" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
@@ -14769,10 +14791,10 @@
         <v>42</v>
       </c>
       <c r="C45" s="17" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="D45" s="25" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="E45" s="24">
         <v>1</v>
@@ -14788,7 +14810,7 @@
         <v>5000</v>
       </c>
       <c r="I45" s="24" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
@@ -14796,10 +14818,10 @@
         <v>43</v>
       </c>
       <c r="C46" s="17" t="s">
+        <v>815</v>
+      </c>
+      <c r="D46" s="25" t="s">
         <v>816</v>
-      </c>
-      <c r="D46" s="25" t="s">
-        <v>817</v>
       </c>
       <c r="E46" s="24">
         <v>1</v>
@@ -14815,7 +14837,7 @@
         <v>298777</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
@@ -14823,10 +14845,10 @@
         <v>44</v>
       </c>
       <c r="C47" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D47" s="21" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="E47" s="22"/>
       <c r="F47" s="22"/>
@@ -14844,10 +14866,10 @@
         <v>45</v>
       </c>
       <c r="C48" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="D48" s="21" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="E48" s="22">
         <v>1</v>
@@ -14863,7 +14885,7 @@
         <v>791792.51</v>
       </c>
       <c r="I48" s="22" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 09:15
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2113" uniqueCount="851">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2116" uniqueCount="857">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2439,18 +2439,6 @@
     <t xml:space="preserve">Telha Trapeizodal TP40 </t>
   </si>
   <si>
-    <t>TELHA GALVALUME C/ RESINA RT-40/0980 -I 0,47</t>
-  </si>
-  <si>
-    <t>CUMEEIRA GALVALUME C/ RESINA RT-40/0980 -I 0,47</t>
-  </si>
-  <si>
-    <t>FIXADOR AUTO PERFURANTE CABECA 5/16 TRAXX -M PONTA 3 12X14X3/4</t>
-  </si>
-  <si>
-    <t>FIXADOR AUTO BROCANTE CABECA 5/16 TRAXX -I PONTA 1 1/4X14X7/8</t>
-  </si>
-  <si>
     <t>Diária bomba de concreto - valor por metro bombeado</t>
   </si>
   <si>
@@ -2577,7 +2565,37 @@
     <t>Fechamento em Alvenaria - Mão de Obra</t>
   </si>
   <si>
-    <t>Telha Termoacústica para cobertura do telhado</t>
+    <t>Topografia do local para locação dos pontos de concretagem dos pilares</t>
+  </si>
+  <si>
+    <t>Topografia</t>
+  </si>
+  <si>
+    <t>Estrtura do Galpão</t>
+  </si>
+  <si>
+    <t>Galpão em estrutura metálica 50 x 40 x 12m - Fechamentos inclusos M.O</t>
+  </si>
+  <si>
+    <t>TELHA FORRO METALICO NATURAL X BRANCO  0.43 EPS 50MM F1 RETARDANTE A CHAMAS</t>
+  </si>
+  <si>
+    <t>TELHA FORRO METALICO NATURAL X BRANCO 0.43 EPS 50MM F1 RETARDANTE A CHAMAS</t>
+  </si>
+  <si>
+    <t>PARAFUSO AUTOBROCANTE 12 X 5" 100UNI.</t>
+  </si>
+  <si>
+    <t>PARAFUSO AUTOBROCANTE 12 X 7/8 100UNI.</t>
+  </si>
+  <si>
+    <t>CUMEEIRA NATURAL 30X30</t>
+  </si>
+  <si>
+    <t>Frete do material de telhado</t>
+  </si>
+  <si>
+    <t>cx</t>
   </si>
 </sst>
 </file>
@@ -2685,7 +2703,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2809,6 +2827,9 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3070,10 +3091,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H45" totalsRowShown="0" dataDxfId="7">
-  <autoFilter ref="B3:H45"/>
-  <sortState ref="B4:H43">
-    <sortCondition ref="H3:H43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H46" totalsRowShown="0" dataDxfId="7">
+  <autoFilter ref="B3:H46"/>
+  <sortState ref="B4:H46">
+    <sortCondition ref="H3:H46"/>
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" name="Item" dataDxfId="6" dataCellStyle="Normal"/>
@@ -12537,11 +12558,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:J48"/>
+  <dimension ref="B3:J49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
-    <col min="3" max="3" width="66.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="90" customWidth="1"/>
     <col min="4" max="4" width="13.5703125" style="14" customWidth="1"/>
     <col min="5" max="5" width="10.7109375" style="14" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" style="15" customWidth="1"/>
@@ -12574,7 +12595,7 @@
         <v>767</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>828</v>
+        <v>824</v>
       </c>
     </row>
     <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -12640,7 +12661,7 @@
       </c>
       <c r="J6" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Pré Moldado",Tabela2[Preço Total])</f>
-        <v>1267174</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
@@ -12834,7 +12855,7 @@
         <v>12</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>849</v>
+        <v>845</v>
       </c>
       <c r="D15" s="24"/>
       <c r="E15" s="24"/>
@@ -12852,65 +12873,71 @@
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="27"/>
-      <c r="C16" s="25" t="s">
-        <v>850</v>
-      </c>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26">
-        <f>F16*D16</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="24" t="s">
-        <v>802</v>
+      <c r="B16" s="27">
+        <v>13</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>800</v>
+      </c>
+      <c r="D16" s="29">
+        <v>4</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>760</v>
+      </c>
+      <c r="F16" s="30">
+        <v>1500</v>
+      </c>
+      <c r="G16" s="30">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>6000</v>
+      </c>
+      <c r="H16" s="29" t="s">
+        <v>771</v>
       </c>
       <c r="J16" s="40"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="27">
-        <v>13</v>
-      </c>
-      <c r="C17" s="28" t="s">
-        <v>800</v>
-      </c>
-      <c r="D17" s="29">
-        <v>4</v>
-      </c>
-      <c r="E17" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>798</v>
+      </c>
+      <c r="D17" s="17">
+        <v>1</v>
+      </c>
+      <c r="E17" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="F17" s="30">
-        <v>1500</v>
-      </c>
-      <c r="G17" s="30">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>6000</v>
-      </c>
-      <c r="H17" s="29" t="s">
+      <c r="F17" s="20">
+        <v>4500</v>
+      </c>
+      <c r="G17" s="20">
+        <f>F17*D17</f>
+        <v>4500</v>
+      </c>
+      <c r="H17" s="17" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="27">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>798</v>
+        <v>769</v>
       </c>
       <c r="D18" s="17">
-        <v>1</v>
+        <v>2100</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="F18" s="20">
-        <v>4500</v>
-      </c>
+        <v>843</v>
+      </c>
+      <c r="F18" s="20"/>
       <c r="G18" s="20">
         <f>F18*D18</f>
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="H18" s="17" t="s">
         <v>771</v>
@@ -12918,16 +12945,16 @@
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="27">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="D19" s="17">
-        <v>2100</v>
+        <v>2300</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>847</v>
+        <v>843</v>
       </c>
       <c r="F19" s="20"/>
       <c r="G19" s="20">
@@ -12938,40 +12965,42 @@
         <v>771</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>848</v>
+        <v>844</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="27">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>770</v>
+        <v>840</v>
       </c>
       <c r="D20" s="17">
-        <v>2300</v>
+        <v>1</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>847</v>
-      </c>
-      <c r="F20" s="20"/>
+        <v>760</v>
+      </c>
+      <c r="F20" s="20">
+        <v>51500</v>
+      </c>
       <c r="G20" s="20">
         <f>F20*D20</f>
-        <v>0</v>
+        <v>51500</v>
       </c>
       <c r="H20" s="17" t="s">
         <v>771</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>848</v>
+        <v>844</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="27">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>844</v>
+        <v>833</v>
       </c>
       <c r="D21" s="17">
         <v>1</v>
@@ -12980,11 +13009,11 @@
         <v>760</v>
       </c>
       <c r="F21" s="20">
-        <v>51500</v>
+        <v>180000</v>
       </c>
       <c r="G21" s="20">
         <f>F21*D21</f>
-        <v>51500</v>
+        <v>180000</v>
       </c>
       <c r="H21" s="17" t="s">
         <v>771</v>
@@ -12992,23 +13021,23 @@
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" s="27">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>837</v>
-      </c>
-      <c r="D22" s="17">
-        <v>1</v>
+        <v>841</v>
+      </c>
+      <c r="D22" s="23">
+        <v>46.8</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="F22" s="20">
-        <v>180000</v>
+        <v>670</v>
       </c>
       <c r="G22" s="20">
         <f>F22*D22</f>
-        <v>180000</v>
+        <v>31355.999999999996</v>
       </c>
       <c r="H22" s="17" t="s">
         <v>771</v>
@@ -13016,13 +13045,13 @@
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" s="27">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="D23" s="23">
-        <v>46.8</v>
+        <v>37.200000000000003</v>
       </c>
       <c r="E23" s="17" t="s">
         <v>759</v>
@@ -13032,7 +13061,7 @@
       </c>
       <c r="G23" s="20">
         <f>F23*D23</f>
-        <v>31355.999999999996</v>
+        <v>24924.000000000004</v>
       </c>
       <c r="H23" s="17" t="s">
         <v>771</v>
@@ -13040,52 +13069,46 @@
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="27">
-        <v>20</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>846</v>
-      </c>
-      <c r="D24" s="23">
-        <v>37.200000000000003</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>759</v>
-      </c>
-      <c r="F24" s="20">
-        <v>670</v>
-      </c>
-      <c r="G24" s="20">
+        <v>22</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>779</v>
+      </c>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19">
         <f>F24*D24</f>
-        <v>24924.000000000004</v>
-      </c>
-      <c r="H24" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="H24" s="22" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="27">
-        <v>22</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>779</v>
-      </c>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19">
+        <v>23</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>788</v>
+      </c>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="26">
         <f>F25*D25</f>
         <v>0</v>
       </c>
-      <c r="H25" s="22" t="s">
-        <v>771</v>
+      <c r="H25" s="24" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="27">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C26" s="25" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="D26" s="24"/>
       <c r="E26" s="24"/>
@@ -13100,10 +13123,10 @@
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" s="27">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="24"/>
@@ -13118,10 +13141,10 @@
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" s="27">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C28" s="25" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="D28" s="24"/>
       <c r="E28" s="24"/>
@@ -13136,42 +13159,49 @@
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" s="27">
-        <v>26</v>
-      </c>
-      <c r="C29" s="25" t="s">
-        <v>791</v>
-      </c>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26">
+        <v>27</v>
+      </c>
+      <c r="C29" s="31" t="s">
+        <v>757</v>
+      </c>
+      <c r="D29" s="27">
+        <f>(2000*1.05)*0.15</f>
+        <v>315</v>
+      </c>
+      <c r="E29" s="27" t="s">
+        <v>759</v>
+      </c>
+      <c r="F29" s="32">
+        <v>670</v>
+      </c>
+      <c r="G29" s="32">
         <f>F29*D29</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="24" t="s">
-        <v>576</v>
+        <v>211050</v>
+      </c>
+      <c r="H29" s="27" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" s="27">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>757</v>
-      </c>
-      <c r="D30" s="27">
-        <f>(2000*1.05)*0.15</f>
-        <v>315</v>
+        <v>777</v>
+      </c>
+      <c r="D30" s="33">
+        <f>2000/13*2</f>
+        <v>307.69230769230768</v>
       </c>
       <c r="E30" s="27" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="F30" s="32">
-        <v>670</v>
+        <v>220.5</v>
       </c>
       <c r="G30" s="32">
         <f>F30*D30</f>
-        <v>211050</v>
+        <v>67846.153846153844</v>
       </c>
       <c r="H30" s="27" t="s">
         <v>635</v>
@@ -13179,24 +13209,23 @@
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" s="27">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>777</v>
-      </c>
-      <c r="D31" s="33">
-        <f>2000/13*2</f>
-        <v>307.69230769230768</v>
+        <v>758</v>
+      </c>
+      <c r="D31" s="27">
+        <v>167</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>760</v>
+        <v>814</v>
       </c>
       <c r="F31" s="32">
-        <v>220.5</v>
+        <v>56.2</v>
       </c>
       <c r="G31" s="32">
         <f>F31*D31</f>
-        <v>67846.153846153844</v>
+        <v>9385.4</v>
       </c>
       <c r="H31" s="27" t="s">
         <v>635</v>
@@ -13204,23 +13233,23 @@
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="27">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="D32" s="27">
-        <v>167</v>
+        <v>1000</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>818</v>
+        <v>763</v>
       </c>
       <c r="F32" s="32">
-        <v>56.2</v>
+        <v>7.3</v>
       </c>
       <c r="G32" s="32">
         <f>F32*D32</f>
-        <v>9385.4</v>
+        <v>7300</v>
       </c>
       <c r="H32" s="27" t="s">
         <v>635</v>
@@ -13228,23 +13257,23 @@
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="27">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>762</v>
+        <v>804</v>
       </c>
       <c r="D33" s="27">
-        <v>1000</v>
+        <v>315</v>
       </c>
       <c r="E33" s="27" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="F33" s="32">
-        <v>7.3</v>
+        <v>50</v>
       </c>
       <c r="G33" s="32">
         <f>F33*D33</f>
-        <v>7300</v>
+        <v>15750</v>
       </c>
       <c r="H33" s="27" t="s">
         <v>635</v>
@@ -13252,23 +13281,23 @@
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="27">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>808</v>
+        <v>768</v>
       </c>
       <c r="D34" s="27">
-        <v>315</v>
+        <v>1</v>
       </c>
       <c r="E34" s="27" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="F34" s="32">
-        <v>50</v>
+        <v>49800</v>
       </c>
       <c r="G34" s="32">
         <f>F34*D34</f>
-        <v>15750</v>
+        <v>49800</v>
       </c>
       <c r="H34" s="27" t="s">
         <v>635</v>
@@ -13276,10 +13305,10 @@
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="27">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C35" s="31" t="s">
-        <v>768</v>
+        <v>849</v>
       </c>
       <c r="D35" s="27">
         <v>1</v>
@@ -13288,46 +13317,44 @@
         <v>760</v>
       </c>
       <c r="F35" s="32">
-        <v>49800</v>
+        <v>1056959.67</v>
       </c>
       <c r="G35" s="32">
         <f>F35*D35</f>
-        <v>49800</v>
+        <v>1056959.67</v>
       </c>
       <c r="H35" s="27" t="s">
-        <v>635</v>
+        <v>848</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="27">
-        <v>33</v>
-      </c>
-      <c r="C36" s="31" t="s">
-        <v>773</v>
-      </c>
-      <c r="D36" s="27">
-        <v>1</v>
-      </c>
-      <c r="E36" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="C36" s="25" t="s">
+        <v>806</v>
+      </c>
+      <c r="D36" s="24">
+        <v>1</v>
+      </c>
+      <c r="E36" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F36" s="32">
-        <v>1267174</v>
-      </c>
-      <c r="G36" s="32">
+      <c r="F36" s="26"/>
+      <c r="G36" s="26">
         <f>F36*D36</f>
-        <v>1267174</v>
-      </c>
-      <c r="H36" s="27" t="s">
-        <v>772</v>
+        <v>0</v>
+      </c>
+      <c r="H36" s="24" t="s">
+        <v>807</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" s="27">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>810</v>
+        <v>819</v>
       </c>
       <c r="D37" s="24">
         <v>1</v>
@@ -13341,68 +13368,70 @@
         <v>0</v>
       </c>
       <c r="H37" s="24" t="s">
-        <v>811</v>
+        <v>807</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" s="27">
-        <v>35</v>
-      </c>
-      <c r="C38" s="25" t="s">
-        <v>823</v>
-      </c>
-      <c r="D38" s="24">
-        <v>1</v>
-      </c>
-      <c r="E38" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="F38" s="26"/>
-      <c r="G38" s="26">
+        <v>36</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>794</v>
+      </c>
+      <c r="D38" s="22"/>
+      <c r="E38" s="22"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19">
         <f>F38*D38</f>
         <v>0</v>
       </c>
-      <c r="H38" s="24" t="s">
-        <v>811</v>
+      <c r="H38" s="22" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="27">
-        <v>36</v>
-      </c>
-      <c r="C39" s="21" t="s">
-        <v>794</v>
-      </c>
-      <c r="D39" s="22"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19">
-        <f>F39*D39</f>
-        <v>0</v>
-      </c>
-      <c r="H39" s="22" t="s">
-        <v>419</v>
+        <v>37</v>
+      </c>
+      <c r="C39" s="48" t="s">
+        <v>850</v>
+      </c>
+      <c r="D39" s="27">
+        <v>1455.89</v>
+      </c>
+      <c r="E39" s="27" t="s">
+        <v>761</v>
+      </c>
+      <c r="F39" s="36">
+        <v>95.9</v>
+      </c>
+      <c r="G39" s="36">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>139619.85100000002</v>
+      </c>
+      <c r="H39" s="27" t="s">
+        <v>802</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" s="27">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C40" s="31" t="s">
-        <v>804</v>
+        <v>851</v>
       </c>
       <c r="D40" s="27">
-        <v>252</v>
+        <v>706.94</v>
       </c>
       <c r="E40" s="27" t="s">
         <v>761</v>
       </c>
       <c r="F40" s="36">
-        <v>269.5</v>
+        <v>95.9</v>
       </c>
       <c r="G40" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>67914</v>
+        <v>67795.546000000002</v>
       </c>
       <c r="H40" s="27" t="s">
         <v>802</v>
@@ -13410,23 +13439,23 @@
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" s="27">
-        <v>38</v>
-      </c>
-      <c r="C41" s="31" t="s">
-        <v>804</v>
+        <v>39</v>
+      </c>
+      <c r="C41" t="s">
+        <v>852</v>
       </c>
       <c r="D41" s="27">
-        <v>84</v>
+        <v>44</v>
       </c>
       <c r="E41" s="27" t="s">
-        <v>761</v>
+        <v>856</v>
       </c>
       <c r="F41" s="36">
-        <v>115.5</v>
+        <v>95</v>
       </c>
       <c r="G41" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>9702</v>
+        <v>4180</v>
       </c>
       <c r="H41" s="27" t="s">
         <v>802</v>
@@ -13434,23 +13463,23 @@
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" s="27">
-        <v>39</v>
-      </c>
-      <c r="C42" s="31" t="s">
-        <v>805</v>
+        <v>40</v>
+      </c>
+      <c r="C42" t="s">
+        <v>853</v>
       </c>
       <c r="D42" s="27">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="E42" s="27" t="s">
-        <v>761</v>
+        <v>856</v>
       </c>
       <c r="F42" s="36">
         <v>35</v>
       </c>
       <c r="G42" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>1470</v>
+        <v>105</v>
       </c>
       <c r="H42" s="27" t="s">
         <v>802</v>
@@ -13458,47 +13487,45 @@
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" s="27">
-        <v>40</v>
-      </c>
-      <c r="C43" s="31" t="s">
-        <v>806</v>
+        <v>41</v>
+      </c>
+      <c r="C43" t="s">
+        <v>854</v>
       </c>
       <c r="D43" s="27">
-        <v>4200</v>
+        <v>126</v>
       </c>
       <c r="E43" s="27" t="s">
         <v>760</v>
       </c>
       <c r="F43" s="36">
-        <v>0.5</v>
+        <v>25.9</v>
       </c>
       <c r="G43" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>2100</v>
+        <v>3263.3999999999996</v>
       </c>
       <c r="H43" s="27" t="s">
         <v>802</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B44" s="27">
-        <v>41</v>
-      </c>
-      <c r="C44" s="31" t="s">
-        <v>807</v>
+      <c r="B44" s="27"/>
+      <c r="C44" t="s">
+        <v>855</v>
       </c>
       <c r="D44" s="27">
-        <v>3100</v>
+        <v>1</v>
       </c>
       <c r="E44" s="27" t="s">
         <v>760</v>
       </c>
       <c r="F44" s="36">
-        <v>0.5</v>
+        <v>1750</v>
       </c>
       <c r="G44" s="36">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>1550</v>
+        <f>F44*D44</f>
+        <v>1750</v>
       </c>
       <c r="H44" s="27" t="s">
         <v>802</v>
@@ -13529,13 +13556,20 @@
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B46" s="24"/>
-      <c r="C46" s="25"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="25" t="s">
+        <v>846</v>
+      </c>
       <c r="D46" s="24"/>
       <c r="E46" s="24"/>
       <c r="F46" s="26"/>
-      <c r="G46" s="26"/>
-      <c r="H46" s="24"/>
+      <c r="G46" s="26">
+        <f>F46*D46</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="24" t="s">
+        <v>847</v>
+      </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" s="24"/>
@@ -13547,9 +13581,18 @@
       <c r="H47" s="24"/>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="G48" s="16">
+      <c r="B48" s="24"/>
+      <c r="C48" s="25"/>
+      <c r="D48" s="24"/>
+      <c r="E48" s="24"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="26"/>
+      <c r="H48" s="24"/>
+    </row>
+    <row r="49" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G49" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>2168460.0538461539</v>
+        <v>2092223.5208461538</v>
       </c>
     </row>
   </sheetData>
@@ -13584,12 +13627,12 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P1" s="14" t="s">
-        <v>834</v>
+        <v>830</v>
       </c>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P2" s="14" t="s">
-        <v>835</v>
+        <v>831</v>
       </c>
     </row>
     <row r="3" spans="2:18" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -13597,7 +13640,7 @@
         <v>753</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>813</v>
+        <v>809</v>
       </c>
       <c r="D3" t="s">
         <v>754</v>
@@ -13618,7 +13661,7 @@
         <v>767</v>
       </c>
       <c r="P3" s="14" t="s">
-        <v>836</v>
+        <v>832</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
@@ -13626,7 +13669,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D4" s="25" t="s">
         <v>796</v>
@@ -13639,19 +13682,19 @@
         <v>0</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>822</v>
+        <v>818</v>
       </c>
       <c r="O4" s="14" t="s">
+        <v>824</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>826</v>
+      </c>
+      <c r="Q4" s="14" t="s">
+        <v>827</v>
+      </c>
+      <c r="R4" s="14" t="s">
         <v>828</v>
-      </c>
-      <c r="P4" s="14" t="s">
-        <v>830</v>
-      </c>
-      <c r="Q4" s="14" t="s">
-        <v>831</v>
-      </c>
-      <c r="R4" s="14" t="s">
-        <v>832</v>
       </c>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
@@ -13659,7 +13702,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D5" s="21" t="s">
         <v>778</v>
@@ -13690,7 +13733,7 @@
         <v>0.33062288469044115</v>
       </c>
       <c r="R5" t="s">
-        <v>833</v>
+        <v>829</v>
       </c>
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.25">
@@ -13698,7 +13741,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>780</v>
@@ -13729,7 +13772,7 @@
         <v>0.60106053136595583</v>
       </c>
       <c r="R6" t="s">
-        <v>833</v>
+        <v>829</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
@@ -13737,10 +13780,10 @@
         <v>4</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>843</v>
+        <v>839</v>
       </c>
       <c r="E7" s="22"/>
       <c r="F7" s="22"/>
@@ -13769,7 +13812,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D8" s="25" t="s">
         <v>792</v>
@@ -13789,10 +13832,10 @@
         <v>643</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>819</v>
+        <v>815</v>
       </c>
       <c r="N8" s="45" t="s">
-        <v>811</v>
+        <v>807</v>
       </c>
       <c r="O8" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
@@ -13808,7 +13851,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D9" s="25" t="s">
         <v>793</v>
@@ -13828,7 +13871,7 @@
         <v>643</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>817</v>
+        <v>813</v>
       </c>
       <c r="N9" s="42" t="s">
         <v>771</v>
@@ -13847,10 +13890,10 @@
         <v>7</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>821</v>
+        <v>817</v>
       </c>
       <c r="E10" s="24"/>
       <c r="F10" s="24"/>
@@ -13879,10 +13922,10 @@
         <v>8</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>840</v>
+        <v>836</v>
       </c>
       <c r="E11" s="22">
         <v>54</v>
@@ -13896,7 +13939,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>841</v>
+        <v>837</v>
       </c>
       <c r="N11" s="41" t="s">
         <v>785</v>
@@ -13915,10 +13958,10 @@
         <v>9</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>842</v>
+        <v>838</v>
       </c>
       <c r="E12" s="22">
         <v>30</v>
@@ -13932,7 +13975,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="22" t="s">
-        <v>841</v>
+        <v>837</v>
       </c>
       <c r="N12" s="41" t="s">
         <v>449</v>
@@ -13951,10 +13994,10 @@
         <v>10</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>839</v>
+        <v>835</v>
       </c>
       <c r="E13" s="24">
         <v>390</v>
@@ -13968,7 +14011,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="22" t="s">
-        <v>841</v>
+        <v>837</v>
       </c>
       <c r="N13" s="41"/>
       <c r="O13" s="40"/>
@@ -13979,10 +14022,10 @@
         <v>11</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>840</v>
+        <v>836</v>
       </c>
       <c r="E14" s="47">
         <f>(84*1.02)*2*1.02</f>
@@ -14016,10 +14059,10 @@
         <v>12</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>839</v>
+        <v>835</v>
       </c>
       <c r="E15" s="22">
         <f>84*7</f>
@@ -14053,7 +14096,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D16" s="25" t="s">
         <v>782</v>
@@ -14087,7 +14130,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D17" s="25" t="s">
         <v>783</v>
@@ -14103,7 +14146,7 @@
         <v>776</v>
       </c>
       <c r="N17" s="41" t="s">
-        <v>822</v>
+        <v>818</v>
       </c>
       <c r="O17" s="40">
         <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
@@ -14119,7 +14162,7 @@
         <v>15</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D18" s="25" t="s">
         <v>784</v>
@@ -14143,10 +14186,10 @@
         <v>16</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>826</v>
+        <v>822</v>
       </c>
       <c r="E19" s="24">
         <v>1</v>
@@ -14169,7 +14212,7 @@
         <v>17</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D20" s="18" t="s">
         <v>797</v>
@@ -14190,7 +14233,7 @@
         <v>18</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D21" s="18" t="s">
         <v>769</v>
@@ -14206,7 +14249,7 @@
         <v>771</v>
       </c>
       <c r="N21" s="41" t="s">
-        <v>829</v>
+        <v>825</v>
       </c>
       <c r="O21" s="43">
         <f>SUM(O5:O17)</f>
@@ -14218,7 +14261,7 @@
         <v>19</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D22" s="18" t="s">
         <v>770</v>
@@ -14241,10 +14284,10 @@
         <v>20</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>838</v>
+        <v>834</v>
       </c>
       <c r="E23" s="17">
         <v>1</v>
@@ -14268,7 +14311,7 @@
         <v>21</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D24" s="18" t="s">
         <v>774</v>
@@ -14289,7 +14332,7 @@
         <v>22</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D25" s="18" t="s">
         <v>775</v>
@@ -14310,7 +14353,7 @@
         <v>23</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D26" s="21" t="s">
         <v>779</v>
@@ -14331,7 +14374,7 @@
         <v>24</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D27" s="25" t="s">
         <v>788</v>
@@ -14352,7 +14395,7 @@
         <v>25</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D28" s="25" t="s">
         <v>789</v>
@@ -14373,7 +14416,7 @@
         <v>26</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D29" s="25" t="s">
         <v>790</v>
@@ -14394,7 +14437,7 @@
         <v>27</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D30" s="25" t="s">
         <v>791</v>
@@ -14415,7 +14458,7 @@
         <v>28</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D31" s="18" t="s">
         <v>757</v>
@@ -14443,7 +14486,7 @@
         <v>29</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D32" s="18" t="s">
         <v>777</v>
@@ -14471,7 +14514,7 @@
         <v>30</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D33" s="18" t="s">
         <v>758</v>
@@ -14499,7 +14542,7 @@
         <v>31</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D34" s="18" t="s">
         <v>762</v>
@@ -14526,10 +14569,10 @@
         <v>32</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="E35" s="23">
         <f>E31</f>
@@ -14554,7 +14597,7 @@
         <v>33</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D36" s="18" t="s">
         <v>768</v>
@@ -14581,10 +14624,10 @@
         <v>34</v>
       </c>
       <c r="C37" s="34" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="D37" s="25" t="s">
-        <v>825</v>
+        <v>821</v>
       </c>
       <c r="E37" s="24">
         <v>110</v>
@@ -14606,7 +14649,7 @@
         <v>35</v>
       </c>
       <c r="C38" s="34" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="D38" s="25" t="s">
         <v>757</v>
@@ -14634,7 +14677,7 @@
         <v>36</v>
       </c>
       <c r="C39" s="34" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="D39" s="18" t="s">
         <v>777</v>
@@ -14662,10 +14705,10 @@
         <v>37</v>
       </c>
       <c r="C40" s="34" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="D40" s="25" t="s">
-        <v>824</v>
+        <v>820</v>
       </c>
       <c r="E40" s="24">
         <v>1</v>
@@ -14689,7 +14732,7 @@
         <v>38</v>
       </c>
       <c r="C41" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D41" s="18" t="s">
         <v>773</v>
@@ -14716,7 +14759,7 @@
         <v>39</v>
       </c>
       <c r="C42" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D42" s="21" t="s">
         <v>795</v>
@@ -14737,10 +14780,10 @@
         <v>40</v>
       </c>
       <c r="C43" s="17" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="D43" s="25" t="s">
-        <v>809</v>
+        <v>805</v>
       </c>
       <c r="E43" s="24">
         <v>1</v>
@@ -14756,7 +14799,7 @@
         <v>46600</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>811</v>
+        <v>807</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.25">
@@ -14764,10 +14807,10 @@
         <v>41</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="D44" s="25" t="s">
-        <v>812</v>
+        <v>808</v>
       </c>
       <c r="E44" s="24">
         <v>1</v>
@@ -14783,7 +14826,7 @@
         <v>8100</v>
       </c>
       <c r="I44" s="24" t="s">
-        <v>811</v>
+        <v>807</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
@@ -14791,10 +14834,10 @@
         <v>42</v>
       </c>
       <c r="C45" s="17" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="D45" s="25" t="s">
-        <v>827</v>
+        <v>823</v>
       </c>
       <c r="E45" s="24">
         <v>1</v>
@@ -14810,7 +14853,7 @@
         <v>5000</v>
       </c>
       <c r="I45" s="24" t="s">
-        <v>811</v>
+        <v>807</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
@@ -14818,10 +14861,10 @@
         <v>43</v>
       </c>
       <c r="C46" s="17" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="D46" s="25" t="s">
-        <v>816</v>
+        <v>812</v>
       </c>
       <c r="E46" s="24">
         <v>1</v>
@@ -14837,7 +14880,7 @@
         <v>298777</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>811</v>
+        <v>807</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
@@ -14845,7 +14888,7 @@
         <v>44</v>
       </c>
       <c r="C47" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D47" s="21" t="s">
         <v>794</v>
@@ -14866,7 +14909,7 @@
         <v>45</v>
       </c>
       <c r="C48" s="17" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D48" s="21" t="s">
         <v>787</v>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 09:18
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2116" uniqueCount="857">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2113" uniqueCount="856">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2524,9 +2524,6 @@
   </si>
   <si>
     <t>C&gt;90%</t>
-  </si>
-  <si>
-    <t>Arrasamento das estacas, Locação dos cálices e concretagem</t>
   </si>
   <si>
     <t>Arrasamento das estacas, locação dos blocos e concretagem dos cálices</t>
@@ -2703,7 +2700,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2830,6 +2827,13 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3091,8 +3095,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H46" totalsRowShown="0" dataDxfId="7">
-  <autoFilter ref="B3:H46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H45" totalsRowShown="0" dataDxfId="7">
+  <autoFilter ref="B3:H45"/>
   <sortState ref="B4:H46">
     <sortCondition ref="H3:H46"/>
   </sortState>
@@ -12558,7 +12562,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:J49"/>
+  <dimension ref="B3:J48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -12617,7 +12621,7 @@
       </c>
       <c r="J4" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
-        <v>298280</v>
+        <v>118280</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
@@ -12694,23 +12698,23 @@
       <c r="B8" s="27">
         <v>5</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="49" t="s">
         <v>793</v>
       </c>
-      <c r="D8" s="24">
-        <v>500</v>
-      </c>
-      <c r="E8" s="24" t="s">
+      <c r="D8" s="50">
+        <v>600</v>
+      </c>
+      <c r="E8" s="50" t="s">
         <v>761</v>
       </c>
-      <c r="F8" s="26">
-        <v>2.35</v>
-      </c>
-      <c r="G8" s="26">
+      <c r="F8" s="51">
+        <v>3.35</v>
+      </c>
+      <c r="G8" s="51">
         <f>F8*D8</f>
-        <v>1175</v>
-      </c>
-      <c r="H8" s="24" t="s">
+        <v>2010</v>
+      </c>
+      <c r="H8" s="50" t="s">
         <v>643</v>
       </c>
       <c r="J8" s="40">
@@ -12803,7 +12807,7 @@
       </c>
       <c r="J12" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Elétrica",Tabela2[Preço Total])</f>
-        <v>1175</v>
+        <v>2010</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
@@ -12855,7 +12859,7 @@
         <v>12</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="D15" s="24"/>
       <c r="E15" s="24"/>
@@ -12901,23 +12905,23 @@
       <c r="B17" s="27">
         <v>14</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="31" t="s">
         <v>798</v>
       </c>
-      <c r="D17" s="17">
-        <v>1</v>
-      </c>
-      <c r="E17" s="17" t="s">
+      <c r="D17" s="27">
+        <v>1</v>
+      </c>
+      <c r="E17" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F17" s="20">
+      <c r="F17" s="32">
         <v>4500</v>
       </c>
-      <c r="G17" s="20">
+      <c r="G17" s="32">
         <f>F17*D17</f>
         <v>4500</v>
       </c>
-      <c r="H17" s="17" t="s">
+      <c r="H17" s="27" t="s">
         <v>771</v>
       </c>
     </row>
@@ -12932,7 +12936,7 @@
         <v>2100</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="F18" s="20"/>
       <c r="G18" s="20">
@@ -12954,7 +12958,7 @@
         <v>2300</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="F19" s="20"/>
       <c r="G19" s="20">
@@ -12965,132 +12969,126 @@
         <v>771</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="27">
         <v>17</v>
       </c>
-      <c r="C20" s="18" t="s">
-        <v>840</v>
-      </c>
-      <c r="D20" s="17">
-        <v>1</v>
-      </c>
-      <c r="E20" s="17" t="s">
+      <c r="C20" s="31" t="s">
+        <v>839</v>
+      </c>
+      <c r="D20" s="27">
+        <v>1</v>
+      </c>
+      <c r="E20" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F20" s="20">
+      <c r="F20" s="32">
         <v>51500</v>
       </c>
-      <c r="G20" s="20">
+      <c r="G20" s="32">
         <f>F20*D20</f>
         <v>51500</v>
       </c>
-      <c r="H20" s="17" t="s">
+      <c r="H20" s="27" t="s">
         <v>771</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="27">
-        <v>18</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>833</v>
-      </c>
-      <c r="D21" s="17">
-        <v>1</v>
-      </c>
-      <c r="E21" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="F21" s="20">
-        <v>180000</v>
-      </c>
-      <c r="G21" s="20">
+        <v>19</v>
+      </c>
+      <c r="C21" s="31" t="s">
+        <v>840</v>
+      </c>
+      <c r="D21" s="33">
+        <v>46.8</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>759</v>
+      </c>
+      <c r="F21" s="32">
+        <v>670</v>
+      </c>
+      <c r="G21" s="32">
         <f>F21*D21</f>
-        <v>180000</v>
-      </c>
-      <c r="H21" s="17" t="s">
+        <v>31355.999999999996</v>
+      </c>
+      <c r="H21" s="27" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" s="27">
-        <v>19</v>
-      </c>
-      <c r="C22" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="31" t="s">
         <v>841</v>
       </c>
-      <c r="D22" s="23">
-        <v>46.8</v>
-      </c>
-      <c r="E22" s="17" t="s">
+      <c r="D22" s="33">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E22" s="27" t="s">
         <v>759</v>
       </c>
-      <c r="F22" s="20">
+      <c r="F22" s="32">
         <v>670</v>
       </c>
-      <c r="G22" s="20">
+      <c r="G22" s="32">
         <f>F22*D22</f>
-        <v>31355.999999999996</v>
-      </c>
-      <c r="H22" s="17" t="s">
+        <v>24924.000000000004</v>
+      </c>
+      <c r="H22" s="27" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" s="27">
-        <v>20</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>842</v>
-      </c>
-      <c r="D23" s="23">
-        <v>37.200000000000003</v>
-      </c>
-      <c r="E23" s="17" t="s">
-        <v>759</v>
-      </c>
-      <c r="F23" s="20">
-        <v>670</v>
-      </c>
-      <c r="G23" s="20">
+        <v>22</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>779</v>
+      </c>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="19">
         <f>F23*D23</f>
-        <v>24924.000000000004</v>
-      </c>
-      <c r="H23" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="H23" s="22" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="27">
-        <v>22</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>779</v>
-      </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19">
+        <v>23</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>788</v>
+      </c>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26">
         <f>F24*D24</f>
         <v>0</v>
       </c>
-      <c r="H24" s="22" t="s">
-        <v>771</v>
+      <c r="H24" s="24" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="27">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="D25" s="24"/>
       <c r="E25" s="24"/>
@@ -13105,10 +13103,10 @@
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="27">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C26" s="25" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="D26" s="24"/>
       <c r="E26" s="24"/>
@@ -13123,10 +13121,10 @@
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" s="27">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="24"/>
@@ -13141,42 +13139,49 @@
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" s="27">
-        <v>26</v>
-      </c>
-      <c r="C28" s="25" t="s">
-        <v>791</v>
-      </c>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26">
+        <v>27</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>757</v>
+      </c>
+      <c r="D28" s="27">
+        <f>(2000*1.05)*0.15</f>
+        <v>315</v>
+      </c>
+      <c r="E28" s="27" t="s">
+        <v>759</v>
+      </c>
+      <c r="F28" s="32">
+        <v>670</v>
+      </c>
+      <c r="G28" s="32">
         <f>F28*D28</f>
-        <v>0</v>
-      </c>
-      <c r="H28" s="24" t="s">
-        <v>576</v>
+        <v>211050</v>
+      </c>
+      <c r="H28" s="27" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" s="27">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>757</v>
-      </c>
-      <c r="D29" s="27">
-        <f>(2000*1.05)*0.15</f>
-        <v>315</v>
+        <v>777</v>
+      </c>
+      <c r="D29" s="33">
+        <f>2000/13*2</f>
+        <v>307.69230769230768</v>
       </c>
       <c r="E29" s="27" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="F29" s="32">
-        <v>670</v>
+        <v>220.5</v>
       </c>
       <c r="G29" s="32">
         <f>F29*D29</f>
-        <v>211050</v>
+        <v>67846.153846153844</v>
       </c>
       <c r="H29" s="27" t="s">
         <v>635</v>
@@ -13184,24 +13189,23 @@
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" s="27">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>777</v>
-      </c>
-      <c r="D30" s="33">
-        <f>2000/13*2</f>
-        <v>307.69230769230768</v>
+        <v>758</v>
+      </c>
+      <c r="D30" s="27">
+        <v>167</v>
       </c>
       <c r="E30" s="27" t="s">
-        <v>760</v>
+        <v>814</v>
       </c>
       <c r="F30" s="32">
-        <v>220.5</v>
+        <v>56.2</v>
       </c>
       <c r="G30" s="32">
         <f>F30*D30</f>
-        <v>67846.153846153844</v>
+        <v>9385.4</v>
       </c>
       <c r="H30" s="27" t="s">
         <v>635</v>
@@ -13209,23 +13213,23 @@
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" s="27">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="D31" s="27">
-        <v>167</v>
+        <v>1000</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>814</v>
+        <v>763</v>
       </c>
       <c r="F31" s="32">
-        <v>56.2</v>
+        <v>7.3</v>
       </c>
       <c r="G31" s="32">
         <f>F31*D31</f>
-        <v>9385.4</v>
+        <v>7300</v>
       </c>
       <c r="H31" s="27" t="s">
         <v>635</v>
@@ -13233,23 +13237,23 @@
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="27">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>762</v>
+        <v>804</v>
       </c>
       <c r="D32" s="27">
-        <v>1000</v>
+        <v>315</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="F32" s="32">
-        <v>7.3</v>
+        <v>50</v>
       </c>
       <c r="G32" s="32">
         <f>F32*D32</f>
-        <v>7300</v>
+        <v>15750</v>
       </c>
       <c r="H32" s="27" t="s">
         <v>635</v>
@@ -13257,23 +13261,23 @@
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="27">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>804</v>
+        <v>768</v>
       </c>
       <c r="D33" s="27">
-        <v>315</v>
+        <v>1</v>
       </c>
       <c r="E33" s="27" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="F33" s="32">
-        <v>50</v>
+        <v>49800</v>
       </c>
       <c r="G33" s="32">
         <f>F33*D33</f>
-        <v>15750</v>
+        <v>49800</v>
       </c>
       <c r="H33" s="27" t="s">
         <v>635</v>
@@ -13281,10 +13285,10 @@
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="27">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>768</v>
+        <v>848</v>
       </c>
       <c r="D34" s="27">
         <v>1</v>
@@ -13293,46 +13297,44 @@
         <v>760</v>
       </c>
       <c r="F34" s="32">
-        <v>49800</v>
+        <v>1056959.67</v>
       </c>
       <c r="G34" s="32">
         <f>F34*D34</f>
-        <v>49800</v>
+        <v>1056959.67</v>
       </c>
       <c r="H34" s="27" t="s">
-        <v>635</v>
+        <v>847</v>
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="27">
-        <v>33</v>
-      </c>
-      <c r="C35" s="31" t="s">
-        <v>849</v>
-      </c>
-      <c r="D35" s="27">
-        <v>1</v>
-      </c>
-      <c r="E35" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="C35" s="25" t="s">
+        <v>806</v>
+      </c>
+      <c r="D35" s="24">
+        <v>1</v>
+      </c>
+      <c r="E35" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F35" s="32">
-        <v>1056959.67</v>
-      </c>
-      <c r="G35" s="32">
+      <c r="F35" s="26"/>
+      <c r="G35" s="26">
         <f>F35*D35</f>
-        <v>1056959.67</v>
-      </c>
-      <c r="H35" s="27" t="s">
-        <v>848</v>
+        <v>0</v>
+      </c>
+      <c r="H35" s="24" t="s">
+        <v>807</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="27">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C36" s="25" t="s">
-        <v>806</v>
+        <v>819</v>
       </c>
       <c r="D36" s="24">
         <v>1</v>
@@ -13351,53 +13353,55 @@
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" s="27">
-        <v>35</v>
-      </c>
-      <c r="C37" s="25" t="s">
-        <v>819</v>
-      </c>
-      <c r="D37" s="24">
-        <v>1</v>
-      </c>
-      <c r="E37" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26">
+        <v>36</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>794</v>
+      </c>
+      <c r="D37" s="22"/>
+      <c r="E37" s="22"/>
+      <c r="F37" s="19"/>
+      <c r="G37" s="19">
         <f>F37*D37</f>
         <v>0</v>
       </c>
-      <c r="H37" s="24" t="s">
-        <v>807</v>
+      <c r="H37" s="22" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" s="27">
-        <v>36</v>
-      </c>
-      <c r="C38" s="21" t="s">
-        <v>794</v>
-      </c>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19">
-        <f>F38*D38</f>
-        <v>0</v>
-      </c>
-      <c r="H38" s="22" t="s">
-        <v>419</v>
+        <v>37</v>
+      </c>
+      <c r="C38" s="48" t="s">
+        <v>849</v>
+      </c>
+      <c r="D38" s="27">
+        <v>1455.89</v>
+      </c>
+      <c r="E38" s="27" t="s">
+        <v>761</v>
+      </c>
+      <c r="F38" s="36">
+        <v>95.9</v>
+      </c>
+      <c r="G38" s="36">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>139619.85100000002</v>
+      </c>
+      <c r="H38" s="27" t="s">
+        <v>802</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="27">
-        <v>37</v>
-      </c>
-      <c r="C39" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="C39" s="31" t="s">
         <v>850</v>
       </c>
       <c r="D39" s="27">
-        <v>1455.89</v>
+        <v>706.94</v>
       </c>
       <c r="E39" s="27" t="s">
         <v>761</v>
@@ -13407,7 +13411,7 @@
       </c>
       <c r="G39" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>139619.85100000002</v>
+        <v>67795.546000000002</v>
       </c>
       <c r="H39" s="27" t="s">
         <v>802</v>
@@ -13415,23 +13419,23 @@
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" s="27">
-        <v>38</v>
-      </c>
-      <c r="C40" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="C40" t="s">
         <v>851</v>
       </c>
       <c r="D40" s="27">
-        <v>706.94</v>
+        <v>44</v>
       </c>
       <c r="E40" s="27" t="s">
-        <v>761</v>
+        <v>855</v>
       </c>
       <c r="F40" s="36">
-        <v>95.9</v>
+        <v>95</v>
       </c>
       <c r="G40" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>67795.546000000002</v>
+        <v>4180</v>
       </c>
       <c r="H40" s="27" t="s">
         <v>802</v>
@@ -13439,23 +13443,23 @@
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" s="27">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C41" t="s">
         <v>852</v>
       </c>
       <c r="D41" s="27">
-        <v>44</v>
+        <v>3</v>
       </c>
       <c r="E41" s="27" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="F41" s="36">
-        <v>95</v>
+        <v>35</v>
       </c>
       <c r="G41" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>4180</v>
+        <v>105</v>
       </c>
       <c r="H41" s="27" t="s">
         <v>802</v>
@@ -13463,56 +13467,56 @@
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" s="27">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C42" t="s">
         <v>853</v>
       </c>
       <c r="D42" s="27">
-        <v>3</v>
+        <v>126</v>
       </c>
       <c r="E42" s="27" t="s">
-        <v>856</v>
+        <v>760</v>
       </c>
       <c r="F42" s="36">
-        <v>35</v>
+        <v>25.9</v>
       </c>
       <c r="G42" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>105</v>
+        <v>3263.3999999999996</v>
       </c>
       <c r="H42" s="27" t="s">
         <v>802</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B43" s="27">
-        <v>41</v>
-      </c>
+      <c r="B43" s="27"/>
       <c r="C43" t="s">
         <v>854</v>
       </c>
       <c r="D43" s="27">
-        <v>126</v>
+        <v>1</v>
       </c>
       <c r="E43" s="27" t="s">
         <v>760</v>
       </c>
       <c r="F43" s="36">
-        <v>25.9</v>
+        <v>1750</v>
       </c>
       <c r="G43" s="36">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>3263.3999999999996</v>
+        <f>F43*D43</f>
+        <v>1750</v>
       </c>
       <c r="H43" s="27" t="s">
         <v>802</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B44" s="27"/>
-      <c r="C44" t="s">
-        <v>855</v>
+      <c r="B44" s="27">
+        <v>42</v>
+      </c>
+      <c r="C44" s="31" t="s">
+        <v>787</v>
       </c>
       <c r="D44" s="27">
         <v>1</v>
@@ -13521,55 +13525,40 @@
         <v>760</v>
       </c>
       <c r="F44" s="36">
-        <v>1750</v>
+        <v>157963.5</v>
       </c>
       <c r="G44" s="36">
         <f>F44*D44</f>
-        <v>1750</v>
+        <v>157963.5</v>
       </c>
       <c r="H44" s="27" t="s">
-        <v>802</v>
+        <v>786</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B45" s="27">
-        <v>42</v>
-      </c>
-      <c r="C45" s="31" t="s">
-        <v>787</v>
-      </c>
-      <c r="D45" s="27">
-        <v>1</v>
-      </c>
-      <c r="E45" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="F45" s="36">
-        <v>157963.5</v>
-      </c>
-      <c r="G45" s="36">
+      <c r="B45" s="27"/>
+      <c r="C45" s="25" t="s">
+        <v>845</v>
+      </c>
+      <c r="D45" s="24"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="26"/>
+      <c r="G45" s="26">
         <f>F45*D45</f>
-        <v>157963.5</v>
-      </c>
-      <c r="H45" s="27" t="s">
-        <v>786</v>
+        <v>0</v>
+      </c>
+      <c r="H45" s="24" t="s">
+        <v>846</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B46" s="27"/>
-      <c r="C46" s="25" t="s">
-        <v>846</v>
-      </c>
+      <c r="B46" s="24"/>
+      <c r="C46" s="25"/>
       <c r="D46" s="24"/>
       <c r="E46" s="24"/>
       <c r="F46" s="26"/>
-      <c r="G46" s="26">
-        <f>F46*D46</f>
-        <v>0</v>
-      </c>
-      <c r="H46" s="24" t="s">
-        <v>847</v>
-      </c>
+      <c r="G46" s="26"/>
+      <c r="H46" s="24"/>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" s="24"/>
@@ -13581,18 +13570,9 @@
       <c r="H47" s="24"/>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B48" s="24"/>
-      <c r="C48" s="25"/>
-      <c r="D48" s="24"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="26"/>
-      <c r="G48" s="26"/>
-      <c r="H48" s="24"/>
-    </row>
-    <row r="49" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G49" s="16">
+      <c r="G48" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>2092223.5208461538</v>
+        <v>1913058.5208461538</v>
       </c>
     </row>
   </sheetData>
@@ -13783,7 +13763,7 @@
         <v>810</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="E7" s="22"/>
       <c r="F7" s="22"/>
@@ -13925,7 +13905,7 @@
         <v>810</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E11" s="22">
         <v>54</v>
@@ -13939,7 +13919,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="N11" s="41" t="s">
         <v>785</v>
@@ -13961,7 +13941,7 @@
         <v>810</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="E12" s="22">
         <v>30</v>
@@ -13975,7 +13955,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="22" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="N12" s="41" t="s">
         <v>449</v>
@@ -13997,7 +13977,7 @@
         <v>810</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="E13" s="24">
         <v>390</v>
@@ -14011,7 +13991,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="22" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="N13" s="41"/>
       <c r="O13" s="40"/>
@@ -14025,7 +14005,7 @@
         <v>810</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E14" s="47">
         <f>(84*1.02)*2*1.02</f>
@@ -14062,7 +14042,7 @@
         <v>810</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="E15" s="22">
         <f>84*7</f>
@@ -14287,7 +14267,7 @@
         <v>810</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="E23" s="17">
         <v>1</v>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 14:19
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2113" uniqueCount="856">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2135" uniqueCount="865">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2370,9 +2370,6 @@
     <t xml:space="preserve">Calha metálica </t>
   </si>
   <si>
-    <t xml:space="preserve">tubulação de drenagem pluvial </t>
-  </si>
-  <si>
     <t xml:space="preserve">Rufo de acabamento </t>
   </si>
   <si>
@@ -2593,6 +2590,36 @@
   </si>
   <si>
     <t>cx</t>
+  </si>
+  <si>
+    <t>Cumeeira TP40</t>
+  </si>
+  <si>
+    <t>Projeto de combate ao incêndio - material, execução e aprovação</t>
+  </si>
+  <si>
+    <t>Rampas Niveladoras para a expedição</t>
+  </si>
+  <si>
+    <t>Sistema de alarme de incêndio</t>
+  </si>
+  <si>
+    <t>Sistema de Alarme de incêndio</t>
+  </si>
+  <si>
+    <t>Calha metálica para o pré moldado (de acordo com o projeto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caixa Parafuso autobrocante 12 x 3/4" 100un </t>
+  </si>
+  <si>
+    <t>Frete para telhas</t>
+  </si>
+  <si>
+    <t>Portas automáticas para as docas</t>
+  </si>
+  <si>
+    <t>Mão de obra para fechamento em alvenaria na parte interna do galpão blocado</t>
   </si>
 </sst>
 </file>
@@ -2804,7 +2831,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2822,9 +2848,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2835,6 +2858,12 @@
     <xf numFmtId="44" fontId="4" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -2842,6 +2871,77 @@
     <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="17">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -2897,33 +2997,6 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -3038,38 +3111,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -3095,43 +3136,43 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H45" totalsRowShown="0" dataDxfId="7">
-  <autoFilter ref="B3:H45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H46" totalsRowShown="0" dataDxfId="9">
+  <autoFilter ref="B3:H46"/>
   <sortState ref="B4:H46">
     <sortCondition ref="H3:H46"/>
   </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" name="Item" dataDxfId="6" dataCellStyle="Normal"/>
-    <tableColumn id="2" name="Descrição" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="2" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="1" dataCellStyle="Moeda">
+    <tableColumn id="1" name="Item" dataDxfId="2" dataCellStyle="Normal"/>
+    <tableColumn id="2" name="Descrição" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="8" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="7" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="6" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="5" dataCellStyle="Moeda">
       <calculatedColumnFormula>F4*D4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="0" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="4" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I48" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:I48"/>
-  <sortState ref="B4:I48">
-    <sortCondition ref="I3:I48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I55" totalsRowShown="0" dataDxfId="16">
+  <autoFilter ref="B3:I55"/>
+  <sortState ref="B4:I51">
+    <sortCondition ref="I3:I51"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" name="Item" dataDxfId="15" dataCellStyle="Normal"/>
-    <tableColumn id="8" name="Local" dataDxfId="14"/>
-    <tableColumn id="2" name="Descrição" dataDxfId="13" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="12" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="11" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="10" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="9" dataCellStyle="Moeda">
+    <tableColumn id="1" name="Item" dataDxfId="0" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Local" dataDxfId="1"/>
+    <tableColumn id="2" name="Descrição" dataDxfId="15" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="14" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="13" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="12" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="11" dataCellStyle="Moeda">
       <calculatedColumnFormula>G4*E4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="8" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="10" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12562,7 +12603,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:J48"/>
+  <dimension ref="B3:J49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -12599,59 +12640,70 @@
         <v>767</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="27">
-        <v>1</v>
-      </c>
-      <c r="C4" s="21" t="s">
+      <c r="B4" s="22">
+        <v>1</v>
+      </c>
+      <c r="C4" s="31" t="s">
         <v>778</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19">
+      <c r="D4" s="27">
+        <v>1</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="F4" s="36">
+        <f>212518+208594</f>
+        <v>421112</v>
+      </c>
+      <c r="G4" s="36">
         <f>F4*D4</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="22" t="s">
-        <v>785</v>
-      </c>
-      <c r="J4" s="40">
+        <v>421112</v>
+      </c>
+      <c r="H4" s="27" t="s">
+        <v>784</v>
+      </c>
+      <c r="J4" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
         <v>118280</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="27">
+      <c r="B5" s="22">
         <v>2</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>780</v>
-      </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19">
+        <v>859</v>
+      </c>
+      <c r="D5" s="22">
+        <v>3</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50">
         <f>F5*D5</f>
         <v>0</v>
       </c>
       <c r="H5" s="22" t="s">
-        <v>449</v>
-      </c>
-      <c r="J5" s="40">
+        <v>784</v>
+      </c>
+      <c r="J5" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Piso",Tabela2[Preço Total])</f>
         <v>361131.5538461539</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="27">
+      <c r="B6" s="22">
         <v>3</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
@@ -12663,181 +12715,187 @@
       <c r="H6" s="22" t="s">
         <v>449</v>
       </c>
-      <c r="J6" s="40">
+      <c r="J6" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Pré Moldado",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="27">
+      <c r="B7" s="22">
         <v>4</v>
       </c>
-      <c r="C7" s="25" t="s">
-        <v>792</v>
-      </c>
-      <c r="D7" s="24">
-        <v>10</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26">
+      <c r="C7" s="21" t="s">
+        <v>837</v>
+      </c>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19">
         <f>F7*D7</f>
         <v>0</v>
       </c>
-      <c r="H7" s="24" t="s">
-        <v>643</v>
-      </c>
-      <c r="J7" s="40">
+      <c r="H7" s="22" t="s">
+        <v>449</v>
+      </c>
+      <c r="J7" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Fechamento Lateral",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="27">
+      <c r="B8" s="22">
         <v>5</v>
       </c>
-      <c r="C8" s="49" t="s">
-        <v>793</v>
-      </c>
-      <c r="D8" s="50">
+      <c r="C8" s="25" t="s">
+        <v>791</v>
+      </c>
+      <c r="D8" s="24">
+        <v>10</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26">
+        <f>F8*D8</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="24" t="s">
+        <v>643</v>
+      </c>
+      <c r="J8" s="39">
+        <f>SUMIF(Tabela2[Aplicação],"AVCB",Tabela2[Preço Total])</f>
+        <v>421112</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="22">
+        <v>6</v>
+      </c>
+      <c r="C9" s="47" t="s">
+        <v>792</v>
+      </c>
+      <c r="D9" s="48">
         <v>600</v>
       </c>
-      <c r="E8" s="50" t="s">
+      <c r="E9" s="48" t="s">
         <v>761</v>
       </c>
-      <c r="F8" s="51">
+      <c r="F9" s="49">
         <v>3.35</v>
       </c>
-      <c r="G8" s="51">
-        <f>F8*D8</f>
+      <c r="G9" s="49">
+        <f>F9*D9</f>
         <v>2010</v>
       </c>
-      <c r="H8" s="50" t="s">
+      <c r="H9" s="48" t="s">
         <v>643</v>
       </c>
-      <c r="J8" s="40">
-        <f>SUMIF(Tabela2[Aplicação],"AVCB",Tabela2[Preço Total])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="27">
-        <v>6</v>
-      </c>
-      <c r="C9" s="25" t="s">
-        <v>796</v>
-      </c>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26">
-        <f>F9*D9</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="24" t="s">
-        <v>799</v>
-      </c>
-      <c r="J9" s="40">
+      <c r="J9" s="39">
         <f>SUMIF(Tabela2[Aplicação],"SPDA",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="27">
+      <c r="B10" s="22">
         <v>7</v>
       </c>
-      <c r="C10" s="21" t="s">
-        <v>803</v>
-      </c>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19">
+      <c r="C10" s="31" t="s">
+        <v>847</v>
+      </c>
+      <c r="D10" s="27">
+        <v>1</v>
+      </c>
+      <c r="E10" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="F10" s="32">
+        <v>1056959.67</v>
+      </c>
+      <c r="G10" s="32">
         <f>F10*D10</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="22" t="s">
-        <v>776</v>
-      </c>
-      <c r="J10" s="40">
+        <v>1056959.67</v>
+      </c>
+      <c r="H10" s="27" t="s">
+        <v>846</v>
+      </c>
+      <c r="J10" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Terraplanagem",Tabela2[Preço Total])</f>
         <v>157963.5</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B11" s="27">
+      <c r="B11" s="22">
         <v>8</v>
       </c>
-      <c r="C11" s="21" t="s">
-        <v>801</v>
-      </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19">
+      <c r="C11" s="25" t="s">
+        <v>795</v>
+      </c>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26">
         <f>F11*D11</f>
         <v>0</v>
       </c>
-      <c r="H11" s="22" t="s">
-        <v>776</v>
-      </c>
-      <c r="J11" s="40">
+      <c r="H11" s="24" t="s">
+        <v>798</v>
+      </c>
+      <c r="J11" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Drenagem",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="27">
+      <c r="B12" s="22">
         <v>9</v>
       </c>
-      <c r="C12" s="25" t="s">
-        <v>782</v>
-      </c>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26">
+      <c r="C12" s="21" t="s">
+        <v>802</v>
+      </c>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19">
         <f>F12*D12</f>
         <v>0</v>
       </c>
-      <c r="H12" s="24" t="s">
+      <c r="H12" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="J12" s="40">
+      <c r="J12" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Elétrica",Tabela2[Preço Total])</f>
         <v>2010</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="27">
+      <c r="B13" s="22">
         <v>10</v>
       </c>
-      <c r="C13" s="25" t="s">
-        <v>783</v>
-      </c>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26">
+      <c r="C13" s="21" t="s">
+        <v>800</v>
+      </c>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19">
         <f>F13*D13</f>
         <v>0</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="H13" s="22" t="s">
         <v>776</v>
       </c>
-      <c r="J13" s="40">
+      <c r="J13" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Pintura",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="27">
+      <c r="B14" s="22">
         <v>11</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="D14" s="24"/>
       <c r="E14" s="24"/>
@@ -12849,17 +12907,17 @@
       <c r="H14" s="24" t="s">
         <v>776</v>
       </c>
-      <c r="J14" s="40">
+      <c r="J14" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Estrura Armazenamento",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B15" s="27">
+      <c r="B15" s="22">
         <v>12</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>844</v>
+        <v>782</v>
       </c>
       <c r="D15" s="24"/>
       <c r="E15" s="24"/>
@@ -12871,242 +12929,242 @@
       <c r="H15" s="24" t="s">
         <v>776</v>
       </c>
-      <c r="J15" s="40">
+      <c r="J15" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Serviço Prévio",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="27">
+      <c r="B16" s="22">
         <v>13</v>
       </c>
-      <c r="C16" s="28" t="s">
-        <v>800</v>
-      </c>
-      <c r="D16" s="29">
+      <c r="C16" s="25" t="s">
+        <v>783</v>
+      </c>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26">
+        <f>F16*D16</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>776</v>
+      </c>
+      <c r="J16" s="39"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="22">
+        <v>14</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>843</v>
+      </c>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26">
+        <f>F17*D17</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="22">
+        <v>15</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>799</v>
+      </c>
+      <c r="D18" s="29">
         <v>4</v>
       </c>
-      <c r="E16" s="29" t="s">
+      <c r="E18" s="29" t="s">
         <v>760</v>
       </c>
-      <c r="F16" s="30">
+      <c r="F18" s="30">
         <v>1500</v>
       </c>
-      <c r="G16" s="30">
+      <c r="G18" s="30">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>6000</v>
       </c>
-      <c r="H16" s="29" t="s">
+      <c r="H18" s="29" t="s">
         <v>771</v>
       </c>
-      <c r="J16" s="40"/>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="27">
-        <v>14</v>
-      </c>
-      <c r="C17" s="31" t="s">
-        <v>798</v>
-      </c>
-      <c r="D17" s="27">
-        <v>1</v>
-      </c>
-      <c r="E17" s="27" t="s">
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="22">
+        <v>16</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>797</v>
+      </c>
+      <c r="D19" s="27">
+        <v>1</v>
+      </c>
+      <c r="E19" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F17" s="32">
+      <c r="F19" s="32">
         <v>4500</v>
       </c>
-      <c r="G17" s="32">
-        <f>F17*D17</f>
+      <c r="G19" s="32">
+        <f>F19*D19</f>
         <v>4500</v>
       </c>
-      <c r="H17" s="27" t="s">
+      <c r="H19" s="27" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="27">
-        <v>15</v>
-      </c>
-      <c r="C18" s="18" t="s">
+      <c r="I19" s="14" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="22">
+        <v>17</v>
+      </c>
+      <c r="C20" s="18" t="s">
         <v>769</v>
       </c>
-      <c r="D18" s="17">
+      <c r="D20" s="17">
         <v>2100</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E20" s="17" t="s">
+        <v>841</v>
+      </c>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20">
+        <f>F20*D20</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="I20" s="14" t="s">
         <v>842</v>
       </c>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20">
-        <f>F18*D18</f>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="22">
+        <v>18</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>770</v>
+      </c>
+      <c r="D21" s="17">
+        <v>2300</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>841</v>
+      </c>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20">
+        <f>F21*D21</f>
         <v>0</v>
       </c>
-      <c r="H18" s="17" t="s">
+      <c r="H21" s="17" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="27">
-        <v>16</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>770</v>
-      </c>
-      <c r="D19" s="17">
-        <v>2300</v>
-      </c>
-      <c r="E19" s="17" t="s">
-        <v>842</v>
-      </c>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20">
-        <f>F19*D19</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="17" t="s">
-        <v>771</v>
-      </c>
-      <c r="I19" s="14" t="s">
-        <v>843</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="27">
-        <v>17</v>
-      </c>
-      <c r="C20" s="31" t="s">
-        <v>839</v>
-      </c>
-      <c r="D20" s="27">
-        <v>1</v>
-      </c>
-      <c r="E20" s="27" t="s">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B22" s="22">
+        <v>19</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>838</v>
+      </c>
+      <c r="D22" s="27">
+        <v>1</v>
+      </c>
+      <c r="E22" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F20" s="32">
+      <c r="F22" s="32">
         <v>51500</v>
-      </c>
-      <c r="G20" s="32">
-        <f>F20*D20</f>
-        <v>51500</v>
-      </c>
-      <c r="H20" s="27" t="s">
-        <v>771</v>
-      </c>
-      <c r="I20" s="14" t="s">
-        <v>843</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="27">
-        <v>19</v>
-      </c>
-      <c r="C21" s="31" t="s">
-        <v>840</v>
-      </c>
-      <c r="D21" s="33">
-        <v>46.8</v>
-      </c>
-      <c r="E21" s="27" t="s">
-        <v>759</v>
-      </c>
-      <c r="F21" s="32">
-        <v>670</v>
-      </c>
-      <c r="G21" s="32">
-        <f>F21*D21</f>
-        <v>31355.999999999996</v>
-      </c>
-      <c r="H21" s="27" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="27">
-        <v>20</v>
-      </c>
-      <c r="C22" s="31" t="s">
-        <v>841</v>
-      </c>
-      <c r="D22" s="33">
-        <v>37.200000000000003</v>
-      </c>
-      <c r="E22" s="27" t="s">
-        <v>759</v>
-      </c>
-      <c r="F22" s="32">
-        <v>670</v>
       </c>
       <c r="G22" s="32">
         <f>F22*D22</f>
-        <v>24924.000000000004</v>
+        <v>51500</v>
       </c>
       <c r="H22" s="27" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="27">
+      <c r="B23" s="22">
+        <v>20</v>
+      </c>
+      <c r="C23" s="31" t="s">
+        <v>839</v>
+      </c>
+      <c r="D23" s="33">
+        <v>46.8</v>
+      </c>
+      <c r="E23" s="27" t="s">
+        <v>759</v>
+      </c>
+      <c r="F23" s="32">
+        <v>670</v>
+      </c>
+      <c r="G23" s="32">
+        <f>F23*D23</f>
+        <v>31355.999999999996</v>
+      </c>
+      <c r="H23" s="27" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="22">
+        <v>21</v>
+      </c>
+      <c r="C24" s="31" t="s">
+        <v>840</v>
+      </c>
+      <c r="D24" s="33">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E24" s="27" t="s">
+        <v>759</v>
+      </c>
+      <c r="F24" s="32">
+        <v>670</v>
+      </c>
+      <c r="G24" s="32">
+        <f>F24*D24</f>
+        <v>24924.000000000004</v>
+      </c>
+      <c r="H24" s="27" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="22">
         <v>22</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="C25" s="21" t="s">
         <v>779</v>
       </c>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19">
-        <f>F23*D23</f>
-        <v>0</v>
-      </c>
-      <c r="H23" s="22" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="27">
-        <v>23</v>
-      </c>
-      <c r="C24" s="25" t="s">
-        <v>788</v>
-      </c>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="26">
-        <f>F24*D24</f>
-        <v>0</v>
-      </c>
-      <c r="H24" s="24" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="27">
-        <v>24</v>
-      </c>
-      <c r="C25" s="25" t="s">
-        <v>789</v>
-      </c>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26">
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19">
         <f>F25*D25</f>
         <v>0</v>
       </c>
-      <c r="H25" s="24" t="s">
-        <v>576</v>
+      <c r="H25" s="22" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="27">
-        <v>25</v>
+      <c r="B26" s="22">
+        <v>23</v>
       </c>
       <c r="C26" s="25" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="D26" s="24"/>
       <c r="E26" s="24"/>
@@ -13120,11 +13178,11 @@
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B27" s="27">
-        <v>26</v>
+      <c r="B27" s="22">
+        <v>24</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="24"/>
@@ -13138,203 +13196,193 @@
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B28" s="27">
+      <c r="B28" s="22">
+        <v>25</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>789</v>
+      </c>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26">
+        <f>F28*D28</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="24" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29" s="22">
+        <v>26</v>
+      </c>
+      <c r="C29" s="25" t="s">
+        <v>790</v>
+      </c>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26">
+        <f>F29*D29</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="24" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B30" s="22">
         <v>27</v>
       </c>
-      <c r="C28" s="31" t="s">
+      <c r="C30" s="31" t="s">
         <v>757</v>
       </c>
-      <c r="D28" s="27">
+      <c r="D30" s="27">
         <f>(2000*1.05)*0.15</f>
         <v>315</v>
       </c>
-      <c r="E28" s="27" t="s">
+      <c r="E30" s="27" t="s">
         <v>759</v>
       </c>
-      <c r="F28" s="32">
+      <c r="F30" s="32">
         <v>670</v>
       </c>
-      <c r="G28" s="32">
-        <f>F28*D28</f>
+      <c r="G30" s="32">
+        <f>F30*D30</f>
         <v>211050</v>
       </c>
-      <c r="H28" s="27" t="s">
+      <c r="H30" s="27" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B29" s="27">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B31" s="22">
         <v>28</v>
       </c>
-      <c r="C29" s="31" t="s">
+      <c r="C31" s="31" t="s">
         <v>777</v>
       </c>
-      <c r="D29" s="33">
+      <c r="D31" s="33">
         <f>2000/13*2</f>
         <v>307.69230769230768</v>
       </c>
-      <c r="E29" s="27" t="s">
+      <c r="E31" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F29" s="32">
+      <c r="F31" s="32">
         <v>220.5</v>
-      </c>
-      <c r="G29" s="32">
-        <f>F29*D29</f>
-        <v>67846.153846153844</v>
-      </c>
-      <c r="H29" s="27" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B30" s="27">
-        <v>29</v>
-      </c>
-      <c r="C30" s="31" t="s">
-        <v>758</v>
-      </c>
-      <c r="D30" s="27">
-        <v>167</v>
-      </c>
-      <c r="E30" s="27" t="s">
-        <v>814</v>
-      </c>
-      <c r="F30" s="32">
-        <v>56.2</v>
-      </c>
-      <c r="G30" s="32">
-        <f>F30*D30</f>
-        <v>9385.4</v>
-      </c>
-      <c r="H30" s="27" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B31" s="27">
-        <v>30</v>
-      </c>
-      <c r="C31" s="31" t="s">
-        <v>762</v>
-      </c>
-      <c r="D31" s="27">
-        <v>1000</v>
-      </c>
-      <c r="E31" s="27" t="s">
-        <v>763</v>
-      </c>
-      <c r="F31" s="32">
-        <v>7.3</v>
       </c>
       <c r="G31" s="32">
         <f>F31*D31</f>
-        <v>7300</v>
+        <v>67846.153846153844</v>
       </c>
       <c r="H31" s="27" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B32" s="27">
-        <v>31</v>
+      <c r="B32" s="22">
+        <v>29</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>804</v>
+        <v>758</v>
       </c>
       <c r="D32" s="27">
-        <v>315</v>
+        <v>167</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>759</v>
+        <v>813</v>
       </c>
       <c r="F32" s="32">
-        <v>50</v>
+        <v>56.2</v>
       </c>
       <c r="G32" s="32">
         <f>F32*D32</f>
-        <v>15750</v>
+        <v>9385.4</v>
       </c>
       <c r="H32" s="27" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B33" s="27">
-        <v>32</v>
+      <c r="B33" s="22">
+        <v>30</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>768</v>
+        <v>762</v>
       </c>
       <c r="D33" s="27">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="E33" s="27" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="F33" s="32">
-        <v>49800</v>
+        <v>7.3</v>
       </c>
       <c r="G33" s="32">
         <f>F33*D33</f>
-        <v>49800</v>
+        <v>7300</v>
       </c>
       <c r="H33" s="27" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="27">
-        <v>33</v>
+      <c r="B34" s="22">
+        <v>31</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>848</v>
+        <v>803</v>
       </c>
       <c r="D34" s="27">
-        <v>1</v>
+        <v>315</v>
       </c>
       <c r="E34" s="27" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="F34" s="32">
-        <v>1056959.67</v>
+        <v>50</v>
       </c>
       <c r="G34" s="32">
         <f>F34*D34</f>
-        <v>1056959.67</v>
+        <v>15750</v>
       </c>
       <c r="H34" s="27" t="s">
-        <v>847</v>
+        <v>635</v>
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="27">
-        <v>34</v>
-      </c>
-      <c r="C35" s="25" t="s">
-        <v>806</v>
-      </c>
-      <c r="D35" s="24">
-        <v>1</v>
-      </c>
-      <c r="E35" s="24" t="s">
+      <c r="B35" s="22">
+        <v>32</v>
+      </c>
+      <c r="C35" s="31" t="s">
+        <v>768</v>
+      </c>
+      <c r="D35" s="27">
+        <v>1</v>
+      </c>
+      <c r="E35" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26">
+      <c r="F35" s="32">
+        <v>49800</v>
+      </c>
+      <c r="G35" s="32">
         <f>F35*D35</f>
-        <v>0</v>
-      </c>
-      <c r="H35" s="24" t="s">
-        <v>807</v>
+        <v>49800</v>
+      </c>
+      <c r="H35" s="27" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B36" s="27">
-        <v>35</v>
+      <c r="B36" s="22">
+        <v>33</v>
       </c>
       <c r="C36" s="25" t="s">
-        <v>819</v>
+        <v>805</v>
       </c>
       <c r="D36" s="24">
         <v>1</v>
@@ -13348,175 +13396,175 @@
         <v>0</v>
       </c>
       <c r="H36" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B37" s="27">
-        <v>36</v>
-      </c>
-      <c r="C37" s="21" t="s">
-        <v>794</v>
-      </c>
-      <c r="D37" s="22"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19">
+      <c r="B37" s="22">
+        <v>34</v>
+      </c>
+      <c r="C37" s="25" t="s">
+        <v>818</v>
+      </c>
+      <c r="D37" s="24">
+        <v>1</v>
+      </c>
+      <c r="E37" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="F37" s="26"/>
+      <c r="G37" s="26">
         <f>F37*D37</f>
         <v>0</v>
       </c>
-      <c r="H37" s="22" t="s">
+      <c r="H37" s="24" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B38" s="22">
+        <v>35</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>793</v>
+      </c>
+      <c r="D38" s="22"/>
+      <c r="E38" s="22"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19">
+        <f>F38*D38</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="22" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B38" s="27">
-        <v>37</v>
-      </c>
-      <c r="C38" s="48" t="s">
-        <v>849</v>
-      </c>
-      <c r="D38" s="27">
+    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B39" s="22">
+        <v>36</v>
+      </c>
+      <c r="C39" s="46" t="s">
+        <v>848</v>
+      </c>
+      <c r="D39" s="27">
         <v>1455.89</v>
       </c>
-      <c r="E38" s="27" t="s">
+      <c r="E39" s="27" t="s">
         <v>761</v>
       </c>
-      <c r="F38" s="36">
+      <c r="F39" s="36">
         <v>95.9</v>
       </c>
-      <c r="G38" s="36">
+      <c r="G39" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>139619.85100000002</v>
       </c>
-      <c r="H38" s="27" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B39" s="27">
-        <v>38</v>
-      </c>
-      <c r="C39" s="31" t="s">
-        <v>850</v>
-      </c>
-      <c r="D39" s="27">
+      <c r="H39" s="27" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B40" s="22">
+        <v>37</v>
+      </c>
+      <c r="C40" s="31" t="s">
+        <v>849</v>
+      </c>
+      <c r="D40" s="27">
         <v>706.94</v>
       </c>
-      <c r="E39" s="27" t="s">
+      <c r="E40" s="27" t="s">
         <v>761</v>
       </c>
-      <c r="F39" s="36">
+      <c r="F40" s="36">
         <v>95.9</v>
       </c>
-      <c r="G39" s="36">
+      <c r="G40" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>67795.546000000002</v>
       </c>
-      <c r="H39" s="27" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B40" s="27">
-        <v>39</v>
-      </c>
-      <c r="C40" t="s">
-        <v>851</v>
-      </c>
-      <c r="D40" s="27">
+      <c r="H40" s="27" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B41" s="22">
+        <v>38</v>
+      </c>
+      <c r="C41" t="s">
+        <v>850</v>
+      </c>
+      <c r="D41" s="27">
         <v>44</v>
       </c>
-      <c r="E40" s="27" t="s">
-        <v>855</v>
-      </c>
-      <c r="F40" s="36">
+      <c r="E41" s="27" t="s">
+        <v>854</v>
+      </c>
+      <c r="F41" s="36">
         <v>95</v>
       </c>
-      <c r="G40" s="36">
+      <c r="G41" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>4180</v>
       </c>
-      <c r="H40" s="27" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B41" s="27">
-        <v>40</v>
-      </c>
-      <c r="C41" t="s">
-        <v>852</v>
-      </c>
-      <c r="D41" s="27">
+      <c r="H41" s="27" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B42" s="22">
+        <v>39</v>
+      </c>
+      <c r="C42" t="s">
+        <v>851</v>
+      </c>
+      <c r="D42" s="27">
         <v>3</v>
       </c>
-      <c r="E41" s="27" t="s">
-        <v>855</v>
-      </c>
-      <c r="F41" s="36">
+      <c r="E42" s="27" t="s">
+        <v>854</v>
+      </c>
+      <c r="F42" s="36">
         <v>35</v>
       </c>
-      <c r="G41" s="36">
+      <c r="G42" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>105</v>
       </c>
-      <c r="H41" s="27" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B42" s="27">
-        <v>41</v>
-      </c>
-      <c r="C42" t="s">
-        <v>853</v>
-      </c>
-      <c r="D42" s="27">
+      <c r="H42" s="27" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B43" s="22">
+        <v>40</v>
+      </c>
+      <c r="C43" t="s">
+        <v>852</v>
+      </c>
+      <c r="D43" s="27">
         <v>126</v>
       </c>
-      <c r="E42" s="27" t="s">
+      <c r="E43" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F42" s="36">
+      <c r="F43" s="36">
         <v>25.9</v>
       </c>
-      <c r="G42" s="36">
+      <c r="G43" s="36">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>3263.3999999999996</v>
       </c>
-      <c r="H42" s="27" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B43" s="27"/>
-      <c r="C43" t="s">
-        <v>854</v>
-      </c>
-      <c r="D43" s="27">
-        <v>1</v>
-      </c>
-      <c r="E43" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="F43" s="36">
-        <v>1750</v>
-      </c>
-      <c r="G43" s="36">
-        <f>F43*D43</f>
-        <v>1750</v>
-      </c>
       <c r="H43" s="27" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B44" s="27">
-        <v>42</v>
-      </c>
-      <c r="C44" s="31" t="s">
-        <v>787</v>
+      <c r="B44" s="22">
+        <v>41</v>
+      </c>
+      <c r="C44" t="s">
+        <v>853</v>
       </c>
       <c r="D44" s="27">
         <v>1</v>
@@ -13525,40 +13573,57 @@
         <v>760</v>
       </c>
       <c r="F44" s="36">
-        <v>157963.5</v>
+        <v>1750</v>
       </c>
       <c r="G44" s="36">
         <f>F44*D44</f>
+        <v>1750</v>
+      </c>
+      <c r="H44" s="27" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B45" s="22">
+        <v>42</v>
+      </c>
+      <c r="C45" s="31" t="s">
+        <v>786</v>
+      </c>
+      <c r="D45" s="27">
+        <v>1</v>
+      </c>
+      <c r="E45" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="F45" s="36">
         <v>157963.5</v>
       </c>
-      <c r="H44" s="27" t="s">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B45" s="27"/>
-      <c r="C45" s="25" t="s">
-        <v>845</v>
-      </c>
-      <c r="D45" s="24"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="26">
+      <c r="G45" s="36">
         <f>F45*D45</f>
-        <v>0</v>
-      </c>
-      <c r="H45" s="24" t="s">
-        <v>846</v>
+        <v>157963.5</v>
+      </c>
+      <c r="H45" s="27" t="s">
+        <v>785</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B46" s="24"/>
-      <c r="C46" s="25"/>
+      <c r="B46" s="22">
+        <v>43</v>
+      </c>
+      <c r="C46" s="25" t="s">
+        <v>844</v>
+      </c>
       <c r="D46" s="24"/>
       <c r="E46" s="24"/>
       <c r="F46" s="26"/>
-      <c r="G46" s="26"/>
-      <c r="H46" s="24"/>
+      <c r="G46" s="26">
+        <f>F46*D46</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="24" t="s">
+        <v>845</v>
+      </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" s="24"/>
@@ -13570,9 +13635,18 @@
       <c r="H47" s="24"/>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="G48" s="16">
+      <c r="B48" s="24"/>
+      <c r="C48" s="25"/>
+      <c r="D48" s="24"/>
+      <c r="E48" s="24"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="26"/>
+      <c r="H48" s="24"/>
+    </row>
+    <row r="49" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G49" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>1913058.5208461538</v>
+        <v>2334170.5208461536</v>
       </c>
     </row>
   </sheetData>
@@ -13586,12 +13660,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R51"/>
+  <dimension ref="B1:R58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
     <col min="3" max="3" width="20" style="14" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="63.85546875" customWidth="1"/>
+    <col min="4" max="4" width="87" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" style="14" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" style="14" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" style="15" customWidth="1"/>
@@ -13607,12 +13681,12 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P1" s="14" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P2" s="14" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="3" spans="2:18" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -13620,7 +13694,7 @@
         <v>753</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="D3" t="s">
         <v>754</v>
@@ -13641,792 +13715,835 @@
         <v>767</v>
       </c>
       <c r="P3" s="14" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B4" s="17">
+      <c r="B4" s="22">
         <v>1</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E4" s="24"/>
       <c r="F4" s="24"/>
       <c r="G4" s="26"/>
       <c r="H4" s="26">
-        <f t="shared" ref="H4:H48" si="0">G4*E4</f>
+        <f>G4*E4</f>
         <v>0</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="O4" s="14" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="P4" s="14" t="s">
+        <v>825</v>
+      </c>
+      <c r="Q4" s="14" t="s">
         <v>826</v>
       </c>
-      <c r="Q4" s="14" t="s">
+      <c r="R4" s="14" t="s">
         <v>827</v>
       </c>
-      <c r="R4" s="14" t="s">
+    </row>
+    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B5" s="22">
+        <v>2</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>809</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>856</v>
+      </c>
+      <c r="E5" s="27">
+        <v>1</v>
+      </c>
+      <c r="F5" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="G5" s="36">
+        <v>486032</v>
+      </c>
+      <c r="H5" s="36">
+        <f>G5*E5</f>
+        <v>486032</v>
+      </c>
+      <c r="I5" s="27" t="s">
+        <v>784</v>
+      </c>
+      <c r="N5" s="37" t="s">
+        <v>772</v>
+      </c>
+      <c r="O5" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Pré Moldado",Tabela24[Preço Total])</f>
+        <v>992504</v>
+      </c>
+      <c r="P5" s="43">
+        <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
+        <v>0.27774553181958522</v>
+      </c>
+      <c r="Q5" s="45">
+        <f>P5</f>
+        <v>0.27774553181958522</v>
+      </c>
+      <c r="R5" t="s">
         <v>828</v>
       </c>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B5" s="17">
-        <v>2</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>778</v>
-      </c>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19">
+    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B6" s="22">
+        <v>3</v>
+      </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="21" t="s">
+        <v>858</v>
+      </c>
+      <c r="E6" s="22">
+        <v>4</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19">
+        <f>G6*E6</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>784</v>
+      </c>
+      <c r="N6" s="44" t="s">
+        <v>785</v>
+      </c>
+      <c r="O6" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Terraplanagem",Tabela24[Preço Total])</f>
+        <v>791792.51</v>
+      </c>
+      <c r="P6" s="43">
+        <f t="shared" si="0"/>
+        <v>0.22157777881067911</v>
+      </c>
+      <c r="Q6" s="45">
+        <f>P6+Q5</f>
+        <v>0.49932331063026436</v>
+      </c>
+      <c r="R6" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B7" s="22">
+        <v>4</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>860</v>
+      </c>
+      <c r="E7" s="27">
+        <v>1</v>
+      </c>
+      <c r="F7" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="G7" s="36">
+        <v>24500</v>
+      </c>
+      <c r="H7" s="36">
+        <f>G7*E7</f>
+        <v>24500</v>
+      </c>
+      <c r="I7" s="27" t="s">
+        <v>772</v>
+      </c>
+      <c r="N7" s="37" t="s">
+        <v>635</v>
+      </c>
+      <c r="O7" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Piso",Tabela24[Preço Total])</f>
+        <v>645545.6</v>
+      </c>
+      <c r="P7" s="43">
+        <f t="shared" si="0"/>
+        <v>0.1806515701556802</v>
+      </c>
+    </row>
+    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B8" s="22">
+        <v>5</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>837</v>
+      </c>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19">
+        <f>G8*E8</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="22" t="s">
+        <v>772</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>814</v>
+      </c>
+      <c r="N8" s="44" t="s">
+        <v>806</v>
+      </c>
+      <c r="O8" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
+        <v>358477</v>
+      </c>
+      <c r="P8" s="43">
+        <f t="shared" si="0"/>
+        <v>0.10031736397041166</v>
+      </c>
+    </row>
+    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B9" s="22">
+        <v>6</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>791</v>
+      </c>
+      <c r="E9" s="24">
+        <v>26</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26">
+        <f>G9*E9</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="24" t="s">
+        <v>643</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>812</v>
+      </c>
+      <c r="N9" s="41" t="s">
+        <v>771</v>
+      </c>
+      <c r="O9" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Fundação",Tabela24[Preço Total])</f>
+        <v>164000</v>
+      </c>
+      <c r="P9" s="43">
+        <f t="shared" si="0"/>
+        <v>4.5894290822416813E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B10" s="22">
+        <v>7</v>
+      </c>
+      <c r="C10" s="27" t="s">
+        <v>809</v>
+      </c>
+      <c r="D10" s="47" t="s">
+        <v>792</v>
+      </c>
+      <c r="E10" s="48">
+        <v>600</v>
+      </c>
+      <c r="F10" s="48" t="s">
+        <v>761</v>
+      </c>
+      <c r="G10" s="49">
+        <v>3.35</v>
+      </c>
+      <c r="H10" s="49">
+        <f>G10*E10</f>
+        <v>2010</v>
+      </c>
+      <c r="I10" s="48" t="s">
+        <v>643</v>
+      </c>
+      <c r="N10" s="41" t="s">
+        <v>776</v>
+      </c>
+      <c r="O10" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
+        <v>66534.056568800006</v>
+      </c>
+      <c r="P10" s="43">
+        <f t="shared" si="0"/>
+        <v>1.8619105742461214E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B11" s="22">
+        <v>8</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>816</v>
+      </c>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26">
+        <f>G11*E11</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="24" t="s">
+        <v>643</v>
+      </c>
+      <c r="N11" s="40" t="s">
+        <v>784</v>
+      </c>
+      <c r="O11" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"AVCB",Tabela24[Preço Total])</f>
+        <v>486032</v>
+      </c>
+      <c r="P11" s="43">
+        <f t="shared" si="0"/>
+        <v>0.13601276803049323</v>
+      </c>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B12" s="22">
+        <v>9</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>834</v>
+      </c>
+      <c r="E12" s="27">
+        <v>54</v>
+      </c>
+      <c r="F12" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="G12" s="36">
+        <v>243.39</v>
+      </c>
+      <c r="H12" s="36">
+        <f>G12*E12</f>
+        <v>13143.06</v>
+      </c>
+      <c r="I12" s="27" t="s">
+        <v>835</v>
+      </c>
+      <c r="N12" s="40" t="s">
+        <v>449</v>
+      </c>
+      <c r="O12" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Drenagem",Tabela24[Preço Total])</f>
+        <v>0</v>
+      </c>
+      <c r="P12" s="43">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I5" s="22" t="s">
-        <v>785</v>
-      </c>
-      <c r="N5" s="37" t="s">
-        <v>772</v>
-      </c>
-      <c r="O5" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Pré Moldado",Tabela24[Preço Total])</f>
-        <v>968004</v>
-      </c>
-      <c r="P5" s="44">
-        <f t="shared" ref="P5:P17" si="1">O5/$O$21</f>
-        <v>0.33062288469044115</v>
-      </c>
-      <c r="Q5" s="46">
-        <f>P5</f>
-        <v>0.33062288469044115</v>
-      </c>
-      <c r="R5" t="s">
-        <v>829</v>
-      </c>
-    </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B6" s="17">
-        <v>3</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>780</v>
-      </c>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19">
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B13" s="22">
+        <v>10</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D13" s="31" t="s">
+        <v>836</v>
+      </c>
+      <c r="E13" s="27">
+        <v>30</v>
+      </c>
+      <c r="F13" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="G13" s="36">
+        <v>119.7</v>
+      </c>
+      <c r="H13" s="36">
+        <f>G13*E13</f>
+        <v>3591</v>
+      </c>
+      <c r="I13" s="27" t="s">
+        <v>835</v>
+      </c>
+      <c r="N13" s="40"/>
+      <c r="O13" s="39"/>
+      <c r="P13" s="43"/>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B14" s="22">
+        <v>11</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>809</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>833</v>
+      </c>
+      <c r="E14" s="48">
+        <v>390</v>
+      </c>
+      <c r="F14" s="27" t="s">
+        <v>761</v>
+      </c>
+      <c r="G14" s="36">
+        <v>38.116666600000002</v>
+      </c>
+      <c r="H14" s="36">
+        <f>G14*E14</f>
+        <v>14865.499974</v>
+      </c>
+      <c r="I14" s="27" t="s">
+        <v>835</v>
+      </c>
+      <c r="N14" s="40" t="s">
+        <v>776</v>
+      </c>
+      <c r="O14" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
+        <v>66534.056568800006</v>
+      </c>
+      <c r="P14" s="43">
+        <f t="shared" si="0"/>
+        <v>1.8619105742461214E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B15" s="22">
+        <v>12</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D15" s="31" t="s">
+        <v>834</v>
+      </c>
+      <c r="E15" s="33">
+        <f>(84*1.02)*2*1.02</f>
+        <v>174.78720000000001</v>
+      </c>
+      <c r="F15" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="G15" s="36">
+        <v>243.39</v>
+      </c>
+      <c r="H15" s="36">
+        <f>G15*E15</f>
+        <v>42541.456608</v>
+      </c>
+      <c r="I15" s="27" t="s">
+        <v>776</v>
+      </c>
+      <c r="N15" s="40" t="s">
+        <v>643</v>
+      </c>
+      <c r="O15" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Elétrica",Tabela24[Preço Total])</f>
+        <v>2010</v>
+      </c>
+      <c r="P15" s="43">
+        <f t="shared" si="0"/>
+        <v>5.6248490581132799E-4</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B16" s="22">
+        <v>13</v>
+      </c>
+      <c r="C16" s="27" t="s">
+        <v>809</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>833</v>
+      </c>
+      <c r="E16" s="27">
+        <f>84*7</f>
+        <v>588</v>
+      </c>
+      <c r="F16" s="27" t="s">
+        <v>761</v>
+      </c>
+      <c r="G16" s="36">
+        <v>38.116666600000002</v>
+      </c>
+      <c r="H16" s="36">
+        <f>G16*E16</f>
+        <v>22412.599960800002</v>
+      </c>
+      <c r="I16" s="27" t="s">
+        <v>776</v>
+      </c>
+      <c r="N16" s="40"/>
+      <c r="O16" s="39"/>
+      <c r="P16" s="43"/>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B17" s="22">
+        <v>14</v>
+      </c>
+      <c r="C17" s="27"/>
+      <c r="D17" s="31" t="s">
+        <v>861</v>
+      </c>
+      <c r="E17" s="27">
+        <v>30</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>854</v>
+      </c>
+      <c r="G17" s="36">
+        <v>24</v>
+      </c>
+      <c r="H17" s="36">
+        <f>G17*E17</f>
+        <v>720</v>
+      </c>
+      <c r="I17" s="27" t="s">
+        <v>776</v>
+      </c>
+      <c r="N17" s="40"/>
+      <c r="O17" s="39"/>
+      <c r="P17" s="43"/>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B18" s="22">
+        <v>15</v>
+      </c>
+      <c r="C18" s="27"/>
+      <c r="D18" s="31" t="s">
+        <v>862</v>
+      </c>
+      <c r="E18" s="27">
+        <v>1</v>
+      </c>
+      <c r="F18" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="G18" s="36">
+        <v>860</v>
+      </c>
+      <c r="H18" s="36">
+        <f>G18*E18</f>
+        <v>860</v>
+      </c>
+      <c r="I18" s="27" t="s">
+        <v>776</v>
+      </c>
+      <c r="N18" s="40"/>
+      <c r="O18" s="39"/>
+      <c r="P18" s="43"/>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B19" s="22">
+        <v>16</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>781</v>
+      </c>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24" t="s">
+        <v>761</v>
+      </c>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26">
+        <f>G19*E19</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="24" t="s">
+        <v>776</v>
+      </c>
+      <c r="N19" s="40" t="s">
+        <v>576</v>
+      </c>
+      <c r="O19" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Pintura",Tabela24[Preço Total])</f>
+        <v>0</v>
+      </c>
+      <c r="P19" s="43">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I6" s="22" t="s">
-        <v>449</v>
-      </c>
-      <c r="N6" s="45" t="s">
-        <v>786</v>
-      </c>
-      <c r="O6" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Terraplanagem",Tabela24[Preço Total])</f>
-        <v>791792.51</v>
-      </c>
-      <c r="P6" s="44">
-        <f t="shared" si="1"/>
-        <v>0.27043764667551473</v>
-      </c>
-      <c r="Q6" s="46">
-        <f>P6+Q5</f>
-        <v>0.60106053136595583</v>
-      </c>
-      <c r="R6" t="s">
-        <v>829</v>
-      </c>
-    </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B7" s="17">
-        <v>4</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>838</v>
-      </c>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19">
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B20" s="22">
+        <v>17</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>782</v>
+      </c>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26">
+        <f>G20*E20</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="24" t="s">
+        <v>776</v>
+      </c>
+      <c r="N20" s="40" t="s">
+        <v>817</v>
+      </c>
+      <c r="O20" s="39">
+        <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
+        <v>0</v>
+      </c>
+      <c r="P20" s="43">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I7" s="22" t="s">
-        <v>449</v>
-      </c>
-      <c r="N7" s="37" t="s">
-        <v>635</v>
-      </c>
-      <c r="O7" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Piso",Tabela24[Preço Total])</f>
-        <v>645545.6</v>
-      </c>
-      <c r="P7" s="44">
-        <f t="shared" si="1"/>
-        <v>0.22048684558247864</v>
-      </c>
-    </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B8" s="17">
-        <v>5</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D8" s="25" t="s">
-        <v>792</v>
-      </c>
-      <c r="E8" s="24">
-        <v>26</v>
-      </c>
-      <c r="F8" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26">
-        <f t="shared" si="0"/>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B21" s="22">
+        <v>18</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>783</v>
+      </c>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26">
+        <f>G21*E21</f>
         <v>0</v>
       </c>
-      <c r="I8" s="24" t="s">
-        <v>643</v>
-      </c>
-      <c r="J8" s="14" t="s">
-        <v>815</v>
-      </c>
-      <c r="N8" s="45" t="s">
-        <v>807</v>
-      </c>
-      <c r="O8" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
-        <v>358477</v>
-      </c>
-      <c r="P8" s="44">
-        <f t="shared" si="1"/>
-        <v>0.12243823355603414</v>
-      </c>
-    </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B9" s="17">
-        <v>6</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D9" s="25" t="s">
-        <v>793</v>
-      </c>
-      <c r="E9" s="24">
-        <v>500</v>
-      </c>
-      <c r="F9" s="24" t="s">
-        <v>761</v>
-      </c>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26">
-        <f t="shared" si="0"/>
+      <c r="I21" s="24" t="s">
+        <v>776</v>
+      </c>
+      <c r="N21" s="40"/>
+      <c r="O21" s="39"/>
+      <c r="P21" s="43"/>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B22" s="22">
+        <v>19</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>821</v>
+      </c>
+      <c r="E22" s="24">
+        <v>1</v>
+      </c>
+      <c r="F22" s="24"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26">
+        <f>G22*E22</f>
         <v>0</v>
       </c>
-      <c r="I9" s="24" t="s">
-        <v>643</v>
-      </c>
-      <c r="J9" s="14" t="s">
-        <v>813</v>
-      </c>
-      <c r="N9" s="42" t="s">
-        <v>771</v>
-      </c>
-      <c r="O9" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Fundação",Tabela24[Preço Total])</f>
-        <v>164000</v>
-      </c>
-      <c r="P9" s="44">
-        <f t="shared" si="1"/>
-        <v>5.6014389495531371E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B10" s="17">
-        <v>7</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D10" s="25" t="s">
-        <v>817</v>
-      </c>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26">
-        <f t="shared" si="0"/>
+      <c r="I22" s="24" t="s">
+        <v>776</v>
+      </c>
+      <c r="N22" s="40"/>
+      <c r="O22" s="39"/>
+      <c r="P22" s="43"/>
+    </row>
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B23" s="22">
+        <v>20</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>796</v>
+      </c>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="20">
+        <f>G23*E23</f>
         <v>0</v>
-      </c>
-      <c r="I10" s="24" t="s">
-        <v>643</v>
-      </c>
-      <c r="N10" s="42" t="s">
-        <v>776</v>
-      </c>
-      <c r="O10" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
-        <v>0</v>
-      </c>
-      <c r="P10" s="44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B11" s="17">
-        <v>8</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>835</v>
-      </c>
-      <c r="E11" s="22">
-        <v>54</v>
-      </c>
-      <c r="F11" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I11" s="22" t="s">
-        <v>836</v>
-      </c>
-      <c r="N11" s="41" t="s">
-        <v>785</v>
-      </c>
-      <c r="O11" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"AVCB",Tabela24[Preço Total])</f>
-        <v>0</v>
-      </c>
-      <c r="P11" s="44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B12" s="17">
-        <v>9</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D12" s="21" t="s">
-        <v>837</v>
-      </c>
-      <c r="E12" s="22">
-        <v>30</v>
-      </c>
-      <c r="F12" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I12" s="22" t="s">
-        <v>836</v>
-      </c>
-      <c r="N12" s="41" t="s">
-        <v>449</v>
-      </c>
-      <c r="O12" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Drenagem",Tabela24[Preço Total])</f>
-        <v>0</v>
-      </c>
-      <c r="P12" s="44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B13" s="17">
-        <v>10</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>834</v>
-      </c>
-      <c r="E13" s="24">
-        <v>390</v>
-      </c>
-      <c r="F13" s="22" t="s">
-        <v>761</v>
-      </c>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I13" s="22" t="s">
-        <v>836</v>
-      </c>
-      <c r="N13" s="41"/>
-      <c r="O13" s="40"/>
-      <c r="P13" s="44"/>
-    </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B14" s="17">
-        <v>11</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>835</v>
-      </c>
-      <c r="E14" s="47">
-        <f>(84*1.02)*2*1.02</f>
-        <v>174.78720000000001</v>
-      </c>
-      <c r="F14" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G14" s="19"/>
-      <c r="H14" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I14" s="22" t="s">
-        <v>776</v>
-      </c>
-      <c r="N14" s="41" t="s">
-        <v>776</v>
-      </c>
-      <c r="O14" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
-        <v>0</v>
-      </c>
-      <c r="P14" s="44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B15" s="17">
-        <v>12</v>
-      </c>
-      <c r="C15" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>834</v>
-      </c>
-      <c r="E15" s="22">
-        <f>84*7</f>
-        <v>588</v>
-      </c>
-      <c r="F15" s="22" t="s">
-        <v>761</v>
-      </c>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I15" s="22" t="s">
-        <v>776</v>
-      </c>
-      <c r="N15" s="41" t="s">
-        <v>643</v>
-      </c>
-      <c r="O15" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Elétrica",Tabela24[Preço Total])</f>
-        <v>0</v>
-      </c>
-      <c r="P15" s="44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B16" s="17">
-        <v>13</v>
-      </c>
-      <c r="C16" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D16" s="25" t="s">
-        <v>782</v>
-      </c>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24" t="s">
-        <v>761</v>
-      </c>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I16" s="24" t="s">
-        <v>776</v>
-      </c>
-      <c r="N16" s="41" t="s">
-        <v>576</v>
-      </c>
-      <c r="O16" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Pintura",Tabela24[Preço Total])</f>
-        <v>0</v>
-      </c>
-      <c r="P16" s="44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B17" s="17">
-        <v>14</v>
-      </c>
-      <c r="C17" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D17" s="25" t="s">
-        <v>783</v>
-      </c>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I17" s="24" t="s">
-        <v>776</v>
-      </c>
-      <c r="N17" s="41" t="s">
-        <v>818</v>
-      </c>
-      <c r="O17" s="40">
-        <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
-        <v>0</v>
-      </c>
-      <c r="P17" s="44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B18" s="17">
-        <v>15</v>
-      </c>
-      <c r="C18" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D18" s="25" t="s">
-        <v>784</v>
-      </c>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I18" s="24" t="s">
-        <v>776</v>
-      </c>
-      <c r="N18" s="41"/>
-      <c r="O18" s="40"/>
-      <c r="P18" s="44"/>
-    </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B19" s="17">
-        <v>16</v>
-      </c>
-      <c r="C19" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D19" s="25" t="s">
-        <v>822</v>
-      </c>
-      <c r="E19" s="24">
-        <v>1</v>
-      </c>
-      <c r="F19" s="24"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I19" s="24" t="s">
-        <v>776</v>
-      </c>
-      <c r="N19" s="41"/>
-      <c r="O19" s="40"/>
-      <c r="P19" s="44"/>
-    </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B20" s="17">
-        <v>17</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D20" s="18" t="s">
-        <v>797</v>
-      </c>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I20" s="17" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B21" s="17">
-        <v>18</v>
-      </c>
-      <c r="C21" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D21" s="18" t="s">
-        <v>769</v>
-      </c>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I21" s="17" t="s">
-        <v>771</v>
-      </c>
-      <c r="N21" s="41" t="s">
-        <v>825</v>
-      </c>
-      <c r="O21" s="43">
-        <f>SUM(O5:O17)</f>
-        <v>2927819.11</v>
-      </c>
-    </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B22" s="17">
-        <v>19</v>
-      </c>
-      <c r="C22" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D22" s="18" t="s">
-        <v>770</v>
-      </c>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I22" s="17" t="s">
-        <v>771</v>
-      </c>
-      <c r="N22" s="41"/>
-      <c r="O22" s="43"/>
-    </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B23" s="17">
-        <v>20</v>
-      </c>
-      <c r="C23" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D23" s="18" t="s">
-        <v>833</v>
-      </c>
-      <c r="E23" s="17">
-        <v>1</v>
-      </c>
-      <c r="F23" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="G23" s="20">
-        <v>164000</v>
-      </c>
-      <c r="H23" s="20">
-        <f t="shared" si="0"/>
-        <v>164000</v>
       </c>
       <c r="I23" s="17" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B24" s="17">
+      <c r="B24" s="22">
         <v>21</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>774</v>
+        <v>769</v>
       </c>
       <c r="E24" s="17"/>
       <c r="F24" s="17"/>
       <c r="G24" s="20"/>
       <c r="H24" s="20">
-        <f t="shared" si="0"/>
+        <f>G24*E24</f>
         <v>0</v>
       </c>
       <c r="I24" s="17" t="s">
         <v>771</v>
       </c>
+      <c r="N24" s="40" t="s">
+        <v>824</v>
+      </c>
+      <c r="O24" s="42">
+        <f>SUM(O5:O20)</f>
+        <v>3573429.2231375999</v>
+      </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B25" s="17">
+      <c r="B25" s="22">
         <v>22</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>775</v>
+        <v>770</v>
       </c>
       <c r="E25" s="17"/>
       <c r="F25" s="17"/>
       <c r="G25" s="20"/>
       <c r="H25" s="20">
-        <f t="shared" si="0"/>
+        <f>G25*E25</f>
         <v>0</v>
       </c>
       <c r="I25" s="17" t="s">
         <v>771</v>
       </c>
+      <c r="N25" s="40"/>
+      <c r="O25" s="42"/>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B26" s="17">
+      <c r="B26" s="22">
         <v>23</v>
       </c>
-      <c r="C26" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D26" s="21" t="s">
+      <c r="C26" s="27" t="s">
+        <v>809</v>
+      </c>
+      <c r="D26" s="31" t="s">
+        <v>832</v>
+      </c>
+      <c r="E26" s="27">
+        <v>1</v>
+      </c>
+      <c r="F26" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="G26" s="32">
+        <v>164000</v>
+      </c>
+      <c r="H26" s="32">
+        <f>G26*E26</f>
+        <v>164000</v>
+      </c>
+      <c r="I26" s="27" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B27" s="22">
+        <v>24</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>774</v>
+      </c>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20">
+        <f>G27*E27</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="17" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B28" s="22">
+        <v>25</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>775</v>
+      </c>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20">
+        <f>G28*E28</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="17" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B29" s="22">
+        <v>26</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D29" s="21" t="s">
         <v>779</v>
       </c>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19">
-        <f t="shared" si="0"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19">
+        <f>G29*E29</f>
         <v>0</v>
       </c>
-      <c r="I26" s="22" t="s">
+      <c r="I29" s="22" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B27" s="17">
-        <v>24</v>
-      </c>
-      <c r="C27" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D27" s="25" t="s">
-        <v>788</v>
-      </c>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I27" s="24" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B28" s="17">
-        <v>25</v>
-      </c>
-      <c r="C28" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D28" s="25" t="s">
-        <v>789</v>
-      </c>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I28" s="24" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B29" s="17">
-        <v>26</v>
-      </c>
-      <c r="C29" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D29" s="25" t="s">
-        <v>790</v>
-      </c>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I29" s="24" t="s">
-        <v>576</v>
-      </c>
-    </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B30" s="17">
+      <c r="B30" s="22">
         <v>27</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="D30" s="25" t="s">
-        <v>791</v>
+        <v>787</v>
       </c>
       <c r="E30" s="24"/>
       <c r="F30" s="24"/>
       <c r="G30" s="26"/>
       <c r="H30" s="26">
-        <f t="shared" si="0"/>
+        <f>G30*E30</f>
         <v>0</v>
       </c>
       <c r="I30" s="24" t="s">
@@ -14434,336 +14551,324 @@
       </c>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B31" s="17">
+      <c r="B31" s="22">
         <v>28</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D31" s="18" t="s">
+        <v>809</v>
+      </c>
+      <c r="D31" s="25" t="s">
+        <v>788</v>
+      </c>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26">
+        <f>G31*E31</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="24" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B32" s="22">
+        <v>29</v>
+      </c>
+      <c r="C32" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D32" s="25" t="s">
+        <v>789</v>
+      </c>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26">
+        <f>G32*E32</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="24" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B33" s="22">
+        <v>30</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D33" s="25" t="s">
+        <v>790</v>
+      </c>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26">
+        <f>G33*E33</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="24" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B34" s="22">
+        <v>31</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>809</v>
+      </c>
+      <c r="D34" s="31" t="s">
         <v>757</v>
       </c>
-      <c r="E31" s="23">
+      <c r="E34" s="33">
         <f>(2150*1.05)*0.15</f>
         <v>338.625</v>
       </c>
-      <c r="F31" s="17" t="s">
+      <c r="F34" s="27" t="s">
         <v>759</v>
       </c>
-      <c r="G31" s="20">
+      <c r="G34" s="32">
         <v>670</v>
       </c>
-      <c r="H31" s="20">
-        <f t="shared" si="0"/>
+      <c r="H34" s="32">
+        <f>G34*E34</f>
         <v>226878.75</v>
       </c>
-      <c r="I31" s="17" t="s">
+      <c r="I34" s="27" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B32" s="17">
-        <v>29</v>
-      </c>
-      <c r="C32" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D32" s="18" t="s">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B35" s="22">
+        <v>32</v>
+      </c>
+      <c r="C35" s="27" t="s">
+        <v>809</v>
+      </c>
+      <c r="D35" s="31" t="s">
         <v>777</v>
       </c>
-      <c r="E32" s="23">
+      <c r="E35" s="33">
         <f>(2150/13)*2</f>
         <v>330.76923076923077</v>
       </c>
-      <c r="F32" s="17" t="s">
+      <c r="F35" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="G32" s="20">
+      <c r="G35" s="32">
         <v>220.5</v>
       </c>
-      <c r="H32" s="20">
-        <f t="shared" si="0"/>
+      <c r="H35" s="32">
+        <f>G35*E35</f>
         <v>72934.61538461539</v>
       </c>
-      <c r="I32" s="17" t="s">
+      <c r="I35" s="27" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B33" s="17">
-        <v>30</v>
-      </c>
-      <c r="C33" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D33" s="18" t="s">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B36" s="22">
+        <v>33</v>
+      </c>
+      <c r="C36" s="27" t="s">
+        <v>809</v>
+      </c>
+      <c r="D36" s="31" t="s">
         <v>758</v>
       </c>
-      <c r="E33" s="17">
+      <c r="E36" s="27">
         <f>2100/12</f>
         <v>175</v>
       </c>
-      <c r="F33" s="17" t="s">
+      <c r="F36" s="27" t="s">
         <v>761</v>
       </c>
-      <c r="G33" s="20">
+      <c r="G36" s="32">
         <v>56.2</v>
       </c>
-      <c r="H33" s="20">
-        <f t="shared" si="0"/>
+      <c r="H36" s="32">
+        <f>G36*E36</f>
         <v>9835</v>
       </c>
-      <c r="I33" s="17" t="s">
+      <c r="I36" s="27" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="17">
-        <v>31</v>
-      </c>
-      <c r="C34" s="17" t="s">
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B37" s="22">
+        <v>34</v>
+      </c>
+      <c r="C37" s="27" t="s">
+        <v>809</v>
+      </c>
+      <c r="D37" s="31" t="s">
+        <v>762</v>
+      </c>
+      <c r="E37" s="27">
+        <v>1000</v>
+      </c>
+      <c r="F37" s="27" t="s">
+        <v>763</v>
+      </c>
+      <c r="G37" s="32">
+        <v>7.3</v>
+      </c>
+      <c r="H37" s="32">
+        <f>G37*E37</f>
+        <v>7300</v>
+      </c>
+      <c r="I37" s="27" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B38" s="22">
+        <v>35</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D38" s="18" t="s">
+        <v>815</v>
+      </c>
+      <c r="E38" s="23">
+        <f>E34</f>
+        <v>338.625</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>766</v>
+      </c>
+      <c r="G38" s="20">
+        <v>50</v>
+      </c>
+      <c r="H38" s="20">
+        <f>G38*E38</f>
+        <v>16931.25</v>
+      </c>
+      <c r="I38" s="17" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B39" s="22">
+        <v>36</v>
+      </c>
+      <c r="C39" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D39" s="18" t="s">
+        <v>768</v>
+      </c>
+      <c r="E39" s="17">
+        <v>1</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G39" s="20">
+        <v>49800</v>
+      </c>
+      <c r="H39" s="20">
+        <f>G39*E39</f>
+        <v>49800</v>
+      </c>
+      <c r="I39" s="17" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B40" s="22">
+        <v>37</v>
+      </c>
+      <c r="C40" s="34" t="s">
         <v>810</v>
       </c>
-      <c r="D34" s="18" t="s">
-        <v>762</v>
-      </c>
-      <c r="E34" s="17">
-        <v>1000</v>
-      </c>
-      <c r="F34" s="17" t="s">
-        <v>763</v>
-      </c>
-      <c r="G34" s="20">
-        <v>7.3</v>
-      </c>
-      <c r="H34" s="20">
-        <f t="shared" si="0"/>
-        <v>7300</v>
-      </c>
-      <c r="I34" s="17" t="s">
+      <c r="D40" s="25" t="s">
+        <v>820</v>
+      </c>
+      <c r="E40" s="24">
+        <v>110</v>
+      </c>
+      <c r="F40" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G40" s="26"/>
+      <c r="H40" s="26">
+        <f>G40*E40</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="24" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B35" s="17">
-        <v>32</v>
-      </c>
-      <c r="C35" s="17" t="s">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B41" s="22">
+        <v>38</v>
+      </c>
+      <c r="C41" s="34" t="s">
         <v>810</v>
       </c>
-      <c r="D35" s="18" t="s">
-        <v>816</v>
-      </c>
-      <c r="E35" s="23">
-        <f>E31</f>
-        <v>338.625</v>
-      </c>
-      <c r="F35" s="17" t="s">
-        <v>766</v>
-      </c>
-      <c r="G35" s="20">
-        <v>50</v>
-      </c>
-      <c r="H35" s="20">
-        <f t="shared" si="0"/>
-        <v>16931.25</v>
-      </c>
-      <c r="I35" s="17" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B36" s="17">
-        <v>33</v>
-      </c>
-      <c r="C36" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D36" s="18" t="s">
-        <v>768</v>
-      </c>
-      <c r="E36" s="17">
-        <v>1</v>
-      </c>
-      <c r="F36" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="G36" s="20">
-        <v>49800</v>
-      </c>
-      <c r="H36" s="20">
-        <f t="shared" si="0"/>
-        <v>49800</v>
-      </c>
-      <c r="I36" s="17" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B37" s="17">
-        <v>34</v>
-      </c>
-      <c r="C37" s="34" t="s">
-        <v>811</v>
-      </c>
-      <c r="D37" s="25" t="s">
-        <v>821</v>
-      </c>
-      <c r="E37" s="24">
-        <v>110</v>
-      </c>
-      <c r="F37" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G37" s="26"/>
-      <c r="H37" s="26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I37" s="24" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B38" s="17">
-        <v>35</v>
-      </c>
-      <c r="C38" s="34" t="s">
-        <v>811</v>
-      </c>
-      <c r="D38" s="25" t="s">
+      <c r="D41" s="25" t="s">
         <v>757</v>
       </c>
-      <c r="E38" s="35">
+      <c r="E41" s="35">
         <f>(1784*0.15)*1.05</f>
         <v>280.97999999999996</v>
       </c>
-      <c r="F38" s="24" t="s">
+      <c r="F41" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="G38" s="26">
+      <c r="G41" s="26">
         <v>670</v>
       </c>
-      <c r="H38" s="26">
-        <f t="shared" si="0"/>
+      <c r="H41" s="26">
+        <f>G41*E41</f>
         <v>188256.59999999998</v>
       </c>
-      <c r="I38" s="24" t="s">
+      <c r="I41" s="24" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="17">
-        <v>36</v>
-      </c>
-      <c r="C39" s="34" t="s">
-        <v>811</v>
-      </c>
-      <c r="D39" s="18" t="s">
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B42" s="22">
+        <v>39</v>
+      </c>
+      <c r="C42" s="34" t="s">
+        <v>810</v>
+      </c>
+      <c r="D42" s="18" t="s">
         <v>777</v>
       </c>
-      <c r="E39" s="35">
+      <c r="E42" s="35">
         <f>1784/13</f>
         <v>137.23076923076923</v>
       </c>
-      <c r="F39" s="24" t="s">
+      <c r="F42" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G39" s="26">
+      <c r="G42" s="26">
         <v>220.5</v>
       </c>
-      <c r="H39" s="26">
-        <f t="shared" si="0"/>
+      <c r="H42" s="26">
+        <f>G42*E42</f>
         <v>30259.384615384613</v>
       </c>
-      <c r="I39" s="24" t="s">
+      <c r="I42" s="24" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B40" s="17">
-        <v>37</v>
-      </c>
-      <c r="C40" s="34" t="s">
-        <v>811</v>
-      </c>
-      <c r="D40" s="25" t="s">
-        <v>820</v>
-      </c>
-      <c r="E40" s="24">
-        <v>1</v>
-      </c>
-      <c r="F40" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G40" s="26">
-        <v>43350</v>
-      </c>
-      <c r="H40" s="26">
-        <f t="shared" si="0"/>
-        <v>43350</v>
-      </c>
-      <c r="I40" s="24" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="17">
-        <v>38</v>
-      </c>
-      <c r="C41" s="17" t="s">
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B43" s="22">
+        <v>40</v>
+      </c>
+      <c r="C43" s="34" t="s">
         <v>810</v>
       </c>
-      <c r="D41" s="18" t="s">
-        <v>773</v>
-      </c>
-      <c r="E41" s="17">
-        <v>1</v>
-      </c>
-      <c r="F41" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="G41" s="20">
-        <v>968004</v>
-      </c>
-      <c r="H41" s="20">
-        <f t="shared" si="0"/>
-        <v>968004</v>
-      </c>
-      <c r="I41" s="17" t="s">
-        <v>772</v>
-      </c>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B42" s="17">
-        <v>39</v>
-      </c>
-      <c r="C42" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D42" s="21" t="s">
-        <v>795</v>
-      </c>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="19"/>
-      <c r="H42" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I42" s="17" t="s">
-        <v>772</v>
-      </c>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B43" s="17">
-        <v>40</v>
-      </c>
-      <c r="C43" s="17" t="s">
-        <v>811</v>
-      </c>
       <c r="D43" s="25" t="s">
-        <v>805</v>
+        <v>819</v>
       </c>
       <c r="E43" s="24">
         <v>1</v>
@@ -14772,52 +14877,52 @@
         <v>760</v>
       </c>
       <c r="G43" s="26">
-        <v>46600</v>
+        <v>43350</v>
       </c>
       <c r="H43" s="26">
-        <f t="shared" si="0"/>
-        <v>46600</v>
+        <f>G43*E43</f>
+        <v>43350</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>807</v>
+        <v>635</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B44" s="17">
+      <c r="B44" s="22">
         <v>41</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>811</v>
-      </c>
-      <c r="D44" s="25" t="s">
-        <v>808</v>
-      </c>
-      <c r="E44" s="24">
-        <v>1</v>
-      </c>
-      <c r="F44" s="24" t="s">
+        <v>809</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="E44" s="17">
+        <v>1</v>
+      </c>
+      <c r="F44" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G44" s="26">
-        <v>8100</v>
-      </c>
-      <c r="H44" s="26">
-        <f t="shared" si="0"/>
-        <v>8100</v>
-      </c>
-      <c r="I44" s="24" t="s">
-        <v>807</v>
+      <c r="G44" s="20">
+        <v>968004</v>
+      </c>
+      <c r="H44" s="20">
+        <f>G44*E44</f>
+        <v>968004</v>
+      </c>
+      <c r="I44" s="17" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B45" s="17">
+      <c r="B45" s="22">
         <v>42</v>
       </c>
       <c r="C45" s="17" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="D45" s="25" t="s">
-        <v>823</v>
+        <v>804</v>
       </c>
       <c r="E45" s="24">
         <v>1</v>
@@ -14826,25 +14931,25 @@
         <v>760</v>
       </c>
       <c r="G45" s="26">
-        <v>5000</v>
+        <v>46600</v>
       </c>
       <c r="H45" s="26">
-        <f t="shared" si="0"/>
-        <v>5000</v>
+        <f>G45*E45</f>
+        <v>46600</v>
       </c>
       <c r="I45" s="24" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B46" s="22">
+        <v>43</v>
+      </c>
+      <c r="C46" s="17" t="s">
+        <v>810</v>
+      </c>
+      <c r="D46" s="25" t="s">
         <v>807</v>
-      </c>
-    </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B46" s="17">
-        <v>43</v>
-      </c>
-      <c r="C46" s="17" t="s">
-        <v>811</v>
-      </c>
-      <c r="D46" s="25" t="s">
-        <v>812</v>
       </c>
       <c r="E46" s="24">
         <v>1</v>
@@ -14853,89 +14958,236 @@
         <v>760</v>
       </c>
       <c r="G46" s="26">
-        <v>298777</v>
+        <v>8100</v>
       </c>
       <c r="H46" s="26">
-        <f t="shared" si="0"/>
-        <v>298777</v>
+        <f>G46*E46</f>
+        <v>8100</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="17">
+      <c r="B47" s="22">
         <v>44</v>
       </c>
       <c r="C47" s="17" t="s">
         <v>810</v>
       </c>
-      <c r="D47" s="21" t="s">
-        <v>794</v>
-      </c>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I47" s="22" t="s">
-        <v>419</v>
+      <c r="D47" s="25" t="s">
+        <v>822</v>
+      </c>
+      <c r="E47" s="24">
+        <v>1</v>
+      </c>
+      <c r="F47" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G47" s="26">
+        <v>5000</v>
+      </c>
+      <c r="H47" s="26">
+        <f>G47*E47</f>
+        <v>5000</v>
+      </c>
+      <c r="I47" s="24" t="s">
+        <v>806</v>
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B48" s="17">
+      <c r="B48" s="22">
         <v>45</v>
       </c>
       <c r="C48" s="17" t="s">
         <v>810</v>
       </c>
-      <c r="D48" s="21" t="s">
-        <v>787</v>
-      </c>
-      <c r="E48" s="22">
-        <v>1</v>
-      </c>
-      <c r="F48" s="22" t="s">
+      <c r="D48" s="25" t="s">
+        <v>811</v>
+      </c>
+      <c r="E48" s="24">
+        <v>1</v>
+      </c>
+      <c r="F48" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G48" s="19">
+      <c r="G48" s="26">
+        <v>298777</v>
+      </c>
+      <c r="H48" s="26">
+        <f>G48*E48</f>
+        <v>298777</v>
+      </c>
+      <c r="I48" s="24" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B49" s="22">
+        <v>46</v>
+      </c>
+      <c r="C49" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D49" s="21" t="s">
+        <v>793</v>
+      </c>
+      <c r="E49" s="22"/>
+      <c r="F49" s="22"/>
+      <c r="G49" s="19"/>
+      <c r="H49" s="19">
+        <f>G49*E49</f>
+        <v>0</v>
+      </c>
+      <c r="I49" s="22" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B50" s="22">
+        <v>47</v>
+      </c>
+      <c r="C50" s="17"/>
+      <c r="D50" s="21" t="s">
+        <v>855</v>
+      </c>
+      <c r="E50" s="22"/>
+      <c r="F50" s="22"/>
+      <c r="G50" s="19"/>
+      <c r="H50" s="19">
+        <f>G50*E50</f>
+        <v>0</v>
+      </c>
+      <c r="I50" s="22" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B51" s="22">
+        <v>48</v>
+      </c>
+      <c r="C51" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D51" s="21" t="s">
+        <v>794</v>
+      </c>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="19"/>
+      <c r="H51" s="19">
+        <f>G51*E51</f>
+        <v>0</v>
+      </c>
+      <c r="I51" s="17" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B52" s="22">
+        <v>49</v>
+      </c>
+      <c r="C52" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D52" s="21" t="s">
+        <v>786</v>
+      </c>
+      <c r="E52" s="22">
+        <v>1</v>
+      </c>
+      <c r="F52" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G52" s="19">
         <v>791792.51</v>
       </c>
-      <c r="H48" s="19">
-        <f t="shared" si="0"/>
+      <c r="H52" s="19">
+        <f>G52*E52</f>
         <v>791792.51</v>
       </c>
-      <c r="I48" s="22" t="s">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B49" s="24"/>
-      <c r="C49" s="34"/>
-      <c r="D49" s="25"/>
-      <c r="E49" s="24"/>
-      <c r="F49" s="24"/>
-      <c r="G49" s="26"/>
-      <c r="H49" s="26"/>
-      <c r="I49" s="25"/>
-    </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B50" s="24"/>
-      <c r="C50" s="34"/>
-      <c r="D50" s="39"/>
-      <c r="E50" s="24"/>
-      <c r="F50" s="24"/>
-      <c r="G50" s="26"/>
-      <c r="H50" s="26"/>
-      <c r="I50" s="25"/>
-    </row>
-    <row r="51" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D51" s="38"/>
-      <c r="H51" s="16">
+      <c r="I52" s="22" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B53" s="22">
+        <v>50</v>
+      </c>
+      <c r="C53" s="17"/>
+      <c r="D53" s="21" t="s">
+        <v>857</v>
+      </c>
+      <c r="E53" s="22">
+        <v>6</v>
+      </c>
+      <c r="F53" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G53" s="19"/>
+      <c r="H53" s="19">
+        <f>G53*E53</f>
+        <v>0</v>
+      </c>
+      <c r="I53" s="17" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B54" s="24"/>
+      <c r="C54" s="34"/>
+      <c r="D54" s="25" t="s">
+        <v>863</v>
+      </c>
+      <c r="E54" s="24"/>
+      <c r="F54" s="24"/>
+      <c r="G54" s="26"/>
+      <c r="H54" s="51">
+        <f>G54*E54</f>
+        <v>0</v>
+      </c>
+      <c r="I54" s="24"/>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B55" s="24"/>
+      <c r="C55" s="34"/>
+      <c r="D55" s="25" t="s">
+        <v>864</v>
+      </c>
+      <c r="E55" s="24"/>
+      <c r="F55" s="24"/>
+      <c r="G55" s="26"/>
+      <c r="H55" s="51">
+        <f>G55*E55</f>
+        <v>0</v>
+      </c>
+      <c r="I55" s="24"/>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B56" s="24"/>
+      <c r="C56" s="34"/>
+      <c r="D56" s="25"/>
+      <c r="E56" s="24"/>
+      <c r="F56" s="24"/>
+      <c r="G56" s="26"/>
+      <c r="H56" s="51"/>
+      <c r="I56" s="24"/>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B57" s="24"/>
+      <c r="C57" s="34"/>
+      <c r="D57" s="25"/>
+      <c r="E57" s="24"/>
+      <c r="F57" s="24"/>
+      <c r="G57" s="26"/>
+      <c r="H57" s="51"/>
+      <c r="I57" s="24"/>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D58" s="38"/>
+      <c r="H58" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>2927819.1100000003</v>
+        <v>3538494.7265427997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 14:26
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -13786,11 +13786,11 @@
       </c>
       <c r="P5" s="43">
         <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
-        <v>0.27774553181958522</v>
+        <v>0.27738443200239088</v>
       </c>
       <c r="Q5" s="45">
         <f>P5</f>
-        <v>0.27774553181958522</v>
+        <v>0.27738443200239088</v>
       </c>
       <c r="R5" t="s">
         <v>828</v>
@@ -13827,11 +13827,11 @@
       </c>
       <c r="P6" s="43">
         <f t="shared" si="0"/>
-        <v>0.22157777881067911</v>
+        <v>0.22128970326577768</v>
       </c>
       <c r="Q6" s="45">
         <f>P6+Q5</f>
-        <v>0.49932331063026436</v>
+        <v>0.49867413526816856</v>
       </c>
       <c r="R6" t="s">
         <v>828</v>
@@ -13868,11 +13868,11 @@
       </c>
       <c r="O7" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Piso",Tabela24[Preço Total])</f>
-        <v>645545.6</v>
+        <v>650197.5</v>
       </c>
       <c r="P7" s="43">
         <f t="shared" si="0"/>
-        <v>0.1806515701556802</v>
+        <v>0.18171681346057503</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
@@ -13907,7 +13907,7 @@
       </c>
       <c r="P8" s="43">
         <f t="shared" si="0"/>
-        <v>0.10031736397041166</v>
+        <v>0.10018694033567732</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
@@ -13946,7 +13946,7 @@
       </c>
       <c r="P9" s="43">
         <f t="shared" si="0"/>
-        <v>4.5894290822416813E-2</v>
+        <v>4.5834623183777706E-2</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
@@ -13984,7 +13984,7 @@
       </c>
       <c r="P10" s="43">
         <f t="shared" si="0"/>
-        <v>1.8619105742461214E-2</v>
+        <v>1.8594898851945721E-2</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
@@ -14016,7 +14016,7 @@
       </c>
       <c r="P11" s="43">
         <f t="shared" si="0"/>
-        <v>0.13601276803049323</v>
+        <v>0.13583593643449907</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
@@ -14122,7 +14122,7 @@
       </c>
       <c r="P14" s="43">
         <f t="shared" si="0"/>
-        <v>1.8619105742461214E-2</v>
+        <v>1.8594898851945721E-2</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
@@ -14161,7 +14161,7 @@
       </c>
       <c r="P15" s="43">
         <f t="shared" si="0"/>
-        <v>5.6248490581132799E-4</v>
+        <v>5.6175361341093404E-4</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
@@ -14413,7 +14413,7 @@
       </c>
       <c r="O24" s="42">
         <f>SUM(O5:O20)</f>
-        <v>3573429.2231375999</v>
+        <v>3578081.1231375998</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -14795,10 +14795,12 @@
       <c r="F40" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G40" s="26"/>
+      <c r="G40" s="26">
+        <v>42.29</v>
+      </c>
       <c r="H40" s="26">
         <f>G40*E40</f>
-        <v>0</v>
+        <v>4651.8999999999996</v>
       </c>
       <c r="I40" s="24" t="s">
         <v>635</v>
@@ -15187,7 +15189,7 @@
       <c r="D58" s="38"/>
       <c r="H58" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>3538494.7265427997</v>
+        <v>3543146.6265428001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 14:32
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2135" uniqueCount="865">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="869">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2620,6 +2620,18 @@
   </si>
   <si>
     <t>Mão de obra para fechamento em alvenaria na parte interna do galpão blocado</t>
+  </si>
+  <si>
+    <t>Mão de obra para concretagem do piso do galpão 2100m²</t>
+  </si>
+  <si>
+    <t>Frente para entrega do Meio fio</t>
+  </si>
+  <si>
+    <t>Mão de obra para concretagem do piso das docas de carregamento DPA IV</t>
+  </si>
+  <si>
+    <t>Solicitar mais um orçamento do Erisvaldo</t>
   </si>
 </sst>
 </file>
@@ -3157,8 +3169,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I55" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:I55"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I57" totalsRowShown="0" dataDxfId="16">
+  <autoFilter ref="B3:I57"/>
   <sortState ref="B4:I51">
     <sortCondition ref="I3:I51"/>
   </sortState>
@@ -13660,7 +13672,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R58"/>
+  <dimension ref="B1:R60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -13671,7 +13683,8 @@
     <col min="7" max="7" width="15.85546875" style="15" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" style="15" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.85546875" style="14" customWidth="1"/>
-    <col min="10" max="13" width="16" style="14" customWidth="1"/>
+    <col min="10" max="10" width="38.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="16" style="14" customWidth="1"/>
     <col min="14" max="14" width="18.42578125" customWidth="1"/>
     <col min="15" max="15" width="25" customWidth="1"/>
     <col min="16" max="16" width="10.5703125" style="14" customWidth="1"/>
@@ -13786,11 +13799,11 @@
       </c>
       <c r="P5" s="43">
         <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
-        <v>0.27738443200239088</v>
+        <v>0.27698576114479873</v>
       </c>
       <c r="Q5" s="45">
         <f>P5</f>
-        <v>0.27738443200239088</v>
+        <v>0.27698576114479873</v>
       </c>
       <c r="R5" t="s">
         <v>828</v>
@@ -13827,11 +13840,11 @@
       </c>
       <c r="P6" s="43">
         <f t="shared" si="0"/>
-        <v>0.22128970326577768</v>
+        <v>0.22097165457378573</v>
       </c>
       <c r="Q6" s="45">
         <f>P6+Q5</f>
-        <v>0.49867413526816856</v>
+        <v>0.49795741571858443</v>
       </c>
       <c r="R6" t="s">
         <v>828</v>
@@ -13868,11 +13881,11 @@
       </c>
       <c r="O7" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Piso",Tabela24[Preço Total])</f>
-        <v>650197.5</v>
+        <v>655347.5</v>
       </c>
       <c r="P7" s="43">
         <f t="shared" si="0"/>
-        <v>0.18171681346057503</v>
+        <v>0.18289289121438398</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
@@ -13907,7 +13920,7 @@
       </c>
       <c r="P8" s="43">
         <f t="shared" si="0"/>
-        <v>0.10018694033567732</v>
+        <v>0.10004294662581108</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
@@ -13946,7 +13959,7 @@
       </c>
       <c r="P9" s="43">
         <f t="shared" si="0"/>
-        <v>4.5834623183777706E-2</v>
+        <v>4.5768747357942119E-2</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
@@ -13984,7 +13997,7 @@
       </c>
       <c r="P10" s="43">
         <f t="shared" si="0"/>
-        <v>1.8594898851945721E-2</v>
+        <v>1.8568173328027054E-2</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
@@ -14016,7 +14029,7 @@
       </c>
       <c r="P11" s="43">
         <f t="shared" si="0"/>
-        <v>0.13583593643449907</v>
+        <v>0.13564070619436175</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
@@ -14122,7 +14135,7 @@
       </c>
       <c r="P14" s="43">
         <f t="shared" si="0"/>
-        <v>1.8594898851945721E-2</v>
+        <v>1.8568173328027054E-2</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
@@ -14161,7 +14174,7 @@
       </c>
       <c r="P15" s="43">
         <f t="shared" si="0"/>
-        <v>5.6175361341093404E-4</v>
+        <v>5.6094623286258327E-4</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
@@ -14413,7 +14426,7 @@
       </c>
       <c r="O24" s="42">
         <f>SUM(O5:O20)</f>
-        <v>3578081.1231375998</v>
+        <v>3583231.1231375998</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -14759,23 +14772,23 @@
       <c r="C39" s="17" t="s">
         <v>809</v>
       </c>
-      <c r="D39" s="18" t="s">
-        <v>768</v>
-      </c>
-      <c r="E39" s="17">
-        <v>1</v>
-      </c>
-      <c r="F39" s="17" t="s">
+      <c r="D39" s="31" t="s">
+        <v>865</v>
+      </c>
+      <c r="E39" s="27">
+        <v>1</v>
+      </c>
+      <c r="F39" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="G39" s="20">
-        <v>49800</v>
-      </c>
-      <c r="H39" s="20">
+      <c r="G39" s="32">
+        <v>53550</v>
+      </c>
+      <c r="H39" s="32">
         <f>G39*E39</f>
-        <v>49800</v>
-      </c>
-      <c r="I39" s="17" t="s">
+        <v>53550</v>
+      </c>
+      <c r="I39" s="27" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14786,23 +14799,23 @@
       <c r="C40" s="34" t="s">
         <v>810</v>
       </c>
-      <c r="D40" s="25" t="s">
+      <c r="D40" s="47" t="s">
         <v>820</v>
       </c>
-      <c r="E40" s="24">
+      <c r="E40" s="48">
         <v>110</v>
       </c>
-      <c r="F40" s="24" t="s">
+      <c r="F40" s="48" t="s">
         <v>760</v>
       </c>
-      <c r="G40" s="26">
+      <c r="G40" s="49">
         <v>42.29</v>
       </c>
-      <c r="H40" s="26">
+      <c r="H40" s="49">
         <f>G40*E40</f>
         <v>4651.8999999999996</v>
       </c>
-      <c r="I40" s="24" t="s">
+      <c r="I40" s="48" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14810,27 +14823,24 @@
       <c r="B41" s="22">
         <v>38</v>
       </c>
-      <c r="C41" s="34" t="s">
-        <v>810</v>
-      </c>
-      <c r="D41" s="25" t="s">
-        <v>757</v>
-      </c>
-      <c r="E41" s="35">
-        <f>(1784*0.15)*1.05</f>
-        <v>280.97999999999996</v>
-      </c>
-      <c r="F41" s="24" t="s">
-        <v>759</v>
-      </c>
-      <c r="G41" s="26">
-        <v>670</v>
-      </c>
-      <c r="H41" s="26">
+      <c r="C41" s="34"/>
+      <c r="D41" s="47" t="s">
+        <v>866</v>
+      </c>
+      <c r="E41" s="48">
+        <v>1</v>
+      </c>
+      <c r="F41" s="48" t="s">
+        <v>760</v>
+      </c>
+      <c r="G41" s="49">
+        <v>1400</v>
+      </c>
+      <c r="H41" s="49">
         <f>G41*E41</f>
-        <v>188256.59999999998</v>
-      </c>
-      <c r="I41" s="24" t="s">
+        <v>1400</v>
+      </c>
+      <c r="I41" s="48" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14841,22 +14851,22 @@
       <c r="C42" s="34" t="s">
         <v>810</v>
       </c>
-      <c r="D42" s="18" t="s">
-        <v>777</v>
+      <c r="D42" s="25" t="s">
+        <v>757</v>
       </c>
       <c r="E42" s="35">
-        <f>1784/13</f>
-        <v>137.23076923076923</v>
+        <f>(1784*0.15)*1.05</f>
+        <v>280.97999999999996</v>
       </c>
       <c r="F42" s="24" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G42" s="26">
-        <v>220.5</v>
+        <v>670</v>
       </c>
       <c r="H42" s="26">
         <f>G42*E42</f>
-        <v>30259.384615384613</v>
+        <v>188256.59999999998</v>
       </c>
       <c r="I42" s="24" t="s">
         <v>635</v>
@@ -14869,21 +14879,22 @@
       <c r="C43" s="34" t="s">
         <v>810</v>
       </c>
-      <c r="D43" s="25" t="s">
-        <v>819</v>
-      </c>
-      <c r="E43" s="24">
-        <v>1</v>
+      <c r="D43" s="18" t="s">
+        <v>777</v>
+      </c>
+      <c r="E43" s="35">
+        <f>1784/13</f>
+        <v>137.23076923076923</v>
       </c>
       <c r="F43" s="24" t="s">
         <v>760</v>
       </c>
       <c r="G43" s="26">
-        <v>43350</v>
+        <v>220.5</v>
       </c>
       <c r="H43" s="26">
         <f>G43*E43</f>
-        <v>43350</v>
+        <v>30259.384615384613</v>
       </c>
       <c r="I43" s="24" t="s">
         <v>635</v>
@@ -14893,27 +14904,27 @@
       <c r="B44" s="22">
         <v>41</v>
       </c>
-      <c r="C44" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D44" s="18" t="s">
-        <v>773</v>
-      </c>
-      <c r="E44" s="17">
-        <v>1</v>
-      </c>
-      <c r="F44" s="17" t="s">
+      <c r="C44" s="34" t="s">
+        <v>810</v>
+      </c>
+      <c r="D44" s="25" t="s">
+        <v>819</v>
+      </c>
+      <c r="E44" s="24">
+        <v>1</v>
+      </c>
+      <c r="F44" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G44" s="20">
-        <v>968004</v>
-      </c>
-      <c r="H44" s="20">
+      <c r="G44" s="26">
+        <v>43350</v>
+      </c>
+      <c r="H44" s="26">
         <f>G44*E44</f>
-        <v>968004</v>
-      </c>
-      <c r="I44" s="17" t="s">
-        <v>772</v>
+        <v>43350</v>
+      </c>
+      <c r="I44" s="24" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
@@ -14921,26 +14932,26 @@
         <v>42</v>
       </c>
       <c r="C45" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D45" s="25" t="s">
-        <v>804</v>
-      </c>
-      <c r="E45" s="24">
-        <v>1</v>
-      </c>
-      <c r="F45" s="24" t="s">
+        <v>809</v>
+      </c>
+      <c r="D45" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="E45" s="17">
+        <v>1</v>
+      </c>
+      <c r="F45" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G45" s="26">
-        <v>46600</v>
-      </c>
-      <c r="H45" s="26">
+      <c r="G45" s="20">
+        <v>968004</v>
+      </c>
+      <c r="H45" s="20">
         <f>G45*E45</f>
-        <v>46600</v>
-      </c>
-      <c r="I45" s="24" t="s">
-        <v>806</v>
+        <v>968004</v>
+      </c>
+      <c r="I45" s="17" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
@@ -14951,7 +14962,7 @@
         <v>810</v>
       </c>
       <c r="D46" s="25" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="E46" s="24">
         <v>1</v>
@@ -14960,11 +14971,11 @@
         <v>760</v>
       </c>
       <c r="G46" s="26">
-        <v>8100</v>
+        <v>46600</v>
       </c>
       <c r="H46" s="26">
         <f>G46*E46</f>
-        <v>8100</v>
+        <v>46600</v>
       </c>
       <c r="I46" s="24" t="s">
         <v>806</v>
@@ -14978,7 +14989,7 @@
         <v>810</v>
       </c>
       <c r="D47" s="25" t="s">
-        <v>822</v>
+        <v>807</v>
       </c>
       <c r="E47" s="24">
         <v>1</v>
@@ -14987,11 +14998,11 @@
         <v>760</v>
       </c>
       <c r="G47" s="26">
-        <v>5000</v>
+        <v>8100</v>
       </c>
       <c r="H47" s="26">
         <f>G47*E47</f>
-        <v>5000</v>
+        <v>8100</v>
       </c>
       <c r="I47" s="24" t="s">
         <v>806</v>
@@ -15005,7 +15016,7 @@
         <v>810</v>
       </c>
       <c r="D48" s="25" t="s">
-        <v>811</v>
+        <v>822</v>
       </c>
       <c r="E48" s="24">
         <v>1</v>
@@ -15014,44 +15025,52 @@
         <v>760</v>
       </c>
       <c r="G48" s="26">
-        <v>298777</v>
+        <v>5000</v>
       </c>
       <c r="H48" s="26">
         <f>G48*E48</f>
-        <v>298777</v>
+        <v>5000</v>
       </c>
       <c r="I48" s="24" t="s">
         <v>806</v>
       </c>
     </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B49" s="22">
         <v>46</v>
       </c>
       <c r="C49" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D49" s="21" t="s">
-        <v>793</v>
-      </c>
-      <c r="E49" s="22"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="19"/>
-      <c r="H49" s="19">
+        <v>810</v>
+      </c>
+      <c r="D49" s="25" t="s">
+        <v>811</v>
+      </c>
+      <c r="E49" s="24">
+        <v>1</v>
+      </c>
+      <c r="F49" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G49" s="26">
+        <v>298777</v>
+      </c>
+      <c r="H49" s="26">
         <f>G49*E49</f>
-        <v>0</v>
-      </c>
-      <c r="I49" s="22" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.25">
+        <v>298777</v>
+      </c>
+      <c r="I49" s="24" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B50" s="22">
         <v>47</v>
       </c>
-      <c r="C50" s="17"/>
+      <c r="C50" s="17" t="s">
+        <v>809</v>
+      </c>
       <c r="D50" s="21" t="s">
-        <v>855</v>
+        <v>793</v>
       </c>
       <c r="E50" s="22"/>
       <c r="F50" s="22"/>
@@ -15061,18 +15080,16 @@
         <v>0</v>
       </c>
       <c r="I50" s="22" t="s">
-        <v>801</v>
-      </c>
-    </row>
-    <row r="51" spans="2:9" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B51" s="22">
         <v>48</v>
       </c>
-      <c r="C51" s="17" t="s">
-        <v>809</v>
-      </c>
+      <c r="C51" s="17"/>
       <c r="D51" s="21" t="s">
-        <v>794</v>
+        <v>855</v>
       </c>
       <c r="E51" s="22"/>
       <c r="F51" s="22"/>
@@ -15081,11 +15098,11 @@
         <f>G51*E51</f>
         <v>0</v>
       </c>
-      <c r="I51" s="17" t="s">
+      <c r="I51" s="22" t="s">
         <v>801</v>
       </c>
     </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B52" s="22">
         <v>49</v>
       </c>
@@ -15093,68 +15110,76 @@
         <v>809</v>
       </c>
       <c r="D52" s="21" t="s">
-        <v>786</v>
-      </c>
-      <c r="E52" s="22">
-        <v>1</v>
-      </c>
-      <c r="F52" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G52" s="19">
-        <v>791792.51</v>
-      </c>
+        <v>794</v>
+      </c>
+      <c r="E52" s="22"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="19"/>
       <c r="H52" s="19">
         <f>G52*E52</f>
-        <v>791792.51</v>
-      </c>
-      <c r="I52" s="22" t="s">
-        <v>785</v>
-      </c>
-    </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="I52" s="17" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B53" s="22">
         <v>50</v>
       </c>
-      <c r="C53" s="17"/>
+      <c r="C53" s="17" t="s">
+        <v>809</v>
+      </c>
       <c r="D53" s="21" t="s">
-        <v>857</v>
+        <v>786</v>
       </c>
       <c r="E53" s="22">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F53" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="G53" s="19"/>
+      <c r="G53" s="19">
+        <v>791792.51</v>
+      </c>
       <c r="H53" s="19">
         <f>G53*E53</f>
-        <v>0</v>
-      </c>
-      <c r="I53" s="17" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="54" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B54" s="24"/>
-      <c r="C54" s="34"/>
-      <c r="D54" s="25" t="s">
-        <v>863</v>
-      </c>
-      <c r="E54" s="24"/>
-      <c r="F54" s="24"/>
-      <c r="G54" s="26"/>
-      <c r="H54" s="51">
+        <v>791792.51</v>
+      </c>
+      <c r="I53" s="22" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B54" s="22">
+        <v>51</v>
+      </c>
+      <c r="C54" s="17"/>
+      <c r="D54" s="21" t="s">
+        <v>857</v>
+      </c>
+      <c r="E54" s="22">
+        <v>6</v>
+      </c>
+      <c r="F54" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G54" s="19"/>
+      <c r="H54" s="19">
         <f>G54*E54</f>
         <v>0</v>
       </c>
-      <c r="I54" s="24"/>
-    </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B55" s="24"/>
+      <c r="I54" s="17" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B55" s="22">
+        <v>52</v>
+      </c>
       <c r="C55" s="34"/>
       <c r="D55" s="25" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="E55" s="24"/>
       <c r="F55" s="24"/>
@@ -15163,33 +15188,76 @@
         <f>G55*E55</f>
         <v>0</v>
       </c>
-      <c r="I55" s="24"/>
-    </row>
-    <row r="56" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B56" s="24"/>
+      <c r="I55" s="17" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B56" s="22"/>
       <c r="C56" s="34"/>
-      <c r="D56" s="25"/>
-      <c r="E56" s="24"/>
-      <c r="F56" s="24"/>
+      <c r="D56" s="25" t="s">
+        <v>867</v>
+      </c>
+      <c r="E56" s="24">
+        <v>1</v>
+      </c>
+      <c r="F56" s="24" t="s">
+        <v>760</v>
+      </c>
       <c r="G56" s="26"/>
-      <c r="H56" s="51"/>
-      <c r="I56" s="24"/>
-    </row>
-    <row r="57" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B57" s="24"/>
+      <c r="H56" s="51">
+        <f>G56*E56</f>
+        <v>0</v>
+      </c>
+      <c r="I56" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="J56" s="14" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="57" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B57" s="22">
+        <v>53</v>
+      </c>
       <c r="C57" s="34"/>
-      <c r="D57" s="25"/>
+      <c r="D57" s="25" t="s">
+        <v>864</v>
+      </c>
       <c r="E57" s="24"/>
       <c r="F57" s="24"/>
       <c r="G57" s="26"/>
-      <c r="H57" s="51"/>
+      <c r="H57" s="51">
+        <f>G57*E57</f>
+        <v>0</v>
+      </c>
       <c r="I57" s="24"/>
     </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D58" s="38"/>
-      <c r="H58" s="16">
+    <row r="58" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B58" s="24"/>
+      <c r="C58" s="34"/>
+      <c r="D58" s="25"/>
+      <c r="E58" s="24"/>
+      <c r="F58" s="24"/>
+      <c r="G58" s="26"/>
+      <c r="H58" s="51"/>
+      <c r="I58" s="24"/>
+    </row>
+    <row r="59" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B59" s="24"/>
+      <c r="C59" s="34"/>
+      <c r="D59" s="25"/>
+      <c r="E59" s="24"/>
+      <c r="F59" s="24"/>
+      <c r="G59" s="26"/>
+      <c r="H59" s="51"/>
+      <c r="I59" s="24"/>
+    </row>
+    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D60" s="38"/>
+      <c r="H60" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>3543146.6265428001</v>
+        <v>3548296.6265428001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 14:33
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -3171,8 +3171,8 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I57" totalsRowShown="0" dataDxfId="16">
   <autoFilter ref="B3:I57"/>
-  <sortState ref="B4:I51">
-    <sortCondition ref="I3:I51"/>
+  <sortState ref="B4:I57">
+    <sortCondition ref="I3:I57"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" name="Item" dataDxfId="0" dataCellStyle="Normal"/>
@@ -13854,27 +13854,23 @@
       <c r="B7" s="22">
         <v>4</v>
       </c>
-      <c r="C7" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D7" s="31" t="s">
-        <v>860</v>
-      </c>
-      <c r="E7" s="27">
-        <v>1</v>
-      </c>
-      <c r="F7" s="27" t="s">
+      <c r="C7" s="17"/>
+      <c r="D7" s="21" t="s">
+        <v>857</v>
+      </c>
+      <c r="E7" s="22">
+        <v>6</v>
+      </c>
+      <c r="F7" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="G7" s="36">
-        <v>24500</v>
-      </c>
-      <c r="H7" s="36">
+      <c r="G7" s="19"/>
+      <c r="H7" s="19">
         <f>G7*E7</f>
-        <v>24500</v>
-      </c>
-      <c r="I7" s="27" t="s">
-        <v>772</v>
+        <v>0</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>253</v>
       </c>
       <c r="N7" s="37" t="s">
         <v>635</v>
@@ -13892,21 +13888,19 @@
       <c r="B8" s="22">
         <v>5</v>
       </c>
-      <c r="C8" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>837</v>
-      </c>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19">
+      <c r="C8" s="34"/>
+      <c r="D8" s="25" t="s">
+        <v>863</v>
+      </c>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="51">
         <f>G8*E8</f>
         <v>0</v>
       </c>
-      <c r="I8" s="22" t="s">
-        <v>772</v>
+      <c r="I8" s="17" t="s">
+        <v>253</v>
       </c>
       <c r="J8" s="14" t="s">
         <v>814</v>
@@ -13927,25 +13921,23 @@
       <c r="B9" s="22">
         <v>6</v>
       </c>
-      <c r="C9" s="17" t="s">
-        <v>809</v>
-      </c>
+      <c r="C9" s="34"/>
       <c r="D9" s="25" t="s">
-        <v>791</v>
+        <v>867</v>
       </c>
       <c r="E9" s="24">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="F9" s="24" t="s">
         <v>760</v>
       </c>
       <c r="G9" s="26"/>
-      <c r="H9" s="26">
+      <c r="H9" s="51">
         <f>G9*E9</f>
         <v>0</v>
       </c>
-      <c r="I9" s="24" t="s">
-        <v>643</v>
+      <c r="I9" s="17" t="s">
+        <v>253</v>
       </c>
       <c r="J9" s="14" t="s">
         <v>812</v>
@@ -13966,26 +13958,24 @@
       <c r="B10" s="22">
         <v>7</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="17" t="s">
         <v>809</v>
       </c>
-      <c r="D10" s="47" t="s">
-        <v>792</v>
-      </c>
-      <c r="E10" s="48">
-        <v>600</v>
-      </c>
-      <c r="F10" s="48" t="s">
-        <v>761</v>
-      </c>
-      <c r="G10" s="49">
-        <v>3.35</v>
-      </c>
-      <c r="H10" s="49">
+      <c r="D10" s="25" t="s">
+        <v>791</v>
+      </c>
+      <c r="E10" s="24">
+        <v>26</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26">
         <f>G10*E10</f>
-        <v>2010</v>
-      </c>
-      <c r="I10" s="48" t="s">
+        <v>0</v>
+      </c>
+      <c r="I10" s="24" t="s">
         <v>643</v>
       </c>
       <c r="N10" s="41" t="s">
@@ -14004,20 +13994,26 @@
       <c r="B11" s="22">
         <v>8</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="27" t="s">
         <v>809</v>
       </c>
-      <c r="D11" s="25" t="s">
-        <v>816</v>
-      </c>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26">
+      <c r="D11" s="47" t="s">
+        <v>792</v>
+      </c>
+      <c r="E11" s="48">
+        <v>600</v>
+      </c>
+      <c r="F11" s="48" t="s">
+        <v>761</v>
+      </c>
+      <c r="G11" s="49">
+        <v>3.35</v>
+      </c>
+      <c r="H11" s="49">
         <f>G11*E11</f>
-        <v>0</v>
-      </c>
-      <c r="I11" s="24" t="s">
+        <v>2010</v>
+      </c>
+      <c r="I11" s="48" t="s">
         <v>643</v>
       </c>
       <c r="N11" s="40" t="s">
@@ -14039,24 +14035,18 @@
       <c r="C12" s="17" t="s">
         <v>809</v>
       </c>
-      <c r="D12" s="31" t="s">
-        <v>834</v>
-      </c>
-      <c r="E12" s="27">
-        <v>54</v>
-      </c>
-      <c r="F12" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="G12" s="36">
-        <v>243.39</v>
-      </c>
-      <c r="H12" s="36">
+      <c r="D12" s="25" t="s">
+        <v>816</v>
+      </c>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26">
         <f>G12*E12</f>
-        <v>13143.06</v>
-      </c>
-      <c r="I12" s="27" t="s">
-        <v>835</v>
+        <v>0</v>
+      </c>
+      <c r="I12" s="24" t="s">
+        <v>643</v>
       </c>
       <c r="N12" s="40" t="s">
         <v>449</v>
@@ -14078,20 +14068,20 @@
         <v>809</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="E13" s="27">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="F13" s="27" t="s">
         <v>760</v>
       </c>
       <c r="G13" s="36">
-        <v>119.7</v>
+        <v>243.39</v>
       </c>
       <c r="H13" s="36">
         <f>G13*E13</f>
-        <v>3591</v>
+        <v>13143.06</v>
       </c>
       <c r="I13" s="27" t="s">
         <v>835</v>
@@ -14104,24 +14094,24 @@
       <c r="B14" s="22">
         <v>11</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="17" t="s">
         <v>809</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>833</v>
-      </c>
-      <c r="E14" s="48">
-        <v>390</v>
+        <v>836</v>
+      </c>
+      <c r="E14" s="27">
+        <v>30</v>
       </c>
       <c r="F14" s="27" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G14" s="36">
-        <v>38.116666600000002</v>
+        <v>119.7</v>
       </c>
       <c r="H14" s="36">
         <f>G14*E14</f>
-        <v>14865.499974</v>
+        <v>3591</v>
       </c>
       <c r="I14" s="27" t="s">
         <v>835</v>
@@ -14142,28 +14132,27 @@
       <c r="B15" s="22">
         <v>12</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="27" t="s">
         <v>809</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>834</v>
-      </c>
-      <c r="E15" s="33">
-        <f>(84*1.02)*2*1.02</f>
-        <v>174.78720000000001</v>
+        <v>833</v>
+      </c>
+      <c r="E15" s="48">
+        <v>390</v>
       </c>
       <c r="F15" s="27" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="G15" s="36">
-        <v>243.39</v>
+        <v>38.116666600000002</v>
       </c>
       <c r="H15" s="36">
         <f>G15*E15</f>
-        <v>42541.456608</v>
+        <v>14865.499974</v>
       </c>
       <c r="I15" s="27" t="s">
-        <v>776</v>
+        <v>835</v>
       </c>
       <c r="N15" s="40" t="s">
         <v>643</v>
@@ -14181,25 +14170,25 @@
       <c r="B16" s="22">
         <v>13</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="17" t="s">
         <v>809</v>
       </c>
       <c r="D16" s="31" t="s">
-        <v>833</v>
-      </c>
-      <c r="E16" s="27">
-        <f>84*7</f>
-        <v>588</v>
+        <v>834</v>
+      </c>
+      <c r="E16" s="33">
+        <f>(84*1.02)*2*1.02</f>
+        <v>174.78720000000001</v>
       </c>
       <c r="F16" s="27" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G16" s="36">
-        <v>38.116666600000002</v>
+        <v>243.39</v>
       </c>
       <c r="H16" s="36">
         <f>G16*E16</f>
-        <v>22412.599960800002</v>
+        <v>42541.456608</v>
       </c>
       <c r="I16" s="27" t="s">
         <v>776</v>
@@ -14212,22 +14201,25 @@
       <c r="B17" s="22">
         <v>14</v>
       </c>
-      <c r="C17" s="27"/>
+      <c r="C17" s="27" t="s">
+        <v>809</v>
+      </c>
       <c r="D17" s="31" t="s">
-        <v>861</v>
+        <v>833</v>
       </c>
       <c r="E17" s="27">
-        <v>30</v>
+        <f>84*7</f>
+        <v>588</v>
       </c>
       <c r="F17" s="27" t="s">
-        <v>854</v>
+        <v>761</v>
       </c>
       <c r="G17" s="36">
-        <v>24</v>
+        <v>38.116666600000002</v>
       </c>
       <c r="H17" s="36">
         <f>G17*E17</f>
-        <v>720</v>
+        <v>22412.599960800002</v>
       </c>
       <c r="I17" s="27" t="s">
         <v>776</v>
@@ -14242,20 +14234,20 @@
       </c>
       <c r="C18" s="27"/>
       <c r="D18" s="31" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E18" s="27">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>760</v>
+        <v>854</v>
       </c>
       <c r="G18" s="36">
-        <v>860</v>
+        <v>24</v>
       </c>
       <c r="H18" s="36">
         <f>G18*E18</f>
-        <v>860</v>
+        <v>720</v>
       </c>
       <c r="I18" s="27" t="s">
         <v>776</v>
@@ -14268,22 +14260,24 @@
       <c r="B19" s="22">
         <v>16</v>
       </c>
-      <c r="C19" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D19" s="25" t="s">
-        <v>781</v>
-      </c>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24" t="s">
-        <v>761</v>
-      </c>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26">
+      <c r="C19" s="27"/>
+      <c r="D19" s="31" t="s">
+        <v>862</v>
+      </c>
+      <c r="E19" s="27">
+        <v>1</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="G19" s="36">
+        <v>860</v>
+      </c>
+      <c r="H19" s="36">
         <f>G19*E19</f>
-        <v>0</v>
-      </c>
-      <c r="I19" s="24" t="s">
+        <v>860</v>
+      </c>
+      <c r="I19" s="27" t="s">
         <v>776</v>
       </c>
       <c r="N19" s="40" t="s">
@@ -14306,10 +14300,12 @@
         <v>809</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
+      <c r="F20" s="24" t="s">
+        <v>761</v>
+      </c>
       <c r="G20" s="26"/>
       <c r="H20" s="26">
         <f>G20*E20</f>
@@ -14338,7 +14334,7 @@
         <v>809</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E21" s="24"/>
       <c r="F21" s="24"/>
@@ -14362,11 +14358,9 @@
         <v>809</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>821</v>
-      </c>
-      <c r="E22" s="24">
-        <v>1</v>
-      </c>
+        <v>783</v>
+      </c>
+      <c r="E22" s="24"/>
       <c r="F22" s="24"/>
       <c r="G22" s="26"/>
       <c r="H22" s="26">
@@ -14387,18 +14381,20 @@
       <c r="C23" s="17" t="s">
         <v>809</v>
       </c>
-      <c r="D23" s="18" t="s">
-        <v>796</v>
-      </c>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20">
+      <c r="D23" s="25" t="s">
+        <v>821</v>
+      </c>
+      <c r="E23" s="24">
+        <v>1</v>
+      </c>
+      <c r="F23" s="24"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26">
         <f>G23*E23</f>
         <v>0</v>
       </c>
-      <c r="I23" s="17" t="s">
-        <v>771</v>
+      <c r="I23" s="24" t="s">
+        <v>776</v>
       </c>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
@@ -14409,7 +14405,7 @@
         <v>809</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>769</v>
+        <v>796</v>
       </c>
       <c r="E24" s="17"/>
       <c r="F24" s="17"/>
@@ -14437,7 +14433,7 @@
         <v>809</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="E25" s="17"/>
       <c r="F25" s="17"/>
@@ -14456,26 +14452,20 @@
       <c r="B26" s="22">
         <v>23</v>
       </c>
-      <c r="C26" s="27" t="s">
+      <c r="C26" s="17" t="s">
         <v>809</v>
       </c>
-      <c r="D26" s="31" t="s">
-        <v>832</v>
-      </c>
-      <c r="E26" s="27">
-        <v>1</v>
-      </c>
-      <c r="F26" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="G26" s="32">
-        <v>164000</v>
-      </c>
-      <c r="H26" s="32">
+      <c r="D26" s="18" t="s">
+        <v>770</v>
+      </c>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="20">
         <f>G26*E26</f>
-        <v>164000</v>
-      </c>
-      <c r="I26" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="I26" s="17" t="s">
         <v>771</v>
       </c>
     </row>
@@ -14483,20 +14473,26 @@
       <c r="B27" s="22">
         <v>24</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="C27" s="27" t="s">
         <v>809</v>
       </c>
-      <c r="D27" s="18" t="s">
-        <v>774</v>
-      </c>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20">
+      <c r="D27" s="31" t="s">
+        <v>832</v>
+      </c>
+      <c r="E27" s="27">
+        <v>1</v>
+      </c>
+      <c r="F27" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="G27" s="32">
+        <v>164000</v>
+      </c>
+      <c r="H27" s="32">
         <f>G27*E27</f>
-        <v>0</v>
-      </c>
-      <c r="I27" s="17" t="s">
+        <v>164000</v>
+      </c>
+      <c r="I27" s="27" t="s">
         <v>771</v>
       </c>
     </row>
@@ -14508,7 +14504,7 @@
         <v>809</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="E28" s="17"/>
       <c r="F28" s="17"/>
@@ -14528,17 +14524,17 @@
       <c r="C29" s="17" t="s">
         <v>809</v>
       </c>
-      <c r="D29" s="21" t="s">
-        <v>779</v>
-      </c>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="19">
+      <c r="D29" s="18" t="s">
+        <v>775</v>
+      </c>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="20">
         <f>G29*E29</f>
         <v>0</v>
       </c>
-      <c r="I29" s="22" t="s">
+      <c r="I29" s="17" t="s">
         <v>771</v>
       </c>
     </row>
@@ -14549,18 +14545,18 @@
       <c r="C30" s="17" t="s">
         <v>809</v>
       </c>
-      <c r="D30" s="25" t="s">
-        <v>787</v>
-      </c>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26">
+      <c r="D30" s="21" t="s">
+        <v>779</v>
+      </c>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="19">
         <f>G30*E30</f>
         <v>0</v>
       </c>
-      <c r="I30" s="24" t="s">
-        <v>576</v>
+      <c r="I30" s="22" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.25">
@@ -14571,7 +14567,7 @@
         <v>809</v>
       </c>
       <c r="D31" s="25" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="E31" s="24"/>
       <c r="F31" s="24"/>
@@ -14592,7 +14588,7 @@
         <v>809</v>
       </c>
       <c r="D32" s="25" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="E32" s="24"/>
       <c r="F32" s="24"/>
@@ -14613,7 +14609,7 @@
         <v>809</v>
       </c>
       <c r="D33" s="25" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="E33" s="24"/>
       <c r="F33" s="24"/>
@@ -14630,28 +14626,21 @@
       <c r="B34" s="22">
         <v>31</v>
       </c>
-      <c r="C34" s="27" t="s">
+      <c r="C34" s="17" t="s">
         <v>809</v>
       </c>
-      <c r="D34" s="31" t="s">
-        <v>757</v>
-      </c>
-      <c r="E34" s="33">
-        <f>(2150*1.05)*0.15</f>
-        <v>338.625</v>
-      </c>
-      <c r="F34" s="27" t="s">
-        <v>759</v>
-      </c>
-      <c r="G34" s="32">
-        <v>670</v>
-      </c>
-      <c r="H34" s="32">
+      <c r="D34" s="25" t="s">
+        <v>790</v>
+      </c>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="26">
         <f>G34*E34</f>
-        <v>226878.75</v>
-      </c>
-      <c r="I34" s="27" t="s">
-        <v>635</v>
+        <v>0</v>
+      </c>
+      <c r="I34" s="24" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.25">
@@ -14662,21 +14651,21 @@
         <v>809</v>
       </c>
       <c r="D35" s="31" t="s">
-        <v>777</v>
+        <v>757</v>
       </c>
       <c r="E35" s="33">
-        <f>(2150/13)*2</f>
-        <v>330.76923076923077</v>
+        <f>(2150*1.05)*0.15</f>
+        <v>338.625</v>
       </c>
       <c r="F35" s="27" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G35" s="32">
-        <v>220.5</v>
+        <v>670</v>
       </c>
       <c r="H35" s="32">
         <f>G35*E35</f>
-        <v>72934.61538461539</v>
+        <v>226878.75</v>
       </c>
       <c r="I35" s="27" t="s">
         <v>635</v>
@@ -14690,21 +14679,21 @@
         <v>809</v>
       </c>
       <c r="D36" s="31" t="s">
-        <v>758</v>
-      </c>
-      <c r="E36" s="27">
-        <f>2100/12</f>
-        <v>175</v>
+        <v>777</v>
+      </c>
+      <c r="E36" s="33">
+        <f>(2150/13)*2</f>
+        <v>330.76923076923077</v>
       </c>
       <c r="F36" s="27" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G36" s="32">
-        <v>56.2</v>
+        <v>220.5</v>
       </c>
       <c r="H36" s="32">
         <f>G36*E36</f>
-        <v>9835</v>
+        <v>72934.61538461539</v>
       </c>
       <c r="I36" s="27" t="s">
         <v>635</v>
@@ -14718,20 +14707,21 @@
         <v>809</v>
       </c>
       <c r="D37" s="31" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="E37" s="27">
-        <v>1000</v>
+        <f>2100/12</f>
+        <v>175</v>
       </c>
       <c r="F37" s="27" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="G37" s="32">
-        <v>7.3</v>
+        <v>56.2</v>
       </c>
       <c r="H37" s="32">
         <f>G37*E37</f>
-        <v>7300</v>
+        <v>9835</v>
       </c>
       <c r="I37" s="27" t="s">
         <v>635</v>
@@ -14741,27 +14731,26 @@
       <c r="B38" s="22">
         <v>35</v>
       </c>
-      <c r="C38" s="17" t="s">
+      <c r="C38" s="27" t="s">
         <v>809</v>
       </c>
-      <c r="D38" s="18" t="s">
-        <v>815</v>
-      </c>
-      <c r="E38" s="23">
-        <f>E34</f>
-        <v>338.625</v>
-      </c>
-      <c r="F38" s="17" t="s">
-        <v>766</v>
-      </c>
-      <c r="G38" s="20">
-        <v>50</v>
-      </c>
-      <c r="H38" s="20">
+      <c r="D38" s="31" t="s">
+        <v>762</v>
+      </c>
+      <c r="E38" s="27">
+        <v>1000</v>
+      </c>
+      <c r="F38" s="27" t="s">
+        <v>763</v>
+      </c>
+      <c r="G38" s="32">
+        <v>7.3</v>
+      </c>
+      <c r="H38" s="32">
         <f>G38*E38</f>
-        <v>16931.25</v>
-      </c>
-      <c r="I38" s="17" t="s">
+        <v>7300</v>
+      </c>
+      <c r="I38" s="27" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14772,23 +14761,24 @@
       <c r="C39" s="17" t="s">
         <v>809</v>
       </c>
-      <c r="D39" s="31" t="s">
-        <v>865</v>
-      </c>
-      <c r="E39" s="27">
-        <v>1</v>
-      </c>
-      <c r="F39" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="G39" s="32">
-        <v>53550</v>
-      </c>
-      <c r="H39" s="32">
+      <c r="D39" s="18" t="s">
+        <v>815</v>
+      </c>
+      <c r="E39" s="23">
+        <f>E35</f>
+        <v>338.625</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>766</v>
+      </c>
+      <c r="G39" s="20">
+        <v>50</v>
+      </c>
+      <c r="H39" s="20">
         <f>G39*E39</f>
-        <v>53550</v>
-      </c>
-      <c r="I39" s="27" t="s">
+        <v>16931.25</v>
+      </c>
+      <c r="I39" s="17" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14796,26 +14786,26 @@
       <c r="B40" s="22">
         <v>37</v>
       </c>
-      <c r="C40" s="34" t="s">
-        <v>810</v>
-      </c>
-      <c r="D40" s="47" t="s">
-        <v>820</v>
-      </c>
-      <c r="E40" s="48">
-        <v>110</v>
-      </c>
-      <c r="F40" s="48" t="s">
+      <c r="C40" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D40" s="31" t="s">
+        <v>865</v>
+      </c>
+      <c r="E40" s="27">
+        <v>1</v>
+      </c>
+      <c r="F40" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="G40" s="49">
-        <v>42.29</v>
-      </c>
-      <c r="H40" s="49">
+      <c r="G40" s="32">
+        <v>53550</v>
+      </c>
+      <c r="H40" s="32">
         <f>G40*E40</f>
-        <v>4651.8999999999996</v>
-      </c>
-      <c r="I40" s="48" t="s">
+        <v>53550</v>
+      </c>
+      <c r="I40" s="27" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14823,22 +14813,24 @@
       <c r="B41" s="22">
         <v>38</v>
       </c>
-      <c r="C41" s="34"/>
+      <c r="C41" s="34" t="s">
+        <v>810</v>
+      </c>
       <c r="D41" s="47" t="s">
-        <v>866</v>
+        <v>820</v>
       </c>
       <c r="E41" s="48">
-        <v>1</v>
+        <v>110</v>
       </c>
       <c r="F41" s="48" t="s">
         <v>760</v>
       </c>
       <c r="G41" s="49">
-        <v>1400</v>
+        <v>42.29</v>
       </c>
       <c r="H41" s="49">
         <f>G41*E41</f>
-        <v>1400</v>
+        <v>4651.8999999999996</v>
       </c>
       <c r="I41" s="48" t="s">
         <v>635</v>
@@ -14848,27 +14840,24 @@
       <c r="B42" s="22">
         <v>39</v>
       </c>
-      <c r="C42" s="34" t="s">
-        <v>810</v>
-      </c>
-      <c r="D42" s="25" t="s">
-        <v>757</v>
-      </c>
-      <c r="E42" s="35">
-        <f>(1784*0.15)*1.05</f>
-        <v>280.97999999999996</v>
-      </c>
-      <c r="F42" s="24" t="s">
-        <v>759</v>
-      </c>
-      <c r="G42" s="26">
-        <v>670</v>
-      </c>
-      <c r="H42" s="26">
+      <c r="C42" s="34"/>
+      <c r="D42" s="47" t="s">
+        <v>866</v>
+      </c>
+      <c r="E42" s="48">
+        <v>1</v>
+      </c>
+      <c r="F42" s="48" t="s">
+        <v>760</v>
+      </c>
+      <c r="G42" s="49">
+        <v>1400</v>
+      </c>
+      <c r="H42" s="49">
         <f>G42*E42</f>
-        <v>188256.59999999998</v>
-      </c>
-      <c r="I42" s="24" t="s">
+        <v>1400</v>
+      </c>
+      <c r="I42" s="48" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14879,22 +14868,22 @@
       <c r="C43" s="34" t="s">
         <v>810</v>
       </c>
-      <c r="D43" s="18" t="s">
-        <v>777</v>
+      <c r="D43" s="25" t="s">
+        <v>757</v>
       </c>
       <c r="E43" s="35">
-        <f>1784/13</f>
-        <v>137.23076923076923</v>
+        <f>(1784*0.15)*1.05</f>
+        <v>280.97999999999996</v>
       </c>
       <c r="F43" s="24" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G43" s="26">
-        <v>220.5</v>
+        <v>670</v>
       </c>
       <c r="H43" s="26">
         <f>G43*E43</f>
-        <v>30259.384615384613</v>
+        <v>188256.59999999998</v>
       </c>
       <c r="I43" s="24" t="s">
         <v>635</v>
@@ -14907,21 +14896,22 @@
       <c r="C44" s="34" t="s">
         <v>810</v>
       </c>
-      <c r="D44" s="25" t="s">
-        <v>819</v>
-      </c>
-      <c r="E44" s="24">
-        <v>1</v>
+      <c r="D44" s="18" t="s">
+        <v>777</v>
+      </c>
+      <c r="E44" s="35">
+        <f>1784/13</f>
+        <v>137.23076923076923</v>
       </c>
       <c r="F44" s="24" t="s">
         <v>760</v>
       </c>
       <c r="G44" s="26">
-        <v>43350</v>
+        <v>220.5</v>
       </c>
       <c r="H44" s="26">
         <f>G44*E44</f>
-        <v>43350</v>
+        <v>30259.384615384613</v>
       </c>
       <c r="I44" s="24" t="s">
         <v>635</v>
@@ -14931,27 +14921,27 @@
       <c r="B45" s="22">
         <v>42</v>
       </c>
-      <c r="C45" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D45" s="18" t="s">
-        <v>773</v>
-      </c>
-      <c r="E45" s="17">
-        <v>1</v>
-      </c>
-      <c r="F45" s="17" t="s">
+      <c r="C45" s="34" t="s">
+        <v>810</v>
+      </c>
+      <c r="D45" s="25" t="s">
+        <v>819</v>
+      </c>
+      <c r="E45" s="24">
+        <v>1</v>
+      </c>
+      <c r="F45" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G45" s="20">
-        <v>968004</v>
-      </c>
-      <c r="H45" s="20">
+      <c r="G45" s="26">
+        <v>43350</v>
+      </c>
+      <c r="H45" s="26">
         <f>G45*E45</f>
-        <v>968004</v>
-      </c>
-      <c r="I45" s="17" t="s">
-        <v>772</v>
+        <v>43350</v>
+      </c>
+      <c r="I45" s="24" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
@@ -14959,26 +14949,26 @@
         <v>43</v>
       </c>
       <c r="C46" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D46" s="25" t="s">
-        <v>804</v>
-      </c>
-      <c r="E46" s="24">
-        <v>1</v>
-      </c>
-      <c r="F46" s="24" t="s">
+        <v>809</v>
+      </c>
+      <c r="D46" s="31" t="s">
+        <v>860</v>
+      </c>
+      <c r="E46" s="27">
+        <v>1</v>
+      </c>
+      <c r="F46" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="G46" s="26">
-        <v>46600</v>
-      </c>
-      <c r="H46" s="26">
+      <c r="G46" s="36">
+        <v>24500</v>
+      </c>
+      <c r="H46" s="36">
         <f>G46*E46</f>
-        <v>46600</v>
-      </c>
-      <c r="I46" s="24" t="s">
-        <v>806</v>
+        <v>24500</v>
+      </c>
+      <c r="I46" s="27" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
@@ -14986,26 +14976,20 @@
         <v>44</v>
       </c>
       <c r="C47" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D47" s="25" t="s">
-        <v>807</v>
-      </c>
-      <c r="E47" s="24">
-        <v>1</v>
-      </c>
-      <c r="F47" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G47" s="26">
-        <v>8100</v>
-      </c>
-      <c r="H47" s="26">
+        <v>809</v>
+      </c>
+      <c r="D47" s="21" t="s">
+        <v>837</v>
+      </c>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="19"/>
+      <c r="H47" s="19">
         <f>G47*E47</f>
-        <v>8100</v>
-      </c>
-      <c r="I47" s="24" t="s">
-        <v>806</v>
+        <v>0</v>
+      </c>
+      <c r="I47" s="22" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.25">
@@ -15013,26 +14997,26 @@
         <v>45</v>
       </c>
       <c r="C48" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D48" s="25" t="s">
-        <v>822</v>
-      </c>
-      <c r="E48" s="24">
-        <v>1</v>
-      </c>
-      <c r="F48" s="24" t="s">
+        <v>809</v>
+      </c>
+      <c r="D48" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="E48" s="17">
+        <v>1</v>
+      </c>
+      <c r="F48" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G48" s="26">
-        <v>5000</v>
-      </c>
-      <c r="H48" s="26">
+      <c r="G48" s="20">
+        <v>968004</v>
+      </c>
+      <c r="H48" s="20">
         <f>G48*E48</f>
-        <v>5000</v>
-      </c>
-      <c r="I48" s="24" t="s">
-        <v>806</v>
+        <v>968004</v>
+      </c>
+      <c r="I48" s="17" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="49" spans="2:10" x14ac:dyDescent="0.25">
@@ -15043,7 +15027,7 @@
         <v>810</v>
       </c>
       <c r="D49" s="25" t="s">
-        <v>811</v>
+        <v>804</v>
       </c>
       <c r="E49" s="24">
         <v>1</v>
@@ -15052,11 +15036,11 @@
         <v>760</v>
       </c>
       <c r="G49" s="26">
-        <v>298777</v>
+        <v>46600</v>
       </c>
       <c r="H49" s="26">
         <f>G49*E49</f>
-        <v>298777</v>
+        <v>46600</v>
       </c>
       <c r="I49" s="24" t="s">
         <v>806</v>
@@ -15067,39 +15051,53 @@
         <v>47</v>
       </c>
       <c r="C50" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D50" s="21" t="s">
-        <v>793</v>
-      </c>
-      <c r="E50" s="22"/>
-      <c r="F50" s="22"/>
-      <c r="G50" s="19"/>
-      <c r="H50" s="19">
+        <v>810</v>
+      </c>
+      <c r="D50" s="25" t="s">
+        <v>807</v>
+      </c>
+      <c r="E50" s="24">
+        <v>1</v>
+      </c>
+      <c r="F50" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G50" s="26">
+        <v>8100</v>
+      </c>
+      <c r="H50" s="26">
         <f>G50*E50</f>
-        <v>0</v>
-      </c>
-      <c r="I50" s="22" t="s">
-        <v>419</v>
+        <v>8100</v>
+      </c>
+      <c r="I50" s="24" t="s">
+        <v>806</v>
       </c>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B51" s="22">
         <v>48</v>
       </c>
-      <c r="C51" s="17"/>
-      <c r="D51" s="21" t="s">
-        <v>855</v>
-      </c>
-      <c r="E51" s="22"/>
-      <c r="F51" s="22"/>
-      <c r="G51" s="19"/>
-      <c r="H51" s="19">
+      <c r="C51" s="17" t="s">
+        <v>810</v>
+      </c>
+      <c r="D51" s="25" t="s">
+        <v>822</v>
+      </c>
+      <c r="E51" s="24">
+        <v>1</v>
+      </c>
+      <c r="F51" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G51" s="26">
+        <v>5000</v>
+      </c>
+      <c r="H51" s="26">
         <f>G51*E51</f>
-        <v>0</v>
-      </c>
-      <c r="I51" s="22" t="s">
-        <v>801</v>
+        <v>5000</v>
+      </c>
+      <c r="I51" s="24" t="s">
+        <v>806</v>
       </c>
     </row>
     <row r="52" spans="2:10" x14ac:dyDescent="0.25">
@@ -15107,20 +15105,26 @@
         <v>49</v>
       </c>
       <c r="C52" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D52" s="21" t="s">
-        <v>794</v>
-      </c>
-      <c r="E52" s="22"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="19"/>
-      <c r="H52" s="19">
+        <v>810</v>
+      </c>
+      <c r="D52" s="25" t="s">
+        <v>811</v>
+      </c>
+      <c r="E52" s="24">
+        <v>1</v>
+      </c>
+      <c r="F52" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G52" s="26">
+        <v>298777</v>
+      </c>
+      <c r="H52" s="26">
         <f>G52*E52</f>
-        <v>0</v>
-      </c>
-      <c r="I52" s="17" t="s">
-        <v>801</v>
+        <v>298777</v>
+      </c>
+      <c r="I52" s="24" t="s">
+        <v>806</v>
       </c>
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.25">
@@ -15131,23 +15135,17 @@
         <v>809</v>
       </c>
       <c r="D53" s="21" t="s">
-        <v>786</v>
-      </c>
-      <c r="E53" s="22">
-        <v>1</v>
-      </c>
-      <c r="F53" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G53" s="19">
-        <v>791792.51</v>
-      </c>
+        <v>793</v>
+      </c>
+      <c r="E53" s="22"/>
+      <c r="F53" s="22"/>
+      <c r="G53" s="19"/>
       <c r="H53" s="19">
         <f>G53*E53</f>
-        <v>791792.51</v>
+        <v>0</v>
       </c>
       <c r="I53" s="22" t="s">
-        <v>785</v>
+        <v>419</v>
       </c>
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
@@ -15156,61 +15154,65 @@
       </c>
       <c r="C54" s="17"/>
       <c r="D54" s="21" t="s">
-        <v>857</v>
-      </c>
-      <c r="E54" s="22">
-        <v>6</v>
-      </c>
-      <c r="F54" s="22" t="s">
-        <v>760</v>
-      </c>
+        <v>855</v>
+      </c>
+      <c r="E54" s="22"/>
+      <c r="F54" s="22"/>
       <c r="G54" s="19"/>
       <c r="H54" s="19">
         <f>G54*E54</f>
         <v>0</v>
       </c>
-      <c r="I54" s="17" t="s">
-        <v>253</v>
+      <c r="I54" s="22" t="s">
+        <v>801</v>
       </c>
     </row>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B55" s="22">
         <v>52</v>
       </c>
-      <c r="C55" s="34"/>
-      <c r="D55" s="25" t="s">
-        <v>863</v>
-      </c>
-      <c r="E55" s="24"/>
-      <c r="F55" s="24"/>
-      <c r="G55" s="26"/>
-      <c r="H55" s="51">
+      <c r="C55" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D55" s="21" t="s">
+        <v>794</v>
+      </c>
+      <c r="E55" s="22"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="19"/>
+      <c r="H55" s="19">
         <f>G55*E55</f>
         <v>0</v>
       </c>
       <c r="I55" s="17" t="s">
-        <v>253</v>
+        <v>801</v>
       </c>
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B56" s="22"/>
-      <c r="C56" s="34"/>
-      <c r="D56" s="25" t="s">
-        <v>867</v>
-      </c>
-      <c r="E56" s="24">
-        <v>1</v>
-      </c>
-      <c r="F56" s="24" t="s">
+      <c r="B56" s="22">
+        <v>53</v>
+      </c>
+      <c r="C56" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D56" s="21" t="s">
+        <v>786</v>
+      </c>
+      <c r="E56" s="22">
+        <v>1</v>
+      </c>
+      <c r="F56" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="G56" s="26"/>
-      <c r="H56" s="51">
+      <c r="G56" s="19">
+        <v>791792.51</v>
+      </c>
+      <c r="H56" s="19">
         <f>G56*E56</f>
-        <v>0</v>
-      </c>
-      <c r="I56" s="17" t="s">
-        <v>253</v>
+        <v>791792.51</v>
+      </c>
+      <c r="I56" s="22" t="s">
+        <v>785</v>
       </c>
       <c r="J56" s="14" t="s">
         <v>868</v>
@@ -15218,7 +15220,7 @@
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B57" s="22">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C57" s="34"/>
       <c r="D57" s="25" t="s">

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 14:35
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="869">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2146" uniqueCount="870">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2628,10 +2628,13 @@
     <t>Frente para entrega do Meio fio</t>
   </si>
   <si>
-    <t>Mão de obra para concretagem do piso das docas de carregamento DPA IV</t>
-  </si>
-  <si>
     <t>Solicitar mais um orçamento do Erisvaldo</t>
+  </si>
+  <si>
+    <t>Mão de obra para concretagem do piso das docas de carregamento DPA IV (interno)</t>
+  </si>
+  <si>
+    <t>Solicitar um extra ao Erisvaldo</t>
   </si>
 </sst>
 </file>
@@ -2739,7 +2742,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2875,6 +2878,9 @@
     </xf>
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -13683,7 +13689,7 @@
     <col min="7" max="7" width="15.85546875" style="15" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" style="15" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.85546875" style="14" customWidth="1"/>
-    <col min="10" max="10" width="38.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="38.140625" style="52" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="16" style="14" customWidth="1"/>
     <col min="14" max="14" width="18.42578125" customWidth="1"/>
     <col min="15" max="15" width="25" customWidth="1"/>
@@ -13727,6 +13733,7 @@
       <c r="I3" t="s">
         <v>767</v>
       </c>
+      <c r="J3" s="52"/>
       <c r="P3" s="14" t="s">
         <v>831</v>
       </c>
@@ -13741,8 +13748,12 @@
       <c r="D4" s="25" t="s">
         <v>795</v>
       </c>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
+      <c r="E4" s="24">
+        <v>1</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>760</v>
+      </c>
       <c r="G4" s="26"/>
       <c r="H4" s="26">
         <f>G4*E4</f>
@@ -13892,8 +13903,12 @@
       <c r="D8" s="25" t="s">
         <v>863</v>
       </c>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
+      <c r="E8" s="24">
+        <v>6</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>760</v>
+      </c>
       <c r="G8" s="26"/>
       <c r="H8" s="51">
         <f>G8*E8</f>
@@ -13902,7 +13917,7 @@
       <c r="I8" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="J8" s="52" t="s">
         <v>814</v>
       </c>
       <c r="N8" s="44" t="s">
@@ -13923,7 +13938,7 @@
       </c>
       <c r="C9" s="34"/>
       <c r="D9" s="25" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="E9" s="24">
         <v>1</v>
@@ -13939,7 +13954,7 @@
       <c r="I9" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="J9" s="14" t="s">
+      <c r="J9" s="52" t="s">
         <v>812</v>
       </c>
       <c r="N9" s="41" t="s">
@@ -14601,7 +14616,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B33" s="22">
         <v>30</v>
       </c>
@@ -14622,7 +14637,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B34" s="22">
         <v>31</v>
       </c>
@@ -14643,7 +14658,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" s="22">
         <v>32</v>
       </c>
@@ -14671,7 +14686,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B36" s="22">
         <v>33</v>
       </c>
@@ -14699,7 +14714,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="22">
         <v>34</v>
       </c>
@@ -14727,7 +14742,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="22">
         <v>35</v>
       </c>
@@ -14754,7 +14769,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B39" s="22">
         <v>36</v>
       </c>
@@ -14782,7 +14797,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B40" s="22">
         <v>37</v>
       </c>
@@ -14809,7 +14824,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B41" s="22">
         <v>38</v>
       </c>
@@ -14836,7 +14851,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B42" s="22">
         <v>39</v>
       </c>
@@ -14861,7 +14876,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B43" s="22">
         <v>40</v>
       </c>
@@ -14889,7 +14904,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B44" s="22">
         <v>41</v>
       </c>
@@ -14917,7 +14932,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B45" s="22">
         <v>42</v>
       </c>
@@ -14943,8 +14958,11 @@
       <c r="I45" s="24" t="s">
         <v>635</v>
       </c>
-    </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J45" s="52" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" s="22">
         <v>43</v>
       </c>
@@ -14971,7 +14989,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B47" s="22">
         <v>44</v>
       </c>
@@ -14992,7 +15010,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B48" s="22">
         <v>45</v>
       </c>
@@ -15214,8 +15232,8 @@
       <c r="I56" s="22" t="s">
         <v>785</v>
       </c>
-      <c r="J56" s="14" t="s">
-        <v>868</v>
+      <c r="J56" s="52" t="s">
+        <v>867</v>
       </c>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 14:39
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2146" uniqueCount="870">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2148" uniqueCount="872">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2635,6 +2635,12 @@
   </si>
   <si>
     <t>Solicitar um extra ao Erisvaldo</t>
+  </si>
+  <si>
+    <t>Concreto para o radier do sistema de tratamento de esgoto do banheiro</t>
+  </si>
+  <si>
+    <t>Ferragem para o Sistema de tratamento de esgoto do banheiro</t>
   </si>
 </sst>
 </file>
@@ -2742,7 +2748,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2881,6 +2887,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3175,8 +3184,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I57" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:I57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I59" totalsRowShown="0" dataDxfId="16">
+  <autoFilter ref="B3:I59"/>
   <sortState ref="B4:I57">
     <sortCondition ref="I3:I57"/>
   </sortState>
@@ -13678,7 +13687,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R60"/>
+  <dimension ref="B1:R62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -13810,11 +13819,11 @@
       </c>
       <c r="P5" s="43">
         <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
-        <v>0.27698576114479873</v>
+        <v>0.25098381953474613</v>
       </c>
       <c r="Q5" s="45">
         <f>P5</f>
-        <v>0.27698576114479873</v>
+        <v>0.25098381953474613</v>
       </c>
       <c r="R5" t="s">
         <v>828</v>
@@ -13851,11 +13860,11 @@
       </c>
       <c r="P6" s="43">
         <f t="shared" si="0"/>
-        <v>0.22097165457378573</v>
+        <v>0.20022801765917683</v>
       </c>
       <c r="Q6" s="45">
         <f>P6+Q5</f>
-        <v>0.49795741571858443</v>
+        <v>0.45121183719392299</v>
       </c>
       <c r="R6" t="s">
         <v>828</v>
@@ -13892,7 +13901,7 @@
       </c>
       <c r="P7" s="43">
         <f t="shared" si="0"/>
-        <v>0.18289289121438398</v>
+        <v>0.16572388491386134</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
@@ -13925,11 +13934,11 @@
       </c>
       <c r="O8" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
-        <v>358477</v>
+        <v>729700</v>
       </c>
       <c r="P8" s="43">
         <f t="shared" si="0"/>
-        <v>0.10004294662581108</v>
+        <v>0.184526100765845</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
@@ -13966,7 +13975,7 @@
       </c>
       <c r="P9" s="43">
         <f t="shared" si="0"/>
-        <v>4.5768747357942119E-2</v>
+        <v>4.1472222181168403E-2</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
@@ -14002,7 +14011,7 @@
       </c>
       <c r="P10" s="43">
         <f t="shared" si="0"/>
-        <v>1.8568173328027054E-2</v>
+        <v>1.6825092540461589E-2</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
@@ -14040,7 +14049,7 @@
       </c>
       <c r="P11" s="43">
         <f t="shared" si="0"/>
-        <v>0.13564070619436175</v>
+        <v>0.12290748226315634</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
@@ -14140,7 +14149,7 @@
       </c>
       <c r="P14" s="43">
         <f t="shared" si="0"/>
-        <v>1.8568173328027054E-2</v>
+        <v>1.6825092540461589E-2</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
@@ -14178,7 +14187,7 @@
       </c>
       <c r="P15" s="43">
         <f t="shared" si="0"/>
-        <v>5.6094623286258327E-4</v>
+        <v>5.0828760112285663E-4</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
@@ -14437,7 +14446,7 @@
       </c>
       <c r="O24" s="42">
         <f>SUM(O5:O20)</f>
-        <v>3583231.1231375998</v>
+        <v>3954454.1231375998</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -15017,23 +15026,23 @@
       <c r="C48" s="17" t="s">
         <v>809</v>
       </c>
-      <c r="D48" s="18" t="s">
+      <c r="D48" s="31" t="s">
         <v>773</v>
       </c>
-      <c r="E48" s="17">
-        <v>1</v>
-      </c>
-      <c r="F48" s="17" t="s">
+      <c r="E48" s="27">
+        <v>1</v>
+      </c>
+      <c r="F48" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="G48" s="20">
+      <c r="G48" s="32">
         <v>968004</v>
       </c>
-      <c r="H48" s="20">
+      <c r="H48" s="32">
         <f>G48*E48</f>
         <v>968004</v>
       </c>
-      <c r="I48" s="17" t="s">
+      <c r="I48" s="27" t="s">
         <v>772</v>
       </c>
     </row>
@@ -15044,23 +15053,23 @@
       <c r="C49" s="17" t="s">
         <v>810</v>
       </c>
-      <c r="D49" s="25" t="s">
+      <c r="D49" s="47" t="s">
         <v>804</v>
       </c>
-      <c r="E49" s="24">
-        <v>1</v>
-      </c>
-      <c r="F49" s="24" t="s">
+      <c r="E49" s="48">
+        <v>1</v>
+      </c>
+      <c r="F49" s="48" t="s">
         <v>760</v>
       </c>
-      <c r="G49" s="26">
+      <c r="G49" s="49">
         <v>46600</v>
       </c>
-      <c r="H49" s="26">
+      <c r="H49" s="49">
         <f>G49*E49</f>
         <v>46600</v>
       </c>
-      <c r="I49" s="24" t="s">
+      <c r="I49" s="48" t="s">
         <v>806</v>
       </c>
     </row>
@@ -15071,23 +15080,23 @@
       <c r="C50" s="17" t="s">
         <v>810</v>
       </c>
-      <c r="D50" s="25" t="s">
+      <c r="D50" s="47" t="s">
         <v>807</v>
       </c>
-      <c r="E50" s="24">
-        <v>1</v>
-      </c>
-      <c r="F50" s="24" t="s">
+      <c r="E50" s="48">
+        <v>1</v>
+      </c>
+      <c r="F50" s="48" t="s">
         <v>760</v>
       </c>
-      <c r="G50" s="26">
+      <c r="G50" s="49">
         <v>8100</v>
       </c>
-      <c r="H50" s="26">
+      <c r="H50" s="49">
         <f>G50*E50</f>
         <v>8100</v>
       </c>
-      <c r="I50" s="24" t="s">
+      <c r="I50" s="48" t="s">
         <v>806</v>
       </c>
     </row>
@@ -15098,23 +15107,23 @@
       <c r="C51" s="17" t="s">
         <v>810</v>
       </c>
-      <c r="D51" s="25" t="s">
+      <c r="D51" s="47" t="s">
         <v>822</v>
       </c>
-      <c r="E51" s="24">
-        <v>1</v>
-      </c>
-      <c r="F51" s="24" t="s">
+      <c r="E51" s="48">
+        <v>1</v>
+      </c>
+      <c r="F51" s="48" t="s">
         <v>760</v>
       </c>
-      <c r="G51" s="26">
+      <c r="G51" s="49">
         <v>5000</v>
       </c>
-      <c r="H51" s="26">
+      <c r="H51" s="49">
         <f>G51*E51</f>
         <v>5000</v>
       </c>
-      <c r="I51" s="24" t="s">
+      <c r="I51" s="48" t="s">
         <v>806</v>
       </c>
     </row>
@@ -15125,23 +15134,23 @@
       <c r="C52" s="17" t="s">
         <v>810</v>
       </c>
-      <c r="D52" s="25" t="s">
+      <c r="D52" s="47" t="s">
         <v>811</v>
       </c>
-      <c r="E52" s="24">
-        <v>1</v>
-      </c>
-      <c r="F52" s="24" t="s">
+      <c r="E52" s="48">
+        <v>1</v>
+      </c>
+      <c r="F52" s="48" t="s">
         <v>760</v>
       </c>
-      <c r="G52" s="26">
-        <v>298777</v>
-      </c>
-      <c r="H52" s="26">
+      <c r="G52" s="49">
+        <v>670000</v>
+      </c>
+      <c r="H52" s="49">
         <f>G52*E52</f>
-        <v>298777</v>
-      </c>
-      <c r="I52" s="24" t="s">
+        <v>670000</v>
+      </c>
+      <c r="I52" s="48" t="s">
         <v>806</v>
       </c>
     </row>
@@ -15149,41 +15158,35 @@
       <c r="B53" s="22">
         <v>50</v>
       </c>
-      <c r="C53" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D53" s="21" t="s">
-        <v>793</v>
-      </c>
-      <c r="E53" s="22"/>
-      <c r="F53" s="22"/>
-      <c r="G53" s="19"/>
-      <c r="H53" s="19">
+      <c r="C53" s="17"/>
+      <c r="D53" s="25" t="s">
+        <v>870</v>
+      </c>
+      <c r="E53" s="24"/>
+      <c r="F53" s="24"/>
+      <c r="G53" s="53"/>
+      <c r="H53" s="53">
         <f>G53*E53</f>
         <v>0</v>
       </c>
-      <c r="I53" s="22" t="s">
-        <v>419</v>
-      </c>
+      <c r="I53" s="24"/>
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B54" s="22">
         <v>51</v>
       </c>
       <c r="C54" s="17"/>
-      <c r="D54" s="21" t="s">
-        <v>855</v>
-      </c>
-      <c r="E54" s="22"/>
-      <c r="F54" s="22"/>
-      <c r="G54" s="19"/>
-      <c r="H54" s="19">
+      <c r="D54" s="25" t="s">
+        <v>871</v>
+      </c>
+      <c r="E54" s="24"/>
+      <c r="F54" s="24"/>
+      <c r="G54" s="53"/>
+      <c r="H54" s="53">
         <f>G54*E54</f>
         <v>0</v>
       </c>
-      <c r="I54" s="22" t="s">
-        <v>801</v>
-      </c>
+      <c r="I54" s="24"/>
     </row>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B55" s="22">
@@ -15193,7 +15196,7 @@
         <v>809</v>
       </c>
       <c r="D55" s="21" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E55" s="22"/>
       <c r="F55" s="22"/>
@@ -15202,82 +15205,122 @@
         <f>G55*E55</f>
         <v>0</v>
       </c>
-      <c r="I55" s="17" t="s">
-        <v>801</v>
+      <c r="I55" s="22" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B56" s="22">
         <v>53</v>
       </c>
-      <c r="C56" s="17" t="s">
-        <v>809</v>
-      </c>
+      <c r="C56" s="17"/>
       <c r="D56" s="21" t="s">
-        <v>786</v>
-      </c>
-      <c r="E56" s="22">
-        <v>1</v>
-      </c>
-      <c r="F56" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G56" s="19">
-        <v>791792.51</v>
-      </c>
+        <v>855</v>
+      </c>
+      <c r="E56" s="22"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="19"/>
       <c r="H56" s="19">
         <f>G56*E56</f>
-        <v>791792.51</v>
+        <v>0</v>
       </c>
       <c r="I56" s="22" t="s">
-        <v>785</v>
-      </c>
-      <c r="J56" s="52" t="s">
-        <v>867</v>
+        <v>801</v>
       </c>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B57" s="22">
         <v>54</v>
       </c>
-      <c r="C57" s="34"/>
-      <c r="D57" s="25" t="s">
-        <v>864</v>
-      </c>
-      <c r="E57" s="24"/>
-      <c r="F57" s="24"/>
-      <c r="G57" s="26"/>
-      <c r="H57" s="51">
+      <c r="C57" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D57" s="21" t="s">
+        <v>794</v>
+      </c>
+      <c r="E57" s="22"/>
+      <c r="F57" s="22"/>
+      <c r="G57" s="19"/>
+      <c r="H57" s="19">
         <f>G57*E57</f>
         <v>0</v>
       </c>
-      <c r="I57" s="24"/>
+      <c r="I57" s="17" t="s">
+        <v>801</v>
+      </c>
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B58" s="24"/>
-      <c r="C58" s="34"/>
-      <c r="D58" s="25"/>
-      <c r="E58" s="24"/>
-      <c r="F58" s="24"/>
-      <c r="G58" s="26"/>
-      <c r="H58" s="51"/>
-      <c r="I58" s="24"/>
+      <c r="B58" s="22">
+        <v>55</v>
+      </c>
+      <c r="C58" s="17" t="s">
+        <v>809</v>
+      </c>
+      <c r="D58" s="21" t="s">
+        <v>786</v>
+      </c>
+      <c r="E58" s="22">
+        <v>1</v>
+      </c>
+      <c r="F58" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G58" s="19">
+        <v>791792.51</v>
+      </c>
+      <c r="H58" s="19">
+        <f>G58*E58</f>
+        <v>791792.51</v>
+      </c>
+      <c r="I58" s="22" t="s">
+        <v>785</v>
+      </c>
+      <c r="J58" s="52" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B59" s="24"/>
+      <c r="B59" s="22">
+        <v>56</v>
+      </c>
       <c r="C59" s="34"/>
-      <c r="D59" s="25"/>
+      <c r="D59" s="25" t="s">
+        <v>864</v>
+      </c>
       <c r="E59" s="24"/>
       <c r="F59" s="24"/>
       <c r="G59" s="26"/>
-      <c r="H59" s="51"/>
+      <c r="H59" s="51">
+        <f>G59*E59</f>
+        <v>0</v>
+      </c>
       <c r="I59" s="24"/>
     </row>
     <row r="60" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="D60" s="38"/>
-      <c r="H60" s="16">
+      <c r="B60" s="24"/>
+      <c r="C60" s="34"/>
+      <c r="D60" s="25"/>
+      <c r="E60" s="24"/>
+      <c r="F60" s="24"/>
+      <c r="G60" s="26"/>
+      <c r="H60" s="51"/>
+      <c r="I60" s="24"/>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B61" s="24"/>
+      <c r="C61" s="34"/>
+      <c r="D61" s="25"/>
+      <c r="E61" s="24"/>
+      <c r="F61" s="24"/>
+      <c r="G61" s="26"/>
+      <c r="H61" s="51"/>
+      <c r="I61" s="24"/>
+    </row>
+    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D62" s="38"/>
+      <c r="H62" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>3548296.6265428001</v>
+        <v>3919519.6265428001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 14:46
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2148" uniqueCount="872">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2154" uniqueCount="872">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2349,12 +2349,6 @@
     <t>Estrutura em pré moldado</t>
   </si>
   <si>
-    <t xml:space="preserve">Concreto para fundação rasa e profunda </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serviço de Hélice Contínua </t>
-  </si>
-  <si>
     <t>Fechamento Lateral</t>
   </si>
   <si>
@@ -2541,6 +2535,9 @@
     <t xml:space="preserve">Tubulação de drenagem pluvial </t>
   </si>
   <si>
+    <t xml:space="preserve">Concreto para fundação profunda </t>
+  </si>
+  <si>
     <t>Execução da fundação profunda</t>
   </si>
   <si>
@@ -2641,6 +2638,9 @@
   </si>
   <si>
     <t>Ferragem para o Sistema de tratamento de esgoto do banheiro</t>
+  </si>
+  <si>
+    <t>Concreto para fundação rasa</t>
   </si>
 </sst>
 </file>
@@ -3184,8 +3184,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I59" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:I59"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I60" totalsRowShown="0" dataDxfId="16">
+  <autoFilter ref="B3:I60"/>
   <sortState ref="B4:I57">
     <sortCondition ref="I3:I57"/>
   </sortState>
@@ -12667,7 +12667,7 @@
         <v>767</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
     </row>
     <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -12675,7 +12675,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="D4" s="27">
         <v>1</v>
@@ -12692,7 +12692,7 @@
         <v>421112</v>
       </c>
       <c r="H4" s="27" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="J4" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
@@ -12704,7 +12704,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="D5" s="22">
         <v>3</v>
@@ -12718,7 +12718,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="22" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="J5" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Piso",Tabela2[Preço Total])</f>
@@ -12730,7 +12730,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
@@ -12752,7 +12752,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
@@ -12774,7 +12774,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="D8" s="24">
         <v>10</v>
@@ -12800,7 +12800,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="D9" s="48">
         <v>600</v>
@@ -12828,7 +12828,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="D10" s="27">
         <v>1</v>
@@ -12844,7 +12844,7 @@
         <v>1056959.67</v>
       </c>
       <c r="H10" s="27" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="J10" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Terraplanagem",Tabela2[Preço Total])</f>
@@ -12856,7 +12856,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="D11" s="24"/>
       <c r="E11" s="24"/>
@@ -12866,7 +12866,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="24" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="J11" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Drenagem",Tabela2[Preço Total])</f>
@@ -12878,7 +12878,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="D12" s="22"/>
       <c r="E12" s="22"/>
@@ -12888,7 +12888,7 @@
         <v>0</v>
       </c>
       <c r="H12" s="22" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="J12" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Elétrica",Tabela2[Preço Total])</f>
@@ -12900,7 +12900,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="D13" s="22"/>
       <c r="E13" s="22"/>
@@ -12910,7 +12910,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="22" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="J13" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Pintura",Tabela2[Preço Total])</f>
@@ -12922,7 +12922,7 @@
         <v>11</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="D14" s="24"/>
       <c r="E14" s="24"/>
@@ -12932,7 +12932,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="24" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="J14" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Estrura Armazenamento",Tabela2[Preço Total])</f>
@@ -12944,7 +12944,7 @@
         <v>12</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="D15" s="24"/>
       <c r="E15" s="24"/>
@@ -12954,7 +12954,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="24" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="J15" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Serviço Prévio",Tabela2[Preço Total])</f>
@@ -12966,7 +12966,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="D16" s="24"/>
       <c r="E16" s="24"/>
@@ -12976,7 +12976,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="24" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="J16" s="39"/>
     </row>
@@ -12985,7 +12985,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D17" s="24"/>
       <c r="E17" s="24"/>
@@ -12995,7 +12995,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="24" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
@@ -13003,7 +13003,7 @@
         <v>15</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="D18" s="29">
         <v>4</v>
@@ -13027,7 +13027,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="D19" s="27">
         <v>1</v>
@@ -13046,7 +13046,7 @@
         <v>771</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
@@ -13060,7 +13060,7 @@
         <v>2100</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="F20" s="20"/>
       <c r="G20" s="20">
@@ -13071,7 +13071,7 @@
         <v>771</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
@@ -13085,7 +13085,7 @@
         <v>2300</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="F21" s="20"/>
       <c r="G21" s="20">
@@ -13101,7 +13101,7 @@
         <v>19</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="D22" s="27">
         <v>1</v>
@@ -13125,7 +13125,7 @@
         <v>20</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D23" s="33">
         <v>46.8</v>
@@ -13149,7 +13149,7 @@
         <v>21</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="D24" s="33">
         <v>37.200000000000003</v>
@@ -13173,7 +13173,7 @@
         <v>22</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
@@ -13191,7 +13191,7 @@
         <v>23</v>
       </c>
       <c r="C26" s="25" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="D26" s="24"/>
       <c r="E26" s="24"/>
@@ -13209,7 +13209,7 @@
         <v>24</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="24"/>
@@ -13227,7 +13227,7 @@
         <v>25</v>
       </c>
       <c r="C28" s="25" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="D28" s="24"/>
       <c r="E28" s="24"/>
@@ -13245,7 +13245,7 @@
         <v>26</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="D29" s="24"/>
       <c r="E29" s="24"/>
@@ -13288,7 +13288,7 @@
         <v>28</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="D31" s="33">
         <f>2000/13*2</f>
@@ -13319,7 +13319,7 @@
         <v>167</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="F32" s="32">
         <v>56.2</v>
@@ -13361,7 +13361,7 @@
         <v>31</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="D34" s="27">
         <v>315</v>
@@ -13409,7 +13409,7 @@
         <v>33</v>
       </c>
       <c r="C36" s="25" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="D36" s="24">
         <v>1</v>
@@ -13423,7 +13423,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="24" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
@@ -13431,7 +13431,7 @@
         <v>34</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="D37" s="24">
         <v>1</v>
@@ -13445,7 +13445,7 @@
         <v>0</v>
       </c>
       <c r="H37" s="24" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
@@ -13453,7 +13453,7 @@
         <v>35</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="D38" s="22"/>
       <c r="E38" s="22"/>
@@ -13471,7 +13471,7 @@
         <v>36</v>
       </c>
       <c r="C39" s="46" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="D39" s="27">
         <v>1455.89</v>
@@ -13487,7 +13487,7 @@
         <v>139619.85100000002</v>
       </c>
       <c r="H39" s="27" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
@@ -13495,7 +13495,7 @@
         <v>37</v>
       </c>
       <c r="C40" s="31" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="D40" s="27">
         <v>706.94</v>
@@ -13511,7 +13511,7 @@
         <v>67795.546000000002</v>
       </c>
       <c r="H40" s="27" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
@@ -13519,13 +13519,13 @@
         <v>38</v>
       </c>
       <c r="C41" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="D41" s="27">
         <v>44</v>
       </c>
       <c r="E41" s="27" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="F41" s="36">
         <v>95</v>
@@ -13535,7 +13535,7 @@
         <v>4180</v>
       </c>
       <c r="H41" s="27" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
@@ -13543,13 +13543,13 @@
         <v>39</v>
       </c>
       <c r="C42" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="D42" s="27">
         <v>3</v>
       </c>
       <c r="E42" s="27" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="F42" s="36">
         <v>35</v>
@@ -13559,7 +13559,7 @@
         <v>105</v>
       </c>
       <c r="H42" s="27" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
@@ -13567,7 +13567,7 @@
         <v>40</v>
       </c>
       <c r="C43" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="D43" s="27">
         <v>126</v>
@@ -13583,7 +13583,7 @@
         <v>3263.3999999999996</v>
       </c>
       <c r="H43" s="27" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
@@ -13591,7 +13591,7 @@
         <v>41</v>
       </c>
       <c r="C44" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="D44" s="27">
         <v>1</v>
@@ -13607,7 +13607,7 @@
         <v>1750</v>
       </c>
       <c r="H44" s="27" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
@@ -13615,7 +13615,7 @@
         <v>42</v>
       </c>
       <c r="C45" s="31" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="D45" s="27">
         <v>1</v>
@@ -13631,7 +13631,7 @@
         <v>157963.5</v>
       </c>
       <c r="H45" s="27" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
@@ -13639,7 +13639,7 @@
         <v>43</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="D46" s="24"/>
       <c r="E46" s="24"/>
@@ -13649,7 +13649,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="24" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
@@ -13687,7 +13687,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R62"/>
+  <dimension ref="B1:R63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -13698,7 +13698,7 @@
     <col min="7" max="7" width="15.85546875" style="15" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" style="15" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.85546875" style="14" customWidth="1"/>
-    <col min="10" max="10" width="38.140625" style="52" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="64.7109375" style="52" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="16" style="14" customWidth="1"/>
     <col min="14" max="14" width="18.42578125" customWidth="1"/>
     <col min="15" max="15" width="25" customWidth="1"/>
@@ -13709,12 +13709,12 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P1" s="14" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P2" s="14" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
     </row>
     <row r="3" spans="2:18" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -13722,7 +13722,7 @@
         <v>753</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="D3" t="s">
         <v>754</v>
@@ -13744,7 +13744,7 @@
       </c>
       <c r="J3" s="52"/>
       <c r="P3" s="14" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
@@ -13752,10 +13752,10 @@
         <v>1</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="E4" s="24">
         <v>1</v>
@@ -13769,19 +13769,19 @@
         <v>0</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="O4" s="14" t="s">
+        <v>821</v>
+      </c>
+      <c r="P4" s="14" t="s">
         <v>823</v>
       </c>
-      <c r="P4" s="14" t="s">
+      <c r="Q4" s="14" t="s">
+        <v>824</v>
+      </c>
+      <c r="R4" s="14" t="s">
         <v>825</v>
-      </c>
-      <c r="Q4" s="14" t="s">
-        <v>826</v>
-      </c>
-      <c r="R4" s="14" t="s">
-        <v>827</v>
       </c>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
@@ -13789,10 +13789,10 @@
         <v>2</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D5" s="31" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="E5" s="27">
         <v>1</v>
@@ -13808,7 +13808,7 @@
         <v>486032</v>
       </c>
       <c r="I5" s="27" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="N5" s="37" t="s">
         <v>772</v>
@@ -13826,7 +13826,7 @@
         <v>0.25098381953474613</v>
       </c>
       <c r="R5" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.25">
@@ -13835,7 +13835,7 @@
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="21" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="E6" s="22">
         <v>4</v>
@@ -13849,10 +13849,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="17" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="N6" s="44" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="O6" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Terraplanagem",Tabela24[Preço Total])</f>
@@ -13867,7 +13867,7 @@
         <v>0.45121183719392299</v>
       </c>
       <c r="R6" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
@@ -13876,7 +13876,7 @@
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="21" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="E7" s="22">
         <v>6</v>
@@ -13910,7 +13910,7 @@
       </c>
       <c r="C8" s="34"/>
       <c r="D8" s="25" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="E8" s="24">
         <v>6</v>
@@ -13927,10 +13927,10 @@
         <v>253</v>
       </c>
       <c r="J8" s="52" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="N8" s="44" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="O8" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
@@ -13947,7 +13947,7 @@
       </c>
       <c r="C9" s="34"/>
       <c r="D9" s="25" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="E9" s="24">
         <v>1</v>
@@ -13964,7 +13964,7 @@
         <v>253</v>
       </c>
       <c r="J9" s="52" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="N9" s="41" t="s">
         <v>771</v>
@@ -13983,10 +13983,10 @@
         <v>7</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="E10" s="24">
         <v>26</v>
@@ -14003,7 +14003,7 @@
         <v>643</v>
       </c>
       <c r="N10" s="41" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="O10" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
@@ -14019,10 +14019,10 @@
         <v>8</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D11" s="47" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="E11" s="48">
         <v>600</v>
@@ -14041,7 +14041,7 @@
         <v>643</v>
       </c>
       <c r="N11" s="40" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="O11" s="39">
         <f>SUMIF(Tabela24[Aplicação],"AVCB",Tabela24[Preço Total])</f>
@@ -14057,10 +14057,10 @@
         <v>9</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="E12" s="24"/>
       <c r="F12" s="24"/>
@@ -14089,10 +14089,10 @@
         <v>10</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="E13" s="27">
         <v>54</v>
@@ -14108,7 +14108,7 @@
         <v>13143.06</v>
       </c>
       <c r="I13" s="27" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="N13" s="40"/>
       <c r="O13" s="39"/>
@@ -14119,10 +14119,10 @@
         <v>11</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="E14" s="27">
         <v>30</v>
@@ -14138,10 +14138,10 @@
         <v>3591</v>
       </c>
       <c r="I14" s="27" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="N14" s="40" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="O14" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
@@ -14157,10 +14157,10 @@
         <v>12</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="E15" s="48">
         <v>390</v>
@@ -14176,7 +14176,7 @@
         <v>14865.499974</v>
       </c>
       <c r="I15" s="27" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="N15" s="40" t="s">
         <v>643</v>
@@ -14195,10 +14195,10 @@
         <v>13</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D16" s="31" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="E16" s="33">
         <f>(84*1.02)*2*1.02</f>
@@ -14215,7 +14215,7 @@
         <v>42541.456608</v>
       </c>
       <c r="I16" s="27" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="N16" s="40"/>
       <c r="O16" s="39"/>
@@ -14226,10 +14226,10 @@
         <v>14</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="E17" s="27">
         <f>84*7</f>
@@ -14246,7 +14246,7 @@
         <v>22412.599960800002</v>
       </c>
       <c r="I17" s="27" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="N17" s="40"/>
       <c r="O17" s="39"/>
@@ -14258,13 +14258,13 @@
       </c>
       <c r="C18" s="27"/>
       <c r="D18" s="31" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="E18" s="27">
         <v>30</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="G18" s="36">
         <v>24</v>
@@ -14274,7 +14274,7 @@
         <v>720</v>
       </c>
       <c r="I18" s="27" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="N18" s="40"/>
       <c r="O18" s="39"/>
@@ -14286,7 +14286,7 @@
       </c>
       <c r="C19" s="27"/>
       <c r="D19" s="31" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E19" s="27">
         <v>1</v>
@@ -14302,7 +14302,7 @@
         <v>860</v>
       </c>
       <c r="I19" s="27" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="N19" s="40" t="s">
         <v>576</v>
@@ -14321,10 +14321,10 @@
         <v>17</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="E20" s="24"/>
       <c r="F20" s="24" t="s">
@@ -14336,10 +14336,10 @@
         <v>0</v>
       </c>
       <c r="I20" s="24" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="N20" s="40" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="O20" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
@@ -14355,10 +14355,10 @@
         <v>18</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="E21" s="24"/>
       <c r="F21" s="24"/>
@@ -14368,7 +14368,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="N21" s="40"/>
       <c r="O21" s="39"/>
@@ -14379,10 +14379,10 @@
         <v>19</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="E22" s="24"/>
       <c r="F22" s="24"/>
@@ -14392,7 +14392,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="24" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="N22" s="40"/>
       <c r="O22" s="39"/>
@@ -14403,10 +14403,10 @@
         <v>20</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="E23" s="24">
         <v>1</v>
@@ -14418,7 +14418,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
@@ -14426,13 +14426,17 @@
         <v>21</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>796</v>
-      </c>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
+        <v>794</v>
+      </c>
+      <c r="E24" s="17">
+        <v>1</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>760</v>
+      </c>
       <c r="G24" s="20"/>
       <c r="H24" s="20">
         <f>G24*E24</f>
@@ -14442,7 +14446,7 @@
         <v>771</v>
       </c>
       <c r="N24" s="40" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="O24" s="42">
         <f>SUM(O5:O20)</f>
@@ -14454,13 +14458,15 @@
         <v>22</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D25" s="18" t="s">
         <v>769</v>
       </c>
       <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
+      <c r="F25" s="17" t="s">
+        <v>840</v>
+      </c>
       <c r="G25" s="20"/>
       <c r="H25" s="20">
         <f>G25*E25</f>
@@ -14469,6 +14475,9 @@
       <c r="I25" s="17" t="s">
         <v>771</v>
       </c>
+      <c r="J25" s="14" t="s">
+        <v>841</v>
+      </c>
       <c r="N25" s="40"/>
       <c r="O25" s="42"/>
     </row>
@@ -14477,13 +14486,15 @@
         <v>23</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D26" s="18" t="s">
         <v>770</v>
       </c>
       <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
+      <c r="F26" s="17" t="s">
+        <v>840</v>
+      </c>
       <c r="G26" s="20"/>
       <c r="H26" s="20">
         <f>G26*E26</f>
@@ -14492,16 +14503,19 @@
       <c r="I26" s="17" t="s">
         <v>771</v>
       </c>
+      <c r="J26" s="14" t="s">
+        <v>841</v>
+      </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B27" s="22">
         <v>24</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D27" s="31" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
       <c r="E27" s="27">
         <v>1</v>
@@ -14525,10 +14539,10 @@
         <v>25</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>774</v>
+        <v>836</v>
       </c>
       <c r="E28" s="17"/>
       <c r="F28" s="17"/>
@@ -14545,11 +14559,9 @@
       <c r="B29" s="22">
         <v>26</v>
       </c>
-      <c r="C29" s="17" t="s">
-        <v>809</v>
-      </c>
+      <c r="C29" s="17"/>
       <c r="D29" s="18" t="s">
-        <v>775</v>
+        <v>871</v>
       </c>
       <c r="E29" s="17"/>
       <c r="F29" s="17"/>
@@ -14558,28 +14570,26 @@
         <f>G29*E29</f>
         <v>0</v>
       </c>
-      <c r="I29" s="17" t="s">
-        <v>771</v>
-      </c>
+      <c r="I29" s="17"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B30" s="22">
         <v>27</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D30" s="21" t="s">
-        <v>779</v>
-      </c>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19">
+        <v>807</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>837</v>
+      </c>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="20">
         <f>G30*E30</f>
         <v>0</v>
       </c>
-      <c r="I30" s="22" t="s">
+      <c r="I30" s="17" t="s">
         <v>771</v>
       </c>
     </row>
@@ -14588,20 +14598,20 @@
         <v>28</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D31" s="25" t="s">
-        <v>787</v>
-      </c>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26">
+        <v>807</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>777</v>
+      </c>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19">
         <f>G31*E31</f>
         <v>0</v>
       </c>
-      <c r="I31" s="24" t="s">
-        <v>576</v>
+      <c r="I31" s="22" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.25">
@@ -14609,10 +14619,10 @@
         <v>29</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D32" s="25" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="E32" s="24"/>
       <c r="F32" s="24"/>
@@ -14630,10 +14640,10 @@
         <v>30</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D33" s="25" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="E33" s="24"/>
       <c r="F33" s="24"/>
@@ -14651,10 +14661,10 @@
         <v>31</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D34" s="25" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="E34" s="24"/>
       <c r="F34" s="24"/>
@@ -14671,28 +14681,21 @@
       <c r="B35" s="22">
         <v>32</v>
       </c>
-      <c r="C35" s="27" t="s">
-        <v>809</v>
-      </c>
-      <c r="D35" s="31" t="s">
-        <v>757</v>
-      </c>
-      <c r="E35" s="33">
-        <f>(2150*1.05)*0.15</f>
-        <v>338.625</v>
-      </c>
-      <c r="F35" s="27" t="s">
-        <v>759</v>
-      </c>
-      <c r="G35" s="32">
-        <v>670</v>
-      </c>
-      <c r="H35" s="32">
+      <c r="C35" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D35" s="25" t="s">
+        <v>788</v>
+      </c>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="26"/>
+      <c r="H35" s="26">
         <f>G35*E35</f>
-        <v>226878.75</v>
-      </c>
-      <c r="I35" s="27" t="s">
-        <v>635</v>
+        <v>0</v>
+      </c>
+      <c r="I35" s="24" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
@@ -14700,24 +14703,24 @@
         <v>33</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D36" s="31" t="s">
-        <v>777</v>
+        <v>757</v>
       </c>
       <c r="E36" s="33">
-        <f>(2150/13)*2</f>
-        <v>330.76923076923077</v>
+        <f>(2150*1.05)*0.15</f>
+        <v>338.625</v>
       </c>
       <c r="F36" s="27" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G36" s="32">
-        <v>220.5</v>
+        <v>670</v>
       </c>
       <c r="H36" s="32">
         <f>G36*E36</f>
-        <v>72934.61538461539</v>
+        <v>226878.75</v>
       </c>
       <c r="I36" s="27" t="s">
         <v>635</v>
@@ -14728,24 +14731,24 @@
         <v>34</v>
       </c>
       <c r="C37" s="27" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D37" s="31" t="s">
-        <v>758</v>
-      </c>
-      <c r="E37" s="27">
-        <f>2100/12</f>
-        <v>175</v>
+        <v>775</v>
+      </c>
+      <c r="E37" s="33">
+        <f>(2150/13)*2</f>
+        <v>330.76923076923077</v>
       </c>
       <c r="F37" s="27" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G37" s="32">
-        <v>56.2</v>
+        <v>220.5</v>
       </c>
       <c r="H37" s="32">
         <f>G37*E37</f>
-        <v>9835</v>
+        <v>72934.61538461539</v>
       </c>
       <c r="I37" s="27" t="s">
         <v>635</v>
@@ -14756,23 +14759,24 @@
         <v>35</v>
       </c>
       <c r="C38" s="27" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D38" s="31" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="E38" s="27">
-        <v>1000</v>
+        <f>2100/12</f>
+        <v>175</v>
       </c>
       <c r="F38" s="27" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="G38" s="32">
-        <v>7.3</v>
+        <v>56.2</v>
       </c>
       <c r="H38" s="32">
         <f>G38*E38</f>
-        <v>7300</v>
+        <v>9835</v>
       </c>
       <c r="I38" s="27" t="s">
         <v>635</v>
@@ -14782,27 +14786,26 @@
       <c r="B39" s="22">
         <v>36</v>
       </c>
-      <c r="C39" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D39" s="18" t="s">
-        <v>815</v>
-      </c>
-      <c r="E39" s="23">
-        <f>E35</f>
-        <v>338.625</v>
-      </c>
-      <c r="F39" s="17" t="s">
-        <v>766</v>
-      </c>
-      <c r="G39" s="20">
-        <v>50</v>
-      </c>
-      <c r="H39" s="20">
+      <c r="C39" s="27" t="s">
+        <v>807</v>
+      </c>
+      <c r="D39" s="31" t="s">
+        <v>762</v>
+      </c>
+      <c r="E39" s="27">
+        <v>1000</v>
+      </c>
+      <c r="F39" s="27" t="s">
+        <v>763</v>
+      </c>
+      <c r="G39" s="32">
+        <v>7.3</v>
+      </c>
+      <c r="H39" s="32">
         <f>G39*E39</f>
-        <v>16931.25</v>
-      </c>
-      <c r="I39" s="17" t="s">
+        <v>7300</v>
+      </c>
+      <c r="I39" s="27" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14811,25 +14814,26 @@
         <v>37</v>
       </c>
       <c r="C40" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D40" s="31" t="s">
-        <v>865</v>
-      </c>
-      <c r="E40" s="27">
-        <v>1</v>
-      </c>
-      <c r="F40" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="G40" s="32">
-        <v>53550</v>
-      </c>
-      <c r="H40" s="32">
+        <v>807</v>
+      </c>
+      <c r="D40" s="18" t="s">
+        <v>813</v>
+      </c>
+      <c r="E40" s="23">
+        <f>E36</f>
+        <v>338.625</v>
+      </c>
+      <c r="F40" s="17" t="s">
+        <v>766</v>
+      </c>
+      <c r="G40" s="20">
+        <v>50</v>
+      </c>
+      <c r="H40" s="20">
         <f>G40*E40</f>
-        <v>53550</v>
-      </c>
-      <c r="I40" s="27" t="s">
+        <v>16931.25</v>
+      </c>
+      <c r="I40" s="17" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14837,26 +14841,26 @@
       <c r="B41" s="22">
         <v>38</v>
       </c>
-      <c r="C41" s="34" t="s">
-        <v>810</v>
-      </c>
-      <c r="D41" s="47" t="s">
-        <v>820</v>
-      </c>
-      <c r="E41" s="48">
-        <v>110</v>
-      </c>
-      <c r="F41" s="48" t="s">
+      <c r="C41" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D41" s="31" t="s">
+        <v>864</v>
+      </c>
+      <c r="E41" s="27">
+        <v>1</v>
+      </c>
+      <c r="F41" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="G41" s="49">
-        <v>42.29</v>
-      </c>
-      <c r="H41" s="49">
+      <c r="G41" s="32">
+        <v>53550</v>
+      </c>
+      <c r="H41" s="32">
         <f>G41*E41</f>
-        <v>4651.8999999999996</v>
-      </c>
-      <c r="I41" s="48" t="s">
+        <v>53550</v>
+      </c>
+      <c r="I41" s="27" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14864,22 +14868,24 @@
       <c r="B42" s="22">
         <v>39</v>
       </c>
-      <c r="C42" s="34"/>
+      <c r="C42" s="34" t="s">
+        <v>808</v>
+      </c>
       <c r="D42" s="47" t="s">
-        <v>866</v>
+        <v>818</v>
       </c>
       <c r="E42" s="48">
-        <v>1</v>
+        <v>110</v>
       </c>
       <c r="F42" s="48" t="s">
         <v>760</v>
       </c>
       <c r="G42" s="49">
-        <v>1400</v>
+        <v>42.29</v>
       </c>
       <c r="H42" s="49">
         <f>G42*E42</f>
-        <v>1400</v>
+        <v>4651.8999999999996</v>
       </c>
       <c r="I42" s="48" t="s">
         <v>635</v>
@@ -14889,27 +14895,24 @@
       <c r="B43" s="22">
         <v>40</v>
       </c>
-      <c r="C43" s="34" t="s">
-        <v>810</v>
-      </c>
-      <c r="D43" s="25" t="s">
-        <v>757</v>
-      </c>
-      <c r="E43" s="35">
-        <f>(1784*0.15)*1.05</f>
-        <v>280.97999999999996</v>
-      </c>
-      <c r="F43" s="24" t="s">
-        <v>759</v>
-      </c>
-      <c r="G43" s="26">
-        <v>670</v>
-      </c>
-      <c r="H43" s="26">
+      <c r="C43" s="34"/>
+      <c r="D43" s="47" t="s">
+        <v>865</v>
+      </c>
+      <c r="E43" s="48">
+        <v>1</v>
+      </c>
+      <c r="F43" s="48" t="s">
+        <v>760</v>
+      </c>
+      <c r="G43" s="49">
+        <v>1400</v>
+      </c>
+      <c r="H43" s="49">
         <f>G43*E43</f>
-        <v>188256.59999999998</v>
-      </c>
-      <c r="I43" s="24" t="s">
+        <v>1400</v>
+      </c>
+      <c r="I43" s="48" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14918,24 +14921,24 @@
         <v>41</v>
       </c>
       <c r="C44" s="34" t="s">
-        <v>810</v>
-      </c>
-      <c r="D44" s="18" t="s">
-        <v>777</v>
+        <v>808</v>
+      </c>
+      <c r="D44" s="25" t="s">
+        <v>757</v>
       </c>
       <c r="E44" s="35">
-        <f>1784/13</f>
-        <v>137.23076923076923</v>
+        <f>(1784*0.15)*1.05</f>
+        <v>280.97999999999996</v>
       </c>
       <c r="F44" s="24" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G44" s="26">
-        <v>220.5</v>
+        <v>670</v>
       </c>
       <c r="H44" s="26">
         <f>G44*E44</f>
-        <v>30259.384615384613</v>
+        <v>188256.59999999998</v>
       </c>
       <c r="I44" s="24" t="s">
         <v>635</v>
@@ -14946,56 +14949,57 @@
         <v>42</v>
       </c>
       <c r="C45" s="34" t="s">
-        <v>810</v>
-      </c>
-      <c r="D45" s="25" t="s">
-        <v>819</v>
-      </c>
-      <c r="E45" s="24">
-        <v>1</v>
+        <v>808</v>
+      </c>
+      <c r="D45" s="18" t="s">
+        <v>775</v>
+      </c>
+      <c r="E45" s="35">
+        <f>1784/13</f>
+        <v>137.23076923076923</v>
       </c>
       <c r="F45" s="24" t="s">
         <v>760</v>
       </c>
       <c r="G45" s="26">
-        <v>43350</v>
+        <v>220.5</v>
       </c>
       <c r="H45" s="26">
         <f>G45*E45</f>
-        <v>43350</v>
+        <v>30259.384615384613</v>
       </c>
       <c r="I45" s="24" t="s">
         <v>635</v>
-      </c>
-      <c r="J45" s="52" t="s">
-        <v>869</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" s="22">
         <v>43</v>
       </c>
-      <c r="C46" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D46" s="31" t="s">
-        <v>860</v>
-      </c>
-      <c r="E46" s="27">
-        <v>1</v>
-      </c>
-      <c r="F46" s="27" t="s">
+      <c r="C46" s="34" t="s">
+        <v>808</v>
+      </c>
+      <c r="D46" s="25" t="s">
+        <v>817</v>
+      </c>
+      <c r="E46" s="24">
+        <v>1</v>
+      </c>
+      <c r="F46" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G46" s="36">
-        <v>24500</v>
-      </c>
-      <c r="H46" s="36">
+      <c r="G46" s="26">
+        <v>43350</v>
+      </c>
+      <c r="H46" s="26">
         <f>G46*E46</f>
-        <v>24500</v>
-      </c>
-      <c r="I46" s="27" t="s">
-        <v>772</v>
+        <v>43350</v>
+      </c>
+      <c r="I46" s="24" t="s">
+        <v>635</v>
+      </c>
+      <c r="J46" s="52" t="s">
+        <v>868</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
@@ -15003,19 +15007,25 @@
         <v>44</v>
       </c>
       <c r="C47" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D47" s="21" t="s">
-        <v>837</v>
-      </c>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="19">
+        <v>807</v>
+      </c>
+      <c r="D47" s="31" t="s">
+        <v>859</v>
+      </c>
+      <c r="E47" s="27">
+        <v>1</v>
+      </c>
+      <c r="F47" s="27" t="s">
+        <v>760</v>
+      </c>
+      <c r="G47" s="36">
+        <v>24500</v>
+      </c>
+      <c r="H47" s="36">
         <f>G47*E47</f>
-        <v>0</v>
-      </c>
-      <c r="I47" s="22" t="s">
+        <v>24500</v>
+      </c>
+      <c r="I47" s="27" t="s">
         <v>772</v>
       </c>
     </row>
@@ -15024,25 +15034,19 @@
         <v>45</v>
       </c>
       <c r="C48" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D48" s="31" t="s">
-        <v>773</v>
-      </c>
-      <c r="E48" s="27">
-        <v>1</v>
-      </c>
-      <c r="F48" s="27" t="s">
-        <v>760</v>
-      </c>
-      <c r="G48" s="32">
-        <v>968004</v>
-      </c>
-      <c r="H48" s="32">
+        <v>807</v>
+      </c>
+      <c r="D48" s="21" t="s">
+        <v>835</v>
+      </c>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="19"/>
+      <c r="H48" s="19">
         <f>G48*E48</f>
-        <v>968004</v>
-      </c>
-      <c r="I48" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="I48" s="22" t="s">
         <v>772</v>
       </c>
     </row>
@@ -15051,26 +15055,26 @@
         <v>46</v>
       </c>
       <c r="C49" s="17" t="s">
-        <v>810</v>
-      </c>
-      <c r="D49" s="47" t="s">
-        <v>804</v>
-      </c>
-      <c r="E49" s="48">
-        <v>1</v>
-      </c>
-      <c r="F49" s="48" t="s">
+        <v>807</v>
+      </c>
+      <c r="D49" s="31" t="s">
+        <v>773</v>
+      </c>
+      <c r="E49" s="27">
+        <v>1</v>
+      </c>
+      <c r="F49" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="G49" s="49">
-        <v>46600</v>
-      </c>
-      <c r="H49" s="49">
+      <c r="G49" s="32">
+        <v>968004</v>
+      </c>
+      <c r="H49" s="32">
         <f>G49*E49</f>
-        <v>46600</v>
-      </c>
-      <c r="I49" s="48" t="s">
-        <v>806</v>
+        <v>968004</v>
+      </c>
+      <c r="I49" s="27" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.25">
@@ -15078,10 +15082,10 @@
         <v>47</v>
       </c>
       <c r="C50" s="17" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="D50" s="47" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="E50" s="48">
         <v>1</v>
@@ -15090,14 +15094,14 @@
         <v>760</v>
       </c>
       <c r="G50" s="49">
-        <v>8100</v>
+        <v>46600</v>
       </c>
       <c r="H50" s="49">
         <f>G50*E50</f>
-        <v>8100</v>
+        <v>46600</v>
       </c>
       <c r="I50" s="48" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.25">
@@ -15105,10 +15109,10 @@
         <v>48</v>
       </c>
       <c r="C51" s="17" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="D51" s="47" t="s">
-        <v>822</v>
+        <v>805</v>
       </c>
       <c r="E51" s="48">
         <v>1</v>
@@ -15117,14 +15121,14 @@
         <v>760</v>
       </c>
       <c r="G51" s="49">
-        <v>5000</v>
+        <v>8100</v>
       </c>
       <c r="H51" s="49">
         <f>G51*E51</f>
-        <v>5000</v>
+        <v>8100</v>
       </c>
       <c r="I51" s="48" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="52" spans="2:10" x14ac:dyDescent="0.25">
@@ -15132,10 +15136,10 @@
         <v>49</v>
       </c>
       <c r="C52" s="17" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="D52" s="47" t="s">
-        <v>811</v>
+        <v>820</v>
       </c>
       <c r="E52" s="48">
         <v>1</v>
@@ -15144,32 +15148,42 @@
         <v>760</v>
       </c>
       <c r="G52" s="49">
-        <v>670000</v>
+        <v>5000</v>
       </c>
       <c r="H52" s="49">
         <f>G52*E52</f>
-        <v>670000</v>
+        <v>5000</v>
       </c>
       <c r="I52" s="48" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B53" s="22">
         <v>50</v>
       </c>
-      <c r="C53" s="17"/>
-      <c r="D53" s="25" t="s">
-        <v>870</v>
-      </c>
-      <c r="E53" s="24"/>
-      <c r="F53" s="24"/>
-      <c r="G53" s="53"/>
-      <c r="H53" s="53">
+      <c r="C53" s="17" t="s">
+        <v>808</v>
+      </c>
+      <c r="D53" s="47" t="s">
+        <v>809</v>
+      </c>
+      <c r="E53" s="48">
+        <v>1</v>
+      </c>
+      <c r="F53" s="48" t="s">
+        <v>760</v>
+      </c>
+      <c r="G53" s="49">
+        <v>670000</v>
+      </c>
+      <c r="H53" s="49">
         <f>G53*E53</f>
-        <v>0</v>
-      </c>
-      <c r="I53" s="24"/>
+        <v>670000</v>
+      </c>
+      <c r="I53" s="48" t="s">
+        <v>804</v>
+      </c>
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B54" s="22">
@@ -15177,7 +15191,7 @@
       </c>
       <c r="C54" s="17"/>
       <c r="D54" s="25" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="E54" s="24"/>
       <c r="F54" s="24"/>
@@ -15192,30 +15206,28 @@
       <c r="B55" s="22">
         <v>52</v>
       </c>
-      <c r="C55" s="17" t="s">
-        <v>809</v>
-      </c>
-      <c r="D55" s="21" t="s">
-        <v>793</v>
-      </c>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
-      <c r="G55" s="19"/>
-      <c r="H55" s="19">
+      <c r="C55" s="17"/>
+      <c r="D55" s="25" t="s">
+        <v>870</v>
+      </c>
+      <c r="E55" s="24"/>
+      <c r="F55" s="24"/>
+      <c r="G55" s="53"/>
+      <c r="H55" s="53">
         <f>G55*E55</f>
         <v>0</v>
       </c>
-      <c r="I55" s="22" t="s">
-        <v>419</v>
-      </c>
+      <c r="I55" s="24"/>
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B56" s="22">
         <v>53</v>
       </c>
-      <c r="C56" s="17"/>
+      <c r="C56" s="17" t="s">
+        <v>807</v>
+      </c>
       <c r="D56" s="21" t="s">
-        <v>855</v>
+        <v>791</v>
       </c>
       <c r="E56" s="22"/>
       <c r="F56" s="22"/>
@@ -15225,18 +15237,16 @@
         <v>0</v>
       </c>
       <c r="I56" s="22" t="s">
-        <v>801</v>
+        <v>419</v>
       </c>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B57" s="22">
         <v>54</v>
       </c>
-      <c r="C57" s="17" t="s">
-        <v>809</v>
-      </c>
+      <c r="C57" s="17"/>
       <c r="D57" s="21" t="s">
-        <v>794</v>
+        <v>854</v>
       </c>
       <c r="E57" s="22"/>
       <c r="F57" s="22"/>
@@ -15245,8 +15255,8 @@
         <f>G57*E57</f>
         <v>0</v>
       </c>
-      <c r="I57" s="17" t="s">
-        <v>801</v>
+      <c r="I57" s="22" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.25">
@@ -15254,56 +15264,67 @@
         <v>55</v>
       </c>
       <c r="C58" s="17" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="D58" s="21" t="s">
-        <v>786</v>
-      </c>
-      <c r="E58" s="22">
-        <v>1</v>
-      </c>
-      <c r="F58" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G58" s="19">
-        <v>791792.51</v>
-      </c>
+        <v>792</v>
+      </c>
+      <c r="E58" s="22"/>
+      <c r="F58" s="22"/>
+      <c r="G58" s="19"/>
       <c r="H58" s="19">
         <f>G58*E58</f>
-        <v>791792.51</v>
-      </c>
-      <c r="I58" s="22" t="s">
-        <v>785</v>
-      </c>
-      <c r="J58" s="52" t="s">
-        <v>867</v>
+        <v>0</v>
+      </c>
+      <c r="I58" s="17" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B59" s="22">
         <v>56</v>
       </c>
-      <c r="C59" s="34"/>
-      <c r="D59" s="25" t="s">
-        <v>864</v>
-      </c>
-      <c r="E59" s="24"/>
-      <c r="F59" s="24"/>
-      <c r="G59" s="26"/>
-      <c r="H59" s="51">
+      <c r="C59" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D59" s="21" t="s">
+        <v>784</v>
+      </c>
+      <c r="E59" s="22">
+        <v>1</v>
+      </c>
+      <c r="F59" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G59" s="19">
+        <v>791792.51</v>
+      </c>
+      <c r="H59" s="19">
         <f>G59*E59</f>
-        <v>0</v>
-      </c>
-      <c r="I59" s="24"/>
+        <v>791792.51</v>
+      </c>
+      <c r="I59" s="22" t="s">
+        <v>783</v>
+      </c>
+      <c r="J59" s="52" t="s">
+        <v>866</v>
+      </c>
     </row>
     <row r="60" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B60" s="24"/>
+      <c r="B60" s="22">
+        <v>57</v>
+      </c>
       <c r="C60" s="34"/>
-      <c r="D60" s="25"/>
+      <c r="D60" s="25" t="s">
+        <v>863</v>
+      </c>
       <c r="E60" s="24"/>
       <c r="F60" s="24"/>
       <c r="G60" s="26"/>
-      <c r="H60" s="51"/>
+      <c r="H60" s="51">
+        <f>G60*E60</f>
+        <v>0</v>
+      </c>
       <c r="I60" s="24"/>
     </row>
     <row r="61" spans="2:10" x14ac:dyDescent="0.25">
@@ -15317,8 +15338,18 @@
       <c r="I61" s="24"/>
     </row>
     <row r="62" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="D62" s="38"/>
-      <c r="H62" s="16">
+      <c r="B62" s="24"/>
+      <c r="C62" s="34"/>
+      <c r="D62" s="25"/>
+      <c r="E62" s="24"/>
+      <c r="F62" s="24"/>
+      <c r="G62" s="26"/>
+      <c r="H62" s="51"/>
+      <c r="I62" s="24"/>
+    </row>
+    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D63" s="38"/>
+      <c r="H63" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
         <v>3919519.6265428001</v>
       </c>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 14:48
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2154" uniqueCount="872">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2157" uniqueCount="872">
   <si>
     <t>Código EAP</t>
   </si>
@@ -13819,11 +13819,11 @@
       </c>
       <c r="P5" s="43">
         <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
-        <v>0.25098381953474613</v>
+        <v>0.24370928566975575</v>
       </c>
       <c r="Q5" s="45">
         <f>P5</f>
-        <v>0.25098381953474613</v>
+        <v>0.24370928566975575</v>
       </c>
       <c r="R5" t="s">
         <v>826</v>
@@ -13860,11 +13860,11 @@
       </c>
       <c r="P6" s="43">
         <f t="shared" si="0"/>
-        <v>0.20022801765917683</v>
+        <v>0.19442459376563009</v>
       </c>
       <c r="Q6" s="45">
         <f>P6+Q5</f>
-        <v>0.45121183719392299</v>
+        <v>0.43813387943538584</v>
       </c>
       <c r="R6" t="s">
         <v>826</v>
@@ -13901,7 +13901,7 @@
       </c>
       <c r="P7" s="43">
         <f t="shared" si="0"/>
-        <v>0.16572388491386134</v>
+        <v>0.16092053139378809</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="P8" s="43">
         <f t="shared" si="0"/>
-        <v>0.184526100765845</v>
+        <v>0.17917778241016738</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
@@ -13971,11 +13971,11 @@
       </c>
       <c r="O9" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Fundação",Tabela24[Preço Total])</f>
-        <v>164000</v>
+        <v>282037.40000000002</v>
       </c>
       <c r="P9" s="43">
         <f t="shared" si="0"/>
-        <v>4.1472222181168403E-2</v>
+        <v>6.9254263243427913E-2</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
@@ -14011,7 +14011,7 @@
       </c>
       <c r="P10" s="43">
         <f t="shared" si="0"/>
-        <v>1.6825092540461589E-2</v>
+        <v>1.6337432795327143E-2</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
@@ -14049,7 +14049,7 @@
       </c>
       <c r="P11" s="43">
         <f t="shared" si="0"/>
-        <v>0.12290748226315634</v>
+        <v>0.11934512257143823</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
@@ -14149,7 +14149,7 @@
       </c>
       <c r="P14" s="43">
         <f t="shared" si="0"/>
-        <v>1.6825092540461589E-2</v>
+        <v>1.6337432795327143E-2</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
@@ -14187,7 +14187,7 @@
       </c>
       <c r="P15" s="43">
         <f t="shared" si="0"/>
-        <v>5.0828760112285663E-4</v>
+        <v>4.9355535513832599E-4</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
@@ -14428,21 +14428,23 @@
       <c r="C24" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="31" t="s">
         <v>794</v>
       </c>
-      <c r="E24" s="17">
-        <v>1</v>
-      </c>
-      <c r="F24" s="17" t="s">
+      <c r="E24" s="27">
+        <v>1</v>
+      </c>
+      <c r="F24" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20">
+      <c r="G24" s="32">
+        <v>6000</v>
+      </c>
+      <c r="H24" s="32">
         <f>G24*E24</f>
-        <v>0</v>
-      </c>
-      <c r="I24" s="17" t="s">
+        <v>6000</v>
+      </c>
+      <c r="I24" s="27" t="s">
         <v>771</v>
       </c>
       <c r="N24" s="40" t="s">
@@ -14450,7 +14452,7 @@
       </c>
       <c r="O24" s="42">
         <f>SUM(O5:O20)</f>
-        <v>3954454.1231375998</v>
+        <v>4072491.5231375997</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -14463,7 +14465,9 @@
       <c r="D25" s="18" t="s">
         <v>769</v>
       </c>
-      <c r="E25" s="17"/>
+      <c r="E25" s="17">
+        <v>4100</v>
+      </c>
       <c r="F25" s="17" t="s">
         <v>839</v>
       </c>
@@ -14491,7 +14495,9 @@
       <c r="D26" s="18" t="s">
         <v>770</v>
       </c>
-      <c r="E26" s="17"/>
+      <c r="E26" s="17">
+        <v>4000</v>
+      </c>
       <c r="F26" s="17" t="s">
         <v>839</v>
       </c>
@@ -14541,17 +14547,23 @@
       <c r="C28" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="D28" s="31" t="s">
         <v>871</v>
       </c>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20">
+      <c r="E28" s="27">
+        <v>99.22</v>
+      </c>
+      <c r="F28" s="27" t="s">
+        <v>759</v>
+      </c>
+      <c r="G28" s="32">
+        <v>670</v>
+      </c>
+      <c r="H28" s="32">
         <f>G28*E28</f>
-        <v>0</v>
-      </c>
-      <c r="I28" s="17" t="s">
+        <v>66477.399999999994</v>
+      </c>
+      <c r="I28" s="27" t="s">
         <v>771</v>
       </c>
     </row>
@@ -14560,17 +14572,25 @@
         <v>26</v>
       </c>
       <c r="C29" s="17"/>
-      <c r="D29" s="18" t="s">
+      <c r="D29" s="31" t="s">
         <v>870</v>
       </c>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="20"/>
-      <c r="H29" s="20">
+      <c r="E29" s="27">
+        <v>68</v>
+      </c>
+      <c r="F29" s="27" t="s">
+        <v>759</v>
+      </c>
+      <c r="G29" s="32">
+        <v>670</v>
+      </c>
+      <c r="H29" s="32">
         <f>G29*E29</f>
-        <v>0</v>
-      </c>
-      <c r="I29" s="17"/>
+        <v>45560</v>
+      </c>
+      <c r="I29" s="27" t="s">
+        <v>771</v>
+      </c>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B30" s="22">
@@ -15351,7 +15371,7 @@
       <c r="D63" s="38"/>
       <c r="H63" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>3919519.6265428001</v>
+        <v>4037557.0265427995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 14:50
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2158" uniqueCount="872">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2159" uniqueCount="873">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2641,6 +2641,9 @@
   </si>
   <si>
     <t xml:space="preserve">Concreto FCK 30 Brita 0 Slump 24±2 fundação profunda </t>
+  </si>
+  <si>
+    <t>Cercado para o sistema de trantamento de esgoto do banheiro</t>
   </si>
 </sst>
 </file>
@@ -3184,8 +3187,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I60" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:I60"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I61" totalsRowShown="0" dataDxfId="16">
+  <autoFilter ref="B3:I61"/>
   <sortState ref="B4:I57">
     <sortCondition ref="I3:I57"/>
   </sortState>
@@ -13687,7 +13690,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R63"/>
+  <dimension ref="B1:R64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -13819,11 +13822,11 @@
       </c>
       <c r="P5" s="43">
         <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
-        <v>0.24037443391160107</v>
+        <v>0.24292488569525772</v>
       </c>
       <c r="Q5" s="45">
         <f>P5</f>
-        <v>0.24037443391160107</v>
+        <v>0.24292488569525772</v>
       </c>
       <c r="R5" t="s">
         <v>826</v>
@@ -13860,11 +13863,11 @@
       </c>
       <c r="P6" s="43">
         <f t="shared" si="0"/>
-        <v>0.19176414036285569</v>
+        <v>0.19379882094793693</v>
       </c>
       <c r="Q6" s="45">
         <f>P6+Q5</f>
-        <v>0.43213857427445679</v>
+        <v>0.43672370664319465</v>
       </c>
       <c r="R6" t="s">
         <v>826</v>
@@ -13897,11 +13900,11 @@
       </c>
       <c r="O7" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Piso",Tabela24[Preço Total])</f>
-        <v>655347.5</v>
+        <v>611997.5</v>
       </c>
       <c r="P7" s="43">
         <f t="shared" si="0"/>
-        <v>0.15871853849242218</v>
+        <v>0.14979226555589042</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
@@ -13938,7 +13941,7 @@
       </c>
       <c r="P8" s="43">
         <f t="shared" si="0"/>
-        <v>0.17672596223823309</v>
+        <v>0.17860108280856254</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
@@ -13975,7 +13978,7 @@
       </c>
       <c r="P9" s="43">
         <f t="shared" si="0"/>
-        <v>8.1990335437343589E-2</v>
+        <v>8.286027985637312E-2</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
@@ -14011,7 +14014,7 @@
       </c>
       <c r="P10" s="43">
         <f t="shared" si="0"/>
-        <v>1.6113875796538599E-2</v>
+        <v>1.6284849317300034E-2</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
@@ -14049,7 +14052,7 @@
       </c>
       <c r="P11" s="43">
         <f t="shared" si="0"/>
-        <v>0.11771203628693012</v>
+        <v>0.1189609996979735</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
@@ -14149,7 +14152,7 @@
       </c>
       <c r="P14" s="43">
         <f t="shared" si="0"/>
-        <v>1.6113875796538599E-2</v>
+        <v>1.6284849317300034E-2</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
@@ -14187,7 +14190,7 @@
       </c>
       <c r="P15" s="43">
         <f t="shared" si="0"/>
-        <v>4.8680167753713651E-4</v>
+        <v>4.9196680340579787E-4</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
@@ -14452,7 +14455,7 @@
       </c>
       <c r="O24" s="42">
         <f>SUM(O5:O20)</f>
-        <v>4128991.5231375997</v>
+        <v>4085641.5231375997</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -15014,12 +15017,10 @@
       <c r="F46" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G46" s="26">
-        <v>43350</v>
-      </c>
+      <c r="G46" s="26"/>
       <c r="H46" s="26">
         <f>G46*E46</f>
-        <v>43350</v>
+        <v>0</v>
       </c>
       <c r="I46" s="24" t="s">
         <v>635</v>
@@ -15246,33 +15247,29 @@
       <c r="I55" s="24"/>
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B56" s="22">
-        <v>53</v>
-      </c>
-      <c r="C56" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D56" s="21" t="s">
-        <v>791</v>
-      </c>
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="19">
+      <c r="B56" s="22"/>
+      <c r="C56" s="17"/>
+      <c r="D56" s="25" t="s">
+        <v>872</v>
+      </c>
+      <c r="E56" s="24"/>
+      <c r="F56" s="24"/>
+      <c r="G56" s="53"/>
+      <c r="H56" s="53">
         <f>G56*E56</f>
         <v>0</v>
       </c>
-      <c r="I56" s="22" t="s">
-        <v>419</v>
-      </c>
+      <c r="I56" s="24"/>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B57" s="22">
-        <v>54</v>
-      </c>
-      <c r="C57" s="17"/>
+        <v>53</v>
+      </c>
+      <c r="C57" s="17" t="s">
+        <v>807</v>
+      </c>
       <c r="D57" s="21" t="s">
-        <v>853</v>
+        <v>791</v>
       </c>
       <c r="E57" s="22"/>
       <c r="F57" s="22"/>
@@ -15282,18 +15279,16 @@
         <v>0</v>
       </c>
       <c r="I57" s="22" t="s">
-        <v>799</v>
+        <v>419</v>
       </c>
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B58" s="22">
-        <v>55</v>
-      </c>
-      <c r="C58" s="17" t="s">
-        <v>807</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="C58" s="17"/>
       <c r="D58" s="21" t="s">
-        <v>792</v>
+        <v>853</v>
       </c>
       <c r="E58" s="22"/>
       <c r="F58" s="22"/>
@@ -15302,65 +15297,76 @@
         <f>G58*E58</f>
         <v>0</v>
       </c>
-      <c r="I58" s="17" t="s">
+      <c r="I58" s="22" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B59" s="22">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C59" s="17" t="s">
         <v>807</v>
       </c>
       <c r="D59" s="21" t="s">
-        <v>784</v>
-      </c>
-      <c r="E59" s="22">
-        <v>1</v>
-      </c>
-      <c r="F59" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G59" s="19">
-        <v>791792.51</v>
-      </c>
+        <v>792</v>
+      </c>
+      <c r="E59" s="22"/>
+      <c r="F59" s="22"/>
+      <c r="G59" s="19"/>
       <c r="H59" s="19">
         <f>G59*E59</f>
-        <v>791792.51</v>
-      </c>
-      <c r="I59" s="22" t="s">
-        <v>783</v>
-      </c>
-      <c r="J59" s="52" t="s">
-        <v>865</v>
+        <v>0</v>
+      </c>
+      <c r="I59" s="17" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="60" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B60" s="22">
+        <v>56</v>
+      </c>
+      <c r="C60" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D60" s="21" t="s">
+        <v>784</v>
+      </c>
+      <c r="E60" s="22">
+        <v>1</v>
+      </c>
+      <c r="F60" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G60" s="19">
+        <v>791792.51</v>
+      </c>
+      <c r="H60" s="19">
+        <f>G60*E60</f>
+        <v>791792.51</v>
+      </c>
+      <c r="I60" s="22" t="s">
+        <v>783</v>
+      </c>
+      <c r="J60" s="52" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B61" s="22">
         <v>57</v>
       </c>
-      <c r="C60" s="34"/>
-      <c r="D60" s="25" t="s">
+      <c r="C61" s="34"/>
+      <c r="D61" s="25" t="s">
         <v>862</v>
       </c>
-      <c r="E60" s="24"/>
-      <c r="F60" s="24"/>
-      <c r="G60" s="26"/>
-      <c r="H60" s="51">
-        <f>G60*E60</f>
-        <v>0</v>
-      </c>
-      <c r="I60" s="24"/>
-    </row>
-    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B61" s="24"/>
-      <c r="C61" s="34"/>
-      <c r="D61" s="25"/>
       <c r="E61" s="24"/>
       <c r="F61" s="24"/>
       <c r="G61" s="26"/>
-      <c r="H61" s="51"/>
+      <c r="H61" s="51">
+        <f>G61*E61</f>
+        <v>0</v>
+      </c>
       <c r="I61" s="24"/>
     </row>
     <row r="62" spans="2:10" x14ac:dyDescent="0.25">
@@ -15374,10 +15380,20 @@
       <c r="I62" s="24"/>
     </row>
     <row r="63" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="D63" s="38"/>
-      <c r="H63" s="16">
+      <c r="B63" s="24"/>
+      <c r="C63" s="34"/>
+      <c r="D63" s="25"/>
+      <c r="E63" s="24"/>
+      <c r="F63" s="24"/>
+      <c r="G63" s="26"/>
+      <c r="H63" s="51"/>
+      <c r="I63" s="24"/>
+    </row>
+    <row r="64" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D64" s="38"/>
+      <c r="H64" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>4094057.0265427995</v>
+        <v>4050707.0265427995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 15:22
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2159" uniqueCount="873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2160" uniqueCount="874">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2644,6 +2644,9 @@
   </si>
   <si>
     <t>Cercado para o sistema de trantamento de esgoto do banheiro</t>
+  </si>
+  <si>
+    <t>Cabo para ligação do sistema de tratamento de esgoto do banheiro</t>
   </si>
 </sst>
 </file>
@@ -3187,8 +3190,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I61" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:I61"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I62" totalsRowShown="0" dataDxfId="16">
+  <autoFilter ref="B3:I62"/>
   <sortState ref="B4:I57">
     <sortCondition ref="I3:I57"/>
   </sortState>
@@ -13690,7 +13693,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R64"/>
+  <dimension ref="B1:R65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -15285,12 +15288,10 @@
       </c>
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B58" s="22">
-        <v>55</v>
-      </c>
+      <c r="B58" s="22"/>
       <c r="C58" s="17"/>
       <c r="D58" s="21" t="s">
-        <v>853</v>
+        <v>873</v>
       </c>
       <c r="E58" s="22"/>
       <c r="F58" s="22"/>
@@ -15299,19 +15300,15 @@
         <f>G58*E58</f>
         <v>0</v>
       </c>
-      <c r="I58" s="22" t="s">
-        <v>799</v>
-      </c>
+      <c r="I58" s="22"/>
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B59" s="22">
-        <v>56</v>
-      </c>
-      <c r="C59" s="17" t="s">
-        <v>807</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="C59" s="17"/>
       <c r="D59" s="21" t="s">
-        <v>792</v>
+        <v>853</v>
       </c>
       <c r="E59" s="22"/>
       <c r="F59" s="22"/>
@@ -15320,65 +15317,76 @@
         <f>G59*E59</f>
         <v>0</v>
       </c>
-      <c r="I59" s="17" t="s">
+      <c r="I59" s="22" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="60" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B60" s="22">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C60" s="17" t="s">
         <v>807</v>
       </c>
       <c r="D60" s="21" t="s">
-        <v>784</v>
-      </c>
-      <c r="E60" s="22">
-        <v>1</v>
-      </c>
-      <c r="F60" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G60" s="19">
-        <v>791792.51</v>
-      </c>
+        <v>792</v>
+      </c>
+      <c r="E60" s="22"/>
+      <c r="F60" s="22"/>
+      <c r="G60" s="19"/>
       <c r="H60" s="19">
         <f>G60*E60</f>
-        <v>791792.51</v>
-      </c>
-      <c r="I60" s="22" t="s">
-        <v>783</v>
-      </c>
-      <c r="J60" s="52" t="s">
-        <v>865</v>
+        <v>0</v>
+      </c>
+      <c r="I60" s="17" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="61" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B61" s="22">
+        <v>57</v>
+      </c>
+      <c r="C61" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D61" s="21" t="s">
+        <v>784</v>
+      </c>
+      <c r="E61" s="22">
+        <v>1</v>
+      </c>
+      <c r="F61" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G61" s="19">
+        <v>791792.51</v>
+      </c>
+      <c r="H61" s="19">
+        <f>G61*E61</f>
+        <v>791792.51</v>
+      </c>
+      <c r="I61" s="22" t="s">
+        <v>783</v>
+      </c>
+      <c r="J61" s="52" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B62" s="22">
         <v>58</v>
       </c>
-      <c r="C61" s="34"/>
-      <c r="D61" s="25" t="s">
+      <c r="C62" s="34"/>
+      <c r="D62" s="25" t="s">
         <v>862</v>
       </c>
-      <c r="E61" s="24"/>
-      <c r="F61" s="24"/>
-      <c r="G61" s="26"/>
-      <c r="H61" s="51">
-        <f>G61*E61</f>
-        <v>0</v>
-      </c>
-      <c r="I61" s="24"/>
-    </row>
-    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B62" s="24"/>
-      <c r="C62" s="34"/>
-      <c r="D62" s="25"/>
       <c r="E62" s="24"/>
       <c r="F62" s="24"/>
       <c r="G62" s="26"/>
-      <c r="H62" s="51"/>
+      <c r="H62" s="51">
+        <f>G62*E62</f>
+        <v>0</v>
+      </c>
       <c r="I62" s="24"/>
     </row>
     <row r="63" spans="2:10" x14ac:dyDescent="0.25">
@@ -15392,8 +15400,18 @@
       <c r="I63" s="24"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="D64" s="38"/>
-      <c r="H64" s="16">
+      <c r="B64" s="24"/>
+      <c r="C64" s="34"/>
+      <c r="D64" s="25"/>
+      <c r="E64" s="24"/>
+      <c r="F64" s="24"/>
+      <c r="G64" s="26"/>
+      <c r="H64" s="51"/>
+      <c r="I64" s="24"/>
+    </row>
+    <row r="65" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D65" s="38"/>
+      <c r="H65" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
         <v>4050707.0265427995</v>
       </c>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 15:23
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -3192,8 +3192,8 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I62" totalsRowShown="0" dataDxfId="16">
   <autoFilter ref="B3:I62"/>
-  <sortState ref="B4:I57">
-    <sortCondition ref="I3:I57"/>
+  <sortState ref="B4:I62">
+    <sortCondition ref="I3:I62"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" name="Item" dataDxfId="0" dataCellStyle="Normal"/>
@@ -13051,9 +13051,6 @@
       <c r="H19" s="27" t="s">
         <v>771</v>
       </c>
-      <c r="I19" s="14" t="s">
-        <v>840</v>
-      </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="22">
@@ -13100,6 +13097,9 @@
       </c>
       <c r="H21" s="17" t="s">
         <v>771</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>840</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
@@ -13524,7 +13524,7 @@
       <c r="B41" s="22">
         <v>38</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="28" t="s">
         <v>848</v>
       </c>
       <c r="D41" s="27">
@@ -13548,7 +13548,7 @@
       <c r="B42" s="22">
         <v>39</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C42" s="28" t="s">
         <v>849</v>
       </c>
       <c r="D42" s="27">
@@ -13572,7 +13572,7 @@
       <c r="B43" s="22">
         <v>40</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="28" t="s">
         <v>850</v>
       </c>
       <c r="D43" s="27">
@@ -13596,7 +13596,7 @@
       <c r="B44" s="22">
         <v>41</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="28" t="s">
         <v>851</v>
       </c>
       <c r="D44" s="27">
@@ -15217,157 +15217,157 @@
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B54" s="22">
-        <v>51</v>
-      </c>
-      <c r="C54" s="17"/>
-      <c r="D54" s="25" t="s">
-        <v>868</v>
-      </c>
-      <c r="E54" s="24"/>
-      <c r="F54" s="24"/>
-      <c r="G54" s="53"/>
-      <c r="H54" s="53">
+        <v>54</v>
+      </c>
+      <c r="C54" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D54" s="21" t="s">
+        <v>791</v>
+      </c>
+      <c r="E54" s="22"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="19"/>
+      <c r="H54" s="19">
         <f>G54*E54</f>
         <v>0</v>
       </c>
-      <c r="I54" s="24"/>
+      <c r="I54" s="22" t="s">
+        <v>419</v>
+      </c>
     </row>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B55" s="22">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C55" s="17"/>
-      <c r="D55" s="25" t="s">
-        <v>869</v>
-      </c>
-      <c r="E55" s="24"/>
-      <c r="F55" s="24"/>
-      <c r="G55" s="53"/>
-      <c r="H55" s="53">
+      <c r="D55" s="21" t="s">
+        <v>853</v>
+      </c>
+      <c r="E55" s="22"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="19"/>
+      <c r="H55" s="19">
         <f>G55*E55</f>
         <v>0</v>
       </c>
-      <c r="I55" s="24"/>
+      <c r="I55" s="22" t="s">
+        <v>799</v>
+      </c>
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B56" s="22">
-        <v>53</v>
-      </c>
-      <c r="C56" s="17"/>
-      <c r="D56" s="25" t="s">
-        <v>872</v>
-      </c>
-      <c r="E56" s="24"/>
-      <c r="F56" s="24"/>
-      <c r="G56" s="53"/>
-      <c r="H56" s="53">
+        <v>56</v>
+      </c>
+      <c r="C56" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D56" s="21" t="s">
+        <v>792</v>
+      </c>
+      <c r="E56" s="22"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="19"/>
+      <c r="H56" s="19">
         <f>G56*E56</f>
         <v>0</v>
       </c>
-      <c r="I56" s="24"/>
+      <c r="I56" s="17" t="s">
+        <v>799</v>
+      </c>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B57" s="22">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C57" s="17" t="s">
         <v>807</v>
       </c>
       <c r="D57" s="21" t="s">
-        <v>791</v>
-      </c>
-      <c r="E57" s="22"/>
-      <c r="F57" s="22"/>
-      <c r="G57" s="19"/>
+        <v>784</v>
+      </c>
+      <c r="E57" s="22">
+        <v>1</v>
+      </c>
+      <c r="F57" s="22" t="s">
+        <v>760</v>
+      </c>
+      <c r="G57" s="19">
+        <v>791792.51</v>
+      </c>
       <c r="H57" s="19">
         <f>G57*E57</f>
-        <v>0</v>
+        <v>791792.51</v>
       </c>
       <c r="I57" s="22" t="s">
-        <v>419</v>
+        <v>783</v>
       </c>
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B58" s="22"/>
+      <c r="B58" s="22">
+        <v>51</v>
+      </c>
       <c r="C58" s="17"/>
-      <c r="D58" s="21" t="s">
-        <v>873</v>
-      </c>
-      <c r="E58" s="22"/>
-      <c r="F58" s="22"/>
-      <c r="G58" s="19"/>
-      <c r="H58" s="19">
+      <c r="D58" s="25" t="s">
+        <v>868</v>
+      </c>
+      <c r="E58" s="24"/>
+      <c r="F58" s="24"/>
+      <c r="G58" s="53"/>
+      <c r="H58" s="53">
         <f>G58*E58</f>
         <v>0</v>
       </c>
-      <c r="I58" s="22"/>
+      <c r="I58" s="24"/>
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B59" s="22">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C59" s="17"/>
-      <c r="D59" s="21" t="s">
-        <v>853</v>
-      </c>
-      <c r="E59" s="22"/>
-      <c r="F59" s="22"/>
-      <c r="G59" s="19"/>
-      <c r="H59" s="19">
+      <c r="D59" s="25" t="s">
+        <v>869</v>
+      </c>
+      <c r="E59" s="24"/>
+      <c r="F59" s="24"/>
+      <c r="G59" s="53"/>
+      <c r="H59" s="53">
         <f>G59*E59</f>
         <v>0</v>
       </c>
-      <c r="I59" s="22" t="s">
-        <v>799</v>
-      </c>
+      <c r="I59" s="24"/>
     </row>
     <row r="60" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B60" s="22">
-        <v>56</v>
-      </c>
-      <c r="C60" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D60" s="21" t="s">
-        <v>792</v>
-      </c>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="19"/>
-      <c r="H60" s="19">
+        <v>53</v>
+      </c>
+      <c r="C60" s="17"/>
+      <c r="D60" s="25" t="s">
+        <v>872</v>
+      </c>
+      <c r="E60" s="24"/>
+      <c r="F60" s="24"/>
+      <c r="G60" s="53"/>
+      <c r="H60" s="53">
         <f>G60*E60</f>
         <v>0</v>
       </c>
-      <c r="I60" s="17" t="s">
-        <v>799</v>
-      </c>
+      <c r="I60" s="24"/>
     </row>
     <row r="61" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B61" s="22">
-        <v>57</v>
-      </c>
-      <c r="C61" s="17" t="s">
-        <v>807</v>
-      </c>
+      <c r="B61" s="22"/>
+      <c r="C61" s="17"/>
       <c r="D61" s="21" t="s">
-        <v>784</v>
-      </c>
-      <c r="E61" s="22">
-        <v>1</v>
-      </c>
-      <c r="F61" s="22" t="s">
-        <v>760</v>
-      </c>
-      <c r="G61" s="19">
-        <v>791792.51</v>
-      </c>
+        <v>873</v>
+      </c>
+      <c r="E61" s="22"/>
+      <c r="F61" s="22"/>
+      <c r="G61" s="19"/>
       <c r="H61" s="19">
         <f>G61*E61</f>
-        <v>791792.51</v>
-      </c>
-      <c r="I61" s="22" t="s">
-        <v>783</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I61" s="22"/>
       <c r="J61" s="52" t="s">
         <v>865</v>
       </c>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 15:28
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -12702,7 +12702,7 @@
       </c>
       <c r="J4" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
-        <v>118280</v>
+        <v>152468</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
@@ -13065,10 +13065,12 @@
       <c r="E20" s="17" t="s">
         <v>839</v>
       </c>
-      <c r="F20" s="20"/>
+      <c r="F20" s="20">
+        <v>7.77</v>
+      </c>
       <c r="G20" s="20">
         <f>F20*D20</f>
-        <v>0</v>
+        <v>16317</v>
       </c>
       <c r="H20" s="17" t="s">
         <v>771</v>
@@ -13090,10 +13092,12 @@
       <c r="E21" s="17" t="s">
         <v>839</v>
       </c>
-      <c r="F21" s="20"/>
+      <c r="F21" s="20">
+        <v>7.77</v>
+      </c>
       <c r="G21" s="20">
         <f>F21*D21</f>
-        <v>0</v>
+        <v>17871</v>
       </c>
       <c r="H21" s="17" t="s">
         <v>771</v>
@@ -13679,7 +13683,7 @@
     <row r="49" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G49" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>2334170.5208461536</v>
+        <v>2368358.5208461536</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 15:29
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -13056,23 +13056,23 @@
       <c r="B20" s="22">
         <v>17</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="31" t="s">
         <v>769</v>
       </c>
-      <c r="D20" s="17">
+      <c r="D20" s="27">
         <v>2100</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="27" t="s">
         <v>839</v>
       </c>
-      <c r="F20" s="20">
+      <c r="F20" s="32">
         <v>7.77</v>
       </c>
-      <c r="G20" s="20">
+      <c r="G20" s="32">
         <f>F20*D20</f>
         <v>16317</v>
       </c>
-      <c r="H20" s="17" t="s">
+      <c r="H20" s="27" t="s">
         <v>771</v>
       </c>
       <c r="I20" s="14" t="s">
@@ -13083,23 +13083,23 @@
       <c r="B21" s="22">
         <v>18</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="31" t="s">
         <v>770</v>
       </c>
-      <c r="D21" s="17">
+      <c r="D21" s="27">
         <v>2300</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="27" t="s">
         <v>839</v>
       </c>
-      <c r="F21" s="20">
+      <c r="F21" s="32">
         <v>7.77</v>
       </c>
-      <c r="G21" s="20">
+      <c r="G21" s="32">
         <f>F21*D21</f>
         <v>17871</v>
       </c>
-      <c r="H21" s="17" t="s">
+      <c r="H21" s="27" t="s">
         <v>771</v>
       </c>
       <c r="I21" s="14" t="s">
@@ -13829,11 +13829,11 @@
       </c>
       <c r="P5" s="43">
         <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
-        <v>0.24292488569525772</v>
+        <v>0.23923953577462048</v>
       </c>
       <c r="Q5" s="45">
         <f>P5</f>
-        <v>0.24292488569525772</v>
+        <v>0.23923953577462048</v>
       </c>
       <c r="R5" t="s">
         <v>826</v>
@@ -13870,11 +13870,11 @@
       </c>
       <c r="P6" s="43">
         <f t="shared" si="0"/>
-        <v>0.19379882094793693</v>
+        <v>0.19085874971004807</v>
       </c>
       <c r="Q6" s="45">
         <f>P6+Q5</f>
-        <v>0.43672370664319465</v>
+        <v>0.43009828548466855</v>
       </c>
       <c r="R6" t="s">
         <v>826</v>
@@ -13911,7 +13911,7 @@
       </c>
       <c r="P7" s="43">
         <f t="shared" si="0"/>
-        <v>0.14979226555589042</v>
+        <v>0.14751980626297556</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="P8" s="43">
         <f t="shared" si="0"/>
-        <v>0.17860108280856254</v>
+        <v>0.17589157248206613</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
@@ -13981,11 +13981,11 @@
       </c>
       <c r="O9" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Fundação",Tabela24[Preço Total])</f>
-        <v>338537.4</v>
+        <v>401474.4</v>
       </c>
       <c r="P9" s="43">
         <f t="shared" si="0"/>
-        <v>8.286027985637312E-2</v>
+        <v>9.6773966736047712E-2</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
@@ -14021,7 +14021,7 @@
       </c>
       <c r="P10" s="43">
         <f t="shared" si="0"/>
-        <v>1.6284849317300034E-2</v>
+        <v>1.6037796126486193E-2</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
@@ -14059,7 +14059,7 @@
       </c>
       <c r="P11" s="43">
         <f t="shared" si="0"/>
-        <v>0.1189609996979735</v>
+        <v>0.11715627347759842</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
@@ -14159,7 +14159,7 @@
       </c>
       <c r="P14" s="43">
         <f t="shared" si="0"/>
-        <v>1.6284849317300034E-2</v>
+        <v>1.6037796126486193E-2</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
@@ -14197,7 +14197,7 @@
       </c>
       <c r="P15" s="43">
         <f t="shared" si="0"/>
-        <v>4.9196680340579787E-4</v>
+        <v>4.8450330367130729E-4</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
@@ -14462,7 +14462,7 @@
       </c>
       <c r="O24" s="42">
         <f>SUM(O5:O20)</f>
-        <v>4085641.5231375997</v>
+        <v>4148578.5231375997</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -14472,21 +14472,23 @@
       <c r="C25" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="D25" s="31" t="s">
         <v>769</v>
       </c>
-      <c r="E25" s="17">
+      <c r="E25" s="27">
         <v>4100</v>
       </c>
-      <c r="F25" s="17" t="s">
+      <c r="F25" s="27" t="s">
         <v>839</v>
       </c>
-      <c r="G25" s="20"/>
-      <c r="H25" s="20">
+      <c r="G25" s="32">
+        <v>7.77</v>
+      </c>
+      <c r="H25" s="32">
         <f>G25*E25</f>
-        <v>0</v>
-      </c>
-      <c r="I25" s="17" t="s">
+        <v>31857</v>
+      </c>
+      <c r="I25" s="27" t="s">
         <v>771</v>
       </c>
       <c r="J25" s="14" t="s">
@@ -14502,21 +14504,23 @@
       <c r="C26" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D26" s="18" t="s">
+      <c r="D26" s="31" t="s">
         <v>770</v>
       </c>
-      <c r="E26" s="17">
+      <c r="E26" s="27">
         <v>4000</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="F26" s="27" t="s">
         <v>839</v>
       </c>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20">
+      <c r="G26" s="32">
+        <v>7.77</v>
+      </c>
+      <c r="H26" s="32">
         <f>G26*E26</f>
-        <v>0</v>
-      </c>
-      <c r="I26" s="17" t="s">
+        <v>31080</v>
+      </c>
+      <c r="I26" s="27" t="s">
         <v>771</v>
       </c>
       <c r="J26" s="14" t="s">
@@ -15417,7 +15421,7 @@
       <c r="D65" s="38"/>
       <c r="H65" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>4050707.0265427995</v>
+        <v>4113644.0265427995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 15:39
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2160" uniqueCount="874">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2158" uniqueCount="873">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2457,15 +2457,9 @@
     <t>Sistema de tratamento para esgoto do banheiro</t>
   </si>
   <si>
-    <t>Verificar final</t>
-  </si>
-  <si>
     <t>pç</t>
   </si>
   <si>
-    <t>R$ 50,00/m³</t>
-  </si>
-  <si>
     <t>Bomba de concreto para volume total do piso</t>
   </si>
   <si>
@@ -2478,9 +2472,6 @@
     <t>Desvio da rede de esgoto existente</t>
   </si>
   <si>
-    <t>Mão de obra para concretagem do piso e instalação do meio-fio</t>
-  </si>
-  <si>
     <t>Meio Fio Padrão Novacap 30x15/12</t>
   </si>
   <si>
@@ -2616,9 +2607,6 @@
     <t>Mão de obra para fechamento em alvenaria na parte interna do galpão blocado</t>
   </si>
   <si>
-    <t>Mão de obra para concretagem do piso do galpão 2100m²</t>
-  </si>
-  <si>
     <t>Frente para entrega do Meio fio</t>
   </si>
   <si>
@@ -2647,6 +2635,15 @@
   </si>
   <si>
     <t>Cabo para ligação do sistema de tratamento de esgoto do banheiro</t>
+  </si>
+  <si>
+    <t>Mão de obra para concretagem do piso e instalação do meio-fio (PÁTIO)</t>
+  </si>
+  <si>
+    <t>Mão de obra para concretagem do piso do galpão 2100m² (DPA IV)</t>
+  </si>
+  <si>
+    <t>Piso pátio</t>
   </si>
 </sst>
 </file>
@@ -12673,7 +12670,7 @@
         <v>767</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
     </row>
     <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -12702,7 +12699,7 @@
       </c>
       <c r="J4" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
-        <v>152468</v>
+        <v>160740</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
@@ -12710,7 +12707,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>857</v>
+        <v>854</v>
       </c>
       <c r="D5" s="22">
         <v>3</v>
@@ -12758,7 +12755,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
@@ -12834,7 +12831,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="D10" s="27">
         <v>1</v>
@@ -12850,7 +12847,7 @@
         <v>1056959.67</v>
       </c>
       <c r="H10" s="27" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="J10" s="39">
         <f>SUMIF(Tabela2[Aplicação],"Terraplanagem",Tabela2[Preço Total])</f>
@@ -12991,7 +12988,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="D17" s="24"/>
       <c r="E17" s="24"/>
@@ -13063,20 +13060,20 @@
         <v>2100</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="F20" s="32">
-        <v>7.77</v>
+        <v>9.65</v>
       </c>
       <c r="G20" s="32">
         <f>F20*D20</f>
-        <v>16317</v>
+        <v>20265</v>
       </c>
       <c r="H20" s="27" t="s">
         <v>771</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
@@ -13090,20 +13087,20 @@
         <v>2300</v>
       </c>
       <c r="E21" s="27" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="F21" s="32">
-        <v>7.77</v>
+        <v>9.65</v>
       </c>
       <c r="G21" s="32">
         <f>F21*D21</f>
-        <v>17871</v>
+        <v>22195</v>
       </c>
       <c r="H21" s="27" t="s">
         <v>771</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
@@ -13111,7 +13108,7 @@
         <v>19</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="D22" s="27">
         <v>1</v>
@@ -13135,7 +13132,7 @@
         <v>20</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="D23" s="33">
         <v>46.8</v>
@@ -13159,7 +13156,7 @@
         <v>21</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="D24" s="33">
         <v>37.200000000000003</v>
@@ -13329,7 +13326,7 @@
         <v>167</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="F32" s="32">
         <v>56.2</v>
@@ -13441,7 +13438,7 @@
         <v>34</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="D37" s="24">
         <v>1</v>
@@ -13481,7 +13478,7 @@
         <v>36</v>
       </c>
       <c r="C39" s="46" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
       <c r="D39" s="27">
         <v>1455.89</v>
@@ -13505,7 +13502,7 @@
         <v>37</v>
       </c>
       <c r="C40" s="31" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
       <c r="D40" s="27">
         <v>706.94</v>
@@ -13529,13 +13526,13 @@
         <v>38</v>
       </c>
       <c r="C41" s="28" t="s">
-        <v>848</v>
+        <v>845</v>
       </c>
       <c r="D41" s="27">
         <v>44</v>
       </c>
       <c r="E41" s="27" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
       <c r="F41" s="36">
         <v>95</v>
@@ -13553,13 +13550,13 @@
         <v>39</v>
       </c>
       <c r="C42" s="28" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
       <c r="D42" s="27">
         <v>3</v>
       </c>
       <c r="E42" s="27" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
       <c r="F42" s="36">
         <v>35</v>
@@ -13577,7 +13574,7 @@
         <v>40</v>
       </c>
       <c r="C43" s="28" t="s">
-        <v>850</v>
+        <v>847</v>
       </c>
       <c r="D43" s="27">
         <v>126</v>
@@ -13601,7 +13598,7 @@
         <v>41</v>
       </c>
       <c r="C44" s="28" t="s">
-        <v>851</v>
+        <v>848</v>
       </c>
       <c r="D44" s="27">
         <v>1</v>
@@ -13649,7 +13646,7 @@
         <v>43</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
       <c r="D46" s="24"/>
       <c r="E46" s="24"/>
@@ -13659,7 +13656,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="24" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
@@ -13683,7 +13680,7 @@
     <row r="49" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G49" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>2368358.5208461536</v>
+        <v>2376630.5208461536</v>
       </c>
     </row>
   </sheetData>
@@ -13719,12 +13716,12 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P1" s="14" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P2" s="14" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
     </row>
     <row r="3" spans="2:18" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -13754,7 +13751,7 @@
       </c>
       <c r="J3" s="52"/>
       <c r="P3" s="14" t="s">
-        <v>829</v>
+        <v>826</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
@@ -13779,19 +13776,19 @@
         <v>0</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="O4" s="14" t="s">
+        <v>818</v>
+      </c>
+      <c r="P4" s="14" t="s">
+        <v>820</v>
+      </c>
+      <c r="Q4" s="14" t="s">
         <v>821</v>
       </c>
-      <c r="P4" s="14" t="s">
-        <v>823</v>
-      </c>
-      <c r="Q4" s="14" t="s">
-        <v>824</v>
-      </c>
       <c r="R4" s="14" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
@@ -13802,7 +13799,7 @@
         <v>807</v>
       </c>
       <c r="D5" s="31" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="E5" s="27">
         <v>1</v>
@@ -13829,14 +13826,14 @@
       </c>
       <c r="P5" s="43">
         <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
-        <v>0.23923953577462048</v>
+        <v>0.23836458165979033</v>
       </c>
       <c r="Q5" s="45">
         <f>P5</f>
-        <v>0.23923953577462048</v>
+        <v>0.23836458165979033</v>
       </c>
       <c r="R5" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.25">
@@ -13845,7 +13842,7 @@
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="21" t="s">
-        <v>856</v>
+        <v>853</v>
       </c>
       <c r="E6" s="22">
         <v>4</v>
@@ -13870,14 +13867,14 @@
       </c>
       <c r="P6" s="43">
         <f t="shared" si="0"/>
-        <v>0.19085874971004807</v>
+        <v>0.19016073527915792</v>
       </c>
       <c r="Q6" s="45">
         <f>P6+Q5</f>
-        <v>0.43009828548466855</v>
+        <v>0.42852531693894824</v>
       </c>
       <c r="R6" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
@@ -13886,7 +13883,7 @@
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="21" t="s">
-        <v>855</v>
+        <v>852</v>
       </c>
       <c r="E7" s="22">
         <v>6</v>
@@ -13911,7 +13908,7 @@
       </c>
       <c r="P7" s="43">
         <f t="shared" si="0"/>
-        <v>0.14751980626297556</v>
+        <v>0.14698029233568582</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
@@ -13920,7 +13917,7 @@
       </c>
       <c r="C8" s="34"/>
       <c r="D8" s="25" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
       <c r="E8" s="24">
         <v>6</v>
@@ -13936,9 +13933,6 @@
       <c r="I8" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="J8" s="52" t="s">
-        <v>812</v>
-      </c>
       <c r="N8" s="44" t="s">
         <v>804</v>
       </c>
@@ -13948,7 +13942,7 @@
       </c>
       <c r="P8" s="43">
         <f t="shared" si="0"/>
-        <v>0.17589157248206613</v>
+        <v>0.17524829646746914</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
@@ -13957,7 +13951,7 @@
       </c>
       <c r="C9" s="34"/>
       <c r="D9" s="25" t="s">
-        <v>866</v>
+        <v>862</v>
       </c>
       <c r="E9" s="24">
         <v>1</v>
@@ -13973,19 +13967,16 @@
       <c r="I9" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="J9" s="52" t="s">
-        <v>810</v>
-      </c>
       <c r="N9" s="41" t="s">
         <v>771</v>
       </c>
       <c r="O9" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Fundação",Tabela24[Preço Total])</f>
-        <v>401474.4</v>
+        <v>416702.4</v>
       </c>
       <c r="P9" s="43">
         <f t="shared" si="0"/>
-        <v>9.6773966736047712E-2</v>
+        <v>0.10007727248719463</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
@@ -14021,7 +14012,7 @@
       </c>
       <c r="P10" s="43">
         <f t="shared" si="0"/>
-        <v>1.6037796126486193E-2</v>
+        <v>1.5979142210158184E-2</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
@@ -14059,7 +14050,7 @@
       </c>
       <c r="P11" s="43">
         <f t="shared" si="0"/>
-        <v>0.11715627347759842</v>
+        <v>0.11672780598694939</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
@@ -14070,7 +14061,7 @@
         <v>807</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="E12" s="24"/>
       <c r="F12" s="24"/>
@@ -14102,7 +14093,7 @@
         <v>807</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="E13" s="27">
         <v>54</v>
@@ -14118,7 +14109,7 @@
         <v>13143.06</v>
       </c>
       <c r="I13" s="27" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="N13" s="40"/>
       <c r="O13" s="39"/>
@@ -14132,7 +14123,7 @@
         <v>807</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="E14" s="27">
         <v>30</v>
@@ -14148,7 +14139,7 @@
         <v>3591</v>
       </c>
       <c r="I14" s="27" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="N14" s="40" t="s">
         <v>774</v>
@@ -14159,7 +14150,7 @@
       </c>
       <c r="P14" s="43">
         <f t="shared" si="0"/>
-        <v>1.6037796126486193E-2</v>
+        <v>1.5979142210158184E-2</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
@@ -14170,7 +14161,7 @@
         <v>807</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="E15" s="48">
         <v>390</v>
@@ -14186,7 +14177,7 @@
         <v>14865.499974</v>
       </c>
       <c r="I15" s="27" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="N15" s="40" t="s">
         <v>643</v>
@@ -14197,7 +14188,7 @@
       </c>
       <c r="P15" s="43">
         <f t="shared" si="0"/>
-        <v>4.8450330367130729E-4</v>
+        <v>4.8273136343649853E-4</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
@@ -14208,7 +14199,7 @@
         <v>807</v>
       </c>
       <c r="D16" s="31" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="E16" s="33">
         <f>(84*1.02)*2*1.02</f>
@@ -14239,7 +14230,7 @@
         <v>807</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="E17" s="27">
         <f>84*7</f>
@@ -14268,13 +14259,13 @@
       </c>
       <c r="C18" s="27"/>
       <c r="D18" s="31" t="s">
-        <v>859</v>
+        <v>856</v>
       </c>
       <c r="E18" s="27">
         <v>30</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
       <c r="G18" s="36">
         <v>24</v>
@@ -14296,7 +14287,7 @@
       </c>
       <c r="C19" s="27"/>
       <c r="D19" s="31" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="E19" s="27">
         <v>1</v>
@@ -14349,7 +14340,7 @@
         <v>774</v>
       </c>
       <c r="N20" s="40" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="O20" s="39">
         <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
@@ -14416,7 +14407,7 @@
         <v>807</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="E23" s="24">
         <v>1</v>
@@ -14458,11 +14449,11 @@
         <v>771</v>
       </c>
       <c r="N24" s="40" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="O24" s="42">
         <f>SUM(O5:O20)</f>
-        <v>4148578.5231375997</v>
+        <v>4163806.5231375997</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -14479,20 +14470,20 @@
         <v>4100</v>
       </c>
       <c r="F25" s="27" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="G25" s="32">
-        <v>7.77</v>
+        <v>9.65</v>
       </c>
       <c r="H25" s="32">
         <f>G25*E25</f>
-        <v>31857</v>
+        <v>39565</v>
       </c>
       <c r="I25" s="27" t="s">
         <v>771</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="N25" s="40"/>
       <c r="O25" s="42"/>
@@ -14511,20 +14502,20 @@
         <v>4000</v>
       </c>
       <c r="F26" s="27" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="G26" s="32">
-        <v>7.77</v>
+        <v>9.65</v>
       </c>
       <c r="H26" s="32">
         <f>G26*E26</f>
-        <v>31080</v>
+        <v>38600</v>
       </c>
       <c r="I26" s="27" t="s">
         <v>771</v>
       </c>
       <c r="J26" s="14" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
@@ -14535,7 +14526,7 @@
         <v>807</v>
       </c>
       <c r="D27" s="31" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="E27" s="27">
         <v>1</v>
@@ -14562,7 +14553,7 @@
         <v>807</v>
       </c>
       <c r="D28" s="31" t="s">
-        <v>871</v>
+        <v>867</v>
       </c>
       <c r="E28" s="27">
         <v>99.22</v>
@@ -14587,7 +14578,7 @@
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="31" t="s">
-        <v>870</v>
+        <v>866</v>
       </c>
       <c r="E29" s="27">
         <v>68</v>
@@ -14614,7 +14605,7 @@
         <v>807</v>
       </c>
       <c r="D30" s="31" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="E30" s="27">
         <v>1</v>
@@ -14857,7 +14848,7 @@
         <v>807</v>
       </c>
       <c r="D40" s="18" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="E40" s="23">
         <f>E36</f>
@@ -14885,7 +14876,7 @@
         <v>807</v>
       </c>
       <c r="D41" s="31" t="s">
-        <v>863</v>
+        <v>871</v>
       </c>
       <c r="E41" s="27">
         <v>1</v>
@@ -14912,7 +14903,7 @@
         <v>808</v>
       </c>
       <c r="D42" s="47" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="E42" s="48">
         <v>110</v>
@@ -14937,7 +14928,7 @@
       </c>
       <c r="C43" s="34"/>
       <c r="D43" s="47" t="s">
-        <v>864</v>
+        <v>860</v>
       </c>
       <c r="E43" s="48">
         <v>1</v>
@@ -15020,7 +15011,7 @@
         <v>808</v>
       </c>
       <c r="D46" s="25" t="s">
-        <v>817</v>
+        <v>870</v>
       </c>
       <c r="E46" s="24">
         <v>1</v>
@@ -15034,10 +15025,10 @@
         <v>0</v>
       </c>
       <c r="I46" s="24" t="s">
-        <v>635</v>
+        <v>872</v>
       </c>
       <c r="J46" s="52" t="s">
-        <v>867</v>
+        <v>863</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
@@ -15048,7 +15039,7 @@
         <v>807</v>
       </c>
       <c r="D47" s="31" t="s">
-        <v>858</v>
+        <v>855</v>
       </c>
       <c r="E47" s="27">
         <v>1</v>
@@ -15075,7 +15066,7 @@
         <v>807</v>
       </c>
       <c r="D48" s="21" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="E48" s="22"/>
       <c r="F48" s="22"/>
@@ -15177,7 +15168,7 @@
         <v>808</v>
       </c>
       <c r="D52" s="47" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="E52" s="48">
         <v>1</v>
@@ -15250,7 +15241,7 @@
       </c>
       <c r="C55" s="17"/>
       <c r="D55" s="21" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
       <c r="E55" s="22"/>
       <c r="F55" s="22"/>
@@ -15317,7 +15308,7 @@
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="25" t="s">
-        <v>868</v>
+        <v>864</v>
       </c>
       <c r="E58" s="24"/>
       <c r="F58" s="24"/>
@@ -15334,7 +15325,7 @@
       </c>
       <c r="C59" s="17"/>
       <c r="D59" s="25" t="s">
-        <v>869</v>
+        <v>865</v>
       </c>
       <c r="E59" s="24"/>
       <c r="F59" s="24"/>
@@ -15351,7 +15342,7 @@
       </c>
       <c r="C60" s="17"/>
       <c r="D60" s="25" t="s">
-        <v>872</v>
+        <v>868</v>
       </c>
       <c r="E60" s="24"/>
       <c r="F60" s="24"/>
@@ -15366,7 +15357,7 @@
       <c r="B61" s="22"/>
       <c r="C61" s="17"/>
       <c r="D61" s="21" t="s">
-        <v>873</v>
+        <v>869</v>
       </c>
       <c r="E61" s="22"/>
       <c r="F61" s="22"/>
@@ -15377,7 +15368,7 @@
       </c>
       <c r="I61" s="22"/>
       <c r="J61" s="52" t="s">
-        <v>865</v>
+        <v>861</v>
       </c>
     </row>
     <row r="62" spans="2:10" x14ac:dyDescent="0.25">
@@ -15386,7 +15377,7 @@
       </c>
       <c r="C62" s="34"/>
       <c r="D62" s="25" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="E62" s="24"/>
       <c r="F62" s="24"/>
@@ -15421,7 +15412,7 @@
       <c r="D65" s="38"/>
       <c r="H65" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>4113644.0265427995</v>
+        <v>4128872.0265427995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 15:50
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2158" uniqueCount="873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2158" uniqueCount="875">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2607,9 +2607,6 @@
     <t>Mão de obra para fechamento em alvenaria na parte interna do galpão blocado</t>
   </si>
   <si>
-    <t>Frente para entrega do Meio fio</t>
-  </si>
-  <si>
     <t>Solicitar mais um orçamento do Erisvaldo</t>
   </si>
   <si>
@@ -2644,6 +2641,15 @@
   </si>
   <si>
     <t>Piso pátio</t>
+  </si>
+  <si>
+    <t>Piso Galpão</t>
+  </si>
+  <si>
+    <t>Piso Pátio de Manobra</t>
+  </si>
+  <si>
+    <t>Frete para entrega do Meio fio</t>
   </si>
 </sst>
 </file>
@@ -2751,7 +2757,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2808,14 +2814,8 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3188,7 +3188,14 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I62" totalsRowShown="0" dataDxfId="16">
-  <autoFilter ref="B3:I62"/>
+  <autoFilter ref="B3:I62">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="Piso"/>
+        <filter val="Piso pátio"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState ref="B4:I62">
     <sortCondition ref="I3:I62"/>
   </sortState>
@@ -12674,402 +12681,402 @@
       </c>
     </row>
     <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="22">
-        <v>1</v>
-      </c>
-      <c r="C4" s="31" t="s">
+      <c r="B4" s="21">
+        <v>1</v>
+      </c>
+      <c r="C4" s="29" t="s">
         <v>776</v>
       </c>
-      <c r="D4" s="27">
-        <v>1</v>
-      </c>
-      <c r="E4" s="27" t="s">
+      <c r="D4" s="25">
+        <v>1</v>
+      </c>
+      <c r="E4" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="F4" s="36">
+      <c r="F4" s="34">
         <f>212518+208594</f>
         <v>421112</v>
       </c>
-      <c r="G4" s="36">
+      <c r="G4" s="34">
         <f>F4*D4</f>
         <v>421112</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="H4" s="25" t="s">
         <v>782</v>
       </c>
-      <c r="J4" s="39">
+      <c r="J4" s="37">
         <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
         <v>160740</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="22">
+      <c r="B5" s="21">
         <v>2</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="20" t="s">
         <v>854</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="21">
         <v>3</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50">
+      <c r="F5" s="48"/>
+      <c r="G5" s="48">
         <f>F5*D5</f>
         <v>0</v>
       </c>
-      <c r="H5" s="22" t="s">
+      <c r="H5" s="21" t="s">
         <v>782</v>
       </c>
-      <c r="J5" s="39">
+      <c r="J5" s="37">
         <f>SUMIF(Tabela2[Aplicação],"Piso",Tabela2[Preço Total])</f>
         <v>361131.5538461539</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="22">
+      <c r="B6" s="21">
         <v>3</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="20" t="s">
         <v>778</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
       <c r="F6" s="19"/>
       <c r="G6" s="19">
         <f>F6*D6</f>
         <v>0</v>
       </c>
-      <c r="H6" s="22" t="s">
+      <c r="H6" s="21" t="s">
         <v>449</v>
       </c>
-      <c r="J6" s="39">
+      <c r="J6" s="37">
         <f>SUMIF(Tabela2[Aplicação],"Pré Moldado",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="22">
+      <c r="B7" s="21">
         <v>4</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="20" t="s">
         <v>832</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
       <c r="F7" s="19"/>
       <c r="G7" s="19">
         <f>F7*D7</f>
         <v>0</v>
       </c>
-      <c r="H7" s="22" t="s">
+      <c r="H7" s="21" t="s">
         <v>449</v>
       </c>
-      <c r="J7" s="39">
+      <c r="J7" s="37">
         <f>SUMIF(Tabela2[Aplicação],"Fechamento Lateral",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="22">
+      <c r="B8" s="21">
         <v>5</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="23" t="s">
         <v>789</v>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="22">
         <v>10</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26">
+      <c r="F8" s="24"/>
+      <c r="G8" s="24">
         <f>F8*D8</f>
         <v>0</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="22" t="s">
         <v>643</v>
       </c>
-      <c r="J8" s="39">
+      <c r="J8" s="37">
         <f>SUMIF(Tabela2[Aplicação],"AVCB",Tabela2[Preço Total])</f>
         <v>421112</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="22">
+      <c r="B9" s="21">
         <v>6</v>
       </c>
-      <c r="C9" s="47" t="s">
+      <c r="C9" s="45" t="s">
         <v>790</v>
       </c>
-      <c r="D9" s="48">
+      <c r="D9" s="46">
         <v>600</v>
       </c>
-      <c r="E9" s="48" t="s">
+      <c r="E9" s="46" t="s">
         <v>761</v>
       </c>
-      <c r="F9" s="49">
+      <c r="F9" s="47">
         <v>3.35</v>
       </c>
-      <c r="G9" s="49">
+      <c r="G9" s="47">
         <f>F9*D9</f>
         <v>2010</v>
       </c>
-      <c r="H9" s="48" t="s">
+      <c r="H9" s="46" t="s">
         <v>643</v>
       </c>
-      <c r="J9" s="39">
+      <c r="J9" s="37">
         <f>SUMIF(Tabela2[Aplicação],"SPDA",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="22">
+      <c r="B10" s="21">
         <v>7</v>
       </c>
-      <c r="C10" s="31" t="s">
+      <c r="C10" s="29" t="s">
         <v>842</v>
       </c>
-      <c r="D10" s="27">
-        <v>1</v>
-      </c>
-      <c r="E10" s="27" t="s">
+      <c r="D10" s="25">
+        <v>1</v>
+      </c>
+      <c r="E10" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="F10" s="32">
+      <c r="F10" s="30">
         <v>1056959.67</v>
       </c>
-      <c r="G10" s="32">
+      <c r="G10" s="30">
         <f>F10*D10</f>
         <v>1056959.67</v>
       </c>
-      <c r="H10" s="27" t="s">
+      <c r="H10" s="25" t="s">
         <v>841</v>
       </c>
-      <c r="J10" s="39">
+      <c r="J10" s="37">
         <f>SUMIF(Tabela2[Aplicação],"Terraplanagem",Tabela2[Preço Total])</f>
         <v>157963.5</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B11" s="22">
+      <c r="B11" s="21">
         <v>8</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="23" t="s">
         <v>793</v>
       </c>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26">
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24">
         <f>F11*D11</f>
         <v>0</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="H11" s="22" t="s">
         <v>796</v>
       </c>
-      <c r="J11" s="39">
+      <c r="J11" s="37">
         <f>SUMIF(Tabela2[Aplicação],"Drenagem",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="22">
+      <c r="B12" s="21">
         <v>9</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="20" t="s">
         <v>800</v>
       </c>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
       <c r="F12" s="19"/>
       <c r="G12" s="19">
         <f>F12*D12</f>
         <v>0</v>
       </c>
-      <c r="H12" s="22" t="s">
+      <c r="H12" s="21" t="s">
         <v>774</v>
       </c>
-      <c r="J12" s="39">
+      <c r="J12" s="37">
         <f>SUMIF(Tabela2[Aplicação],"Elétrica",Tabela2[Preço Total])</f>
         <v>2010</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="22">
+      <c r="B13" s="21">
         <v>10</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="20" t="s">
         <v>798</v>
       </c>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
       <c r="F13" s="19"/>
       <c r="G13" s="19">
         <f>F13*D13</f>
         <v>0</v>
       </c>
-      <c r="H13" s="22" t="s">
+      <c r="H13" s="21" t="s">
         <v>774</v>
       </c>
-      <c r="J13" s="39">
+      <c r="J13" s="37">
         <f>SUMIF(Tabela2[Aplicação],"Pintura",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="22">
+      <c r="B14" s="21">
         <v>11</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="23" t="s">
         <v>779</v>
       </c>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26">
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24">
         <f>F14*D14</f>
         <v>0</v>
       </c>
-      <c r="H14" s="24" t="s">
+      <c r="H14" s="22" t="s">
         <v>774</v>
       </c>
-      <c r="J14" s="39">
+      <c r="J14" s="37">
         <f>SUMIF(Tabela2[Aplicação],"Estrura Armazenamento",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B15" s="22">
+      <c r="B15" s="21">
         <v>12</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="23" t="s">
         <v>780</v>
       </c>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26">
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24">
         <f>F15*D15</f>
         <v>0</v>
       </c>
-      <c r="H15" s="24" t="s">
+      <c r="H15" s="22" t="s">
         <v>774</v>
       </c>
-      <c r="J15" s="39">
+      <c r="J15" s="37">
         <f>SUMIF(Tabela2[Aplicação],"Serviço Prévio",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="22">
+      <c r="B16" s="21">
         <v>13</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="23" t="s">
         <v>781</v>
       </c>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26">
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24">
         <f>F16*D16</f>
         <v>0</v>
       </c>
-      <c r="H16" s="24" t="s">
+      <c r="H16" s="22" t="s">
         <v>774</v>
       </c>
-      <c r="J16" s="39"/>
+      <c r="J16" s="37"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="22">
+      <c r="B17" s="21">
         <v>14</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="23" t="s">
         <v>838</v>
       </c>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26">
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24">
         <f>F17*D17</f>
         <v>0</v>
       </c>
-      <c r="H17" s="24" t="s">
+      <c r="H17" s="22" t="s">
         <v>774</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="22">
+      <c r="B18" s="21">
         <v>15</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="26" t="s">
         <v>797</v>
       </c>
-      <c r="D18" s="29">
+      <c r="D18" s="27">
         <v>4</v>
       </c>
-      <c r="E18" s="29" t="s">
+      <c r="E18" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="F18" s="30">
+      <c r="F18" s="28">
         <v>1500</v>
       </c>
-      <c r="G18" s="30">
+      <c r="G18" s="28">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>6000</v>
       </c>
-      <c r="H18" s="29" t="s">
+      <c r="H18" s="27" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="22">
+      <c r="B19" s="21">
         <v>16</v>
       </c>
-      <c r="C19" s="31" t="s">
+      <c r="C19" s="29" t="s">
         <v>795</v>
       </c>
-      <c r="D19" s="27">
-        <v>1</v>
-      </c>
-      <c r="E19" s="27" t="s">
+      <c r="D19" s="25">
+        <v>1</v>
+      </c>
+      <c r="E19" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="F19" s="32">
+      <c r="F19" s="30">
         <v>4500</v>
       </c>
-      <c r="G19" s="32">
+      <c r="G19" s="30">
         <f>F19*D19</f>
         <v>4500</v>
       </c>
-      <c r="H19" s="27" t="s">
+      <c r="H19" s="25" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="22">
+      <c r="B20" s="21">
         <v>17</v>
       </c>
-      <c r="C20" s="31" t="s">
+      <c r="C20" s="29" t="s">
         <v>769</v>
       </c>
-      <c r="D20" s="27">
+      <c r="D20" s="25">
         <v>2100</v>
       </c>
-      <c r="E20" s="27" t="s">
+      <c r="E20" s="25" t="s">
         <v>836</v>
       </c>
-      <c r="F20" s="32">
+      <c r="F20" s="30">
         <v>9.65</v>
       </c>
-      <c r="G20" s="32">
+      <c r="G20" s="30">
         <f>F20*D20</f>
         <v>20265</v>
       </c>
-      <c r="H20" s="27" t="s">
+      <c r="H20" s="25" t="s">
         <v>771</v>
       </c>
       <c r="I20" s="14" t="s">
@@ -13077,26 +13084,26 @@
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="22">
+      <c r="B21" s="21">
         <v>18</v>
       </c>
-      <c r="C21" s="31" t="s">
+      <c r="C21" s="29" t="s">
         <v>770</v>
       </c>
-      <c r="D21" s="27">
+      <c r="D21" s="25">
         <v>2300</v>
       </c>
-      <c r="E21" s="27" t="s">
+      <c r="E21" s="25" t="s">
         <v>836</v>
       </c>
-      <c r="F21" s="32">
+      <c r="F21" s="30">
         <v>9.65</v>
       </c>
-      <c r="G21" s="32">
+      <c r="G21" s="30">
         <f>F21*D21</f>
         <v>22195</v>
       </c>
-      <c r="H21" s="27" t="s">
+      <c r="H21" s="25" t="s">
         <v>771</v>
       </c>
       <c r="I21" s="14" t="s">
@@ -13104,578 +13111,578 @@
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="22">
+      <c r="B22" s="21">
         <v>19</v>
       </c>
-      <c r="C22" s="31" t="s">
+      <c r="C22" s="29" t="s">
         <v>833</v>
       </c>
-      <c r="D22" s="27">
-        <v>1</v>
-      </c>
-      <c r="E22" s="27" t="s">
+      <c r="D22" s="25">
+        <v>1</v>
+      </c>
+      <c r="E22" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="F22" s="32">
+      <c r="F22" s="30">
         <v>51500</v>
       </c>
-      <c r="G22" s="32">
+      <c r="G22" s="30">
         <f>F22*D22</f>
         <v>51500</v>
       </c>
-      <c r="H22" s="27" t="s">
+      <c r="H22" s="25" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="22">
+      <c r="B23" s="21">
         <v>20</v>
       </c>
-      <c r="C23" s="31" t="s">
+      <c r="C23" s="29" t="s">
         <v>834</v>
       </c>
-      <c r="D23" s="33">
+      <c r="D23" s="31">
         <v>46.8</v>
       </c>
-      <c r="E23" s="27" t="s">
+      <c r="E23" s="25" t="s">
         <v>759</v>
       </c>
-      <c r="F23" s="32">
+      <c r="F23" s="30">
         <v>670</v>
       </c>
-      <c r="G23" s="32">
+      <c r="G23" s="30">
         <f>F23*D23</f>
         <v>31355.999999999996</v>
       </c>
-      <c r="H23" s="27" t="s">
+      <c r="H23" s="25" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="22">
+      <c r="B24" s="21">
         <v>21</v>
       </c>
-      <c r="C24" s="31" t="s">
+      <c r="C24" s="29" t="s">
         <v>835</v>
       </c>
-      <c r="D24" s="33">
+      <c r="D24" s="31">
         <v>37.200000000000003</v>
       </c>
-      <c r="E24" s="27" t="s">
+      <c r="E24" s="25" t="s">
         <v>759</v>
       </c>
-      <c r="F24" s="32">
+      <c r="F24" s="30">
         <v>670</v>
       </c>
-      <c r="G24" s="32">
+      <c r="G24" s="30">
         <f>F24*D24</f>
         <v>24924.000000000004</v>
       </c>
-      <c r="H24" s="27" t="s">
+      <c r="H24" s="25" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="22">
+      <c r="B25" s="21">
         <v>22</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="20" t="s">
         <v>777</v>
       </c>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
       <c r="F25" s="19"/>
       <c r="G25" s="19">
         <f>F25*D25</f>
         <v>0</v>
       </c>
-      <c r="H25" s="22" t="s">
+      <c r="H25" s="21" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="22">
+      <c r="B26" s="21">
         <v>23</v>
       </c>
-      <c r="C26" s="25" t="s">
+      <c r="C26" s="23" t="s">
         <v>785</v>
       </c>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26">
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24">
         <f>F26*D26</f>
         <v>0</v>
       </c>
-      <c r="H26" s="24" t="s">
+      <c r="H26" s="22" t="s">
         <v>576</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B27" s="22">
+      <c r="B27" s="21">
         <v>24</v>
       </c>
-      <c r="C27" s="25" t="s">
+      <c r="C27" s="23" t="s">
         <v>786</v>
       </c>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26">
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24">
         <f>F27*D27</f>
         <v>0</v>
       </c>
-      <c r="H27" s="24" t="s">
+      <c r="H27" s="22" t="s">
         <v>576</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B28" s="22">
+      <c r="B28" s="21">
         <v>25</v>
       </c>
-      <c r="C28" s="25" t="s">
+      <c r="C28" s="23" t="s">
         <v>787</v>
       </c>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26">
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24">
         <f>F28*D28</f>
         <v>0</v>
       </c>
-      <c r="H28" s="24" t="s">
+      <c r="H28" s="22" t="s">
         <v>576</v>
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B29" s="22">
+      <c r="B29" s="21">
         <v>26</v>
       </c>
-      <c r="C29" s="25" t="s">
+      <c r="C29" s="23" t="s">
         <v>788</v>
       </c>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26">
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24">
         <f>F29*D29</f>
         <v>0</v>
       </c>
-      <c r="H29" s="24" t="s">
+      <c r="H29" s="22" t="s">
         <v>576</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B30" s="22">
+      <c r="B30" s="21">
         <v>27</v>
       </c>
-      <c r="C30" s="31" t="s">
+      <c r="C30" s="29" t="s">
         <v>757</v>
       </c>
-      <c r="D30" s="27">
+      <c r="D30" s="25">
         <f>(2000*1.05)*0.15</f>
         <v>315</v>
       </c>
-      <c r="E30" s="27" t="s">
+      <c r="E30" s="25" t="s">
         <v>759</v>
       </c>
-      <c r="F30" s="32">
+      <c r="F30" s="30">
         <v>670</v>
       </c>
-      <c r="G30" s="32">
+      <c r="G30" s="30">
         <f>F30*D30</f>
         <v>211050</v>
       </c>
-      <c r="H30" s="27" t="s">
+      <c r="H30" s="25" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B31" s="22">
+      <c r="B31" s="21">
         <v>28</v>
       </c>
-      <c r="C31" s="31" t="s">
+      <c r="C31" s="29" t="s">
         <v>775</v>
       </c>
-      <c r="D31" s="33">
+      <c r="D31" s="31">
         <f>2000/13*2</f>
         <v>307.69230769230768</v>
       </c>
-      <c r="E31" s="27" t="s">
+      <c r="E31" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="F31" s="32">
+      <c r="F31" s="30">
         <v>220.5</v>
       </c>
-      <c r="G31" s="32">
+      <c r="G31" s="30">
         <f>F31*D31</f>
         <v>67846.153846153844</v>
       </c>
-      <c r="H31" s="27" t="s">
+      <c r="H31" s="25" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B32" s="22">
+      <c r="B32" s="21">
         <v>29</v>
       </c>
-      <c r="C32" s="31" t="s">
+      <c r="C32" s="29" t="s">
         <v>758</v>
       </c>
-      <c r="D32" s="27">
+      <c r="D32" s="25">
         <v>167</v>
       </c>
-      <c r="E32" s="27" t="s">
+      <c r="E32" s="25" t="s">
         <v>810</v>
       </c>
-      <c r="F32" s="32">
+      <c r="F32" s="30">
         <v>56.2</v>
       </c>
-      <c r="G32" s="32">
+      <c r="G32" s="30">
         <f>F32*D32</f>
         <v>9385.4</v>
       </c>
-      <c r="H32" s="27" t="s">
+      <c r="H32" s="25" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B33" s="22">
+      <c r="B33" s="21">
         <v>30</v>
       </c>
-      <c r="C33" s="31" t="s">
+      <c r="C33" s="29" t="s">
         <v>762</v>
       </c>
-      <c r="D33" s="27">
+      <c r="D33" s="25">
         <v>1000</v>
       </c>
-      <c r="E33" s="27" t="s">
+      <c r="E33" s="25" t="s">
         <v>763</v>
       </c>
-      <c r="F33" s="32">
+      <c r="F33" s="30">
         <v>7.3</v>
       </c>
-      <c r="G33" s="32">
+      <c r="G33" s="30">
         <f>F33*D33</f>
         <v>7300</v>
       </c>
-      <c r="H33" s="27" t="s">
+      <c r="H33" s="25" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="22">
+      <c r="B34" s="21">
         <v>31</v>
       </c>
-      <c r="C34" s="31" t="s">
+      <c r="C34" s="29" t="s">
         <v>801</v>
       </c>
-      <c r="D34" s="27">
+      <c r="D34" s="25">
         <v>315</v>
       </c>
-      <c r="E34" s="27" t="s">
+      <c r="E34" s="25" t="s">
         <v>759</v>
       </c>
-      <c r="F34" s="32">
+      <c r="F34" s="30">
         <v>50</v>
       </c>
-      <c r="G34" s="32">
+      <c r="G34" s="30">
         <f>F34*D34</f>
         <v>15750</v>
       </c>
-      <c r="H34" s="27" t="s">
+      <c r="H34" s="25" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="22">
+      <c r="B35" s="21">
         <v>32</v>
       </c>
-      <c r="C35" s="31" t="s">
+      <c r="C35" s="29" t="s">
         <v>768</v>
       </c>
-      <c r="D35" s="27">
-        <v>1</v>
-      </c>
-      <c r="E35" s="27" t="s">
+      <c r="D35" s="25">
+        <v>1</v>
+      </c>
+      <c r="E35" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="F35" s="32">
+      <c r="F35" s="30">
         <v>49800</v>
       </c>
-      <c r="G35" s="32">
+      <c r="G35" s="30">
         <f>F35*D35</f>
         <v>49800</v>
       </c>
-      <c r="H35" s="27" t="s">
+      <c r="H35" s="25" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B36" s="22">
+      <c r="B36" s="21">
         <v>33</v>
       </c>
-      <c r="C36" s="25" t="s">
+      <c r="C36" s="23" t="s">
         <v>803</v>
       </c>
-      <c r="D36" s="24">
-        <v>1</v>
-      </c>
-      <c r="E36" s="24" t="s">
+      <c r="D36" s="22">
+        <v>1</v>
+      </c>
+      <c r="E36" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26">
+      <c r="F36" s="24"/>
+      <c r="G36" s="24">
         <f>F36*D36</f>
         <v>0</v>
       </c>
-      <c r="H36" s="24" t="s">
+      <c r="H36" s="22" t="s">
         <v>804</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B37" s="22">
+      <c r="B37" s="21">
         <v>34</v>
       </c>
-      <c r="C37" s="25" t="s">
+      <c r="C37" s="23" t="s">
         <v>814</v>
       </c>
-      <c r="D37" s="24">
-        <v>1</v>
-      </c>
-      <c r="E37" s="24" t="s">
+      <c r="D37" s="22">
+        <v>1</v>
+      </c>
+      <c r="E37" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26">
+      <c r="F37" s="24"/>
+      <c r="G37" s="24">
         <f>F37*D37</f>
         <v>0</v>
       </c>
-      <c r="H37" s="24" t="s">
+      <c r="H37" s="22" t="s">
         <v>804</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B38" s="22">
+      <c r="B38" s="21">
         <v>35</v>
       </c>
-      <c r="C38" s="21" t="s">
+      <c r="C38" s="20" t="s">
         <v>791</v>
       </c>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="21"/>
       <c r="F38" s="19"/>
       <c r="G38" s="19">
         <f>F38*D38</f>
         <v>0</v>
       </c>
-      <c r="H38" s="22" t="s">
+      <c r="H38" s="21" t="s">
         <v>419</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B39" s="22">
+      <c r="B39" s="21">
         <v>36</v>
       </c>
-      <c r="C39" s="46" t="s">
+      <c r="C39" s="44" t="s">
         <v>843</v>
       </c>
-      <c r="D39" s="27">
+      <c r="D39" s="25">
         <v>1455.89</v>
       </c>
-      <c r="E39" s="27" t="s">
+      <c r="E39" s="25" t="s">
         <v>761</v>
       </c>
-      <c r="F39" s="36">
+      <c r="F39" s="34">
         <v>95.9</v>
       </c>
-      <c r="G39" s="36">
+      <c r="G39" s="34">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>139619.85100000002</v>
       </c>
-      <c r="H39" s="27" t="s">
+      <c r="H39" s="25" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B40" s="22">
+      <c r="B40" s="21">
         <v>37</v>
       </c>
-      <c r="C40" s="31" t="s">
+      <c r="C40" s="29" t="s">
         <v>844</v>
       </c>
-      <c r="D40" s="27">
+      <c r="D40" s="25">
         <v>706.94</v>
       </c>
-      <c r="E40" s="27" t="s">
+      <c r="E40" s="25" t="s">
         <v>761</v>
       </c>
-      <c r="F40" s="36">
+      <c r="F40" s="34">
         <v>95.9</v>
       </c>
-      <c r="G40" s="36">
+      <c r="G40" s="34">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>67795.546000000002</v>
       </c>
-      <c r="H40" s="27" t="s">
+      <c r="H40" s="25" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B41" s="22">
+      <c r="B41" s="21">
         <v>38</v>
       </c>
-      <c r="C41" s="28" t="s">
+      <c r="C41" s="26" t="s">
         <v>845</v>
       </c>
-      <c r="D41" s="27">
+      <c r="D41" s="25">
         <v>44</v>
       </c>
-      <c r="E41" s="27" t="s">
+      <c r="E41" s="25" t="s">
         <v>849</v>
       </c>
-      <c r="F41" s="36">
+      <c r="F41" s="34">
         <v>95</v>
       </c>
-      <c r="G41" s="36">
+      <c r="G41" s="34">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>4180</v>
       </c>
-      <c r="H41" s="27" t="s">
+      <c r="H41" s="25" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B42" s="22">
+      <c r="B42" s="21">
         <v>39</v>
       </c>
-      <c r="C42" s="28" t="s">
+      <c r="C42" s="26" t="s">
         <v>846</v>
       </c>
-      <c r="D42" s="27">
+      <c r="D42" s="25">
         <v>3</v>
       </c>
-      <c r="E42" s="27" t="s">
+      <c r="E42" s="25" t="s">
         <v>849</v>
       </c>
-      <c r="F42" s="36">
+      <c r="F42" s="34">
         <v>35</v>
       </c>
-      <c r="G42" s="36">
+      <c r="G42" s="34">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>105</v>
       </c>
-      <c r="H42" s="27" t="s">
+      <c r="H42" s="25" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B43" s="22">
+      <c r="B43" s="21">
         <v>40</v>
       </c>
-      <c r="C43" s="28" t="s">
+      <c r="C43" s="26" t="s">
         <v>847</v>
       </c>
-      <c r="D43" s="27">
+      <c r="D43" s="25">
         <v>126</v>
       </c>
-      <c r="E43" s="27" t="s">
+      <c r="E43" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="F43" s="36">
+      <c r="F43" s="34">
         <v>25.9</v>
       </c>
-      <c r="G43" s="36">
+      <c r="G43" s="34">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>3263.3999999999996</v>
       </c>
-      <c r="H43" s="27" t="s">
+      <c r="H43" s="25" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B44" s="22">
+      <c r="B44" s="21">
         <v>41</v>
       </c>
-      <c r="C44" s="28" t="s">
+      <c r="C44" s="26" t="s">
         <v>848</v>
       </c>
-      <c r="D44" s="27">
-        <v>1</v>
-      </c>
-      <c r="E44" s="27" t="s">
+      <c r="D44" s="25">
+        <v>1</v>
+      </c>
+      <c r="E44" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="F44" s="36">
+      <c r="F44" s="34">
         <v>1750</v>
       </c>
-      <c r="G44" s="36">
+      <c r="G44" s="34">
         <f>F44*D44</f>
         <v>1750</v>
       </c>
-      <c r="H44" s="27" t="s">
+      <c r="H44" s="25" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B45" s="22">
+      <c r="B45" s="21">
         <v>42</v>
       </c>
-      <c r="C45" s="31" t="s">
+      <c r="C45" s="29" t="s">
         <v>784</v>
       </c>
-      <c r="D45" s="27">
-        <v>1</v>
-      </c>
-      <c r="E45" s="27" t="s">
+      <c r="D45" s="25">
+        <v>1</v>
+      </c>
+      <c r="E45" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="F45" s="36">
+      <c r="F45" s="34">
         <v>157963.5</v>
       </c>
-      <c r="G45" s="36">
+      <c r="G45" s="34">
         <f>F45*D45</f>
         <v>157963.5</v>
       </c>
-      <c r="H45" s="27" t="s">
+      <c r="H45" s="25" t="s">
         <v>783</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B46" s="22">
+      <c r="B46" s="21">
         <v>43</v>
       </c>
-      <c r="C46" s="25" t="s">
+      <c r="C46" s="23" t="s">
         <v>839</v>
       </c>
-      <c r="D46" s="24"/>
-      <c r="E46" s="24"/>
-      <c r="F46" s="26"/>
-      <c r="G46" s="26">
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="24"/>
+      <c r="G46" s="24">
         <f>F46*D46</f>
         <v>0</v>
       </c>
-      <c r="H46" s="24" t="s">
+      <c r="H46" s="22" t="s">
         <v>840</v>
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B47" s="24"/>
-      <c r="C47" s="25"/>
-      <c r="D47" s="24"/>
-      <c r="E47" s="24"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="26"/>
-      <c r="H47" s="24"/>
+      <c r="B47" s="22"/>
+      <c r="C47" s="23"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="24"/>
+      <c r="G47" s="24"/>
+      <c r="H47" s="22"/>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B48" s="24"/>
-      <c r="C48" s="25"/>
-      <c r="D48" s="24"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="26"/>
-      <c r="G48" s="26"/>
-      <c r="H48" s="24"/>
+      <c r="B48" s="22"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="24"/>
+      <c r="G48" s="24"/>
+      <c r="H48" s="22"/>
     </row>
     <row r="49" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G49" s="16">
@@ -13705,7 +13712,7 @@
     <col min="7" max="7" width="15.85546875" style="15" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" style="15" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.85546875" style="14" customWidth="1"/>
-    <col min="10" max="10" width="64.7109375" style="52" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="64.7109375" style="50" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="16" style="14" customWidth="1"/>
     <col min="14" max="14" width="18.42578125" customWidth="1"/>
     <col min="15" max="15" width="25" customWidth="1"/>
@@ -13749,33 +13756,33 @@
       <c r="I3" t="s">
         <v>767</v>
       </c>
-      <c r="J3" s="52"/>
+      <c r="J3" s="50"/>
       <c r="P3" s="14" t="s">
         <v>826</v>
       </c>
     </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B4" s="22">
+    <row r="4" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="21">
         <v>1</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="23" t="s">
         <v>793</v>
       </c>
-      <c r="E4" s="24">
-        <v>1</v>
-      </c>
-      <c r="F4" s="24" t="s">
+      <c r="E4" s="22">
+        <v>1</v>
+      </c>
+      <c r="F4" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26">
+      <c r="G4" s="24"/>
+      <c r="H4" s="24">
         <f>G4*E4</f>
         <v>0</v>
       </c>
-      <c r="I4" s="24" t="s">
+      <c r="I4" s="22" t="s">
         <v>813</v>
       </c>
       <c r="O4" s="14" t="s">
@@ -13791,63 +13798,63 @@
         <v>822</v>
       </c>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B5" s="22">
+    <row r="5" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="21">
         <v>2</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="25" t="s">
         <v>807</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="29" t="s">
         <v>851</v>
       </c>
-      <c r="E5" s="27">
-        <v>1</v>
-      </c>
-      <c r="F5" s="27" t="s">
+      <c r="E5" s="25">
+        <v>1</v>
+      </c>
+      <c r="F5" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G5" s="36">
+      <c r="G5" s="34">
         <v>486032</v>
       </c>
-      <c r="H5" s="36">
+      <c r="H5" s="34">
         <f>G5*E5</f>
         <v>486032</v>
       </c>
-      <c r="I5" s="27" t="s">
+      <c r="I5" s="25" t="s">
         <v>782</v>
       </c>
-      <c r="N5" s="37" t="s">
+      <c r="N5" s="35" t="s">
         <v>772</v>
       </c>
-      <c r="O5" s="39">
+      <c r="O5" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Pré Moldado",Tabela24[Preço Total])</f>
         <v>992504</v>
       </c>
-      <c r="P5" s="43">
+      <c r="P5" s="41">
         <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
-        <v>0.23836458165979033</v>
-      </c>
-      <c r="Q5" s="45">
+        <v>0.27943619534004144</v>
+      </c>
+      <c r="Q5" s="43">
         <f>P5</f>
-        <v>0.23836458165979033</v>
+        <v>0.27943619534004144</v>
       </c>
       <c r="R5" t="s">
         <v>823</v>
       </c>
     </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B6" s="22">
+    <row r="6" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="21">
         <v>3</v>
       </c>
       <c r="C6" s="17"/>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="20" t="s">
         <v>853</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="21">
         <v>4</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="21" t="s">
         <v>760</v>
       </c>
       <c r="G6" s="19"/>
@@ -13858,37 +13865,37 @@
       <c r="I6" s="17" t="s">
         <v>782</v>
       </c>
-      <c r="N6" s="44" t="s">
+      <c r="N6" s="42" t="s">
         <v>783</v>
       </c>
-      <c r="O6" s="39">
+      <c r="O6" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Terraplanagem",Tabela24[Preço Total])</f>
         <v>791792.51</v>
       </c>
-      <c r="P6" s="43">
+      <c r="P6" s="41">
         <f t="shared" si="0"/>
-        <v>0.19016073527915792</v>
-      </c>
-      <c r="Q6" s="45">
+        <v>0.22292654386596095</v>
+      </c>
+      <c r="Q6" s="43">
         <f>P6+Q5</f>
-        <v>0.42852531693894824</v>
+        <v>0.50236273920600238</v>
       </c>
       <c r="R6" t="s">
         <v>823</v>
       </c>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B7" s="22">
+    <row r="7" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="21">
         <v>4</v>
       </c>
       <c r="C7" s="17"/>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="20" t="s">
         <v>852</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="21">
         <v>6</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="21" t="s">
         <v>760</v>
       </c>
       <c r="G7" s="19"/>
@@ -13899,1373 +13906,1373 @@
       <c r="I7" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="N7" s="37" t="s">
+      <c r="N7" s="35" t="s">
         <v>635</v>
       </c>
-      <c r="O7" s="39">
+      <c r="O7" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Piso",Tabela24[Preço Total])</f>
-        <v>611997.5</v>
-      </c>
-      <c r="P7" s="43">
+        <v>0</v>
+      </c>
+      <c r="P7" s="41">
         <f t="shared" si="0"/>
-        <v>0.14698029233568582</v>
-      </c>
-    </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B8" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="21">
         <v>5</v>
       </c>
-      <c r="C8" s="34"/>
-      <c r="D8" s="25" t="s">
+      <c r="C8" s="32"/>
+      <c r="D8" s="23" t="s">
         <v>858</v>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="22">
         <v>6</v>
       </c>
-      <c r="F8" s="24" t="s">
+      <c r="F8" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="G8" s="26"/>
-      <c r="H8" s="51">
+      <c r="G8" s="24"/>
+      <c r="H8" s="49">
         <f>G8*E8</f>
         <v>0</v>
       </c>
       <c r="I8" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="N8" s="44" t="s">
+      <c r="N8" s="42" t="s">
         <v>804</v>
       </c>
-      <c r="O8" s="39">
+      <c r="O8" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
         <v>729700</v>
       </c>
-      <c r="P8" s="43">
+      <c r="P8" s="41">
         <f t="shared" si="0"/>
-        <v>0.17524829646746914</v>
-      </c>
-    </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B9" s="22">
+        <v>0.20544460449492216</v>
+      </c>
+    </row>
+    <row r="9" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="21">
         <v>6</v>
       </c>
-      <c r="C9" s="34"/>
-      <c r="D9" s="25" t="s">
-        <v>862</v>
-      </c>
-      <c r="E9" s="24">
-        <v>1</v>
-      </c>
-      <c r="F9" s="24" t="s">
+      <c r="C9" s="32"/>
+      <c r="D9" s="23" t="s">
+        <v>861</v>
+      </c>
+      <c r="E9" s="22">
+        <v>1</v>
+      </c>
+      <c r="F9" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="G9" s="26"/>
-      <c r="H9" s="51">
+      <c r="G9" s="24"/>
+      <c r="H9" s="49">
         <f>G9*E9</f>
         <v>0</v>
       </c>
       <c r="I9" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="N9" s="41" t="s">
+      <c r="N9" s="39" t="s">
         <v>771</v>
       </c>
-      <c r="O9" s="39">
+      <c r="O9" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Fundação",Tabela24[Preço Total])</f>
         <v>416702.4</v>
       </c>
-      <c r="P9" s="43">
+      <c r="P9" s="41">
         <f t="shared" si="0"/>
-        <v>0.10007727248719463</v>
-      </c>
-    </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B10" s="22">
+        <v>0.11732117275604338</v>
+      </c>
+    </row>
+    <row r="10" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="21">
         <v>7</v>
       </c>
       <c r="C10" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="23" t="s">
         <v>789</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="22">
         <v>26</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="F10" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26">
+      <c r="G10" s="24"/>
+      <c r="H10" s="24">
         <f>G10*E10</f>
         <v>0</v>
       </c>
-      <c r="I10" s="24" t="s">
+      <c r="I10" s="22" t="s">
         <v>643</v>
       </c>
-      <c r="N10" s="41" t="s">
+      <c r="N10" s="39" t="s">
         <v>774</v>
       </c>
-      <c r="O10" s="39">
+      <c r="O10" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
         <v>66534.056568800006</v>
       </c>
-      <c r="P10" s="43">
+      <c r="P10" s="41">
         <f t="shared" si="0"/>
-        <v>1.5979142210158184E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B11" s="22">
+        <v>1.8732442013457442E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="21">
         <v>8</v>
       </c>
-      <c r="C11" s="27" t="s">
+      <c r="C11" s="25" t="s">
         <v>807</v>
       </c>
-      <c r="D11" s="47" t="s">
+      <c r="D11" s="45" t="s">
         <v>790</v>
       </c>
-      <c r="E11" s="48">
+      <c r="E11" s="46">
         <v>600</v>
       </c>
-      <c r="F11" s="48" t="s">
+      <c r="F11" s="46" t="s">
         <v>761</v>
       </c>
-      <c r="G11" s="49">
+      <c r="G11" s="47">
         <v>3.35</v>
       </c>
-      <c r="H11" s="49">
+      <c r="H11" s="47">
         <f>G11*E11</f>
         <v>2010</v>
       </c>
-      <c r="I11" s="48" t="s">
+      <c r="I11" s="46" t="s">
         <v>643</v>
       </c>
-      <c r="N11" s="40" t="s">
+      <c r="N11" s="38" t="s">
         <v>782</v>
       </c>
-      <c r="O11" s="39">
+      <c r="O11" s="37">
         <f>SUMIF(Tabela24[Aplicação],"AVCB",Tabela24[Preço Total])</f>
         <v>486032</v>
       </c>
-      <c r="P11" s="43">
+      <c r="P11" s="41">
         <f t="shared" si="0"/>
-        <v>0.11672780598694939</v>
-      </c>
-    </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B12" s="22">
+        <v>0.13684069071108126</v>
+      </c>
+    </row>
+    <row r="12" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="21">
         <v>9</v>
       </c>
       <c r="C12" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="23" t="s">
         <v>812</v>
       </c>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26">
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24">
         <f>G12*E12</f>
         <v>0</v>
       </c>
-      <c r="I12" s="24" t="s">
+      <c r="I12" s="22" t="s">
         <v>643</v>
       </c>
-      <c r="N12" s="40" t="s">
+      <c r="N12" s="38" t="s">
         <v>449</v>
       </c>
-      <c r="O12" s="39">
+      <c r="O12" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Drenagem",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
-      <c r="P12" s="43">
+      <c r="P12" s="41">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B13" s="22">
+    <row r="13" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="21">
         <v>10</v>
       </c>
       <c r="C13" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D13" s="31" t="s">
+      <c r="D13" s="29" t="s">
         <v>829</v>
       </c>
-      <c r="E13" s="27">
+      <c r="E13" s="25">
         <v>54</v>
       </c>
-      <c r="F13" s="27" t="s">
+      <c r="F13" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G13" s="36">
+      <c r="G13" s="34">
         <v>243.39</v>
       </c>
-      <c r="H13" s="36">
+      <c r="H13" s="34">
         <f>G13*E13</f>
         <v>13143.06</v>
       </c>
-      <c r="I13" s="27" t="s">
+      <c r="I13" s="25" t="s">
         <v>830</v>
       </c>
-      <c r="N13" s="40"/>
-      <c r="O13" s="39"/>
-      <c r="P13" s="43"/>
-    </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B14" s="22">
+      <c r="N13" s="38"/>
+      <c r="O13" s="37"/>
+      <c r="P13" s="41"/>
+    </row>
+    <row r="14" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="21">
         <v>11</v>
       </c>
       <c r="C14" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D14" s="31" t="s">
+      <c r="D14" s="29" t="s">
         <v>831</v>
       </c>
-      <c r="E14" s="27">
+      <c r="E14" s="25">
         <v>30</v>
       </c>
-      <c r="F14" s="27" t="s">
+      <c r="F14" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G14" s="36">
+      <c r="G14" s="34">
         <v>119.7</v>
       </c>
-      <c r="H14" s="36">
+      <c r="H14" s="34">
         <f>G14*E14</f>
         <v>3591</v>
       </c>
-      <c r="I14" s="27" t="s">
+      <c r="I14" s="25" t="s">
         <v>830</v>
       </c>
-      <c r="N14" s="40" t="s">
+      <c r="N14" s="38" t="s">
         <v>774</v>
       </c>
-      <c r="O14" s="39">
+      <c r="O14" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
         <v>66534.056568800006</v>
       </c>
-      <c r="P14" s="43">
+      <c r="P14" s="41">
         <f t="shared" si="0"/>
-        <v>1.5979142210158184E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B15" s="22">
+        <v>1.8732442013457442E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="21">
         <v>12</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="25" t="s">
         <v>807</v>
       </c>
-      <c r="D15" s="31" t="s">
+      <c r="D15" s="29" t="s">
         <v>828</v>
       </c>
-      <c r="E15" s="48">
+      <c r="E15" s="46">
         <v>390</v>
       </c>
-      <c r="F15" s="27" t="s">
+      <c r="F15" s="25" t="s">
         <v>761</v>
       </c>
-      <c r="G15" s="36">
+      <c r="G15" s="34">
         <v>38.116666600000002</v>
       </c>
-      <c r="H15" s="36">
+      <c r="H15" s="34">
         <f>G15*E15</f>
         <v>14865.499974</v>
       </c>
-      <c r="I15" s="27" t="s">
+      <c r="I15" s="25" t="s">
         <v>830</v>
       </c>
-      <c r="N15" s="40" t="s">
+      <c r="N15" s="38" t="s">
         <v>643</v>
       </c>
-      <c r="O15" s="39">
+      <c r="O15" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Elétrica",Tabela24[Preço Total])</f>
         <v>2010</v>
       </c>
-      <c r="P15" s="43">
+      <c r="P15" s="41">
         <f t="shared" si="0"/>
-        <v>4.8273136343649853E-4</v>
-      </c>
-    </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B16" s="22">
+        <v>5.6590880503603334E-4</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="21">
         <v>13</v>
       </c>
       <c r="C16" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D16" s="31" t="s">
+      <c r="D16" s="29" t="s">
         <v>829</v>
       </c>
-      <c r="E16" s="33">
+      <c r="E16" s="31">
         <f>(84*1.02)*2*1.02</f>
         <v>174.78720000000001</v>
       </c>
-      <c r="F16" s="27" t="s">
+      <c r="F16" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G16" s="36">
+      <c r="G16" s="34">
         <v>243.39</v>
       </c>
-      <c r="H16" s="36">
+      <c r="H16" s="34">
         <f>G16*E16</f>
         <v>42541.456608</v>
       </c>
-      <c r="I16" s="27" t="s">
+      <c r="I16" s="25" t="s">
         <v>774</v>
       </c>
-      <c r="N16" s="40"/>
-      <c r="O16" s="39"/>
-      <c r="P16" s="43"/>
-    </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B17" s="22">
+      <c r="N16" s="38"/>
+      <c r="O16" s="37"/>
+      <c r="P16" s="41"/>
+    </row>
+    <row r="17" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="21">
         <v>14</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="25" t="s">
         <v>807</v>
       </c>
-      <c r="D17" s="31" t="s">
+      <c r="D17" s="29" t="s">
         <v>828</v>
       </c>
-      <c r="E17" s="27">
+      <c r="E17" s="25">
         <f>84*7</f>
         <v>588</v>
       </c>
-      <c r="F17" s="27" t="s">
+      <c r="F17" s="25" t="s">
         <v>761</v>
       </c>
-      <c r="G17" s="36">
+      <c r="G17" s="34">
         <v>38.116666600000002</v>
       </c>
-      <c r="H17" s="36">
+      <c r="H17" s="34">
         <f>G17*E17</f>
         <v>22412.599960800002</v>
       </c>
-      <c r="I17" s="27" t="s">
+      <c r="I17" s="25" t="s">
         <v>774</v>
       </c>
-      <c r="N17" s="40"/>
-      <c r="O17" s="39"/>
-      <c r="P17" s="43"/>
-    </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B18" s="22">
+      <c r="N17" s="38"/>
+      <c r="O17" s="37"/>
+      <c r="P17" s="41"/>
+    </row>
+    <row r="18" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="21">
         <v>15</v>
       </c>
-      <c r="C18" s="27"/>
-      <c r="D18" s="31" t="s">
+      <c r="C18" s="25"/>
+      <c r="D18" s="29" t="s">
         <v>856</v>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="25">
         <v>30</v>
       </c>
-      <c r="F18" s="27" t="s">
+      <c r="F18" s="25" t="s">
         <v>849</v>
       </c>
-      <c r="G18" s="36">
+      <c r="G18" s="34">
         <v>24</v>
       </c>
-      <c r="H18" s="36">
+      <c r="H18" s="34">
         <f>G18*E18</f>
         <v>720</v>
       </c>
-      <c r="I18" s="27" t="s">
+      <c r="I18" s="25" t="s">
         <v>774</v>
       </c>
-      <c r="N18" s="40"/>
-      <c r="O18" s="39"/>
-      <c r="P18" s="43"/>
-    </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B19" s="22">
+      <c r="N18" s="38"/>
+      <c r="O18" s="37"/>
+      <c r="P18" s="41"/>
+    </row>
+    <row r="19" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="21">
         <v>16</v>
       </c>
-      <c r="C19" s="27"/>
-      <c r="D19" s="31" t="s">
+      <c r="C19" s="25"/>
+      <c r="D19" s="29" t="s">
         <v>857</v>
       </c>
-      <c r="E19" s="27">
-        <v>1</v>
-      </c>
-      <c r="F19" s="27" t="s">
+      <c r="E19" s="25">
+        <v>1</v>
+      </c>
+      <c r="F19" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G19" s="36">
+      <c r="G19" s="34">
         <v>860</v>
       </c>
-      <c r="H19" s="36">
+      <c r="H19" s="34">
         <f>G19*E19</f>
         <v>860</v>
       </c>
-      <c r="I19" s="27" t="s">
+      <c r="I19" s="25" t="s">
         <v>774</v>
       </c>
-      <c r="N19" s="40" t="s">
+      <c r="N19" s="38" t="s">
         <v>576</v>
       </c>
-      <c r="O19" s="39">
+      <c r="O19" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Pintura",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
-      <c r="P19" s="43">
+      <c r="P19" s="41">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B20" s="22">
+    <row r="20" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="21">
         <v>17</v>
       </c>
       <c r="C20" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D20" s="25" t="s">
+      <c r="D20" s="23" t="s">
         <v>779</v>
       </c>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24" t="s">
+      <c r="E20" s="22"/>
+      <c r="F20" s="22" t="s">
         <v>761</v>
       </c>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26">
+      <c r="G20" s="24"/>
+      <c r="H20" s="24">
         <f>G20*E20</f>
         <v>0</v>
       </c>
-      <c r="I20" s="24" t="s">
+      <c r="I20" s="22" t="s">
         <v>774</v>
       </c>
-      <c r="N20" s="40" t="s">
+      <c r="N20" s="38" t="s">
         <v>813</v>
       </c>
-      <c r="O20" s="39">
+      <c r="O20" s="37">
         <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
-      <c r="P20" s="43">
+      <c r="P20" s="41">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B21" s="22">
+    <row r="21" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="21">
         <v>18</v>
       </c>
       <c r="C21" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D21" s="25" t="s">
+      <c r="D21" s="23" t="s">
         <v>780</v>
       </c>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="26">
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24">
         <f>G21*E21</f>
         <v>0</v>
       </c>
-      <c r="I21" s="24" t="s">
+      <c r="I21" s="22" t="s">
         <v>774</v>
       </c>
-      <c r="N21" s="40"/>
-      <c r="O21" s="39"/>
-      <c r="P21" s="43"/>
-    </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B22" s="22">
+      <c r="N21" s="38"/>
+      <c r="O21" s="37"/>
+      <c r="P21" s="41"/>
+    </row>
+    <row r="22" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="21">
         <v>19</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D22" s="25" t="s">
+      <c r="D22" s="23" t="s">
         <v>781</v>
       </c>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="26">
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24">
         <f>G22*E22</f>
         <v>0</v>
       </c>
-      <c r="I22" s="24" t="s">
+      <c r="I22" s="22" t="s">
         <v>774</v>
       </c>
-      <c r="N22" s="40"/>
-      <c r="O22" s="39"/>
-      <c r="P22" s="43"/>
-    </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B23" s="22">
+      <c r="N22" s="38"/>
+      <c r="O22" s="37"/>
+      <c r="P22" s="41"/>
+    </row>
+    <row r="23" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="21">
         <v>20</v>
       </c>
       <c r="C23" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D23" s="25" t="s">
+      <c r="D23" s="23" t="s">
         <v>816</v>
       </c>
-      <c r="E23" s="24">
-        <v>1</v>
-      </c>
-      <c r="F23" s="24"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26">
+      <c r="E23" s="22">
+        <v>1</v>
+      </c>
+      <c r="F23" s="22"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24">
         <f>G23*E23</f>
         <v>0</v>
       </c>
-      <c r="I23" s="24" t="s">
+      <c r="I23" s="22" t="s">
         <v>774</v>
       </c>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B24" s="22">
+    <row r="24" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="21">
         <v>21</v>
       </c>
       <c r="C24" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D24" s="31" t="s">
+      <c r="D24" s="29" t="s">
         <v>794</v>
       </c>
-      <c r="E24" s="27">
-        <v>1</v>
-      </c>
-      <c r="F24" s="27" t="s">
+      <c r="E24" s="25">
+        <v>1</v>
+      </c>
+      <c r="F24" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G24" s="32">
+      <c r="G24" s="30">
         <v>6000</v>
       </c>
-      <c r="H24" s="32">
+      <c r="H24" s="30">
         <f>G24*E24</f>
         <v>6000</v>
       </c>
-      <c r="I24" s="27" t="s">
+      <c r="I24" s="25" t="s">
         <v>771</v>
       </c>
-      <c r="N24" s="40" t="s">
+      <c r="N24" s="38" t="s">
         <v>819</v>
       </c>
-      <c r="O24" s="42">
+      <c r="O24" s="40">
         <f>SUM(O5:O20)</f>
-        <v>4163806.5231375997</v>
-      </c>
-    </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B25" s="22">
+        <v>3551809.0231375997</v>
+      </c>
+    </row>
+    <row r="25" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="21">
         <v>22</v>
       </c>
       <c r="C25" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D25" s="31" t="s">
+      <c r="D25" s="29" t="s">
         <v>769</v>
       </c>
-      <c r="E25" s="27">
+      <c r="E25" s="25">
         <v>4100</v>
       </c>
-      <c r="F25" s="27" t="s">
+      <c r="F25" s="25" t="s">
         <v>836</v>
       </c>
-      <c r="G25" s="32">
+      <c r="G25" s="30">
         <v>9.65</v>
       </c>
-      <c r="H25" s="32">
+      <c r="H25" s="30">
         <f>G25*E25</f>
         <v>39565</v>
       </c>
-      <c r="I25" s="27" t="s">
+      <c r="I25" s="25" t="s">
         <v>771</v>
       </c>
       <c r="J25" s="14" t="s">
         <v>837</v>
       </c>
-      <c r="N25" s="40"/>
-      <c r="O25" s="42"/>
-    </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B26" s="22">
+      <c r="N25" s="38"/>
+      <c r="O25" s="40"/>
+    </row>
+    <row r="26" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="21">
         <v>23</v>
       </c>
       <c r="C26" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D26" s="31" t="s">
+      <c r="D26" s="29" t="s">
         <v>770</v>
       </c>
-      <c r="E26" s="27">
+      <c r="E26" s="25">
         <v>4000</v>
       </c>
-      <c r="F26" s="27" t="s">
+      <c r="F26" s="25" t="s">
         <v>836</v>
       </c>
-      <c r="G26" s="32">
+      <c r="G26" s="30">
         <v>9.65</v>
       </c>
-      <c r="H26" s="32">
+      <c r="H26" s="30">
         <f>G26*E26</f>
         <v>38600</v>
       </c>
-      <c r="I26" s="27" t="s">
+      <c r="I26" s="25" t="s">
         <v>771</v>
       </c>
       <c r="J26" s="14" t="s">
         <v>837</v>
       </c>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B27" s="22">
+    <row r="27" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="21">
         <v>24</v>
       </c>
-      <c r="C27" s="27" t="s">
+      <c r="C27" s="25" t="s">
         <v>807</v>
       </c>
-      <c r="D27" s="31" t="s">
+      <c r="D27" s="29" t="s">
         <v>827</v>
       </c>
-      <c r="E27" s="27">
-        <v>1</v>
-      </c>
-      <c r="F27" s="27" t="s">
+      <c r="E27" s="25">
+        <v>1</v>
+      </c>
+      <c r="F27" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G27" s="32">
+      <c r="G27" s="30">
         <v>164000</v>
       </c>
-      <c r="H27" s="32">
+      <c r="H27" s="30">
         <f>G27*E27</f>
         <v>164000</v>
       </c>
-      <c r="I27" s="27" t="s">
+      <c r="I27" s="25" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B28" s="22">
+    <row r="28" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="21">
         <v>25</v>
       </c>
       <c r="C28" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D28" s="31" t="s">
-        <v>867</v>
-      </c>
-      <c r="E28" s="27">
+      <c r="D28" s="29" t="s">
+        <v>866</v>
+      </c>
+      <c r="E28" s="25">
         <v>99.22</v>
       </c>
-      <c r="F28" s="27" t="s">
+      <c r="F28" s="25" t="s">
         <v>759</v>
       </c>
-      <c r="G28" s="32">
+      <c r="G28" s="30">
         <v>670</v>
       </c>
-      <c r="H28" s="32">
+      <c r="H28" s="30">
         <f>G28*E28</f>
         <v>66477.399999999994</v>
       </c>
-      <c r="I28" s="27" t="s">
+      <c r="I28" s="25" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B29" s="22">
+    <row r="29" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="21">
         <v>26</v>
       </c>
       <c r="C29" s="17"/>
-      <c r="D29" s="31" t="s">
-        <v>866</v>
-      </c>
-      <c r="E29" s="27">
+      <c r="D29" s="29" t="s">
+        <v>865</v>
+      </c>
+      <c r="E29" s="25">
         <v>68</v>
       </c>
-      <c r="F29" s="27" t="s">
+      <c r="F29" s="25" t="s">
         <v>759</v>
       </c>
-      <c r="G29" s="32">
+      <c r="G29" s="30">
         <v>670</v>
       </c>
-      <c r="H29" s="32">
+      <c r="H29" s="30">
         <f>G29*E29</f>
         <v>45560</v>
       </c>
-      <c r="I29" s="27" t="s">
+      <c r="I29" s="25" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B30" s="22">
+    <row r="30" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="21">
         <v>27</v>
       </c>
       <c r="C30" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D30" s="31" t="s">
+      <c r="D30" s="29" t="s">
         <v>833</v>
       </c>
-      <c r="E30" s="27">
-        <v>1</v>
-      </c>
-      <c r="F30" s="27" t="s">
+      <c r="E30" s="25">
+        <v>1</v>
+      </c>
+      <c r="F30" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G30" s="32">
+      <c r="G30" s="30">
         <v>56500</v>
       </c>
-      <c r="H30" s="32">
+      <c r="H30" s="30">
         <f>G30*E30</f>
         <v>56500</v>
       </c>
-      <c r="I30" s="27" t="s">
+      <c r="I30" s="25" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B31" s="22">
+    <row r="31" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="21">
         <v>28</v>
       </c>
       <c r="C31" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="D31" s="20" t="s">
         <v>777</v>
       </c>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
       <c r="G31" s="19"/>
       <c r="H31" s="19">
         <f>G31*E31</f>
         <v>0</v>
       </c>
-      <c r="I31" s="22" t="s">
+      <c r="I31" s="21" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B32" s="22">
+    <row r="32" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="21">
         <v>29</v>
       </c>
       <c r="C32" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D32" s="25" t="s">
+      <c r="D32" s="23" t="s">
         <v>785</v>
       </c>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26">
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24">
         <f>G32*E32</f>
         <v>0</v>
       </c>
-      <c r="I32" s="24" t="s">
+      <c r="I32" s="22" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B33" s="22">
+    <row r="33" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="21">
         <v>30</v>
       </c>
       <c r="C33" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D33" s="25" t="s">
+      <c r="D33" s="23" t="s">
         <v>786</v>
       </c>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26">
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24">
         <f>G33*E33</f>
         <v>0</v>
       </c>
-      <c r="I33" s="24" t="s">
+      <c r="I33" s="22" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B34" s="22">
+    <row r="34" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="21">
         <v>31</v>
       </c>
       <c r="C34" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D34" s="25" t="s">
+      <c r="D34" s="23" t="s">
         <v>787</v>
       </c>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26">
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24">
         <f>G34*E34</f>
         <v>0</v>
       </c>
-      <c r="I34" s="24" t="s">
+      <c r="I34" s="22" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B35" s="22">
+    <row r="35" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="21">
         <v>32</v>
       </c>
       <c r="C35" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D35" s="25" t="s">
+      <c r="D35" s="23" t="s">
         <v>788</v>
       </c>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="26">
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24">
         <f>G35*E35</f>
         <v>0</v>
       </c>
-      <c r="I35" s="24" t="s">
+      <c r="I35" s="22" t="s">
         <v>576</v>
       </c>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B36" s="22">
+      <c r="B36" s="21">
         <v>33</v>
       </c>
-      <c r="C36" s="27" t="s">
+      <c r="C36" s="25" t="s">
         <v>807</v>
       </c>
-      <c r="D36" s="31" t="s">
+      <c r="D36" s="29" t="s">
         <v>757</v>
       </c>
-      <c r="E36" s="33">
+      <c r="E36" s="31">
         <f>(2150*1.05)*0.15</f>
         <v>338.625</v>
       </c>
-      <c r="F36" s="27" t="s">
+      <c r="F36" s="25" t="s">
         <v>759</v>
       </c>
-      <c r="G36" s="32">
+      <c r="G36" s="30">
         <v>670</v>
       </c>
-      <c r="H36" s="32">
+      <c r="H36" s="30">
         <f>G36*E36</f>
         <v>226878.75</v>
       </c>
-      <c r="I36" s="27" t="s">
-        <v>635</v>
+      <c r="I36" s="25" t="s">
+        <v>872</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="22">
+      <c r="B37" s="21">
         <v>34</v>
       </c>
-      <c r="C37" s="27" t="s">
+      <c r="C37" s="25" t="s">
         <v>807</v>
       </c>
-      <c r="D37" s="31" t="s">
+      <c r="D37" s="29" t="s">
         <v>775</v>
       </c>
-      <c r="E37" s="33">
+      <c r="E37" s="31">
         <f>(2150/13)*2</f>
         <v>330.76923076923077</v>
       </c>
-      <c r="F37" s="27" t="s">
+      <c r="F37" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G37" s="32">
+      <c r="G37" s="30">
         <v>220.5</v>
       </c>
-      <c r="H37" s="32">
+      <c r="H37" s="30">
         <f>G37*E37</f>
         <v>72934.61538461539</v>
       </c>
-      <c r="I37" s="27" t="s">
-        <v>635</v>
+      <c r="I37" s="25" t="s">
+        <v>872</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="22">
+      <c r="B38" s="21">
         <v>35</v>
       </c>
-      <c r="C38" s="27" t="s">
+      <c r="C38" s="25" t="s">
         <v>807</v>
       </c>
-      <c r="D38" s="31" t="s">
+      <c r="D38" s="29" t="s">
         <v>758</v>
       </c>
-      <c r="E38" s="27">
+      <c r="E38" s="25">
         <f>2100/12</f>
         <v>175</v>
       </c>
-      <c r="F38" s="27" t="s">
+      <c r="F38" s="25" t="s">
         <v>761</v>
       </c>
-      <c r="G38" s="32">
+      <c r="G38" s="30">
         <v>56.2</v>
       </c>
-      <c r="H38" s="32">
+      <c r="H38" s="30">
         <f>G38*E38</f>
         <v>9835</v>
       </c>
-      <c r="I38" s="27" t="s">
-        <v>635</v>
+      <c r="I38" s="25" t="s">
+        <v>872</v>
       </c>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="22">
+      <c r="B39" s="21">
         <v>36</v>
       </c>
-      <c r="C39" s="27" t="s">
+      <c r="C39" s="25" t="s">
         <v>807</v>
       </c>
-      <c r="D39" s="31" t="s">
+      <c r="D39" s="29" t="s">
         <v>762</v>
       </c>
-      <c r="E39" s="27">
+      <c r="E39" s="25">
         <v>1000</v>
       </c>
-      <c r="F39" s="27" t="s">
+      <c r="F39" s="25" t="s">
         <v>763</v>
       </c>
-      <c r="G39" s="32">
+      <c r="G39" s="30">
         <v>7.3</v>
       </c>
-      <c r="H39" s="32">
+      <c r="H39" s="30">
         <f>G39*E39</f>
         <v>7300</v>
       </c>
-      <c r="I39" s="27" t="s">
-        <v>635</v>
+      <c r="I39" s="25" t="s">
+        <v>872</v>
       </c>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B40" s="22">
+      <c r="B40" s="21">
         <v>37</v>
       </c>
       <c r="C40" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D40" s="18" t="s">
+      <c r="D40" s="29" t="s">
         <v>811</v>
       </c>
-      <c r="E40" s="23">
+      <c r="E40" s="31">
         <f>E36</f>
         <v>338.625</v>
       </c>
-      <c r="F40" s="17" t="s">
+      <c r="F40" s="25" t="s">
         <v>766</v>
       </c>
-      <c r="G40" s="20">
+      <c r="G40" s="30">
         <v>50</v>
       </c>
-      <c r="H40" s="20">
+      <c r="H40" s="30">
         <f>G40*E40</f>
         <v>16931.25</v>
       </c>
-      <c r="I40" s="17" t="s">
-        <v>635</v>
+      <c r="I40" s="25" t="s">
+        <v>872</v>
       </c>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B41" s="22">
+      <c r="B41" s="21">
         <v>38</v>
       </c>
       <c r="C41" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D41" s="31" t="s">
-        <v>871</v>
-      </c>
-      <c r="E41" s="27">
-        <v>1</v>
-      </c>
-      <c r="F41" s="27" t="s">
+      <c r="D41" s="29" t="s">
+        <v>870</v>
+      </c>
+      <c r="E41" s="25">
+        <v>1</v>
+      </c>
+      <c r="F41" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G41" s="32">
+      <c r="G41" s="30">
         <v>53550</v>
       </c>
-      <c r="H41" s="32">
+      <c r="H41" s="30">
         <f>G41*E41</f>
         <v>53550</v>
       </c>
-      <c r="I41" s="27" t="s">
-        <v>635</v>
+      <c r="I41" s="25" t="s">
+        <v>872</v>
       </c>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B42" s="22">
+      <c r="B42" s="21">
         <v>39</v>
       </c>
-      <c r="C42" s="34" t="s">
+      <c r="C42" s="32" t="s">
         <v>808</v>
       </c>
-      <c r="D42" s="47" t="s">
+      <c r="D42" s="45" t="s">
         <v>815</v>
       </c>
-      <c r="E42" s="48">
+      <c r="E42" s="46">
         <v>110</v>
       </c>
-      <c r="F42" s="48" t="s">
+      <c r="F42" s="46" t="s">
         <v>760</v>
       </c>
-      <c r="G42" s="49">
+      <c r="G42" s="47">
         <v>42.29</v>
       </c>
-      <c r="H42" s="49">
+      <c r="H42" s="47">
         <f>G42*E42</f>
         <v>4651.8999999999996</v>
       </c>
-      <c r="I42" s="48" t="s">
-        <v>635</v>
+      <c r="I42" s="46" t="s">
+        <v>873</v>
       </c>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B43" s="22">
+      <c r="B43" s="21">
         <v>40</v>
       </c>
-      <c r="C43" s="34"/>
-      <c r="D43" s="47" t="s">
-        <v>860</v>
-      </c>
-      <c r="E43" s="48">
-        <v>1</v>
-      </c>
-      <c r="F43" s="48" t="s">
+      <c r="C43" s="32"/>
+      <c r="D43" s="45" t="s">
+        <v>874</v>
+      </c>
+      <c r="E43" s="46">
+        <v>1</v>
+      </c>
+      <c r="F43" s="46" t="s">
         <v>760</v>
       </c>
-      <c r="G43" s="49">
+      <c r="G43" s="47">
         <v>1400</v>
       </c>
-      <c r="H43" s="49">
+      <c r="H43" s="47">
         <f>G43*E43</f>
         <v>1400</v>
       </c>
-      <c r="I43" s="48" t="s">
-        <v>635</v>
+      <c r="I43" s="46" t="s">
+        <v>873</v>
       </c>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B44" s="22">
+      <c r="B44" s="21">
         <v>41</v>
       </c>
-      <c r="C44" s="34" t="s">
+      <c r="C44" s="32" t="s">
         <v>808</v>
       </c>
-      <c r="D44" s="25" t="s">
+      <c r="D44" s="23" t="s">
         <v>757</v>
       </c>
-      <c r="E44" s="35">
+      <c r="E44" s="33">
         <f>(1784*0.15)*1.05</f>
         <v>280.97999999999996</v>
       </c>
-      <c r="F44" s="24" t="s">
+      <c r="F44" s="22" t="s">
         <v>759</v>
       </c>
-      <c r="G44" s="26">
+      <c r="G44" s="24">
         <v>670</v>
       </c>
-      <c r="H44" s="26">
+      <c r="H44" s="24">
         <f>G44*E44</f>
         <v>188256.59999999998</v>
       </c>
-      <c r="I44" s="24" t="s">
-        <v>635</v>
+      <c r="I44" s="46" t="s">
+        <v>873</v>
       </c>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B45" s="22">
+      <c r="B45" s="21">
         <v>42</v>
       </c>
-      <c r="C45" s="34" t="s">
+      <c r="C45" s="32" t="s">
         <v>808</v>
       </c>
       <c r="D45" s="18" t="s">
         <v>775</v>
       </c>
-      <c r="E45" s="35">
+      <c r="E45" s="33">
         <f>1784/13</f>
         <v>137.23076923076923</v>
       </c>
-      <c r="F45" s="24" t="s">
+      <c r="F45" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="G45" s="26">
+      <c r="G45" s="24">
         <v>220.5</v>
       </c>
-      <c r="H45" s="26">
+      <c r="H45" s="24">
         <f>G45*E45</f>
         <v>30259.384615384613</v>
       </c>
-      <c r="I45" s="24" t="s">
-        <v>635</v>
+      <c r="I45" s="46" t="s">
+        <v>873</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B46" s="22">
+      <c r="B46" s="21">
         <v>43</v>
       </c>
-      <c r="C46" s="34" t="s">
+      <c r="C46" s="32" t="s">
         <v>808</v>
       </c>
-      <c r="D46" s="25" t="s">
-        <v>870</v>
-      </c>
-      <c r="E46" s="24">
-        <v>1</v>
-      </c>
-      <c r="F46" s="24" t="s">
+      <c r="D46" s="23" t="s">
+        <v>869</v>
+      </c>
+      <c r="E46" s="22">
+        <v>1</v>
+      </c>
+      <c r="F46" s="22" t="s">
         <v>760</v>
       </c>
-      <c r="G46" s="26"/>
-      <c r="H46" s="26">
+      <c r="G46" s="24"/>
+      <c r="H46" s="24">
         <f>G46*E46</f>
         <v>0</v>
       </c>
-      <c r="I46" s="24" t="s">
-        <v>872</v>
-      </c>
-      <c r="J46" s="52" t="s">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B47" s="22">
+      <c r="I46" s="22" t="s">
+        <v>871</v>
+      </c>
+      <c r="J46" s="50" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="21">
         <v>44</v>
       </c>
       <c r="C47" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D47" s="31" t="s">
+      <c r="D47" s="29" t="s">
         <v>855</v>
       </c>
-      <c r="E47" s="27">
-        <v>1</v>
-      </c>
-      <c r="F47" s="27" t="s">
+      <c r="E47" s="25">
+        <v>1</v>
+      </c>
+      <c r="F47" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G47" s="36">
+      <c r="G47" s="34">
         <v>24500</v>
       </c>
-      <c r="H47" s="36">
+      <c r="H47" s="34">
         <f>G47*E47</f>
         <v>24500</v>
       </c>
-      <c r="I47" s="27" t="s">
+      <c r="I47" s="25" t="s">
         <v>772</v>
       </c>
     </row>
-    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B48" s="22">
+    <row r="48" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="21">
         <v>45</v>
       </c>
       <c r="C48" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D48" s="21" t="s">
+      <c r="D48" s="20" t="s">
         <v>832</v>
       </c>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
+      <c r="E48" s="21"/>
+      <c r="F48" s="21"/>
       <c r="G48" s="19"/>
       <c r="H48" s="19">
         <f>G48*E48</f>
         <v>0</v>
       </c>
-      <c r="I48" s="22" t="s">
+      <c r="I48" s="21" t="s">
         <v>772</v>
       </c>
     </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B49" s="22">
+    <row r="49" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="21">
         <v>46</v>
       </c>
       <c r="C49" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D49" s="31" t="s">
+      <c r="D49" s="29" t="s">
         <v>773</v>
       </c>
-      <c r="E49" s="27">
-        <v>1</v>
-      </c>
-      <c r="F49" s="27" t="s">
+      <c r="E49" s="25">
+        <v>1</v>
+      </c>
+      <c r="F49" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="G49" s="32">
+      <c r="G49" s="30">
         <v>968004</v>
       </c>
-      <c r="H49" s="32">
+      <c r="H49" s="30">
         <f>G49*E49</f>
         <v>968004</v>
       </c>
-      <c r="I49" s="27" t="s">
+      <c r="I49" s="25" t="s">
         <v>772</v>
       </c>
     </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B50" s="22">
+    <row r="50" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="21">
         <v>47</v>
       </c>
       <c r="C50" s="17" t="s">
         <v>808</v>
       </c>
-      <c r="D50" s="47" t="s">
+      <c r="D50" s="45" t="s">
         <v>802</v>
       </c>
-      <c r="E50" s="48">
-        <v>1</v>
-      </c>
-      <c r="F50" s="48" t="s">
+      <c r="E50" s="46">
+        <v>1</v>
+      </c>
+      <c r="F50" s="46" t="s">
         <v>760</v>
       </c>
-      <c r="G50" s="49">
+      <c r="G50" s="47">
         <v>46600</v>
       </c>
-      <c r="H50" s="49">
+      <c r="H50" s="47">
         <f>G50*E50</f>
         <v>46600</v>
       </c>
-      <c r="I50" s="48" t="s">
+      <c r="I50" s="46" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B51" s="22">
+    <row r="51" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="21">
         <v>48</v>
       </c>
       <c r="C51" s="17" t="s">
         <v>808</v>
       </c>
-      <c r="D51" s="47" t="s">
+      <c r="D51" s="45" t="s">
         <v>805</v>
       </c>
-      <c r="E51" s="48">
-        <v>1</v>
-      </c>
-      <c r="F51" s="48" t="s">
+      <c r="E51" s="46">
+        <v>1</v>
+      </c>
+      <c r="F51" s="46" t="s">
         <v>760</v>
       </c>
-      <c r="G51" s="49">
+      <c r="G51" s="47">
         <v>8100</v>
       </c>
-      <c r="H51" s="49">
+      <c r="H51" s="47">
         <f>G51*E51</f>
         <v>8100</v>
       </c>
-      <c r="I51" s="48" t="s">
+      <c r="I51" s="46" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B52" s="22">
+    <row r="52" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="21">
         <v>49</v>
       </c>
       <c r="C52" s="17" t="s">
         <v>808</v>
       </c>
-      <c r="D52" s="47" t="s">
+      <c r="D52" s="45" t="s">
         <v>817</v>
       </c>
-      <c r="E52" s="48">
-        <v>1</v>
-      </c>
-      <c r="F52" s="48" t="s">
+      <c r="E52" s="46">
+        <v>1</v>
+      </c>
+      <c r="F52" s="46" t="s">
         <v>760</v>
       </c>
-      <c r="G52" s="49">
+      <c r="G52" s="47">
         <v>5000</v>
       </c>
-      <c r="H52" s="49">
+      <c r="H52" s="47">
         <f>G52*E52</f>
         <v>5000</v>
       </c>
-      <c r="I52" s="48" t="s">
+      <c r="I52" s="46" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B53" s="22">
+    <row r="53" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="21">
         <v>50</v>
       </c>
       <c r="C53" s="17" t="s">
         <v>808</v>
       </c>
-      <c r="D53" s="47" t="s">
+      <c r="D53" s="45" t="s">
         <v>809</v>
       </c>
-      <c r="E53" s="48">
-        <v>1</v>
-      </c>
-      <c r="F53" s="48" t="s">
+      <c r="E53" s="46">
+        <v>1</v>
+      </c>
+      <c r="F53" s="46" t="s">
         <v>760</v>
       </c>
-      <c r="G53" s="49">
+      <c r="G53" s="47">
         <v>670000</v>
       </c>
-      <c r="H53" s="49">
+      <c r="H53" s="47">
         <f>G53*E53</f>
         <v>670000</v>
       </c>
-      <c r="I53" s="48" t="s">
+      <c r="I53" s="46" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B54" s="22">
+    <row r="54" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="21">
         <v>54</v>
       </c>
       <c r="C54" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D54" s="21" t="s">
+      <c r="D54" s="20" t="s">
         <v>791</v>
       </c>
-      <c r="E54" s="22"/>
-      <c r="F54" s="22"/>
+      <c r="E54" s="21"/>
+      <c r="F54" s="21"/>
       <c r="G54" s="19"/>
       <c r="H54" s="19">
         <f>G54*E54</f>
         <v>0</v>
       </c>
-      <c r="I54" s="22" t="s">
+      <c r="I54" s="21" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B55" s="22">
+    <row r="55" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="21">
         <v>55</v>
       </c>
       <c r="C55" s="17"/>
-      <c r="D55" s="21" t="s">
+      <c r="D55" s="20" t="s">
         <v>850</v>
       </c>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
+      <c r="E55" s="21"/>
+      <c r="F55" s="21"/>
       <c r="G55" s="19"/>
       <c r="H55" s="19">
         <f>G55*E55</f>
         <v>0</v>
       </c>
-      <c r="I55" s="22" t="s">
+      <c r="I55" s="21" t="s">
         <v>799</v>
       </c>
     </row>
-    <row r="56" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B56" s="22">
+    <row r="56" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="21">
         <v>56</v>
       </c>
       <c r="C56" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D56" s="21" t="s">
+      <c r="D56" s="20" t="s">
         <v>792</v>
       </c>
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
+      <c r="E56" s="21"/>
+      <c r="F56" s="21"/>
       <c r="G56" s="19"/>
       <c r="H56" s="19">
         <f>G56*E56</f>
@@ -15275,20 +15282,20 @@
         <v>799</v>
       </c>
     </row>
-    <row r="57" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B57" s="22">
+    <row r="57" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="21">
         <v>57</v>
       </c>
       <c r="C57" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D57" s="21" t="s">
+      <c r="D57" s="20" t="s">
         <v>784</v>
       </c>
-      <c r="E57" s="22">
-        <v>1</v>
-      </c>
-      <c r="F57" s="22" t="s">
+      <c r="E57" s="21">
+        <v>1</v>
+      </c>
+      <c r="F57" s="21" t="s">
         <v>760</v>
       </c>
       <c r="G57" s="19">
@@ -15298,118 +15305,118 @@
         <f>G57*E57</f>
         <v>791792.51</v>
       </c>
-      <c r="I57" s="22" t="s">
+      <c r="I57" s="21" t="s">
         <v>783</v>
       </c>
     </row>
-    <row r="58" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B58" s="22">
+    <row r="58" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="21">
         <v>51</v>
       </c>
       <c r="C58" s="17"/>
-      <c r="D58" s="25" t="s">
-        <v>864</v>
-      </c>
-      <c r="E58" s="24"/>
-      <c r="F58" s="24"/>
-      <c r="G58" s="53"/>
-      <c r="H58" s="53">
+      <c r="D58" s="23" t="s">
+        <v>863</v>
+      </c>
+      <c r="E58" s="22"/>
+      <c r="F58" s="22"/>
+      <c r="G58" s="51"/>
+      <c r="H58" s="51">
         <f>G58*E58</f>
         <v>0</v>
       </c>
-      <c r="I58" s="24"/>
-    </row>
-    <row r="59" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B59" s="22">
+      <c r="I58" s="22"/>
+    </row>
+    <row r="59" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B59" s="21">
         <v>52</v>
       </c>
       <c r="C59" s="17"/>
-      <c r="D59" s="25" t="s">
-        <v>865</v>
-      </c>
-      <c r="E59" s="24"/>
-      <c r="F59" s="24"/>
-      <c r="G59" s="53"/>
-      <c r="H59" s="53">
+      <c r="D59" s="23" t="s">
+        <v>864</v>
+      </c>
+      <c r="E59" s="22"/>
+      <c r="F59" s="22"/>
+      <c r="G59" s="51"/>
+      <c r="H59" s="51">
         <f>G59*E59</f>
         <v>0</v>
       </c>
-      <c r="I59" s="24"/>
-    </row>
-    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B60" s="22">
+      <c r="I59" s="22"/>
+    </row>
+    <row r="60" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B60" s="21">
         <v>53</v>
       </c>
       <c r="C60" s="17"/>
-      <c r="D60" s="25" t="s">
-        <v>868</v>
-      </c>
-      <c r="E60" s="24"/>
-      <c r="F60" s="24"/>
-      <c r="G60" s="53"/>
-      <c r="H60" s="53">
+      <c r="D60" s="23" t="s">
+        <v>867</v>
+      </c>
+      <c r="E60" s="22"/>
+      <c r="F60" s="22"/>
+      <c r="G60" s="51"/>
+      <c r="H60" s="51">
         <f>G60*E60</f>
         <v>0</v>
       </c>
-      <c r="I60" s="24"/>
-    </row>
-    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B61" s="22"/>
+      <c r="I60" s="22"/>
+    </row>
+    <row r="61" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="21"/>
       <c r="C61" s="17"/>
-      <c r="D61" s="21" t="s">
-        <v>869</v>
-      </c>
-      <c r="E61" s="22"/>
-      <c r="F61" s="22"/>
+      <c r="D61" s="20" t="s">
+        <v>868</v>
+      </c>
+      <c r="E61" s="21"/>
+      <c r="F61" s="21"/>
       <c r="G61" s="19"/>
       <c r="H61" s="19">
         <f>G61*E61</f>
         <v>0</v>
       </c>
-      <c r="I61" s="22"/>
-      <c r="J61" s="52" t="s">
-        <v>861</v>
-      </c>
-    </row>
-    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B62" s="22">
+      <c r="I61" s="21"/>
+      <c r="J61" s="50" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="62" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="21">
         <v>58</v>
       </c>
-      <c r="C62" s="34"/>
-      <c r="D62" s="25" t="s">
+      <c r="C62" s="32"/>
+      <c r="D62" s="23" t="s">
         <v>859</v>
       </c>
-      <c r="E62" s="24"/>
-      <c r="F62" s="24"/>
-      <c r="G62" s="26"/>
-      <c r="H62" s="51">
+      <c r="E62" s="22"/>
+      <c r="F62" s="22"/>
+      <c r="G62" s="24"/>
+      <c r="H62" s="49">
         <f>G62*E62</f>
         <v>0</v>
       </c>
-      <c r="I62" s="24"/>
+      <c r="I62" s="22"/>
     </row>
     <row r="63" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B63" s="24"/>
-      <c r="C63" s="34"/>
-      <c r="D63" s="25"/>
-      <c r="E63" s="24"/>
-      <c r="F63" s="24"/>
-      <c r="G63" s="26"/>
-      <c r="H63" s="51"/>
-      <c r="I63" s="24"/>
+      <c r="B63" s="22"/>
+      <c r="C63" s="32"/>
+      <c r="D63" s="23"/>
+      <c r="E63" s="22"/>
+      <c r="F63" s="22"/>
+      <c r="G63" s="24"/>
+      <c r="H63" s="49"/>
+      <c r="I63" s="22"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B64" s="24"/>
-      <c r="C64" s="34"/>
-      <c r="D64" s="25"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="24"/>
-      <c r="G64" s="26"/>
-      <c r="H64" s="51"/>
-      <c r="I64" s="24"/>
+      <c r="B64" s="22"/>
+      <c r="C64" s="32"/>
+      <c r="D64" s="23"/>
+      <c r="E64" s="22"/>
+      <c r="F64" s="22"/>
+      <c r="G64" s="24"/>
+      <c r="H64" s="49"/>
+      <c r="I64" s="22"/>
     </row>
     <row r="65" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D65" s="38"/>
+      <c r="D65" s="36"/>
       <c r="H65" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
         <v>4128872.0265427995</v>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 15:55
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2158" uniqueCount="875">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2157" uniqueCount="873">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2613,9 +2613,6 @@
     <t>Mão de obra para concretagem do piso das docas de carregamento DPA IV (interno)</t>
   </si>
   <si>
-    <t>Solicitar um extra ao Erisvaldo</t>
-  </si>
-  <si>
     <t>Concreto para o radier do sistema de tratamento de esgoto do banheiro</t>
   </si>
   <si>
@@ -2638,9 +2635,6 @@
   </si>
   <si>
     <t>Mão de obra para concretagem do piso do galpão 2100m² (DPA IV)</t>
-  </si>
-  <si>
-    <t>Piso pátio</t>
   </si>
   <si>
     <t>Piso Galpão</t>
@@ -2757,7 +2751,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2810,7 +2804,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2843,9 +2836,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="44" fontId="3" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2894,13 +2884,19 @@
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="18">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -3166,28 +3162,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H46" totalsRowShown="0" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H46" totalsRowShown="0" dataDxfId="10">
   <autoFilter ref="B3:H46"/>
   <sortState ref="B4:H46">
     <sortCondition ref="H3:H46"/>
   </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" name="Item" dataDxfId="2" dataCellStyle="Normal"/>
-    <tableColumn id="2" name="Descrição" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="8" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="6" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="5" dataCellStyle="Moeda">
+    <tableColumn id="1" name="Item" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="2" name="Descrição" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="9" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="8" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="7" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="6" dataCellStyle="Moeda">
       <calculatedColumnFormula>F4*D4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="5" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I62" totalsRowShown="0" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I62" totalsRowShown="0" headerRowDxfId="0" dataDxfId="17">
   <autoFilter ref="B3:I62">
     <filterColumn colId="7">
       <filters>
@@ -3200,16 +3196,16 @@
     <sortCondition ref="I3:I62"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" name="Item" dataDxfId="0" dataCellStyle="Normal"/>
-    <tableColumn id="8" name="Local" dataDxfId="1"/>
-    <tableColumn id="2" name="Descrição" dataDxfId="15" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="14" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="13" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="12" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="11" dataCellStyle="Moeda">
+    <tableColumn id="1" name="Item" dataDxfId="1" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Local" dataDxfId="2"/>
+    <tableColumn id="2" name="Descrição" dataDxfId="16" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="15" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="14" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="13" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="12" dataCellStyle="Moeda">
       <calculatedColumnFormula>G4*E4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="10" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="11" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12681,402 +12677,402 @@
       </c>
     </row>
     <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="21">
-        <v>1</v>
-      </c>
-      <c r="C4" s="29" t="s">
+      <c r="B4" s="20">
+        <v>1</v>
+      </c>
+      <c r="C4" s="28" t="s">
         <v>776</v>
       </c>
-      <c r="D4" s="25">
-        <v>1</v>
-      </c>
-      <c r="E4" s="25" t="s">
+      <c r="D4" s="24">
+        <v>1</v>
+      </c>
+      <c r="E4" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F4" s="34">
+      <c r="F4" s="32">
         <f>212518+208594</f>
         <v>421112</v>
       </c>
-      <c r="G4" s="34">
+      <c r="G4" s="32">
         <f>F4*D4</f>
         <v>421112</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="24" t="s">
         <v>782</v>
       </c>
-      <c r="J4" s="37">
+      <c r="J4" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
         <v>160740</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="21">
+      <c r="B5" s="20">
         <v>2</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="19" t="s">
         <v>854</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="20">
         <v>3</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="E5" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48">
+      <c r="F5" s="46"/>
+      <c r="G5" s="46">
         <f>F5*D5</f>
         <v>0</v>
       </c>
-      <c r="H5" s="21" t="s">
+      <c r="H5" s="20" t="s">
         <v>782</v>
       </c>
-      <c r="J5" s="37">
+      <c r="J5" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Piso",Tabela2[Preço Total])</f>
         <v>361131.5538461539</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="21">
+      <c r="B6" s="20">
         <v>3</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="19" t="s">
         <v>778</v>
       </c>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19">
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18">
         <f>F6*D6</f>
         <v>0</v>
       </c>
-      <c r="H6" s="21" t="s">
+      <c r="H6" s="20" t="s">
         <v>449</v>
       </c>
-      <c r="J6" s="37">
+      <c r="J6" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Pré Moldado",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="21">
+      <c r="B7" s="20">
         <v>4</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="19" t="s">
         <v>832</v>
       </c>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19">
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18">
         <f>F7*D7</f>
         <v>0</v>
       </c>
-      <c r="H7" s="21" t="s">
+      <c r="H7" s="20" t="s">
         <v>449</v>
       </c>
-      <c r="J7" s="37">
+      <c r="J7" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Fechamento Lateral",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="21">
+      <c r="B8" s="20">
         <v>5</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="22" t="s">
         <v>789</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="21">
         <v>10</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24">
+      <c r="F8" s="23"/>
+      <c r="G8" s="23">
         <f>F8*D8</f>
         <v>0</v>
       </c>
-      <c r="H8" s="22" t="s">
+      <c r="H8" s="21" t="s">
         <v>643</v>
       </c>
-      <c r="J8" s="37">
+      <c r="J8" s="35">
         <f>SUMIF(Tabela2[Aplicação],"AVCB",Tabela2[Preço Total])</f>
         <v>421112</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="21">
+      <c r="B9" s="20">
         <v>6</v>
       </c>
-      <c r="C9" s="45" t="s">
+      <c r="C9" s="43" t="s">
         <v>790</v>
       </c>
-      <c r="D9" s="46">
+      <c r="D9" s="44">
         <v>600</v>
       </c>
-      <c r="E9" s="46" t="s">
+      <c r="E9" s="44" t="s">
         <v>761</v>
       </c>
-      <c r="F9" s="47">
+      <c r="F9" s="45">
         <v>3.35</v>
       </c>
-      <c r="G9" s="47">
+      <c r="G9" s="45">
         <f>F9*D9</f>
         <v>2010</v>
       </c>
-      <c r="H9" s="46" t="s">
+      <c r="H9" s="44" t="s">
         <v>643</v>
       </c>
-      <c r="J9" s="37">
+      <c r="J9" s="35">
         <f>SUMIF(Tabela2[Aplicação],"SPDA",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="21">
+      <c r="B10" s="20">
         <v>7</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="28" t="s">
         <v>842</v>
       </c>
-      <c r="D10" s="25">
-        <v>1</v>
-      </c>
-      <c r="E10" s="25" t="s">
+      <c r="D10" s="24">
+        <v>1</v>
+      </c>
+      <c r="E10" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F10" s="30">
+      <c r="F10" s="29">
         <v>1056959.67</v>
       </c>
-      <c r="G10" s="30">
+      <c r="G10" s="29">
         <f>F10*D10</f>
         <v>1056959.67</v>
       </c>
-      <c r="H10" s="25" t="s">
+      <c r="H10" s="24" t="s">
         <v>841</v>
       </c>
-      <c r="J10" s="37">
+      <c r="J10" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Terraplanagem",Tabela2[Preço Total])</f>
         <v>157963.5</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B11" s="21">
+      <c r="B11" s="20">
         <v>8</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="22" t="s">
         <v>793</v>
       </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24">
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23">
         <f>F11*D11</f>
         <v>0</v>
       </c>
-      <c r="H11" s="22" t="s">
+      <c r="H11" s="21" t="s">
         <v>796</v>
       </c>
-      <c r="J11" s="37">
+      <c r="J11" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Drenagem",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="21">
+      <c r="B12" s="20">
         <v>9</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="19" t="s">
         <v>800</v>
       </c>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19">
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18">
         <f>F12*D12</f>
         <v>0</v>
       </c>
-      <c r="H12" s="21" t="s">
+      <c r="H12" s="20" t="s">
         <v>774</v>
       </c>
-      <c r="J12" s="37">
+      <c r="J12" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Elétrica",Tabela2[Preço Total])</f>
         <v>2010</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="21">
+      <c r="B13" s="20">
         <v>10</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="19" t="s">
         <v>798</v>
       </c>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19">
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18">
         <f>F13*D13</f>
         <v>0</v>
       </c>
-      <c r="H13" s="21" t="s">
+      <c r="H13" s="20" t="s">
         <v>774</v>
       </c>
-      <c r="J13" s="37">
+      <c r="J13" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Pintura",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="21">
+      <c r="B14" s="20">
         <v>11</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="C14" s="22" t="s">
         <v>779</v>
       </c>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24">
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23">
         <f>F14*D14</f>
         <v>0</v>
       </c>
-      <c r="H14" s="22" t="s">
+      <c r="H14" s="21" t="s">
         <v>774</v>
       </c>
-      <c r="J14" s="37">
+      <c r="J14" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Estrura Armazenamento",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B15" s="21">
+      <c r="B15" s="20">
         <v>12</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="22" t="s">
         <v>780</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24">
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23">
         <f>F15*D15</f>
         <v>0</v>
       </c>
-      <c r="H15" s="22" t="s">
+      <c r="H15" s="21" t="s">
         <v>774</v>
       </c>
-      <c r="J15" s="37">
+      <c r="J15" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Serviço Prévio",Tabela2[Preço Total])</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="21">
+      <c r="B16" s="20">
         <v>13</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="22" t="s">
         <v>781</v>
       </c>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24">
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23">
         <f>F16*D16</f>
         <v>0</v>
       </c>
-      <c r="H16" s="22" t="s">
+      <c r="H16" s="21" t="s">
         <v>774</v>
       </c>
-      <c r="J16" s="37"/>
+      <c r="J16" s="35"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="21">
+      <c r="B17" s="20">
         <v>14</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="22" t="s">
         <v>838</v>
       </c>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24">
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23">
         <f>F17*D17</f>
         <v>0</v>
       </c>
-      <c r="H17" s="22" t="s">
+      <c r="H17" s="21" t="s">
         <v>774</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="21">
+      <c r="B18" s="20">
         <v>15</v>
       </c>
-      <c r="C18" s="26" t="s">
+      <c r="C18" s="25" t="s">
         <v>797</v>
       </c>
-      <c r="D18" s="27">
+      <c r="D18" s="26">
         <v>4</v>
       </c>
-      <c r="E18" s="27" t="s">
+      <c r="E18" s="26" t="s">
         <v>760</v>
       </c>
-      <c r="F18" s="28">
+      <c r="F18" s="27">
         <v>1500</v>
       </c>
-      <c r="G18" s="28">
+      <c r="G18" s="27">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>6000</v>
       </c>
-      <c r="H18" s="27" t="s">
+      <c r="H18" s="26" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="21">
+      <c r="B19" s="20">
         <v>16</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="C19" s="28" t="s">
         <v>795</v>
       </c>
-      <c r="D19" s="25">
-        <v>1</v>
-      </c>
-      <c r="E19" s="25" t="s">
+      <c r="D19" s="24">
+        <v>1</v>
+      </c>
+      <c r="E19" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F19" s="30">
+      <c r="F19" s="29">
         <v>4500</v>
       </c>
-      <c r="G19" s="30">
+      <c r="G19" s="29">
         <f>F19*D19</f>
         <v>4500</v>
       </c>
-      <c r="H19" s="25" t="s">
+      <c r="H19" s="24" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="21">
+      <c r="B20" s="20">
         <v>17</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="C20" s="28" t="s">
         <v>769</v>
       </c>
-      <c r="D20" s="25">
+      <c r="D20" s="24">
         <v>2100</v>
       </c>
-      <c r="E20" s="25" t="s">
+      <c r="E20" s="24" t="s">
         <v>836</v>
       </c>
-      <c r="F20" s="30">
+      <c r="F20" s="29">
         <v>9.65</v>
       </c>
-      <c r="G20" s="30">
+      <c r="G20" s="29">
         <f>F20*D20</f>
         <v>20265</v>
       </c>
-      <c r="H20" s="25" t="s">
+      <c r="H20" s="24" t="s">
         <v>771</v>
       </c>
       <c r="I20" s="14" t="s">
@@ -13084,26 +13080,26 @@
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="21">
+      <c r="B21" s="20">
         <v>18</v>
       </c>
-      <c r="C21" s="29" t="s">
+      <c r="C21" s="28" t="s">
         <v>770</v>
       </c>
-      <c r="D21" s="25">
+      <c r="D21" s="24">
         <v>2300</v>
       </c>
-      <c r="E21" s="25" t="s">
+      <c r="E21" s="24" t="s">
         <v>836</v>
       </c>
-      <c r="F21" s="30">
+      <c r="F21" s="29">
         <v>9.65</v>
       </c>
-      <c r="G21" s="30">
+      <c r="G21" s="29">
         <f>F21*D21</f>
         <v>22195</v>
       </c>
-      <c r="H21" s="25" t="s">
+      <c r="H21" s="24" t="s">
         <v>771</v>
       </c>
       <c r="I21" s="14" t="s">
@@ -13111,578 +13107,578 @@
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="21">
+      <c r="B22" s="20">
         <v>19</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C22" s="28" t="s">
         <v>833</v>
       </c>
-      <c r="D22" s="25">
-        <v>1</v>
-      </c>
-      <c r="E22" s="25" t="s">
+      <c r="D22" s="24">
+        <v>1</v>
+      </c>
+      <c r="E22" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F22" s="30">
+      <c r="F22" s="29">
         <v>51500</v>
       </c>
-      <c r="G22" s="30">
+      <c r="G22" s="29">
         <f>F22*D22</f>
         <v>51500</v>
       </c>
-      <c r="H22" s="25" t="s">
+      <c r="H22" s="24" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="21">
+      <c r="B23" s="20">
         <v>20</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="C23" s="28" t="s">
         <v>834</v>
       </c>
-      <c r="D23" s="31">
+      <c r="D23" s="30">
         <v>46.8</v>
       </c>
-      <c r="E23" s="25" t="s">
+      <c r="E23" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="F23" s="30">
+      <c r="F23" s="29">
         <v>670</v>
       </c>
-      <c r="G23" s="30">
+      <c r="G23" s="29">
         <f>F23*D23</f>
         <v>31355.999999999996</v>
       </c>
-      <c r="H23" s="25" t="s">
+      <c r="H23" s="24" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="21">
+      <c r="B24" s="20">
         <v>21</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="28" t="s">
         <v>835</v>
       </c>
-      <c r="D24" s="31">
+      <c r="D24" s="30">
         <v>37.200000000000003</v>
       </c>
-      <c r="E24" s="25" t="s">
+      <c r="E24" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="F24" s="30">
+      <c r="F24" s="29">
         <v>670</v>
       </c>
-      <c r="G24" s="30">
+      <c r="G24" s="29">
         <f>F24*D24</f>
         <v>24924.000000000004</v>
       </c>
-      <c r="H24" s="25" t="s">
+      <c r="H24" s="24" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="21">
+      <c r="B25" s="20">
         <v>22</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="19" t="s">
         <v>777</v>
       </c>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19">
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18">
         <f>F25*D25</f>
         <v>0</v>
       </c>
-      <c r="H25" s="21" t="s">
+      <c r="H25" s="20" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="21">
+      <c r="B26" s="20">
         <v>23</v>
       </c>
-      <c r="C26" s="23" t="s">
+      <c r="C26" s="22" t="s">
         <v>785</v>
       </c>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24">
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23">
         <f>F26*D26</f>
         <v>0</v>
       </c>
-      <c r="H26" s="22" t="s">
+      <c r="H26" s="21" t="s">
         <v>576</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B27" s="21">
+      <c r="B27" s="20">
         <v>24</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="C27" s="22" t="s">
         <v>786</v>
       </c>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24">
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23">
         <f>F27*D27</f>
         <v>0</v>
       </c>
-      <c r="H27" s="22" t="s">
+      <c r="H27" s="21" t="s">
         <v>576</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B28" s="21">
+      <c r="B28" s="20">
         <v>25</v>
       </c>
-      <c r="C28" s="23" t="s">
+      <c r="C28" s="22" t="s">
         <v>787</v>
       </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24">
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23">
         <f>F28*D28</f>
         <v>0</v>
       </c>
-      <c r="H28" s="22" t="s">
+      <c r="H28" s="21" t="s">
         <v>576</v>
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B29" s="21">
+      <c r="B29" s="20">
         <v>26</v>
       </c>
-      <c r="C29" s="23" t="s">
+      <c r="C29" s="22" t="s">
         <v>788</v>
       </c>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24">
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23">
         <f>F29*D29</f>
         <v>0</v>
       </c>
-      <c r="H29" s="22" t="s">
+      <c r="H29" s="21" t="s">
         <v>576</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B30" s="21">
+      <c r="B30" s="20">
         <v>27</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="C30" s="28" t="s">
         <v>757</v>
       </c>
-      <c r="D30" s="25">
+      <c r="D30" s="24">
         <f>(2000*1.05)*0.15</f>
         <v>315</v>
       </c>
-      <c r="E30" s="25" t="s">
+      <c r="E30" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="F30" s="30">
+      <c r="F30" s="29">
         <v>670</v>
       </c>
-      <c r="G30" s="30">
+      <c r="G30" s="29">
         <f>F30*D30</f>
         <v>211050</v>
       </c>
-      <c r="H30" s="25" t="s">
+      <c r="H30" s="24" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B31" s="21">
+      <c r="B31" s="20">
         <v>28</v>
       </c>
-      <c r="C31" s="29" t="s">
+      <c r="C31" s="28" t="s">
         <v>775</v>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="30">
         <f>2000/13*2</f>
         <v>307.69230769230768</v>
       </c>
-      <c r="E31" s="25" t="s">
+      <c r="E31" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F31" s="30">
+      <c r="F31" s="29">
         <v>220.5</v>
       </c>
-      <c r="G31" s="30">
+      <c r="G31" s="29">
         <f>F31*D31</f>
         <v>67846.153846153844</v>
       </c>
-      <c r="H31" s="25" t="s">
+      <c r="H31" s="24" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B32" s="21">
+      <c r="B32" s="20">
         <v>29</v>
       </c>
-      <c r="C32" s="29" t="s">
+      <c r="C32" s="28" t="s">
         <v>758</v>
       </c>
-      <c r="D32" s="25">
+      <c r="D32" s="24">
         <v>167</v>
       </c>
-      <c r="E32" s="25" t="s">
+      <c r="E32" s="24" t="s">
         <v>810</v>
       </c>
-      <c r="F32" s="30">
+      <c r="F32" s="29">
         <v>56.2</v>
       </c>
-      <c r="G32" s="30">
+      <c r="G32" s="29">
         <f>F32*D32</f>
         <v>9385.4</v>
       </c>
-      <c r="H32" s="25" t="s">
+      <c r="H32" s="24" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B33" s="21">
+      <c r="B33" s="20">
         <v>30</v>
       </c>
-      <c r="C33" s="29" t="s">
+      <c r="C33" s="28" t="s">
         <v>762</v>
       </c>
-      <c r="D33" s="25">
+      <c r="D33" s="24">
         <v>1000</v>
       </c>
-      <c r="E33" s="25" t="s">
+      <c r="E33" s="24" t="s">
         <v>763</v>
       </c>
-      <c r="F33" s="30">
+      <c r="F33" s="29">
         <v>7.3</v>
       </c>
-      <c r="G33" s="30">
+      <c r="G33" s="29">
         <f>F33*D33</f>
         <v>7300</v>
       </c>
-      <c r="H33" s="25" t="s">
+      <c r="H33" s="24" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="21">
+      <c r="B34" s="20">
         <v>31</v>
       </c>
-      <c r="C34" s="29" t="s">
+      <c r="C34" s="28" t="s">
         <v>801</v>
       </c>
-      <c r="D34" s="25">
+      <c r="D34" s="24">
         <v>315</v>
       </c>
-      <c r="E34" s="25" t="s">
+      <c r="E34" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="F34" s="30">
+      <c r="F34" s="29">
         <v>50</v>
       </c>
-      <c r="G34" s="30">
+      <c r="G34" s="29">
         <f>F34*D34</f>
         <v>15750</v>
       </c>
-      <c r="H34" s="25" t="s">
+      <c r="H34" s="24" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="21">
+      <c r="B35" s="20">
         <v>32</v>
       </c>
-      <c r="C35" s="29" t="s">
+      <c r="C35" s="28" t="s">
         <v>768</v>
       </c>
-      <c r="D35" s="25">
-        <v>1</v>
-      </c>
-      <c r="E35" s="25" t="s">
+      <c r="D35" s="24">
+        <v>1</v>
+      </c>
+      <c r="E35" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F35" s="30">
+      <c r="F35" s="29">
         <v>49800</v>
       </c>
-      <c r="G35" s="30">
+      <c r="G35" s="29">
         <f>F35*D35</f>
         <v>49800</v>
       </c>
-      <c r="H35" s="25" t="s">
+      <c r="H35" s="24" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B36" s="21">
+      <c r="B36" s="20">
         <v>33</v>
       </c>
-      <c r="C36" s="23" t="s">
+      <c r="C36" s="22" t="s">
         <v>803</v>
       </c>
-      <c r="D36" s="22">
-        <v>1</v>
-      </c>
-      <c r="E36" s="22" t="s">
+      <c r="D36" s="21">
+        <v>1</v>
+      </c>
+      <c r="E36" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="F36" s="24"/>
-      <c r="G36" s="24">
+      <c r="F36" s="23"/>
+      <c r="G36" s="23">
         <f>F36*D36</f>
         <v>0</v>
       </c>
-      <c r="H36" s="22" t="s">
+      <c r="H36" s="21" t="s">
         <v>804</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B37" s="21">
+      <c r="B37" s="20">
         <v>34</v>
       </c>
-      <c r="C37" s="23" t="s">
+      <c r="C37" s="22" t="s">
         <v>814</v>
       </c>
-      <c r="D37" s="22">
-        <v>1</v>
-      </c>
-      <c r="E37" s="22" t="s">
+      <c r="D37" s="21">
+        <v>1</v>
+      </c>
+      <c r="E37" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="F37" s="24"/>
-      <c r="G37" s="24">
+      <c r="F37" s="23"/>
+      <c r="G37" s="23">
         <f>F37*D37</f>
         <v>0</v>
       </c>
-      <c r="H37" s="22" t="s">
+      <c r="H37" s="21" t="s">
         <v>804</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B38" s="21">
+      <c r="B38" s="20">
         <v>35</v>
       </c>
-      <c r="C38" s="20" t="s">
+      <c r="C38" s="19" t="s">
         <v>791</v>
       </c>
-      <c r="D38" s="21"/>
-      <c r="E38" s="21"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19">
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18">
         <f>F38*D38</f>
         <v>0</v>
       </c>
-      <c r="H38" s="21" t="s">
+      <c r="H38" s="20" t="s">
         <v>419</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B39" s="21">
+      <c r="B39" s="20">
         <v>36</v>
       </c>
-      <c r="C39" s="44" t="s">
+      <c r="C39" s="42" t="s">
         <v>843</v>
       </c>
-      <c r="D39" s="25">
+      <c r="D39" s="24">
         <v>1455.89</v>
       </c>
-      <c r="E39" s="25" t="s">
+      <c r="E39" s="24" t="s">
         <v>761</v>
       </c>
-      <c r="F39" s="34">
+      <c r="F39" s="32">
         <v>95.9</v>
       </c>
-      <c r="G39" s="34">
+      <c r="G39" s="32">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>139619.85100000002</v>
       </c>
-      <c r="H39" s="25" t="s">
+      <c r="H39" s="24" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B40" s="21">
+      <c r="B40" s="20">
         <v>37</v>
       </c>
-      <c r="C40" s="29" t="s">
+      <c r="C40" s="28" t="s">
         <v>844</v>
       </c>
-      <c r="D40" s="25">
+      <c r="D40" s="24">
         <v>706.94</v>
       </c>
-      <c r="E40" s="25" t="s">
+      <c r="E40" s="24" t="s">
         <v>761</v>
       </c>
-      <c r="F40" s="34">
+      <c r="F40" s="32">
         <v>95.9</v>
       </c>
-      <c r="G40" s="34">
+      <c r="G40" s="32">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>67795.546000000002</v>
       </c>
-      <c r="H40" s="25" t="s">
+      <c r="H40" s="24" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B41" s="21">
+      <c r="B41" s="20">
         <v>38</v>
       </c>
-      <c r="C41" s="26" t="s">
+      <c r="C41" s="25" t="s">
         <v>845</v>
       </c>
-      <c r="D41" s="25">
+      <c r="D41" s="24">
         <v>44</v>
       </c>
-      <c r="E41" s="25" t="s">
+      <c r="E41" s="24" t="s">
         <v>849</v>
       </c>
-      <c r="F41" s="34">
+      <c r="F41" s="32">
         <v>95</v>
       </c>
-      <c r="G41" s="34">
+      <c r="G41" s="32">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>4180</v>
       </c>
-      <c r="H41" s="25" t="s">
+      <c r="H41" s="24" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B42" s="21">
+      <c r="B42" s="20">
         <v>39</v>
       </c>
-      <c r="C42" s="26" t="s">
+      <c r="C42" s="25" t="s">
         <v>846</v>
       </c>
-      <c r="D42" s="25">
+      <c r="D42" s="24">
         <v>3</v>
       </c>
-      <c r="E42" s="25" t="s">
+      <c r="E42" s="24" t="s">
         <v>849</v>
       </c>
-      <c r="F42" s="34">
+      <c r="F42" s="32">
         <v>35</v>
       </c>
-      <c r="G42" s="34">
+      <c r="G42" s="32">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>105</v>
       </c>
-      <c r="H42" s="25" t="s">
+      <c r="H42" s="24" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B43" s="21">
+      <c r="B43" s="20">
         <v>40</v>
       </c>
-      <c r="C43" s="26" t="s">
+      <c r="C43" s="25" t="s">
         <v>847</v>
       </c>
-      <c r="D43" s="25">
+      <c r="D43" s="24">
         <v>126</v>
       </c>
-      <c r="E43" s="25" t="s">
+      <c r="E43" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F43" s="34">
+      <c r="F43" s="32">
         <v>25.9</v>
       </c>
-      <c r="G43" s="34">
+      <c r="G43" s="32">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
         <v>3263.3999999999996</v>
       </c>
-      <c r="H43" s="25" t="s">
+      <c r="H43" s="24" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B44" s="21">
+      <c r="B44" s="20">
         <v>41</v>
       </c>
-      <c r="C44" s="26" t="s">
+      <c r="C44" s="25" t="s">
         <v>848</v>
       </c>
-      <c r="D44" s="25">
-        <v>1</v>
-      </c>
-      <c r="E44" s="25" t="s">
+      <c r="D44" s="24">
+        <v>1</v>
+      </c>
+      <c r="E44" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F44" s="34">
+      <c r="F44" s="32">
         <v>1750</v>
       </c>
-      <c r="G44" s="34">
+      <c r="G44" s="32">
         <f>F44*D44</f>
         <v>1750</v>
       </c>
-      <c r="H44" s="25" t="s">
+      <c r="H44" s="24" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B45" s="21">
+      <c r="B45" s="20">
         <v>42</v>
       </c>
-      <c r="C45" s="29" t="s">
+      <c r="C45" s="28" t="s">
         <v>784</v>
       </c>
-      <c r="D45" s="25">
-        <v>1</v>
-      </c>
-      <c r="E45" s="25" t="s">
+      <c r="D45" s="24">
+        <v>1</v>
+      </c>
+      <c r="E45" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="F45" s="34">
+      <c r="F45" s="32">
         <v>157963.5</v>
       </c>
-      <c r="G45" s="34">
+      <c r="G45" s="32">
         <f>F45*D45</f>
         <v>157963.5</v>
       </c>
-      <c r="H45" s="25" t="s">
+      <c r="H45" s="24" t="s">
         <v>783</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B46" s="21">
+      <c r="B46" s="20">
         <v>43</v>
       </c>
-      <c r="C46" s="23" t="s">
+      <c r="C46" s="22" t="s">
         <v>839</v>
       </c>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="24"/>
-      <c r="G46" s="24">
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="23"/>
+      <c r="G46" s="23">
         <f>F46*D46</f>
         <v>0</v>
       </c>
-      <c r="H46" s="22" t="s">
+      <c r="H46" s="21" t="s">
         <v>840</v>
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B47" s="22"/>
-      <c r="C47" s="23"/>
-      <c r="D47" s="22"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="24"/>
-      <c r="G47" s="24"/>
-      <c r="H47" s="22"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="23"/>
+      <c r="H47" s="21"/>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B48" s="22"/>
-      <c r="C48" s="23"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="24"/>
-      <c r="G48" s="24"/>
-      <c r="H48" s="22"/>
+      <c r="B48" s="21"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="21"/>
+      <c r="E48" s="21"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="23"/>
+      <c r="H48" s="21"/>
     </row>
     <row r="49" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G49" s="16">
@@ -13712,7 +13708,7 @@
     <col min="7" max="7" width="15.85546875" style="15" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" style="15" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.85546875" style="14" customWidth="1"/>
-    <col min="10" max="10" width="64.7109375" style="50" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="64.7109375" style="48" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="16" style="14" customWidth="1"/>
     <col min="14" max="14" width="18.42578125" customWidth="1"/>
     <col min="15" max="15" width="25" customWidth="1"/>
@@ -13738,7 +13734,7 @@
       <c r="C3" s="14" t="s">
         <v>806</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="14" t="s">
         <v>754</v>
       </c>
       <c r="E3" s="14" t="s">
@@ -13753,36 +13749,35 @@
       <c r="H3" s="14" t="s">
         <v>765</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="14" t="s">
         <v>767</v>
       </c>
-      <c r="J3" s="50"/>
       <c r="P3" s="14" t="s">
         <v>826</v>
       </c>
     </row>
     <row r="4" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="21">
+      <c r="B4" s="20">
         <v>1</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="22" t="s">
         <v>793</v>
       </c>
-      <c r="E4" s="22">
-        <v>1</v>
-      </c>
-      <c r="F4" s="22" t="s">
+      <c r="E4" s="21">
+        <v>1</v>
+      </c>
+      <c r="F4" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24">
+      <c r="G4" s="23"/>
+      <c r="H4" s="23">
         <f>G4*E4</f>
         <v>0</v>
       </c>
-      <c r="I4" s="22" t="s">
+      <c r="I4" s="21" t="s">
         <v>813</v>
       </c>
       <c r="O4" s="14" t="s">
@@ -13799,43 +13794,43 @@
       </c>
     </row>
     <row r="5" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="21">
+      <c r="B5" s="20">
         <v>2</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="28" t="s">
         <v>851</v>
       </c>
-      <c r="E5" s="25">
-        <v>1</v>
-      </c>
-      <c r="F5" s="25" t="s">
+      <c r="E5" s="24">
+        <v>1</v>
+      </c>
+      <c r="F5" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G5" s="34">
+      <c r="G5" s="32">
         <v>486032</v>
       </c>
-      <c r="H5" s="34">
+      <c r="H5" s="32">
         <f>G5*E5</f>
         <v>486032</v>
       </c>
-      <c r="I5" s="25" t="s">
+      <c r="I5" s="24" t="s">
         <v>782</v>
       </c>
-      <c r="N5" s="35" t="s">
+      <c r="N5" s="33" t="s">
         <v>772</v>
       </c>
-      <c r="O5" s="37">
+      <c r="O5" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Pré Moldado",Tabela24[Preço Total])</f>
         <v>992504</v>
       </c>
-      <c r="P5" s="41">
+      <c r="P5" s="39">
         <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
         <v>0.27943619534004144</v>
       </c>
-      <c r="Q5" s="43">
+      <c r="Q5" s="41">
         <f>P5</f>
         <v>0.27943619534004144</v>
       </c>
@@ -13844,39 +13839,39 @@
       </c>
     </row>
     <row r="6" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="21">
+      <c r="B6" s="20">
         <v>3</v>
       </c>
       <c r="C6" s="17"/>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="19" t="s">
         <v>853</v>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="20">
         <v>4</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19">
+      <c r="G6" s="18"/>
+      <c r="H6" s="18">
         <f>G6*E6</f>
         <v>0</v>
       </c>
       <c r="I6" s="17" t="s">
         <v>782</v>
       </c>
-      <c r="N6" s="42" t="s">
+      <c r="N6" s="40" t="s">
         <v>783</v>
       </c>
-      <c r="O6" s="37">
+      <c r="O6" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Terraplanagem",Tabela24[Preço Total])</f>
         <v>791792.51</v>
       </c>
-      <c r="P6" s="41">
+      <c r="P6" s="39">
         <f t="shared" si="0"/>
         <v>0.22292654386596095</v>
       </c>
-      <c r="Q6" s="43">
+      <c r="Q6" s="41">
         <f>P6+Q5</f>
         <v>0.50236273920600238</v>
       </c>
@@ -13885,640 +13880,640 @@
       </c>
     </row>
     <row r="7" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="21">
+      <c r="B7" s="20">
         <v>4</v>
       </c>
       <c r="C7" s="17"/>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="19" t="s">
         <v>852</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="20">
         <v>6</v>
       </c>
-      <c r="F7" s="21" t="s">
+      <c r="F7" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19">
+      <c r="G7" s="18"/>
+      <c r="H7" s="18">
         <f>G7*E7</f>
         <v>0</v>
       </c>
       <c r="I7" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="N7" s="35" t="s">
+      <c r="N7" s="33" t="s">
         <v>635</v>
       </c>
-      <c r="O7" s="37">
+      <c r="O7" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Piso",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
-      <c r="P7" s="41">
+      <c r="P7" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="21">
+      <c r="B8" s="20">
         <v>5</v>
       </c>
-      <c r="C8" s="32"/>
-      <c r="D8" s="23" t="s">
+      <c r="C8" s="31"/>
+      <c r="D8" s="22" t="s">
         <v>858</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="21">
         <v>6</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="G8" s="24"/>
-      <c r="H8" s="49">
+      <c r="G8" s="23"/>
+      <c r="H8" s="47">
         <f>G8*E8</f>
         <v>0</v>
       </c>
       <c r="I8" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="N8" s="42" t="s">
+      <c r="N8" s="40" t="s">
         <v>804</v>
       </c>
-      <c r="O8" s="37">
+      <c r="O8" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
         <v>729700</v>
       </c>
-      <c r="P8" s="41">
+      <c r="P8" s="39">
         <f t="shared" si="0"/>
         <v>0.20544460449492216</v>
       </c>
     </row>
     <row r="9" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="21">
+      <c r="B9" s="20">
         <v>6</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="23" t="s">
+      <c r="C9" s="31"/>
+      <c r="D9" s="22" t="s">
         <v>861</v>
       </c>
-      <c r="E9" s="22">
-        <v>1</v>
-      </c>
-      <c r="F9" s="22" t="s">
+      <c r="E9" s="21">
+        <v>1</v>
+      </c>
+      <c r="F9" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="G9" s="24"/>
-      <c r="H9" s="49">
+      <c r="G9" s="23"/>
+      <c r="H9" s="47">
         <f>G9*E9</f>
         <v>0</v>
       </c>
       <c r="I9" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="N9" s="39" t="s">
+      <c r="N9" s="37" t="s">
         <v>771</v>
       </c>
-      <c r="O9" s="37">
+      <c r="O9" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Fundação",Tabela24[Preço Total])</f>
         <v>416702.4</v>
       </c>
-      <c r="P9" s="41">
+      <c r="P9" s="39">
         <f t="shared" si="0"/>
         <v>0.11732117275604338</v>
       </c>
     </row>
     <row r="10" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="21">
+      <c r="B10" s="20">
         <v>7</v>
       </c>
       <c r="C10" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="22" t="s">
         <v>789</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="21">
         <v>26</v>
       </c>
-      <c r="F10" s="22" t="s">
+      <c r="F10" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24">
+      <c r="G10" s="23"/>
+      <c r="H10" s="23">
         <f>G10*E10</f>
         <v>0</v>
       </c>
-      <c r="I10" s="22" t="s">
+      <c r="I10" s="21" t="s">
         <v>643</v>
       </c>
-      <c r="N10" s="39" t="s">
+      <c r="N10" s="37" t="s">
         <v>774</v>
       </c>
-      <c r="O10" s="37">
+      <c r="O10" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
         <v>66534.056568800006</v>
       </c>
-      <c r="P10" s="41">
+      <c r="P10" s="39">
         <f t="shared" si="0"/>
         <v>1.8732442013457442E-2</v>
       </c>
     </row>
     <row r="11" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="21">
+      <c r="B11" s="20">
         <v>8</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D11" s="45" t="s">
+      <c r="D11" s="43" t="s">
         <v>790</v>
       </c>
-      <c r="E11" s="46">
+      <c r="E11" s="44">
         <v>600</v>
       </c>
-      <c r="F11" s="46" t="s">
+      <c r="F11" s="44" t="s">
         <v>761</v>
       </c>
-      <c r="G11" s="47">
+      <c r="G11" s="45">
         <v>3.35</v>
       </c>
-      <c r="H11" s="47">
+      <c r="H11" s="45">
         <f>G11*E11</f>
         <v>2010</v>
       </c>
-      <c r="I11" s="46" t="s">
+      <c r="I11" s="44" t="s">
         <v>643</v>
       </c>
-      <c r="N11" s="38" t="s">
+      <c r="N11" s="36" t="s">
         <v>782</v>
       </c>
-      <c r="O11" s="37">
+      <c r="O11" s="35">
         <f>SUMIF(Tabela24[Aplicação],"AVCB",Tabela24[Preço Total])</f>
         <v>486032</v>
       </c>
-      <c r="P11" s="41">
+      <c r="P11" s="39">
         <f t="shared" si="0"/>
         <v>0.13684069071108126</v>
       </c>
     </row>
     <row r="12" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="21">
+      <c r="B12" s="20">
         <v>9</v>
       </c>
       <c r="C12" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="22" t="s">
         <v>812</v>
       </c>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24">
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23">
         <f>G12*E12</f>
         <v>0</v>
       </c>
-      <c r="I12" s="22" t="s">
+      <c r="I12" s="21" t="s">
         <v>643</v>
       </c>
-      <c r="N12" s="38" t="s">
+      <c r="N12" s="36" t="s">
         <v>449</v>
       </c>
-      <c r="O12" s="37">
+      <c r="O12" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Drenagem",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
-      <c r="P12" s="41">
+      <c r="P12" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="21">
+      <c r="B13" s="20">
         <v>10</v>
       </c>
       <c r="C13" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D13" s="29" t="s">
+      <c r="D13" s="28" t="s">
         <v>829</v>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="24">
         <v>54</v>
       </c>
-      <c r="F13" s="25" t="s">
+      <c r="F13" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G13" s="34">
+      <c r="G13" s="32">
         <v>243.39</v>
       </c>
-      <c r="H13" s="34">
+      <c r="H13" s="32">
         <f>G13*E13</f>
         <v>13143.06</v>
       </c>
-      <c r="I13" s="25" t="s">
+      <c r="I13" s="24" t="s">
         <v>830</v>
       </c>
-      <c r="N13" s="38"/>
-      <c r="O13" s="37"/>
-      <c r="P13" s="41"/>
+      <c r="N13" s="36"/>
+      <c r="O13" s="35"/>
+      <c r="P13" s="39"/>
     </row>
     <row r="14" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="21">
+      <c r="B14" s="20">
         <v>11</v>
       </c>
       <c r="C14" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D14" s="29" t="s">
+      <c r="D14" s="28" t="s">
         <v>831</v>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="24">
         <v>30</v>
       </c>
-      <c r="F14" s="25" t="s">
+      <c r="F14" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G14" s="34">
+      <c r="G14" s="32">
         <v>119.7</v>
       </c>
-      <c r="H14" s="34">
+      <c r="H14" s="32">
         <f>G14*E14</f>
         <v>3591</v>
       </c>
-      <c r="I14" s="25" t="s">
+      <c r="I14" s="24" t="s">
         <v>830</v>
       </c>
-      <c r="N14" s="38" t="s">
+      <c r="N14" s="36" t="s">
         <v>774</v>
       </c>
-      <c r="O14" s="37">
+      <c r="O14" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Fechamento Lateral",Tabela24[Preço Total])</f>
         <v>66534.056568800006</v>
       </c>
-      <c r="P14" s="41">
+      <c r="P14" s="39">
         <f t="shared" si="0"/>
         <v>1.8732442013457442E-2</v>
       </c>
     </row>
     <row r="15" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="21">
+      <c r="B15" s="20">
         <v>12</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D15" s="29" t="s">
+      <c r="D15" s="28" t="s">
         <v>828</v>
       </c>
-      <c r="E15" s="46">
+      <c r="E15" s="44">
         <v>390</v>
       </c>
-      <c r="F15" s="25" t="s">
+      <c r="F15" s="24" t="s">
         <v>761</v>
       </c>
-      <c r="G15" s="34">
+      <c r="G15" s="32">
         <v>38.116666600000002</v>
       </c>
-      <c r="H15" s="34">
+      <c r="H15" s="32">
         <f>G15*E15</f>
         <v>14865.499974</v>
       </c>
-      <c r="I15" s="25" t="s">
+      <c r="I15" s="24" t="s">
         <v>830</v>
       </c>
-      <c r="N15" s="38" t="s">
+      <c r="N15" s="36" t="s">
         <v>643</v>
       </c>
-      <c r="O15" s="37">
+      <c r="O15" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Elétrica",Tabela24[Preço Total])</f>
         <v>2010</v>
       </c>
-      <c r="P15" s="41">
+      <c r="P15" s="39">
         <f t="shared" si="0"/>
         <v>5.6590880503603334E-4</v>
       </c>
     </row>
     <row r="16" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="21">
+      <c r="B16" s="20">
         <v>13</v>
       </c>
       <c r="C16" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D16" s="29" t="s">
+      <c r="D16" s="28" t="s">
         <v>829</v>
       </c>
-      <c r="E16" s="31">
+      <c r="E16" s="30">
         <f>(84*1.02)*2*1.02</f>
         <v>174.78720000000001</v>
       </c>
-      <c r="F16" s="25" t="s">
+      <c r="F16" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G16" s="34">
+      <c r="G16" s="32">
         <v>243.39</v>
       </c>
-      <c r="H16" s="34">
+      <c r="H16" s="32">
         <f>G16*E16</f>
         <v>42541.456608</v>
       </c>
-      <c r="I16" s="25" t="s">
+      <c r="I16" s="24" t="s">
         <v>774</v>
       </c>
-      <c r="N16" s="38"/>
-      <c r="O16" s="37"/>
-      <c r="P16" s="41"/>
+      <c r="N16" s="36"/>
+      <c r="O16" s="35"/>
+      <c r="P16" s="39"/>
     </row>
     <row r="17" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="21">
+      <c r="B17" s="20">
         <v>14</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D17" s="29" t="s">
+      <c r="D17" s="28" t="s">
         <v>828</v>
       </c>
-      <c r="E17" s="25">
+      <c r="E17" s="24">
         <f>84*7</f>
         <v>588</v>
       </c>
-      <c r="F17" s="25" t="s">
+      <c r="F17" s="24" t="s">
         <v>761</v>
       </c>
-      <c r="G17" s="34">
+      <c r="G17" s="32">
         <v>38.116666600000002</v>
       </c>
-      <c r="H17" s="34">
+      <c r="H17" s="32">
         <f>G17*E17</f>
         <v>22412.599960800002</v>
       </c>
-      <c r="I17" s="25" t="s">
+      <c r="I17" s="24" t="s">
         <v>774</v>
       </c>
-      <c r="N17" s="38"/>
-      <c r="O17" s="37"/>
-      <c r="P17" s="41"/>
+      <c r="N17" s="36"/>
+      <c r="O17" s="35"/>
+      <c r="P17" s="39"/>
     </row>
     <row r="18" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="21">
+      <c r="B18" s="20">
         <v>15</v>
       </c>
-      <c r="C18" s="25"/>
-      <c r="D18" s="29" t="s">
+      <c r="C18" s="24"/>
+      <c r="D18" s="28" t="s">
         <v>856</v>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="24">
         <v>30</v>
       </c>
-      <c r="F18" s="25" t="s">
+      <c r="F18" s="24" t="s">
         <v>849</v>
       </c>
-      <c r="G18" s="34">
+      <c r="G18" s="32">
         <v>24</v>
       </c>
-      <c r="H18" s="34">
+      <c r="H18" s="32">
         <f>G18*E18</f>
         <v>720</v>
       </c>
-      <c r="I18" s="25" t="s">
+      <c r="I18" s="24" t="s">
         <v>774</v>
       </c>
-      <c r="N18" s="38"/>
-      <c r="O18" s="37"/>
-      <c r="P18" s="41"/>
+      <c r="N18" s="36"/>
+      <c r="O18" s="35"/>
+      <c r="P18" s="39"/>
     </row>
     <row r="19" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="21">
+      <c r="B19" s="20">
         <v>16</v>
       </c>
-      <c r="C19" s="25"/>
-      <c r="D19" s="29" t="s">
+      <c r="C19" s="24"/>
+      <c r="D19" s="28" t="s">
         <v>857</v>
       </c>
-      <c r="E19" s="25">
-        <v>1</v>
-      </c>
-      <c r="F19" s="25" t="s">
+      <c r="E19" s="24">
+        <v>1</v>
+      </c>
+      <c r="F19" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G19" s="34">
+      <c r="G19" s="32">
         <v>860</v>
       </c>
-      <c r="H19" s="34">
+      <c r="H19" s="32">
         <f>G19*E19</f>
         <v>860</v>
       </c>
-      <c r="I19" s="25" t="s">
+      <c r="I19" s="24" t="s">
         <v>774</v>
       </c>
-      <c r="N19" s="38" t="s">
+      <c r="N19" s="36" t="s">
         <v>576</v>
       </c>
-      <c r="O19" s="37">
+      <c r="O19" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Pintura",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
-      <c r="P19" s="41">
+      <c r="P19" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="21">
+      <c r="B20" s="20">
         <v>17</v>
       </c>
       <c r="C20" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D20" s="23" t="s">
+      <c r="D20" s="22" t="s">
         <v>779</v>
       </c>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22" t="s">
+      <c r="E20" s="21"/>
+      <c r="F20" s="21" t="s">
         <v>761</v>
       </c>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24">
+      <c r="G20" s="23"/>
+      <c r="H20" s="23">
         <f>G20*E20</f>
         <v>0</v>
       </c>
-      <c r="I20" s="22" t="s">
+      <c r="I20" s="21" t="s">
         <v>774</v>
       </c>
-      <c r="N20" s="38" t="s">
+      <c r="N20" s="36" t="s">
         <v>813</v>
       </c>
-      <c r="O20" s="37">
+      <c r="O20" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
         <v>0</v>
       </c>
-      <c r="P20" s="41">
+      <c r="P20" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="21">
+      <c r="B21" s="20">
         <v>18</v>
       </c>
       <c r="C21" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="D21" s="22" t="s">
         <v>780</v>
       </c>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24">
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23">
         <f>G21*E21</f>
         <v>0</v>
       </c>
-      <c r="I21" s="22" t="s">
+      <c r="I21" s="21" t="s">
         <v>774</v>
       </c>
-      <c r="N21" s="38"/>
-      <c r="O21" s="37"/>
-      <c r="P21" s="41"/>
+      <c r="N21" s="36"/>
+      <c r="O21" s="35"/>
+      <c r="P21" s="39"/>
     </row>
     <row r="22" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="21">
+      <c r="B22" s="20">
         <v>19</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D22" s="23" t="s">
+      <c r="D22" s="22" t="s">
         <v>781</v>
       </c>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24">
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23">
         <f>G22*E22</f>
         <v>0</v>
       </c>
-      <c r="I22" s="22" t="s">
+      <c r="I22" s="21" t="s">
         <v>774</v>
       </c>
-      <c r="N22" s="38"/>
-      <c r="O22" s="37"/>
-      <c r="P22" s="41"/>
+      <c r="N22" s="36"/>
+      <c r="O22" s="35"/>
+      <c r="P22" s="39"/>
     </row>
     <row r="23" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="21">
+      <c r="B23" s="20">
         <v>20</v>
       </c>
       <c r="C23" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D23" s="23" t="s">
+      <c r="D23" s="22" t="s">
         <v>816</v>
       </c>
-      <c r="E23" s="22">
-        <v>1</v>
-      </c>
-      <c r="F23" s="22"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24">
+      <c r="E23" s="21">
+        <v>1</v>
+      </c>
+      <c r="F23" s="21"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23">
         <f>G23*E23</f>
         <v>0</v>
       </c>
-      <c r="I23" s="22" t="s">
+      <c r="I23" s="21" t="s">
         <v>774</v>
       </c>
     </row>
     <row r="24" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="21">
+      <c r="B24" s="20">
         <v>21</v>
       </c>
       <c r="C24" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D24" s="29" t="s">
+      <c r="D24" s="28" t="s">
         <v>794</v>
       </c>
-      <c r="E24" s="25">
-        <v>1</v>
-      </c>
-      <c r="F24" s="25" t="s">
+      <c r="E24" s="24">
+        <v>1</v>
+      </c>
+      <c r="F24" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G24" s="30">
+      <c r="G24" s="29">
         <v>6000</v>
       </c>
-      <c r="H24" s="30">
+      <c r="H24" s="29">
         <f>G24*E24</f>
         <v>6000</v>
       </c>
-      <c r="I24" s="25" t="s">
+      <c r="I24" s="24" t="s">
         <v>771</v>
       </c>
-      <c r="N24" s="38" t="s">
+      <c r="N24" s="36" t="s">
         <v>819</v>
       </c>
-      <c r="O24" s="40">
+      <c r="O24" s="38">
         <f>SUM(O5:O20)</f>
         <v>3551809.0231375997</v>
       </c>
     </row>
     <row r="25" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="21">
+      <c r="B25" s="20">
         <v>22</v>
       </c>
       <c r="C25" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D25" s="29" t="s">
+      <c r="D25" s="28" t="s">
         <v>769</v>
       </c>
-      <c r="E25" s="25">
+      <c r="E25" s="24">
         <v>4100</v>
       </c>
-      <c r="F25" s="25" t="s">
+      <c r="F25" s="24" t="s">
         <v>836</v>
       </c>
-      <c r="G25" s="30">
+      <c r="G25" s="29">
         <v>9.65</v>
       </c>
-      <c r="H25" s="30">
+      <c r="H25" s="29">
         <f>G25*E25</f>
         <v>39565</v>
       </c>
-      <c r="I25" s="25" t="s">
+      <c r="I25" s="24" t="s">
         <v>771</v>
       </c>
       <c r="J25" s="14" t="s">
         <v>837</v>
       </c>
-      <c r="N25" s="38"/>
-      <c r="O25" s="40"/>
+      <c r="N25" s="36"/>
+      <c r="O25" s="38"/>
     </row>
     <row r="26" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="21">
+      <c r="B26" s="20">
         <v>23</v>
       </c>
       <c r="C26" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D26" s="29" t="s">
+      <c r="D26" s="28" t="s">
         <v>770</v>
       </c>
-      <c r="E26" s="25">
+      <c r="E26" s="24">
         <v>4000</v>
       </c>
-      <c r="F26" s="25" t="s">
+      <c r="F26" s="24" t="s">
         <v>836</v>
       </c>
-      <c r="G26" s="30">
+      <c r="G26" s="29">
         <v>9.65</v>
       </c>
-      <c r="H26" s="30">
+      <c r="H26" s="29">
         <f>G26*E26</f>
         <v>38600</v>
       </c>
-      <c r="I26" s="25" t="s">
+      <c r="I26" s="24" t="s">
         <v>771</v>
       </c>
       <c r="J26" s="14" t="s">
@@ -14526,755 +14521,752 @@
       </c>
     </row>
     <row r="27" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="21">
+      <c r="B27" s="20">
         <v>24</v>
       </c>
-      <c r="C27" s="25" t="s">
+      <c r="C27" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D27" s="29" t="s">
+      <c r="D27" s="28" t="s">
         <v>827</v>
       </c>
-      <c r="E27" s="25">
-        <v>1</v>
-      </c>
-      <c r="F27" s="25" t="s">
+      <c r="E27" s="24">
+        <v>1</v>
+      </c>
+      <c r="F27" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G27" s="30">
+      <c r="G27" s="29">
         <v>164000</v>
       </c>
-      <c r="H27" s="30">
+      <c r="H27" s="29">
         <f>G27*E27</f>
         <v>164000</v>
       </c>
-      <c r="I27" s="25" t="s">
+      <c r="I27" s="24" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="28" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="21">
+      <c r="B28" s="20">
         <v>25</v>
       </c>
       <c r="C28" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D28" s="29" t="s">
-        <v>866</v>
-      </c>
-      <c r="E28" s="25">
+      <c r="D28" s="28" t="s">
+        <v>865</v>
+      </c>
+      <c r="E28" s="24">
         <v>99.22</v>
       </c>
-      <c r="F28" s="25" t="s">
+      <c r="F28" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="G28" s="30">
+      <c r="G28" s="29">
         <v>670</v>
       </c>
-      <c r="H28" s="30">
+      <c r="H28" s="29">
         <f>G28*E28</f>
         <v>66477.399999999994</v>
       </c>
-      <c r="I28" s="25" t="s">
+      <c r="I28" s="24" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="29" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="21">
+      <c r="B29" s="20">
         <v>26</v>
       </c>
       <c r="C29" s="17"/>
-      <c r="D29" s="29" t="s">
-        <v>865</v>
-      </c>
-      <c r="E29" s="25">
+      <c r="D29" s="28" t="s">
+        <v>864</v>
+      </c>
+      <c r="E29" s="24">
         <v>68</v>
       </c>
-      <c r="F29" s="25" t="s">
+      <c r="F29" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="G29" s="30">
+      <c r="G29" s="29">
         <v>670</v>
       </c>
-      <c r="H29" s="30">
+      <c r="H29" s="29">
         <f>G29*E29</f>
         <v>45560</v>
       </c>
-      <c r="I29" s="25" t="s">
+      <c r="I29" s="24" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="30" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="21">
+      <c r="B30" s="20">
         <v>27</v>
       </c>
       <c r="C30" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D30" s="29" t="s">
+      <c r="D30" s="28" t="s">
         <v>833</v>
       </c>
-      <c r="E30" s="25">
-        <v>1</v>
-      </c>
-      <c r="F30" s="25" t="s">
+      <c r="E30" s="24">
+        <v>1</v>
+      </c>
+      <c r="F30" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G30" s="30">
+      <c r="G30" s="29">
         <v>56500</v>
       </c>
-      <c r="H30" s="30">
+      <c r="H30" s="29">
         <f>G30*E30</f>
         <v>56500</v>
       </c>
-      <c r="I30" s="25" t="s">
+      <c r="I30" s="24" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="31" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="21">
+      <c r="B31" s="20">
         <v>28</v>
       </c>
       <c r="C31" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="19" t="s">
         <v>777</v>
       </c>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="19">
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18">
         <f>G31*E31</f>
         <v>0</v>
       </c>
-      <c r="I31" s="21" t="s">
+      <c r="I31" s="20" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="32" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="21">
+      <c r="B32" s="20">
         <v>29</v>
       </c>
       <c r="C32" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D32" s="23" t="s">
+      <c r="D32" s="22" t="s">
         <v>785</v>
       </c>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24">
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="23">
         <f>G32*E32</f>
         <v>0</v>
       </c>
-      <c r="I32" s="22" t="s">
+      <c r="I32" s="21" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="33" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="21">
+    <row r="33" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="20">
         <v>30</v>
       </c>
       <c r="C33" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D33" s="23" t="s">
+      <c r="D33" s="22" t="s">
         <v>786</v>
       </c>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24">
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23">
         <f>G33*E33</f>
         <v>0</v>
       </c>
-      <c r="I33" s="22" t="s">
+      <c r="I33" s="21" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="34" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="21">
+    <row r="34" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="20">
         <v>31</v>
       </c>
       <c r="C34" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D34" s="23" t="s">
+      <c r="D34" s="22" t="s">
         <v>787</v>
       </c>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24">
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23">
         <f>G34*E34</f>
         <v>0</v>
       </c>
-      <c r="I34" s="22" t="s">
+      <c r="I34" s="21" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="35" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="21">
+    <row r="35" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="20">
         <v>32</v>
       </c>
       <c r="C35" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D35" s="23" t="s">
+      <c r="D35" s="22" t="s">
         <v>788</v>
       </c>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="24"/>
-      <c r="H35" s="24">
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="23">
         <f>G35*E35</f>
         <v>0</v>
       </c>
-      <c r="I35" s="22" t="s">
+      <c r="I35" s="21" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B36" s="21">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B36" s="20">
         <v>33</v>
       </c>
-      <c r="C36" s="25" t="s">
+      <c r="C36" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D36" s="29" t="s">
+      <c r="D36" s="28" t="s">
         <v>757</v>
       </c>
-      <c r="E36" s="31">
+      <c r="E36" s="30">
         <f>(2150*1.05)*0.15</f>
         <v>338.625</v>
       </c>
-      <c r="F36" s="25" t="s">
+      <c r="F36" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="G36" s="30">
+      <c r="G36" s="29">
         <v>670</v>
       </c>
-      <c r="H36" s="30">
+      <c r="H36" s="29">
         <f>G36*E36</f>
         <v>226878.75</v>
       </c>
-      <c r="I36" s="25" t="s">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="21">
+      <c r="I36" s="24" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B37" s="20">
         <v>34</v>
       </c>
-      <c r="C37" s="25" t="s">
+      <c r="C37" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D37" s="29" t="s">
+      <c r="D37" s="28" t="s">
         <v>775</v>
       </c>
-      <c r="E37" s="31">
+      <c r="E37" s="30">
         <f>(2150/13)*2</f>
         <v>330.76923076923077</v>
       </c>
-      <c r="F37" s="25" t="s">
+      <c r="F37" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G37" s="30">
+      <c r="G37" s="29">
         <v>220.5</v>
       </c>
-      <c r="H37" s="30">
+      <c r="H37" s="29">
         <f>G37*E37</f>
         <v>72934.61538461539</v>
       </c>
-      <c r="I37" s="25" t="s">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="21">
+      <c r="I37" s="24" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B38" s="20">
         <v>35</v>
       </c>
-      <c r="C38" s="25" t="s">
+      <c r="C38" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D38" s="29" t="s">
+      <c r="D38" s="28" t="s">
         <v>758</v>
       </c>
-      <c r="E38" s="25">
+      <c r="E38" s="24">
         <f>2100/12</f>
         <v>175</v>
       </c>
-      <c r="F38" s="25" t="s">
+      <c r="F38" s="24" t="s">
         <v>761</v>
       </c>
-      <c r="G38" s="30">
+      <c r="G38" s="29">
         <v>56.2</v>
       </c>
-      <c r="H38" s="30">
+      <c r="H38" s="29">
         <f>G38*E38</f>
         <v>9835</v>
       </c>
-      <c r="I38" s="25" t="s">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="21">
+      <c r="I38" s="24" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B39" s="20">
         <v>36</v>
       </c>
-      <c r="C39" s="25" t="s">
+      <c r="C39" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D39" s="29" t="s">
+      <c r="D39" s="28" t="s">
         <v>762</v>
       </c>
-      <c r="E39" s="25">
+      <c r="E39" s="24">
         <v>1000</v>
       </c>
-      <c r="F39" s="25" t="s">
+      <c r="F39" s="24" t="s">
         <v>763</v>
       </c>
-      <c r="G39" s="30">
+      <c r="G39" s="29">
         <v>7.3</v>
       </c>
-      <c r="H39" s="30">
+      <c r="H39" s="29">
         <f>G39*E39</f>
         <v>7300</v>
       </c>
-      <c r="I39" s="25" t="s">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B40" s="21">
+      <c r="I39" s="24" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B40" s="20">
         <v>37</v>
       </c>
       <c r="C40" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D40" s="29" t="s">
+      <c r="D40" s="28" t="s">
         <v>811</v>
       </c>
-      <c r="E40" s="31">
+      <c r="E40" s="30">
         <f>E36</f>
         <v>338.625</v>
       </c>
-      <c r="F40" s="25" t="s">
+      <c r="F40" s="24" t="s">
         <v>766</v>
       </c>
-      <c r="G40" s="30">
+      <c r="G40" s="29">
         <v>50</v>
       </c>
-      <c r="H40" s="30">
+      <c r="H40" s="29">
         <f>G40*E40</f>
         <v>16931.25</v>
       </c>
-      <c r="I40" s="25" t="s">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B41" s="21">
+      <c r="I40" s="24" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B41" s="20">
         <v>38</v>
       </c>
       <c r="C41" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D41" s="29" t="s">
-        <v>870</v>
-      </c>
-      <c r="E41" s="25">
-        <v>1</v>
-      </c>
-      <c r="F41" s="25" t="s">
+      <c r="D41" s="28" t="s">
+        <v>869</v>
+      </c>
+      <c r="E41" s="24">
+        <v>1</v>
+      </c>
+      <c r="F41" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G41" s="30">
+      <c r="G41" s="29">
         <v>53550</v>
       </c>
-      <c r="H41" s="30">
+      <c r="H41" s="29">
         <f>G41*E41</f>
         <v>53550</v>
       </c>
-      <c r="I41" s="25" t="s">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B42" s="21">
+      <c r="I41" s="24" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B42" s="20">
         <v>39</v>
       </c>
-      <c r="C42" s="32" t="s">
+      <c r="C42" s="31" t="s">
         <v>808</v>
       </c>
-      <c r="D42" s="45" t="s">
+      <c r="D42" s="43" t="s">
         <v>815</v>
       </c>
-      <c r="E42" s="46">
+      <c r="E42" s="44">
         <v>110</v>
       </c>
-      <c r="F42" s="46" t="s">
+      <c r="F42" s="44" t="s">
         <v>760</v>
       </c>
-      <c r="G42" s="47">
+      <c r="G42" s="45">
         <v>42.29</v>
       </c>
-      <c r="H42" s="47">
+      <c r="H42" s="45">
         <f>G42*E42</f>
         <v>4651.8999999999996</v>
       </c>
-      <c r="I42" s="46" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B43" s="21">
+      <c r="I42" s="44" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B43" s="20">
         <v>40</v>
       </c>
-      <c r="C43" s="32"/>
-      <c r="D43" s="45" t="s">
-        <v>874</v>
-      </c>
-      <c r="E43" s="46">
-        <v>1</v>
-      </c>
-      <c r="F43" s="46" t="s">
+      <c r="C43" s="31"/>
+      <c r="D43" s="43" t="s">
+        <v>872</v>
+      </c>
+      <c r="E43" s="44">
+        <v>1</v>
+      </c>
+      <c r="F43" s="44" t="s">
         <v>760</v>
       </c>
-      <c r="G43" s="47">
+      <c r="G43" s="45">
         <v>1400</v>
       </c>
-      <c r="H43" s="47">
+      <c r="H43" s="45">
         <f>G43*E43</f>
         <v>1400</v>
       </c>
-      <c r="I43" s="46" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B44" s="21">
+      <c r="I43" s="44" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B44" s="20">
         <v>41</v>
       </c>
-      <c r="C44" s="32" t="s">
+      <c r="C44" s="31" t="s">
         <v>808</v>
       </c>
-      <c r="D44" s="23" t="s">
+      <c r="D44" s="43" t="s">
         <v>757</v>
       </c>
-      <c r="E44" s="33">
-        <f>(1784*0.15)*1.05</f>
-        <v>280.97999999999996</v>
-      </c>
-      <c r="F44" s="22" t="s">
+      <c r="E44" s="50">
+        <f>((1260+960)*0.15)*1.1</f>
+        <v>366.3</v>
+      </c>
+      <c r="F44" s="44" t="s">
         <v>759</v>
       </c>
-      <c r="G44" s="24">
+      <c r="G44" s="45">
         <v>670</v>
       </c>
-      <c r="H44" s="24">
+      <c r="H44" s="45">
         <f>G44*E44</f>
-        <v>188256.59999999998</v>
-      </c>
-      <c r="I44" s="46" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B45" s="21">
+        <v>245421</v>
+      </c>
+      <c r="I44" s="44" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B45" s="20">
         <v>42</v>
       </c>
-      <c r="C45" s="32" t="s">
+      <c r="C45" s="31" t="s">
         <v>808</v>
       </c>
-      <c r="D45" s="18" t="s">
+      <c r="D45" s="28" t="s">
         <v>775</v>
       </c>
-      <c r="E45" s="33">
-        <f>1784/13</f>
-        <v>137.23076923076923</v>
-      </c>
-      <c r="F45" s="22" t="s">
+      <c r="E45" s="50">
+        <f>(1260+960)/13*1.05</f>
+        <v>179.30769230769232</v>
+      </c>
+      <c r="F45" s="44" t="s">
         <v>760</v>
       </c>
-      <c r="G45" s="24">
+      <c r="G45" s="45">
         <v>220.5</v>
       </c>
-      <c r="H45" s="24">
+      <c r="H45" s="45">
         <f>G45*E45</f>
-        <v>30259.384615384613</v>
-      </c>
-      <c r="I45" s="46" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B46" s="21">
+        <v>39537.346153846156</v>
+      </c>
+      <c r="I45" s="44" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B46" s="20">
         <v>43</v>
       </c>
-      <c r="C46" s="32" t="s">
+      <c r="C46" s="31" t="s">
         <v>808</v>
       </c>
-      <c r="D46" s="23" t="s">
-        <v>869</v>
-      </c>
-      <c r="E46" s="22">
-        <v>1</v>
-      </c>
-      <c r="F46" s="22" t="s">
+      <c r="D46" s="22" t="s">
+        <v>868</v>
+      </c>
+      <c r="E46" s="21">
+        <v>1</v>
+      </c>
+      <c r="F46" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="G46" s="24"/>
-      <c r="H46" s="24">
+      <c r="G46" s="23"/>
+      <c r="H46" s="23">
         <f>G46*E46</f>
         <v>0</v>
       </c>
-      <c r="I46" s="22" t="s">
+      <c r="I46" s="44" t="s">
         <v>871</v>
       </c>
-      <c r="J46" s="50" t="s">
-        <v>862</v>
-      </c>
-    </row>
-    <row r="47" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="21">
+    </row>
+    <row r="47" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="20">
         <v>44</v>
       </c>
       <c r="C47" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D47" s="29" t="s">
+      <c r="D47" s="28" t="s">
         <v>855</v>
       </c>
-      <c r="E47" s="25">
-        <v>1</v>
-      </c>
-      <c r="F47" s="25" t="s">
+      <c r="E47" s="24">
+        <v>1</v>
+      </c>
+      <c r="F47" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G47" s="34">
+      <c r="G47" s="32">
         <v>24500</v>
       </c>
-      <c r="H47" s="34">
+      <c r="H47" s="32">
         <f>G47*E47</f>
         <v>24500</v>
       </c>
-      <c r="I47" s="25" t="s">
+      <c r="I47" s="24" t="s">
         <v>772</v>
       </c>
     </row>
-    <row r="48" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="21">
+    <row r="48" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="20">
         <v>45</v>
       </c>
       <c r="C48" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D48" s="20" t="s">
+      <c r="D48" s="19" t="s">
         <v>832</v>
       </c>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
-      <c r="G48" s="19"/>
-      <c r="H48" s="19">
+      <c r="E48" s="20"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="18"/>
+      <c r="H48" s="18">
         <f>G48*E48</f>
         <v>0</v>
       </c>
-      <c r="I48" s="21" t="s">
+      <c r="I48" s="20" t="s">
         <v>772</v>
       </c>
     </row>
     <row r="49" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="21">
+      <c r="B49" s="20">
         <v>46</v>
       </c>
       <c r="C49" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D49" s="29" t="s">
+      <c r="D49" s="28" t="s">
         <v>773</v>
       </c>
-      <c r="E49" s="25">
-        <v>1</v>
-      </c>
-      <c r="F49" s="25" t="s">
+      <c r="E49" s="24">
+        <v>1</v>
+      </c>
+      <c r="F49" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G49" s="30">
+      <c r="G49" s="29">
         <v>968004</v>
       </c>
-      <c r="H49" s="30">
+      <c r="H49" s="29">
         <f>G49*E49</f>
         <v>968004</v>
       </c>
-      <c r="I49" s="25" t="s">
+      <c r="I49" s="24" t="s">
         <v>772</v>
       </c>
     </row>
     <row r="50" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="21">
+      <c r="B50" s="20">
         <v>47</v>
       </c>
       <c r="C50" s="17" t="s">
         <v>808</v>
       </c>
-      <c r="D50" s="45" t="s">
+      <c r="D50" s="43" t="s">
         <v>802</v>
       </c>
-      <c r="E50" s="46">
-        <v>1</v>
-      </c>
-      <c r="F50" s="46" t="s">
+      <c r="E50" s="44">
+        <v>1</v>
+      </c>
+      <c r="F50" s="44" t="s">
         <v>760</v>
       </c>
-      <c r="G50" s="47">
+      <c r="G50" s="45">
         <v>46600</v>
       </c>
-      <c r="H50" s="47">
+      <c r="H50" s="45">
         <f>G50*E50</f>
         <v>46600</v>
       </c>
-      <c r="I50" s="46" t="s">
+      <c r="I50" s="44" t="s">
         <v>804</v>
       </c>
     </row>
     <row r="51" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="21">
+      <c r="B51" s="20">
         <v>48</v>
       </c>
       <c r="C51" s="17" t="s">
         <v>808</v>
       </c>
-      <c r="D51" s="45" t="s">
+      <c r="D51" s="43" t="s">
         <v>805</v>
       </c>
-      <c r="E51" s="46">
-        <v>1</v>
-      </c>
-      <c r="F51" s="46" t="s">
+      <c r="E51" s="44">
+        <v>1</v>
+      </c>
+      <c r="F51" s="44" t="s">
         <v>760</v>
       </c>
-      <c r="G51" s="47">
+      <c r="G51" s="45">
         <v>8100</v>
       </c>
-      <c r="H51" s="47">
+      <c r="H51" s="45">
         <f>G51*E51</f>
         <v>8100</v>
       </c>
-      <c r="I51" s="46" t="s">
+      <c r="I51" s="44" t="s">
         <v>804</v>
       </c>
     </row>
     <row r="52" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="21">
+      <c r="B52" s="20">
         <v>49</v>
       </c>
       <c r="C52" s="17" t="s">
         <v>808</v>
       </c>
-      <c r="D52" s="45" t="s">
+      <c r="D52" s="43" t="s">
         <v>817</v>
       </c>
-      <c r="E52" s="46">
-        <v>1</v>
-      </c>
-      <c r="F52" s="46" t="s">
+      <c r="E52" s="44">
+        <v>1</v>
+      </c>
+      <c r="F52" s="44" t="s">
         <v>760</v>
       </c>
-      <c r="G52" s="47">
+      <c r="G52" s="45">
         <v>5000</v>
       </c>
-      <c r="H52" s="47">
+      <c r="H52" s="45">
         <f>G52*E52</f>
         <v>5000</v>
       </c>
-      <c r="I52" s="46" t="s">
+      <c r="I52" s="44" t="s">
         <v>804</v>
       </c>
     </row>
     <row r="53" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="21">
+      <c r="B53" s="20">
         <v>50</v>
       </c>
       <c r="C53" s="17" t="s">
         <v>808</v>
       </c>
-      <c r="D53" s="45" t="s">
+      <c r="D53" s="43" t="s">
         <v>809</v>
       </c>
-      <c r="E53" s="46">
-        <v>1</v>
-      </c>
-      <c r="F53" s="46" t="s">
+      <c r="E53" s="44">
+        <v>1</v>
+      </c>
+      <c r="F53" s="44" t="s">
         <v>760</v>
       </c>
-      <c r="G53" s="47">
+      <c r="G53" s="45">
         <v>670000</v>
       </c>
-      <c r="H53" s="47">
+      <c r="H53" s="45">
         <f>G53*E53</f>
         <v>670000</v>
       </c>
-      <c r="I53" s="46" t="s">
+      <c r="I53" s="44" t="s">
         <v>804</v>
       </c>
     </row>
     <row r="54" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="21">
+      <c r="B54" s="20">
         <v>54</v>
       </c>
       <c r="C54" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D54" s="20" t="s">
+      <c r="D54" s="19" t="s">
         <v>791</v>
       </c>
-      <c r="E54" s="21"/>
-      <c r="F54" s="21"/>
-      <c r="G54" s="19"/>
-      <c r="H54" s="19">
+      <c r="E54" s="20"/>
+      <c r="F54" s="20"/>
+      <c r="G54" s="18"/>
+      <c r="H54" s="18">
         <f>G54*E54</f>
         <v>0</v>
       </c>
-      <c r="I54" s="21" t="s">
+      <c r="I54" s="20" t="s">
         <v>419</v>
       </c>
     </row>
     <row r="55" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="21">
+      <c r="B55" s="20">
         <v>55</v>
       </c>
       <c r="C55" s="17"/>
-      <c r="D55" s="20" t="s">
+      <c r="D55" s="19" t="s">
         <v>850</v>
       </c>
-      <c r="E55" s="21"/>
-      <c r="F55" s="21"/>
-      <c r="G55" s="19"/>
-      <c r="H55" s="19">
+      <c r="E55" s="20"/>
+      <c r="F55" s="20"/>
+      <c r="G55" s="18"/>
+      <c r="H55" s="18">
         <f>G55*E55</f>
         <v>0</v>
       </c>
-      <c r="I55" s="21" t="s">
+      <c r="I55" s="20" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="56" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="21">
+      <c r="B56" s="20">
         <v>56</v>
       </c>
       <c r="C56" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D56" s="20" t="s">
+      <c r="D56" s="19" t="s">
         <v>792</v>
       </c>
-      <c r="E56" s="21"/>
-      <c r="F56" s="21"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="19">
+      <c r="E56" s="20"/>
+      <c r="F56" s="20"/>
+      <c r="G56" s="18"/>
+      <c r="H56" s="18">
         <f>G56*E56</f>
         <v>0</v>
       </c>
@@ -15283,143 +15275,143 @@
       </c>
     </row>
     <row r="57" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="21">
+      <c r="B57" s="20">
         <v>57</v>
       </c>
       <c r="C57" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D57" s="20" t="s">
+      <c r="D57" s="19" t="s">
         <v>784</v>
       </c>
-      <c r="E57" s="21">
-        <v>1</v>
-      </c>
-      <c r="F57" s="21" t="s">
+      <c r="E57" s="20">
+        <v>1</v>
+      </c>
+      <c r="F57" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="G57" s="19">
+      <c r="G57" s="18">
         <v>791792.51</v>
       </c>
-      <c r="H57" s="19">
+      <c r="H57" s="18">
         <f>G57*E57</f>
         <v>791792.51</v>
       </c>
-      <c r="I57" s="21" t="s">
+      <c r="I57" s="20" t="s">
         <v>783</v>
       </c>
     </row>
     <row r="58" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="21">
+      <c r="B58" s="20">
         <v>51</v>
       </c>
       <c r="C58" s="17"/>
-      <c r="D58" s="23" t="s">
-        <v>863</v>
-      </c>
-      <c r="E58" s="22"/>
-      <c r="F58" s="22"/>
-      <c r="G58" s="51"/>
-      <c r="H58" s="51">
+      <c r="D58" s="22" t="s">
+        <v>862</v>
+      </c>
+      <c r="E58" s="21"/>
+      <c r="F58" s="21"/>
+      <c r="G58" s="49"/>
+      <c r="H58" s="49">
         <f>G58*E58</f>
         <v>0</v>
       </c>
-      <c r="I58" s="22"/>
+      <c r="I58" s="21"/>
     </row>
     <row r="59" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="21">
+      <c r="B59" s="20">
         <v>52</v>
       </c>
       <c r="C59" s="17"/>
-      <c r="D59" s="23" t="s">
-        <v>864</v>
-      </c>
-      <c r="E59" s="22"/>
-      <c r="F59" s="22"/>
-      <c r="G59" s="51"/>
-      <c r="H59" s="51">
+      <c r="D59" s="22" t="s">
+        <v>863</v>
+      </c>
+      <c r="E59" s="21"/>
+      <c r="F59" s="21"/>
+      <c r="G59" s="49"/>
+      <c r="H59" s="49">
         <f>G59*E59</f>
         <v>0</v>
       </c>
-      <c r="I59" s="22"/>
+      <c r="I59" s="21"/>
     </row>
     <row r="60" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="21">
+      <c r="B60" s="20">
         <v>53</v>
       </c>
       <c r="C60" s="17"/>
-      <c r="D60" s="23" t="s">
-        <v>867</v>
-      </c>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="51"/>
-      <c r="H60" s="51">
+      <c r="D60" s="22" t="s">
+        <v>866</v>
+      </c>
+      <c r="E60" s="21"/>
+      <c r="F60" s="21"/>
+      <c r="G60" s="49"/>
+      <c r="H60" s="49">
         <f>G60*E60</f>
         <v>0</v>
       </c>
-      <c r="I60" s="22"/>
+      <c r="I60" s="21"/>
     </row>
     <row r="61" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="21"/>
+      <c r="B61" s="20"/>
       <c r="C61" s="17"/>
-      <c r="D61" s="20" t="s">
-        <v>868</v>
-      </c>
-      <c r="E61" s="21"/>
-      <c r="F61" s="21"/>
-      <c r="G61" s="19"/>
-      <c r="H61" s="19">
+      <c r="D61" s="19" t="s">
+        <v>867</v>
+      </c>
+      <c r="E61" s="20"/>
+      <c r="F61" s="20"/>
+      <c r="G61" s="18"/>
+      <c r="H61" s="18">
         <f>G61*E61</f>
         <v>0</v>
       </c>
-      <c r="I61" s="21"/>
-      <c r="J61" s="50" t="s">
+      <c r="I61" s="20"/>
+      <c r="J61" s="48" t="s">
         <v>860</v>
       </c>
     </row>
     <row r="62" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="21">
+      <c r="B62" s="20">
         <v>58</v>
       </c>
-      <c r="C62" s="32"/>
-      <c r="D62" s="23" t="s">
+      <c r="C62" s="31"/>
+      <c r="D62" s="22" t="s">
         <v>859</v>
       </c>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
-      <c r="G62" s="24"/>
-      <c r="H62" s="49">
+      <c r="E62" s="21"/>
+      <c r="F62" s="21"/>
+      <c r="G62" s="23"/>
+      <c r="H62" s="47">
         <f>G62*E62</f>
         <v>0</v>
       </c>
-      <c r="I62" s="22"/>
+      <c r="I62" s="21"/>
     </row>
     <row r="63" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B63" s="22"/>
-      <c r="C63" s="32"/>
-      <c r="D63" s="23"/>
-      <c r="E63" s="22"/>
-      <c r="F63" s="22"/>
-      <c r="G63" s="24"/>
-      <c r="H63" s="49"/>
-      <c r="I63" s="22"/>
+      <c r="B63" s="21"/>
+      <c r="C63" s="31"/>
+      <c r="D63" s="22"/>
+      <c r="E63" s="21"/>
+      <c r="F63" s="21"/>
+      <c r="G63" s="23"/>
+      <c r="H63" s="47"/>
+      <c r="I63" s="21"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B64" s="22"/>
-      <c r="C64" s="32"/>
-      <c r="D64" s="23"/>
-      <c r="E64" s="22"/>
-      <c r="F64" s="22"/>
-      <c r="G64" s="24"/>
-      <c r="H64" s="49"/>
-      <c r="I64" s="22"/>
+      <c r="B64" s="21"/>
+      <c r="C64" s="31"/>
+      <c r="D64" s="22"/>
+      <c r="E64" s="21"/>
+      <c r="F64" s="21"/>
+      <c r="G64" s="23"/>
+      <c r="H64" s="47"/>
+      <c r="I64" s="21"/>
     </row>
     <row r="65" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D65" s="36"/>
+      <c r="D65" s="34"/>
       <c r="H65" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>4128872.0265427995</v>
+        <v>4195314.3880812619</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 15:56
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -2637,13 +2637,13 @@
     <t>Mão de obra para concretagem do piso do galpão 2100m² (DPA IV)</t>
   </si>
   <si>
-    <t>Piso Galpão</t>
-  </si>
-  <si>
     <t>Piso Pátio de Manobra</t>
   </si>
   <si>
     <t>Frete para entrega do Meio fio</t>
+  </si>
+  <si>
+    <t>Piso Galpão DPA IV</t>
   </si>
 </sst>
 </file>
@@ -14756,7 +14756,7 @@
         <v>226878.75</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.25">
@@ -14784,7 +14784,7 @@
         <v>72934.61538461539</v>
       </c>
       <c r="I37" s="24" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.25">
@@ -14812,7 +14812,7 @@
         <v>9835</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
@@ -14839,7 +14839,7 @@
         <v>7300</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.25">
@@ -14867,7 +14867,7 @@
         <v>16931.25</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.25">
@@ -14894,7 +14894,7 @@
         <v>53550</v>
       </c>
       <c r="I41" s="24" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.25">
@@ -14921,7 +14921,7 @@
         <v>4651.8999999999996</v>
       </c>
       <c r="I42" s="44" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.25">
@@ -14930,7 +14930,7 @@
       </c>
       <c r="C43" s="31"/>
       <c r="D43" s="43" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="E43" s="44">
         <v>1</v>
@@ -14946,7 +14946,7 @@
         <v>1400</v>
       </c>
       <c r="I43" s="44" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.25">
@@ -14974,7 +14974,7 @@
         <v>245421</v>
       </c>
       <c r="I44" s="44" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
@@ -15002,7 +15002,7 @@
         <v>39537.346153846156</v>
       </c>
       <c r="I45" s="44" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
@@ -15027,7 +15027,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="44" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="47" spans="2:9" hidden="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:09
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2157" uniqueCount="873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2162" uniqueCount="873">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2607,9 +2607,6 @@
     <t>Mão de obra para fechamento em alvenaria na parte interna do galpão blocado</t>
   </si>
   <si>
-    <t>Solicitar mais um orçamento do Erisvaldo</t>
-  </si>
-  <si>
     <t>Mão de obra para concretagem do piso das docas de carregamento DPA IV (interno)</t>
   </si>
   <si>
@@ -2631,9 +2628,6 @@
     <t>Cabo para ligação do sistema de tratamento de esgoto do banheiro</t>
   </si>
   <si>
-    <t>Mão de obra para concretagem do piso e instalação do meio-fio (PÁTIO)</t>
-  </si>
-  <si>
     <t>Mão de obra para concretagem do piso do galpão 2100m² (DPA IV)</t>
   </si>
   <si>
@@ -2644,6 +2638,12 @@
   </si>
   <si>
     <t>Piso Galpão DPA IV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mão de obra para concretagem do piso e instalação do meio-fio </t>
+  </si>
+  <si>
+    <t>Docas de Carregamento</t>
   </si>
 </sst>
 </file>
@@ -3183,15 +3183,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I62" totalsRowShown="0" headerRowDxfId="0" dataDxfId="17">
-  <autoFilter ref="B3:I62">
-    <filterColumn colId="7">
-      <filters>
-        <filter val="Piso"/>
-        <filter val="Piso pátio"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I65" totalsRowShown="0" headerRowDxfId="0" dataDxfId="17">
+  <autoFilter ref="B3:I65"/>
   <sortState ref="B4:I62">
     <sortCondition ref="I3:I62"/>
   </sortState>
@@ -13697,7 +13690,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R65"/>
+  <dimension ref="B1:R68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -13756,7 +13749,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="4" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B4" s="20">
         <v>1</v>
       </c>
@@ -13793,7 +13786,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="5" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B5" s="20">
         <v>2</v>
       </c>
@@ -13838,7 +13831,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="6" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B6" s="20">
         <v>3</v>
       </c>
@@ -13879,7 +13872,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="7" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B7" s="20">
         <v>4</v>
       </c>
@@ -13913,7 +13906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B8" s="20">
         <v>5</v>
       </c>
@@ -13947,13 +13940,13 @@
         <v>0.20544460449492216</v>
       </c>
     </row>
-    <row r="9" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B9" s="20">
         <v>6</v>
       </c>
       <c r="C9" s="31"/>
       <c r="D9" s="22" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="E9" s="21">
         <v>1</v>
@@ -13981,7 +13974,7 @@
         <v>0.11732117275604338</v>
       </c>
     </row>
-    <row r="10" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B10" s="20">
         <v>7</v>
       </c>
@@ -14017,7 +14010,7 @@
         <v>1.8732442013457442E-2</v>
       </c>
     </row>
-    <row r="11" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B11" s="20">
         <v>8</v>
       </c>
@@ -14055,7 +14048,7 @@
         <v>0.13684069071108126</v>
       </c>
     </row>
-    <row r="12" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B12" s="20">
         <v>9</v>
       </c>
@@ -14087,7 +14080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B13" s="20">
         <v>10</v>
       </c>
@@ -14117,7 +14110,7 @@
       <c r="O13" s="35"/>
       <c r="P13" s="39"/>
     </row>
-    <row r="14" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B14" s="20">
         <v>11</v>
       </c>
@@ -14155,7 +14148,7 @@
         <v>1.8732442013457442E-2</v>
       </c>
     </row>
-    <row r="15" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B15" s="20">
         <v>12</v>
       </c>
@@ -14193,7 +14186,7 @@
         <v>5.6590880503603334E-4</v>
       </c>
     </row>
-    <row r="16" spans="2:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B16" s="20">
         <v>13</v>
       </c>
@@ -14224,7 +14217,7 @@
       <c r="O16" s="35"/>
       <c r="P16" s="39"/>
     </row>
-    <row r="17" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" s="20">
         <v>14</v>
       </c>
@@ -14255,7 +14248,7 @@
       <c r="O17" s="35"/>
       <c r="P17" s="39"/>
     </row>
-    <row r="18" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" s="20">
         <v>15</v>
       </c>
@@ -14283,7 +14276,7 @@
       <c r="O18" s="35"/>
       <c r="P18" s="39"/>
     </row>
-    <row r="19" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B19" s="20">
         <v>16</v>
       </c>
@@ -14319,7 +14312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="20">
         <v>17</v>
       </c>
@@ -14353,7 +14346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B21" s="20">
         <v>18</v>
       </c>
@@ -14377,7 +14370,7 @@
       <c r="O21" s="35"/>
       <c r="P21" s="39"/>
     </row>
-    <row r="22" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B22" s="20">
         <v>19</v>
       </c>
@@ -14401,7 +14394,7 @@
       <c r="O22" s="35"/>
       <c r="P22" s="39"/>
     </row>
-    <row r="23" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B23" s="20">
         <v>20</v>
       </c>
@@ -14424,7 +14417,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="24" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B24" s="20">
         <v>21</v>
       </c>
@@ -14458,7 +14451,7 @@
         <v>3551809.0231375997</v>
       </c>
     </row>
-    <row r="25" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B25" s="20">
         <v>22</v>
       </c>
@@ -14490,7 +14483,7 @@
       <c r="N25" s="36"/>
       <c r="O25" s="38"/>
     </row>
-    <row r="26" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B26" s="20">
         <v>23</v>
       </c>
@@ -14520,7 +14513,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="27" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B27" s="20">
         <v>24</v>
       </c>
@@ -14547,7 +14540,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="28" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B28" s="20">
         <v>25</v>
       </c>
@@ -14555,7 +14548,7 @@
         <v>807</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="E28" s="24">
         <v>99.22</v>
@@ -14574,13 +14567,13 @@
         <v>771</v>
       </c>
     </row>
-    <row r="29" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B29" s="20">
         <v>26</v>
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="28" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="E29" s="24">
         <v>68</v>
@@ -14599,7 +14592,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="30" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B30" s="20">
         <v>27</v>
       </c>
@@ -14626,7 +14619,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="31" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B31" s="20">
         <v>28</v>
       </c>
@@ -14647,7 +14640,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="32" spans="2:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B32" s="20">
         <v>29</v>
       </c>
@@ -14668,7 +14661,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="33" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" s="20">
         <v>30</v>
       </c>
@@ -14689,7 +14682,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="34" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" s="20">
         <v>31</v>
       </c>
@@ -14710,7 +14703,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="35" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" s="20">
         <v>32</v>
       </c>
@@ -14756,7 +14749,7 @@
         <v>226878.75</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.25">
@@ -14784,7 +14777,7 @@
         <v>72934.61538461539</v>
       </c>
       <c r="I37" s="24" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.25">
@@ -14812,7 +14805,7 @@
         <v>9835</v>
       </c>
       <c r="I38" s="24" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
@@ -14839,7 +14832,7 @@
         <v>7300</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.25">
@@ -14867,7 +14860,7 @@
         <v>16931.25</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.25">
@@ -14878,7 +14871,7 @@
         <v>807</v>
       </c>
       <c r="D41" s="28" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="E41" s="24">
         <v>1</v>
@@ -14894,7 +14887,7 @@
         <v>53550</v>
       </c>
       <c r="I41" s="24" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.25">
@@ -14921,7 +14914,7 @@
         <v>4651.8999999999996</v>
       </c>
       <c r="I42" s="44" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.25">
@@ -14930,7 +14923,7 @@
       </c>
       <c r="C43" s="31"/>
       <c r="D43" s="43" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="E43" s="44">
         <v>1</v>
@@ -14946,7 +14939,7 @@
         <v>1400</v>
       </c>
       <c r="I43" s="44" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.25">
@@ -14974,7 +14967,7 @@
         <v>245421</v>
       </c>
       <c r="I44" s="44" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
@@ -15002,7 +14995,7 @@
         <v>39537.346153846156</v>
       </c>
       <c r="I45" s="44" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
@@ -15013,7 +15006,7 @@
         <v>808</v>
       </c>
       <c r="D46" s="22" t="s">
-        <v>868</v>
+        <v>871</v>
       </c>
       <c r="E46" s="21">
         <v>1</v>
@@ -15021,180 +15014,150 @@
       <c r="F46" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="G46" s="23"/>
-      <c r="H46" s="23">
+      <c r="G46" s="49"/>
+      <c r="H46" s="49">
         <f>G46*E46</f>
         <v>0</v>
       </c>
-      <c r="I46" s="44" t="s">
-        <v>870</v>
-      </c>
-    </row>
-    <row r="47" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="20">
-        <v>44</v>
-      </c>
-      <c r="C47" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D47" s="28" t="s">
-        <v>855</v>
-      </c>
-      <c r="E47" s="24">
-        <v>1</v>
-      </c>
-      <c r="F47" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G47" s="32">
-        <v>24500</v>
-      </c>
-      <c r="H47" s="32">
+      <c r="I46" s="21" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B47" s="20"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="22" t="s">
+        <v>757</v>
+      </c>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="49"/>
+      <c r="H47" s="49">
         <f>G47*E47</f>
-        <v>24500</v>
-      </c>
-      <c r="I47" s="24" t="s">
-        <v>772</v>
-      </c>
-    </row>
-    <row r="48" spans="2:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="20">
-        <v>45</v>
-      </c>
-      <c r="C48" s="17" t="s">
-        <v>807</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I47" s="21" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B48" s="20"/>
+      <c r="C48" s="31"/>
       <c r="D48" s="19" t="s">
-        <v>832</v>
-      </c>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="18"/>
-      <c r="H48" s="18">
+        <v>775</v>
+      </c>
+      <c r="E48" s="21"/>
+      <c r="F48" s="21"/>
+      <c r="G48" s="49"/>
+      <c r="H48" s="49">
         <f>G48*E48</f>
         <v>0</v>
       </c>
-      <c r="I48" s="20" t="s">
+      <c r="I48" s="21" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B49" s="20"/>
+      <c r="C49" s="31"/>
+      <c r="D49" s="19" t="s">
+        <v>758</v>
+      </c>
+      <c r="E49" s="21"/>
+      <c r="F49" s="21"/>
+      <c r="G49" s="49"/>
+      <c r="H49" s="49">
+        <f>G49*E49</f>
+        <v>0</v>
+      </c>
+      <c r="I49" s="21" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B50" s="20">
+        <v>44</v>
+      </c>
+      <c r="C50" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D50" s="28" t="s">
+        <v>855</v>
+      </c>
+      <c r="E50" s="24">
+        <v>1</v>
+      </c>
+      <c r="F50" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G50" s="32">
+        <v>24500</v>
+      </c>
+      <c r="H50" s="32">
+        <f>G50*E50</f>
+        <v>24500</v>
+      </c>
+      <c r="I50" s="24" t="s">
         <v>772</v>
       </c>
     </row>
-    <row r="49" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="20">
+    <row r="51" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B51" s="20">
+        <v>45</v>
+      </c>
+      <c r="C51" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D51" s="19" t="s">
+        <v>832</v>
+      </c>
+      <c r="E51" s="20"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="18"/>
+      <c r="H51" s="18">
+        <f>G51*E51</f>
+        <v>0</v>
+      </c>
+      <c r="I51" s="20" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B52" s="20">
         <v>46</v>
       </c>
-      <c r="C49" s="17" t="s">
+      <c r="C52" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D49" s="28" t="s">
+      <c r="D52" s="28" t="s">
         <v>773</v>
       </c>
-      <c r="E49" s="24">
-        <v>1</v>
-      </c>
-      <c r="F49" s="24" t="s">
+      <c r="E52" s="24">
+        <v>1</v>
+      </c>
+      <c r="F52" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G49" s="29">
+      <c r="G52" s="29">
         <v>968004</v>
       </c>
-      <c r="H49" s="29">
-        <f>G49*E49</f>
+      <c r="H52" s="29">
+        <f>G52*E52</f>
         <v>968004</v>
       </c>
-      <c r="I49" s="24" t="s">
+      <c r="I52" s="24" t="s">
         <v>772</v>
       </c>
     </row>
-    <row r="50" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="20">
+    <row r="53" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B53" s="20">
         <v>47</v>
-      </c>
-      <c r="C50" s="17" t="s">
-        <v>808</v>
-      </c>
-      <c r="D50" s="43" t="s">
-        <v>802</v>
-      </c>
-      <c r="E50" s="44">
-        <v>1</v>
-      </c>
-      <c r="F50" s="44" t="s">
-        <v>760</v>
-      </c>
-      <c r="G50" s="45">
-        <v>46600</v>
-      </c>
-      <c r="H50" s="45">
-        <f>G50*E50</f>
-        <v>46600</v>
-      </c>
-      <c r="I50" s="44" t="s">
-        <v>804</v>
-      </c>
-    </row>
-    <row r="51" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="20">
-        <v>48</v>
-      </c>
-      <c r="C51" s="17" t="s">
-        <v>808</v>
-      </c>
-      <c r="D51" s="43" t="s">
-        <v>805</v>
-      </c>
-      <c r="E51" s="44">
-        <v>1</v>
-      </c>
-      <c r="F51" s="44" t="s">
-        <v>760</v>
-      </c>
-      <c r="G51" s="45">
-        <v>8100</v>
-      </c>
-      <c r="H51" s="45">
-        <f>G51*E51</f>
-        <v>8100</v>
-      </c>
-      <c r="I51" s="44" t="s">
-        <v>804</v>
-      </c>
-    </row>
-    <row r="52" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="20">
-        <v>49</v>
-      </c>
-      <c r="C52" s="17" t="s">
-        <v>808</v>
-      </c>
-      <c r="D52" s="43" t="s">
-        <v>817</v>
-      </c>
-      <c r="E52" s="44">
-        <v>1</v>
-      </c>
-      <c r="F52" s="44" t="s">
-        <v>760</v>
-      </c>
-      <c r="G52" s="45">
-        <v>5000</v>
-      </c>
-      <c r="H52" s="45">
-        <f>G52*E52</f>
-        <v>5000</v>
-      </c>
-      <c r="I52" s="44" t="s">
-        <v>804</v>
-      </c>
-    </row>
-    <row r="53" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="20">
-        <v>50</v>
       </c>
       <c r="C53" s="17" t="s">
         <v>808</v>
       </c>
       <c r="D53" s="43" t="s">
-        <v>809</v>
+        <v>802</v>
       </c>
       <c r="E53" s="44">
         <v>1</v>
@@ -15203,213 +15166,293 @@
         <v>760</v>
       </c>
       <c r="G53" s="45">
-        <v>670000</v>
+        <v>46600</v>
       </c>
       <c r="H53" s="45">
         <f>G53*E53</f>
-        <v>670000</v>
+        <v>46600</v>
       </c>
       <c r="I53" s="44" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="54" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B54" s="20">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C54" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D54" s="19" t="s">
-        <v>791</v>
-      </c>
-      <c r="E54" s="20"/>
-      <c r="F54" s="20"/>
-      <c r="G54" s="18"/>
-      <c r="H54" s="18">
+        <v>808</v>
+      </c>
+      <c r="D54" s="43" t="s">
+        <v>805</v>
+      </c>
+      <c r="E54" s="44">
+        <v>1</v>
+      </c>
+      <c r="F54" s="44" t="s">
+        <v>760</v>
+      </c>
+      <c r="G54" s="45">
+        <v>8100</v>
+      </c>
+      <c r="H54" s="45">
         <f>G54*E54</f>
-        <v>0</v>
-      </c>
-      <c r="I54" s="20" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="55" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+        <v>8100</v>
+      </c>
+      <c r="I54" s="44" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B55" s="20">
-        <v>55</v>
-      </c>
-      <c r="C55" s="17"/>
-      <c r="D55" s="19" t="s">
-        <v>850</v>
-      </c>
-      <c r="E55" s="20"/>
-      <c r="F55" s="20"/>
-      <c r="G55" s="18"/>
-      <c r="H55" s="18">
+        <v>49</v>
+      </c>
+      <c r="C55" s="17" t="s">
+        <v>808</v>
+      </c>
+      <c r="D55" s="43" t="s">
+        <v>817</v>
+      </c>
+      <c r="E55" s="44">
+        <v>1</v>
+      </c>
+      <c r="F55" s="44" t="s">
+        <v>760</v>
+      </c>
+      <c r="G55" s="45">
+        <v>5000</v>
+      </c>
+      <c r="H55" s="45">
         <f>G55*E55</f>
-        <v>0</v>
-      </c>
-      <c r="I55" s="20" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="56" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+        <v>5000</v>
+      </c>
+      <c r="I55" s="44" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B56" s="20">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C56" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D56" s="19" t="s">
-        <v>792</v>
-      </c>
-      <c r="E56" s="20"/>
-      <c r="F56" s="20"/>
-      <c r="G56" s="18"/>
-      <c r="H56" s="18">
+        <v>808</v>
+      </c>
+      <c r="D56" s="43" t="s">
+        <v>809</v>
+      </c>
+      <c r="E56" s="44">
+        <v>1</v>
+      </c>
+      <c r="F56" s="44" t="s">
+        <v>760</v>
+      </c>
+      <c r="G56" s="45">
+        <v>670000</v>
+      </c>
+      <c r="H56" s="45">
         <f>G56*E56</f>
-        <v>0</v>
-      </c>
-      <c r="I56" s="17" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="57" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+        <v>670000</v>
+      </c>
+      <c r="I56" s="44" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" s="20">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C57" s="17" t="s">
         <v>807</v>
       </c>
       <c r="D57" s="19" t="s">
-        <v>784</v>
-      </c>
-      <c r="E57" s="20">
-        <v>1</v>
-      </c>
-      <c r="F57" s="20" t="s">
-        <v>760</v>
-      </c>
-      <c r="G57" s="18">
-        <v>791792.51</v>
-      </c>
+        <v>791</v>
+      </c>
+      <c r="E57" s="20"/>
+      <c r="F57" s="20"/>
+      <c r="G57" s="18"/>
       <c r="H57" s="18">
         <f>G57*E57</f>
-        <v>791792.51</v>
+        <v>0</v>
       </c>
       <c r="I57" s="20" t="s">
-        <v>783</v>
-      </c>
-    </row>
-    <row r="58" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B58" s="20">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C58" s="17"/>
-      <c r="D58" s="22" t="s">
-        <v>862</v>
-      </c>
-      <c r="E58" s="21"/>
-      <c r="F58" s="21"/>
-      <c r="G58" s="49"/>
-      <c r="H58" s="49">
+      <c r="D58" s="19" t="s">
+        <v>850</v>
+      </c>
+      <c r="E58" s="20"/>
+      <c r="F58" s="20"/>
+      <c r="G58" s="18"/>
+      <c r="H58" s="18">
         <f>G58*E58</f>
         <v>0</v>
       </c>
-      <c r="I58" s="21"/>
-    </row>
-    <row r="59" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="I58" s="20" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B59" s="20">
-        <v>52</v>
-      </c>
-      <c r="C59" s="17"/>
-      <c r="D59" s="22" t="s">
-        <v>863</v>
-      </c>
-      <c r="E59" s="21"/>
-      <c r="F59" s="21"/>
-      <c r="G59" s="49"/>
-      <c r="H59" s="49">
+        <v>53</v>
+      </c>
+      <c r="C59" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D59" s="19" t="s">
+        <v>792</v>
+      </c>
+      <c r="E59" s="20"/>
+      <c r="F59" s="20"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="18">
         <f>G59*E59</f>
         <v>0</v>
       </c>
-      <c r="I59" s="21"/>
-    </row>
-    <row r="60" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="I59" s="17" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B60" s="20">
-        <v>53</v>
-      </c>
-      <c r="C60" s="17"/>
-      <c r="D60" s="22" t="s">
-        <v>866</v>
-      </c>
-      <c r="E60" s="21"/>
-      <c r="F60" s="21"/>
-      <c r="G60" s="49"/>
-      <c r="H60" s="49">
+        <v>54</v>
+      </c>
+      <c r="C60" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D60" s="19" t="s">
+        <v>784</v>
+      </c>
+      <c r="E60" s="20">
+        <v>1</v>
+      </c>
+      <c r="F60" s="20" t="s">
+        <v>760</v>
+      </c>
+      <c r="G60" s="18">
+        <v>791792.51</v>
+      </c>
+      <c r="H60" s="18">
         <f>G60*E60</f>
-        <v>0</v>
-      </c>
-      <c r="I60" s="21"/>
-    </row>
-    <row r="61" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="20"/>
+        <v>791792.51</v>
+      </c>
+      <c r="I60" s="20" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B61" s="20">
+        <v>55</v>
+      </c>
       <c r="C61" s="17"/>
-      <c r="D61" s="19" t="s">
-        <v>867</v>
-      </c>
-      <c r="E61" s="20"/>
-      <c r="F61" s="20"/>
-      <c r="G61" s="18"/>
-      <c r="H61" s="18">
+      <c r="D61" s="22" t="s">
+        <v>861</v>
+      </c>
+      <c r="E61" s="21"/>
+      <c r="F61" s="21"/>
+      <c r="G61" s="49"/>
+      <c r="H61" s="49">
         <f>G61*E61</f>
         <v>0</v>
       </c>
-      <c r="I61" s="20"/>
-      <c r="J61" s="48" t="s">
-        <v>860</v>
-      </c>
-    </row>
-    <row r="62" spans="2:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="I61" s="21"/>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B62" s="20">
-        <v>58</v>
-      </c>
-      <c r="C62" s="31"/>
+        <v>56</v>
+      </c>
+      <c r="C62" s="17"/>
       <c r="D62" s="22" t="s">
-        <v>859</v>
+        <v>862</v>
       </c>
       <c r="E62" s="21"/>
       <c r="F62" s="21"/>
-      <c r="G62" s="23"/>
-      <c r="H62" s="47">
+      <c r="G62" s="49"/>
+      <c r="H62" s="49">
         <f>G62*E62</f>
         <v>0</v>
       </c>
       <c r="I62" s="21"/>
     </row>
-    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B63" s="21"/>
-      <c r="C63" s="31"/>
-      <c r="D63" s="22"/>
+    <row r="63" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B63" s="20">
+        <v>57</v>
+      </c>
+      <c r="C63" s="17"/>
+      <c r="D63" s="22" t="s">
+        <v>865</v>
+      </c>
       <c r="E63" s="21"/>
       <c r="F63" s="21"/>
-      <c r="G63" s="23"/>
-      <c r="H63" s="47"/>
+      <c r="G63" s="49"/>
+      <c r="H63" s="49">
+        <f>G63*E63</f>
+        <v>0</v>
+      </c>
       <c r="I63" s="21"/>
     </row>
-    <row r="64" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B64" s="21"/>
-      <c r="C64" s="31"/>
-      <c r="D64" s="22"/>
-      <c r="E64" s="21"/>
-      <c r="F64" s="21"/>
-      <c r="G64" s="23"/>
-      <c r="H64" s="47"/>
-      <c r="I64" s="21"/>
-    </row>
-    <row r="65" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D65" s="34"/>
-      <c r="H65" s="16">
+    <row r="64" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B64" s="20">
+        <v>58</v>
+      </c>
+      <c r="C64" s="17"/>
+      <c r="D64" s="19" t="s">
+        <v>866</v>
+      </c>
+      <c r="E64" s="20"/>
+      <c r="F64" s="20"/>
+      <c r="G64" s="18"/>
+      <c r="H64" s="18">
+        <f>G64*E64</f>
+        <v>0</v>
+      </c>
+      <c r="I64" s="20"/>
+    </row>
+    <row r="65" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B65" s="20">
+        <v>59</v>
+      </c>
+      <c r="C65" s="31"/>
+      <c r="D65" s="22" t="s">
+        <v>859</v>
+      </c>
+      <c r="E65" s="21"/>
+      <c r="F65" s="21"/>
+      <c r="G65" s="23"/>
+      <c r="H65" s="47">
+        <f>G65*E65</f>
+        <v>0</v>
+      </c>
+      <c r="I65" s="21"/>
+    </row>
+    <row r="66" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B66" s="21"/>
+      <c r="C66" s="31"/>
+      <c r="D66" s="22"/>
+      <c r="E66" s="21"/>
+      <c r="F66" s="21"/>
+      <c r="G66" s="23"/>
+      <c r="H66" s="47"/>
+      <c r="I66" s="21"/>
+    </row>
+    <row r="67" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B67" s="21"/>
+      <c r="C67" s="31"/>
+      <c r="D67" s="22"/>
+      <c r="E67" s="21"/>
+      <c r="F67" s="21"/>
+      <c r="G67" s="23"/>
+      <c r="H67" s="47"/>
+      <c r="I67" s="21"/>
+    </row>
+    <row r="68" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D68" s="34"/>
+      <c r="H68" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
         <v>4195314.3880812619</v>
       </c>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:14
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2162" uniqueCount="873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2167" uniqueCount="875">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2607,6 +2607,9 @@
     <t>Mão de obra para fechamento em alvenaria na parte interna do galpão blocado</t>
   </si>
   <si>
+    <t>Mão de obra para concretagem do piso do galpão 2100m²</t>
+  </si>
+  <si>
     <t>Mão de obra para concretagem do piso das docas de carregamento DPA IV (interno)</t>
   </si>
   <si>
@@ -2628,9 +2631,6 @@
     <t>Cabo para ligação do sistema de tratamento de esgoto do banheiro</t>
   </si>
   <si>
-    <t>Mão de obra para concretagem do piso do galpão 2100m² (DPA IV)</t>
-  </si>
-  <si>
     <t>Piso Pátio de Manobra</t>
   </si>
   <si>
@@ -2644,6 +2644,12 @@
   </si>
   <si>
     <t>Docas de Carregamento</t>
+  </si>
+  <si>
+    <t>Tratamento de Esgoto</t>
+  </si>
+  <si>
+    <t>Serviço Preliminar</t>
   </si>
 </sst>
 </file>
@@ -3185,8 +3191,8 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I65" totalsRowShown="0" headerRowDxfId="0" dataDxfId="17">
   <autoFilter ref="B3:I65"/>
-  <sortState ref="B4:I62">
-    <sortCondition ref="I3:I62"/>
+  <sortState ref="B4:I66">
+    <sortCondition ref="I3:I66"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" name="Item" dataDxfId="1" dataCellStyle="Normal"/>
@@ -13820,12 +13826,12 @@
         <v>992504</v>
       </c>
       <c r="P5" s="39">
-        <f t="shared" ref="P5:P20" si="0">O5/$O$24</f>
-        <v>0.27943619534004144</v>
+        <f>O5/$O$24</f>
+        <v>0.35168875187413606</v>
       </c>
       <c r="Q5" s="41">
         <f>P5</f>
-        <v>0.27943619534004144</v>
+        <v>0.35168875187413606</v>
       </c>
       <c r="R5" t="s">
         <v>823</v>
@@ -13861,12 +13867,12 @@
         <v>791792.51</v>
       </c>
       <c r="P6" s="39">
-        <f t="shared" si="0"/>
-        <v>0.22292654386596095</v>
+        <f>O6/$O$24</f>
+        <v>0.28056765472500805</v>
       </c>
       <c r="Q6" s="41">
         <f>P6+Q5</f>
-        <v>0.50236273920600238</v>
+        <v>0.63225640659914406</v>
       </c>
       <c r="R6" t="s">
         <v>823</v>
@@ -13902,7 +13908,7 @@
         <v>0</v>
       </c>
       <c r="P7" s="39">
-        <f t="shared" si="0"/>
+        <f>O7/$O$24</f>
         <v>0</v>
       </c>
     </row>
@@ -13933,11 +13939,11 @@
       </c>
       <c r="O8" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
-        <v>729700</v>
+        <v>0</v>
       </c>
       <c r="P8" s="39">
-        <f t="shared" si="0"/>
-        <v>0.20544460449492216</v>
+        <f>O8/$O$24</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
@@ -13946,7 +13952,7 @@
       </c>
       <c r="C9" s="31"/>
       <c r="D9" s="22" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="E9" s="21">
         <v>1</v>
@@ -13960,7 +13966,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="17" t="s">
-        <v>253</v>
+        <v>872</v>
       </c>
       <c r="N9" s="37" t="s">
         <v>771</v>
@@ -13970,33 +13976,27 @@
         <v>416702.4</v>
       </c>
       <c r="P9" s="39">
-        <f t="shared" si="0"/>
-        <v>0.11732117275604338</v>
+        <f>O9/$O$24</f>
+        <v>0.14765637917726981</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B10" s="20">
         <v>7</v>
       </c>
-      <c r="C10" s="17" t="s">
-        <v>807</v>
-      </c>
+      <c r="C10" s="31"/>
       <c r="D10" s="22" t="s">
-        <v>789</v>
-      </c>
-      <c r="E10" s="21">
-        <v>26</v>
-      </c>
-      <c r="F10" s="21" t="s">
-        <v>760</v>
-      </c>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23">
+        <v>757</v>
+      </c>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49">
         <f>G10*E10</f>
         <v>0</v>
       </c>
       <c r="I10" s="21" t="s">
-        <v>643</v>
+        <v>872</v>
       </c>
       <c r="N10" s="37" t="s">
         <v>774</v>
@@ -14006,35 +14006,27 @@
         <v>66534.056568800006</v>
       </c>
       <c r="P10" s="39">
-        <f t="shared" si="0"/>
-        <v>1.8732442013457442E-2</v>
+        <f t="shared" ref="P10:P12" si="0">O10/$O$24</f>
+        <v>2.3576005045626455E-2</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B11" s="20">
         <v>8</v>
       </c>
-      <c r="C11" s="24" t="s">
-        <v>807</v>
-      </c>
-      <c r="D11" s="43" t="s">
-        <v>790</v>
-      </c>
-      <c r="E11" s="44">
-        <v>600</v>
-      </c>
-      <c r="F11" s="44" t="s">
-        <v>761</v>
-      </c>
-      <c r="G11" s="45">
-        <v>3.35</v>
-      </c>
-      <c r="H11" s="45">
+      <c r="C11" s="31"/>
+      <c r="D11" s="19" t="s">
+        <v>775</v>
+      </c>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="49">
         <f>G11*E11</f>
-        <v>2010</v>
-      </c>
-      <c r="I11" s="44" t="s">
-        <v>643</v>
+        <v>0</v>
+      </c>
+      <c r="I11" s="21" t="s">
+        <v>872</v>
       </c>
       <c r="N11" s="36" t="s">
         <v>782</v>
@@ -14045,28 +14037,26 @@
       </c>
       <c r="P11" s="39">
         <f t="shared" si="0"/>
-        <v>0.13684069071108126</v>
+        <v>0.17222297084030905</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B12" s="20">
         <v>9</v>
       </c>
-      <c r="C12" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D12" s="22" t="s">
-        <v>812</v>
+      <c r="C12" s="31"/>
+      <c r="D12" s="19" t="s">
+        <v>758</v>
       </c>
       <c r="E12" s="21"/>
       <c r="F12" s="21"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23">
+      <c r="G12" s="49"/>
+      <c r="H12" s="49">
         <f>G12*E12</f>
         <v>0</v>
       </c>
       <c r="I12" s="21" t="s">
-        <v>643</v>
+        <v>872</v>
       </c>
       <c r="N12" s="36" t="s">
         <v>449</v>
@@ -14087,24 +14077,22 @@
       <c r="C13" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D13" s="28" t="s">
-        <v>829</v>
-      </c>
-      <c r="E13" s="24">
-        <v>54</v>
-      </c>
-      <c r="F13" s="24" t="s">
+      <c r="D13" s="22" t="s">
+        <v>789</v>
+      </c>
+      <c r="E13" s="21">
+        <v>26</v>
+      </c>
+      <c r="F13" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="G13" s="32">
-        <v>243.39</v>
-      </c>
-      <c r="H13" s="32">
+      <c r="G13" s="23"/>
+      <c r="H13" s="23">
         <f>G13*E13</f>
-        <v>13143.06</v>
-      </c>
-      <c r="I13" s="24" t="s">
-        <v>830</v>
+        <v>0</v>
+      </c>
+      <c r="I13" s="21" t="s">
+        <v>643</v>
       </c>
       <c r="N13" s="36"/>
       <c r="O13" s="35"/>
@@ -14114,27 +14102,27 @@
       <c r="B14" s="20">
         <v>11</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D14" s="28" t="s">
-        <v>831</v>
-      </c>
-      <c r="E14" s="24">
-        <v>30</v>
-      </c>
-      <c r="F14" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G14" s="32">
-        <v>119.7</v>
-      </c>
-      <c r="H14" s="32">
+      <c r="D14" s="43" t="s">
+        <v>790</v>
+      </c>
+      <c r="E14" s="44">
+        <v>600</v>
+      </c>
+      <c r="F14" s="44" t="s">
+        <v>761</v>
+      </c>
+      <c r="G14" s="45">
+        <v>3.35</v>
+      </c>
+      <c r="H14" s="45">
         <f>G14*E14</f>
-        <v>3591</v>
-      </c>
-      <c r="I14" s="24" t="s">
-        <v>830</v>
+        <v>2010</v>
+      </c>
+      <c r="I14" s="44" t="s">
+        <v>643</v>
       </c>
       <c r="N14" s="36" t="s">
         <v>774</v>
@@ -14144,35 +14132,29 @@
         <v>66534.056568800006</v>
       </c>
       <c r="P14" s="39">
-        <f t="shared" si="0"/>
-        <v>1.8732442013457442E-2</v>
+        <f>O14/$O$24</f>
+        <v>2.3576005045626455E-2</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B15" s="20">
         <v>12</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D15" s="28" t="s">
-        <v>828</v>
-      </c>
-      <c r="E15" s="44">
-        <v>390</v>
-      </c>
-      <c r="F15" s="24" t="s">
-        <v>761</v>
-      </c>
-      <c r="G15" s="32">
-        <v>38.116666600000002</v>
-      </c>
-      <c r="H15" s="32">
+      <c r="D15" s="22" t="s">
+        <v>812</v>
+      </c>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23">
         <f>G15*E15</f>
-        <v>14865.499974</v>
-      </c>
-      <c r="I15" s="24" t="s">
-        <v>830</v>
+        <v>0</v>
+      </c>
+      <c r="I15" s="21" t="s">
+        <v>643</v>
       </c>
       <c r="N15" s="36" t="s">
         <v>643</v>
@@ -14182,8 +14164,8 @@
         <v>2010</v>
       </c>
       <c r="P15" s="39">
-        <f t="shared" si="0"/>
-        <v>5.6590880503603334E-4</v>
+        <f>O15/$O$24</f>
+        <v>7.1223329202402556E-4</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
@@ -14196,9 +14178,8 @@
       <c r="D16" s="28" t="s">
         <v>829</v>
       </c>
-      <c r="E16" s="30">
-        <f>(84*1.02)*2*1.02</f>
-        <v>174.78720000000001</v>
+      <c r="E16" s="24">
+        <v>54</v>
       </c>
       <c r="F16" s="24" t="s">
         <v>760</v>
@@ -14208,10 +14189,10 @@
       </c>
       <c r="H16" s="32">
         <f>G16*E16</f>
-        <v>42541.456608</v>
+        <v>13143.06</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>774</v>
+        <v>830</v>
       </c>
       <c r="N16" s="36"/>
       <c r="O16" s="35"/>
@@ -14221,28 +14202,27 @@
       <c r="B17" s="20">
         <v>14</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="17" t="s">
         <v>807</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>828</v>
+        <v>831</v>
       </c>
       <c r="E17" s="24">
-        <f>84*7</f>
-        <v>588</v>
+        <v>30</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G17" s="32">
-        <v>38.116666600000002</v>
+        <v>119.7</v>
       </c>
       <c r="H17" s="32">
         <f>G17*E17</f>
-        <v>22412.599960800002</v>
+        <v>3591</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>774</v>
+        <v>830</v>
       </c>
       <c r="N17" s="36"/>
       <c r="O17" s="35"/>
@@ -14252,25 +14232,27 @@
       <c r="B18" s="20">
         <v>15</v>
       </c>
-      <c r="C18" s="24"/>
+      <c r="C18" s="24" t="s">
+        <v>807</v>
+      </c>
       <c r="D18" s="28" t="s">
-        <v>856</v>
-      </c>
-      <c r="E18" s="24">
-        <v>30</v>
+        <v>828</v>
+      </c>
+      <c r="E18" s="44">
+        <v>390</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>849</v>
+        <v>761</v>
       </c>
       <c r="G18" s="32">
-        <v>24</v>
+        <v>38.116666600000002</v>
       </c>
       <c r="H18" s="32">
         <f>G18*E18</f>
-        <v>720</v>
+        <v>14865.499974</v>
       </c>
       <c r="I18" s="24" t="s">
-        <v>774</v>
+        <v>830</v>
       </c>
       <c r="N18" s="36"/>
       <c r="O18" s="35"/>
@@ -14280,22 +14262,25 @@
       <c r="B19" s="20">
         <v>16</v>
       </c>
-      <c r="C19" s="24"/>
+      <c r="C19" s="17" t="s">
+        <v>807</v>
+      </c>
       <c r="D19" s="28" t="s">
-        <v>857</v>
-      </c>
-      <c r="E19" s="24">
-        <v>1</v>
+        <v>829</v>
+      </c>
+      <c r="E19" s="30">
+        <f>(84*1.02)*2*1.02</f>
+        <v>174.78720000000001</v>
       </c>
       <c r="F19" s="24" t="s">
         <v>760</v>
       </c>
       <c r="G19" s="32">
-        <v>860</v>
+        <v>243.39</v>
       </c>
       <c r="H19" s="32">
         <f>G19*E19</f>
-        <v>860</v>
+        <v>42541.456608</v>
       </c>
       <c r="I19" s="24" t="s">
         <v>774</v>
@@ -14308,7 +14293,7 @@
         <v>0</v>
       </c>
       <c r="P19" s="39">
-        <f t="shared" si="0"/>
+        <f>O19/$O$24</f>
         <v>0</v>
       </c>
     </row>
@@ -14316,22 +14301,27 @@
       <c r="B20" s="20">
         <v>17</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="24" t="s">
         <v>807</v>
       </c>
-      <c r="D20" s="22" t="s">
-        <v>779</v>
-      </c>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21" t="s">
+      <c r="D20" s="28" t="s">
+        <v>828</v>
+      </c>
+      <c r="E20" s="24">
+        <f>84*7</f>
+        <v>588</v>
+      </c>
+      <c r="F20" s="24" t="s">
         <v>761</v>
       </c>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23">
+      <c r="G20" s="32">
+        <v>38.116666600000002</v>
+      </c>
+      <c r="H20" s="32">
         <f>G20*E20</f>
-        <v>0</v>
-      </c>
-      <c r="I20" s="21" t="s">
+        <v>22412.599960800002</v>
+      </c>
+      <c r="I20" s="24" t="s">
         <v>774</v>
       </c>
       <c r="N20" s="36" t="s">
@@ -14342,7 +14332,7 @@
         <v>0</v>
       </c>
       <c r="P20" s="39">
-        <f t="shared" si="0"/>
+        <f>O20/$O$24</f>
         <v>0</v>
       </c>
     </row>
@@ -14350,20 +14340,24 @@
       <c r="B21" s="20">
         <v>18</v>
       </c>
-      <c r="C21" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>780</v>
-      </c>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="23">
+      <c r="C21" s="24"/>
+      <c r="D21" s="28" t="s">
+        <v>856</v>
+      </c>
+      <c r="E21" s="24">
+        <v>30</v>
+      </c>
+      <c r="F21" s="24" t="s">
+        <v>849</v>
+      </c>
+      <c r="G21" s="32">
+        <v>24</v>
+      </c>
+      <c r="H21" s="32">
         <f>G21*E21</f>
-        <v>0</v>
-      </c>
-      <c r="I21" s="21" t="s">
+        <v>720</v>
+      </c>
+      <c r="I21" s="24" t="s">
         <v>774</v>
       </c>
       <c r="N21" s="36"/>
@@ -14374,20 +14368,24 @@
       <c r="B22" s="20">
         <v>19</v>
       </c>
-      <c r="C22" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>781</v>
-      </c>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="23">
+      <c r="C22" s="24"/>
+      <c r="D22" s="28" t="s">
+        <v>857</v>
+      </c>
+      <c r="E22" s="24">
+        <v>1</v>
+      </c>
+      <c r="F22" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G22" s="32">
+        <v>860</v>
+      </c>
+      <c r="H22" s="32">
         <f>G22*E22</f>
-        <v>0</v>
-      </c>
-      <c r="I22" s="21" t="s">
+        <v>860</v>
+      </c>
+      <c r="I22" s="24" t="s">
         <v>774</v>
       </c>
       <c r="N22" s="36"/>
@@ -14402,12 +14400,12 @@
         <v>807</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>816</v>
-      </c>
-      <c r="E23" s="21">
-        <v>1</v>
-      </c>
-      <c r="F23" s="21"/>
+        <v>779</v>
+      </c>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21" t="s">
+        <v>761</v>
+      </c>
       <c r="G23" s="23"/>
       <c r="H23" s="23">
         <f>G23*E23</f>
@@ -14424,31 +14422,25 @@
       <c r="C24" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D24" s="28" t="s">
-        <v>794</v>
-      </c>
-      <c r="E24" s="24">
-        <v>1</v>
-      </c>
-      <c r="F24" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G24" s="29">
-        <v>6000</v>
-      </c>
-      <c r="H24" s="29">
+      <c r="D24" s="22" t="s">
+        <v>780</v>
+      </c>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="23">
         <f>G24*E24</f>
-        <v>6000</v>
-      </c>
-      <c r="I24" s="24" t="s">
-        <v>771</v>
+        <v>0</v>
+      </c>
+      <c r="I24" s="21" t="s">
+        <v>774</v>
       </c>
       <c r="N24" s="36" t="s">
         <v>819</v>
       </c>
       <c r="O24" s="38">
         <f>SUM(O5:O20)</f>
-        <v>3551809.0231375997</v>
+        <v>2822109.0231376002</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -14458,24 +14450,18 @@
       <c r="C25" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D25" s="28" t="s">
-        <v>769</v>
-      </c>
-      <c r="E25" s="24">
-        <v>4100</v>
-      </c>
-      <c r="F25" s="24" t="s">
-        <v>836</v>
-      </c>
-      <c r="G25" s="29">
-        <v>9.65</v>
-      </c>
-      <c r="H25" s="29">
+      <c r="D25" s="22" t="s">
+        <v>781</v>
+      </c>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23">
         <f>G25*E25</f>
-        <v>39565</v>
-      </c>
-      <c r="I25" s="24" t="s">
-        <v>771</v>
+        <v>0</v>
+      </c>
+      <c r="I25" s="21" t="s">
+        <v>774</v>
       </c>
       <c r="J25" s="14" t="s">
         <v>837</v>
@@ -14490,24 +14476,20 @@
       <c r="C26" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D26" s="28" t="s">
-        <v>770</v>
-      </c>
-      <c r="E26" s="24">
-        <v>4000</v>
-      </c>
-      <c r="F26" s="24" t="s">
-        <v>836</v>
-      </c>
-      <c r="G26" s="29">
-        <v>9.65</v>
-      </c>
-      <c r="H26" s="29">
+      <c r="D26" s="22" t="s">
+        <v>816</v>
+      </c>
+      <c r="E26" s="21">
+        <v>1</v>
+      </c>
+      <c r="F26" s="21"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23">
         <f>G26*E26</f>
-        <v>38600</v>
-      </c>
-      <c r="I26" s="24" t="s">
-        <v>771</v>
+        <v>0</v>
+      </c>
+      <c r="I26" s="21" t="s">
+        <v>774</v>
       </c>
       <c r="J26" s="14" t="s">
         <v>837</v>
@@ -14517,11 +14499,11 @@
       <c r="B27" s="20">
         <v>24</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C27" s="17" t="s">
         <v>807</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>827</v>
+        <v>794</v>
       </c>
       <c r="E27" s="24">
         <v>1</v>
@@ -14530,11 +14512,11 @@
         <v>760</v>
       </c>
       <c r="G27" s="29">
-        <v>164000</v>
+        <v>6000</v>
       </c>
       <c r="H27" s="29">
         <f>G27*E27</f>
-        <v>164000</v>
+        <v>6000</v>
       </c>
       <c r="I27" s="24" t="s">
         <v>771</v>
@@ -14548,20 +14530,20 @@
         <v>807</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>864</v>
+        <v>769</v>
       </c>
       <c r="E28" s="24">
-        <v>99.22</v>
+        <v>4100</v>
       </c>
       <c r="F28" s="24" t="s">
-        <v>759</v>
+        <v>836</v>
       </c>
       <c r="G28" s="29">
-        <v>670</v>
+        <v>9.65</v>
       </c>
       <c r="H28" s="29">
         <f>G28*E28</f>
-        <v>66477.399999999994</v>
+        <v>39565</v>
       </c>
       <c r="I28" s="24" t="s">
         <v>771</v>
@@ -14571,22 +14553,24 @@
       <c r="B29" s="20">
         <v>26</v>
       </c>
-      <c r="C29" s="17"/>
+      <c r="C29" s="17" t="s">
+        <v>807</v>
+      </c>
       <c r="D29" s="28" t="s">
-        <v>863</v>
+        <v>770</v>
       </c>
       <c r="E29" s="24">
-        <v>68</v>
+        <v>4000</v>
       </c>
       <c r="F29" s="24" t="s">
-        <v>759</v>
+        <v>836</v>
       </c>
       <c r="G29" s="29">
-        <v>670</v>
+        <v>9.65</v>
       </c>
       <c r="H29" s="29">
         <f>G29*E29</f>
-        <v>45560</v>
+        <v>38600</v>
       </c>
       <c r="I29" s="24" t="s">
         <v>771</v>
@@ -14596,11 +14580,11 @@
       <c r="B30" s="20">
         <v>27</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="24" t="s">
         <v>807</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>833</v>
+        <v>827</v>
       </c>
       <c r="E30" s="24">
         <v>1</v>
@@ -14609,11 +14593,11 @@
         <v>760</v>
       </c>
       <c r="G30" s="29">
-        <v>56500</v>
+        <v>164000</v>
       </c>
       <c r="H30" s="29">
         <f>G30*E30</f>
-        <v>56500</v>
+        <v>164000</v>
       </c>
       <c r="I30" s="24" t="s">
         <v>771</v>
@@ -14626,17 +14610,23 @@
       <c r="C31" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D31" s="19" t="s">
-        <v>777</v>
-      </c>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="18"/>
-      <c r="H31" s="18">
+      <c r="D31" s="28" t="s">
+        <v>865</v>
+      </c>
+      <c r="E31" s="24">
+        <v>99.22</v>
+      </c>
+      <c r="F31" s="24" t="s">
+        <v>759</v>
+      </c>
+      <c r="G31" s="29">
+        <v>670</v>
+      </c>
+      <c r="H31" s="29">
         <f>G31*E31</f>
-        <v>0</v>
-      </c>
-      <c r="I31" s="20" t="s">
+        <v>66477.399999999994</v>
+      </c>
+      <c r="I31" s="24" t="s">
         <v>771</v>
       </c>
     </row>
@@ -14644,21 +14634,25 @@
       <c r="B32" s="20">
         <v>29</v>
       </c>
-      <c r="C32" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D32" s="22" t="s">
-        <v>785</v>
-      </c>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23">
+      <c r="C32" s="17"/>
+      <c r="D32" s="28" t="s">
+        <v>864</v>
+      </c>
+      <c r="E32" s="24">
+        <v>68</v>
+      </c>
+      <c r="F32" s="24" t="s">
+        <v>759</v>
+      </c>
+      <c r="G32" s="29">
+        <v>670</v>
+      </c>
+      <c r="H32" s="29">
         <f>G32*E32</f>
-        <v>0</v>
-      </c>
-      <c r="I32" s="21" t="s">
-        <v>576</v>
+        <v>45560</v>
+      </c>
+      <c r="I32" s="24" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.25">
@@ -14668,18 +14662,24 @@
       <c r="C33" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D33" s="22" t="s">
-        <v>786</v>
-      </c>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="23">
+      <c r="D33" s="28" t="s">
+        <v>833</v>
+      </c>
+      <c r="E33" s="24">
+        <v>1</v>
+      </c>
+      <c r="F33" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G33" s="29">
+        <v>56500</v>
+      </c>
+      <c r="H33" s="29">
         <f>G33*E33</f>
-        <v>0</v>
-      </c>
-      <c r="I33" s="21" t="s">
-        <v>576</v>
+        <v>56500</v>
+      </c>
+      <c r="I33" s="24" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.25">
@@ -14689,18 +14689,18 @@
       <c r="C34" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D34" s="22" t="s">
-        <v>787</v>
-      </c>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="23">
+      <c r="D34" s="19" t="s">
+        <v>777</v>
+      </c>
+      <c r="E34" s="20"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18">
         <f>G34*E34</f>
         <v>0</v>
       </c>
-      <c r="I34" s="21" t="s">
-        <v>576</v>
+      <c r="I34" s="20" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.25">
@@ -14711,7 +14711,7 @@
         <v>807</v>
       </c>
       <c r="D35" s="22" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="E35" s="21"/>
       <c r="F35" s="21"/>
@@ -14728,84 +14728,63 @@
       <c r="B36" s="20">
         <v>33</v>
       </c>
-      <c r="C36" s="24" t="s">
+      <c r="C36" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D36" s="28" t="s">
-        <v>757</v>
-      </c>
-      <c r="E36" s="30">
-        <f>(2150*1.05)*0.15</f>
-        <v>338.625</v>
-      </c>
-      <c r="F36" s="24" t="s">
-        <v>759</v>
-      </c>
-      <c r="G36" s="29">
-        <v>670</v>
-      </c>
-      <c r="H36" s="29">
+      <c r="D36" s="22" t="s">
+        <v>786</v>
+      </c>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23">
         <f>G36*E36</f>
-        <v>226878.75</v>
-      </c>
-      <c r="I36" s="24" t="s">
-        <v>870</v>
+        <v>0</v>
+      </c>
+      <c r="I36" s="21" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B37" s="20">
         <v>34</v>
       </c>
-      <c r="C37" s="24" t="s">
+      <c r="C37" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D37" s="28" t="s">
-        <v>775</v>
-      </c>
-      <c r="E37" s="30">
-        <f>(2150/13)*2</f>
-        <v>330.76923076923077</v>
-      </c>
-      <c r="F37" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G37" s="29">
-        <v>220.5</v>
-      </c>
-      <c r="H37" s="29">
+      <c r="D37" s="22" t="s">
+        <v>787</v>
+      </c>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="23">
         <f>G37*E37</f>
-        <v>72934.61538461539</v>
-      </c>
-      <c r="I37" s="24" t="s">
-        <v>870</v>
+        <v>0</v>
+      </c>
+      <c r="I37" s="21" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B38" s="20">
         <v>35</v>
       </c>
-      <c r="C38" s="24" t="s">
+      <c r="C38" s="17" t="s">
         <v>807</v>
       </c>
-      <c r="D38" s="28" t="s">
-        <v>758</v>
-      </c>
-      <c r="E38" s="24">
-        <f>2100/12</f>
-        <v>175</v>
-      </c>
-      <c r="F38" s="24" t="s">
-        <v>761</v>
-      </c>
-      <c r="G38" s="29">
-        <v>56.2</v>
-      </c>
-      <c r="H38" s="29">
+      <c r="D38" s="22" t="s">
+        <v>788</v>
+      </c>
+      <c r="E38" s="21"/>
+      <c r="F38" s="21"/>
+      <c r="G38" s="23"/>
+      <c r="H38" s="23">
         <f>G38*E38</f>
-        <v>9835</v>
-      </c>
-      <c r="I38" s="24" t="s">
-        <v>870</v>
+        <v>0</v>
+      </c>
+      <c r="I38" s="21" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
@@ -14816,20 +14795,21 @@
         <v>807</v>
       </c>
       <c r="D39" s="28" t="s">
-        <v>762</v>
-      </c>
-      <c r="E39" s="24">
-        <v>1000</v>
+        <v>757</v>
+      </c>
+      <c r="E39" s="30">
+        <f>(2150*1.05)*0.15</f>
+        <v>338.625</v>
       </c>
       <c r="F39" s="24" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="G39" s="29">
-        <v>7.3</v>
+        <v>670</v>
       </c>
       <c r="H39" s="29">
         <f>G39*E39</f>
-        <v>7300</v>
+        <v>226878.75</v>
       </c>
       <c r="I39" s="24" t="s">
         <v>870</v>
@@ -14839,25 +14819,25 @@
       <c r="B40" s="20">
         <v>37</v>
       </c>
-      <c r="C40" s="17" t="s">
+      <c r="C40" s="24" t="s">
         <v>807</v>
       </c>
       <c r="D40" s="28" t="s">
-        <v>811</v>
+        <v>775</v>
       </c>
       <c r="E40" s="30">
-        <f>E36</f>
-        <v>338.625</v>
+        <f>(2150/13)*2</f>
+        <v>330.76923076923077</v>
       </c>
       <c r="F40" s="24" t="s">
-        <v>766</v>
+        <v>760</v>
       </c>
       <c r="G40" s="29">
-        <v>50</v>
+        <v>220.5</v>
       </c>
       <c r="H40" s="29">
         <f>G40*E40</f>
-        <v>16931.25</v>
+        <v>72934.61538461539</v>
       </c>
       <c r="I40" s="24" t="s">
         <v>870</v>
@@ -14867,24 +14847,25 @@
       <c r="B41" s="20">
         <v>38</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="C41" s="24" t="s">
         <v>807</v>
       </c>
       <c r="D41" s="28" t="s">
-        <v>867</v>
+        <v>758</v>
       </c>
       <c r="E41" s="24">
-        <v>1</v>
+        <f>2100/12</f>
+        <v>175</v>
       </c>
       <c r="F41" s="24" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="G41" s="29">
-        <v>53550</v>
+        <v>56.2</v>
       </c>
       <c r="H41" s="29">
         <f>G41*E41</f>
-        <v>53550</v>
+        <v>9835</v>
       </c>
       <c r="I41" s="24" t="s">
         <v>870</v>
@@ -14894,80 +14875,82 @@
       <c r="B42" s="20">
         <v>39</v>
       </c>
-      <c r="C42" s="31" t="s">
-        <v>808</v>
-      </c>
-      <c r="D42" s="43" t="s">
-        <v>815</v>
-      </c>
-      <c r="E42" s="44">
-        <v>110</v>
-      </c>
-      <c r="F42" s="44" t="s">
-        <v>760</v>
-      </c>
-      <c r="G42" s="45">
-        <v>42.29</v>
-      </c>
-      <c r="H42" s="45">
+      <c r="C42" s="24" t="s">
+        <v>807</v>
+      </c>
+      <c r="D42" s="28" t="s">
+        <v>762</v>
+      </c>
+      <c r="E42" s="24">
+        <v>1000</v>
+      </c>
+      <c r="F42" s="24" t="s">
+        <v>763</v>
+      </c>
+      <c r="G42" s="29">
+        <v>7.3</v>
+      </c>
+      <c r="H42" s="29">
         <f>G42*E42</f>
-        <v>4651.8999999999996</v>
-      </c>
-      <c r="I42" s="44" t="s">
-        <v>868</v>
+        <v>7300</v>
+      </c>
+      <c r="I42" s="24" t="s">
+        <v>870</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B43" s="20">
         <v>40</v>
       </c>
-      <c r="C43" s="31"/>
-      <c r="D43" s="43" t="s">
-        <v>869</v>
-      </c>
-      <c r="E43" s="44">
-        <v>1</v>
-      </c>
-      <c r="F43" s="44" t="s">
-        <v>760</v>
-      </c>
-      <c r="G43" s="45">
-        <v>1400</v>
-      </c>
-      <c r="H43" s="45">
+      <c r="C43" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D43" s="28" t="s">
+        <v>811</v>
+      </c>
+      <c r="E43" s="30">
+        <f>E39</f>
+        <v>338.625</v>
+      </c>
+      <c r="F43" s="24" t="s">
+        <v>766</v>
+      </c>
+      <c r="G43" s="29">
+        <v>50</v>
+      </c>
+      <c r="H43" s="29">
         <f>G43*E43</f>
-        <v>1400</v>
-      </c>
-      <c r="I43" s="44" t="s">
-        <v>868</v>
+        <v>16931.25</v>
+      </c>
+      <c r="I43" s="24" t="s">
+        <v>870</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B44" s="20">
         <v>41</v>
       </c>
-      <c r="C44" s="31" t="s">
-        <v>808</v>
-      </c>
-      <c r="D44" s="43" t="s">
-        <v>757</v>
-      </c>
-      <c r="E44" s="50">
-        <f>((1260+960)*0.15)*1.1</f>
-        <v>366.3</v>
-      </c>
-      <c r="F44" s="44" t="s">
-        <v>759</v>
-      </c>
-      <c r="G44" s="45">
-        <v>670</v>
-      </c>
-      <c r="H44" s="45">
+      <c r="C44" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D44" s="28" t="s">
+        <v>860</v>
+      </c>
+      <c r="E44" s="24">
+        <v>1</v>
+      </c>
+      <c r="F44" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G44" s="29">
+        <v>53550</v>
+      </c>
+      <c r="H44" s="29">
         <f>G44*E44</f>
-        <v>245421</v>
-      </c>
-      <c r="I44" s="44" t="s">
-        <v>868</v>
+        <v>53550</v>
+      </c>
+      <c r="I44" s="24" t="s">
+        <v>870</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
@@ -14977,22 +14960,21 @@
       <c r="C45" s="31" t="s">
         <v>808</v>
       </c>
-      <c r="D45" s="28" t="s">
-        <v>775</v>
-      </c>
-      <c r="E45" s="50">
-        <f>(1260+960)/13*1.05</f>
-        <v>179.30769230769232</v>
+      <c r="D45" s="43" t="s">
+        <v>815</v>
+      </c>
+      <c r="E45" s="44">
+        <v>110</v>
       </c>
       <c r="F45" s="44" t="s">
         <v>760</v>
       </c>
       <c r="G45" s="45">
-        <v>220.5</v>
+        <v>42.29</v>
       </c>
       <c r="H45" s="45">
         <f>G45*E45</f>
-        <v>39537.346153846156</v>
+        <v>4651.8999999999996</v>
       </c>
       <c r="I45" s="44" t="s">
         <v>868</v>
@@ -15002,81 +14984,111 @@
       <c r="B46" s="20">
         <v>43</v>
       </c>
-      <c r="C46" s="31" t="s">
+      <c r="C46" s="31"/>
+      <c r="D46" s="43" t="s">
+        <v>869</v>
+      </c>
+      <c r="E46" s="44">
+        <v>1</v>
+      </c>
+      <c r="F46" s="44" t="s">
+        <v>760</v>
+      </c>
+      <c r="G46" s="45">
+        <v>1400</v>
+      </c>
+      <c r="H46" s="45">
+        <f>G46*E46</f>
+        <v>1400</v>
+      </c>
+      <c r="I46" s="44" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B47" s="20">
+        <v>44</v>
+      </c>
+      <c r="C47" s="31" t="s">
         <v>808</v>
       </c>
-      <c r="D46" s="22" t="s">
+      <c r="D47" s="43" t="s">
+        <v>757</v>
+      </c>
+      <c r="E47" s="50">
+        <f>((1260+960)*0.15)*1.1</f>
+        <v>366.3</v>
+      </c>
+      <c r="F47" s="44" t="s">
+        <v>759</v>
+      </c>
+      <c r="G47" s="45">
+        <v>670</v>
+      </c>
+      <c r="H47" s="45">
+        <f>G47*E47</f>
+        <v>245421</v>
+      </c>
+      <c r="I47" s="44" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B48" s="20">
+        <v>45</v>
+      </c>
+      <c r="C48" s="31" t="s">
+        <v>808</v>
+      </c>
+      <c r="D48" s="28" t="s">
+        <v>775</v>
+      </c>
+      <c r="E48" s="50">
+        <f>(1260+960)/13*1.05</f>
+        <v>179.30769230769232</v>
+      </c>
+      <c r="F48" s="44" t="s">
+        <v>760</v>
+      </c>
+      <c r="G48" s="45">
+        <v>220.5</v>
+      </c>
+      <c r="H48" s="45">
+        <f>G48*E48</f>
+        <v>39537.346153846156</v>
+      </c>
+      <c r="I48" s="44" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B49" s="20">
+        <v>46</v>
+      </c>
+      <c r="C49" s="31" t="s">
+        <v>808</v>
+      </c>
+      <c r="D49" s="22" t="s">
         <v>871</v>
       </c>
-      <c r="E46" s="21">
-        <v>1</v>
-      </c>
-      <c r="F46" s="21" t="s">
+      <c r="E49" s="21">
+        <v>1</v>
+      </c>
+      <c r="F49" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="G46" s="49"/>
-      <c r="H46" s="49">
-        <f>G46*E46</f>
-        <v>0</v>
-      </c>
-      <c r="I46" s="21" t="s">
-        <v>868</v>
-      </c>
-    </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="20"/>
-      <c r="C47" s="31"/>
-      <c r="D47" s="22" t="s">
-        <v>757</v>
-      </c>
-      <c r="E47" s="21"/>
-      <c r="F47" s="21"/>
-      <c r="G47" s="49"/>
-      <c r="H47" s="49">
-        <f>G47*E47</f>
-        <v>0</v>
-      </c>
-      <c r="I47" s="21" t="s">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B48" s="20"/>
-      <c r="C48" s="31"/>
-      <c r="D48" s="19" t="s">
-        <v>775</v>
-      </c>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
-      <c r="G48" s="49"/>
-      <c r="H48" s="49">
-        <f>G48*E48</f>
-        <v>0</v>
-      </c>
-      <c r="I48" s="21" t="s">
-        <v>872</v>
-      </c>
-    </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B49" s="20"/>
-      <c r="C49" s="31"/>
-      <c r="D49" s="19" t="s">
-        <v>758</v>
-      </c>
-      <c r="E49" s="21"/>
-      <c r="F49" s="21"/>
       <c r="G49" s="49"/>
       <c r="H49" s="49">
         <f>G49*E49</f>
         <v>0</v>
       </c>
       <c r="I49" s="21" t="s">
-        <v>872</v>
+        <v>868</v>
       </c>
     </row>
     <row r="50" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B50" s="20">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C50" s="17" t="s">
         <v>807</v>
@@ -15103,7 +15115,7 @@
     </row>
     <row r="51" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B51" s="20">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C51" s="17" t="s">
         <v>807</v>
@@ -15124,7 +15136,7 @@
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B52" s="20">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C52" s="17" t="s">
         <v>807</v>
@@ -15151,7 +15163,7 @@
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B53" s="20">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C53" s="17" t="s">
         <v>808</v>
@@ -15173,12 +15185,12 @@
         <v>46600</v>
       </c>
       <c r="I53" s="44" t="s">
-        <v>804</v>
+        <v>874</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B54" s="20">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C54" s="17" t="s">
         <v>808</v>
@@ -15200,12 +15212,12 @@
         <v>8100</v>
       </c>
       <c r="I54" s="44" t="s">
-        <v>804</v>
+        <v>874</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B55" s="20">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C55" s="17" t="s">
         <v>808</v>
@@ -15227,12 +15239,12 @@
         <v>5000</v>
       </c>
       <c r="I55" s="44" t="s">
-        <v>804</v>
+        <v>874</v>
       </c>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B56" s="20">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C56" s="17" t="s">
         <v>808</v>
@@ -15254,12 +15266,12 @@
         <v>670000</v>
       </c>
       <c r="I56" s="44" t="s">
-        <v>804</v>
+        <v>874</v>
       </c>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" s="20">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C57" s="17" t="s">
         <v>807</v>
@@ -15280,7 +15292,7 @@
     </row>
     <row r="58" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B58" s="20">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="19" t="s">
@@ -15299,7 +15311,7 @@
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B59" s="20">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C59" s="17" t="s">
         <v>807</v>
@@ -15320,7 +15332,7 @@
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B60" s="20">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C60" s="17" t="s">
         <v>807</v>
@@ -15347,11 +15359,11 @@
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B61" s="20">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C61" s="17"/>
       <c r="D61" s="22" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="E61" s="21"/>
       <c r="F61" s="21"/>
@@ -15360,15 +15372,17 @@
         <f>G61*E61</f>
         <v>0</v>
       </c>
-      <c r="I61" s="21"/>
+      <c r="I61" s="21" t="s">
+        <v>873</v>
+      </c>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B62" s="20">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C62" s="17"/>
       <c r="D62" s="22" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="E62" s="21"/>
       <c r="F62" s="21"/>
@@ -15377,15 +15391,17 @@
         <f>G62*E62</f>
         <v>0</v>
       </c>
-      <c r="I62" s="21"/>
+      <c r="I62" s="21" t="s">
+        <v>873</v>
+      </c>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" s="20">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C63" s="17"/>
       <c r="D63" s="22" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="E63" s="21"/>
       <c r="F63" s="21"/>
@@ -15394,15 +15410,17 @@
         <f>G63*E63</f>
         <v>0</v>
       </c>
-      <c r="I63" s="21"/>
+      <c r="I63" s="21" t="s">
+        <v>873</v>
+      </c>
     </row>
     <row r="64" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B64" s="20">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C64" s="17"/>
       <c r="D64" s="19" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="E64" s="20"/>
       <c r="F64" s="20"/>
@@ -15411,11 +15429,13 @@
         <f>G64*E64</f>
         <v>0</v>
       </c>
-      <c r="I64" s="20"/>
+      <c r="I64" s="21" t="s">
+        <v>873</v>
+      </c>
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" s="20">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C65" s="31"/>
       <c r="D65" s="22" t="s">
@@ -15428,7 +15448,9 @@
         <f>G65*E65</f>
         <v>0</v>
       </c>
-      <c r="I65" s="21"/>
+      <c r="I65" s="21" t="s">
+        <v>873</v>
+      </c>
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B66" s="21"/>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:18
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2167" uniqueCount="875">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2170" uniqueCount="875">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2610,9 +2610,6 @@
     <t>Mão de obra para concretagem do piso do galpão 2100m²</t>
   </si>
   <si>
-    <t>Mão de obra para concretagem do piso das docas de carregamento DPA IV (interno)</t>
-  </si>
-  <si>
     <t>Concreto para o radier do sistema de tratamento de esgoto do banheiro</t>
   </si>
   <si>
@@ -2650,6 +2647,9 @@
   </si>
   <si>
     <t>Serviço Preliminar</t>
+  </si>
+  <si>
+    <t>Mão de obra para concretagem do piso das docas de carregamento (1075m²)</t>
   </si>
 </sst>
 </file>
@@ -13702,7 +13702,7 @@
     <col min="2" max="2" width="9.140625" style="14"/>
     <col min="3" max="3" width="20" style="14" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="87" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="14" customWidth="1"/>
+    <col min="5" max="5" width="16" style="14" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" style="14" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" style="15" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" style="15" bestFit="1" customWidth="1"/>
@@ -13952,7 +13952,7 @@
       </c>
       <c r="C9" s="31"/>
       <c r="D9" s="22" t="s">
-        <v>861</v>
+        <v>874</v>
       </c>
       <c r="E9" s="21">
         <v>1</v>
@@ -13966,7 +13966,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="17" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="N9" s="37" t="s">
         <v>771</v>
@@ -13985,18 +13985,25 @@
         <v>7</v>
       </c>
       <c r="C10" s="31"/>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="43" t="s">
         <v>757</v>
       </c>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="49"/>
-      <c r="H10" s="49">
+      <c r="E10" s="50">
+        <f>(1075*0.15)*1.1</f>
+        <v>177.37500000000003</v>
+      </c>
+      <c r="F10" s="44" t="s">
+        <v>759</v>
+      </c>
+      <c r="G10" s="45">
+        <v>670</v>
+      </c>
+      <c r="H10" s="45">
         <f>G10*E10</f>
-        <v>0</v>
-      </c>
-      <c r="I10" s="21" t="s">
-        <v>872</v>
+        <v>118841.25000000001</v>
+      </c>
+      <c r="I10" s="44" t="s">
+        <v>871</v>
       </c>
       <c r="N10" s="37" t="s">
         <v>774</v>
@@ -14015,18 +14022,25 @@
         <v>8</v>
       </c>
       <c r="C11" s="31"/>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="28" t="s">
         <v>775</v>
       </c>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="49"/>
-      <c r="H11" s="49">
+      <c r="E11" s="50">
+        <f>1075/13*2</f>
+        <v>165.38461538461539</v>
+      </c>
+      <c r="F11" s="44" t="s">
+        <v>760</v>
+      </c>
+      <c r="G11" s="45">
+        <v>220.5</v>
+      </c>
+      <c r="H11" s="45">
         <f>G11*E11</f>
-        <v>0</v>
-      </c>
-      <c r="I11" s="21" t="s">
-        <v>872</v>
+        <v>36467.307692307695</v>
+      </c>
+      <c r="I11" s="44" t="s">
+        <v>871</v>
       </c>
       <c r="N11" s="36" t="s">
         <v>782</v>
@@ -14045,18 +14059,25 @@
         <v>9</v>
       </c>
       <c r="C12" s="31"/>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="28" t="s">
         <v>758</v>
       </c>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="49"/>
-      <c r="H12" s="49">
+      <c r="E12" s="50">
+        <f>(20*53)/12</f>
+        <v>88.333333333333329</v>
+      </c>
+      <c r="F12" s="44" t="s">
+        <v>760</v>
+      </c>
+      <c r="G12" s="45">
+        <v>56.2</v>
+      </c>
+      <c r="H12" s="45">
         <f>G12*E12</f>
-        <v>0</v>
-      </c>
-      <c r="I12" s="21" t="s">
-        <v>872</v>
+        <v>4964.333333333333</v>
+      </c>
+      <c r="I12" s="44" t="s">
+        <v>871</v>
       </c>
       <c r="N12" s="36" t="s">
         <v>449</v>
@@ -14611,7 +14632,7 @@
         <v>807</v>
       </c>
       <c r="D31" s="28" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="E31" s="24">
         <v>99.22</v>
@@ -14636,7 +14657,7 @@
       </c>
       <c r="C32" s="17"/>
       <c r="D32" s="28" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="E32" s="24">
         <v>68</v>
@@ -14812,7 +14833,7 @@
         <v>226878.75</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.25">
@@ -14840,7 +14861,7 @@
         <v>72934.61538461539</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.25">
@@ -14858,7 +14879,7 @@
         <v>175</v>
       </c>
       <c r="F41" s="24" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G41" s="29">
         <v>56.2</v>
@@ -14868,7 +14889,7 @@
         <v>9835</v>
       </c>
       <c r="I41" s="24" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.25">
@@ -14895,7 +14916,7 @@
         <v>7300</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.25">
@@ -14923,7 +14944,7 @@
         <v>16931.25</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.25">
@@ -14950,7 +14971,7 @@
         <v>53550</v>
       </c>
       <c r="I44" s="24" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
@@ -14977,7 +14998,7 @@
         <v>4651.8999999999996</v>
       </c>
       <c r="I45" s="44" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
@@ -14986,7 +15007,7 @@
       </c>
       <c r="C46" s="31"/>
       <c r="D46" s="43" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="E46" s="44">
         <v>1</v>
@@ -15002,7 +15023,7 @@
         <v>1400</v>
       </c>
       <c r="I46" s="44" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
@@ -15030,7 +15051,7 @@
         <v>245421</v>
       </c>
       <c r="I47" s="44" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.25">
@@ -15058,7 +15079,7 @@
         <v>39537.346153846156</v>
       </c>
       <c r="I48" s="44" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.25">
@@ -15069,7 +15090,7 @@
         <v>808</v>
       </c>
       <c r="D49" s="22" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="E49" s="21">
         <v>1</v>
@@ -15083,7 +15104,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="21" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="50" spans="2:9" x14ac:dyDescent="0.25">
@@ -15185,7 +15206,7 @@
         <v>46600</v>
       </c>
       <c r="I53" s="44" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.25">
@@ -15212,7 +15233,7 @@
         <v>8100</v>
       </c>
       <c r="I54" s="44" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
@@ -15239,7 +15260,7 @@
         <v>5000</v>
       </c>
       <c r="I55" s="44" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.25">
@@ -15266,7 +15287,7 @@
         <v>670000</v>
       </c>
       <c r="I56" s="44" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.25">
@@ -15363,7 +15384,7 @@
       </c>
       <c r="C61" s="17"/>
       <c r="D61" s="22" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E61" s="21"/>
       <c r="F61" s="21"/>
@@ -15373,7 +15394,7 @@
         <v>0</v>
       </c>
       <c r="I61" s="21" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.25">
@@ -15382,7 +15403,7 @@
       </c>
       <c r="C62" s="17"/>
       <c r="D62" s="22" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="E62" s="21"/>
       <c r="F62" s="21"/>
@@ -15392,7 +15413,7 @@
         <v>0</v>
       </c>
       <c r="I62" s="21" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
@@ -15401,7 +15422,7 @@
       </c>
       <c r="C63" s="17"/>
       <c r="D63" s="22" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="E63" s="21"/>
       <c r="F63" s="21"/>
@@ -15411,7 +15432,7 @@
         <v>0</v>
       </c>
       <c r="I63" s="21" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="64" spans="2:9" x14ac:dyDescent="0.25">
@@ -15420,7 +15441,7 @@
       </c>
       <c r="C64" s="17"/>
       <c r="D64" s="19" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="E64" s="20"/>
       <c r="F64" s="20"/>
@@ -15430,7 +15451,7 @@
         <v>0</v>
       </c>
       <c r="I64" s="21" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
@@ -15449,7 +15470,7 @@
         <v>0</v>
       </c>
       <c r="I65" s="21" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.25">
@@ -15476,7 +15497,7 @@
       <c r="D68" s="34"/>
       <c r="H68" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>4195314.3880812619</v>
+        <v>4355587.2791069029</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:19
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2170" uniqueCount="875">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2168" uniqueCount="876">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2650,6 +2650,9 @@
   </si>
   <si>
     <t>Mão de obra para concretagem do piso das docas de carregamento (1075m²)</t>
+  </si>
+  <si>
+    <t>Mão de obra para montagem e cobertura da frente das docas de carregamento</t>
   </si>
 </sst>
 </file>
@@ -14472,7 +14475,7 @@
         <v>807</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>781</v>
+        <v>875</v>
       </c>
       <c r="E25" s="21"/>
       <c r="F25" s="21"/>
@@ -14482,11 +14485,9 @@
         <v>0</v>
       </c>
       <c r="I25" s="21" t="s">
-        <v>774</v>
-      </c>
-      <c r="J25" s="14" t="s">
-        <v>837</v>
-      </c>
+        <v>871</v>
+      </c>
+      <c r="J25" s="14"/>
       <c r="N25" s="36"/>
       <c r="O25" s="38"/>
     </row>
@@ -14512,9 +14513,7 @@
       <c r="I26" s="21" t="s">
         <v>774</v>
       </c>
-      <c r="J26" s="14" t="s">
-        <v>837</v>
-      </c>
+      <c r="J26" s="14"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B27" s="20">

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:21
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2168" uniqueCount="876">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2172" uniqueCount="876">
   <si>
     <t>Código EAP</t>
   </si>
@@ -14450,7 +14450,9 @@
         <v>780</v>
       </c>
       <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
+      <c r="F24" s="21" t="s">
+        <v>761</v>
+      </c>
       <c r="G24" s="23"/>
       <c r="H24" s="23">
         <f>G24*E24</f>
@@ -14478,7 +14480,9 @@
         <v>875</v>
       </c>
       <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
+      <c r="F25" s="21" t="s">
+        <v>760</v>
+      </c>
       <c r="G25" s="23"/>
       <c r="H25" s="23">
         <f>G25*E25</f>
@@ -14504,7 +14508,9 @@
       <c r="E26" s="21">
         <v>1</v>
       </c>
-      <c r="F26" s="21"/>
+      <c r="F26" s="21" t="s">
+        <v>760</v>
+      </c>
       <c r="G26" s="23"/>
       <c r="H26" s="23">
         <f>G26*E26</f>
@@ -14713,7 +14719,9 @@
         <v>777</v>
       </c>
       <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
+      <c r="F34" s="20" t="s">
+        <v>760</v>
+      </c>
       <c r="G34" s="18"/>
       <c r="H34" s="18">
         <f>G34*E34</f>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:34
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2172" uniqueCount="876">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2178" uniqueCount="879">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2403,9 +2403,6 @@
     <t>SPDA do galpão completo</t>
   </si>
   <si>
-    <t>Telha Trapeizodal TP40 Fechamento Telhado</t>
-  </si>
-  <si>
     <t>Estrutura drive-in</t>
   </si>
   <si>
@@ -2577,9 +2574,6 @@
     <t>cx</t>
   </si>
   <si>
-    <t>Cumeeira TP40</t>
-  </si>
-  <si>
     <t>Projeto de combate ao incêndio - material, execução e aprovação</t>
   </si>
   <si>
@@ -2653,6 +2647,21 @@
   </si>
   <si>
     <t>Mão de obra para montagem e cobertura da frente das docas de carregamento</t>
+  </si>
+  <si>
+    <t>Parafuso de fixação telha/terça 4700 peças</t>
+  </si>
+  <si>
+    <t>Parafuso de costura telha/telha 3200 peças</t>
+  </si>
+  <si>
+    <t>cumeeiras tp40 0.50mm largura util 980mm galvalume</t>
+  </si>
+  <si>
+    <t>telha tp40 0.50mm comp 7300mm largura util 980mm galvalume</t>
+  </si>
+  <si>
+    <t>telhas tp40 0.50mm comp 5600mm largura util 980mm galvalume</t>
   </si>
 </sst>
 </file>
@@ -2760,7 +2769,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2895,6 +2904,9 @@
     </xf>
     <xf numFmtId="1" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3192,8 +3204,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I65" totalsRowShown="0" headerRowDxfId="0" dataDxfId="17">
-  <autoFilter ref="B3:I65"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I68" totalsRowShown="0" headerRowDxfId="0" dataDxfId="17">
+  <autoFilter ref="B3:I68"/>
   <sortState ref="B4:I66">
     <sortCondition ref="I3:I66"/>
   </sortState>
@@ -12675,7 +12687,7 @@
         <v>767</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
     </row>
     <row r="4" spans="2:10" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -12712,7 +12724,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="D5" s="20">
         <v>3</v>
@@ -12760,7 +12772,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="D7" s="20"/>
       <c r="E7" s="20"/>
@@ -12836,7 +12848,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="D10" s="24">
         <v>1</v>
@@ -12852,7 +12864,7 @@
         <v>1056959.67</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="J10" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Terraplanagem",Tabela2[Preço Total])</f>
@@ -12864,7 +12876,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
@@ -12874,7 +12886,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="21" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="J11" s="35">
         <f>SUMIF(Tabela2[Aplicação],"Drenagem",Tabela2[Preço Total])</f>
@@ -12886,7 +12898,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="D12" s="20"/>
       <c r="E12" s="20"/>
@@ -12908,7 +12920,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="D13" s="20"/>
       <c r="E13" s="20"/>
@@ -12993,7 +13005,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="D17" s="21"/>
       <c r="E17" s="21"/>
@@ -13011,7 +13023,7 @@
         <v>15</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="D18" s="26">
         <v>4</v>
@@ -13035,7 +13047,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="D19" s="24">
         <v>1</v>
@@ -13065,7 +13077,7 @@
         <v>2100</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="F20" s="29">
         <v>9.65</v>
@@ -13078,7 +13090,7 @@
         <v>771</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
@@ -13092,7 +13104,7 @@
         <v>2300</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="F21" s="29">
         <v>9.65</v>
@@ -13105,7 +13117,7 @@
         <v>771</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
@@ -13113,7 +13125,7 @@
         <v>19</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="D22" s="24">
         <v>1</v>
@@ -13137,7 +13149,7 @@
         <v>20</v>
       </c>
       <c r="C23" s="28" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D23" s="30">
         <v>46.8</v>
@@ -13161,7 +13173,7 @@
         <v>21</v>
       </c>
       <c r="C24" s="28" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D24" s="30">
         <v>37.200000000000003</v>
@@ -13331,7 +13343,7 @@
         <v>167</v>
       </c>
       <c r="E32" s="24" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="F32" s="29">
         <v>56.2</v>
@@ -13373,7 +13385,7 @@
         <v>31</v>
       </c>
       <c r="C34" s="28" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="D34" s="24">
         <v>315</v>
@@ -13421,7 +13433,7 @@
         <v>33</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="D36" s="21">
         <v>1</v>
@@ -13435,7 +13447,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="21" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
@@ -13443,7 +13455,7 @@
         <v>34</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="D37" s="21">
         <v>1</v>
@@ -13457,7 +13469,7 @@
         <v>0</v>
       </c>
       <c r="H37" s="21" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
@@ -13483,7 +13495,7 @@
         <v>36</v>
       </c>
       <c r="C39" s="42" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D39" s="24">
         <v>1455.89</v>
@@ -13499,7 +13511,7 @@
         <v>139619.85100000002</v>
       </c>
       <c r="H39" s="24" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
@@ -13507,7 +13519,7 @@
         <v>37</v>
       </c>
       <c r="C40" s="28" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="D40" s="24">
         <v>706.94</v>
@@ -13523,7 +13535,7 @@
         <v>67795.546000000002</v>
       </c>
       <c r="H40" s="24" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
@@ -13531,13 +13543,13 @@
         <v>38</v>
       </c>
       <c r="C41" s="25" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="D41" s="24">
         <v>44</v>
       </c>
       <c r="E41" s="24" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="F41" s="32">
         <v>95</v>
@@ -13547,7 +13559,7 @@
         <v>4180</v>
       </c>
       <c r="H41" s="24" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
@@ -13555,13 +13567,13 @@
         <v>39</v>
       </c>
       <c r="C42" s="25" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="D42" s="24">
         <v>3</v>
       </c>
       <c r="E42" s="24" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="F42" s="32">
         <v>35</v>
@@ -13571,7 +13583,7 @@
         <v>105</v>
       </c>
       <c r="H42" s="24" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
@@ -13579,7 +13591,7 @@
         <v>40</v>
       </c>
       <c r="C43" s="25" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="D43" s="24">
         <v>126</v>
@@ -13595,7 +13607,7 @@
         <v>3263.3999999999996</v>
       </c>
       <c r="H43" s="24" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
@@ -13603,7 +13615,7 @@
         <v>41</v>
       </c>
       <c r="C44" s="25" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="D44" s="24">
         <v>1</v>
@@ -13619,7 +13631,7 @@
         <v>1750</v>
       </c>
       <c r="H44" s="24" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
@@ -13651,7 +13663,7 @@
         <v>43</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D46" s="21"/>
       <c r="E46" s="21"/>
@@ -13661,7 +13673,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="21" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
@@ -13699,7 +13711,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R68"/>
+  <dimension ref="B1:R71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -13721,12 +13733,12 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P1" s="14" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="P2" s="14" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="3" spans="2:18" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -13734,7 +13746,7 @@
         <v>753</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>754</v>
@@ -13755,7 +13767,7 @@
         <v>767</v>
       </c>
       <c r="P3" s="14" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
@@ -13763,10 +13775,10 @@
         <v>1</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="E4" s="21">
         <v>1</v>
@@ -13780,19 +13792,19 @@
         <v>0</v>
       </c>
       <c r="I4" s="21" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="O4" s="14" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="P4" s="14" t="s">
+        <v>819</v>
+      </c>
+      <c r="Q4" s="14" t="s">
         <v>820</v>
       </c>
-      <c r="Q4" s="14" t="s">
+      <c r="R4" s="14" t="s">
         <v>821</v>
-      </c>
-      <c r="R4" s="14" t="s">
-        <v>822</v>
       </c>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
@@ -13800,10 +13812,10 @@
         <v>2</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="E5" s="24">
         <v>1</v>
@@ -13837,7 +13849,7 @@
         <v>0.35168875187413606</v>
       </c>
       <c r="R5" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.25">
@@ -13846,7 +13858,7 @@
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="19" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="E6" s="20">
         <v>4</v>
@@ -13878,7 +13890,7 @@
         <v>0.63225640659914406</v>
       </c>
       <c r="R6" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.25">
@@ -13887,7 +13899,7 @@
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="19" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="E7" s="20">
         <v>6</v>
@@ -13921,7 +13933,7 @@
       </c>
       <c r="C8" s="31"/>
       <c r="D8" s="22" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="E8" s="21">
         <v>6</v>
@@ -13938,7 +13950,7 @@
         <v>253</v>
       </c>
       <c r="N8" s="40" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="O8" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Prévio",Tabela24[Preço Total])</f>
@@ -13955,7 +13967,7 @@
       </c>
       <c r="C9" s="31"/>
       <c r="D9" s="22" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="E9" s="21">
         <v>1</v>
@@ -13969,7 +13981,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="17" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="N9" s="37" t="s">
         <v>771</v>
@@ -14006,7 +14018,7 @@
         <v>118841.25000000001</v>
       </c>
       <c r="I10" s="44" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="N10" s="37" t="s">
         <v>774</v>
@@ -14043,7 +14055,7 @@
         <v>36467.307692307695</v>
       </c>
       <c r="I11" s="44" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="N11" s="36" t="s">
         <v>782</v>
@@ -14080,7 +14092,7 @@
         <v>4964.333333333333</v>
       </c>
       <c r="I12" s="44" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="N12" s="36" t="s">
         <v>449</v>
@@ -14099,7 +14111,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D13" s="22" t="s">
         <v>789</v>
@@ -14127,7 +14139,7 @@
         <v>11</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D14" s="43" t="s">
         <v>790</v>
@@ -14165,10 +14177,10 @@
         <v>12</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="E15" s="21"/>
       <c r="F15" s="21"/>
@@ -14197,10 +14209,10 @@
         <v>13</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="E16" s="24">
         <v>54</v>
@@ -14216,7 +14228,7 @@
         <v>13143.06</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="N16" s="36"/>
       <c r="O16" s="35"/>
@@ -14227,10 +14239,10 @@
         <v>14</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="E17" s="24">
         <v>30</v>
@@ -14246,7 +14258,7 @@
         <v>3591</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="N17" s="36"/>
       <c r="O17" s="35"/>
@@ -14257,10 +14269,10 @@
         <v>15</v>
       </c>
       <c r="C18" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="E18" s="44">
         <v>390</v>
@@ -14276,7 +14288,7 @@
         <v>14865.499974</v>
       </c>
       <c r="I18" s="24" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="N18" s="36"/>
       <c r="O18" s="35"/>
@@ -14287,10 +14299,10 @@
         <v>16</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D19" s="28" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="E19" s="30">
         <f>(84*1.02)*2*1.02</f>
@@ -14326,10 +14338,10 @@
         <v>17</v>
       </c>
       <c r="C20" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="E20" s="24">
         <f>84*7</f>
@@ -14349,7 +14361,7 @@
         <v>774</v>
       </c>
       <c r="N20" s="36" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="O20" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
@@ -14366,13 +14378,13 @@
       </c>
       <c r="C21" s="24"/>
       <c r="D21" s="28" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="E21" s="24">
         <v>30</v>
       </c>
       <c r="F21" s="24" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="G21" s="32">
         <v>24</v>
@@ -14394,7 +14406,7 @@
       </c>
       <c r="C22" s="24"/>
       <c r="D22" s="28" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="E22" s="24">
         <v>1</v>
@@ -14421,7 +14433,7 @@
         <v>20</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D23" s="22" t="s">
         <v>779</v>
@@ -14444,7 +14456,7 @@
         <v>21</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D24" s="22" t="s">
         <v>780</v>
@@ -14462,7 +14474,7 @@
         <v>774</v>
       </c>
       <c r="N24" s="36" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="O24" s="38">
         <f>SUM(O5:O20)</f>
@@ -14474,10 +14486,10 @@
         <v>22</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="E25" s="21"/>
       <c r="F25" s="21" t="s">
@@ -14489,7 +14501,7 @@
         <v>0</v>
       </c>
       <c r="I25" s="21" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="J25" s="14"/>
       <c r="N25" s="36"/>
@@ -14500,10 +14512,10 @@
         <v>23</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D26" s="22" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="E26" s="21">
         <v>1</v>
@@ -14526,10 +14538,10 @@
         <v>24</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E27" s="24">
         <v>1</v>
@@ -14553,7 +14565,7 @@
         <v>25</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D28" s="28" t="s">
         <v>769</v>
@@ -14562,7 +14574,7 @@
         <v>4100</v>
       </c>
       <c r="F28" s="24" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="G28" s="29">
         <v>9.65</v>
@@ -14580,7 +14592,7 @@
         <v>26</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D29" s="28" t="s">
         <v>770</v>
@@ -14589,7 +14601,7 @@
         <v>4000</v>
       </c>
       <c r="F29" s="24" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="G29" s="29">
         <v>9.65</v>
@@ -14607,10 +14619,10 @@
         <v>27</v>
       </c>
       <c r="C30" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="E30" s="24">
         <v>1</v>
@@ -14634,10 +14646,10 @@
         <v>28</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D31" s="28" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="E31" s="24">
         <v>99.22</v>
@@ -14662,7 +14674,7 @@
       </c>
       <c r="C32" s="17"/>
       <c r="D32" s="28" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="E32" s="24">
         <v>68</v>
@@ -14686,10 +14698,10 @@
         <v>30</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D33" s="28" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="E33" s="24">
         <v>1</v>
@@ -14713,7 +14725,7 @@
         <v>31</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D34" s="19" t="s">
         <v>777</v>
@@ -14736,7 +14748,7 @@
         <v>32</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D35" s="22" t="s">
         <v>785</v>
@@ -14757,7 +14769,7 @@
         <v>33</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D36" s="22" t="s">
         <v>786</v>
@@ -14778,7 +14790,7 @@
         <v>34</v>
       </c>
       <c r="C37" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D37" s="22" t="s">
         <v>787</v>
@@ -14799,7 +14811,7 @@
         <v>35</v>
       </c>
       <c r="C38" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D38" s="22" t="s">
         <v>788</v>
@@ -14820,7 +14832,7 @@
         <v>36</v>
       </c>
       <c r="C39" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D39" s="28" t="s">
         <v>757</v>
@@ -14840,7 +14852,7 @@
         <v>226878.75</v>
       </c>
       <c r="I39" s="24" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.25">
@@ -14848,7 +14860,7 @@
         <v>37</v>
       </c>
       <c r="C40" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D40" s="28" t="s">
         <v>775</v>
@@ -14868,7 +14880,7 @@
         <v>72934.61538461539</v>
       </c>
       <c r="I40" s="24" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.25">
@@ -14876,7 +14888,7 @@
         <v>38</v>
       </c>
       <c r="C41" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D41" s="28" t="s">
         <v>758</v>
@@ -14896,7 +14908,7 @@
         <v>9835</v>
       </c>
       <c r="I41" s="24" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.25">
@@ -14904,7 +14916,7 @@
         <v>39</v>
       </c>
       <c r="C42" s="24" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D42" s="28" t="s">
         <v>762</v>
@@ -14923,7 +14935,7 @@
         <v>7300</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.25">
@@ -14931,10 +14943,10 @@
         <v>40</v>
       </c>
       <c r="C43" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D43" s="28" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="E43" s="30">
         <f>E39</f>
@@ -14951,7 +14963,7 @@
         <v>16931.25</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.25">
@@ -14959,10 +14971,10 @@
         <v>41</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D44" s="28" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="E44" s="24">
         <v>1</v>
@@ -14978,7 +14990,7 @@
         <v>53550</v>
       </c>
       <c r="I44" s="24" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
@@ -14986,10 +14998,10 @@
         <v>42</v>
       </c>
       <c r="C45" s="31" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D45" s="43" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E45" s="44">
         <v>110</v>
@@ -15005,7 +15017,7 @@
         <v>4651.8999999999996</v>
       </c>
       <c r="I45" s="44" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
@@ -15014,7 +15026,7 @@
       </c>
       <c r="C46" s="31"/>
       <c r="D46" s="43" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="E46" s="44">
         <v>1</v>
@@ -15030,7 +15042,7 @@
         <v>1400</v>
       </c>
       <c r="I46" s="44" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
@@ -15038,7 +15050,7 @@
         <v>44</v>
       </c>
       <c r="C47" s="31" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D47" s="43" t="s">
         <v>757</v>
@@ -15058,7 +15070,7 @@
         <v>245421</v>
       </c>
       <c r="I47" s="44" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.25">
@@ -15066,7 +15078,7 @@
         <v>45</v>
       </c>
       <c r="C48" s="31" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D48" s="28" t="s">
         <v>775</v>
@@ -15086,7 +15098,7 @@
         <v>39537.346153846156</v>
       </c>
       <c r="I48" s="44" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.25">
@@ -15094,10 +15106,10 @@
         <v>46</v>
       </c>
       <c r="C49" s="31" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D49" s="22" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="E49" s="21">
         <v>1</v>
@@ -15111,7 +15123,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="21" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
     </row>
     <row r="50" spans="2:9" x14ac:dyDescent="0.25">
@@ -15119,10 +15131,10 @@
         <v>47</v>
       </c>
       <c r="C50" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D50" s="28" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="E50" s="24">
         <v>1</v>
@@ -15146,10 +15158,10 @@
         <v>48</v>
       </c>
       <c r="C51" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D51" s="19" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E51" s="20"/>
       <c r="F51" s="20"/>
@@ -15167,7 +15179,7 @@
         <v>49</v>
       </c>
       <c r="C52" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D52" s="28" t="s">
         <v>773</v>
@@ -15194,10 +15206,10 @@
         <v>50</v>
       </c>
       <c r="C53" s="17" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D53" s="43" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="E53" s="44">
         <v>1</v>
@@ -15213,7 +15225,7 @@
         <v>46600</v>
       </c>
       <c r="I53" s="44" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.25">
@@ -15221,10 +15233,10 @@
         <v>51</v>
       </c>
       <c r="C54" s="17" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D54" s="43" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="E54" s="44">
         <v>1</v>
@@ -15240,7 +15252,7 @@
         <v>8100</v>
       </c>
       <c r="I54" s="44" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
@@ -15248,10 +15260,10 @@
         <v>52</v>
       </c>
       <c r="C55" s="17" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="D55" s="43" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="E55" s="44">
         <v>1</v>
@@ -15267,7 +15279,7 @@
         <v>5000</v>
       </c>
       <c r="I55" s="44" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.25">
@@ -15275,10 +15287,10 @@
         <v>53</v>
       </c>
       <c r="C56" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D56" s="43" t="s">
         <v>808</v>
-      </c>
-      <c r="D56" s="43" t="s">
-        <v>809</v>
       </c>
       <c r="E56" s="44">
         <v>1</v>
@@ -15294,7 +15306,7 @@
         <v>670000</v>
       </c>
       <c r="I56" s="44" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.25">
@@ -15302,7 +15314,7 @@
         <v>54</v>
       </c>
       <c r="C57" s="17" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="D57" s="19" t="s">
         <v>791</v>
@@ -15324,185 +15336,240 @@
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="19" t="s">
-        <v>850</v>
-      </c>
-      <c r="E58" s="20"/>
-      <c r="F58" s="20"/>
+        <v>876</v>
+      </c>
+      <c r="E58" s="20">
+        <v>87</v>
+      </c>
+      <c r="F58" s="20" t="s">
+        <v>760</v>
+      </c>
       <c r="G58" s="18"/>
       <c r="H58" s="18">
         <f>G58*E58</f>
         <v>0</v>
       </c>
       <c r="I58" s="20" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B59" s="20">
-        <v>56</v>
-      </c>
-      <c r="C59" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D59" s="19" t="s">
-        <v>792</v>
-      </c>
-      <c r="E59" s="20"/>
-      <c r="F59" s="20"/>
+      <c r="B59" s="20"/>
+      <c r="C59" s="17"/>
+      <c r="D59" s="51" t="s">
+        <v>877</v>
+      </c>
+      <c r="E59" s="20">
+        <v>174</v>
+      </c>
+      <c r="F59" s="20" t="s">
+        <v>760</v>
+      </c>
       <c r="G59" s="18"/>
       <c r="H59" s="18">
         <f>G59*E59</f>
         <v>0</v>
       </c>
-      <c r="I59" s="17" t="s">
-        <v>799</v>
+      <c r="I59" s="20" t="s">
+        <v>798</v>
       </c>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B60" s="20">
-        <v>57</v>
-      </c>
-      <c r="C60" s="17" t="s">
-        <v>807</v>
-      </c>
+      <c r="B60" s="20"/>
+      <c r="C60" s="17"/>
       <c r="D60" s="19" t="s">
-        <v>784</v>
+        <v>878</v>
       </c>
       <c r="E60" s="20">
-        <v>1</v>
+        <v>174</v>
       </c>
       <c r="F60" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="G60" s="18">
-        <v>791792.51</v>
-      </c>
+      <c r="G60" s="18"/>
       <c r="H60" s="18">
         <f>G60*E60</f>
-        <v>791792.51</v>
+        <v>0</v>
       </c>
       <c r="I60" s="20" t="s">
-        <v>783</v>
+        <v>798</v>
       </c>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B61" s="20">
-        <v>58</v>
-      </c>
+      <c r="B61" s="20"/>
       <c r="C61" s="17"/>
-      <c r="D61" s="22" t="s">
-        <v>861</v>
-      </c>
-      <c r="E61" s="21"/>
-      <c r="F61" s="21"/>
-      <c r="G61" s="49"/>
-      <c r="H61" s="49">
+      <c r="D61" s="51" t="s">
+        <v>874</v>
+      </c>
+      <c r="E61" s="20"/>
+      <c r="F61" s="20"/>
+      <c r="G61" s="18"/>
+      <c r="H61" s="18">
         <f>G61*E61</f>
         <v>0</v>
       </c>
-      <c r="I61" s="21" t="s">
-        <v>872</v>
-      </c>
+      <c r="I61" s="20"/>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B62" s="20">
-        <v>59</v>
-      </c>
+      <c r="B62" s="20"/>
       <c r="C62" s="17"/>
-      <c r="D62" s="22" t="s">
-        <v>862</v>
-      </c>
-      <c r="E62" s="21"/>
-      <c r="F62" s="21"/>
-      <c r="G62" s="49"/>
-      <c r="H62" s="49">
+      <c r="D62" s="19" t="s">
+        <v>875</v>
+      </c>
+      <c r="E62" s="20"/>
+      <c r="F62" s="20"/>
+      <c r="G62" s="18"/>
+      <c r="H62" s="18">
         <f>G62*E62</f>
         <v>0</v>
       </c>
-      <c r="I62" s="21" t="s">
-        <v>872</v>
-      </c>
+      <c r="I62" s="20"/>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" s="20">
-        <v>60</v>
-      </c>
-      <c r="C63" s="17"/>
-      <c r="D63" s="22" t="s">
-        <v>865</v>
-      </c>
-      <c r="E63" s="21"/>
-      <c r="F63" s="21"/>
-      <c r="G63" s="49"/>
-      <c r="H63" s="49">
+        <v>57</v>
+      </c>
+      <c r="C63" s="17" t="s">
+        <v>806</v>
+      </c>
+      <c r="D63" s="19" t="s">
+        <v>784</v>
+      </c>
+      <c r="E63" s="20">
+        <v>1</v>
+      </c>
+      <c r="F63" s="20" t="s">
+        <v>760</v>
+      </c>
+      <c r="G63" s="18">
+        <v>791792.51</v>
+      </c>
+      <c r="H63" s="18">
         <f>G63*E63</f>
-        <v>0</v>
-      </c>
-      <c r="I63" s="21" t="s">
-        <v>872</v>
+        <v>791792.51</v>
+      </c>
+      <c r="I63" s="20" t="s">
+        <v>783</v>
       </c>
     </row>
     <row r="64" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B64" s="20">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C64" s="17"/>
-      <c r="D64" s="19" t="s">
-        <v>866</v>
-      </c>
-      <c r="E64" s="20"/>
-      <c r="F64" s="20"/>
-      <c r="G64" s="18"/>
-      <c r="H64" s="18">
+      <c r="D64" s="22" t="s">
+        <v>859</v>
+      </c>
+      <c r="E64" s="21"/>
+      <c r="F64" s="21"/>
+      <c r="G64" s="49"/>
+      <c r="H64" s="49">
         <f>G64*E64</f>
         <v>0</v>
       </c>
       <c r="I64" s="21" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" s="20">
-        <v>62</v>
-      </c>
-      <c r="C65" s="31"/>
+        <v>59</v>
+      </c>
+      <c r="C65" s="17"/>
       <c r="D65" s="22" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="E65" s="21"/>
       <c r="F65" s="21"/>
-      <c r="G65" s="23"/>
-      <c r="H65" s="47">
+      <c r="G65" s="49"/>
+      <c r="H65" s="49">
         <f>G65*E65</f>
         <v>0</v>
       </c>
       <c r="I65" s="21" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B66" s="21"/>
-      <c r="C66" s="31"/>
-      <c r="D66" s="22"/>
+      <c r="B66" s="20">
+        <v>60</v>
+      </c>
+      <c r="C66" s="17"/>
+      <c r="D66" s="22" t="s">
+        <v>863</v>
+      </c>
       <c r="E66" s="21"/>
       <c r="F66" s="21"/>
-      <c r="G66" s="23"/>
-      <c r="H66" s="47"/>
-      <c r="I66" s="21"/>
+      <c r="G66" s="49"/>
+      <c r="H66" s="49">
+        <f>G66*E66</f>
+        <v>0</v>
+      </c>
+      <c r="I66" s="21" t="s">
+        <v>870</v>
+      </c>
     </row>
     <row r="67" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B67" s="21"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="22"/>
-      <c r="E67" s="21"/>
-      <c r="F67" s="21"/>
-      <c r="G67" s="23"/>
-      <c r="H67" s="47"/>
-      <c r="I67" s="21"/>
+      <c r="B67" s="20">
+        <v>61</v>
+      </c>
+      <c r="C67" s="17"/>
+      <c r="D67" s="19" t="s">
+        <v>864</v>
+      </c>
+      <c r="E67" s="20"/>
+      <c r="F67" s="20"/>
+      <c r="G67" s="18"/>
+      <c r="H67" s="18">
+        <f>G67*E67</f>
+        <v>0</v>
+      </c>
+      <c r="I67" s="21" t="s">
+        <v>870</v>
+      </c>
     </row>
     <row r="68" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D68" s="34"/>
-      <c r="H68" s="16">
+      <c r="B68" s="20">
+        <v>62</v>
+      </c>
+      <c r="C68" s="31"/>
+      <c r="D68" s="22" t="s">
+        <v>857</v>
+      </c>
+      <c r="E68" s="21"/>
+      <c r="F68" s="21"/>
+      <c r="G68" s="23"/>
+      <c r="H68" s="47">
+        <f>G68*E68</f>
+        <v>0</v>
+      </c>
+      <c r="I68" s="21" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="69" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B69" s="21"/>
+      <c r="C69" s="31"/>
+      <c r="D69" s="22"/>
+      <c r="E69" s="21"/>
+      <c r="F69" s="21"/>
+      <c r="G69" s="23"/>
+      <c r="H69" s="47"/>
+      <c r="I69" s="21"/>
+    </row>
+    <row r="70" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B70" s="21"/>
+      <c r="C70" s="31"/>
+      <c r="D70" s="22"/>
+      <c r="E70" s="21"/>
+      <c r="F70" s="21"/>
+      <c r="G70" s="23"/>
+      <c r="H70" s="47"/>
+      <c r="I70" s="21"/>
+    </row>
+    <row r="71" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D71" s="34"/>
+      <c r="H71" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
         <v>4355587.2791069029</v>
       </c>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:36
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2178" uniqueCount="879">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2180" uniqueCount="879">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2649,12 +2649,6 @@
     <t>Mão de obra para montagem e cobertura da frente das docas de carregamento</t>
   </si>
   <si>
-    <t>Parafuso de fixação telha/terça 4700 peças</t>
-  </si>
-  <si>
-    <t>Parafuso de costura telha/telha 3200 peças</t>
-  </si>
-  <si>
     <t>cumeeiras tp40 0.50mm largura util 980mm galvalume</t>
   </si>
   <si>
@@ -2662,6 +2656,12 @@
   </si>
   <si>
     <t>telhas tp40 0.50mm comp 5600mm largura util 980mm galvalume</t>
+  </si>
+  <si>
+    <t>Parafuso de fixação telha/terça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parafuso de costura telha/telha </t>
   </si>
 </sst>
 </file>
@@ -15336,7 +15336,7 @@
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="19" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="E58" s="20">
         <v>87</v>
@@ -15344,20 +15344,24 @@
       <c r="F58" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="G58" s="18"/>
+      <c r="G58" s="18">
+        <v>34.99</v>
+      </c>
       <c r="H58" s="18">
         <f>G58*E58</f>
-        <v>0</v>
+        <v>3044.13</v>
       </c>
       <c r="I58" s="20" t="s">
         <v>798</v>
       </c>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B59" s="20"/>
+      <c r="B59" s="20">
+        <v>56</v>
+      </c>
       <c r="C59" s="17"/>
       <c r="D59" s="51" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="E59" s="20">
         <v>174</v>
@@ -15365,20 +15369,24 @@
       <c r="F59" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="G59" s="18"/>
+      <c r="G59" s="18">
+        <v>255.5</v>
+      </c>
       <c r="H59" s="18">
         <f>G59*E59</f>
-        <v>0</v>
+        <v>44457</v>
       </c>
       <c r="I59" s="20" t="s">
         <v>798</v>
       </c>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B60" s="20"/>
+      <c r="B60" s="20">
+        <v>57</v>
+      </c>
       <c r="C60" s="17"/>
       <c r="D60" s="19" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="E60" s="20">
         <v>174</v>
@@ -15386,23 +15394,31 @@
       <c r="F60" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="G60" s="18"/>
+      <c r="G60" s="18">
+        <v>196</v>
+      </c>
       <c r="H60" s="18">
         <f>G60*E60</f>
-        <v>0</v>
+        <v>34104</v>
       </c>
       <c r="I60" s="20" t="s">
         <v>798</v>
       </c>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B61" s="20"/>
+      <c r="B61" s="20">
+        <v>58</v>
+      </c>
       <c r="C61" s="17"/>
       <c r="D61" s="51" t="s">
-        <v>874</v>
-      </c>
-      <c r="E61" s="20"/>
-      <c r="F61" s="20"/>
+        <v>877</v>
+      </c>
+      <c r="E61" s="20">
+        <v>4700</v>
+      </c>
+      <c r="F61" s="20" t="s">
+        <v>760</v>
+      </c>
       <c r="G61" s="18"/>
       <c r="H61" s="18">
         <f>G61*E61</f>
@@ -15411,13 +15427,19 @@
       <c r="I61" s="20"/>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B62" s="20"/>
+      <c r="B62" s="20">
+        <v>59</v>
+      </c>
       <c r="C62" s="17"/>
       <c r="D62" s="19" t="s">
-        <v>875</v>
-      </c>
-      <c r="E62" s="20"/>
-      <c r="F62" s="20"/>
+        <v>878</v>
+      </c>
+      <c r="E62" s="20">
+        <v>3200</v>
+      </c>
+      <c r="F62" s="20" t="s">
+        <v>760</v>
+      </c>
       <c r="G62" s="18"/>
       <c r="H62" s="18">
         <f>G62*E62</f>
@@ -15427,7 +15449,7 @@
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" s="20">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C63" s="17" t="s">
         <v>806</v>
@@ -15454,7 +15476,7 @@
     </row>
     <row r="64" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B64" s="20">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C64" s="17"/>
       <c r="D64" s="22" t="s">
@@ -15473,7 +15495,7 @@
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" s="20">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C65" s="17"/>
       <c r="D65" s="22" t="s">
@@ -15492,7 +15514,7 @@
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B66" s="20">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C66" s="17"/>
       <c r="D66" s="22" t="s">
@@ -15511,7 +15533,7 @@
     </row>
     <row r="67" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B67" s="20">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C67" s="17"/>
       <c r="D67" s="19" t="s">
@@ -15530,7 +15552,7 @@
     </row>
     <row r="68" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B68" s="20">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C68" s="31"/>
       <c r="D68" s="22" t="s">
@@ -15571,7 +15593,7 @@
       <c r="D71" s="34"/>
       <c r="H71" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>4355587.2791069029</v>
+        <v>4437192.4091069028</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:39
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2180" uniqueCount="879">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2182" uniqueCount="879">
   <si>
     <t>Código EAP</t>
   </si>
@@ -15419,12 +15419,16 @@
       <c r="F61" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="G61" s="18"/>
+      <c r="G61" s="18">
+        <v>0.5</v>
+      </c>
       <c r="H61" s="18">
         <f>G61*E61</f>
-        <v>0</v>
-      </c>
-      <c r="I61" s="20"/>
+        <v>2350</v>
+      </c>
+      <c r="I61" s="20" t="s">
+        <v>798</v>
+      </c>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B62" s="20">
@@ -15440,12 +15444,16 @@
       <c r="F62" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="G62" s="18"/>
+      <c r="G62" s="18">
+        <v>0.5</v>
+      </c>
       <c r="H62" s="18">
         <f>G62*E62</f>
-        <v>0</v>
-      </c>
-      <c r="I62" s="20"/>
+        <v>1600</v>
+      </c>
+      <c r="I62" s="20" t="s">
+        <v>798</v>
+      </c>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" s="20">
@@ -15593,7 +15601,7 @@
       <c r="D71" s="34"/>
       <c r="H71" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>4437192.4091069028</v>
+        <v>4441142.4091069028</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:40
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -2769,7 +2769,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2904,9 +2904,6 @@
     </xf>
     <xf numFmtId="1" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -15335,23 +15332,23 @@
         <v>55</v>
       </c>
       <c r="C58" s="17"/>
-      <c r="D58" s="19" t="s">
+      <c r="D58" s="28" t="s">
         <v>874</v>
       </c>
-      <c r="E58" s="20">
+      <c r="E58" s="24">
         <v>87</v>
       </c>
-      <c r="F58" s="20" t="s">
+      <c r="F58" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G58" s="18">
+      <c r="G58" s="32">
         <v>34.99</v>
       </c>
-      <c r="H58" s="18">
+      <c r="H58" s="32">
         <f>G58*E58</f>
         <v>3044.13</v>
       </c>
-      <c r="I58" s="20" t="s">
+      <c r="I58" s="24" t="s">
         <v>798</v>
       </c>
     </row>
@@ -15360,23 +15357,23 @@
         <v>56</v>
       </c>
       <c r="C59" s="17"/>
-      <c r="D59" s="51" t="s">
+      <c r="D59" s="42" t="s">
         <v>875</v>
       </c>
-      <c r="E59" s="20">
+      <c r="E59" s="24">
         <v>174</v>
       </c>
-      <c r="F59" s="20" t="s">
+      <c r="F59" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G59" s="18">
+      <c r="G59" s="32">
         <v>255.5</v>
       </c>
-      <c r="H59" s="18">
+      <c r="H59" s="32">
         <f>G59*E59</f>
         <v>44457</v>
       </c>
-      <c r="I59" s="20" t="s">
+      <c r="I59" s="24" t="s">
         <v>798</v>
       </c>
     </row>
@@ -15385,23 +15382,23 @@
         <v>57</v>
       </c>
       <c r="C60" s="17"/>
-      <c r="D60" s="19" t="s">
+      <c r="D60" s="28" t="s">
         <v>876</v>
       </c>
-      <c r="E60" s="20">
+      <c r="E60" s="24">
         <v>174</v>
       </c>
-      <c r="F60" s="20" t="s">
+      <c r="F60" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G60" s="18">
+      <c r="G60" s="32">
         <v>196</v>
       </c>
-      <c r="H60" s="18">
+      <c r="H60" s="32">
         <f>G60*E60</f>
         <v>34104</v>
       </c>
-      <c r="I60" s="20" t="s">
+      <c r="I60" s="24" t="s">
         <v>798</v>
       </c>
     </row>
@@ -15410,23 +15407,23 @@
         <v>58</v>
       </c>
       <c r="C61" s="17"/>
-      <c r="D61" s="51" t="s">
+      <c r="D61" s="42" t="s">
         <v>877</v>
       </c>
-      <c r="E61" s="20">
+      <c r="E61" s="24">
         <v>4700</v>
       </c>
-      <c r="F61" s="20" t="s">
+      <c r="F61" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G61" s="18">
+      <c r="G61" s="32">
         <v>0.5</v>
       </c>
-      <c r="H61" s="18">
+      <c r="H61" s="32">
         <f>G61*E61</f>
         <v>2350</v>
       </c>
-      <c r="I61" s="20" t="s">
+      <c r="I61" s="24" t="s">
         <v>798</v>
       </c>
     </row>
@@ -15435,23 +15432,23 @@
         <v>59</v>
       </c>
       <c r="C62" s="17"/>
-      <c r="D62" s="19" t="s">
+      <c r="D62" s="28" t="s">
         <v>878</v>
       </c>
-      <c r="E62" s="20">
+      <c r="E62" s="24">
         <v>3200</v>
       </c>
-      <c r="F62" s="20" t="s">
+      <c r="F62" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G62" s="18">
+      <c r="G62" s="32">
         <v>0.5</v>
       </c>
-      <c r="H62" s="18">
+      <c r="H62" s="32">
         <f>G62*E62</f>
         <v>1600</v>
       </c>
-      <c r="I62" s="20" t="s">
+      <c r="I62" s="24" t="s">
         <v>798</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:41
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -14227,9 +14227,17 @@
       <c r="I16" s="24" t="s">
         <v>829</v>
       </c>
-      <c r="N16" s="36"/>
-      <c r="O16" s="35"/>
-      <c r="P16" s="39"/>
+      <c r="N16" s="36" t="s">
+        <v>576</v>
+      </c>
+      <c r="O16" s="35">
+        <f>SUMIF(Tabela24[Aplicação],"Pintura",Tabela24[Preço Total])</f>
+        <v>0</v>
+      </c>
+      <c r="P16" s="39">
+        <f>O16/$O$24</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" s="20">
@@ -14257,9 +14265,17 @@
       <c r="I17" s="24" t="s">
         <v>829</v>
       </c>
-      <c r="N17" s="36"/>
-      <c r="O17" s="35"/>
-      <c r="P17" s="39"/>
+      <c r="N17" s="36" t="s">
+        <v>812</v>
+      </c>
+      <c r="O17" s="35">
+        <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
+        <v>0</v>
+      </c>
+      <c r="P17" s="39">
+        <f>O17/$O$24</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" s="20">
@@ -14318,17 +14334,6 @@
       <c r="I19" s="24" t="s">
         <v>774</v>
       </c>
-      <c r="N19" s="36" t="s">
-        <v>576</v>
-      </c>
-      <c r="O19" s="35">
-        <f>SUMIF(Tabela24[Aplicação],"Pintura",Tabela24[Preço Total])</f>
-        <v>0</v>
-      </c>
-      <c r="P19" s="39">
-        <f>O19/$O$24</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="20">
@@ -14356,17 +14361,6 @@
       </c>
       <c r="I20" s="24" t="s">
         <v>774</v>
-      </c>
-      <c r="N20" s="36" t="s">
-        <v>812</v>
-      </c>
-      <c r="O20" s="35">
-        <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
-        <v>0</v>
-      </c>
-      <c r="P20" s="39">
-        <f>O20/$O$24</f>
-        <v>0</v>
       </c>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.25">
@@ -14474,7 +14468,7 @@
         <v>818</v>
       </c>
       <c r="O24" s="38">
-        <f>SUM(O5:O20)</f>
+        <f>SUM(O5:O18)</f>
         <v>2822109.0231376002</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza planilha 09/10/2026 16:52
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2182" uniqueCount="879">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2186" uniqueCount="881">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2662,6 +2662,12 @@
   </si>
   <si>
     <t xml:space="preserve">Parafuso de costura telha/telha </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sondagem SPT após realização do aterro </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Necessário por desencargo de consciência </t>
   </si>
 </sst>
 </file>
@@ -2769,7 +2775,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2905,6 +2911,12 @@
     <xf numFmtId="1" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -2913,6 +2925,105 @@
   </cellStyles>
   <dxfs count="18">
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2937,20 +3048,18 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
+        <color rgb="FF404040"/>
         <name val="Calibri"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
       </font>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -3069,103 +3178,6 @@
         <scheme val="minor"/>
       </font>
     </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.249977111117893"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF404040"/>
-        <name val="Calibri"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3180,43 +3192,43 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H46" totalsRowShown="0" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H46" totalsRowShown="0" dataDxfId="17">
   <autoFilter ref="B3:H46"/>
   <sortState ref="B4:H46">
     <sortCondition ref="H3:H46"/>
   </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" name="Item" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="2" name="Descrição" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="9" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="8" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="7" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="6" dataCellStyle="Moeda">
+    <tableColumn id="1" name="Item" dataDxfId="10" dataCellStyle="Normal"/>
+    <tableColumn id="2" name="Descrição" dataDxfId="11" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="16" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="15" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="14" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="13" dataCellStyle="Moeda">
       <calculatedColumnFormula>F4*D4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="12" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I68" totalsRowShown="0" headerRowDxfId="0" dataDxfId="17">
-  <autoFilter ref="B3:I68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B3:I69" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="B3:I69"/>
   <sortState ref="B4:I66">
     <sortCondition ref="I3:I66"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" name="Item" dataDxfId="1" dataCellStyle="Normal"/>
-    <tableColumn id="8" name="Local" dataDxfId="2"/>
-    <tableColumn id="2" name="Descrição" dataDxfId="16" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="15" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="14" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="13" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="12" dataCellStyle="Moeda">
+    <tableColumn id="1" name="Item" dataDxfId="7" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Local" dataDxfId="6"/>
+    <tableColumn id="2" name="Descrição" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="2" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="1" dataCellStyle="Moeda">
       <calculatedColumnFormula>G4*E4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="11" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="0" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12647,7 +12659,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:J49"/>
+  <dimension ref="B3:J75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -13697,6 +13709,12 @@
         <v>2376630.5208461536</v>
       </c>
     </row>
+    <row r="75" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H75" s="52">
+        <f>SUM('Expansão DMP'!G49,H71)</f>
+        <v>2376630.5208461536</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -13708,7 +13726,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:R71"/>
+  <dimension ref="B1:R76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="14"/>
@@ -13839,11 +13857,11 @@
       </c>
       <c r="P5" s="39">
         <f>O5/$O$24</f>
-        <v>0.35168875187413606</v>
+        <v>0.35094262345617866</v>
       </c>
       <c r="Q5" s="41">
         <f>P5</f>
-        <v>0.35168875187413606</v>
+        <v>0.35094262345617866</v>
       </c>
       <c r="R5" t="s">
         <v>822</v>
@@ -13880,11 +13898,11 @@
       </c>
       <c r="P6" s="39">
         <f>O6/$O$24</f>
-        <v>0.28056765472500805</v>
+        <v>0.27997241390699945</v>
       </c>
       <c r="Q6" s="41">
         <f>P6+Q5</f>
-        <v>0.63225640659914406</v>
+        <v>0.63091503736317811</v>
       </c>
       <c r="R6" t="s">
         <v>822</v>
@@ -13985,11 +14003,11 @@
       </c>
       <c r="O9" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Fundação",Tabela24[Preço Total])</f>
-        <v>416702.4</v>
+        <v>422702.4</v>
       </c>
       <c r="P9" s="39">
         <f>O9/$O$24</f>
-        <v>0.14765637917726981</v>
+        <v>0.14946467641160441</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
@@ -14026,7 +14044,7 @@
       </c>
       <c r="P10" s="39">
         <f t="shared" ref="P10:P12" si="0">O10/$O$24</f>
-        <v>2.3576005045626455E-2</v>
+        <v>2.3525987161196801E-2</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
@@ -14063,7 +14081,7 @@
       </c>
       <c r="P11" s="39">
         <f t="shared" si="0"/>
-        <v>0.17222297084030905</v>
+        <v>0.17185758965571263</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
@@ -14166,7 +14184,7 @@
       </c>
       <c r="P14" s="39">
         <f>O14/$O$24</f>
-        <v>2.3576005045626455E-2</v>
+        <v>2.3525987161196801E-2</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
@@ -14198,7 +14216,7 @@
       </c>
       <c r="P15" s="39">
         <f>O15/$O$24</f>
-        <v>7.1223329202402556E-4</v>
+        <v>7.1072224711126505E-4</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
@@ -14469,7 +14487,7 @@
       </c>
       <c r="O24" s="38">
         <f>SUM(O5:O18)</f>
-        <v>2822109.0231376002</v>
+        <v>2828109.0231376002</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -14684,7 +14702,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B33" s="20">
         <v>30</v>
       </c>
@@ -14711,7 +14729,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B34" s="20">
         <v>31</v>
       </c>
@@ -14734,36 +14752,41 @@
         <v>771</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B35" s="20">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B35" s="20"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="19" t="s">
+        <v>879</v>
+      </c>
+      <c r="E35" s="20">
+        <v>4</v>
+      </c>
+      <c r="F35" s="20" t="s">
+        <v>760</v>
+      </c>
+      <c r="G35" s="18">
+        <v>1500</v>
+      </c>
+      <c r="H35" s="18">
+        <f>G35*E35</f>
+        <v>6000</v>
+      </c>
+      <c r="I35" s="20" t="s">
+        <v>771</v>
+      </c>
+      <c r="J35" s="48" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B36" s="20">
         <v>32</v>
-      </c>
-      <c r="C35" s="17" t="s">
-        <v>806</v>
-      </c>
-      <c r="D35" s="22" t="s">
-        <v>785</v>
-      </c>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
-      <c r="G35" s="23"/>
-      <c r="H35" s="23">
-        <f>G35*E35</f>
-        <v>0</v>
-      </c>
-      <c r="I35" s="21" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B36" s="20">
-        <v>33</v>
       </c>
       <c r="C36" s="17" t="s">
         <v>806</v>
       </c>
       <c r="D36" s="22" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="E36" s="21"/>
       <c r="F36" s="21"/>
@@ -14776,15 +14799,15 @@
         <v>576</v>
       </c>
     </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="20">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C37" s="17" t="s">
         <v>806</v>
       </c>
       <c r="D37" s="22" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="E37" s="21"/>
       <c r="F37" s="21"/>
@@ -14797,15 +14820,15 @@
         <v>576</v>
       </c>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="20">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C38" s="17" t="s">
         <v>806</v>
       </c>
       <c r="D38" s="22" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="E38" s="21"/>
       <c r="F38" s="21"/>
@@ -14818,416 +14841,410 @@
         <v>576</v>
       </c>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B39" s="20">
+        <v>35</v>
+      </c>
+      <c r="C39" s="17" t="s">
+        <v>806</v>
+      </c>
+      <c r="D39" s="22" t="s">
+        <v>788</v>
+      </c>
+      <c r="E39" s="21"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="23">
+        <f>G39*E39</f>
+        <v>0</v>
+      </c>
+      <c r="I39" s="21" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B40" s="20">
         <v>36</v>
       </c>
-      <c r="C39" s="24" t="s">
+      <c r="C40" s="24" t="s">
         <v>806</v>
       </c>
-      <c r="D39" s="28" t="s">
+      <c r="D40" s="28" t="s">
         <v>757</v>
       </c>
-      <c r="E39" s="30">
+      <c r="E40" s="30">
         <f>(2150*1.05)*0.15</f>
         <v>338.625</v>
       </c>
-      <c r="F39" s="24" t="s">
+      <c r="F40" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="G39" s="29">
+      <c r="G40" s="29">
         <v>670</v>
       </c>
-      <c r="H39" s="29">
-        <f>G39*E39</f>
+      <c r="H40" s="29">
+        <f>G40*E40</f>
         <v>226878.75</v>
       </c>
-      <c r="I39" s="24" t="s">
+      <c r="I40" s="24" t="s">
         <v>867</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B40" s="20">
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B41" s="20">
         <v>37</v>
       </c>
-      <c r="C40" s="24" t="s">
+      <c r="C41" s="24" t="s">
         <v>806</v>
       </c>
-      <c r="D40" s="28" t="s">
+      <c r="D41" s="28" t="s">
         <v>775</v>
       </c>
-      <c r="E40" s="30">
+      <c r="E41" s="30">
         <f>(2150/13)*2</f>
         <v>330.76923076923077</v>
       </c>
-      <c r="F40" s="24" t="s">
+      <c r="F41" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G40" s="29">
+      <c r="G41" s="29">
         <v>220.5</v>
       </c>
-      <c r="H40" s="29">
-        <f>G40*E40</f>
+      <c r="H41" s="29">
+        <f>G41*E41</f>
         <v>72934.61538461539</v>
       </c>
-      <c r="I40" s="24" t="s">
+      <c r="I41" s="24" t="s">
         <v>867</v>
       </c>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="20">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B42" s="20">
         <v>38</v>
       </c>
-      <c r="C41" s="24" t="s">
+      <c r="C42" s="24" t="s">
         <v>806</v>
       </c>
-      <c r="D41" s="28" t="s">
+      <c r="D42" s="28" t="s">
         <v>758</v>
       </c>
-      <c r="E41" s="24">
+      <c r="E42" s="24">
         <f>2100/12</f>
         <v>175</v>
       </c>
-      <c r="F41" s="24" t="s">
+      <c r="F42" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G41" s="29">
+      <c r="G42" s="29">
         <v>56.2</v>
-      </c>
-      <c r="H41" s="29">
-        <f>G41*E41</f>
-        <v>9835</v>
-      </c>
-      <c r="I41" s="24" t="s">
-        <v>867</v>
-      </c>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B42" s="20">
-        <v>39</v>
-      </c>
-      <c r="C42" s="24" t="s">
-        <v>806</v>
-      </c>
-      <c r="D42" s="28" t="s">
-        <v>762</v>
-      </c>
-      <c r="E42" s="24">
-        <v>1000</v>
-      </c>
-      <c r="F42" s="24" t="s">
-        <v>763</v>
-      </c>
-      <c r="G42" s="29">
-        <v>7.3</v>
       </c>
       <c r="H42" s="29">
         <f>G42*E42</f>
-        <v>7300</v>
+        <v>9835</v>
       </c>
       <c r="I42" s="24" t="s">
         <v>867</v>
       </c>
     </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B43" s="20">
-        <v>40</v>
-      </c>
-      <c r="C43" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C43" s="24" t="s">
         <v>806</v>
       </c>
       <c r="D43" s="28" t="s">
-        <v>810</v>
-      </c>
-      <c r="E43" s="30">
-        <f>E39</f>
-        <v>338.625</v>
+        <v>762</v>
+      </c>
+      <c r="E43" s="24">
+        <v>1000</v>
       </c>
       <c r="F43" s="24" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="G43" s="29">
-        <v>50</v>
+        <v>7.3</v>
       </c>
       <c r="H43" s="29">
         <f>G43*E43</f>
-        <v>16931.25</v>
+        <v>7300</v>
       </c>
       <c r="I43" s="24" t="s">
         <v>867</v>
       </c>
     </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B44" s="20">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C44" s="17" t="s">
         <v>806</v>
       </c>
       <c r="D44" s="28" t="s">
-        <v>858</v>
-      </c>
-      <c r="E44" s="24">
-        <v>1</v>
+        <v>810</v>
+      </c>
+      <c r="E44" s="30">
+        <f>E40</f>
+        <v>338.625</v>
       </c>
       <c r="F44" s="24" t="s">
-        <v>760</v>
+        <v>766</v>
       </c>
       <c r="G44" s="29">
-        <v>53550</v>
+        <v>50</v>
       </c>
       <c r="H44" s="29">
         <f>G44*E44</f>
-        <v>53550</v>
+        <v>16931.25</v>
       </c>
       <c r="I44" s="24" t="s">
         <v>867</v>
       </c>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B45" s="20">
+        <v>41</v>
+      </c>
+      <c r="C45" s="17" t="s">
+        <v>806</v>
+      </c>
+      <c r="D45" s="28" t="s">
+        <v>858</v>
+      </c>
+      <c r="E45" s="24">
+        <v>1</v>
+      </c>
+      <c r="F45" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G45" s="29">
+        <v>53550</v>
+      </c>
+      <c r="H45" s="29">
+        <f>G45*E45</f>
+        <v>53550</v>
+      </c>
+      <c r="I45" s="24" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B46" s="20">
         <v>42</v>
       </c>
-      <c r="C45" s="31" t="s">
+      <c r="C46" s="31" t="s">
         <v>807</v>
       </c>
-      <c r="D45" s="43" t="s">
+      <c r="D46" s="43" t="s">
         <v>814</v>
       </c>
-      <c r="E45" s="44">
+      <c r="E46" s="44">
         <v>110</v>
-      </c>
-      <c r="F45" s="44" t="s">
-        <v>760</v>
-      </c>
-      <c r="G45" s="45">
-        <v>42.29</v>
-      </c>
-      <c r="H45" s="45">
-        <f>G45*E45</f>
-        <v>4651.8999999999996</v>
-      </c>
-      <c r="I45" s="44" t="s">
-        <v>865</v>
-      </c>
-    </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B46" s="20">
-        <v>43</v>
-      </c>
-      <c r="C46" s="31"/>
-      <c r="D46" s="43" t="s">
-        <v>866</v>
-      </c>
-      <c r="E46" s="44">
-        <v>1</v>
       </c>
       <c r="F46" s="44" t="s">
         <v>760</v>
       </c>
       <c r="G46" s="45">
-        <v>1400</v>
+        <v>42.29</v>
       </c>
       <c r="H46" s="45">
         <f>G46*E46</f>
-        <v>1400</v>
+        <v>4651.8999999999996</v>
       </c>
       <c r="I46" s="44" t="s">
         <v>865</v>
       </c>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B47" s="20">
+        <v>43</v>
+      </c>
+      <c r="C47" s="31"/>
+      <c r="D47" s="43" t="s">
+        <v>866</v>
+      </c>
+      <c r="E47" s="44">
+        <v>1</v>
+      </c>
+      <c r="F47" s="44" t="s">
+        <v>760</v>
+      </c>
+      <c r="G47" s="45">
+        <v>1400</v>
+      </c>
+      <c r="H47" s="45">
+        <f>G47*E47</f>
+        <v>1400</v>
+      </c>
+      <c r="I47" s="44" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B48" s="20">
         <v>44</v>
       </c>
-      <c r="C47" s="31" t="s">
+      <c r="C48" s="31" t="s">
         <v>807</v>
       </c>
-      <c r="D47" s="43" t="s">
+      <c r="D48" s="43" t="s">
         <v>757</v>
       </c>
-      <c r="E47" s="50">
+      <c r="E48" s="50">
         <f>((1260+960)*0.15)*1.1</f>
         <v>366.3</v>
       </c>
-      <c r="F47" s="44" t="s">
+      <c r="F48" s="44" t="s">
         <v>759</v>
       </c>
-      <c r="G47" s="45">
+      <c r="G48" s="45">
         <v>670</v>
       </c>
-      <c r="H47" s="45">
-        <f>G47*E47</f>
+      <c r="H48" s="45">
+        <f>G48*E48</f>
         <v>245421</v>
       </c>
-      <c r="I47" s="44" t="s">
+      <c r="I48" s="44" t="s">
         <v>865</v>
       </c>
     </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B48" s="20">
+    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B49" s="20">
         <v>45</v>
       </c>
-      <c r="C48" s="31" t="s">
+      <c r="C49" s="31" t="s">
         <v>807</v>
       </c>
-      <c r="D48" s="28" t="s">
+      <c r="D49" s="28" t="s">
         <v>775</v>
       </c>
-      <c r="E48" s="50">
+      <c r="E49" s="50">
         <f>(1260+960)/13*1.05</f>
         <v>179.30769230769232</v>
       </c>
-      <c r="F48" s="44" t="s">
+      <c r="F49" s="44" t="s">
         <v>760</v>
       </c>
-      <c r="G48" s="45">
+      <c r="G49" s="45">
         <v>220.5</v>
       </c>
-      <c r="H48" s="45">
-        <f>G48*E48</f>
+      <c r="H49" s="45">
+        <f>G49*E49</f>
         <v>39537.346153846156</v>
       </c>
-      <c r="I48" s="44" t="s">
-        <v>865</v>
-      </c>
-    </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B49" s="20">
-        <v>46</v>
-      </c>
-      <c r="C49" s="31" t="s">
-        <v>807</v>
-      </c>
-      <c r="D49" s="22" t="s">
-        <v>868</v>
-      </c>
-      <c r="E49" s="21">
-        <v>1</v>
-      </c>
-      <c r="F49" s="21" t="s">
-        <v>760</v>
-      </c>
-      <c r="G49" s="49"/>
-      <c r="H49" s="49">
-        <f>G49*E49</f>
-        <v>0</v>
-      </c>
-      <c r="I49" s="21" t="s">
+      <c r="I49" s="44" t="s">
         <v>865</v>
       </c>
     </row>
     <row r="50" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B50" s="20">
-        <v>47</v>
-      </c>
-      <c r="C50" s="17" t="s">
-        <v>806</v>
-      </c>
-      <c r="D50" s="28" t="s">
-        <v>853</v>
-      </c>
-      <c r="E50" s="24">
-        <v>1</v>
-      </c>
-      <c r="F50" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="C50" s="31" t="s">
+        <v>807</v>
+      </c>
+      <c r="D50" s="22" t="s">
+        <v>868</v>
+      </c>
+      <c r="E50" s="21">
+        <v>1</v>
+      </c>
+      <c r="F50" s="21" t="s">
         <v>760</v>
       </c>
-      <c r="G50" s="32">
-        <v>24500</v>
-      </c>
-      <c r="H50" s="32">
+      <c r="G50" s="49"/>
+      <c r="H50" s="49">
         <f>G50*E50</f>
-        <v>24500</v>
-      </c>
-      <c r="I50" s="24" t="s">
-        <v>772</v>
+        <v>0</v>
+      </c>
+      <c r="I50" s="21" t="s">
+        <v>865</v>
       </c>
     </row>
     <row r="51" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B51" s="20">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C51" s="17" t="s">
         <v>806</v>
       </c>
-      <c r="D51" s="19" t="s">
-        <v>831</v>
-      </c>
-      <c r="E51" s="20"/>
-      <c r="F51" s="20"/>
-      <c r="G51" s="18"/>
-      <c r="H51" s="18">
+      <c r="D51" s="28" t="s">
+        <v>853</v>
+      </c>
+      <c r="E51" s="24">
+        <v>1</v>
+      </c>
+      <c r="F51" s="24" t="s">
+        <v>760</v>
+      </c>
+      <c r="G51" s="32">
+        <v>24500</v>
+      </c>
+      <c r="H51" s="32">
         <f>G51*E51</f>
-        <v>0</v>
-      </c>
-      <c r="I51" s="20" t="s">
+        <v>24500</v>
+      </c>
+      <c r="I51" s="24" t="s">
         <v>772</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B52" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C52" s="17" t="s">
         <v>806</v>
       </c>
-      <c r="D52" s="28" t="s">
-        <v>773</v>
-      </c>
-      <c r="E52" s="24">
-        <v>1</v>
-      </c>
-      <c r="F52" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G52" s="29">
-        <v>968004</v>
-      </c>
-      <c r="H52" s="29">
+      <c r="D52" s="19" t="s">
+        <v>831</v>
+      </c>
+      <c r="E52" s="20"/>
+      <c r="F52" s="20"/>
+      <c r="G52" s="18"/>
+      <c r="H52" s="18">
         <f>G52*E52</f>
-        <v>968004</v>
-      </c>
-      <c r="I52" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="I52" s="20" t="s">
         <v>772</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B53" s="20">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C53" s="17" t="s">
-        <v>807</v>
-      </c>
-      <c r="D53" s="43" t="s">
-        <v>801</v>
-      </c>
-      <c r="E53" s="44">
-        <v>1</v>
-      </c>
-      <c r="F53" s="44" t="s">
+        <v>806</v>
+      </c>
+      <c r="D53" s="28" t="s">
+        <v>773</v>
+      </c>
+      <c r="E53" s="24">
+        <v>1</v>
+      </c>
+      <c r="F53" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G53" s="45">
-        <v>46600</v>
-      </c>
-      <c r="H53" s="45">
+      <c r="G53" s="29">
+        <v>968004</v>
+      </c>
+      <c r="H53" s="29">
         <f>G53*E53</f>
-        <v>46600</v>
-      </c>
-      <c r="I53" s="44" t="s">
-        <v>871</v>
+        <v>968004</v>
+      </c>
+      <c r="I53" s="24" t="s">
+        <v>772</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B54" s="20">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C54" s="17" t="s">
         <v>807</v>
       </c>
       <c r="D54" s="43" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="E54" s="44">
         <v>1</v>
@@ -15236,11 +15253,11 @@
         <v>760</v>
       </c>
       <c r="G54" s="45">
-        <v>8100</v>
+        <v>46600</v>
       </c>
       <c r="H54" s="45">
         <f>G54*E54</f>
-        <v>8100</v>
+        <v>46600</v>
       </c>
       <c r="I54" s="44" t="s">
         <v>871</v>
@@ -15248,13 +15265,13 @@
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B55" s="20">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C55" s="17" t="s">
         <v>807</v>
       </c>
       <c r="D55" s="43" t="s">
-        <v>816</v>
+        <v>804</v>
       </c>
       <c r="E55" s="44">
         <v>1</v>
@@ -15263,11 +15280,11 @@
         <v>760</v>
       </c>
       <c r="G55" s="45">
-        <v>5000</v>
+        <v>8100</v>
       </c>
       <c r="H55" s="45">
         <f>G55*E55</f>
-        <v>5000</v>
+        <v>8100</v>
       </c>
       <c r="I55" s="44" t="s">
         <v>871</v>
@@ -15275,13 +15292,13 @@
     </row>
     <row r="56" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B56" s="20">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C56" s="17" t="s">
         <v>807</v>
       </c>
       <c r="D56" s="43" t="s">
-        <v>808</v>
+        <v>816</v>
       </c>
       <c r="E56" s="44">
         <v>1</v>
@@ -15290,11 +15307,11 @@
         <v>760</v>
       </c>
       <c r="G56" s="45">
-        <v>670000</v>
+        <v>5000</v>
       </c>
       <c r="H56" s="45">
         <f>G56*E56</f>
-        <v>670000</v>
+        <v>5000</v>
       </c>
       <c r="I56" s="44" t="s">
         <v>871</v>
@@ -15302,70 +15319,72 @@
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" s="20">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C57" s="17" t="s">
-        <v>806</v>
-      </c>
-      <c r="D57" s="19" t="s">
-        <v>791</v>
-      </c>
-      <c r="E57" s="20"/>
-      <c r="F57" s="20"/>
-      <c r="G57" s="18"/>
-      <c r="H57" s="18">
+        <v>807</v>
+      </c>
+      <c r="D57" s="43" t="s">
+        <v>808</v>
+      </c>
+      <c r="E57" s="44">
+        <v>1</v>
+      </c>
+      <c r="F57" s="44" t="s">
+        <v>760</v>
+      </c>
+      <c r="G57" s="45">
+        <v>670000</v>
+      </c>
+      <c r="H57" s="45">
         <f>G57*E57</f>
-        <v>0</v>
-      </c>
-      <c r="I57" s="20" t="s">
-        <v>419</v>
+        <v>670000</v>
+      </c>
+      <c r="I57" s="44" t="s">
+        <v>871</v>
       </c>
     </row>
     <row r="58" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B58" s="20">
-        <v>55</v>
-      </c>
-      <c r="C58" s="17"/>
-      <c r="D58" s="28" t="s">
-        <v>874</v>
-      </c>
-      <c r="E58" s="24">
-        <v>87</v>
-      </c>
-      <c r="F58" s="24" t="s">
-        <v>760</v>
-      </c>
-      <c r="G58" s="32">
-        <v>34.99</v>
-      </c>
-      <c r="H58" s="32">
+        <v>54</v>
+      </c>
+      <c r="C58" s="17" t="s">
+        <v>806</v>
+      </c>
+      <c r="D58" s="19" t="s">
+        <v>791</v>
+      </c>
+      <c r="E58" s="20"/>
+      <c r="F58" s="20"/>
+      <c r="G58" s="18"/>
+      <c r="H58" s="18">
         <f>G58*E58</f>
-        <v>3044.13</v>
-      </c>
-      <c r="I58" s="24" t="s">
-        <v>798</v>
+        <v>0</v>
+      </c>
+      <c r="I58" s="20" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B59" s="20">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C59" s="17"/>
-      <c r="D59" s="42" t="s">
-        <v>875</v>
+      <c r="D59" s="28" t="s">
+        <v>874</v>
       </c>
       <c r="E59" s="24">
-        <v>174</v>
+        <v>87</v>
       </c>
       <c r="F59" s="24" t="s">
         <v>760</v>
       </c>
       <c r="G59" s="32">
-        <v>255.5</v>
+        <v>34.99</v>
       </c>
       <c r="H59" s="32">
         <f>G59*E59</f>
-        <v>44457</v>
+        <v>3044.13</v>
       </c>
       <c r="I59" s="24" t="s">
         <v>798</v>
@@ -15373,11 +15392,11 @@
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B60" s="20">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C60" s="17"/>
-      <c r="D60" s="28" t="s">
-        <v>876</v>
+      <c r="D60" s="42" t="s">
+        <v>875</v>
       </c>
       <c r="E60" s="24">
         <v>174</v>
@@ -15386,11 +15405,11 @@
         <v>760</v>
       </c>
       <c r="G60" s="32">
-        <v>196</v>
+        <v>255.5</v>
       </c>
       <c r="H60" s="32">
         <f>G60*E60</f>
-        <v>34104</v>
+        <v>44457</v>
       </c>
       <c r="I60" s="24" t="s">
         <v>798</v>
@@ -15398,24 +15417,24 @@
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B61" s="20">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C61" s="17"/>
-      <c r="D61" s="42" t="s">
-        <v>877</v>
+      <c r="D61" s="28" t="s">
+        <v>876</v>
       </c>
       <c r="E61" s="24">
-        <v>4700</v>
+        <v>174</v>
       </c>
       <c r="F61" s="24" t="s">
         <v>760</v>
       </c>
       <c r="G61" s="32">
-        <v>0.5</v>
+        <v>196</v>
       </c>
       <c r="H61" s="32">
         <f>G61*E61</f>
-        <v>2350</v>
+        <v>34104</v>
       </c>
       <c r="I61" s="24" t="s">
         <v>798</v>
@@ -15423,14 +15442,14 @@
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B62" s="20">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C62" s="17"/>
-      <c r="D62" s="28" t="s">
-        <v>878</v>
+      <c r="D62" s="42" t="s">
+        <v>877</v>
       </c>
       <c r="E62" s="24">
-        <v>3200</v>
+        <v>4700</v>
       </c>
       <c r="F62" s="24" t="s">
         <v>760</v>
@@ -15440,7 +15459,7 @@
       </c>
       <c r="H62" s="32">
         <f>G62*E62</f>
-        <v>1600</v>
+        <v>2350</v>
       </c>
       <c r="I62" s="24" t="s">
         <v>798</v>
@@ -15448,57 +15467,63 @@
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" s="20">
-        <v>60</v>
-      </c>
-      <c r="C63" s="17" t="s">
-        <v>806</v>
-      </c>
-      <c r="D63" s="19" t="s">
-        <v>784</v>
-      </c>
-      <c r="E63" s="20">
-        <v>1</v>
-      </c>
-      <c r="F63" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C63" s="17"/>
+      <c r="D63" s="28" t="s">
+        <v>878</v>
+      </c>
+      <c r="E63" s="24">
+        <v>3200</v>
+      </c>
+      <c r="F63" s="24" t="s">
         <v>760</v>
       </c>
-      <c r="G63" s="18">
-        <v>791792.51</v>
-      </c>
-      <c r="H63" s="18">
+      <c r="G63" s="32">
+        <v>0.5</v>
+      </c>
+      <c r="H63" s="32">
         <f>G63*E63</f>
-        <v>791792.51</v>
-      </c>
-      <c r="I63" s="20" t="s">
-        <v>783</v>
+        <v>1600</v>
+      </c>
+      <c r="I63" s="24" t="s">
+        <v>798</v>
       </c>
     </row>
     <row r="64" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B64" s="20">
-        <v>61</v>
-      </c>
-      <c r="C64" s="17"/>
-      <c r="D64" s="22" t="s">
-        <v>859</v>
-      </c>
-      <c r="E64" s="21"/>
-      <c r="F64" s="21"/>
-      <c r="G64" s="49"/>
-      <c r="H64" s="49">
+        <v>60</v>
+      </c>
+      <c r="C64" s="17" t="s">
+        <v>806</v>
+      </c>
+      <c r="D64" s="19" t="s">
+        <v>784</v>
+      </c>
+      <c r="E64" s="20">
+        <v>1</v>
+      </c>
+      <c r="F64" s="20" t="s">
+        <v>760</v>
+      </c>
+      <c r="G64" s="18">
+        <v>791792.51</v>
+      </c>
+      <c r="H64" s="18">
         <f>G64*E64</f>
-        <v>0</v>
-      </c>
-      <c r="I64" s="21" t="s">
-        <v>870</v>
+        <v>791792.51</v>
+      </c>
+      <c r="I64" s="20" t="s">
+        <v>783</v>
       </c>
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" s="20">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C65" s="17"/>
       <c r="D65" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="E65" s="21"/>
       <c r="F65" s="21"/>
@@ -15513,11 +15538,11 @@
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B66" s="20">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C66" s="17"/>
       <c r="D66" s="22" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="E66" s="21"/>
       <c r="F66" s="21"/>
@@ -15532,16 +15557,16 @@
     </row>
     <row r="67" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B67" s="20">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C67" s="17"/>
-      <c r="D67" s="19" t="s">
-        <v>864</v>
-      </c>
-      <c r="E67" s="20"/>
-      <c r="F67" s="20"/>
-      <c r="G67" s="18"/>
-      <c r="H67" s="18">
+      <c r="D67" s="22" t="s">
+        <v>863</v>
+      </c>
+      <c r="E67" s="21"/>
+      <c r="F67" s="21"/>
+      <c r="G67" s="49"/>
+      <c r="H67" s="49">
         <f>G67*E67</f>
         <v>0</v>
       </c>
@@ -15551,16 +15576,16 @@
     </row>
     <row r="68" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B68" s="20">
-        <v>65</v>
-      </c>
-      <c r="C68" s="31"/>
-      <c r="D68" s="22" t="s">
-        <v>857</v>
-      </c>
-      <c r="E68" s="21"/>
-      <c r="F68" s="21"/>
-      <c r="G68" s="23"/>
-      <c r="H68" s="47">
+        <v>64</v>
+      </c>
+      <c r="C68" s="17"/>
+      <c r="D68" s="19" t="s">
+        <v>864</v>
+      </c>
+      <c r="E68" s="20"/>
+      <c r="F68" s="20"/>
+      <c r="G68" s="18"/>
+      <c r="H68" s="18">
         <f>G68*E68</f>
         <v>0</v>
       </c>
@@ -15569,14 +15594,23 @@
       </c>
     </row>
     <row r="69" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B69" s="21"/>
+      <c r="B69" s="20">
+        <v>65</v>
+      </c>
       <c r="C69" s="31"/>
-      <c r="D69" s="22"/>
+      <c r="D69" s="22" t="s">
+        <v>857</v>
+      </c>
       <c r="E69" s="21"/>
       <c r="F69" s="21"/>
       <c r="G69" s="23"/>
-      <c r="H69" s="47"/>
-      <c r="I69" s="21"/>
+      <c r="H69" s="47">
+        <f>G69*E69</f>
+        <v>0</v>
+      </c>
+      <c r="I69" s="21" t="s">
+        <v>870</v>
+      </c>
     </row>
     <row r="70" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B70" s="21"/>
@@ -15589,10 +15623,26 @@
       <c r="I70" s="21"/>
     </row>
     <row r="71" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="D71" s="34"/>
-      <c r="H71" s="16">
+      <c r="B71" s="21"/>
+      <c r="C71" s="31"/>
+      <c r="D71" s="22"/>
+      <c r="E71" s="21"/>
+      <c r="F71" s="21"/>
+      <c r="G71" s="23"/>
+      <c r="H71" s="47"/>
+      <c r="I71" s="21"/>
+    </row>
+    <row r="72" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D72" s="34"/>
+      <c r="H72" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>4441142.4091069028</v>
+        <v>4447142.4091069028</v>
+      </c>
+    </row>
+    <row r="76" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="H76" s="51">
+        <f>SUM('Expansão DMP'!G49,H72)</f>
+        <v>6823772.9299530564</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 12:16
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2343" uniqueCount="920">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2346" uniqueCount="922">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2788,6 +2788,12 @@
   </si>
   <si>
     <t>Mão de obra para fechamento em alvenaria e telhas na fachada do galpão DPA IV</t>
+  </si>
+  <si>
+    <t>Realocação da estação de abastecimento de gás das empilhadeiras</t>
+  </si>
+  <si>
+    <t>Combate ao Incêndio</t>
   </si>
 </sst>
 </file>
@@ -3403,8 +3409,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H52" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="B3:H52"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H53" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="B3:H53"/>
   <sortState ref="B4:H53">
     <sortCondition ref="H3:H53"/>
   </sortState>
@@ -12912,7 +12918,7 @@
       </c>
       <c r="G2" s="20"/>
       <c r="H2" s="20">
-        <f>G2*E2</f>
+        <f t="shared" ref="H2:H33" si="0">G2*E2</f>
         <v>0</v>
       </c>
       <c r="I2" s="18" t="s">
@@ -12942,11 +12948,11 @@
         <v>486032</v>
       </c>
       <c r="H3" s="25">
-        <f>G3*E3</f>
+        <f t="shared" si="0"/>
         <v>486032</v>
       </c>
-      <c r="I3" s="21" t="s">
-        <v>779</v>
+      <c r="I3" s="53" t="s">
+        <v>921</v>
       </c>
       <c r="J3" s="39"/>
       <c r="K3" s="39"/>
@@ -12969,11 +12975,11 @@
         <v>8650</v>
       </c>
       <c r="H4" s="25">
-        <f>G4*E4</f>
+        <f t="shared" si="0"/>
         <v>8650</v>
       </c>
-      <c r="I4" s="21" t="s">
-        <v>779</v>
+      <c r="I4" s="53" t="s">
+        <v>921</v>
       </c>
       <c r="J4" s="39"/>
       <c r="K4" s="39"/>
@@ -12996,7 +13002,7 @@
         <v>21938</v>
       </c>
       <c r="H5" s="25">
-        <f>G5*E5</f>
+        <f t="shared" si="0"/>
         <v>131628</v>
       </c>
       <c r="I5" s="21" t="s">
@@ -13023,7 +13029,7 @@
         <v>11180</v>
       </c>
       <c r="H6" s="25">
-        <f>G6*E6</f>
+        <f t="shared" si="0"/>
         <v>11180</v>
       </c>
       <c r="I6" s="21" t="s">
@@ -13050,7 +13056,7 @@
         <v>55.57</v>
       </c>
       <c r="H7" s="25">
-        <f>G7*E7</f>
+        <f t="shared" si="0"/>
         <v>13892.5</v>
       </c>
       <c r="I7" s="21" t="s">
@@ -13077,7 +13083,7 @@
         <v>13855.22</v>
       </c>
       <c r="H8" s="38">
-        <f>G8*E8</f>
+        <f t="shared" si="0"/>
         <v>83131.319999999992</v>
       </c>
       <c r="I8" s="21" t="s">
@@ -13104,7 +13110,7 @@
         <v>111260.98</v>
       </c>
       <c r="H9" s="38">
-        <f>G9*E9</f>
+        <f t="shared" si="0"/>
         <v>111260.98</v>
       </c>
       <c r="I9" s="21" t="s">
@@ -13131,7 +13137,7 @@
         <v>55.57</v>
       </c>
       <c r="H10" s="38">
-        <f>G10*E10</f>
+        <f t="shared" si="0"/>
         <v>16671</v>
       </c>
       <c r="I10" s="21" t="s">
@@ -13158,7 +13164,7 @@
         <v>27412.5</v>
       </c>
       <c r="H11" s="38">
-        <f>G11*E11</f>
+        <f t="shared" si="0"/>
         <v>27412.5</v>
       </c>
       <c r="I11" s="21" t="s">
@@ -13186,7 +13192,7 @@
         <v>670</v>
       </c>
       <c r="H12" s="31">
-        <f>G12*E12</f>
+        <f t="shared" si="0"/>
         <v>118841.25000000001</v>
       </c>
       <c r="I12" s="30" t="s">
@@ -13214,7 +13220,7 @@
         <v>220.5</v>
       </c>
       <c r="H13" s="31">
-        <f>G13*E13</f>
+        <f t="shared" si="0"/>
         <v>36467.307692307695</v>
       </c>
       <c r="I13" s="30" t="s">
@@ -13242,7 +13248,7 @@
         <v>56.2</v>
       </c>
       <c r="H14" s="31">
-        <f>G14*E14</f>
+        <f t="shared" si="0"/>
         <v>4964.333333333333</v>
       </c>
       <c r="I14" s="30" t="s">
@@ -13270,7 +13276,7 @@
         <v>50</v>
       </c>
       <c r="H15" s="31">
-        <f>G15*E15</f>
+        <f t="shared" si="0"/>
         <v>8868.7500000000018</v>
       </c>
       <c r="I15" s="30" t="s">
@@ -13297,7 +13303,7 @@
         <v>67000</v>
       </c>
       <c r="H16" s="31">
-        <f>G16*E16</f>
+        <f t="shared" si="0"/>
         <v>67000</v>
       </c>
       <c r="I16" s="30" t="s">
@@ -13324,7 +13330,7 @@
         <v>48600</v>
       </c>
       <c r="H17" s="38">
-        <f>G17*E17</f>
+        <f t="shared" si="0"/>
         <v>48600</v>
       </c>
       <c r="I17" s="30" t="s">
@@ -13349,7 +13355,7 @@
         <v>48600</v>
       </c>
       <c r="H18" s="38">
-        <f>G18*E18</f>
+        <f t="shared" si="0"/>
         <v>48600</v>
       </c>
       <c r="I18" s="30" t="s">
@@ -13376,7 +13382,7 @@
         <v>243.39</v>
       </c>
       <c r="H19" s="38">
-        <f>G19*E19</f>
+        <f t="shared" si="0"/>
         <v>12169.5</v>
       </c>
       <c r="I19" s="30" t="s">
@@ -13404,7 +13410,7 @@
         <v>38.119999999999997</v>
       </c>
       <c r="H20" s="38">
-        <f>G20*E20</f>
+        <f t="shared" si="0"/>
         <v>6709.12</v>
       </c>
       <c r="I20" s="30" t="s">
@@ -13431,7 +13437,7 @@
         <v>24</v>
       </c>
       <c r="H21" s="38">
-        <f>G21*E21</f>
+        <f t="shared" si="0"/>
         <v>240</v>
       </c>
       <c r="I21" s="30" t="s">
@@ -13463,7 +13469,7 @@
         <v>243.39</v>
       </c>
       <c r="H22" s="38">
-        <f>G22*E22</f>
+        <f t="shared" si="0"/>
         <v>8762.0399999999991</v>
       </c>
       <c r="I22" s="30" t="s">
@@ -13492,7 +13498,7 @@
         <v>38.119999999999997</v>
       </c>
       <c r="H23" s="38">
-        <f>G23*E23</f>
+        <f t="shared" si="0"/>
         <v>2744.64</v>
       </c>
       <c r="I23" s="30" t="s">
@@ -13521,7 +13527,7 @@
         <v>32</v>
       </c>
       <c r="H24" s="38">
-        <f>G24*E24</f>
+        <f t="shared" si="0"/>
         <v>1152</v>
       </c>
       <c r="I24" s="30" t="s">
@@ -13550,7 +13556,7 @@
         <v>419</v>
       </c>
       <c r="H25" s="38">
-        <f>G25*E25</f>
+        <f t="shared" si="0"/>
         <v>1676</v>
       </c>
       <c r="I25" s="30" t="s">
@@ -13580,7 +13586,7 @@
         <v>38.119999999999997</v>
       </c>
       <c r="H26" s="38">
-        <f>G26*E26</f>
+        <f t="shared" si="0"/>
         <v>1829.7599999999998</v>
       </c>
       <c r="I26" s="30" t="s">
@@ -13607,7 +13613,7 @@
         <v>65000</v>
       </c>
       <c r="H27" s="31">
-        <f>G27*E27</f>
+        <f t="shared" si="0"/>
         <v>130000</v>
       </c>
       <c r="I27" s="30" t="s">
@@ -13636,7 +13642,7 @@
         <v>198.72</v>
       </c>
       <c r="H28" s="25">
-        <f>G28*E28</f>
+        <f t="shared" si="0"/>
         <v>11525.76</v>
       </c>
       <c r="I28" s="21" t="s">
@@ -13665,7 +13671,7 @@
         <v>484.24</v>
       </c>
       <c r="H29" s="25">
-        <f>G29*E29</f>
+        <f t="shared" si="0"/>
         <v>15011.44</v>
       </c>
       <c r="I29" s="21" t="s">
@@ -13694,7 +13700,7 @@
         <v>703.93</v>
       </c>
       <c r="H30" s="25">
-        <f>G30*E30</f>
+        <f t="shared" si="0"/>
         <v>19710.039999999997</v>
       </c>
       <c r="I30" s="21" t="s">
@@ -13724,7 +13730,7 @@
         <v>49.05</v>
       </c>
       <c r="H31" s="25">
-        <f>G31*E31</f>
+        <f t="shared" si="0"/>
         <v>4120.2</v>
       </c>
       <c r="I31" s="21" t="s">
@@ -13753,7 +13759,7 @@
         <v>151.19999999999999</v>
       </c>
       <c r="H32" s="25">
-        <f>G32*E32</f>
+        <f t="shared" si="0"/>
         <v>453.59999999999997</v>
       </c>
       <c r="I32" s="21" t="s">
@@ -13782,7 +13788,7 @@
         <v>48.38</v>
       </c>
       <c r="H33" s="25">
-        <f>G33*E33</f>
+        <f t="shared" si="0"/>
         <v>96.76</v>
       </c>
       <c r="I33" s="21" t="s">
@@ -13811,7 +13817,7 @@
         <v>27.14</v>
       </c>
       <c r="H34" s="25">
-        <f>G34*E34</f>
+        <f t="shared" ref="H34:H65" si="1">G34*E34</f>
         <v>814.2</v>
       </c>
       <c r="I34" s="21" t="s">
@@ -13840,7 +13846,7 @@
         <v>703.93</v>
       </c>
       <c r="H35" s="25">
-        <f>G35*E35</f>
+        <f t="shared" si="1"/>
         <v>8447.16</v>
       </c>
       <c r="I35" s="21" t="s">
@@ -13870,7 +13876,7 @@
         <v>484.24</v>
       </c>
       <c r="H36" s="25">
-        <f>G36*E36</f>
+        <f t="shared" si="1"/>
         <v>6295.12</v>
       </c>
       <c r="I36" s="21" t="s">
@@ -13897,7 +13903,7 @@
         <v>37375</v>
       </c>
       <c r="H37" s="38">
-        <f>G37*E37</f>
+        <f t="shared" si="1"/>
         <v>37375</v>
       </c>
       <c r="I37" s="30" t="s">
@@ -13925,7 +13931,7 @@
         <v>243.39</v>
       </c>
       <c r="H38" s="25">
-        <f>G38*E38</f>
+        <f t="shared" si="1"/>
         <v>26286.12</v>
       </c>
       <c r="I38" s="21" t="s">
@@ -13953,7 +13959,7 @@
         <v>119.7</v>
       </c>
       <c r="H39" s="25">
-        <f>G39*E39</f>
+        <f t="shared" si="1"/>
         <v>3591</v>
       </c>
       <c r="I39" s="21" t="s">
@@ -13980,7 +13986,7 @@
         <v>38.116666600000002</v>
       </c>
       <c r="H40" s="25">
-        <f>G40*E40</f>
+        <f t="shared" si="1"/>
         <v>14865.499974</v>
       </c>
       <c r="I40" s="21" t="s">
@@ -14008,7 +14014,7 @@
         <v>243.39</v>
       </c>
       <c r="H41" s="25">
-        <f>G41*E41</f>
+        <f t="shared" si="1"/>
         <v>42541.456608</v>
       </c>
       <c r="I41" s="21" t="s">
@@ -14037,7 +14043,7 @@
         <v>38.116666600000002</v>
       </c>
       <c r="H42" s="25">
-        <f>G42*E42</f>
+        <f t="shared" si="1"/>
         <v>22412.599960800002</v>
       </c>
       <c r="I42" s="21" t="s">
@@ -14064,7 +14070,7 @@
         <v>24</v>
       </c>
       <c r="H43" s="25">
-        <f>G43*E43</f>
+        <f t="shared" si="1"/>
         <v>720</v>
       </c>
       <c r="I43" s="21" t="s">
@@ -14091,7 +14097,7 @@
         <v>860</v>
       </c>
       <c r="H44" s="25">
-        <f>G44*E44</f>
+        <f t="shared" si="1"/>
         <v>860</v>
       </c>
       <c r="I44" s="21" t="s">
@@ -14118,7 +14124,7 @@
         <v>23.90625</v>
       </c>
       <c r="H45" s="31">
-        <f>G45*E45</f>
+        <f t="shared" si="1"/>
         <v>3346.875</v>
       </c>
       <c r="I45" s="30" t="s">
@@ -14145,7 +14151,7 @@
         <v>26</v>
       </c>
       <c r="H46" s="31">
-        <f>G46*E46</f>
+        <f t="shared" si="1"/>
         <v>1716</v>
       </c>
       <c r="I46" s="30" t="s">
@@ -14173,7 +14179,7 @@
         <v>31000</v>
       </c>
       <c r="H47" s="31">
-        <f>G47*E47</f>
+        <f t="shared" si="1"/>
         <v>31000</v>
       </c>
       <c r="I47" s="30" t="s">
@@ -14200,7 +14206,7 @@
         <v>6000</v>
       </c>
       <c r="H48" s="23">
-        <f>G48*E48</f>
+        <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="I48" s="21" t="s">
@@ -14227,7 +14233,7 @@
         <v>9.65</v>
       </c>
       <c r="H49" s="23">
-        <f>G49*E49</f>
+        <f t="shared" si="1"/>
         <v>39565</v>
       </c>
       <c r="I49" s="21" t="s">
@@ -14254,7 +14260,7 @@
         <v>9.65</v>
       </c>
       <c r="H50" s="23">
-        <f>G50*E50</f>
+        <f t="shared" si="1"/>
         <v>38600</v>
       </c>
       <c r="I50" s="21" t="s">
@@ -14284,7 +14290,7 @@
         <v>164000</v>
       </c>
       <c r="H51" s="23">
-        <f>G51*E51</f>
+        <f t="shared" si="1"/>
         <v>164000</v>
       </c>
       <c r="I51" s="21" t="s">
@@ -14314,7 +14320,7 @@
         <v>670</v>
       </c>
       <c r="H52" s="23">
-        <f>G52*E52</f>
+        <f t="shared" si="1"/>
         <v>66477.399999999994</v>
       </c>
       <c r="I52" s="21" t="s">
@@ -14341,7 +14347,7 @@
         <v>670</v>
       </c>
       <c r="H53" s="23">
-        <f>G53*E53</f>
+        <f t="shared" si="1"/>
         <v>45560</v>
       </c>
       <c r="I53" s="21" t="s">
@@ -14368,7 +14374,7 @@
         <v>56500</v>
       </c>
       <c r="H54" s="23">
-        <f>G54*E54</f>
+        <f t="shared" si="1"/>
         <v>56500</v>
       </c>
       <c r="I54" s="21" t="s">
@@ -14392,11 +14398,11 @@
         <v>760</v>
       </c>
       <c r="G55" s="25">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="H55" s="25">
-        <f>G55*E55</f>
-        <v>6000</v>
+        <f t="shared" si="1"/>
+        <v>6250</v>
       </c>
       <c r="I55" s="21" t="s">
         <v>771</v>
@@ -14422,7 +14428,7 @@
         <v>1500</v>
       </c>
       <c r="H56" s="25">
-        <f>G56*E56</f>
+        <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="I56" s="21" t="s">
@@ -14449,7 +14455,7 @@
         <v>420</v>
       </c>
       <c r="H57" s="31">
-        <f>G57*E57</f>
+        <f t="shared" si="1"/>
         <v>10920</v>
       </c>
       <c r="I57" s="21" t="s">
@@ -14479,7 +14485,7 @@
         <v>15</v>
       </c>
       <c r="H58" s="31">
-        <f>G58*E58</f>
+        <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="I58" s="21" t="s">
@@ -14502,7 +14508,7 @@
       </c>
       <c r="G59" s="34"/>
       <c r="H59" s="34">
-        <f>G59*E59</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I59" s="17" t="s">
@@ -14529,7 +14535,7 @@
         <v>380</v>
       </c>
       <c r="H60" s="31">
-        <f>G60*E60</f>
+        <f t="shared" si="1"/>
         <v>3040</v>
       </c>
       <c r="I60" s="30" t="s">
@@ -14556,7 +14562,7 @@
         <v>290</v>
       </c>
       <c r="H61" s="31">
-        <f>G61*E61</f>
+        <f t="shared" si="1"/>
         <v>1160</v>
       </c>
       <c r="I61" s="30" t="s">
@@ -14583,7 +14589,7 @@
         <v>290</v>
       </c>
       <c r="H62" s="31">
-        <f>G62*E62</f>
+        <f t="shared" si="1"/>
         <v>1160</v>
       </c>
       <c r="I62" s="30" t="s">
@@ -14611,7 +14617,7 @@
         <v>670</v>
       </c>
       <c r="H63" s="23">
-        <f>G63*E63</f>
+        <f t="shared" si="1"/>
         <v>226878.75</v>
       </c>
       <c r="I63" s="21" t="s">
@@ -14639,7 +14645,7 @@
         <v>220.5</v>
       </c>
       <c r="H64" s="23">
-        <f>G64*E64</f>
+        <f t="shared" si="1"/>
         <v>72934.61538461539</v>
       </c>
       <c r="I64" s="21" t="s">
@@ -14667,7 +14673,7 @@
         <v>56.2</v>
       </c>
       <c r="H65" s="23">
-        <f>G65*E65</f>
+        <f t="shared" si="1"/>
         <v>9835</v>
       </c>
       <c r="I65" s="21" t="s">
@@ -14694,7 +14700,7 @@
         <v>7.3</v>
       </c>
       <c r="H66" s="23">
-        <f>G66*E66</f>
+        <f t="shared" ref="H66:H97" si="2">G66*E66</f>
         <v>7300</v>
       </c>
       <c r="I66" s="21" t="s">
@@ -14722,7 +14728,7 @@
         <v>50</v>
       </c>
       <c r="H67" s="23">
-        <f>G67*E67</f>
+        <f t="shared" si="2"/>
         <v>16931.25</v>
       </c>
       <c r="I67" s="21" t="s">
@@ -14749,7 +14755,7 @@
         <v>53550</v>
       </c>
       <c r="H68" s="23">
-        <f>G68*E68</f>
+        <f t="shared" si="2"/>
         <v>53550</v>
       </c>
       <c r="I68" s="21" t="s">
@@ -14776,7 +14782,7 @@
         <v>42.29</v>
       </c>
       <c r="H69" s="31">
-        <f>G69*E69</f>
+        <f t="shared" si="2"/>
         <v>4651.8999999999996</v>
       </c>
       <c r="I69" s="30" t="s">
@@ -14803,7 +14809,7 @@
         <v>1400</v>
       </c>
       <c r="H70" s="31">
-        <f>G70*E70</f>
+        <f t="shared" si="2"/>
         <v>1400</v>
       </c>
       <c r="I70" s="30" t="s">
@@ -14831,7 +14837,7 @@
         <v>670</v>
       </c>
       <c r="H71" s="31">
-        <f>G71*E71</f>
+        <f t="shared" si="2"/>
         <v>245421</v>
       </c>
       <c r="I71" s="30" t="s">
@@ -14859,7 +14865,7 @@
         <v>220.5</v>
       </c>
       <c r="H72" s="31">
-        <f>G72*E72</f>
+        <f t="shared" si="2"/>
         <v>39537.346153846156</v>
       </c>
       <c r="I72" s="30" t="s">
@@ -14886,7 +14892,7 @@
         <v>62525</v>
       </c>
       <c r="H73" s="31">
-        <f>G73*E73</f>
+        <f t="shared" si="2"/>
         <v>62525</v>
       </c>
       <c r="I73" s="30" t="s">
@@ -14913,7 +14919,7 @@
         <v>24500</v>
       </c>
       <c r="H74" s="25">
-        <f>G74*E74</f>
+        <f t="shared" si="2"/>
         <v>24500</v>
       </c>
       <c r="I74" s="21" t="s">
@@ -14940,7 +14946,7 @@
         <v>968004</v>
       </c>
       <c r="H75" s="23">
-        <f>G75*E75</f>
+        <f t="shared" si="2"/>
         <v>968004</v>
       </c>
       <c r="I75" s="21" t="s">
@@ -14967,7 +14973,7 @@
         <v>32000</v>
       </c>
       <c r="H76" s="38">
-        <f>G76*E76</f>
+        <f t="shared" si="2"/>
         <v>32000</v>
       </c>
       <c r="I76" s="30" t="s">
@@ -14994,7 +15000,7 @@
         <v>10000</v>
       </c>
       <c r="H77" s="38">
-        <f>G77*E77</f>
+        <f t="shared" si="2"/>
         <v>10000</v>
       </c>
       <c r="I77" s="30" t="s">
@@ -15021,7 +15027,7 @@
         <v>46600</v>
       </c>
       <c r="H78" s="31">
-        <f>G78*E78</f>
+        <f t="shared" si="2"/>
         <v>46600</v>
       </c>
       <c r="I78" s="30" t="s">
@@ -15048,7 +15054,7 @@
         <v>8100</v>
       </c>
       <c r="H79" s="31">
-        <f>G79*E79</f>
+        <f t="shared" si="2"/>
         <v>8100</v>
       </c>
       <c r="I79" s="30" t="s">
@@ -15075,7 +15081,7 @@
         <v>5000</v>
       </c>
       <c r="H80" s="31">
-        <f>G80*E80</f>
+        <f t="shared" si="2"/>
         <v>5000</v>
       </c>
       <c r="I80" s="30" t="s">
@@ -15102,7 +15108,7 @@
         <v>27000</v>
       </c>
       <c r="H81" s="31">
-        <f>G81*E81</f>
+        <f t="shared" si="2"/>
         <v>27000</v>
       </c>
       <c r="I81" s="30" t="s">
@@ -15129,7 +15135,7 @@
         <v>16</v>
       </c>
       <c r="H82" s="31">
-        <f>G82*E82</f>
+        <f t="shared" si="2"/>
         <v>5120</v>
       </c>
       <c r="I82" s="30" t="s">
@@ -15156,7 +15162,7 @@
         <v>3400</v>
       </c>
       <c r="H83" s="31">
-        <f>G83*E83</f>
+        <f t="shared" si="2"/>
         <v>3400</v>
       </c>
       <c r="I83" s="30" t="s">
@@ -15183,7 +15189,7 @@
         <v>8000</v>
       </c>
       <c r="H84" s="31">
-        <f>G84*E84</f>
+        <f t="shared" si="2"/>
         <v>8000</v>
       </c>
       <c r="I84" s="30" t="s">
@@ -15210,7 +15216,7 @@
         <v>2500</v>
       </c>
       <c r="H85" s="31">
-        <f>G85*E85</f>
+        <f t="shared" si="2"/>
         <v>2500</v>
       </c>
       <c r="I85" s="30" t="s">
@@ -15239,7 +15245,7 @@
         <v>102</v>
       </c>
       <c r="H86" s="31">
-        <f>G86*E86</f>
+        <f t="shared" si="2"/>
         <v>11730</v>
       </c>
       <c r="I86" s="21" t="s">
@@ -15266,7 +15272,7 @@
         <v>34.99</v>
       </c>
       <c r="H87" s="25">
-        <f>G87*E87</f>
+        <f t="shared" si="2"/>
         <v>3044.13</v>
       </c>
       <c r="I87" s="21" t="s">
@@ -15293,7 +15299,7 @@
         <v>255.5</v>
       </c>
       <c r="H88" s="25">
-        <f>G88*E88</f>
+        <f t="shared" si="2"/>
         <v>44457</v>
       </c>
       <c r="I88" s="21" t="s">
@@ -15320,7 +15326,7 @@
         <v>196</v>
       </c>
       <c r="H89" s="25">
-        <f>G89*E89</f>
+        <f t="shared" si="2"/>
         <v>34104</v>
       </c>
       <c r="I89" s="21" t="s">
@@ -15347,7 +15353,7 @@
         <v>0.5</v>
       </c>
       <c r="H90" s="25">
-        <f>G90*E90</f>
+        <f t="shared" si="2"/>
         <v>2350</v>
       </c>
       <c r="I90" s="21" t="s">
@@ -15374,7 +15380,7 @@
         <v>0.5</v>
       </c>
       <c r="H91" s="25">
-        <f>G91*E91</f>
+        <f t="shared" si="2"/>
         <v>1600</v>
       </c>
       <c r="I91" s="21" t="s">
@@ -15401,7 +15407,7 @@
         <v>908615.35</v>
       </c>
       <c r="H92" s="25">
-        <f>G92*E92</f>
+        <f t="shared" si="2"/>
         <v>908615.35</v>
       </c>
       <c r="I92" s="21" t="s">
@@ -15430,7 +15436,7 @@
         <v>124.25</v>
       </c>
       <c r="H93" s="31">
-        <f>G93*E93</f>
+        <f t="shared" si="2"/>
         <v>93187.5</v>
       </c>
       <c r="I93" s="30" t="s">
@@ -15459,7 +15465,7 @@
         <v>55.57</v>
       </c>
       <c r="H94" s="31">
-        <f>G94*E94</f>
+        <f t="shared" si="2"/>
         <v>13892.5</v>
       </c>
       <c r="I94" s="30" t="s">
@@ -15486,7 +15492,7 @@
         <v>4430</v>
       </c>
       <c r="H95" s="31">
-        <f>G95*E95</f>
+        <f t="shared" si="2"/>
         <v>4430</v>
       </c>
       <c r="I95" s="30" t="s">
@@ -15513,7 +15519,7 @@
         <v>670000</v>
       </c>
       <c r="H96" s="31">
-        <f>G96*E96</f>
+        <f t="shared" si="2"/>
         <v>670000</v>
       </c>
       <c r="I96" s="30" t="s">
@@ -15542,7 +15548,7 @@
         <v>670</v>
       </c>
       <c r="H97" s="31">
-        <f>G97*E97</f>
+        <f t="shared" si="2"/>
         <v>7879.2</v>
       </c>
       <c r="I97" s="30" t="s">
@@ -15569,7 +15575,7 @@
         <v>9.99</v>
       </c>
       <c r="H98" s="31">
-        <f>G98*E98</f>
+        <f t="shared" ref="H98:H129" si="3">G98*E98</f>
         <v>5994</v>
       </c>
       <c r="I98" s="30" t="s">
@@ -15599,7 +15605,7 @@
       <c r="F100" s="27"/>
       <c r="H100" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>5773126.7741069021</v>
+        <v>5773376.7741069021</v>
       </c>
     </row>
     <row r="101" spans="2:12" x14ac:dyDescent="0.25">
@@ -15636,7 +15642,7 @@
       </c>
       <c r="D2" s="60">
         <f>'DPA IV'!H100</f>
-        <v>5773126.7741069021</v>
+        <v>5773376.7741069021</v>
       </c>
     </row>
     <row r="3" spans="3:7" x14ac:dyDescent="0.25">
@@ -15668,8 +15674,8 @@
         <v>992504</v>
       </c>
       <c r="E5" s="64">
-        <f>D5/$D$2</f>
-        <v>0.17191792919765556</v>
+        <f t="shared" ref="E5:E21" si="0">D5/$D$2</f>
+        <v>0.17191048477059301</v>
       </c>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
@@ -15683,8 +15689,8 @@
         <v>908615.35</v>
       </c>
       <c r="E6" s="64">
-        <f>D6/$D$2</f>
-        <v>0.15738704268114084</v>
+        <f t="shared" si="0"/>
+        <v>0.15738022747364447</v>
       </c>
       <c r="F6" s="14"/>
       <c r="G6" s="14"/>
@@ -15698,8 +15704,8 @@
         <v>893801.0010256411</v>
       </c>
       <c r="E7" s="64">
-        <f>D7/$D$2</f>
-        <v>0.15482095509047805</v>
+        <f t="shared" si="0"/>
+        <v>0.1548142510002572</v>
       </c>
       <c r="F7" s="61"/>
       <c r="G7" s="14"/>
@@ -15713,8 +15719,8 @@
         <v>795383.2</v>
       </c>
       <c r="E8" s="64">
-        <f>D8/$D$2</f>
-        <v>0.1377733819335788</v>
+        <f t="shared" si="0"/>
+        <v>0.13776741604102907</v>
       </c>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
@@ -15725,11 +15731,11 @@
       </c>
       <c r="D9" s="58">
         <f>SUMIF(Tabela24[Aplicação],"AVCB",Tabela24[Preço Total])</f>
-        <v>494682</v>
+        <v>0</v>
       </c>
       <c r="E9" s="64">
-        <f>D9/$D$2</f>
-        <v>8.5687014915158677E-2</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="F9" s="61"/>
       <c r="G9" s="14"/>
@@ -15740,11 +15746,11 @@
       </c>
       <c r="D10" s="58">
         <f>SUMIF(Tabela24[Aplicação],"Fundação",Tabela24[Preço Total])</f>
-        <v>428702.4</v>
+        <v>428952.4</v>
       </c>
       <c r="E10" s="64">
-        <f>D10/$D$2</f>
-        <v>7.425826883323898E-2</v>
+        <f t="shared" si="0"/>
+        <v>7.4298355500339877E-2</v>
       </c>
       <c r="F10" s="61"/>
       <c r="G10" s="14"/>
@@ -15758,8 +15764,8 @@
         <v>387429.61538461538</v>
       </c>
       <c r="E11" s="64">
-        <f>D11/$D$2</f>
-        <v>6.7109147355342874E-2</v>
+        <f t="shared" si="0"/>
+        <v>6.7106241380642931E-2</v>
       </c>
       <c r="F11" s="61"/>
       <c r="G11" s="14"/>
@@ -15773,8 +15779,8 @@
         <v>353535.24615384615</v>
       </c>
       <c r="E12" s="64">
-        <f>D12/$D$2</f>
-        <v>6.1238088125743224E-2</v>
+        <f t="shared" si="0"/>
+        <v>6.1235436380909919E-2</v>
       </c>
       <c r="F12" s="14"/>
       <c r="G12" s="14"/>
@@ -15788,8 +15794,8 @@
         <v>117450</v>
       </c>
       <c r="E13" s="64">
-        <f>D13/$D$2</f>
-        <v>2.034426136747524E-2</v>
+        <f t="shared" si="0"/>
+        <v>2.0343380415903764E-2</v>
       </c>
       <c r="F13" s="14"/>
       <c r="G13" s="14"/>
@@ -15803,8 +15809,8 @@
         <v>103849.27999999998</v>
       </c>
       <c r="E14" s="64">
-        <f>D14/$D$2</f>
-        <v>1.7988394168958012E-2</v>
+        <f t="shared" si="0"/>
+        <v>1.7987615231653521E-2</v>
       </c>
       <c r="F14" s="61"/>
       <c r="G14" s="14"/>
@@ -15818,8 +15824,8 @@
         <v>102596.93156880001</v>
       </c>
       <c r="E15" s="64">
-        <f>D15/$D$2</f>
-        <v>1.7771466933474998E-2</v>
+        <f t="shared" si="0"/>
+        <v>1.7770697389600212E-2</v>
       </c>
       <c r="F15" s="61"/>
       <c r="G15" s="14"/>
@@ -15833,8 +15839,8 @@
         <v>85555.13</v>
       </c>
       <c r="E16" s="64">
-        <f>D16/$D$2</f>
-        <v>1.4819548114502529E-2</v>
+        <f t="shared" si="0"/>
+        <v>1.4818906395249899E-2</v>
       </c>
       <c r="F16" s="14"/>
       <c r="G16" s="14"/>
@@ -15848,8 +15854,8 @@
         <v>44742.619974000001</v>
       </c>
       <c r="E17" s="64">
-        <f>D17/$D$2</f>
-        <v>7.7501537251313257E-3</v>
+        <f t="shared" si="0"/>
+        <v>7.74981812631159E-3</v>
       </c>
       <c r="F17" s="61"/>
       <c r="G17" s="14"/>
@@ -15863,8 +15869,8 @@
         <v>42000</v>
       </c>
       <c r="E18" s="64">
-        <f>D18/$D$2</f>
-        <v>7.2750870790460626E-3</v>
+        <f t="shared" si="0"/>
+        <v>7.2747720516641813E-3</v>
       </c>
       <c r="F18" s="14"/>
       <c r="G18" s="14"/>
@@ -15878,8 +15884,8 @@
         <v>16920</v>
       </c>
       <c r="E19" s="64">
-        <f>D19/$D$2</f>
-        <v>2.9308207947014138E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.9306938836704275E-3</v>
       </c>
       <c r="F19" s="61"/>
       <c r="G19" s="14"/>
@@ -15893,8 +15899,8 @@
         <v>5360</v>
       </c>
       <c r="E20" s="64">
-        <f>D20/$D$2</f>
-        <v>9.2843968437349752E-4</v>
+        <f t="shared" si="0"/>
+        <v>9.2839948087904784E-4</v>
       </c>
       <c r="F20" s="61"/>
       <c r="G20" s="14"/>
@@ -15908,7 +15914,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="64">
-        <f>D21/$D$2</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F21" s="14"/>
@@ -15931,7 +15937,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:I81"/>
+  <dimension ref="B3:I82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.28515625" style="47" customWidth="1"/>
@@ -15984,7 +15990,7 @@
       </c>
       <c r="F4" s="20"/>
       <c r="G4" s="20">
-        <f t="shared" ref="G4:G21" si="0">F4*D4</f>
+        <f>F4*D4</f>
         <v>0</v>
       </c>
       <c r="H4" s="50" t="s">
@@ -16012,11 +16018,11 @@
         <v>421112</v>
       </c>
       <c r="G5" s="25">
-        <f t="shared" si="0"/>
+        <f>F5*D5</f>
         <v>421112</v>
       </c>
       <c r="H5" s="53" t="s">
-        <v>779</v>
+        <v>921</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
@@ -16036,11 +16042,11 @@
         <v>6650</v>
       </c>
       <c r="G6" s="25">
-        <f t="shared" si="0"/>
+        <f>F6*D6</f>
         <v>6650</v>
       </c>
       <c r="H6" s="53" t="s">
-        <v>779</v>
+        <v>921</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
@@ -16060,7 +16066,7 @@
         <v>198.72</v>
       </c>
       <c r="G7" s="25">
-        <f t="shared" si="0"/>
+        <f>F7*D7</f>
         <v>1987.2</v>
       </c>
       <c r="H7" s="53" t="s">
@@ -16084,7 +16090,7 @@
         <v>484.24</v>
       </c>
       <c r="G8" s="25">
-        <f t="shared" si="0"/>
+        <f>F8*D8</f>
         <v>12106</v>
       </c>
       <c r="H8" s="53" t="s">
@@ -16108,7 +16114,7 @@
         <v>703.93</v>
       </c>
       <c r="G9" s="25">
-        <f t="shared" si="0"/>
+        <f>F9*D9</f>
         <v>5631.44</v>
       </c>
       <c r="H9" s="53" t="s">
@@ -16132,7 +16138,7 @@
         <v>49.05</v>
       </c>
       <c r="G10" s="25">
-        <f t="shared" si="0"/>
+        <f>F10*D10</f>
         <v>1177.1999999999998</v>
       </c>
       <c r="H10" s="53" t="s">
@@ -16156,7 +16162,7 @@
         <v>151.19999999999999</v>
       </c>
       <c r="G11" s="25">
-        <f t="shared" si="0"/>
+        <f>F11*D11</f>
         <v>302.39999999999998</v>
       </c>
       <c r="H11" s="53" t="s">
@@ -16180,7 +16186,7 @@
         <v>48.38</v>
       </c>
       <c r="G12" s="25">
-        <f t="shared" si="0"/>
+        <f>F12*D12</f>
         <v>96.76</v>
       </c>
       <c r="H12" s="53" t="s">
@@ -16204,7 +16210,7 @@
         <v>27.14</v>
       </c>
       <c r="G13" s="25">
-        <f t="shared" si="0"/>
+        <f>F13*D13</f>
         <v>325.68</v>
       </c>
       <c r="H13" s="53" t="s">
@@ -16215,24 +16221,24 @@
       <c r="B14" s="48">
         <v>11</v>
       </c>
-      <c r="C14" s="42" t="s">
-        <v>850</v>
-      </c>
-      <c r="D14" s="43">
-        <v>10</v>
-      </c>
-      <c r="E14" s="43" t="s">
+      <c r="C14" s="52" t="s">
+        <v>816</v>
+      </c>
+      <c r="D14" s="53">
+        <v>1</v>
+      </c>
+      <c r="E14" s="53" t="s">
         <v>760</v>
       </c>
-      <c r="F14" s="31">
-        <v>420</v>
-      </c>
-      <c r="G14" s="31">
-        <f t="shared" si="0"/>
-        <v>4200</v>
+      <c r="F14" s="25">
+        <v>1056959.67</v>
+      </c>
+      <c r="G14" s="25">
+        <f>F14*D14</f>
+        <v>1056959.67</v>
       </c>
       <c r="H14" s="53" t="s">
-        <v>903</v>
+        <v>892</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
@@ -16240,43 +16246,48 @@
         <v>12</v>
       </c>
       <c r="C15" s="52" t="s">
-        <v>899</v>
-      </c>
-      <c r="D15" s="43">
-        <v>200</v>
-      </c>
-      <c r="E15" s="43" t="s">
-        <v>761</v>
-      </c>
-      <c r="F15" s="31">
-        <v>15</v>
-      </c>
-      <c r="G15" s="31">
-        <f t="shared" si="0"/>
-        <v>3000</v>
+        <v>893</v>
+      </c>
+      <c r="D15" s="53">
+        <v>1</v>
+      </c>
+      <c r="E15" s="53" t="s">
+        <v>760</v>
+      </c>
+      <c r="F15" s="25">
+        <v>163890</v>
+      </c>
+      <c r="G15" s="25">
+        <f>F15*D15</f>
+        <v>163890</v>
       </c>
       <c r="H15" s="53" t="s">
-        <v>903</v>
+        <v>892</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="48">
         <v>13</v>
       </c>
-      <c r="C16" s="54" t="s">
-        <v>851</v>
-      </c>
-      <c r="D16" s="55"/>
-      <c r="E16" s="55" t="s">
+      <c r="C16" s="52" t="s">
+        <v>805</v>
+      </c>
+      <c r="D16" s="56">
+        <f>50*1.02</f>
+        <v>51</v>
+      </c>
+      <c r="E16" s="53" t="s">
         <v>760</v>
       </c>
-      <c r="F16" s="37"/>
-      <c r="G16" s="37">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H16" s="48" t="s">
-        <v>903</v>
+      <c r="F16" s="25">
+        <v>243.39</v>
+      </c>
+      <c r="G16" s="25">
+        <f>F16*D16</f>
+        <v>12412.89</v>
+      </c>
+      <c r="H16" s="53" t="s">
+        <v>806</v>
       </c>
       <c r="I16" s="51" t="s">
         <v>852</v>
@@ -16287,23 +16298,23 @@
         <v>14</v>
       </c>
       <c r="C17" s="52" t="s">
-        <v>816</v>
-      </c>
-      <c r="D17" s="53">
-        <v>1</v>
+        <v>807</v>
+      </c>
+      <c r="D17" s="56">
+        <v>51</v>
       </c>
       <c r="E17" s="53" t="s">
         <v>760</v>
       </c>
       <c r="F17" s="25">
-        <v>1056959.67</v>
+        <v>119.7</v>
       </c>
       <c r="G17" s="25">
-        <f t="shared" si="0"/>
-        <v>1056959.67</v>
+        <f>F17*D17</f>
+        <v>6104.7</v>
       </c>
       <c r="H17" s="53" t="s">
-        <v>892</v>
+        <v>806</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
@@ -16311,23 +16322,24 @@
         <v>15</v>
       </c>
       <c r="C18" s="52" t="s">
-        <v>893</v>
-      </c>
-      <c r="D18" s="53">
-        <v>1</v>
+        <v>805</v>
+      </c>
+      <c r="D18" s="56">
+        <f>(40*1.02)*4</f>
+        <v>163.19999999999999</v>
       </c>
       <c r="E18" s="53" t="s">
         <v>760</v>
       </c>
       <c r="F18" s="25">
-        <v>163890</v>
+        <v>243.39</v>
       </c>
       <c r="G18" s="25">
-        <f t="shared" si="0"/>
-        <v>163890</v>
+        <f>F18*D18</f>
+        <v>39721.247999999992</v>
       </c>
       <c r="H18" s="53" t="s">
-        <v>892</v>
+        <v>774</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
@@ -16335,72 +16347,70 @@
         <v>16</v>
       </c>
       <c r="C19" s="52" t="s">
-        <v>805</v>
-      </c>
-      <c r="D19" s="56">
-        <f>50*1.02</f>
-        <v>51</v>
-      </c>
-      <c r="E19" s="53" t="s">
-        <v>760</v>
-      </c>
-      <c r="F19" s="25">
-        <v>243.39</v>
-      </c>
-      <c r="G19" s="25">
-        <f t="shared" si="0"/>
-        <v>12412.89</v>
-      </c>
-      <c r="H19" s="53" t="s">
-        <v>806</v>
+        <v>875</v>
+      </c>
+      <c r="D19" s="53">
+        <v>180</v>
+      </c>
+      <c r="E19" s="43" t="s">
+        <v>761</v>
+      </c>
+      <c r="F19" s="31">
+        <v>23.90625</v>
+      </c>
+      <c r="G19" s="31">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>4303.125</v>
+      </c>
+      <c r="H19" s="43" t="s">
+        <v>774</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="48">
         <v>17</v>
       </c>
-      <c r="C20" s="52" t="s">
-        <v>807</v>
-      </c>
-      <c r="D20" s="56">
-        <v>51</v>
-      </c>
-      <c r="E20" s="53" t="s">
-        <v>760</v>
-      </c>
-      <c r="F20" s="25">
-        <v>119.7</v>
-      </c>
-      <c r="G20" s="25">
-        <f t="shared" si="0"/>
-        <v>6104.7</v>
-      </c>
-      <c r="H20" s="53" t="s">
-        <v>806</v>
+      <c r="C20" s="42" t="s">
+        <v>778</v>
+      </c>
+      <c r="D20" s="43">
+        <v>50</v>
+      </c>
+      <c r="E20" s="43" t="s">
+        <v>761</v>
+      </c>
+      <c r="F20" s="31">
+        <v>32</v>
+      </c>
+      <c r="G20" s="31">
+        <f>F20*D20</f>
+        <v>1600</v>
+      </c>
+      <c r="H20" s="43" t="s">
+        <v>774</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="48">
         <v>18</v>
       </c>
-      <c r="C21" s="52" t="s">
-        <v>805</v>
-      </c>
-      <c r="D21" s="56">
-        <f>(40*1.02)*4</f>
-        <v>163.19999999999999</v>
-      </c>
-      <c r="E21" s="53" t="s">
-        <v>760</v>
-      </c>
-      <c r="F21" s="25">
-        <v>243.39</v>
-      </c>
-      <c r="G21" s="25">
-        <f t="shared" si="0"/>
-        <v>39721.247999999992</v>
-      </c>
-      <c r="H21" s="53" t="s">
+      <c r="C21" s="42" t="s">
+        <v>871</v>
+      </c>
+      <c r="D21" s="43">
+        <v>6</v>
+      </c>
+      <c r="E21" s="43" t="s">
+        <v>761</v>
+      </c>
+      <c r="F21" s="31">
+        <v>419</v>
+      </c>
+      <c r="G21" s="31">
+        <f>F21*D21</f>
+        <v>2514</v>
+      </c>
+      <c r="H21" s="43" t="s">
         <v>774</v>
       </c>
     </row>
@@ -16408,21 +16418,22 @@
       <c r="B22" s="48">
         <v>19</v>
       </c>
-      <c r="C22" s="52" t="s">
-        <v>875</v>
-      </c>
-      <c r="D22" s="53">
-        <v>180</v>
+      <c r="C22" s="42" t="s">
+        <v>813</v>
+      </c>
+      <c r="D22" s="43">
+        <v>1</v>
       </c>
       <c r="E22" s="43" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="F22" s="31">
-        <v>23.90625</v>
+        <f>23500+7500</f>
+        <v>31000</v>
       </c>
       <c r="G22" s="31">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>4303.125</v>
+        <f>F22*D22</f>
+        <v>31000</v>
       </c>
       <c r="H22" s="43" t="s">
         <v>774</v>
@@ -16432,96 +16443,95 @@
       <c r="B23" s="48">
         <v>20</v>
       </c>
-      <c r="C23" s="42" t="s">
-        <v>778</v>
-      </c>
-      <c r="D23" s="43">
-        <v>50</v>
-      </c>
-      <c r="E23" s="43" t="s">
-        <v>761</v>
-      </c>
-      <c r="F23" s="31">
-        <v>32</v>
-      </c>
-      <c r="G23" s="31">
-        <f>F23*D23</f>
-        <v>1600</v>
-      </c>
-      <c r="H23" s="43" t="s">
-        <v>774</v>
+      <c r="C23" s="44" t="s">
+        <v>790</v>
+      </c>
+      <c r="D23" s="45">
+        <v>4</v>
+      </c>
+      <c r="E23" s="45" t="s">
+        <v>760</v>
+      </c>
+      <c r="F23" s="46">
+        <v>1500</v>
+      </c>
+      <c r="G23" s="46">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>6000</v>
+      </c>
+      <c r="H23" s="45" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="48">
         <v>21</v>
       </c>
-      <c r="C24" s="42" t="s">
-        <v>871</v>
-      </c>
-      <c r="D24" s="43">
-        <v>6</v>
-      </c>
-      <c r="E24" s="43" t="s">
-        <v>761</v>
-      </c>
-      <c r="F24" s="31">
-        <v>419</v>
-      </c>
-      <c r="G24" s="31">
+      <c r="C24" s="52" t="s">
+        <v>789</v>
+      </c>
+      <c r="D24" s="53">
+        <v>1</v>
+      </c>
+      <c r="E24" s="53" t="s">
+        <v>760</v>
+      </c>
+      <c r="F24" s="25">
+        <v>4500</v>
+      </c>
+      <c r="G24" s="25">
         <f>F24*D24</f>
-        <v>2514</v>
-      </c>
-      <c r="H24" s="43" t="s">
-        <v>774</v>
+        <v>4500</v>
+      </c>
+      <c r="H24" s="53" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="48">
         <v>22</v>
       </c>
-      <c r="C25" s="42" t="s">
-        <v>813</v>
-      </c>
-      <c r="D25" s="43">
-        <v>1</v>
-      </c>
-      <c r="E25" s="43" t="s">
-        <v>760</v>
-      </c>
-      <c r="F25" s="31">
-        <f>23500+7500</f>
-        <v>31000</v>
-      </c>
-      <c r="G25" s="31">
+      <c r="C25" s="52" t="s">
+        <v>769</v>
+      </c>
+      <c r="D25" s="53">
+        <v>2100</v>
+      </c>
+      <c r="E25" s="53" t="s">
+        <v>811</v>
+      </c>
+      <c r="F25" s="25">
+        <v>9.65</v>
+      </c>
+      <c r="G25" s="25">
         <f>F25*D25</f>
-        <v>31000</v>
-      </c>
-      <c r="H25" s="43" t="s">
-        <v>774</v>
+        <v>20265</v>
+      </c>
+      <c r="H25" s="53" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="48">
         <v>23</v>
       </c>
-      <c r="C26" s="44" t="s">
-        <v>790</v>
-      </c>
-      <c r="D26" s="45">
-        <v>4</v>
-      </c>
-      <c r="E26" s="45" t="s">
-        <v>760</v>
-      </c>
-      <c r="F26" s="46">
-        <v>1500</v>
-      </c>
-      <c r="G26" s="46">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>6000</v>
-      </c>
-      <c r="H26" s="45" t="s">
+      <c r="C26" s="52" t="s">
+        <v>770</v>
+      </c>
+      <c r="D26" s="53">
+        <v>2300</v>
+      </c>
+      <c r="E26" s="53" t="s">
+        <v>811</v>
+      </c>
+      <c r="F26" s="25">
+        <v>9.65</v>
+      </c>
+      <c r="G26" s="25">
+        <f>F26*D26</f>
+        <v>22195</v>
+      </c>
+      <c r="H26" s="53" t="s">
         <v>771</v>
       </c>
     </row>
@@ -16530,7 +16540,7 @@
         <v>24</v>
       </c>
       <c r="C27" s="52" t="s">
-        <v>789</v>
+        <v>808</v>
       </c>
       <c r="D27" s="53">
         <v>1</v>
@@ -16539,11 +16549,11 @@
         <v>760</v>
       </c>
       <c r="F27" s="25">
-        <v>4500</v>
+        <v>51500</v>
       </c>
       <c r="G27" s="25">
-        <f t="shared" ref="G27:G44" si="1">F27*D27</f>
-        <v>4500</v>
+        <f>F27*D27</f>
+        <v>51500</v>
       </c>
       <c r="H27" s="53" t="s">
         <v>771</v>
@@ -16554,20 +16564,20 @@
         <v>25</v>
       </c>
       <c r="C28" s="52" t="s">
-        <v>769</v>
-      </c>
-      <c r="D28" s="53">
-        <v>2100</v>
+        <v>809</v>
+      </c>
+      <c r="D28" s="56">
+        <v>46.8</v>
       </c>
       <c r="E28" s="53" t="s">
-        <v>811</v>
+        <v>759</v>
       </c>
       <c r="F28" s="25">
-        <v>9.65</v>
+        <v>670</v>
       </c>
       <c r="G28" s="25">
-        <f t="shared" si="1"/>
-        <v>20265</v>
+        <f>F28*D28</f>
+        <v>31355.999999999996</v>
       </c>
       <c r="H28" s="53" t="s">
         <v>771</v>
@@ -16581,20 +16591,20 @@
         <v>26</v>
       </c>
       <c r="C29" s="52" t="s">
-        <v>770</v>
-      </c>
-      <c r="D29" s="53">
-        <v>2300</v>
+        <v>810</v>
+      </c>
+      <c r="D29" s="56">
+        <v>37.200000000000003</v>
       </c>
       <c r="E29" s="53" t="s">
-        <v>811</v>
+        <v>759</v>
       </c>
       <c r="F29" s="25">
-        <v>9.65</v>
+        <v>670</v>
       </c>
       <c r="G29" s="25">
-        <f t="shared" si="1"/>
-        <v>22195</v>
+        <f>F29*D29</f>
+        <v>24924.000000000004</v>
       </c>
       <c r="H29" s="53" t="s">
         <v>771</v>
@@ -16608,20 +16618,20 @@
         <v>27</v>
       </c>
       <c r="C30" s="52" t="s">
-        <v>808</v>
+        <v>844</v>
       </c>
       <c r="D30" s="53">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="E30" s="53" t="s">
         <v>760</v>
       </c>
       <c r="F30" s="25">
-        <v>51500</v>
+        <v>120</v>
       </c>
       <c r="G30" s="25">
-        <f t="shared" si="1"/>
-        <v>51500</v>
+        <f>F30*D30</f>
+        <v>3600</v>
       </c>
       <c r="H30" s="53" t="s">
         <v>771</v>
@@ -16631,24 +16641,24 @@
       <c r="B31" s="48">
         <v>28</v>
       </c>
-      <c r="C31" s="52" t="s">
-        <v>809</v>
-      </c>
-      <c r="D31" s="56">
-        <v>46.8</v>
-      </c>
-      <c r="E31" s="53" t="s">
-        <v>759</v>
-      </c>
-      <c r="F31" s="25">
-        <v>670</v>
-      </c>
-      <c r="G31" s="25">
-        <f t="shared" si="1"/>
-        <v>31355.999999999996</v>
+      <c r="C31" s="42" t="s">
+        <v>850</v>
+      </c>
+      <c r="D31" s="43">
+        <v>10</v>
+      </c>
+      <c r="E31" s="43" t="s">
+        <v>760</v>
+      </c>
+      <c r="F31" s="31">
+        <v>420</v>
+      </c>
+      <c r="G31" s="31">
+        <f>F31*D31</f>
+        <v>4200</v>
       </c>
       <c r="H31" s="53" t="s">
-        <v>771</v>
+        <v>903</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
@@ -16656,47 +16666,43 @@
         <v>29</v>
       </c>
       <c r="C32" s="52" t="s">
-        <v>810</v>
-      </c>
-      <c r="D32" s="56">
-        <v>37.200000000000003</v>
-      </c>
-      <c r="E32" s="53" t="s">
-        <v>759</v>
-      </c>
-      <c r="F32" s="25">
-        <v>670</v>
-      </c>
-      <c r="G32" s="25">
-        <f t="shared" si="1"/>
-        <v>24924.000000000004</v>
+        <v>899</v>
+      </c>
+      <c r="D32" s="43">
+        <v>200</v>
+      </c>
+      <c r="E32" s="43" t="s">
+        <v>761</v>
+      </c>
+      <c r="F32" s="31">
+        <v>15</v>
+      </c>
+      <c r="G32" s="31">
+        <f>F32*D32</f>
+        <v>3000</v>
       </c>
       <c r="H32" s="53" t="s">
-        <v>771</v>
+        <v>903</v>
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="48">
         <v>30</v>
       </c>
-      <c r="C33" s="52" t="s">
-        <v>844</v>
-      </c>
-      <c r="D33" s="53">
-        <v>30</v>
-      </c>
-      <c r="E33" s="53" t="s">
+      <c r="C33" s="54" t="s">
+        <v>851</v>
+      </c>
+      <c r="D33" s="55"/>
+      <c r="E33" s="55" t="s">
         <v>760</v>
       </c>
-      <c r="F33" s="25">
-        <v>120</v>
-      </c>
-      <c r="G33" s="25">
-        <f t="shared" si="1"/>
-        <v>3600</v>
-      </c>
-      <c r="H33" s="53" t="s">
-        <v>771</v>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37">
+        <f>F33*D33</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="48" t="s">
+        <v>903</v>
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
@@ -16716,7 +16722,7 @@
         <v>280</v>
       </c>
       <c r="G34" s="31">
-        <f t="shared" si="1"/>
+        <f>F34*D34</f>
         <v>2240</v>
       </c>
       <c r="H34" s="43" t="s">
@@ -16740,7 +16746,7 @@
         <v>380</v>
       </c>
       <c r="G35" s="31">
-        <f t="shared" si="1"/>
+        <f>F35*D35</f>
         <v>1900</v>
       </c>
       <c r="H35" s="43" t="s">
@@ -16764,7 +16770,7 @@
         <v>290</v>
       </c>
       <c r="G36" s="31">
-        <f t="shared" si="1"/>
+        <f>F36*D36</f>
         <v>580</v>
       </c>
       <c r="H36" s="43" t="s">
@@ -16788,7 +16794,7 @@
         <v>290</v>
       </c>
       <c r="G37" s="31">
-        <f t="shared" si="1"/>
+        <f>F37*D37</f>
         <v>580</v>
       </c>
       <c r="H37" s="43" t="s">
@@ -16813,7 +16819,7 @@
         <v>670</v>
       </c>
       <c r="G38" s="25">
-        <f t="shared" si="1"/>
+        <f>F38*D38</f>
         <v>211050</v>
       </c>
       <c r="H38" s="53" t="s">
@@ -16838,7 +16844,7 @@
         <v>220.5</v>
       </c>
       <c r="G39" s="25">
-        <f t="shared" si="1"/>
+        <f>F39*D39</f>
         <v>67846.153846153844</v>
       </c>
       <c r="H39" s="53" t="s">
@@ -16862,7 +16868,7 @@
         <v>56.2</v>
       </c>
       <c r="G40" s="25">
-        <f t="shared" si="1"/>
+        <f>F40*D40</f>
         <v>9385.4</v>
       </c>
       <c r="H40" s="53" t="s">
@@ -16886,7 +16892,7 @@
         <v>7.3</v>
       </c>
       <c r="G41" s="25">
-        <f t="shared" si="1"/>
+        <f>F41*D41</f>
         <v>7300</v>
       </c>
       <c r="H41" s="53" t="s">
@@ -16910,7 +16916,7 @@
         <v>50</v>
       </c>
       <c r="G42" s="25">
-        <f t="shared" si="1"/>
+        <f>F42*D42</f>
         <v>15750</v>
       </c>
       <c r="H42" s="53" t="s">
@@ -16934,7 +16940,7 @@
         <v>49800</v>
       </c>
       <c r="G43" s="25">
-        <f t="shared" si="1"/>
+        <f>F43*D43</f>
         <v>49800</v>
       </c>
       <c r="H43" s="53" t="s">
@@ -16946,7 +16952,7 @@
         <v>41</v>
       </c>
       <c r="C44" s="52" t="s">
-        <v>786</v>
+        <v>920</v>
       </c>
       <c r="D44" s="53">
         <v>1</v>
@@ -16955,49 +16961,49 @@
         <v>760</v>
       </c>
       <c r="F44" s="25">
-        <v>404191.96</v>
+        <v>15000</v>
       </c>
       <c r="G44" s="25">
-        <f t="shared" si="1"/>
-        <v>404191.96</v>
+        <f>F44*D44</f>
+        <v>15000</v>
       </c>
       <c r="H44" s="53" t="s">
-        <v>419</v>
+        <v>837</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B45" s="48">
         <v>42</v>
       </c>
-      <c r="C45" s="57" t="s">
-        <v>845</v>
+      <c r="C45" s="52" t="s">
+        <v>786</v>
       </c>
       <c r="D45" s="53">
-        <v>1455.89</v>
+        <v>1</v>
       </c>
       <c r="E45" s="53" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="F45" s="25">
-        <v>95.9</v>
+        <v>404191.96</v>
       </c>
       <c r="G45" s="25">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>139619.85100000002</v>
+        <f>F45*D45</f>
+        <v>404191.96</v>
       </c>
       <c r="H45" s="53" t="s">
-        <v>791</v>
+        <v>837</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" s="48">
         <v>43</v>
       </c>
-      <c r="C46" s="52" t="s">
-        <v>846</v>
+      <c r="C46" s="57" t="s">
+        <v>845</v>
       </c>
       <c r="D46" s="53">
-        <v>706.94</v>
+        <v>1455.89</v>
       </c>
       <c r="E46" s="53" t="s">
         <v>761</v>
@@ -17007,7 +17013,7 @@
       </c>
       <c r="G46" s="25">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>67795.546000000002</v>
+        <v>139619.85100000002</v>
       </c>
       <c r="H46" s="53" t="s">
         <v>791</v>
@@ -17017,21 +17023,21 @@
       <c r="B47" s="48">
         <v>44</v>
       </c>
-      <c r="C47" s="44" t="s">
-        <v>847</v>
+      <c r="C47" s="52" t="s">
+        <v>846</v>
       </c>
       <c r="D47" s="53">
-        <v>44</v>
+        <v>706.94</v>
       </c>
       <c r="E47" s="53" t="s">
-        <v>818</v>
+        <v>761</v>
       </c>
       <c r="F47" s="25">
-        <v>95</v>
+        <v>95.9</v>
       </c>
       <c r="G47" s="25">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>4180</v>
+        <v>67795.546000000002</v>
       </c>
       <c r="H47" s="53" t="s">
         <v>791</v>
@@ -17042,20 +17048,20 @@
         <v>45</v>
       </c>
       <c r="C48" s="44" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="D48" s="53">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="E48" s="53" t="s">
         <v>818</v>
       </c>
       <c r="F48" s="25">
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="G48" s="25">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>105</v>
+        <v>4180</v>
       </c>
       <c r="H48" s="53" t="s">
         <v>791</v>
@@ -17066,20 +17072,20 @@
         <v>46</v>
       </c>
       <c r="C49" s="44" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="D49" s="53">
-        <v>126</v>
+        <v>3</v>
       </c>
       <c r="E49" s="53" t="s">
-        <v>760</v>
+        <v>818</v>
       </c>
       <c r="F49" s="25">
-        <v>25.9</v>
+        <v>35</v>
       </c>
       <c r="G49" s="25">
         <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>3263.3999999999996</v>
+        <v>105</v>
       </c>
       <c r="H49" s="53" t="s">
         <v>791</v>
@@ -17090,20 +17096,20 @@
         <v>47</v>
       </c>
       <c r="C50" s="44" t="s">
-        <v>817</v>
+        <v>849</v>
       </c>
       <c r="D50" s="53">
-        <v>1</v>
+        <v>126</v>
       </c>
       <c r="E50" s="53" t="s">
         <v>760</v>
       </c>
       <c r="F50" s="25">
-        <v>1750</v>
+        <v>25.9</v>
       </c>
       <c r="G50" s="25">
-        <f>F50*D50</f>
-        <v>1750</v>
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>3263.3999999999996</v>
       </c>
       <c r="H50" s="53" t="s">
         <v>791</v>
@@ -17113,8 +17119,8 @@
       <c r="B51" s="48">
         <v>48</v>
       </c>
-      <c r="C51" s="52" t="s">
-        <v>781</v>
+      <c r="C51" s="44" t="s">
+        <v>817</v>
       </c>
       <c r="D51" s="53">
         <v>1</v>
@@ -17123,48 +17129,63 @@
         <v>760</v>
       </c>
       <c r="F51" s="25">
-        <v>174417.38</v>
+        <v>1750</v>
       </c>
       <c r="G51" s="25">
         <f>F51*D51</f>
-        <v>174417.38</v>
+        <v>1750</v>
       </c>
       <c r="H51" s="53" t="s">
-        <v>780</v>
+        <v>791</v>
       </c>
     </row>
     <row r="52" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B52" s="48">
-        <v>51</v>
-      </c>
-      <c r="C52" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="C52" s="52" t="s">
+        <v>781</v>
+      </c>
+      <c r="D52" s="53">
+        <v>1</v>
+      </c>
+      <c r="E52" s="53" t="s">
+        <v>760</v>
+      </c>
+      <c r="F52" s="25">
+        <v>174417.38</v>
+      </c>
+      <c r="G52" s="25">
+        <f>F52*D52</f>
+        <v>174417.38</v>
+      </c>
+      <c r="H52" s="53" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B53" s="48">
+        <v>50</v>
+      </c>
+      <c r="C53" s="42" t="s">
         <v>814</v>
       </c>
-      <c r="D52" s="43">
-        <v>1</v>
-      </c>
-      <c r="E52" s="43" t="s">
+      <c r="D53" s="43">
+        <v>1</v>
+      </c>
+      <c r="E53" s="43" t="s">
         <v>760</v>
       </c>
-      <c r="F52" s="31">
+      <c r="F53" s="31">
         <v>5000</v>
       </c>
-      <c r="G52" s="31">
-        <f>F52*D52</f>
+      <c r="G53" s="31">
+        <f>F53*D53</f>
         <v>5000</v>
       </c>
-      <c r="H52" s="43" t="s">
+      <c r="H53" s="43" t="s">
         <v>815</v>
       </c>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B53" s="50"/>
-      <c r="C53" s="49"/>
-      <c r="D53" s="50"/>
-      <c r="E53" s="50"/>
-      <c r="F53" s="20"/>
-      <c r="G53" s="20"/>
-      <c r="H53" s="50"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B54" s="50"/>
@@ -17176,15 +17197,24 @@
       <c r="H54" s="50"/>
     </row>
     <row r="55" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="G55" s="16">
+      <c r="B55" s="50"/>
+      <c r="C55" s="49"/>
+      <c r="D55" s="50"/>
+      <c r="E55" s="50"/>
+      <c r="F55" s="20"/>
+      <c r="G55" s="20"/>
+      <c r="H55" s="50"/>
+    </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G56" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>3106189.0038461541</v>
-      </c>
-    </row>
-    <row r="81" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H81" s="36">
-        <f>SUM('Expansão DMP'!G55,H77)</f>
-        <v>3106189.0038461541</v>
+        <v>3121189.0038461541</v>
+      </c>
+    </row>
+    <row r="82" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H82" s="36">
+        <f>SUM('Expansão DMP'!G56,H78)</f>
+        <v>3121189.0038461541</v>
       </c>
     </row>
   </sheetData>
@@ -17212,8 +17242,8 @@
         <v>909</v>
       </c>
       <c r="D2" s="62">
-        <f>'Expansão DMP'!G55</f>
-        <v>3106189.0038461541</v>
+        <f>'Expansão DMP'!G56</f>
+        <v>3121189.0038461541</v>
       </c>
       <c r="G2" s="14" t="s">
         <v>914</v>
@@ -17268,12 +17298,12 @@
         <v>1220849.67</v>
       </c>
       <c r="E7" s="64">
-        <f>D7/$D$2</f>
-        <v>0.39303779277059958</v>
+        <f t="shared" ref="E7:E20" si="0">D7/$D$2</f>
+        <v>0.39114890783466844</v>
       </c>
       <c r="F7" s="64">
         <f>E7</f>
-        <v>0.39303779277059958</v>
+        <v>0.39114890783466844</v>
       </c>
       <c r="G7" s="14" t="s">
         <v>914</v>
@@ -17285,15 +17315,15 @@
       </c>
       <c r="D8" s="63">
         <f>SUMIF(Tabela2[Aplicação],"AVCB",Tabela2[Preço Total])</f>
-        <v>427762</v>
+        <v>0</v>
       </c>
       <c r="E8" s="64">
-        <f>D8/$D$2</f>
-        <v>0.13771280481333728</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="F8" s="64">
-        <f>F7+E8</f>
-        <v>0.53075059758393683</v>
+        <f t="shared" ref="F8:F20" si="1">F7+E8</f>
+        <v>0.39114890783466844</v>
       </c>
       <c r="G8" s="14" t="s">
         <v>914</v>
@@ -17305,15 +17335,15 @@
       </c>
       <c r="D9" s="63">
         <f>SUMIF(Tabela2[Aplicação],"SPDA",Tabela2[Preço Total])</f>
-        <v>404191.96</v>
+        <v>0</v>
       </c>
       <c r="E9" s="64">
-        <f>D9/$D$2</f>
-        <v>0.1301247153664894</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="F9" s="64">
-        <f>F8+E9</f>
-        <v>0.66087531295042623</v>
+        <f t="shared" si="1"/>
+        <v>0.39114890783466844</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>914</v>
@@ -17328,12 +17358,12 @@
         <v>361131.5538461539</v>
       </c>
       <c r="E10" s="64">
-        <f>D10/$D$2</f>
-        <v>0.11626193814960795</v>
+        <f t="shared" si="0"/>
+        <v>0.11570319945416364</v>
       </c>
       <c r="F10" s="64">
-        <f>F9+E10</f>
-        <v>0.77713725110003418</v>
+        <f t="shared" si="1"/>
+        <v>0.50685210728883212</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>914</v>
@@ -17348,12 +17378,12 @@
         <v>216713.79700000002</v>
       </c>
       <c r="E11" s="64">
-        <f>D11/$D$2</f>
-        <v>6.9768387155984407E-2</v>
+        <f t="shared" si="0"/>
+        <v>6.9433089996456365E-2</v>
       </c>
       <c r="F11" s="64">
-        <f>F10+E11</f>
-        <v>0.84690563825601861</v>
+        <f t="shared" si="1"/>
+        <v>0.57628519728528849</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>915</v>
@@ -17368,12 +17398,12 @@
         <v>174417.38</v>
       </c>
       <c r="E12" s="64">
-        <f>D12/$D$2</f>
-        <v>5.6151567011547728E-2</v>
+        <f t="shared" si="0"/>
+        <v>5.588171039468303E-2</v>
       </c>
       <c r="F12" s="64">
-        <f>F11+E12</f>
-        <v>0.90305720526756639</v>
+        <f t="shared" si="1"/>
+        <v>0.63216690767997152</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>915</v>
@@ -17388,12 +17418,12 @@
         <v>164340</v>
       </c>
       <c r="E13" s="64">
-        <f>D13/$D$2</f>
-        <v>5.2907276342975415E-2</v>
+        <f t="shared" si="0"/>
+        <v>5.2653011335580258E-2</v>
       </c>
       <c r="F13" s="64">
-        <f>F12+E13</f>
-        <v>0.95596448161054182</v>
+        <f t="shared" si="1"/>
+        <v>0.68481991901555173</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>916</v>
@@ -17408,12 +17438,12 @@
         <v>79138.372999999992</v>
       </c>
       <c r="E14" s="64">
-        <f>D14/$D$2</f>
-        <v>2.547764250726825E-2</v>
+        <f t="shared" si="0"/>
+        <v>2.5355200502910905E-2</v>
       </c>
       <c r="F14" s="64">
-        <f>F13+E14</f>
-        <v>0.98144212411781007</v>
+        <f t="shared" si="1"/>
+        <v>0.71017511951846268</v>
       </c>
       <c r="G14" s="14" t="s">
         <v>916</v>
@@ -17428,12 +17458,12 @@
         <v>21626.68</v>
       </c>
       <c r="E15" s="64">
-        <f>D15/$D$2</f>
-        <v>6.9624481875447215E-3</v>
+        <f t="shared" si="0"/>
+        <v>6.9289876304671223E-3</v>
       </c>
       <c r="F15" s="64">
-        <f>F14+E15</f>
-        <v>0.98840457230535483</v>
+        <f t="shared" si="1"/>
+        <v>0.7171041071489298</v>
       </c>
       <c r="G15" s="14" t="s">
         <v>916</v>
@@ -17448,12 +17478,12 @@
         <v>18517.59</v>
       </c>
       <c r="E16" s="64">
-        <f>D16/$D$2</f>
-        <v>5.9615142469022645E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.9328640390509165E-3</v>
       </c>
       <c r="F16" s="64">
-        <f>F15+E16</f>
-        <v>0.99436608655225711</v>
+        <f t="shared" si="1"/>
+        <v>0.72303697118798071</v>
       </c>
       <c r="G16" s="14" t="s">
         <v>916</v>
@@ -17468,12 +17498,12 @@
         <v>7200</v>
       </c>
       <c r="E17" s="64">
-        <f>D17/$D$2</f>
-        <v>2.3179529613570828E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.3068132019969444E-3</v>
       </c>
       <c r="F17" s="64">
-        <f>F16+E17</f>
-        <v>0.99668403951361417</v>
+        <f t="shared" si="1"/>
+        <v>0.72534378438997771</v>
       </c>
       <c r="G17" s="14" t="s">
         <v>916</v>
@@ -17488,12 +17518,12 @@
         <v>5300</v>
       </c>
       <c r="E18" s="64">
-        <f>D18/$D$2</f>
-        <v>1.7062709298878527E-3</v>
+        <f t="shared" si="0"/>
+        <v>1.6980708292477509E-3</v>
       </c>
       <c r="F18" s="64">
-        <f>F17+E18</f>
-        <v>0.99839031044350202</v>
+        <f t="shared" si="1"/>
+        <v>0.72704185521922549</v>
       </c>
       <c r="G18" s="14" t="s">
         <v>916</v>
@@ -17508,12 +17538,12 @@
         <v>5000</v>
       </c>
       <c r="E19" s="64">
-        <f>D19/$D$2</f>
-        <v>1.6096895564979741E-3</v>
+        <f t="shared" si="0"/>
+        <v>1.6019536124978781E-3</v>
       </c>
       <c r="F19" s="64">
-        <f>F18+E19</f>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.72864380883172342</v>
       </c>
       <c r="G19" s="14" t="s">
         <v>916</v>
@@ -17528,12 +17558,12 @@
         <v>0</v>
       </c>
       <c r="E20" s="64">
-        <f>D20/$D$2</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F20" s="64">
-        <f>F19+E20</f>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.72864380883172342</v>
       </c>
       <c r="G20" s="14" t="s">
         <v>916</v>

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 14:00
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tiago.melo\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Engenharia\000 - Projetos e Acompanhamentos\2026 - Projetos\08 - Ampliações\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -15575,7 +15575,7 @@
         <v>9.99</v>
       </c>
       <c r="H98" s="31">
-        <f t="shared" ref="H98:H129" si="3">G98*E98</f>
+        <f t="shared" ref="H98" si="3">G98*E98</f>
         <v>5994</v>
       </c>
       <c r="I98" s="30" t="s">
@@ -15990,7 +15990,7 @@
       </c>
       <c r="F4" s="20"/>
       <c r="G4" s="20">
-        <f>F4*D4</f>
+        <f t="shared" ref="G4:G18" si="0">F4*D4</f>
         <v>0</v>
       </c>
       <c r="H4" s="50" t="s">
@@ -16018,7 +16018,7 @@
         <v>421112</v>
       </c>
       <c r="G5" s="25">
-        <f>F5*D5</f>
+        <f t="shared" si="0"/>
         <v>421112</v>
       </c>
       <c r="H5" s="53" t="s">
@@ -16042,7 +16042,7 @@
         <v>6650</v>
       </c>
       <c r="G6" s="25">
-        <f>F6*D6</f>
+        <f t="shared" si="0"/>
         <v>6650</v>
       </c>
       <c r="H6" s="53" t="s">
@@ -16066,7 +16066,7 @@
         <v>198.72</v>
       </c>
       <c r="G7" s="25">
-        <f>F7*D7</f>
+        <f t="shared" si="0"/>
         <v>1987.2</v>
       </c>
       <c r="H7" s="53" t="s">
@@ -16090,7 +16090,7 @@
         <v>484.24</v>
       </c>
       <c r="G8" s="25">
-        <f>F8*D8</f>
+        <f t="shared" si="0"/>
         <v>12106</v>
       </c>
       <c r="H8" s="53" t="s">
@@ -16114,7 +16114,7 @@
         <v>703.93</v>
       </c>
       <c r="G9" s="25">
-        <f>F9*D9</f>
+        <f t="shared" si="0"/>
         <v>5631.44</v>
       </c>
       <c r="H9" s="53" t="s">
@@ -16138,7 +16138,7 @@
         <v>49.05</v>
       </c>
       <c r="G10" s="25">
-        <f>F10*D10</f>
+        <f t="shared" si="0"/>
         <v>1177.1999999999998</v>
       </c>
       <c r="H10" s="53" t="s">
@@ -16162,7 +16162,7 @@
         <v>151.19999999999999</v>
       </c>
       <c r="G11" s="25">
-        <f>F11*D11</f>
+        <f t="shared" si="0"/>
         <v>302.39999999999998</v>
       </c>
       <c r="H11" s="53" t="s">
@@ -16186,7 +16186,7 @@
         <v>48.38</v>
       </c>
       <c r="G12" s="25">
-        <f>F12*D12</f>
+        <f t="shared" si="0"/>
         <v>96.76</v>
       </c>
       <c r="H12" s="53" t="s">
@@ -16210,7 +16210,7 @@
         <v>27.14</v>
       </c>
       <c r="G13" s="25">
-        <f>F13*D13</f>
+        <f t="shared" si="0"/>
         <v>325.68</v>
       </c>
       <c r="H13" s="53" t="s">
@@ -16234,7 +16234,7 @@
         <v>1056959.67</v>
       </c>
       <c r="G14" s="25">
-        <f>F14*D14</f>
+        <f t="shared" si="0"/>
         <v>1056959.67</v>
       </c>
       <c r="H14" s="53" t="s">
@@ -16258,7 +16258,7 @@
         <v>163890</v>
       </c>
       <c r="G15" s="25">
-        <f>F15*D15</f>
+        <f t="shared" si="0"/>
         <v>163890</v>
       </c>
       <c r="H15" s="53" t="s">
@@ -16283,7 +16283,7 @@
         <v>243.39</v>
       </c>
       <c r="G16" s="25">
-        <f>F16*D16</f>
+        <f t="shared" si="0"/>
         <v>12412.89</v>
       </c>
       <c r="H16" s="53" t="s">
@@ -16310,7 +16310,7 @@
         <v>119.7</v>
       </c>
       <c r="G17" s="25">
-        <f>F17*D17</f>
+        <f t="shared" si="0"/>
         <v>6104.7</v>
       </c>
       <c r="H17" s="53" t="s">
@@ -16335,7 +16335,7 @@
         <v>243.39</v>
       </c>
       <c r="G18" s="25">
-        <f>F18*D18</f>
+        <f t="shared" si="0"/>
         <v>39721.247999999992</v>
       </c>
       <c r="H18" s="53" t="s">
@@ -16480,7 +16480,7 @@
         <v>4500</v>
       </c>
       <c r="G24" s="25">
-        <f>F24*D24</f>
+        <f t="shared" ref="G24:G45" si="1">F24*D24</f>
         <v>4500</v>
       </c>
       <c r="H24" s="53" t="s">
@@ -16504,7 +16504,7 @@
         <v>9.65</v>
       </c>
       <c r="G25" s="25">
-        <f>F25*D25</f>
+        <f t="shared" si="1"/>
         <v>20265</v>
       </c>
       <c r="H25" s="53" t="s">
@@ -16528,7 +16528,7 @@
         <v>9.65</v>
       </c>
       <c r="G26" s="25">
-        <f>F26*D26</f>
+        <f t="shared" si="1"/>
         <v>22195</v>
       </c>
       <c r="H26" s="53" t="s">
@@ -16552,7 +16552,7 @@
         <v>51500</v>
       </c>
       <c r="G27" s="25">
-        <f>F27*D27</f>
+        <f t="shared" si="1"/>
         <v>51500</v>
       </c>
       <c r="H27" s="53" t="s">
@@ -16576,7 +16576,7 @@
         <v>670</v>
       </c>
       <c r="G28" s="25">
-        <f>F28*D28</f>
+        <f t="shared" si="1"/>
         <v>31355.999999999996</v>
       </c>
       <c r="H28" s="53" t="s">
@@ -16603,7 +16603,7 @@
         <v>670</v>
       </c>
       <c r="G29" s="25">
-        <f>F29*D29</f>
+        <f t="shared" si="1"/>
         <v>24924.000000000004</v>
       </c>
       <c r="H29" s="53" t="s">
@@ -16630,7 +16630,7 @@
         <v>120</v>
       </c>
       <c r="G30" s="25">
-        <f>F30*D30</f>
+        <f t="shared" si="1"/>
         <v>3600</v>
       </c>
       <c r="H30" s="53" t="s">
@@ -16654,7 +16654,7 @@
         <v>420</v>
       </c>
       <c r="G31" s="31">
-        <f>F31*D31</f>
+        <f t="shared" si="1"/>
         <v>4200</v>
       </c>
       <c r="H31" s="53" t="s">
@@ -16678,7 +16678,7 @@
         <v>15</v>
       </c>
       <c r="G32" s="31">
-        <f>F32*D32</f>
+        <f t="shared" si="1"/>
         <v>3000</v>
       </c>
       <c r="H32" s="53" t="s">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="F33" s="37"/>
       <c r="G33" s="37">
-        <f>F33*D33</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H33" s="48" t="s">
@@ -16722,7 +16722,7 @@
         <v>280</v>
       </c>
       <c r="G34" s="31">
-        <f>F34*D34</f>
+        <f t="shared" si="1"/>
         <v>2240</v>
       </c>
       <c r="H34" s="43" t="s">
@@ -16746,7 +16746,7 @@
         <v>380</v>
       </c>
       <c r="G35" s="31">
-        <f>F35*D35</f>
+        <f t="shared" si="1"/>
         <v>1900</v>
       </c>
       <c r="H35" s="43" t="s">
@@ -16770,7 +16770,7 @@
         <v>290</v>
       </c>
       <c r="G36" s="31">
-        <f>F36*D36</f>
+        <f t="shared" si="1"/>
         <v>580</v>
       </c>
       <c r="H36" s="43" t="s">
@@ -16794,7 +16794,7 @@
         <v>290</v>
       </c>
       <c r="G37" s="31">
-        <f>F37*D37</f>
+        <f t="shared" si="1"/>
         <v>580</v>
       </c>
       <c r="H37" s="43" t="s">
@@ -16819,7 +16819,7 @@
         <v>670</v>
       </c>
       <c r="G38" s="25">
-        <f>F38*D38</f>
+        <f t="shared" si="1"/>
         <v>211050</v>
       </c>
       <c r="H38" s="53" t="s">
@@ -16844,7 +16844,7 @@
         <v>220.5</v>
       </c>
       <c r="G39" s="25">
-        <f>F39*D39</f>
+        <f t="shared" si="1"/>
         <v>67846.153846153844</v>
       </c>
       <c r="H39" s="53" t="s">
@@ -16868,7 +16868,7 @@
         <v>56.2</v>
       </c>
       <c r="G40" s="25">
-        <f>F40*D40</f>
+        <f t="shared" si="1"/>
         <v>9385.4</v>
       </c>
       <c r="H40" s="53" t="s">
@@ -16892,7 +16892,7 @@
         <v>7.3</v>
       </c>
       <c r="G41" s="25">
-        <f>F41*D41</f>
+        <f t="shared" si="1"/>
         <v>7300</v>
       </c>
       <c r="H41" s="53" t="s">
@@ -16916,7 +16916,7 @@
         <v>50</v>
       </c>
       <c r="G42" s="25">
-        <f>F42*D42</f>
+        <f t="shared" si="1"/>
         <v>15750</v>
       </c>
       <c r="H42" s="53" t="s">
@@ -16940,7 +16940,7 @@
         <v>49800</v>
       </c>
       <c r="G43" s="25">
-        <f>F43*D43</f>
+        <f t="shared" si="1"/>
         <v>49800</v>
       </c>
       <c r="H43" s="53" t="s">
@@ -16964,7 +16964,7 @@
         <v>15000</v>
       </c>
       <c r="G44" s="25">
-        <f>F44*D44</f>
+        <f t="shared" si="1"/>
         <v>15000</v>
       </c>
       <c r="H44" s="53" t="s">
@@ -16988,7 +16988,7 @@
         <v>404191.96</v>
       </c>
       <c r="G45" s="25">
-        <f>F45*D45</f>
+        <f t="shared" si="1"/>
         <v>404191.96</v>
       </c>
       <c r="H45" s="53" t="s">

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 14:04
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -16480,7 +16480,7 @@
         <v>4500</v>
       </c>
       <c r="G24" s="25">
-        <f t="shared" ref="G24:G45" si="1">F24*D24</f>
+        <f t="shared" ref="G24:G50" si="1">F24*D24</f>
         <v>4500</v>
       </c>
       <c r="H24" s="53" t="s">
@@ -17012,7 +17012,7 @@
         <v>95.9</v>
       </c>
       <c r="G46" s="25">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <f t="shared" si="1"/>
         <v>139619.85100000002</v>
       </c>
       <c r="H46" s="53" t="s">
@@ -17036,7 +17036,7 @@
         <v>95.9</v>
       </c>
       <c r="G47" s="25">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <f t="shared" si="1"/>
         <v>67795.546000000002</v>
       </c>
       <c r="H47" s="53" t="s">
@@ -17060,7 +17060,7 @@
         <v>95</v>
       </c>
       <c r="G48" s="25">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <f t="shared" si="1"/>
         <v>4180</v>
       </c>
       <c r="H48" s="53" t="s">
@@ -17084,7 +17084,7 @@
         <v>35</v>
       </c>
       <c r="G49" s="25">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <f t="shared" si="1"/>
         <v>105</v>
       </c>
       <c r="H49" s="53" t="s">
@@ -17108,7 +17108,7 @@
         <v>25.9</v>
       </c>
       <c r="G50" s="25">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <f t="shared" si="1"/>
         <v>3263.3999999999996</v>
       </c>
       <c r="H50" s="53" t="s">

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 14:26
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2346" uniqueCount="922">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2361" uniqueCount="926">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2649,9 +2649,6 @@
     <t>Mão de obra para desmontagem da cobertura de enlonamento de caminhões e lateral do blocado</t>
   </si>
   <si>
-    <t>Categoria</t>
-  </si>
-  <si>
     <t>Rufo de acabamento galvanizado 140 x 140 x 20mm #20</t>
   </si>
   <si>
@@ -2794,6 +2791,21 @@
   </si>
   <si>
     <t>Combate ao Incêndio</t>
+  </si>
+  <si>
+    <t>Locação de empilhadeira retrátil</t>
+  </si>
+  <si>
+    <t>Grupo</t>
+  </si>
+  <si>
+    <t>Retirada de reservatório de água</t>
+  </si>
+  <si>
+    <t>Desmontagem da cobertura de enlonamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grupo Serviço premilinar </t>
   </si>
 </sst>
 </file>
@@ -2804,7 +2816,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="\R\$\ #,##0.00"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2841,6 +2853,12 @@
       <sz val="11"/>
       <color rgb="FF404040"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF404040"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -2901,7 +2919,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3081,13 +3099,30 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="21">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -3386,44 +3421,45 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B1:J98" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B1:J98" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
   <autoFilter ref="B1:J98"/>
   <sortState ref="B2:J98">
     <sortCondition ref="I1:I98"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" name="Item" dataDxfId="17" dataCellStyle="Normal"/>
-    <tableColumn id="8" name="Local" dataDxfId="16"/>
-    <tableColumn id="2" name="Insumo ou Serviço" dataDxfId="15" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="14" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="13" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="12" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="11" dataCellStyle="Moeda">
+    <tableColumn id="1" name="Item" dataDxfId="18" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Local" dataDxfId="17"/>
+    <tableColumn id="2" name="Insumo ou Serviço" dataDxfId="16" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="15" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="14" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="13" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="12" dataCellStyle="Moeda">
       <calculatedColumnFormula>G2*E2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="10" dataCellStyle="Normal"/>
-    <tableColumn id="11" name="Categoria" dataDxfId="9"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="11" dataCellStyle="Normal"/>
+    <tableColumn id="11" name="Grupo" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:H53" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="B3:H53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:I54" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="B3:I54"/>
   <sortState ref="B4:H53">
     <sortCondition ref="H3:H53"/>
   </sortState>
-  <tableColumns count="7">
-    <tableColumn id="1" name="Item" dataDxfId="6" dataCellStyle="Normal"/>
-    <tableColumn id="2" name="Descrição" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="2" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="1" dataCellStyle="Moeda">
+  <tableColumns count="8">
+    <tableColumn id="1" name="Item" dataDxfId="7" dataCellStyle="Normal"/>
+    <tableColumn id="2" name="Descrição" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="3" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="2" dataCellStyle="Moeda">
       <calculatedColumnFormula>F4*D4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="0" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="1" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Grupo Serviço premilinar " dataDxfId="0" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12866,7 +12902,7 @@
     <col min="7" max="7" width="18.42578125" style="15" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.42578125" style="15" customWidth="1"/>
     <col min="9" max="9" width="23.85546875" style="14" customWidth="1"/>
-    <col min="10" max="10" width="24.42578125" style="14" customWidth="1"/>
+    <col min="10" max="10" width="43.7109375" style="14" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.28515625" style="14" customWidth="1"/>
     <col min="12" max="12" width="55.5703125" style="33" customWidth="1"/>
     <col min="13" max="13" width="54.42578125" style="14" customWidth="1"/>
@@ -12899,7 +12935,7 @@
         <v>767</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>873</v>
+        <v>922</v>
       </c>
     </row>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
@@ -12952,7 +12988,7 @@
         <v>486032</v>
       </c>
       <c r="I3" s="53" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="J3" s="39"/>
       <c r="K3" s="39"/>
@@ -12979,7 +13015,7 @@
         <v>8650</v>
       </c>
       <c r="I4" s="53" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="J4" s="39"/>
       <c r="K4" s="39"/>
@@ -13017,7 +13053,7 @@
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="22" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="E6" s="21">
         <v>1</v>
@@ -13044,7 +13080,7 @@
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="29" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="E7" s="21">
         <v>250</v>
@@ -13071,7 +13107,7 @@
       </c>
       <c r="C8" s="18"/>
       <c r="D8" s="29" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="E8" s="30">
         <v>6</v>
@@ -13098,7 +13134,7 @@
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="29" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="E9" s="30">
         <v>1</v>
@@ -13125,7 +13161,7 @@
       </c>
       <c r="C10" s="18"/>
       <c r="D10" s="29" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="E10" s="30">
         <v>300</v>
@@ -13318,7 +13354,7 @@
       </c>
       <c r="C17" s="18"/>
       <c r="D17" s="29" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="E17" s="30">
         <v>1</v>
@@ -13343,7 +13379,7 @@
       <c r="B18" s="17"/>
       <c r="C18" s="18"/>
       <c r="D18" s="29" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="E18" s="30">
         <v>1</v>
@@ -13370,7 +13406,7 @@
       </c>
       <c r="C19" s="18"/>
       <c r="D19" s="29" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="E19" s="30">
         <v>50</v>
@@ -13397,7 +13433,7 @@
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="29" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="E20" s="30">
         <f>44*4</f>
@@ -13446,7 +13482,7 @@
       <c r="J21" s="39"/>
       <c r="K21" s="39"/>
       <c r="L21" s="33" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
@@ -13454,10 +13490,10 @@
         <v>21</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="D22" s="29" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="E22" s="30">
         <v>36</v>
@@ -13483,7 +13519,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="D23" s="29" t="s">
         <v>856</v>
@@ -13512,7 +13548,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="D24" s="29" t="s">
         <v>778</v>
@@ -13541,7 +13577,7 @@
         <v>24</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="D25" s="29" t="s">
         <v>871</v>
@@ -13570,7 +13606,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="D26" s="29" t="s">
         <v>857</v>
@@ -13601,7 +13637,7 @@
       </c>
       <c r="C27" s="17"/>
       <c r="D27" s="29" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="E27" s="30">
         <v>2</v>
@@ -13627,7 +13663,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D28" s="22" t="s">
         <v>861</v>
@@ -13636,7 +13672,7 @@
         <v>58</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="G28" s="25">
         <v>198.72</v>
@@ -13656,7 +13692,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D29" s="22" t="s">
         <v>864</v>
@@ -13665,7 +13701,7 @@
         <v>31</v>
       </c>
       <c r="F29" s="21" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="G29" s="25">
         <v>484.24</v>
@@ -13685,7 +13721,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D30" s="22" t="s">
         <v>867</v>
@@ -13714,7 +13750,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D31" s="22" t="s">
         <v>862</v>
@@ -13744,7 +13780,7 @@
         <v>31</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D32" s="22" t="s">
         <v>865</v>
@@ -13773,7 +13809,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D33" s="22" t="s">
         <v>866</v>
@@ -13802,7 +13838,7 @@
         <v>33</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D34" s="22" t="s">
         <v>863</v>
@@ -13831,7 +13867,7 @@
         <v>34</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="D35" s="22" t="s">
         <v>869</v>
@@ -13840,7 +13876,7 @@
         <v>12</v>
       </c>
       <c r="F35" s="21" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="G35" s="25">
         <v>703.93</v>
@@ -13860,7 +13896,7 @@
         <v>35</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="D36" s="22" t="s">
         <v>870</v>
@@ -13870,7 +13906,7 @@
         <v>13</v>
       </c>
       <c r="F36" s="21" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="G36" s="25">
         <v>484.24</v>
@@ -13891,7 +13927,7 @@
       </c>
       <c r="C37" s="18"/>
       <c r="D37" s="29" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="E37" s="30">
         <v>1</v>
@@ -14112,7 +14148,7 @@
       </c>
       <c r="C45" s="17"/>
       <c r="D45" s="29" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="E45" s="30">
         <v>140</v>
@@ -14459,7 +14495,7 @@
         <v>10920</v>
       </c>
       <c r="I57" s="21" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="J57" s="39"/>
       <c r="K57" s="39"/>
@@ -14473,7 +14509,7 @@
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="22" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="E58" s="30">
         <v>400</v>
@@ -14489,7 +14525,7 @@
         <v>6000</v>
       </c>
       <c r="I58" s="21" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="J58" s="39"/>
       <c r="K58" s="39"/>
@@ -14512,7 +14548,7 @@
         <v>0</v>
       </c>
       <c r="I59" s="17" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="J59" s="39"/>
       <c r="K59" s="39"/>
@@ -14961,7 +14997,7 @@
       </c>
       <c r="C76" s="18"/>
       <c r="D76" s="29" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="E76" s="30">
         <v>1</v>
@@ -14988,7 +15024,7 @@
       </c>
       <c r="C77" s="18"/>
       <c r="D77" s="29" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="E77" s="30">
         <v>1</v>
@@ -15033,7 +15069,9 @@
       <c r="I78" s="30" t="s">
         <v>837</v>
       </c>
-      <c r="J78" s="39"/>
+      <c r="J78" s="65" t="s">
+        <v>923</v>
+      </c>
       <c r="K78" s="39"/>
     </row>
     <row r="79" spans="2:11" x14ac:dyDescent="0.25">
@@ -15060,7 +15098,9 @@
       <c r="I79" s="30" t="s">
         <v>837</v>
       </c>
-      <c r="J79" s="39"/>
+      <c r="J79" s="65" t="s">
+        <v>923</v>
+      </c>
       <c r="K79" s="39"/>
     </row>
     <row r="80" spans="2:11" x14ac:dyDescent="0.25">
@@ -15087,7 +15127,9 @@
       <c r="I80" s="30" t="s">
         <v>837</v>
       </c>
-      <c r="J80" s="39"/>
+      <c r="J80" s="65" t="s">
+        <v>923</v>
+      </c>
       <c r="K80" s="39"/>
     </row>
     <row r="81" spans="2:12" x14ac:dyDescent="0.25">
@@ -15114,7 +15156,9 @@
       <c r="I81" s="30" t="s">
         <v>837</v>
       </c>
-      <c r="J81" s="39"/>
+      <c r="J81" s="65" t="s">
+        <v>924</v>
+      </c>
       <c r="K81" s="39"/>
     </row>
     <row r="82" spans="2:12" x14ac:dyDescent="0.25">
@@ -15123,7 +15167,7 @@
       </c>
       <c r="C82" s="17"/>
       <c r="D82" s="29" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="E82" s="30">
         <v>320</v>
@@ -15141,7 +15185,9 @@
       <c r="I82" s="30" t="s">
         <v>837</v>
       </c>
-      <c r="J82" s="39"/>
+      <c r="J82" s="65" t="s">
+        <v>923</v>
+      </c>
       <c r="K82" s="39"/>
     </row>
     <row r="83" spans="2:12" x14ac:dyDescent="0.25">
@@ -15150,7 +15196,7 @@
       </c>
       <c r="C83" s="17"/>
       <c r="D83" s="29" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="E83" s="30">
         <v>1</v>
@@ -15168,7 +15214,9 @@
       <c r="I83" s="30" t="s">
         <v>837</v>
       </c>
-      <c r="J83" s="39"/>
+      <c r="J83" s="65" t="s">
+        <v>923</v>
+      </c>
       <c r="K83" s="39"/>
     </row>
     <row r="84" spans="2:12" x14ac:dyDescent="0.25">
@@ -15177,7 +15225,7 @@
       </c>
       <c r="C84" s="17"/>
       <c r="D84" s="29" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="E84" s="30">
         <v>1</v>
@@ -15195,7 +15243,9 @@
       <c r="I84" s="30" t="s">
         <v>837</v>
       </c>
-      <c r="J84" s="39"/>
+      <c r="J84" s="65" t="s">
+        <v>923</v>
+      </c>
       <c r="K84" s="39"/>
     </row>
     <row r="85" spans="2:12" x14ac:dyDescent="0.25">
@@ -15204,7 +15254,7 @@
       </c>
       <c r="C85" s="17"/>
       <c r="D85" s="29" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="E85" s="30">
         <v>1</v>
@@ -15222,7 +15272,9 @@
       <c r="I85" s="30" t="s">
         <v>837</v>
       </c>
-      <c r="J85" s="39"/>
+      <c r="J85" s="65" t="s">
+        <v>924</v>
+      </c>
       <c r="K85" s="39"/>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.25">
@@ -15230,10 +15282,10 @@
         <v>85</v>
       </c>
       <c r="C86" s="17" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="D86" s="22" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="E86" s="35">
         <v>115</v>
@@ -15421,10 +15473,10 @@
         <v>93</v>
       </c>
       <c r="C93" s="17" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="D93" s="29" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="E93" s="30">
         <v>750</v>
@@ -15450,10 +15502,10 @@
         <v>94</v>
       </c>
       <c r="C94" s="17" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="D94" s="29" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="E94" s="30">
         <v>250</v>
@@ -15480,7 +15532,7 @@
       </c>
       <c r="C95" s="17"/>
       <c r="D95" s="29" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="E95" s="30">
         <v>1</v>
@@ -15638,7 +15690,7 @@
   <sheetData>
     <row r="2" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C2" s="59" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="D2" s="60">
         <f>'DPA IV'!H100</f>
@@ -15653,16 +15705,16 @@
         <v>767</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>802</v>
       </c>
       <c r="F4" s="14" t="s">
+        <v>906</v>
+      </c>
+      <c r="G4" s="14" t="s">
         <v>907</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>908</v>
       </c>
     </row>
     <row r="5" spans="3:7" x14ac:dyDescent="0.25">
@@ -15862,7 +15914,7 @@
     </row>
     <row r="18" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C18" s="33" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="D18" s="58">
         <f>SUMIF(Tabela24[Aplicação],"Sala Coordenação",Tabela24[Preço Total])</f>
@@ -15877,7 +15929,7 @@
     </row>
     <row r="19" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C19" s="33" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="D19" s="58">
         <f>SUMIF(Tabela24[Aplicação],"Iluminação Galpão",Tabela24[Preço Total])</f>
@@ -15937,7 +15989,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:I82"/>
+  <dimension ref="B3:J83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.28515625" style="47" customWidth="1"/>
@@ -15948,11 +16000,12 @@
     <col min="6" max="6" width="17.28515625" style="15" customWidth="1"/>
     <col min="7" max="7" width="18.28515625" style="15" customWidth="1"/>
     <col min="8" max="8" width="27.42578125" style="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="67.28515625" style="15" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="47"/>
+    <col min="9" max="9" width="66.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="67.28515625" style="15" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="47"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:10" s="15" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
         <v>753</v>
       </c>
@@ -15974,13 +16027,16 @@
       <c r="H3" s="15" t="s">
         <v>767</v>
       </c>
-    </row>
-    <row r="4" spans="2:9" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I3" s="15" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" s="15" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="48">
         <v>1</v>
       </c>
       <c r="C4" s="49" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="D4" s="50">
         <v>1</v>
@@ -15996,11 +16052,12 @@
       <c r="H4" s="50" t="s">
         <v>798</v>
       </c>
-      <c r="I4" s="51" t="s">
+      <c r="I4" s="48"/>
+      <c r="J4" s="51" t="s">
         <v>860</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="48">
         <v>2</v>
       </c>
@@ -16022,10 +16079,11 @@
         <v>421112</v>
       </c>
       <c r="H5" s="53" t="s">
-        <v>921</v>
-      </c>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+        <v>920</v>
+      </c>
+      <c r="I5" s="48"/>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="48">
         <v>3</v>
       </c>
@@ -16046,10 +16104,11 @@
         <v>6650</v>
       </c>
       <c r="H6" s="53" t="s">
-        <v>921</v>
-      </c>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+        <v>920</v>
+      </c>
+      <c r="I6" s="48"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="48">
         <v>4</v>
       </c>
@@ -16060,7 +16119,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="53" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="F7" s="25">
         <v>198.72</v>
@@ -16072,8 +16131,9 @@
       <c r="H7" s="53" t="s">
         <v>868</v>
       </c>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I7" s="48"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" s="48">
         <v>5</v>
       </c>
@@ -16084,7 +16144,7 @@
         <v>25</v>
       </c>
       <c r="E8" s="53" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="F8" s="25">
         <v>484.24</v>
@@ -16096,8 +16156,9 @@
       <c r="H8" s="53" t="s">
         <v>868</v>
       </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I8" s="48"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="48">
         <v>6</v>
       </c>
@@ -16120,8 +16181,9 @@
       <c r="H9" s="53" t="s">
         <v>868</v>
       </c>
-    </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I9" s="48"/>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="48">
         <v>7</v>
       </c>
@@ -16144,8 +16206,9 @@
       <c r="H10" s="53" t="s">
         <v>868</v>
       </c>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I10" s="48"/>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="48">
         <v>8</v>
       </c>
@@ -16168,8 +16231,9 @@
       <c r="H11" s="53" t="s">
         <v>868</v>
       </c>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I11" s="48"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="48">
         <v>9</v>
       </c>
@@ -16192,8 +16256,9 @@
       <c r="H12" s="53" t="s">
         <v>868</v>
       </c>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I12" s="48"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="48">
         <v>10</v>
       </c>
@@ -16216,8 +16281,9 @@
       <c r="H13" s="53" t="s">
         <v>868</v>
       </c>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I13" s="48"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="48">
         <v>11</v>
       </c>
@@ -16238,15 +16304,16 @@
         <v>1056959.67</v>
       </c>
       <c r="H14" s="53" t="s">
-        <v>892</v>
-      </c>
-    </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+        <v>891</v>
+      </c>
+      <c r="I14" s="48"/>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="48">
         <v>12</v>
       </c>
       <c r="C15" s="52" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="D15" s="53">
         <v>1</v>
@@ -16262,10 +16329,11 @@
         <v>163890</v>
       </c>
       <c r="H15" s="53" t="s">
-        <v>892</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+        <v>891</v>
+      </c>
+      <c r="I15" s="48"/>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="48">
         <v>13</v>
       </c>
@@ -16289,11 +16357,12 @@
       <c r="H16" s="53" t="s">
         <v>806</v>
       </c>
-      <c r="I16" s="51" t="s">
+      <c r="I16" s="48"/>
+      <c r="J16" s="51" t="s">
         <v>852</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="48">
         <v>14</v>
       </c>
@@ -16316,8 +16385,9 @@
       <c r="H17" s="53" t="s">
         <v>806</v>
       </c>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I17" s="48"/>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="48">
         <v>15</v>
       </c>
@@ -16341,13 +16411,14 @@
       <c r="H18" s="53" t="s">
         <v>774</v>
       </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I18" s="48"/>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="48">
         <v>16</v>
       </c>
       <c r="C19" s="52" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="D19" s="53">
         <v>180</v>
@@ -16365,8 +16436,9 @@
       <c r="H19" s="43" t="s">
         <v>774</v>
       </c>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I19" s="48"/>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="48">
         <v>17</v>
       </c>
@@ -16389,8 +16461,9 @@
       <c r="H20" s="43" t="s">
         <v>774</v>
       </c>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I20" s="48"/>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="48">
         <v>18</v>
       </c>
@@ -16413,8 +16486,9 @@
       <c r="H21" s="43" t="s">
         <v>774</v>
       </c>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I21" s="48"/>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="48">
         <v>19</v>
       </c>
@@ -16438,8 +16512,9 @@
       <c r="H22" s="43" t="s">
         <v>774</v>
       </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I22" s="48"/>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" s="48">
         <v>20</v>
       </c>
@@ -16462,8 +16537,9 @@
       <c r="H23" s="45" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I23" s="48"/>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B24" s="48">
         <v>21</v>
       </c>
@@ -16480,14 +16556,15 @@
         <v>4500</v>
       </c>
       <c r="G24" s="25">
-        <f t="shared" ref="G24:G50" si="1">F24*D24</f>
+        <f t="shared" ref="G24:G51" si="1">F24*D24</f>
         <v>4500</v>
       </c>
       <c r="H24" s="53" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I24" s="48"/>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B25" s="48">
         <v>22</v>
       </c>
@@ -16510,8 +16587,9 @@
       <c r="H25" s="53" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I25" s="48"/>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B26" s="48">
         <v>23</v>
       </c>
@@ -16534,8 +16612,9 @@
       <c r="H26" s="53" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I26" s="48"/>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B27" s="48">
         <v>24</v>
       </c>
@@ -16558,8 +16637,9 @@
       <c r="H27" s="53" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I27" s="48"/>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B28" s="48">
         <v>25</v>
       </c>
@@ -16582,11 +16662,12 @@
       <c r="H28" s="53" t="s">
         <v>771</v>
       </c>
-      <c r="I28" s="15" t="s">
+      <c r="I28" s="48"/>
+      <c r="J28" s="15" t="s">
         <v>812</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B29" s="48">
         <v>26</v>
       </c>
@@ -16609,11 +16690,12 @@
       <c r="H29" s="53" t="s">
         <v>771</v>
       </c>
-      <c r="I29" s="15" t="s">
+      <c r="I29" s="48"/>
+      <c r="J29" s="15" t="s">
         <v>812</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="48">
         <v>27</v>
       </c>
@@ -16636,8 +16718,9 @@
       <c r="H30" s="53" t="s">
         <v>771</v>
       </c>
-    </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="I30" s="48"/>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B31" s="48">
         <v>28</v>
       </c>
@@ -16658,15 +16741,16 @@
         <v>4200</v>
       </c>
       <c r="H31" s="53" t="s">
-        <v>903</v>
-      </c>
-    </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+        <v>902</v>
+      </c>
+      <c r="I31" s="48"/>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B32" s="48">
         <v>29</v>
       </c>
       <c r="C32" s="52" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="D32" s="43">
         <v>200</v>
@@ -16682,10 +16766,11 @@
         <v>3000</v>
       </c>
       <c r="H32" s="53" t="s">
-        <v>903</v>
-      </c>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
+        <v>902</v>
+      </c>
+      <c r="I32" s="48"/>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" s="48">
         <v>30</v>
       </c>
@@ -16702,10 +16787,11 @@
         <v>0</v>
       </c>
       <c r="H33" s="48" t="s">
-        <v>903</v>
-      </c>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
+        <v>902</v>
+      </c>
+      <c r="I33" s="48"/>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" s="48">
         <v>31</v>
       </c>
@@ -16728,8 +16814,9 @@
       <c r="H34" s="43" t="s">
         <v>576</v>
       </c>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I34" s="48"/>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" s="48">
         <v>32</v>
       </c>
@@ -16752,8 +16839,9 @@
       <c r="H35" s="43" t="s">
         <v>576</v>
       </c>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I35" s="48"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" s="48">
         <v>33</v>
       </c>
@@ -16776,8 +16864,9 @@
       <c r="H36" s="43" t="s">
         <v>576</v>
       </c>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I36" s="48"/>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B37" s="48">
         <v>34</v>
       </c>
@@ -16800,8 +16889,9 @@
       <c r="H37" s="43" t="s">
         <v>576</v>
       </c>
-    </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I37" s="48"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B38" s="48">
         <v>35</v>
       </c>
@@ -16825,8 +16915,9 @@
       <c r="H38" s="53" t="s">
         <v>635</v>
       </c>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I38" s="48"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B39" s="48">
         <v>36</v>
       </c>
@@ -16850,8 +16941,9 @@
       <c r="H39" s="53" t="s">
         <v>635</v>
       </c>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I39" s="48"/>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B40" s="48">
         <v>37</v>
       </c>
@@ -16874,8 +16966,9 @@
       <c r="H40" s="53" t="s">
         <v>635</v>
       </c>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I40" s="48"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B41" s="48">
         <v>38</v>
       </c>
@@ -16898,8 +16991,9 @@
       <c r="H41" s="53" t="s">
         <v>635</v>
       </c>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I41" s="48"/>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B42" s="48">
         <v>39</v>
       </c>
@@ -16922,8 +17016,9 @@
       <c r="H42" s="53" t="s">
         <v>635</v>
       </c>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I42" s="48"/>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B43" s="48">
         <v>40</v>
       </c>
@@ -16946,13 +17041,14 @@
       <c r="H43" s="53" t="s">
         <v>635</v>
       </c>
-    </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I43" s="48"/>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B44" s="48">
         <v>41</v>
       </c>
       <c r="C44" s="52" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="D44" s="53">
         <v>1</v>
@@ -16970,8 +17066,11 @@
       <c r="H44" s="53" t="s">
         <v>837</v>
       </c>
-    </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I44" s="48" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B45" s="48">
         <v>42</v>
       </c>
@@ -16994,157 +17093,168 @@
       <c r="H45" s="53" t="s">
         <v>837</v>
       </c>
-    </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I45" s="48" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B46" s="48">
         <v>43</v>
       </c>
-      <c r="C46" s="57" t="s">
+      <c r="C46" s="52" t="s">
+        <v>921</v>
+      </c>
+      <c r="D46" s="53">
+        <v>1</v>
+      </c>
+      <c r="E46" s="53" t="s">
+        <v>760</v>
+      </c>
+      <c r="F46" s="25">
+        <v>14503</v>
+      </c>
+      <c r="G46" s="25">
+        <f>F46*D46</f>
+        <v>14503</v>
+      </c>
+      <c r="H46" s="53" t="s">
+        <v>837</v>
+      </c>
+      <c r="I46" s="48" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B47" s="48">
+        <v>44</v>
+      </c>
+      <c r="C47" s="57" t="s">
         <v>845</v>
       </c>
-      <c r="D46" s="53">
+      <c r="D47" s="53">
         <v>1455.89</v>
       </c>
-      <c r="E46" s="53" t="s">
+      <c r="E47" s="53" t="s">
         <v>761</v>
       </c>
-      <c r="F46" s="25">
+      <c r="F47" s="25">
         <v>95.9</v>
       </c>
-      <c r="G46" s="25">
+      <c r="G47" s="25">
         <f t="shared" si="1"/>
         <v>139619.85100000002</v>
       </c>
-      <c r="H46" s="53" t="s">
+      <c r="H47" s="53" t="s">
         <v>791</v>
       </c>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B47" s="48">
-        <v>44</v>
-      </c>
-      <c r="C47" s="52" t="s">
+      <c r="I47" s="48"/>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B48" s="48">
+        <v>45</v>
+      </c>
+      <c r="C48" s="52" t="s">
         <v>846</v>
       </c>
-      <c r="D47" s="53">
+      <c r="D48" s="53">
         <v>706.94</v>
       </c>
-      <c r="E47" s="53" t="s">
+      <c r="E48" s="53" t="s">
         <v>761</v>
       </c>
-      <c r="F47" s="25">
+      <c r="F48" s="25">
         <v>95.9</v>
       </c>
-      <c r="G47" s="25">
+      <c r="G48" s="25">
         <f t="shared" si="1"/>
         <v>67795.546000000002</v>
       </c>
-      <c r="H47" s="53" t="s">
+      <c r="H48" s="53" t="s">
         <v>791</v>
       </c>
-    </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B48" s="48">
-        <v>45</v>
-      </c>
-      <c r="C48" s="44" t="s">
+      <c r="I48" s="48"/>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B49" s="48">
+        <v>46</v>
+      </c>
+      <c r="C49" s="44" t="s">
         <v>847</v>
       </c>
-      <c r="D48" s="53">
+      <c r="D49" s="53">
         <v>44</v>
       </c>
-      <c r="E48" s="53" t="s">
+      <c r="E49" s="53" t="s">
         <v>818</v>
       </c>
-      <c r="F48" s="25">
+      <c r="F49" s="25">
         <v>95</v>
       </c>
-      <c r="G48" s="25">
+      <c r="G49" s="25">
         <f t="shared" si="1"/>
         <v>4180</v>
       </c>
-      <c r="H48" s="53" t="s">
+      <c r="H49" s="53" t="s">
         <v>791</v>
       </c>
-    </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B49" s="48">
-        <v>46</v>
-      </c>
-      <c r="C49" s="44" t="s">
+      <c r="I49" s="48"/>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B50" s="48">
+        <v>47</v>
+      </c>
+      <c r="C50" s="44" t="s">
         <v>848</v>
       </c>
-      <c r="D49" s="53">
+      <c r="D50" s="53">
         <v>3</v>
       </c>
-      <c r="E49" s="53" t="s">
+      <c r="E50" s="53" t="s">
         <v>818</v>
       </c>
-      <c r="F49" s="25">
+      <c r="F50" s="25">
         <v>35</v>
       </c>
-      <c r="G49" s="25">
+      <c r="G50" s="25">
         <f t="shared" si="1"/>
         <v>105</v>
       </c>
-      <c r="H49" s="53" t="s">
+      <c r="H50" s="53" t="s">
         <v>791</v>
       </c>
-    </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B50" s="48">
-        <v>47</v>
-      </c>
-      <c r="C50" s="44" t="s">
+      <c r="I50" s="48"/>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B51" s="48">
+        <v>48</v>
+      </c>
+      <c r="C51" s="44" t="s">
         <v>849</v>
       </c>
-      <c r="D50" s="53">
+      <c r="D51" s="53">
         <v>126</v>
       </c>
-      <c r="E50" s="53" t="s">
+      <c r="E51" s="53" t="s">
         <v>760</v>
       </c>
-      <c r="F50" s="25">
+      <c r="F51" s="25">
         <v>25.9</v>
       </c>
-      <c r="G50" s="25">
+      <c r="G51" s="25">
         <f t="shared" si="1"/>
         <v>3263.3999999999996</v>
       </c>
-      <c r="H50" s="53" t="s">
-        <v>791</v>
-      </c>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B51" s="48">
-        <v>48</v>
-      </c>
-      <c r="C51" s="44" t="s">
-        <v>817</v>
-      </c>
-      <c r="D51" s="53">
-        <v>1</v>
-      </c>
-      <c r="E51" s="53" t="s">
-        <v>760</v>
-      </c>
-      <c r="F51" s="25">
-        <v>1750</v>
-      </c>
-      <c r="G51" s="25">
-        <f>F51*D51</f>
-        <v>1750</v>
-      </c>
       <c r="H51" s="53" t="s">
         <v>791</v>
       </c>
-    </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I51" s="48"/>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B52" s="48">
         <v>49</v>
       </c>
-      <c r="C52" s="52" t="s">
-        <v>781</v>
+      <c r="C52" s="44" t="s">
+        <v>817</v>
       </c>
       <c r="D52" s="53">
         <v>1</v>
@@ -17153,50 +17263,68 @@
         <v>760</v>
       </c>
       <c r="F52" s="25">
-        <v>174417.38</v>
+        <v>1750</v>
       </c>
       <c r="G52" s="25">
         <f>F52*D52</f>
-        <v>174417.38</v>
+        <v>1750</v>
       </c>
       <c r="H52" s="53" t="s">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
+        <v>791</v>
+      </c>
+      <c r="I52" s="48"/>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B53" s="48">
         <v>50</v>
       </c>
-      <c r="C53" s="42" t="s">
+      <c r="C53" s="52" t="s">
+        <v>781</v>
+      </c>
+      <c r="D53" s="53">
+        <v>1</v>
+      </c>
+      <c r="E53" s="53" t="s">
+        <v>760</v>
+      </c>
+      <c r="F53" s="25">
+        <v>174417.38</v>
+      </c>
+      <c r="G53" s="25">
+        <f>F53*D53</f>
+        <v>174417.38</v>
+      </c>
+      <c r="H53" s="53" t="s">
+        <v>780</v>
+      </c>
+      <c r="I53" s="48"/>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B54" s="48">
+        <v>51</v>
+      </c>
+      <c r="C54" s="42" t="s">
         <v>814</v>
       </c>
-      <c r="D53" s="43">
-        <v>1</v>
-      </c>
-      <c r="E53" s="43" t="s">
+      <c r="D54" s="43">
+        <v>1</v>
+      </c>
+      <c r="E54" s="43" t="s">
         <v>760</v>
       </c>
-      <c r="F53" s="31">
+      <c r="F54" s="31">
         <v>5000</v>
       </c>
-      <c r="G53" s="31">
-        <f>F53*D53</f>
+      <c r="G54" s="31">
+        <f>F54*D54</f>
         <v>5000</v>
       </c>
-      <c r="H53" s="43" t="s">
+      <c r="H54" s="43" t="s">
         <v>815</v>
       </c>
-    </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B54" s="50"/>
-      <c r="C54" s="49"/>
-      <c r="D54" s="50"/>
-      <c r="E54" s="50"/>
-      <c r="F54" s="20"/>
-      <c r="G54" s="20"/>
-      <c r="H54" s="50"/>
-    </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="I54" s="48"/>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B55" s="50"/>
       <c r="C55" s="49"/>
       <c r="D55" s="50"/>
@@ -17204,18 +17332,30 @@
       <c r="F55" s="20"/>
       <c r="G55" s="20"/>
       <c r="H55" s="50"/>
-    </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="G56" s="16">
+      <c r="I55" s="50"/>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B56" s="50"/>
+      <c r="C56" s="49"/>
+      <c r="D56" s="50"/>
+      <c r="E56" s="50"/>
+      <c r="F56" s="20"/>
+      <c r="G56" s="20"/>
+      <c r="H56" s="50"/>
+      <c r="I56" s="50"/>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="G57" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>3121189.0038461541</v>
-      </c>
-    </row>
-    <row r="82" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H82" s="36">
-        <f>SUM('Expansão DMP'!G56,H78)</f>
-        <v>3121189.0038461541</v>
-      </c>
+        <v>3135692.0038461541</v>
+      </c>
+    </row>
+    <row r="83" spans="8:9" x14ac:dyDescent="0.25">
+      <c r="H83" s="36">
+        <f>SUM('Expansão DMP'!G57,H79)</f>
+        <v>3135692.0038461541</v>
+      </c>
+      <c r="I83" s="36"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -17239,14 +17379,14 @@
   <sheetData>
     <row r="2" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C2" s="59" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="D2" s="62">
-        <f>'Expansão DMP'!G56</f>
-        <v>3121189.0038461541</v>
+        <f>'Expansão DMP'!G57</f>
+        <v>3135692.0038461541</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="H2" s="61">
         <v>0.8</v>
@@ -17256,7 +17396,7 @@
       <c r="C3" s="59"/>
       <c r="D3" s="62"/>
       <c r="G3" s="14" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="H3" s="61">
         <v>0.81</v>
@@ -17266,7 +17406,7 @@
       <c r="C4" s="59"/>
       <c r="D4" s="62"/>
       <c r="G4" s="14" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="H4" s="61">
         <v>0.91</v>
@@ -17277,21 +17417,21 @@
         <v>767</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>802</v>
       </c>
       <c r="F6" s="14" t="s">
+        <v>906</v>
+      </c>
+      <c r="G6" s="14" t="s">
         <v>907</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>908</v>
       </c>
     </row>
     <row r="7" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="D7" s="63">
         <f>SUMIF(Tabela2[Aplicação],"Estrutura Metálica",Tabela2[Preço Total])</f>
@@ -17299,14 +17439,14 @@
       </c>
       <c r="E7" s="64">
         <f t="shared" ref="E7:E20" si="0">D7/$D$2</f>
-        <v>0.39114890783466844</v>
+        <v>0.38933979118565826</v>
       </c>
       <c r="F7" s="64">
         <f>E7</f>
-        <v>0.39114890783466844</v>
+        <v>0.38933979118565826</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
     <row r="8" spans="3:8" x14ac:dyDescent="0.25">
@@ -17323,10 +17463,10 @@
       </c>
       <c r="F8" s="64">
         <f t="shared" ref="F8:F20" si="1">F7+E8</f>
-        <v>0.39114890783466844</v>
+        <v>0.38933979118565826</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
     <row r="9" spans="3:8" x14ac:dyDescent="0.25">
@@ -17343,10 +17483,10 @@
       </c>
       <c r="F9" s="64">
         <f t="shared" si="1"/>
-        <v>0.39114890783466844</v>
+        <v>0.38933979118565826</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
     <row r="10" spans="3:8" x14ac:dyDescent="0.25">
@@ -17359,14 +17499,14 @@
       </c>
       <c r="E10" s="64">
         <f t="shared" si="0"/>
-        <v>0.11570319945416364</v>
+        <v>0.11516805649381374</v>
       </c>
       <c r="F10" s="64">
         <f t="shared" si="1"/>
-        <v>0.50685210728883212</v>
+        <v>0.50450784767947199</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
     <row r="11" spans="3:8" x14ac:dyDescent="0.25">
@@ -17379,14 +17519,14 @@
       </c>
       <c r="E11" s="64">
         <f t="shared" si="0"/>
-        <v>6.9433089996456365E-2</v>
+        <v>6.9111952555985984E-2</v>
       </c>
       <c r="F11" s="64">
         <f t="shared" si="1"/>
-        <v>0.57628519728528849</v>
+        <v>0.573619800235458</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
     </row>
     <row r="12" spans="3:8" x14ac:dyDescent="0.25">
@@ -17399,14 +17539,14 @@
       </c>
       <c r="E12" s="64">
         <f t="shared" si="0"/>
-        <v>5.588171039468303E-2</v>
+        <v>5.56232499193366E-2</v>
       </c>
       <c r="F12" s="64">
         <f t="shared" si="1"/>
-        <v>0.63216690767997152</v>
+        <v>0.62924305015479465</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
     </row>
     <row r="13" spans="3:8" x14ac:dyDescent="0.25">
@@ -17419,14 +17559,14 @@
       </c>
       <c r="E13" s="64">
         <f t="shared" si="0"/>
-        <v>5.2653011335580258E-2</v>
+        <v>5.2409484030454853E-2</v>
       </c>
       <c r="F13" s="64">
         <f t="shared" si="1"/>
-        <v>0.68481991901555173</v>
+        <v>0.68165253418524951</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="14" spans="3:8" x14ac:dyDescent="0.25">
@@ -17439,14 +17579,14 @@
       </c>
       <c r="E14" s="64">
         <f t="shared" si="0"/>
-        <v>2.5355200502910905E-2</v>
+        <v>2.5237929268222461E-2</v>
       </c>
       <c r="F14" s="64">
         <f t="shared" si="1"/>
-        <v>0.71017511951846268</v>
+        <v>0.70689046345347195</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="15" spans="3:8" x14ac:dyDescent="0.25">
@@ -17459,14 +17599,14 @@
       </c>
       <c r="E15" s="64">
         <f t="shared" si="0"/>
-        <v>6.9289876304671223E-3</v>
+        <v>6.8969401246912346E-3</v>
       </c>
       <c r="F15" s="64">
         <f t="shared" si="1"/>
-        <v>0.7171041071489298</v>
+        <v>0.71378740357816317</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="16" spans="3:8" x14ac:dyDescent="0.25">
@@ -17479,19 +17619,19 @@
       </c>
       <c r="E16" s="64">
         <f t="shared" si="0"/>
-        <v>5.9328640390509165E-3</v>
+        <v>5.9054237397317185E-3</v>
       </c>
       <c r="F16" s="64">
         <f t="shared" si="1"/>
-        <v>0.72303697118798071</v>
+        <v>0.71969282731789486</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="17" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="D17" s="63">
         <f>SUMIF(Tabela2[Aplicação],"Iluminação Galpão",Tabela2[Preço Total])</f>
@@ -17499,14 +17639,14 @@
       </c>
       <c r="E17" s="64">
         <f t="shared" si="0"/>
-        <v>2.3068132019969444E-3</v>
+        <v>2.296143878661768E-3</v>
       </c>
       <c r="F17" s="64">
         <f t="shared" si="1"/>
-        <v>0.72534378438997771</v>
+        <v>0.72198897119655658</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="18" spans="3:7" x14ac:dyDescent="0.25">
@@ -17519,14 +17659,14 @@
       </c>
       <c r="E18" s="64">
         <f t="shared" si="0"/>
-        <v>1.6980708292477509E-3</v>
+        <v>1.6902170217926904E-3</v>
       </c>
       <c r="F18" s="64">
         <f t="shared" si="1"/>
-        <v>0.72704185521922549</v>
+        <v>0.72367918821834931</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="19" spans="3:7" x14ac:dyDescent="0.25">
@@ -17539,14 +17679,14 @@
       </c>
       <c r="E19" s="64">
         <f t="shared" si="0"/>
-        <v>1.6019536124978781E-3</v>
+        <v>1.5945443601817833E-3</v>
       </c>
       <c r="F19" s="64">
         <f t="shared" si="1"/>
-        <v>0.72864380883172342</v>
+        <v>0.72527373257853112</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="20" spans="3:7" x14ac:dyDescent="0.25">
@@ -17563,10 +17703,10 @@
       </c>
       <c r="F20" s="64">
         <f t="shared" si="1"/>
-        <v>0.72864380883172342</v>
+        <v>0.72527373257853112</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="21" spans="3:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 14:29
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2361" uniqueCount="926">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2362" uniqueCount="925">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2794,9 +2794,6 @@
   </si>
   <si>
     <t>Locação de empilhadeira retrátil</t>
-  </si>
-  <si>
-    <t>Grupo</t>
   </si>
   <si>
     <t>Retirada de reservatório de água</t>
@@ -3437,7 +3434,7 @@
       <calculatedColumnFormula>G2*E2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" name="Aplicação" dataDxfId="11" dataCellStyle="Normal"/>
-    <tableColumn id="11" name="Grupo" dataDxfId="10"/>
+    <tableColumn id="11" name="Grupo Serviço premilinar " dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12935,7 +12932,7 @@
         <v>767</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>922</v>
+        <v>924</v>
       </c>
     </row>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
@@ -15070,7 +15067,7 @@
         <v>837</v>
       </c>
       <c r="J78" s="65" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="K78" s="39"/>
     </row>
@@ -15099,7 +15096,7 @@
         <v>837</v>
       </c>
       <c r="J79" s="65" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="K79" s="39"/>
     </row>
@@ -15128,7 +15125,7 @@
         <v>837</v>
       </c>
       <c r="J80" s="65" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="K80" s="39"/>
     </row>
@@ -15157,7 +15154,7 @@
         <v>837</v>
       </c>
       <c r="J81" s="65" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="K81" s="39"/>
     </row>
@@ -15186,7 +15183,7 @@
         <v>837</v>
       </c>
       <c r="J82" s="65" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="K82" s="39"/>
     </row>
@@ -15215,7 +15212,7 @@
         <v>837</v>
       </c>
       <c r="J83" s="65" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="K83" s="39"/>
     </row>
@@ -15244,7 +15241,7 @@
         <v>837</v>
       </c>
       <c r="J84" s="65" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="K84" s="39"/>
     </row>
@@ -15273,7 +15270,7 @@
         <v>837</v>
       </c>
       <c r="J85" s="65" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="K85" s="39"/>
     </row>
@@ -15303,7 +15300,9 @@
       <c r="I86" s="21" t="s">
         <v>837</v>
       </c>
-      <c r="J86" s="39"/>
+      <c r="J86" s="65" t="s">
+        <v>922</v>
+      </c>
       <c r="K86" s="39"/>
     </row>
     <row r="87" spans="2:12" x14ac:dyDescent="0.25">
@@ -16028,7 +16027,7 @@
         <v>767</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="4" spans="2:10" s="15" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Atualiza planilha e roteiro 22/10/2026 14:38
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2362" uniqueCount="925">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2364" uniqueCount="927">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2803,6 +2803,12 @@
   </si>
   <si>
     <t xml:space="preserve">Grupo Serviço premilinar </t>
+  </si>
+  <si>
+    <t>Prazo de execução:</t>
+  </si>
+  <si>
+    <t>300 dias</t>
   </si>
 </sst>
 </file>
@@ -12847,7 +12853,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:O104"/>
+  <dimension ref="B1:O105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" customWidth="1"/>
@@ -15616,21 +15622,37 @@
       <c r="K99" s="27"/>
     </row>
     <row r="100" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D100" s="21"/>
-      <c r="E100" s="22"/>
-      <c r="F100" s="22"/>
-      <c r="H100" s="16">
+      <c r="B100" s="18"/>
+      <c r="C100" s="18"/>
+      <c r="D100" s="19"/>
+      <c r="E100" s="18"/>
+      <c r="F100" s="18"/>
+      <c r="G100" s="20" t="s">
+        <v>925</v>
+      </c>
+      <c r="H100" s="23" t="s">
+        <v>926</v>
+      </c>
+      <c r="I100" s="18"/>
+      <c r="J100" s="27"/>
+      <c r="K100" s="27"/>
+    </row>
+    <row r="101" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D101" s="21"/>
+      <c r="E101" s="22"/>
+      <c r="F101" s="22"/>
+      <c r="H101" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
         <v>5833096.2741069021</v>
       </c>
     </row>
-    <row r="101" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D101" s="28"/>
-      <c r="E101" s="29"/>
-      <c r="F101" s="29"/>
-    </row>
-    <row r="104" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="H104" s="26"/>
+    <row r="102" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D102" s="28"/>
+      <c r="E102" s="29"/>
+      <c r="F102" s="29"/>
+    </row>
+    <row r="105" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H105" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -15657,7 +15679,7 @@
         <v>910</v>
       </c>
       <c r="D2" s="37">
-        <f>'DPA IV'!H100</f>
+        <f>'DPA IV'!H101</f>
         <v>5833096.2741069021</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 14:41
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2364" uniqueCount="927">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2366" uniqueCount="929">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2809,6 +2809,12 @@
   </si>
   <si>
     <t>300 dias</t>
+  </si>
+  <si>
+    <t>Prazo de Execução:</t>
+  </si>
+  <si>
+    <t>180 dias</t>
   </si>
 </sst>
 </file>
@@ -17330,8 +17336,12 @@
       <c r="C56" s="32"/>
       <c r="D56" s="33"/>
       <c r="E56" s="33"/>
-      <c r="F56" s="20"/>
-      <c r="G56" s="20"/>
+      <c r="F56" s="20" t="s">
+        <v>927</v>
+      </c>
+      <c r="G56" s="20" t="s">
+        <v>928</v>
+      </c>
       <c r="H56" s="33"/>
       <c r="I56" s="33"/>
     </row>

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 14:57
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,18 +9,19 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
     <sheet name="DPA IV" sheetId="6" r:id="rId2"/>
     <sheet name=" ABC DPA IV" sheetId="7" r:id="rId3"/>
     <sheet name="Expansão DMP" sheetId="3" r:id="rId4"/>
-    <sheet name="ABC DMP" sheetId="8" r:id="rId5"/>
+    <sheet name="Prazo de Execução" sheetId="9" r:id="rId5"/>
+    <sheet name="ABC DMP" sheetId="8" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">' ABC DPA IV'!$C$4:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ABC DMP'!$C$6:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ABC DMP'!$C$6:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">EAP_Cronograma!$A$1:$M$367</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
@@ -17336,12 +17337,6 @@
       <c r="C56" s="32"/>
       <c r="D56" s="33"/>
       <c r="E56" s="33"/>
-      <c r="F56" s="20" t="s">
-        <v>927</v>
-      </c>
-      <c r="G56" s="20" t="s">
-        <v>928</v>
-      </c>
       <c r="H56" s="33"/>
       <c r="I56" s="33"/>
     </row>
@@ -17368,6 +17363,27 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A2:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>927</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>928</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="C2:H28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 15:19
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2366" uniqueCount="929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2372" uniqueCount="931">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2816,6 +2816,12 @@
   </si>
   <si>
     <t>180 dias</t>
+  </si>
+  <si>
+    <t>Montagem da estrutura</t>
+  </si>
+  <si>
+    <t>Frete</t>
   </si>
 </sst>
 </file>
@@ -3414,8 +3420,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:I54" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="B3:I54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:I56" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="B3:I56"/>
   <sortState ref="B4:H53">
     <sortCondition ref="H3:H53"/>
   </sortState>
@@ -15982,7 +15988,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:J83"/>
+  <dimension ref="B3:J85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.28515625" style="30" customWidth="1"/>
@@ -16039,7 +16045,7 @@
       </c>
       <c r="F4" s="20"/>
       <c r="G4" s="20">
-        <f t="shared" ref="G4:G18" si="0">F4*D4</f>
+        <f t="shared" ref="G4:G20" si="0">F4*D4</f>
         <v>0</v>
       </c>
       <c r="H4" s="33" t="s">
@@ -16050,79 +16056,77 @@
         <v>860</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" s="15" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="31">
         <v>2</v>
       </c>
-      <c r="C5" s="43" t="s">
-        <v>776</v>
-      </c>
-      <c r="D5" s="31">
-        <v>1</v>
-      </c>
-      <c r="E5" s="31" t="s">
+      <c r="C5" s="32" t="s">
+        <v>929</v>
+      </c>
+      <c r="D5" s="33">
+        <v>1</v>
+      </c>
+      <c r="E5" s="33" t="s">
         <v>760</v>
       </c>
-      <c r="F5" s="44">
-        <f>212518+208594</f>
-        <v>421112</v>
-      </c>
-      <c r="G5" s="44">
-        <f t="shared" si="0"/>
-        <v>421112</v>
-      </c>
-      <c r="H5" s="31" t="s">
-        <v>920</v>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20">
+        <f>F5*D5</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="33" t="s">
+        <v>798</v>
       </c>
       <c r="I5" s="31"/>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J5" s="34"/>
+    </row>
+    <row r="6" spans="2:10" s="15" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="31">
         <v>3</v>
       </c>
-      <c r="C6" s="43" t="s">
-        <v>822</v>
-      </c>
-      <c r="D6" s="31">
-        <v>1</v>
-      </c>
-      <c r="E6" s="31" t="s">
+      <c r="C6" s="32" t="s">
+        <v>930</v>
+      </c>
+      <c r="D6" s="33">
+        <v>1</v>
+      </c>
+      <c r="E6" s="33" t="s">
         <v>760</v>
       </c>
-      <c r="F6" s="44">
-        <v>6650</v>
-      </c>
-      <c r="G6" s="44">
-        <f t="shared" si="0"/>
-        <v>6650</v>
-      </c>
-      <c r="H6" s="31" t="s">
-        <v>920</v>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20">
+        <f>F6*D6</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="33" t="s">
+        <v>798</v>
       </c>
       <c r="I6" s="31"/>
+      <c r="J6" s="34"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="31">
         <v>4</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>861</v>
+        <v>776</v>
       </c>
       <c r="D7" s="31">
-        <v>10</v>
-      </c>
-      <c r="E7" s="31" t="s">
-        <v>881</v>
+        <v>1</v>
+      </c>
+      <c r="E7" s="33" t="s">
+        <v>760</v>
       </c>
       <c r="F7" s="44">
-        <v>198.72</v>
+        <f>212518+208594</f>
+        <v>421112</v>
       </c>
       <c r="G7" s="44">
         <f t="shared" si="0"/>
-        <v>1987.2</v>
+        <v>421112</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>868</v>
+        <v>920</v>
       </c>
       <c r="I7" s="31"/>
     </row>
@@ -16131,23 +16135,23 @@
         <v>5</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>864</v>
+        <v>822</v>
       </c>
       <c r="D8" s="31">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>881</v>
+        <v>760</v>
       </c>
       <c r="F8" s="44">
-        <v>484.24</v>
+        <v>6650</v>
       </c>
       <c r="G8" s="44">
         <f t="shared" si="0"/>
-        <v>12106</v>
+        <v>6650</v>
       </c>
       <c r="H8" s="31" t="s">
-        <v>868</v>
+        <v>920</v>
       </c>
       <c r="I8" s="31"/>
     </row>
@@ -16156,20 +16160,20 @@
         <v>6</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>867</v>
+        <v>861</v>
       </c>
       <c r="D9" s="31">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>760</v>
+        <v>881</v>
       </c>
       <c r="F9" s="44">
-        <v>703.93</v>
+        <v>198.72</v>
       </c>
       <c r="G9" s="44">
         <f t="shared" si="0"/>
-        <v>5631.44</v>
+        <v>1987.2</v>
       </c>
       <c r="H9" s="31" t="s">
         <v>868</v>
@@ -16181,20 +16185,20 @@
         <v>7</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="D10" s="31">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>760</v>
+        <v>881</v>
       </c>
       <c r="F10" s="44">
-        <v>49.05</v>
+        <v>484.24</v>
       </c>
       <c r="G10" s="44">
         <f t="shared" si="0"/>
-        <v>1177.1999999999998</v>
+        <v>12106</v>
       </c>
       <c r="H10" s="31" t="s">
         <v>868</v>
@@ -16206,20 +16210,20 @@
         <v>8</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
       <c r="D11" s="31">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E11" s="31" t="s">
         <v>760</v>
       </c>
       <c r="F11" s="44">
-        <v>151.19999999999999</v>
+        <v>703.93</v>
       </c>
       <c r="G11" s="44">
         <f t="shared" si="0"/>
-        <v>302.39999999999998</v>
+        <v>5631.44</v>
       </c>
       <c r="H11" s="31" t="s">
         <v>868</v>
@@ -16231,20 +16235,20 @@
         <v>9</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>866</v>
+        <v>862</v>
       </c>
       <c r="D12" s="31">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="E12" s="31" t="s">
         <v>760</v>
       </c>
       <c r="F12" s="44">
-        <v>48.38</v>
+        <v>49.05</v>
       </c>
       <c r="G12" s="44">
         <f t="shared" si="0"/>
-        <v>96.76</v>
+        <v>1177.1999999999998</v>
       </c>
       <c r="H12" s="31" t="s">
         <v>868</v>
@@ -16256,20 +16260,20 @@
         <v>10</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>863</v>
+        <v>865</v>
       </c>
       <c r="D13" s="31">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E13" s="31" t="s">
         <v>760</v>
       </c>
       <c r="F13" s="44">
-        <v>27.14</v>
+        <v>151.19999999999999</v>
       </c>
       <c r="G13" s="44">
         <f t="shared" si="0"/>
-        <v>325.68</v>
+        <v>302.39999999999998</v>
       </c>
       <c r="H13" s="31" t="s">
         <v>868</v>
@@ -16281,23 +16285,23 @@
         <v>11</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>816</v>
+        <v>866</v>
       </c>
       <c r="D14" s="31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="31" t="s">
         <v>760</v>
       </c>
       <c r="F14" s="44">
-        <v>1056959.67</v>
+        <v>48.38</v>
       </c>
       <c r="G14" s="44">
         <f t="shared" si="0"/>
-        <v>1056959.67</v>
+        <v>96.76</v>
       </c>
       <c r="H14" s="31" t="s">
-        <v>891</v>
+        <v>868</v>
       </c>
       <c r="I14" s="31"/>
     </row>
@@ -16306,23 +16310,23 @@
         <v>12</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>892</v>
+        <v>863</v>
       </c>
       <c r="D15" s="31">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E15" s="31" t="s">
         <v>760</v>
       </c>
       <c r="F15" s="44">
-        <v>163890</v>
+        <v>27.14</v>
       </c>
       <c r="G15" s="44">
         <f t="shared" si="0"/>
-        <v>163890</v>
+        <v>325.68</v>
       </c>
       <c r="H15" s="31" t="s">
-        <v>891</v>
+        <v>868</v>
       </c>
       <c r="I15" s="31"/>
     </row>
@@ -16331,52 +16335,48 @@
         <v>13</v>
       </c>
       <c r="C16" s="43" t="s">
-        <v>805</v>
-      </c>
-      <c r="D16" s="45">
-        <f>50*1.02</f>
-        <v>51</v>
+        <v>816</v>
+      </c>
+      <c r="D16" s="31">
+        <v>1</v>
       </c>
       <c r="E16" s="31" t="s">
         <v>760</v>
       </c>
       <c r="F16" s="44">
-        <v>243.39</v>
+        <v>1056959.67</v>
       </c>
       <c r="G16" s="44">
         <f t="shared" si="0"/>
-        <v>12412.89</v>
+        <v>1056959.67</v>
       </c>
       <c r="H16" s="31" t="s">
-        <v>806</v>
+        <v>891</v>
       </c>
       <c r="I16" s="31"/>
-      <c r="J16" s="34" t="s">
-        <v>852</v>
-      </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="31">
         <v>14</v>
       </c>
       <c r="C17" s="43" t="s">
-        <v>807</v>
-      </c>
-      <c r="D17" s="45">
-        <v>51</v>
+        <v>892</v>
+      </c>
+      <c r="D17" s="31">
+        <v>1</v>
       </c>
       <c r="E17" s="31" t="s">
         <v>760</v>
       </c>
       <c r="F17" s="44">
-        <v>119.7</v>
+        <v>163890</v>
       </c>
       <c r="G17" s="44">
         <f t="shared" si="0"/>
-        <v>6104.7</v>
+        <v>163890</v>
       </c>
       <c r="H17" s="31" t="s">
-        <v>806</v>
+        <v>891</v>
       </c>
       <c r="I17" s="31"/>
     </row>
@@ -16388,8 +16388,8 @@
         <v>805</v>
       </c>
       <c r="D18" s="45">
-        <f>(40*1.02)*4</f>
-        <v>163.19999999999999</v>
+        <f>50*1.02</f>
+        <v>51</v>
       </c>
       <c r="E18" s="31" t="s">
         <v>760</v>
@@ -16399,35 +16399,38 @@
       </c>
       <c r="G18" s="44">
         <f t="shared" si="0"/>
-        <v>39721.247999999992</v>
+        <v>12412.89</v>
       </c>
       <c r="H18" s="31" t="s">
-        <v>774</v>
+        <v>806</v>
       </c>
       <c r="I18" s="31"/>
+      <c r="J18" s="34" t="s">
+        <v>852</v>
+      </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="31">
         <v>16</v>
       </c>
       <c r="C19" s="43" t="s">
-        <v>874</v>
-      </c>
-      <c r="D19" s="31">
-        <v>180</v>
-      </c>
-      <c r="E19" s="33" t="s">
-        <v>761</v>
-      </c>
-      <c r="F19" s="25">
-        <v>23.90625</v>
-      </c>
-      <c r="G19" s="25">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>4303.125</v>
-      </c>
-      <c r="H19" s="33" t="s">
-        <v>774</v>
+        <v>807</v>
+      </c>
+      <c r="D19" s="45">
+        <v>51</v>
+      </c>
+      <c r="E19" s="31" t="s">
+        <v>760</v>
+      </c>
+      <c r="F19" s="44">
+        <v>119.7</v>
+      </c>
+      <c r="G19" s="44">
+        <f t="shared" si="0"/>
+        <v>6104.7</v>
+      </c>
+      <c r="H19" s="31" t="s">
+        <v>806</v>
       </c>
       <c r="I19" s="31"/>
     </row>
@@ -16435,23 +16438,24 @@
       <c r="B20" s="31">
         <v>17</v>
       </c>
-      <c r="C20" s="32" t="s">
-        <v>778</v>
-      </c>
-      <c r="D20" s="33">
-        <v>50</v>
-      </c>
-      <c r="E20" s="33" t="s">
-        <v>761</v>
-      </c>
-      <c r="F20" s="25">
-        <v>32</v>
-      </c>
-      <c r="G20" s="25">
-        <f>F20*D20</f>
-        <v>1600</v>
-      </c>
-      <c r="H20" s="33" t="s">
+      <c r="C20" s="43" t="s">
+        <v>805</v>
+      </c>
+      <c r="D20" s="45">
+        <f>(40*1.02)*4</f>
+        <v>163.19999999999999</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>760</v>
+      </c>
+      <c r="F20" s="44">
+        <v>243.39</v>
+      </c>
+      <c r="G20" s="44">
+        <f t="shared" si="0"/>
+        <v>39721.247999999992</v>
+      </c>
+      <c r="H20" s="31" t="s">
         <v>774</v>
       </c>
       <c r="I20" s="31"/>
@@ -16460,21 +16464,21 @@
       <c r="B21" s="31">
         <v>18</v>
       </c>
-      <c r="C21" s="32" t="s">
-        <v>871</v>
-      </c>
-      <c r="D21" s="33">
-        <v>6</v>
+      <c r="C21" s="43" t="s">
+        <v>874</v>
+      </c>
+      <c r="D21" s="31">
+        <v>180</v>
       </c>
       <c r="E21" s="33" t="s">
         <v>761</v>
       </c>
       <c r="F21" s="25">
-        <v>419</v>
+        <v>23.90625</v>
       </c>
       <c r="G21" s="25">
-        <f>F21*D21</f>
-        <v>2514</v>
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>4303.125</v>
       </c>
       <c r="H21" s="33" t="s">
         <v>774</v>
@@ -16486,21 +16490,20 @@
         <v>19</v>
       </c>
       <c r="C22" s="32" t="s">
-        <v>813</v>
+        <v>778</v>
       </c>
       <c r="D22" s="33">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="F22" s="25">
-        <f>23500+7500</f>
-        <v>31000</v>
+        <v>32</v>
       </c>
       <c r="G22" s="25">
         <f>F22*D22</f>
-        <v>31000</v>
+        <v>1600</v>
       </c>
       <c r="H22" s="33" t="s">
         <v>774</v>
@@ -16511,24 +16514,24 @@
       <c r="B23" s="31">
         <v>20</v>
       </c>
-      <c r="C23" s="46" t="s">
-        <v>790</v>
-      </c>
-      <c r="D23" s="47">
-        <v>4</v>
-      </c>
-      <c r="E23" s="47" t="s">
-        <v>760</v>
-      </c>
-      <c r="F23" s="48">
-        <v>1500</v>
-      </c>
-      <c r="G23" s="48">
-        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
-        <v>6000</v>
-      </c>
-      <c r="H23" s="47" t="s">
-        <v>771</v>
+      <c r="C23" s="32" t="s">
+        <v>871</v>
+      </c>
+      <c r="D23" s="33">
+        <v>6</v>
+      </c>
+      <c r="E23" s="33" t="s">
+        <v>761</v>
+      </c>
+      <c r="F23" s="25">
+        <v>419</v>
+      </c>
+      <c r="G23" s="25">
+        <f>F23*D23</f>
+        <v>2514</v>
+      </c>
+      <c r="H23" s="33" t="s">
+        <v>774</v>
       </c>
       <c r="I23" s="31"/>
     </row>
@@ -16536,24 +16539,25 @@
       <c r="B24" s="31">
         <v>21</v>
       </c>
-      <c r="C24" s="43" t="s">
-        <v>789</v>
-      </c>
-      <c r="D24" s="31">
-        <v>1</v>
-      </c>
-      <c r="E24" s="31" t="s">
+      <c r="C24" s="32" t="s">
+        <v>813</v>
+      </c>
+      <c r="D24" s="33">
+        <v>1</v>
+      </c>
+      <c r="E24" s="33" t="s">
         <v>760</v>
       </c>
-      <c r="F24" s="44">
-        <v>4500</v>
-      </c>
-      <c r="G24" s="44">
-        <f t="shared" ref="G24:G51" si="1">F24*D24</f>
-        <v>4500</v>
-      </c>
-      <c r="H24" s="31" t="s">
-        <v>771</v>
+      <c r="F24" s="25">
+        <f>23500+7500</f>
+        <v>31000</v>
+      </c>
+      <c r="G24" s="25">
+        <f>F24*D24</f>
+        <v>31000</v>
+      </c>
+      <c r="H24" s="33" t="s">
+        <v>774</v>
       </c>
       <c r="I24" s="31"/>
     </row>
@@ -16561,23 +16565,23 @@
       <c r="B25" s="31">
         <v>22</v>
       </c>
-      <c r="C25" s="43" t="s">
-        <v>769</v>
-      </c>
-      <c r="D25" s="31">
-        <v>2100</v>
-      </c>
-      <c r="E25" s="31" t="s">
-        <v>811</v>
-      </c>
-      <c r="F25" s="44">
-        <v>9.65</v>
-      </c>
-      <c r="G25" s="44">
-        <f t="shared" si="1"/>
-        <v>20265</v>
-      </c>
-      <c r="H25" s="31" t="s">
+      <c r="C25" s="46" t="s">
+        <v>790</v>
+      </c>
+      <c r="D25" s="47">
+        <v>4</v>
+      </c>
+      <c r="E25" s="47" t="s">
+        <v>760</v>
+      </c>
+      <c r="F25" s="48">
+        <v>1500</v>
+      </c>
+      <c r="G25" s="48">
+        <f>Tabela2[[#This Row],[Preço Unitário]]*Tabela2[[#This Row],[Quantidade]]</f>
+        <v>6000</v>
+      </c>
+      <c r="H25" s="47" t="s">
         <v>771</v>
       </c>
       <c r="I25" s="31"/>
@@ -16587,20 +16591,20 @@
         <v>23</v>
       </c>
       <c r="C26" s="43" t="s">
-        <v>770</v>
+        <v>789</v>
       </c>
       <c r="D26" s="31">
-        <v>2300</v>
+        <v>1</v>
       </c>
       <c r="E26" s="31" t="s">
-        <v>811</v>
+        <v>760</v>
       </c>
       <c r="F26" s="44">
-        <v>9.65</v>
+        <v>4500</v>
       </c>
       <c r="G26" s="44">
-        <f t="shared" si="1"/>
-        <v>22195</v>
+        <f t="shared" ref="G26:G53" si="1">F26*D26</f>
+        <v>4500</v>
       </c>
       <c r="H26" s="31" t="s">
         <v>771</v>
@@ -16612,20 +16616,20 @@
         <v>24</v>
       </c>
       <c r="C27" s="43" t="s">
-        <v>808</v>
+        <v>769</v>
       </c>
       <c r="D27" s="31">
-        <v>1</v>
+        <v>2100</v>
       </c>
       <c r="E27" s="31" t="s">
-        <v>760</v>
+        <v>811</v>
       </c>
       <c r="F27" s="44">
-        <v>51500</v>
+        <v>9.65</v>
       </c>
       <c r="G27" s="44">
         <f t="shared" si="1"/>
-        <v>51500</v>
+        <v>20265</v>
       </c>
       <c r="H27" s="31" t="s">
         <v>771</v>
@@ -16637,129 +16641,129 @@
         <v>25</v>
       </c>
       <c r="C28" s="43" t="s">
-        <v>809</v>
-      </c>
-      <c r="D28" s="45">
-        <v>46.8</v>
+        <v>770</v>
+      </c>
+      <c r="D28" s="31">
+        <v>2300</v>
       </c>
       <c r="E28" s="31" t="s">
-        <v>759</v>
+        <v>811</v>
       </c>
       <c r="F28" s="44">
-        <v>670</v>
+        <v>9.65</v>
       </c>
       <c r="G28" s="44">
         <f t="shared" si="1"/>
-        <v>31355.999999999996</v>
+        <v>22195</v>
       </c>
       <c r="H28" s="31" t="s">
         <v>771</v>
       </c>
       <c r="I28" s="31"/>
-      <c r="J28" s="15" t="s">
-        <v>812</v>
-      </c>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B29" s="31">
         <v>26</v>
       </c>
       <c r="C29" s="43" t="s">
-        <v>810</v>
-      </c>
-      <c r="D29" s="45">
-        <v>37.200000000000003</v>
+        <v>808</v>
+      </c>
+      <c r="D29" s="31">
+        <v>1</v>
       </c>
       <c r="E29" s="31" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="F29" s="44">
-        <v>670</v>
+        <v>51500</v>
       </c>
       <c r="G29" s="44">
         <f t="shared" si="1"/>
-        <v>24924.000000000004</v>
+        <v>51500</v>
       </c>
       <c r="H29" s="31" t="s">
         <v>771</v>
       </c>
       <c r="I29" s="31"/>
-      <c r="J29" s="15" t="s">
-        <v>812</v>
-      </c>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="31">
         <v>27</v>
       </c>
       <c r="C30" s="43" t="s">
-        <v>844</v>
-      </c>
-      <c r="D30" s="31">
-        <v>30</v>
+        <v>809</v>
+      </c>
+      <c r="D30" s="45">
+        <v>46.8</v>
       </c>
       <c r="E30" s="31" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="F30" s="44">
-        <v>120</v>
+        <v>670</v>
       </c>
       <c r="G30" s="44">
         <f t="shared" si="1"/>
-        <v>3600</v>
+        <v>31355.999999999996</v>
       </c>
       <c r="H30" s="31" t="s">
         <v>771</v>
       </c>
       <c r="I30" s="31"/>
+      <c r="J30" s="15" t="s">
+        <v>812</v>
+      </c>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B31" s="31">
         <v>28</v>
       </c>
-      <c r="C31" s="32" t="s">
-        <v>850</v>
-      </c>
-      <c r="D31" s="33">
-        <v>10</v>
-      </c>
-      <c r="E31" s="33" t="s">
-        <v>760</v>
-      </c>
-      <c r="F31" s="25">
-        <v>420</v>
-      </c>
-      <c r="G31" s="25">
+      <c r="C31" s="43" t="s">
+        <v>810</v>
+      </c>
+      <c r="D31" s="45">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E31" s="31" t="s">
+        <v>759</v>
+      </c>
+      <c r="F31" s="44">
+        <v>670</v>
+      </c>
+      <c r="G31" s="44">
         <f t="shared" si="1"/>
-        <v>4200</v>
+        <v>24924.000000000004</v>
       </c>
       <c r="H31" s="31" t="s">
-        <v>902</v>
+        <v>771</v>
       </c>
       <c r="I31" s="31"/>
+      <c r="J31" s="15" t="s">
+        <v>812</v>
+      </c>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B32" s="31">
         <v>29</v>
       </c>
       <c r="C32" s="43" t="s">
-        <v>898</v>
-      </c>
-      <c r="D32" s="33">
-        <v>200</v>
-      </c>
-      <c r="E32" s="33" t="s">
-        <v>761</v>
-      </c>
-      <c r="F32" s="25">
-        <v>15</v>
-      </c>
-      <c r="G32" s="25">
+        <v>844</v>
+      </c>
+      <c r="D32" s="31">
+        <v>30</v>
+      </c>
+      <c r="E32" s="31" t="s">
+        <v>760</v>
+      </c>
+      <c r="F32" s="44">
+        <v>120</v>
+      </c>
+      <c r="G32" s="44">
         <f t="shared" si="1"/>
-        <v>3000</v>
+        <v>3600</v>
       </c>
       <c r="H32" s="31" t="s">
-        <v>902</v>
+        <v>771</v>
       </c>
       <c r="I32" s="31"/>
     </row>
@@ -16768,21 +16772,20 @@
         <v>30</v>
       </c>
       <c r="C33" s="32" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="D33" s="33">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E33" s="33" t="s">
         <v>760</v>
       </c>
       <c r="F33" s="25">
-        <f>119439/2</f>
-        <v>59719.5</v>
+        <v>420</v>
       </c>
       <c r="G33" s="25">
         <f t="shared" si="1"/>
-        <v>59719.5</v>
+        <v>4200</v>
       </c>
       <c r="H33" s="31" t="s">
         <v>902</v>
@@ -16793,24 +16796,24 @@
       <c r="B34" s="31">
         <v>31</v>
       </c>
-      <c r="C34" s="32" t="s">
-        <v>782</v>
+      <c r="C34" s="43" t="s">
+        <v>898</v>
       </c>
       <c r="D34" s="33">
-        <v>8</v>
+        <v>200</v>
       </c>
       <c r="E34" s="33" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="F34" s="25">
-        <v>280</v>
+        <v>15</v>
       </c>
       <c r="G34" s="25">
         <f t="shared" si="1"/>
-        <v>2240</v>
-      </c>
-      <c r="H34" s="33" t="s">
-        <v>576</v>
+        <v>3000</v>
+      </c>
+      <c r="H34" s="31" t="s">
+        <v>902</v>
       </c>
       <c r="I34" s="31"/>
     </row>
@@ -16819,23 +16822,24 @@
         <v>32</v>
       </c>
       <c r="C35" s="32" t="s">
-        <v>783</v>
+        <v>851</v>
       </c>
       <c r="D35" s="33">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E35" s="33" t="s">
         <v>760</v>
       </c>
       <c r="F35" s="25">
-        <v>380</v>
+        <f>119439/2</f>
+        <v>59719.5</v>
       </c>
       <c r="G35" s="25">
         <f t="shared" si="1"/>
-        <v>1900</v>
-      </c>
-      <c r="H35" s="33" t="s">
-        <v>576</v>
+        <v>59719.5</v>
+      </c>
+      <c r="H35" s="31" t="s">
+        <v>902</v>
       </c>
       <c r="I35" s="31"/>
     </row>
@@ -16844,20 +16848,20 @@
         <v>33</v>
       </c>
       <c r="C36" s="32" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="D36" s="33">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E36" s="33" t="s">
         <v>760</v>
       </c>
       <c r="F36" s="25">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="G36" s="25">
         <f t="shared" si="1"/>
-        <v>580</v>
+        <v>2240</v>
       </c>
       <c r="H36" s="33" t="s">
         <v>576</v>
@@ -16869,20 +16873,20 @@
         <v>34</v>
       </c>
       <c r="C37" s="32" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="D37" s="33">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E37" s="33" t="s">
         <v>760</v>
       </c>
       <c r="F37" s="25">
-        <v>290</v>
+        <v>380</v>
       </c>
       <c r="G37" s="25">
         <f t="shared" si="1"/>
-        <v>580</v>
+        <v>1900</v>
       </c>
       <c r="H37" s="33" t="s">
         <v>576</v>
@@ -16893,25 +16897,24 @@
       <c r="B38" s="31">
         <v>35</v>
       </c>
-      <c r="C38" s="43" t="s">
-        <v>757</v>
-      </c>
-      <c r="D38" s="31">
-        <f>(2000*1.05)*0.15</f>
-        <v>315</v>
-      </c>
-      <c r="E38" s="31" t="s">
-        <v>759</v>
-      </c>
-      <c r="F38" s="44">
-        <v>670</v>
-      </c>
-      <c r="G38" s="44">
+      <c r="C38" s="32" t="s">
+        <v>784</v>
+      </c>
+      <c r="D38" s="33">
+        <v>2</v>
+      </c>
+      <c r="E38" s="33" t="s">
+        <v>760</v>
+      </c>
+      <c r="F38" s="25">
+        <v>290</v>
+      </c>
+      <c r="G38" s="25">
         <f t="shared" si="1"/>
-        <v>211050</v>
-      </c>
-      <c r="H38" s="31" t="s">
-        <v>635</v>
+        <v>580</v>
+      </c>
+      <c r="H38" s="33" t="s">
+        <v>576</v>
       </c>
       <c r="I38" s="31"/>
     </row>
@@ -16919,25 +16922,24 @@
       <c r="B39" s="31">
         <v>36</v>
       </c>
-      <c r="C39" s="43" t="s">
-        <v>775</v>
-      </c>
-      <c r="D39" s="45">
-        <f>2000/13*2</f>
-        <v>307.69230769230768</v>
-      </c>
-      <c r="E39" s="31" t="s">
+      <c r="C39" s="32" t="s">
+        <v>785</v>
+      </c>
+      <c r="D39" s="33">
+        <v>2</v>
+      </c>
+      <c r="E39" s="33" t="s">
         <v>760</v>
       </c>
-      <c r="F39" s="44">
-        <v>220.5</v>
-      </c>
-      <c r="G39" s="44">
+      <c r="F39" s="25">
+        <v>290</v>
+      </c>
+      <c r="G39" s="25">
         <f t="shared" si="1"/>
-        <v>67846.153846153844</v>
-      </c>
-      <c r="H39" s="31" t="s">
-        <v>635</v>
+        <v>580</v>
+      </c>
+      <c r="H39" s="33" t="s">
+        <v>576</v>
       </c>
       <c r="I39" s="31"/>
     </row>
@@ -16946,20 +16948,21 @@
         <v>37</v>
       </c>
       <c r="C40" s="43" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="D40" s="31">
-        <v>167</v>
+        <f>(2000*1.05)*0.15</f>
+        <v>315</v>
       </c>
       <c r="E40" s="31" t="s">
-        <v>797</v>
+        <v>759</v>
       </c>
       <c r="F40" s="44">
-        <v>56.2</v>
+        <v>670</v>
       </c>
       <c r="G40" s="44">
         <f t="shared" si="1"/>
-        <v>9385.4</v>
+        <v>211050</v>
       </c>
       <c r="H40" s="31" t="s">
         <v>635</v>
@@ -16971,20 +16974,21 @@
         <v>38</v>
       </c>
       <c r="C41" s="43" t="s">
-        <v>762</v>
-      </c>
-      <c r="D41" s="31">
-        <v>1000</v>
+        <v>775</v>
+      </c>
+      <c r="D41" s="45">
+        <f>2000/13*2</f>
+        <v>307.69230769230768</v>
       </c>
       <c r="E41" s="31" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="F41" s="44">
-        <v>7.3</v>
+        <v>220.5</v>
       </c>
       <c r="G41" s="44">
         <f t="shared" si="1"/>
-        <v>7300</v>
+        <v>67846.153846153844</v>
       </c>
       <c r="H41" s="31" t="s">
         <v>635</v>
@@ -16996,20 +17000,20 @@
         <v>39</v>
       </c>
       <c r="C42" s="43" t="s">
-        <v>792</v>
+        <v>758</v>
       </c>
       <c r="D42" s="31">
-        <v>315</v>
+        <v>167</v>
       </c>
       <c r="E42" s="31" t="s">
-        <v>759</v>
+        <v>797</v>
       </c>
       <c r="F42" s="44">
-        <v>50</v>
+        <v>56.2</v>
       </c>
       <c r="G42" s="44">
         <f t="shared" si="1"/>
-        <v>15750</v>
+        <v>9385.4</v>
       </c>
       <c r="H42" s="31" t="s">
         <v>635</v>
@@ -17021,20 +17025,20 @@
         <v>40</v>
       </c>
       <c r="C43" s="43" t="s">
-        <v>768</v>
+        <v>762</v>
       </c>
       <c r="D43" s="31">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="E43" s="31" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="F43" s="44">
-        <v>49800</v>
+        <v>7.3</v>
       </c>
       <c r="G43" s="44">
         <f t="shared" si="1"/>
-        <v>49800</v>
+        <v>7300</v>
       </c>
       <c r="H43" s="31" t="s">
         <v>635</v>
@@ -17046,34 +17050,32 @@
         <v>41</v>
       </c>
       <c r="C44" s="43" t="s">
-        <v>919</v>
+        <v>792</v>
       </c>
       <c r="D44" s="31">
-        <v>1</v>
+        <v>315</v>
       </c>
       <c r="E44" s="31" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="F44" s="44">
-        <v>15000</v>
+        <v>50</v>
       </c>
       <c r="G44" s="44">
         <f t="shared" si="1"/>
-        <v>15000</v>
+        <v>15750</v>
       </c>
       <c r="H44" s="31" t="s">
-        <v>837</v>
-      </c>
-      <c r="I44" s="31" t="s">
-        <v>919</v>
-      </c>
+        <v>635</v>
+      </c>
+      <c r="I44" s="31"/>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B45" s="31">
         <v>42</v>
       </c>
       <c r="C45" s="43" t="s">
-        <v>786</v>
+        <v>768</v>
       </c>
       <c r="D45" s="31">
         <v>1</v>
@@ -17082,25 +17084,23 @@
         <v>760</v>
       </c>
       <c r="F45" s="44">
-        <v>404191.96</v>
+        <v>49800</v>
       </c>
       <c r="G45" s="44">
         <f t="shared" si="1"/>
-        <v>404191.96</v>
+        <v>49800</v>
       </c>
       <c r="H45" s="31" t="s">
-        <v>837</v>
-      </c>
-      <c r="I45" s="31" t="s">
-        <v>786</v>
-      </c>
+        <v>635</v>
+      </c>
+      <c r="I45" s="31"/>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B46" s="31">
         <v>43</v>
       </c>
       <c r="C46" s="43" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="D46" s="31">
         <v>1</v>
@@ -17109,88 +17109,92 @@
         <v>760</v>
       </c>
       <c r="F46" s="44">
-        <v>14503</v>
+        <v>15000</v>
       </c>
       <c r="G46" s="44">
-        <f>F46*D46</f>
-        <v>14503</v>
+        <f t="shared" si="1"/>
+        <v>15000</v>
       </c>
       <c r="H46" s="31" t="s">
         <v>837</v>
       </c>
       <c r="I46" s="31" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B47" s="31">
         <v>44</v>
       </c>
-      <c r="C47" s="49" t="s">
-        <v>845</v>
+      <c r="C47" s="43" t="s">
+        <v>786</v>
       </c>
       <c r="D47" s="31">
-        <v>1455.89</v>
+        <v>1</v>
       </c>
       <c r="E47" s="31" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="F47" s="44">
-        <v>95.9</v>
+        <v>404191.96</v>
       </c>
       <c r="G47" s="44">
         <f t="shared" si="1"/>
-        <v>139619.85100000002</v>
+        <v>404191.96</v>
       </c>
       <c r="H47" s="31" t="s">
-        <v>791</v>
-      </c>
-      <c r="I47" s="31"/>
+        <v>837</v>
+      </c>
+      <c r="I47" s="31" t="s">
+        <v>786</v>
+      </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B48" s="31">
         <v>45</v>
       </c>
       <c r="C48" s="43" t="s">
-        <v>846</v>
+        <v>921</v>
       </c>
       <c r="D48" s="31">
-        <v>706.94</v>
+        <v>1</v>
       </c>
       <c r="E48" s="31" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="F48" s="44">
-        <v>95.9</v>
+        <v>14503</v>
       </c>
       <c r="G48" s="44">
-        <f t="shared" si="1"/>
-        <v>67795.546000000002</v>
+        <f>F48*D48</f>
+        <v>14503</v>
       </c>
       <c r="H48" s="31" t="s">
-        <v>791</v>
-      </c>
-      <c r="I48" s="31"/>
+        <v>837</v>
+      </c>
+      <c r="I48" s="31" t="s">
+        <v>921</v>
+      </c>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B49" s="31">
         <v>46</v>
       </c>
-      <c r="C49" s="46" t="s">
-        <v>847</v>
+      <c r="C49" s="49" t="s">
+        <v>845</v>
       </c>
       <c r="D49" s="31">
-        <v>44</v>
+        <v>1455.89</v>
       </c>
       <c r="E49" s="31" t="s">
-        <v>818</v>
+        <v>761</v>
       </c>
       <c r="F49" s="44">
-        <v>95</v>
+        <v>95.9</v>
       </c>
       <c r="G49" s="44">
         <f t="shared" si="1"/>
-        <v>4180</v>
+        <v>139619.85100000002</v>
       </c>
       <c r="H49" s="31" t="s">
         <v>791</v>
@@ -17201,21 +17205,21 @@
       <c r="B50" s="31">
         <v>47</v>
       </c>
-      <c r="C50" s="46" t="s">
-        <v>848</v>
+      <c r="C50" s="43" t="s">
+        <v>846</v>
       </c>
       <c r="D50" s="31">
-        <v>3</v>
+        <v>706.94</v>
       </c>
       <c r="E50" s="31" t="s">
-        <v>818</v>
+        <v>761</v>
       </c>
       <c r="F50" s="44">
-        <v>35</v>
+        <v>95.9</v>
       </c>
       <c r="G50" s="44">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>67795.546000000002</v>
       </c>
       <c r="H50" s="31" t="s">
         <v>791</v>
@@ -17227,20 +17231,20 @@
         <v>48</v>
       </c>
       <c r="C51" s="46" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="D51" s="31">
-        <v>126</v>
+        <v>44</v>
       </c>
       <c r="E51" s="31" t="s">
-        <v>760</v>
+        <v>818</v>
       </c>
       <c r="F51" s="44">
-        <v>25.9</v>
+        <v>95</v>
       </c>
       <c r="G51" s="44">
         <f t="shared" si="1"/>
-        <v>3263.3999999999996</v>
+        <v>4180</v>
       </c>
       <c r="H51" s="31" t="s">
         <v>791</v>
@@ -17252,20 +17256,20 @@
         <v>49</v>
       </c>
       <c r="C52" s="46" t="s">
-        <v>817</v>
+        <v>848</v>
       </c>
       <c r="D52" s="31">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E52" s="31" t="s">
-        <v>760</v>
+        <v>818</v>
       </c>
       <c r="F52" s="44">
-        <v>1750</v>
+        <v>35</v>
       </c>
       <c r="G52" s="44">
-        <f>F52*D52</f>
-        <v>1750</v>
+        <f t="shared" si="1"/>
+        <v>105</v>
       </c>
       <c r="H52" s="31" t="s">
         <v>791</v>
@@ -17276,24 +17280,24 @@
       <c r="B53" s="31">
         <v>50</v>
       </c>
-      <c r="C53" s="43" t="s">
-        <v>781</v>
+      <c r="C53" s="46" t="s">
+        <v>849</v>
       </c>
       <c r="D53" s="31">
-        <v>1</v>
+        <v>126</v>
       </c>
       <c r="E53" s="31" t="s">
         <v>760</v>
       </c>
       <c r="F53" s="44">
-        <v>174417.38</v>
+        <v>25.9</v>
       </c>
       <c r="G53" s="44">
-        <f>F53*D53</f>
-        <v>174417.38</v>
+        <f t="shared" si="1"/>
+        <v>3263.3999999999996</v>
       </c>
       <c r="H53" s="31" t="s">
-        <v>780</v>
+        <v>791</v>
       </c>
       <c r="I53" s="31"/>
     </row>
@@ -17301,57 +17305,107 @@
       <c r="B54" s="31">
         <v>51</v>
       </c>
-      <c r="C54" s="32" t="s">
+      <c r="C54" s="46" t="s">
+        <v>817</v>
+      </c>
+      <c r="D54" s="31">
+        <v>1</v>
+      </c>
+      <c r="E54" s="31" t="s">
+        <v>760</v>
+      </c>
+      <c r="F54" s="44">
+        <v>1750</v>
+      </c>
+      <c r="G54" s="44">
+        <f>F54*D54</f>
+        <v>1750</v>
+      </c>
+      <c r="H54" s="31" t="s">
+        <v>791</v>
+      </c>
+      <c r="I54" s="31"/>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B55" s="31">
+        <v>52</v>
+      </c>
+      <c r="C55" s="43" t="s">
+        <v>781</v>
+      </c>
+      <c r="D55" s="31">
+        <v>1</v>
+      </c>
+      <c r="E55" s="31" t="s">
+        <v>760</v>
+      </c>
+      <c r="F55" s="44">
+        <v>174417.38</v>
+      </c>
+      <c r="G55" s="44">
+        <f>F55*D55</f>
+        <v>174417.38</v>
+      </c>
+      <c r="H55" s="31" t="s">
+        <v>780</v>
+      </c>
+      <c r="I55" s="31"/>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B56" s="31">
+        <v>53</v>
+      </c>
+      <c r="C56" s="32" t="s">
         <v>814</v>
       </c>
-      <c r="D54" s="33">
-        <v>1</v>
-      </c>
-      <c r="E54" s="33" t="s">
+      <c r="D56" s="33">
+        <v>1</v>
+      </c>
+      <c r="E56" s="33" t="s">
         <v>760</v>
       </c>
-      <c r="F54" s="25">
+      <c r="F56" s="25">
         <v>5000</v>
       </c>
-      <c r="G54" s="25">
-        <f>F54*D54</f>
+      <c r="G56" s="25">
+        <f>F56*D56</f>
         <v>5000</v>
       </c>
-      <c r="H54" s="33" t="s">
+      <c r="H56" s="33" t="s">
         <v>815</v>
       </c>
-      <c r="I54" s="31"/>
-    </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B55" s="33"/>
-      <c r="C55" s="32"/>
-      <c r="D55" s="33"/>
-      <c r="E55" s="33"/>
-      <c r="F55" s="20"/>
-      <c r="G55" s="20"/>
-      <c r="H55" s="33"/>
-      <c r="I55" s="33"/>
-    </row>
-    <row r="56" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B56" s="33"/>
-      <c r="C56" s="32"/>
-      <c r="D56" s="33"/>
-      <c r="E56" s="33"/>
-      <c r="H56" s="33"/>
-      <c r="I56" s="33"/>
+      <c r="I56" s="31"/>
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="G57" s="16">
+      <c r="B57" s="33"/>
+      <c r="C57" s="32"/>
+      <c r="D57" s="33"/>
+      <c r="E57" s="33"/>
+      <c r="F57" s="20"/>
+      <c r="G57" s="20"/>
+      <c r="H57" s="33"/>
+      <c r="I57" s="33"/>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B58" s="33"/>
+      <c r="C58" s="32"/>
+      <c r="D58" s="33"/>
+      <c r="E58" s="33"/>
+      <c r="H58" s="33"/>
+      <c r="I58" s="33"/>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="G59" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
         <v>3195411.5038461541</v>
       </c>
     </row>
-    <row r="83" spans="8:9" x14ac:dyDescent="0.25">
-      <c r="H83" s="26">
-        <f>SUM('Expansão DMP'!G57,H79)</f>
+    <row r="85" spans="8:9" x14ac:dyDescent="0.25">
+      <c r="H85" s="26">
+        <f>SUM('Expansão DMP'!G59,H81)</f>
         <v>3195411.5038461541</v>
       </c>
-      <c r="I83" s="26"/>
+      <c r="I85" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -17399,7 +17453,7 @@
         <v>908</v>
       </c>
       <c r="D2" s="39">
-        <f>'Expansão DMP'!G57</f>
+        <f>'Expansão DMP'!G59</f>
         <v>3195411.5038461541</v>
       </c>
       <c r="G2" s="14" t="s">

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 15:25
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -16043,10 +16043,12 @@
       <c r="E4" s="33" t="s">
         <v>760</v>
       </c>
-      <c r="F4" s="20"/>
+      <c r="F4" s="20">
+        <v>1019077.5</v>
+      </c>
       <c r="G4" s="20">
         <f t="shared" ref="G4:G20" si="0">F4*D4</f>
-        <v>0</v>
+        <v>1019077.5</v>
       </c>
       <c r="H4" s="33" t="s">
         <v>798</v>
@@ -16069,10 +16071,12 @@
       <c r="E5" s="33" t="s">
         <v>760</v>
       </c>
-      <c r="F5" s="20"/>
+      <c r="F5" s="20">
+        <v>70700</v>
+      </c>
       <c r="G5" s="20">
         <f>F5*D5</f>
-        <v>0</v>
+        <v>70700</v>
       </c>
       <c r="H5" s="33" t="s">
         <v>798</v>
@@ -16093,10 +16097,12 @@
       <c r="E6" s="33" t="s">
         <v>760</v>
       </c>
-      <c r="F6" s="20"/>
+      <c r="F6" s="20">
+        <v>88200</v>
+      </c>
       <c r="G6" s="20">
         <f>F6*D6</f>
-        <v>0</v>
+        <v>88200</v>
       </c>
       <c r="H6" s="33" t="s">
         <v>798</v>
@@ -17397,13 +17403,13 @@
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
       <c r="G59" s="16">
         <f>SUM(Tabela2[Preço Total])</f>
-        <v>3195411.5038461541</v>
+        <v>4373389.0038461545</v>
       </c>
     </row>
     <row r="85" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H85" s="26">
         <f>SUM('Expansão DMP'!G59,H81)</f>
-        <v>3195411.5038461541</v>
+        <v>4373389.0038461545</v>
       </c>
       <c r="I85" s="26"/>
     </row>
@@ -17454,7 +17460,7 @@
       </c>
       <c r="D2" s="39">
         <f>'Expansão DMP'!G59</f>
-        <v>3195411.5038461541</v>
+        <v>4373389.0038461545</v>
       </c>
       <c r="G2" s="14" t="s">
         <v>913</v>
@@ -17510,11 +17516,11 @@
       </c>
       <c r="E7" s="41">
         <f t="shared" ref="E7:E20" si="0">D7/$D$2</f>
-        <v>0.38206336446198724</v>
+        <v>0.27915414542962674</v>
       </c>
       <c r="F7" s="41">
         <f>E7</f>
-        <v>0.38206336446198724</v>
+        <v>0.27915414542962674</v>
       </c>
       <c r="G7" s="14" t="s">
         <v>913</v>
@@ -17534,7 +17540,7 @@
       </c>
       <c r="F8" s="41">
         <f t="shared" ref="F8:F20" si="1">F7+E8</f>
-        <v>0.38206336446198724</v>
+        <v>0.27915414542962674</v>
       </c>
       <c r="G8" s="14" t="s">
         <v>913</v>
@@ -17554,7 +17560,7 @@
       </c>
       <c r="F9" s="41">
         <f t="shared" si="1"/>
-        <v>0.38206336446198724</v>
+        <v>0.27915414542962674</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>913</v>
@@ -17570,11 +17576,11 @@
       </c>
       <c r="E10" s="41">
         <f t="shared" si="0"/>
-        <v>0.11301566430848679</v>
+        <v>8.2574761478697328E-2</v>
       </c>
       <c r="F10" s="41">
         <f t="shared" si="1"/>
-        <v>0.49507902877047405</v>
+        <v>0.36172890690832404</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>913</v>
@@ -17590,11 +17596,11 @@
       </c>
       <c r="E11" s="41">
         <f t="shared" si="0"/>
-        <v>6.782030944657759E-2</v>
+        <v>4.9552828895259984E-2</v>
       </c>
       <c r="F11" s="41">
         <f t="shared" si="1"/>
-        <v>0.56289933821705163</v>
+        <v>0.41128173580358401</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>914</v>
@@ -17610,11 +17616,11 @@
       </c>
       <c r="E12" s="41">
         <f t="shared" si="0"/>
-        <v>5.4583699091670254E-2</v>
+        <v>3.9881515192590811E-2</v>
       </c>
       <c r="F12" s="41">
         <f t="shared" si="1"/>
-        <v>0.61748303730872189</v>
+        <v>0.45116325099617482</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>914</v>
@@ -17630,11 +17636,11 @@
       </c>
       <c r="E13" s="41">
         <f t="shared" si="0"/>
-        <v>5.1429995730500534E-2</v>
+        <v>3.7577265561209404E-2</v>
       </c>
       <c r="F13" s="41">
         <f t="shared" si="1"/>
-        <v>0.66891303303922245</v>
+        <v>0.48874051655738421</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>915</v>
@@ -17650,11 +17656,11 @@
       </c>
       <c r="E14" s="41">
         <f t="shared" si="0"/>
-        <v>2.4766254019160026E-2</v>
+        <v>1.809543421140954E-2</v>
       </c>
       <c r="F14" s="41">
         <f t="shared" si="1"/>
-        <v>0.69367928705838244</v>
+        <v>0.50683595076879373</v>
       </c>
       <c r="G14" s="14" t="s">
         <v>915</v>
@@ -17670,11 +17676,11 @@
       </c>
       <c r="E15" s="41">
         <f t="shared" si="0"/>
-        <v>6.7680422299190787E-3</v>
+        <v>4.945062051644738E-3</v>
       </c>
       <c r="F15" s="41">
         <f t="shared" si="1"/>
-        <v>0.70044732928830156</v>
+        <v>0.51178101282043842</v>
       </c>
       <c r="G15" s="14" t="s">
         <v>915</v>
@@ -17690,11 +17696,11 @@
       </c>
       <c r="E16" s="41">
         <f t="shared" si="0"/>
-        <v>5.7950564356770073E-3</v>
+        <v>4.2341511317001077E-3</v>
       </c>
       <c r="F16" s="41">
         <f t="shared" si="1"/>
-        <v>0.70624238572397857</v>
+        <v>0.51601516395213853</v>
       </c>
       <c r="G16" s="14" t="s">
         <v>915</v>
@@ -17710,11 +17716,11 @@
       </c>
       <c r="E17" s="41">
         <f t="shared" si="0"/>
-        <v>2.0942373124541988E-2</v>
+        <v>1.5301520157742197E-2</v>
       </c>
       <c r="F17" s="41">
         <f t="shared" si="1"/>
-        <v>0.72718475884852052</v>
+        <v>0.53131668410988075</v>
       </c>
       <c r="G17" s="14" t="s">
         <v>915</v>
@@ -17730,11 +17736,11 @@
       </c>
       <c r="E18" s="41">
         <f t="shared" si="0"/>
-        <v>1.6586283155144994E-3</v>
+        <v>1.2118748172959099E-3</v>
       </c>
       <c r="F18" s="41">
         <f t="shared" si="1"/>
-        <v>0.72884338716403507</v>
+        <v>0.53252855892717665</v>
       </c>
       <c r="G18" s="14" t="s">
         <v>915</v>
@@ -17750,11 +17756,11 @@
       </c>
       <c r="E19" s="41">
         <f t="shared" si="0"/>
-        <v>1.5647436938816032E-3</v>
+        <v>1.1432781295244432E-3</v>
       </c>
       <c r="F19" s="41">
         <f t="shared" si="1"/>
-        <v>0.73040813085791667</v>
+        <v>0.53367183705670107</v>
       </c>
       <c r="G19" s="14" t="s">
         <v>915</v>
@@ -17766,15 +17772,15 @@
       </c>
       <c r="D20" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Armazenamento",Tabela2[Preço Total])</f>
-        <v>0</v>
+        <v>1177977.5</v>
       </c>
       <c r="E20" s="41">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.26935118256437596</v>
       </c>
       <c r="F20" s="41">
         <f t="shared" si="1"/>
-        <v>0.73040813085791667</v>
+        <v>0.80302301962107703</v>
       </c>
       <c r="G20" s="14" t="s">
         <v>915</v>

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 15:30
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2372" uniqueCount="931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2378" uniqueCount="931">
   <si>
     <t>Código EAP</t>
   </si>
@@ -3397,8 +3397,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B1:J98" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
-  <autoFilter ref="B1:J98"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B1:J100" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+  <autoFilter ref="B1:J100"/>
   <sortState ref="B2:J98">
     <sortCondition ref="I1:I98"/>
   </sortState>
@@ -12866,7 +12866,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:O105"/>
+  <dimension ref="B1:O107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" customWidth="1"/>
@@ -12928,10 +12928,13 @@
       <c r="F2" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G2" s="20"/>
+      <c r="G2" s="20">
+        <f>1204691.84+68961.33</f>
+        <v>1273653.1700000002</v>
+      </c>
       <c r="H2" s="20">
-        <f t="shared" ref="H2:H33" si="0">G2*E2</f>
-        <v>0</v>
+        <f t="shared" ref="H2:H35" si="0">G2*E2</f>
+        <v>1273653.1700000002</v>
       </c>
       <c r="I2" s="18" t="s">
         <v>798</v>
@@ -12947,24 +12950,24 @@
         <v>2</v>
       </c>
       <c r="C3" s="17"/>
-      <c r="D3" s="50" t="s">
-        <v>819</v>
-      </c>
-      <c r="E3" s="17">
-        <v>1</v>
-      </c>
-      <c r="F3" s="17" t="s">
+      <c r="D3" s="19" t="s">
+        <v>929</v>
+      </c>
+      <c r="E3" s="18">
+        <v>1</v>
+      </c>
+      <c r="F3" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G3" s="44">
-        <v>486032</v>
-      </c>
-      <c r="H3" s="44">
-        <f t="shared" si="0"/>
-        <v>486032</v>
-      </c>
-      <c r="I3" s="31" t="s">
-        <v>920</v>
+      <c r="G3" s="20">
+        <v>185900</v>
+      </c>
+      <c r="H3" s="20">
+        <f>G3*E3</f>
+        <v>185900</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>798</v>
       </c>
       <c r="J3" s="27"/>
       <c r="K3" s="27"/>
@@ -12974,24 +12977,24 @@
         <v>3</v>
       </c>
       <c r="C4" s="17"/>
-      <c r="D4" s="50" t="s">
-        <v>821</v>
-      </c>
-      <c r="E4" s="17">
-        <v>1</v>
-      </c>
-      <c r="F4" s="17" t="s">
+      <c r="D4" s="19" t="s">
+        <v>930</v>
+      </c>
+      <c r="E4" s="18">
+        <v>1</v>
+      </c>
+      <c r="F4" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G4" s="44">
-        <v>8650</v>
-      </c>
-      <c r="H4" s="44">
-        <f t="shared" si="0"/>
-        <v>8650</v>
-      </c>
-      <c r="I4" s="31" t="s">
-        <v>920</v>
+      <c r="G4" s="20">
+        <v>88200</v>
+      </c>
+      <c r="H4" s="20">
+        <f>G4*E4</f>
+        <v>88200</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>798</v>
       </c>
       <c r="J4" s="27"/>
       <c r="K4" s="27"/>
@@ -13002,23 +13005,23 @@
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="50" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="E5" s="17">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>760</v>
       </c>
       <c r="G5" s="44">
-        <v>21938</v>
+        <v>486032</v>
       </c>
       <c r="H5" s="44">
         <f t="shared" si="0"/>
-        <v>131628</v>
-      </c>
-      <c r="I5" s="17" t="s">
-        <v>835</v>
+        <v>486032</v>
+      </c>
+      <c r="I5" s="31" t="s">
+        <v>920</v>
       </c>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
@@ -13029,7 +13032,7 @@
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="50" t="s">
-        <v>899</v>
+        <v>821</v>
       </c>
       <c r="E6" s="17">
         <v>1</v>
@@ -13038,14 +13041,14 @@
         <v>760</v>
       </c>
       <c r="G6" s="44">
-        <v>11180</v>
+        <v>8650</v>
       </c>
       <c r="H6" s="44">
         <f t="shared" si="0"/>
-        <v>11180</v>
-      </c>
-      <c r="I6" s="17" t="s">
-        <v>835</v>
+        <v>8650</v>
+      </c>
+      <c r="I6" s="31" t="s">
+        <v>920</v>
       </c>
       <c r="J6" s="27"/>
       <c r="K6" s="27"/>
@@ -13055,21 +13058,21 @@
         <v>6</v>
       </c>
       <c r="C7" s="17"/>
-      <c r="D7" s="19" t="s">
-        <v>889</v>
+      <c r="D7" s="50" t="s">
+        <v>820</v>
       </c>
       <c r="E7" s="17">
-        <v>250</v>
+        <v>6</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G7" s="44">
-        <v>55.57</v>
+        <v>21938</v>
       </c>
       <c r="H7" s="44">
         <f t="shared" si="0"/>
-        <v>13892.5</v>
+        <v>131628</v>
       </c>
       <c r="I7" s="17" t="s">
         <v>835</v>
@@ -13081,22 +13084,22 @@
       <c r="B8" s="17">
         <v>7</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="19" t="s">
-        <v>888</v>
-      </c>
-      <c r="E8" s="18">
-        <v>6</v>
-      </c>
-      <c r="F8" s="18" t="s">
+      <c r="C8" s="17"/>
+      <c r="D8" s="50" t="s">
+        <v>899</v>
+      </c>
+      <c r="E8" s="17">
+        <v>1</v>
+      </c>
+      <c r="F8" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G8" s="25">
-        <v>13855.22</v>
-      </c>
-      <c r="H8" s="51">
+      <c r="G8" s="44">
+        <v>11180</v>
+      </c>
+      <c r="H8" s="44">
         <f t="shared" si="0"/>
-        <v>83131.319999999992</v>
+        <v>11180</v>
       </c>
       <c r="I8" s="17" t="s">
         <v>835</v>
@@ -13108,22 +13111,22 @@
       <c r="B9" s="17">
         <v>8</v>
       </c>
-      <c r="C9" s="18"/>
+      <c r="C9" s="17"/>
       <c r="D9" s="19" t="s">
-        <v>886</v>
-      </c>
-      <c r="E9" s="18">
-        <v>1</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>760</v>
-      </c>
-      <c r="G9" s="25">
-        <v>111260.98</v>
-      </c>
-      <c r="H9" s="51">
+        <v>889</v>
+      </c>
+      <c r="E9" s="17">
+        <v>250</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>761</v>
+      </c>
+      <c r="G9" s="44">
+        <v>55.57</v>
+      </c>
+      <c r="H9" s="44">
         <f t="shared" si="0"/>
-        <v>111260.98</v>
+        <v>13892.5</v>
       </c>
       <c r="I9" s="17" t="s">
         <v>835</v>
@@ -13137,20 +13140,20 @@
       </c>
       <c r="C10" s="18"/>
       <c r="D10" s="19" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="E10" s="18">
-        <v>300</v>
+        <v>6</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G10" s="25">
-        <v>55.57</v>
+        <v>13855.22</v>
       </c>
       <c r="H10" s="51">
         <f t="shared" si="0"/>
-        <v>16671</v>
+        <v>83131.319999999992</v>
       </c>
       <c r="I10" s="17" t="s">
         <v>835</v>
@@ -13164,7 +13167,7 @@
       </c>
       <c r="C11" s="18"/>
       <c r="D11" s="19" t="s">
-        <v>838</v>
+        <v>886</v>
       </c>
       <c r="E11" s="18">
         <v>1</v>
@@ -13173,11 +13176,11 @@
         <v>760</v>
       </c>
       <c r="G11" s="25">
-        <v>27412.5</v>
+        <v>111260.98</v>
       </c>
       <c r="H11" s="51">
         <f t="shared" si="0"/>
-        <v>27412.5</v>
+        <v>111260.98</v>
       </c>
       <c r="I11" s="17" t="s">
         <v>835</v>
@@ -13191,23 +13194,22 @@
       </c>
       <c r="C12" s="18"/>
       <c r="D12" s="19" t="s">
-        <v>757</v>
-      </c>
-      <c r="E12" s="52">
-        <f>(1075*0.15)*1.1</f>
-        <v>177.37500000000003</v>
+        <v>887</v>
+      </c>
+      <c r="E12" s="18">
+        <v>300</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="G12" s="25">
-        <v>670</v>
-      </c>
-      <c r="H12" s="25">
+        <v>55.57</v>
+      </c>
+      <c r="H12" s="51">
         <f t="shared" si="0"/>
-        <v>118841.25000000001</v>
-      </c>
-      <c r="I12" s="18" t="s">
+        <v>16671</v>
+      </c>
+      <c r="I12" s="17" t="s">
         <v>835</v>
       </c>
       <c r="J12" s="27"/>
@@ -13218,24 +13220,23 @@
         <v>12</v>
       </c>
       <c r="C13" s="18"/>
-      <c r="D13" s="50" t="s">
-        <v>775</v>
-      </c>
-      <c r="E13" s="52">
-        <f>1075/13*2</f>
-        <v>165.38461538461539</v>
+      <c r="D13" s="19" t="s">
+        <v>838</v>
+      </c>
+      <c r="E13" s="18">
+        <v>1</v>
       </c>
       <c r="F13" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G13" s="25">
-        <v>220.5</v>
-      </c>
-      <c r="H13" s="25">
+        <v>27412.5</v>
+      </c>
+      <c r="H13" s="51">
         <f t="shared" si="0"/>
-        <v>36467.307692307695</v>
-      </c>
-      <c r="I13" s="18" t="s">
+        <v>27412.5</v>
+      </c>
+      <c r="I13" s="17" t="s">
         <v>835</v>
       </c>
       <c r="J13" s="27"/>
@@ -13246,22 +13247,22 @@
         <v>13</v>
       </c>
       <c r="C14" s="18"/>
-      <c r="D14" s="50" t="s">
-        <v>758</v>
+      <c r="D14" s="19" t="s">
+        <v>757</v>
       </c>
       <c r="E14" s="52">
-        <f>(20*53)/12</f>
-        <v>88.333333333333329</v>
+        <f>(1075*0.15)*1.1</f>
+        <v>177.37500000000003</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G14" s="25">
-        <v>56.2</v>
+        <v>670</v>
       </c>
       <c r="H14" s="25">
         <f t="shared" si="0"/>
-        <v>4964.333333333333</v>
+        <v>118841.25000000001</v>
       </c>
       <c r="I14" s="18" t="s">
         <v>835</v>
@@ -13275,21 +13276,21 @@
       </c>
       <c r="C15" s="18"/>
       <c r="D15" s="50" t="s">
-        <v>792</v>
+        <v>775</v>
       </c>
       <c r="E15" s="52">
-        <f>E12</f>
-        <v>177.37500000000003</v>
+        <f>1075/13*2</f>
+        <v>165.38461538461539</v>
       </c>
       <c r="F15" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G15" s="25">
-        <v>50</v>
+        <v>220.5</v>
       </c>
       <c r="H15" s="25">
         <f t="shared" si="0"/>
-        <v>8868.7500000000018</v>
+        <v>36467.307692307695</v>
       </c>
       <c r="I15" s="18" t="s">
         <v>835</v>
@@ -13301,22 +13302,23 @@
       <c r="B16" s="17">
         <v>15</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="19" t="s">
-        <v>839</v>
-      </c>
-      <c r="E16" s="18">
-        <v>1</v>
+      <c r="C16" s="18"/>
+      <c r="D16" s="50" t="s">
+        <v>758</v>
+      </c>
+      <c r="E16" s="52">
+        <f>(20*53)/12</f>
+        <v>88.333333333333329</v>
       </c>
       <c r="F16" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G16" s="25">
-        <v>67000</v>
+        <v>56.2</v>
       </c>
       <c r="H16" s="25">
         <f t="shared" si="0"/>
-        <v>67000</v>
+        <v>4964.333333333333</v>
       </c>
       <c r="I16" s="18" t="s">
         <v>835</v>
@@ -13329,160 +13331,158 @@
         <v>16</v>
       </c>
       <c r="C17" s="18"/>
-      <c r="D17" s="19" t="s">
-        <v>884</v>
-      </c>
-      <c r="E17" s="18">
-        <v>1</v>
+      <c r="D17" s="50" t="s">
+        <v>792</v>
+      </c>
+      <c r="E17" s="52">
+        <f>E14</f>
+        <v>177.37500000000003</v>
       </c>
       <c r="F17" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G17" s="25">
+        <v>50</v>
+      </c>
+      <c r="H17" s="25">
+        <f t="shared" si="0"/>
+        <v>8868.7500000000018</v>
+      </c>
+      <c r="I17" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="17">
+        <v>17</v>
+      </c>
+      <c r="C18" s="17"/>
+      <c r="D18" s="19" t="s">
+        <v>839</v>
+      </c>
+      <c r="E18" s="18">
+        <v>1</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G18" s="25">
+        <v>67000</v>
+      </c>
+      <c r="H18" s="25">
+        <f t="shared" si="0"/>
+        <v>67000</v>
+      </c>
+      <c r="I18" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B19" s="17">
+        <v>18</v>
+      </c>
+      <c r="C19" s="18"/>
+      <c r="D19" s="19" t="s">
+        <v>884</v>
+      </c>
+      <c r="E19" s="18">
+        <v>1</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G19" s="25">
         <v>48600</v>
       </c>
-      <c r="H17" s="51">
+      <c r="H19" s="51">
         <f t="shared" si="0"/>
         <v>48600</v>
       </c>
-      <c r="I17" s="18" t="s">
+      <c r="I19" s="18" t="s">
         <v>835</v>
       </c>
-      <c r="J17" s="27"/>
-      <c r="K17" s="27"/>
-    </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B18" s="17"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="19" t="s">
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B20" s="17">
+        <v>19</v>
+      </c>
+      <c r="C20" s="18"/>
+      <c r="D20" s="19" t="s">
         <v>918</v>
       </c>
-      <c r="E18" s="18">
-        <v>1</v>
-      </c>
-      <c r="F18" s="18" t="s">
+      <c r="E20" s="18">
+        <v>1</v>
+      </c>
+      <c r="F20" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G18" s="25">
+      <c r="G20" s="25">
         <v>48600</v>
       </c>
-      <c r="H18" s="51">
+      <c r="H20" s="51">
         <f t="shared" si="0"/>
         <v>48600</v>
       </c>
-      <c r="I18" s="18" t="s">
+      <c r="I20" s="18" t="s">
         <v>835</v>
       </c>
-      <c r="J18" s="27"/>
-      <c r="K18" s="27"/>
-    </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B19" s="17">
-        <v>17</v>
-      </c>
-      <c r="C19" s="18"/>
-      <c r="D19" s="19" t="s">
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B21" s="17">
+        <v>20</v>
+      </c>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19" t="s">
         <v>885</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E21" s="18">
         <v>50</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F21" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G19" s="25">
+      <c r="G21" s="25">
         <v>243.39</v>
       </c>
-      <c r="H19" s="51">
+      <c r="H21" s="51">
         <f t="shared" si="0"/>
         <v>12169.5</v>
       </c>
-      <c r="I19" s="18" t="s">
-        <v>835</v>
-      </c>
-      <c r="J19" s="27"/>
-      <c r="K19" s="27"/>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="17">
-        <v>18</v>
-      </c>
-      <c r="C20" s="18"/>
-      <c r="D20" s="19" t="s">
-        <v>880</v>
-      </c>
-      <c r="E20" s="18">
-        <f>44*4</f>
-        <v>176</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>760</v>
-      </c>
-      <c r="G20" s="25">
-        <v>38.119999999999997</v>
-      </c>
-      <c r="H20" s="51">
-        <f t="shared" si="0"/>
-        <v>6709.12</v>
-      </c>
-      <c r="I20" s="18" t="s">
-        <v>835</v>
-      </c>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B21" s="17">
-        <v>19</v>
-      </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="19" t="s">
-        <v>824</v>
-      </c>
-      <c r="E21" s="18">
-        <v>10</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>760</v>
-      </c>
-      <c r="G21" s="25">
-        <v>24</v>
-      </c>
-      <c r="H21" s="51">
-        <f t="shared" si="0"/>
-        <v>240</v>
-      </c>
       <c r="I21" s="18" t="s">
         <v>835</v>
       </c>
       <c r="J21" s="27"/>
       <c r="K21" s="27"/>
-      <c r="L21" s="24" t="s">
-        <v>890</v>
-      </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="17">
         <v>21</v>
       </c>
-      <c r="C22" s="18" t="s">
-        <v>877</v>
-      </c>
+      <c r="C22" s="18"/>
       <c r="D22" s="19" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="E22" s="18">
-        <v>36</v>
+        <f>44*4</f>
+        <v>176</v>
       </c>
       <c r="F22" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G22" s="25">
-        <v>243.39</v>
+        <v>38.119999999999997</v>
       </c>
       <c r="H22" s="51">
         <f t="shared" si="0"/>
-        <v>8762.0399999999991</v>
+        <v>6709.12</v>
       </c>
       <c r="I22" s="18" t="s">
         <v>835</v>
@@ -13494,30 +13494,31 @@
       <c r="B23" s="17">
         <v>22</v>
       </c>
-      <c r="C23" s="18" t="s">
-        <v>877</v>
-      </c>
+      <c r="C23" s="18"/>
       <c r="D23" s="19" t="s">
-        <v>856</v>
+        <v>824</v>
       </c>
       <c r="E23" s="18">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G23" s="25">
-        <v>38.119999999999997</v>
+        <v>24</v>
       </c>
       <c r="H23" s="51">
         <f t="shared" si="0"/>
-        <v>2744.64</v>
+        <v>240</v>
       </c>
       <c r="I23" s="18" t="s">
         <v>835</v>
       </c>
       <c r="J23" s="27"/>
       <c r="K23" s="27"/>
+      <c r="L23" s="24" t="s">
+        <v>890</v>
+      </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="17">
@@ -13527,20 +13528,20 @@
         <v>877</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>778</v>
+        <v>876</v>
       </c>
       <c r="E24" s="18">
         <v>36</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G24" s="25">
-        <v>32</v>
+        <v>243.39</v>
       </c>
       <c r="H24" s="51">
         <f t="shared" si="0"/>
-        <v>1152</v>
+        <v>8762.0399999999991</v>
       </c>
       <c r="I24" s="18" t="s">
         <v>835</v>
@@ -13556,20 +13557,20 @@
         <v>877</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>871</v>
+        <v>856</v>
       </c>
       <c r="E25" s="18">
-        <v>4</v>
+        <v>72</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="G25" s="25">
-        <v>419</v>
+        <v>38.119999999999997</v>
       </c>
       <c r="H25" s="51">
         <f t="shared" si="0"/>
-        <v>1676</v>
+        <v>2744.64</v>
       </c>
       <c r="I25" s="18" t="s">
         <v>835</v>
@@ -13585,21 +13586,20 @@
         <v>877</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>857</v>
+        <v>778</v>
       </c>
       <c r="E26" s="18">
-        <f>8*6</f>
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="F26" s="18" t="s">
         <v>761</v>
       </c>
       <c r="G26" s="25">
-        <v>38.119999999999997</v>
+        <v>32</v>
       </c>
       <c r="H26" s="51">
         <f t="shared" si="0"/>
-        <v>1829.7599999999998</v>
+        <v>1152</v>
       </c>
       <c r="I26" s="18" t="s">
         <v>835</v>
@@ -13611,22 +13611,24 @@
       <c r="B27" s="17">
         <v>26</v>
       </c>
-      <c r="C27" s="17"/>
+      <c r="C27" s="18" t="s">
+        <v>877</v>
+      </c>
       <c r="D27" s="19" t="s">
-        <v>917</v>
+        <v>871</v>
       </c>
       <c r="E27" s="18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F27" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G27" s="25">
-        <v>65000</v>
-      </c>
-      <c r="H27" s="25">
+        <v>419</v>
+      </c>
+      <c r="H27" s="51">
         <f t="shared" si="0"/>
-        <v>130000</v>
+        <v>1676</v>
       </c>
       <c r="I27" s="18" t="s">
         <v>835</v>
@@ -13638,27 +13640,28 @@
       <c r="B28" s="17">
         <v>27</v>
       </c>
-      <c r="C28" s="17" t="s">
-        <v>878</v>
-      </c>
-      <c r="D28" s="50" t="s">
-        <v>861</v>
-      </c>
-      <c r="E28" s="17">
-        <v>58</v>
-      </c>
-      <c r="F28" s="17" t="s">
-        <v>881</v>
-      </c>
-      <c r="G28" s="44">
-        <v>198.72</v>
-      </c>
-      <c r="H28" s="44">
+      <c r="C28" s="18" t="s">
+        <v>877</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>857</v>
+      </c>
+      <c r="E28" s="18">
+        <f>8*6</f>
+        <v>48</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G28" s="25">
+        <v>38.119999999999997</v>
+      </c>
+      <c r="H28" s="51">
         <f t="shared" si="0"/>
-        <v>11525.76</v>
-      </c>
-      <c r="I28" s="17" t="s">
-        <v>868</v>
+        <v>1829.7599999999998</v>
+      </c>
+      <c r="I28" s="18" t="s">
+        <v>835</v>
       </c>
       <c r="J28" s="27"/>
       <c r="K28" s="27"/>
@@ -13667,27 +13670,25 @@
       <c r="B29" s="17">
         <v>28</v>
       </c>
-      <c r="C29" s="17" t="s">
-        <v>879</v>
-      </c>
-      <c r="D29" s="50" t="s">
-        <v>864</v>
-      </c>
-      <c r="E29" s="17">
-        <v>31</v>
-      </c>
-      <c r="F29" s="17" t="s">
-        <v>881</v>
-      </c>
-      <c r="G29" s="44">
-        <v>484.24</v>
-      </c>
-      <c r="H29" s="44">
+      <c r="C29" s="17"/>
+      <c r="D29" s="19" t="s">
+        <v>917</v>
+      </c>
+      <c r="E29" s="18">
+        <v>2</v>
+      </c>
+      <c r="F29" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G29" s="25">
+        <v>65000</v>
+      </c>
+      <c r="H29" s="25">
         <f t="shared" si="0"/>
-        <v>15011.44</v>
-      </c>
-      <c r="I29" s="17" t="s">
-        <v>868</v>
+        <v>130000</v>
+      </c>
+      <c r="I29" s="18" t="s">
+        <v>835</v>
       </c>
       <c r="J29" s="27"/>
       <c r="K29" s="27"/>
@@ -13697,23 +13698,23 @@
         <v>29</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D30" s="50" t="s">
-        <v>867</v>
+        <v>861</v>
       </c>
       <c r="E30" s="17">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="F30" s="17" t="s">
-        <v>760</v>
+        <v>881</v>
       </c>
       <c r="G30" s="44">
-        <v>703.93</v>
+        <v>198.72</v>
       </c>
       <c r="H30" s="44">
         <f t="shared" si="0"/>
-        <v>19710.039999999997</v>
+        <v>11525.76</v>
       </c>
       <c r="I30" s="17" t="s">
         <v>868</v>
@@ -13726,24 +13727,23 @@
         <v>30</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="D31" s="50" t="s">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="E31" s="17">
-        <f>28*3</f>
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="F31" s="17" t="s">
-        <v>760</v>
+        <v>881</v>
       </c>
       <c r="G31" s="44">
-        <v>49.05</v>
+        <v>484.24</v>
       </c>
       <c r="H31" s="44">
         <f t="shared" si="0"/>
-        <v>4120.2</v>
+        <v>15011.44</v>
       </c>
       <c r="I31" s="17" t="s">
         <v>868</v>
@@ -13759,20 +13759,20 @@
         <v>879</v>
       </c>
       <c r="D32" s="50" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
       <c r="E32" s="17">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="F32" s="17" t="s">
         <v>760</v>
       </c>
       <c r="G32" s="44">
-        <v>151.19999999999999</v>
+        <v>703.93</v>
       </c>
       <c r="H32" s="44">
         <f t="shared" si="0"/>
-        <v>453.59999999999997</v>
+        <v>19710.039999999997</v>
       </c>
       <c r="I32" s="17" t="s">
         <v>868</v>
@@ -13785,23 +13785,24 @@
         <v>32</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D33" s="50" t="s">
-        <v>866</v>
+        <v>862</v>
       </c>
       <c r="E33" s="17">
-        <v>2</v>
+        <f>28*3</f>
+        <v>84</v>
       </c>
       <c r="F33" s="17" t="s">
         <v>760</v>
       </c>
       <c r="G33" s="44">
-        <v>48.38</v>
+        <v>49.05</v>
       </c>
       <c r="H33" s="44">
         <f t="shared" si="0"/>
-        <v>96.76</v>
+        <v>4120.2</v>
       </c>
       <c r="I33" s="17" t="s">
         <v>868</v>
@@ -13814,23 +13815,23 @@
         <v>33</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="D34" s="50" t="s">
-        <v>863</v>
+        <v>865</v>
       </c>
       <c r="E34" s="17">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="F34" s="17" t="s">
         <v>760</v>
       </c>
       <c r="G34" s="44">
-        <v>27.14</v>
+        <v>151.19999999999999</v>
       </c>
       <c r="H34" s="44">
-        <f t="shared" ref="H34:H65" si="1">G34*E34</f>
-        <v>814.2</v>
+        <f t="shared" si="0"/>
+        <v>453.59999999999997</v>
       </c>
       <c r="I34" s="17" t="s">
         <v>868</v>
@@ -13843,23 +13844,23 @@
         <v>34</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>882</v>
+        <v>879</v>
       </c>
       <c r="D35" s="50" t="s">
-        <v>869</v>
+        <v>866</v>
       </c>
       <c r="E35" s="17">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F35" s="17" t="s">
-        <v>881</v>
+        <v>760</v>
       </c>
       <c r="G35" s="44">
-        <v>703.93</v>
+        <v>48.38</v>
       </c>
       <c r="H35" s="44">
-        <f t="shared" si="1"/>
-        <v>8447.16</v>
+        <f t="shared" si="0"/>
+        <v>96.76</v>
       </c>
       <c r="I35" s="17" t="s">
         <v>868</v>
@@ -13872,24 +13873,23 @@
         <v>35</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>882</v>
+        <v>878</v>
       </c>
       <c r="D36" s="50" t="s">
-        <v>870</v>
+        <v>863</v>
       </c>
       <c r="E36" s="17">
-        <f>78/6</f>
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>881</v>
+        <v>760</v>
       </c>
       <c r="G36" s="44">
-        <v>484.24</v>
+        <v>27.14</v>
       </c>
       <c r="H36" s="44">
-        <f t="shared" si="1"/>
-        <v>6295.12</v>
+        <f t="shared" ref="H36:H67" si="1">G36*E36</f>
+        <v>814.2</v>
       </c>
       <c r="I36" s="17" t="s">
         <v>868</v>
@@ -13901,24 +13901,26 @@
       <c r="B37" s="17">
         <v>36</v>
       </c>
-      <c r="C37" s="18"/>
-      <c r="D37" s="19" t="s">
-        <v>883</v>
-      </c>
-      <c r="E37" s="18">
-        <v>1</v>
-      </c>
-      <c r="F37" s="18" t="s">
-        <v>760</v>
-      </c>
-      <c r="G37" s="25">
-        <v>37375</v>
-      </c>
-      <c r="H37" s="51">
+      <c r="C37" s="17" t="s">
+        <v>882</v>
+      </c>
+      <c r="D37" s="50" t="s">
+        <v>869</v>
+      </c>
+      <c r="E37" s="17">
+        <v>12</v>
+      </c>
+      <c r="F37" s="17" t="s">
+        <v>881</v>
+      </c>
+      <c r="G37" s="44">
+        <v>703.93</v>
+      </c>
+      <c r="H37" s="44">
         <f t="shared" si="1"/>
-        <v>37375</v>
-      </c>
-      <c r="I37" s="18" t="s">
+        <v>8447.16</v>
+      </c>
+      <c r="I37" s="17" t="s">
         <v>868</v>
       </c>
       <c r="J37" s="27"/>
@@ -13928,54 +13930,55 @@
       <c r="B38" s="17">
         <v>37</v>
       </c>
-      <c r="C38" s="17"/>
+      <c r="C38" s="17" t="s">
+        <v>882</v>
+      </c>
       <c r="D38" s="50" t="s">
-        <v>805</v>
+        <v>870</v>
       </c>
       <c r="E38" s="17">
-        <f>54*2</f>
-        <v>108</v>
+        <f>78/6</f>
+        <v>13</v>
       </c>
       <c r="F38" s="17" t="s">
-        <v>760</v>
+        <v>881</v>
       </c>
       <c r="G38" s="44">
-        <v>243.39</v>
+        <v>484.24</v>
       </c>
       <c r="H38" s="44">
         <f t="shared" si="1"/>
-        <v>26286.12</v>
+        <v>6295.12</v>
       </c>
       <c r="I38" s="17" t="s">
-        <v>806</v>
+        <v>868</v>
       </c>
       <c r="J38" s="27"/>
       <c r="K38" s="27"/>
-      <c r="L38" s="14"/>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="17">
         <v>38</v>
       </c>
-      <c r="C39" s="17"/>
-      <c r="D39" s="50" t="s">
-        <v>807</v>
-      </c>
-      <c r="E39" s="17">
-        <v>30</v>
-      </c>
-      <c r="F39" s="17" t="s">
+      <c r="C39" s="18"/>
+      <c r="D39" s="19" t="s">
+        <v>883</v>
+      </c>
+      <c r="E39" s="18">
+        <v>1</v>
+      </c>
+      <c r="F39" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G39" s="44">
-        <v>119.7</v>
-      </c>
-      <c r="H39" s="44">
+      <c r="G39" s="25">
+        <v>37375</v>
+      </c>
+      <c r="H39" s="51">
         <f t="shared" si="1"/>
-        <v>3591</v>
-      </c>
-      <c r="I39" s="17" t="s">
-        <v>806</v>
+        <v>37375</v>
+      </c>
+      <c r="I39" s="18" t="s">
+        <v>868</v>
       </c>
       <c r="J39" s="27"/>
       <c r="K39" s="27"/>
@@ -13986,26 +13989,28 @@
       </c>
       <c r="C40" s="17"/>
       <c r="D40" s="50" t="s">
-        <v>804</v>
-      </c>
-      <c r="E40" s="18">
-        <v>390</v>
+        <v>805</v>
+      </c>
+      <c r="E40" s="17">
+        <f>54*2</f>
+        <v>108</v>
       </c>
       <c r="F40" s="17" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G40" s="44">
-        <v>38.116666600000002</v>
+        <v>243.39</v>
       </c>
       <c r="H40" s="44">
         <f t="shared" si="1"/>
-        <v>14865.499974</v>
+        <v>26286.12</v>
       </c>
       <c r="I40" s="17" t="s">
         <v>806</v>
       </c>
       <c r="J40" s="27"/>
       <c r="K40" s="27"/>
+      <c r="L40" s="14"/>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="17">
@@ -14013,28 +14018,26 @@
       </c>
       <c r="C41" s="17"/>
       <c r="D41" s="50" t="s">
-        <v>805</v>
-      </c>
-      <c r="E41" s="53">
-        <f>(84*1.02)*2*1.02</f>
-        <v>174.78720000000001</v>
+        <v>807</v>
+      </c>
+      <c r="E41" s="17">
+        <v>30</v>
       </c>
       <c r="F41" s="17" t="s">
         <v>760</v>
       </c>
       <c r="G41" s="44">
-        <v>243.39</v>
+        <v>119.7</v>
       </c>
       <c r="H41" s="44">
         <f t="shared" si="1"/>
-        <v>42541.456608</v>
+        <v>3591</v>
       </c>
       <c r="I41" s="17" t="s">
-        <v>774</v>
+        <v>806</v>
       </c>
       <c r="J41" s="27"/>
       <c r="K41" s="27"/>
-      <c r="L41" s="14"/>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="17">
@@ -14044,9 +14047,8 @@
       <c r="D42" s="50" t="s">
         <v>804</v>
       </c>
-      <c r="E42" s="17">
-        <f>84*7</f>
-        <v>588</v>
+      <c r="E42" s="18">
+        <v>390</v>
       </c>
       <c r="F42" s="17" t="s">
         <v>761</v>
@@ -14056,10 +14058,10 @@
       </c>
       <c r="H42" s="44">
         <f t="shared" si="1"/>
-        <v>22412.599960800002</v>
+        <v>14865.499974</v>
       </c>
       <c r="I42" s="17" t="s">
-        <v>774</v>
+        <v>806</v>
       </c>
       <c r="J42" s="27"/>
       <c r="K42" s="27"/>
@@ -14070,26 +14072,28 @@
       </c>
       <c r="C43" s="17"/>
       <c r="D43" s="50" t="s">
-        <v>824</v>
-      </c>
-      <c r="E43" s="17">
-        <v>30</v>
+        <v>805</v>
+      </c>
+      <c r="E43" s="53">
+        <f>(84*1.02)*2*1.02</f>
+        <v>174.78720000000001</v>
       </c>
       <c r="F43" s="17" t="s">
-        <v>818</v>
+        <v>760</v>
       </c>
       <c r="G43" s="44">
-        <v>24</v>
+        <v>243.39</v>
       </c>
       <c r="H43" s="44">
         <f t="shared" si="1"/>
-        <v>720</v>
+        <v>42541.456608</v>
       </c>
       <c r="I43" s="17" t="s">
         <v>774</v>
       </c>
       <c r="J43" s="27"/>
       <c r="K43" s="27"/>
+      <c r="L43" s="14"/>
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="17">
@@ -14097,20 +14101,21 @@
       </c>
       <c r="C44" s="17"/>
       <c r="D44" s="50" t="s">
-        <v>825</v>
+        <v>804</v>
       </c>
       <c r="E44" s="17">
-        <v>1</v>
+        <f>84*7</f>
+        <v>588</v>
       </c>
       <c r="F44" s="17" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="G44" s="44">
-        <v>860</v>
+        <v>38.116666600000002</v>
       </c>
       <c r="H44" s="44">
         <f t="shared" si="1"/>
-        <v>860</v>
+        <v>22412.599960800002</v>
       </c>
       <c r="I44" s="17" t="s">
         <v>774</v>
@@ -14123,23 +14128,23 @@
         <v>44</v>
       </c>
       <c r="C45" s="17"/>
-      <c r="D45" s="19" t="s">
-        <v>873</v>
-      </c>
-      <c r="E45" s="18">
-        <v>140</v>
-      </c>
-      <c r="F45" s="18" t="s">
-        <v>761</v>
-      </c>
-      <c r="G45" s="25">
-        <v>23.90625</v>
-      </c>
-      <c r="H45" s="25">
+      <c r="D45" s="50" t="s">
+        <v>824</v>
+      </c>
+      <c r="E45" s="17">
+        <v>30</v>
+      </c>
+      <c r="F45" s="17" t="s">
+        <v>818</v>
+      </c>
+      <c r="G45" s="44">
+        <v>24</v>
+      </c>
+      <c r="H45" s="44">
         <f t="shared" si="1"/>
-        <v>3346.875</v>
-      </c>
-      <c r="I45" s="18" t="s">
+        <v>720</v>
+      </c>
+      <c r="I45" s="17" t="s">
         <v>774</v>
       </c>
       <c r="J45" s="27"/>
@@ -14150,23 +14155,23 @@
         <v>45</v>
       </c>
       <c r="C46" s="17"/>
-      <c r="D46" s="19" t="s">
-        <v>778</v>
-      </c>
-      <c r="E46" s="18">
-        <v>66</v>
-      </c>
-      <c r="F46" s="18" t="s">
-        <v>761</v>
-      </c>
-      <c r="G46" s="25">
-        <v>26</v>
-      </c>
-      <c r="H46" s="25">
+      <c r="D46" s="50" t="s">
+        <v>825</v>
+      </c>
+      <c r="E46" s="17">
+        <v>1</v>
+      </c>
+      <c r="F46" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G46" s="44">
+        <v>860</v>
+      </c>
+      <c r="H46" s="44">
         <f t="shared" si="1"/>
-        <v>1716</v>
-      </c>
-      <c r="I46" s="18" t="s">
+        <v>860</v>
+      </c>
+      <c r="I46" s="17" t="s">
         <v>774</v>
       </c>
       <c r="J46" s="27"/>
@@ -14178,21 +14183,20 @@
       </c>
       <c r="C47" s="17"/>
       <c r="D47" s="19" t="s">
-        <v>800</v>
+        <v>873</v>
       </c>
       <c r="E47" s="18">
-        <v>1</v>
+        <v>140</v>
       </c>
       <c r="F47" s="18" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="G47" s="25">
-        <f>7500+7000+6500+10000</f>
-        <v>31000</v>
+        <v>23.90625</v>
       </c>
       <c r="H47" s="25">
         <f t="shared" si="1"/>
-        <v>31000</v>
+        <v>3346.875</v>
       </c>
       <c r="I47" s="18" t="s">
         <v>774</v>
@@ -14205,24 +14209,24 @@
         <v>47</v>
       </c>
       <c r="C48" s="17"/>
-      <c r="D48" s="50" t="s">
-        <v>788</v>
-      </c>
-      <c r="E48" s="17">
-        <v>1</v>
-      </c>
-      <c r="F48" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="G48" s="54">
-        <v>6000</v>
-      </c>
-      <c r="H48" s="54">
+      <c r="D48" s="19" t="s">
+        <v>778</v>
+      </c>
+      <c r="E48" s="18">
+        <v>66</v>
+      </c>
+      <c r="F48" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G48" s="25">
+        <v>26</v>
+      </c>
+      <c r="H48" s="25">
         <f t="shared" si="1"/>
-        <v>6000</v>
-      </c>
-      <c r="I48" s="17" t="s">
-        <v>771</v>
+        <v>1716</v>
+      </c>
+      <c r="I48" s="18" t="s">
+        <v>774</v>
       </c>
       <c r="J48" s="27"/>
       <c r="K48" s="27"/>
@@ -14232,24 +14236,25 @@
         <v>48</v>
       </c>
       <c r="C49" s="17"/>
-      <c r="D49" s="50" t="s">
-        <v>769</v>
-      </c>
-      <c r="E49" s="17">
-        <v>4100</v>
-      </c>
-      <c r="F49" s="17" t="s">
-        <v>811</v>
-      </c>
-      <c r="G49" s="54">
-        <v>9.65</v>
-      </c>
-      <c r="H49" s="54">
+      <c r="D49" s="19" t="s">
+        <v>800</v>
+      </c>
+      <c r="E49" s="18">
+        <v>1</v>
+      </c>
+      <c r="F49" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G49" s="25">
+        <f>7500+7000+6500+10000</f>
+        <v>31000</v>
+      </c>
+      <c r="H49" s="25">
         <f t="shared" si="1"/>
-        <v>39565</v>
-      </c>
-      <c r="I49" s="17" t="s">
-        <v>771</v>
+        <v>31000</v>
+      </c>
+      <c r="I49" s="18" t="s">
+        <v>774</v>
       </c>
       <c r="J49" s="27"/>
       <c r="K49" s="27"/>
@@ -14260,29 +14265,26 @@
       </c>
       <c r="C50" s="17"/>
       <c r="D50" s="50" t="s">
-        <v>770</v>
+        <v>788</v>
       </c>
       <c r="E50" s="17">
-        <v>4000</v>
+        <v>1</v>
       </c>
       <c r="F50" s="17" t="s">
-        <v>811</v>
+        <v>760</v>
       </c>
       <c r="G50" s="54">
-        <v>9.65</v>
+        <v>6000</v>
       </c>
       <c r="H50" s="54">
         <f t="shared" si="1"/>
-        <v>38600</v>
+        <v>6000</v>
       </c>
       <c r="I50" s="17" t="s">
         <v>771</v>
       </c>
       <c r="J50" s="27"/>
       <c r="K50" s="27"/>
-      <c r="L50" s="14" t="s">
-        <v>812</v>
-      </c>
     </row>
     <row r="51" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B51" s="17">
@@ -14290,29 +14292,26 @@
       </c>
       <c r="C51" s="17"/>
       <c r="D51" s="50" t="s">
-        <v>803</v>
+        <v>769</v>
       </c>
       <c r="E51" s="17">
-        <v>1</v>
+        <v>4100</v>
       </c>
       <c r="F51" s="17" t="s">
-        <v>760</v>
+        <v>811</v>
       </c>
       <c r="G51" s="54">
-        <v>164000</v>
+        <v>9.65</v>
       </c>
       <c r="H51" s="54">
         <f t="shared" si="1"/>
-        <v>164000</v>
+        <v>39565</v>
       </c>
       <c r="I51" s="17" t="s">
         <v>771</v>
       </c>
       <c r="J51" s="27"/>
       <c r="K51" s="27"/>
-      <c r="L51" s="14" t="s">
-        <v>812</v>
-      </c>
     </row>
     <row r="52" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B52" s="17">
@@ -14320,26 +14319,29 @@
       </c>
       <c r="C52" s="17"/>
       <c r="D52" s="50" t="s">
-        <v>830</v>
-      </c>
-      <c r="E52" s="53">
-        <v>99.22</v>
+        <v>770</v>
+      </c>
+      <c r="E52" s="17">
+        <v>4000</v>
       </c>
       <c r="F52" s="17" t="s">
-        <v>759</v>
+        <v>811</v>
       </c>
       <c r="G52" s="54">
-        <v>670</v>
+        <v>9.65</v>
       </c>
       <c r="H52" s="54">
         <f t="shared" si="1"/>
-        <v>66477.399999999994</v>
+        <v>38600</v>
       </c>
       <c r="I52" s="17" t="s">
         <v>771</v>
       </c>
       <c r="J52" s="27"/>
       <c r="K52" s="27"/>
+      <c r="L52" s="14" t="s">
+        <v>812</v>
+      </c>
     </row>
     <row r="53" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B53" s="17">
@@ -14347,26 +14349,29 @@
       </c>
       <c r="C53" s="17"/>
       <c r="D53" s="50" t="s">
-        <v>829</v>
+        <v>803</v>
       </c>
       <c r="E53" s="17">
-        <v>68</v>
+        <v>1</v>
       </c>
       <c r="F53" s="17" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="G53" s="54">
-        <v>670</v>
+        <v>164000</v>
       </c>
       <c r="H53" s="54">
         <f t="shared" si="1"/>
-        <v>45560</v>
+        <v>164000</v>
       </c>
       <c r="I53" s="17" t="s">
         <v>771</v>
       </c>
       <c r="J53" s="27"/>
       <c r="K53" s="27"/>
+      <c r="L53" s="14" t="s">
+        <v>812</v>
+      </c>
     </row>
     <row r="54" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B54" s="17">
@@ -14374,20 +14379,20 @@
       </c>
       <c r="C54" s="17"/>
       <c r="D54" s="50" t="s">
-        <v>808</v>
-      </c>
-      <c r="E54" s="17">
-        <v>1</v>
+        <v>830</v>
+      </c>
+      <c r="E54" s="53">
+        <v>99.22</v>
       </c>
       <c r="F54" s="17" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G54" s="54">
-        <v>56500</v>
+        <v>670</v>
       </c>
       <c r="H54" s="54">
         <f t="shared" si="1"/>
-        <v>56500</v>
+        <v>66477.399999999994</v>
       </c>
       <c r="I54" s="17" t="s">
         <v>771</v>
@@ -14401,20 +14406,20 @@
       </c>
       <c r="C55" s="17"/>
       <c r="D55" s="50" t="s">
-        <v>777</v>
+        <v>829</v>
       </c>
       <c r="E55" s="17">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="F55" s="17" t="s">
-        <v>760</v>
-      </c>
-      <c r="G55" s="44">
-        <v>125</v>
-      </c>
-      <c r="H55" s="44">
+        <v>759</v>
+      </c>
+      <c r="G55" s="54">
+        <v>670</v>
+      </c>
+      <c r="H55" s="54">
         <f t="shared" si="1"/>
-        <v>6250</v>
+        <v>45560</v>
       </c>
       <c r="I55" s="17" t="s">
         <v>771</v>
@@ -14428,20 +14433,20 @@
       </c>
       <c r="C56" s="17"/>
       <c r="D56" s="50" t="s">
-        <v>842</v>
+        <v>808</v>
       </c>
       <c r="E56" s="17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F56" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G56" s="44">
-        <v>1500</v>
-      </c>
-      <c r="H56" s="44">
+      <c r="G56" s="54">
+        <v>56500</v>
+      </c>
+      <c r="H56" s="54">
         <f t="shared" si="1"/>
-        <v>6000</v>
+        <v>56500</v>
       </c>
       <c r="I56" s="17" t="s">
         <v>771</v>
@@ -14454,30 +14459,27 @@
         <v>56</v>
       </c>
       <c r="C57" s="17"/>
-      <c r="D57" s="19" t="s">
-        <v>850</v>
-      </c>
-      <c r="E57" s="18">
-        <v>26</v>
-      </c>
-      <c r="F57" s="18" t="s">
+      <c r="D57" s="50" t="s">
+        <v>777</v>
+      </c>
+      <c r="E57" s="17">
+        <v>50</v>
+      </c>
+      <c r="F57" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G57" s="25">
-        <v>420</v>
-      </c>
-      <c r="H57" s="25">
+      <c r="G57" s="44">
+        <v>125</v>
+      </c>
+      <c r="H57" s="44">
         <f t="shared" si="1"/>
-        <v>10920</v>
+        <v>6250</v>
       </c>
       <c r="I57" s="17" t="s">
-        <v>901</v>
+        <v>771</v>
       </c>
       <c r="J57" s="27"/>
       <c r="K57" s="27"/>
-      <c r="L57" s="24" t="s">
-        <v>843</v>
-      </c>
     </row>
     <row r="58" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B58" s="17">
@@ -14485,23 +14487,23 @@
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="50" t="s">
-        <v>898</v>
-      </c>
-      <c r="E58" s="18">
-        <v>400</v>
-      </c>
-      <c r="F58" s="18" t="s">
-        <v>761</v>
-      </c>
-      <c r="G58" s="25">
-        <v>15</v>
-      </c>
-      <c r="H58" s="25">
+        <v>842</v>
+      </c>
+      <c r="E58" s="17">
+        <v>4</v>
+      </c>
+      <c r="F58" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G58" s="44">
+        <v>1500</v>
+      </c>
+      <c r="H58" s="44">
         <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="I58" s="17" t="s">
-        <v>901</v>
+        <v>771</v>
       </c>
       <c r="J58" s="27"/>
       <c r="K58" s="27"/>
@@ -14512,51 +14514,53 @@
       </c>
       <c r="C59" s="17"/>
       <c r="D59" s="19" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="E59" s="18">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="F59" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G59" s="25">
-        <f>119439/2</f>
-        <v>59719.5</v>
+        <v>420</v>
       </c>
       <c r="H59" s="25">
         <f t="shared" si="1"/>
-        <v>59719.5</v>
+        <v>10920</v>
       </c>
       <c r="I59" s="17" t="s">
         <v>901</v>
       </c>
       <c r="J59" s="27"/>
       <c r="K59" s="27"/>
+      <c r="L59" s="24" t="s">
+        <v>843</v>
+      </c>
     </row>
     <row r="60" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B60" s="17">
         <v>59</v>
       </c>
       <c r="C60" s="17"/>
-      <c r="D60" s="19" t="s">
-        <v>783</v>
+      <c r="D60" s="50" t="s">
+        <v>898</v>
       </c>
       <c r="E60" s="18">
-        <v>8</v>
+        <v>400</v>
       </c>
       <c r="F60" s="18" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="G60" s="25">
-        <v>380</v>
+        <v>15</v>
       </c>
       <c r="H60" s="25">
         <f t="shared" si="1"/>
-        <v>3040</v>
-      </c>
-      <c r="I60" s="18" t="s">
-        <v>576</v>
+        <v>6000</v>
+      </c>
+      <c r="I60" s="17" t="s">
+        <v>901</v>
       </c>
       <c r="J60" s="27"/>
       <c r="K60" s="27"/>
@@ -14567,23 +14571,24 @@
       </c>
       <c r="C61" s="17"/>
       <c r="D61" s="19" t="s">
-        <v>784</v>
+        <v>851</v>
       </c>
       <c r="E61" s="18">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F61" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G61" s="25">
-        <v>290</v>
+        <f>119439/2</f>
+        <v>59719.5</v>
       </c>
       <c r="H61" s="25">
         <f t="shared" si="1"/>
-        <v>1160</v>
-      </c>
-      <c r="I61" s="18" t="s">
-        <v>576</v>
+        <v>59719.5</v>
+      </c>
+      <c r="I61" s="17" t="s">
+        <v>901</v>
       </c>
       <c r="J61" s="27"/>
       <c r="K61" s="27"/>
@@ -14594,20 +14599,20 @@
       </c>
       <c r="C62" s="17"/>
       <c r="D62" s="19" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="E62" s="18">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F62" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G62" s="25">
-        <v>290</v>
+        <v>380</v>
       </c>
       <c r="H62" s="25">
         <f t="shared" si="1"/>
-        <v>1160</v>
+        <v>3040</v>
       </c>
       <c r="I62" s="18" t="s">
         <v>576</v>
@@ -14620,25 +14625,24 @@
         <v>62</v>
       </c>
       <c r="C63" s="17"/>
-      <c r="D63" s="50" t="s">
-        <v>757</v>
-      </c>
-      <c r="E63" s="53">
-        <f>(2150*1.05)*0.15</f>
-        <v>338.625</v>
-      </c>
-      <c r="F63" s="17" t="s">
-        <v>759</v>
-      </c>
-      <c r="G63" s="54">
-        <v>670</v>
-      </c>
-      <c r="H63" s="54">
+      <c r="D63" s="19" t="s">
+        <v>784</v>
+      </c>
+      <c r="E63" s="18">
+        <v>4</v>
+      </c>
+      <c r="F63" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G63" s="25">
+        <v>290</v>
+      </c>
+      <c r="H63" s="25">
         <f t="shared" si="1"/>
-        <v>226878.75</v>
-      </c>
-      <c r="I63" s="17" t="s">
-        <v>833</v>
+        <v>1160</v>
+      </c>
+      <c r="I63" s="18" t="s">
+        <v>576</v>
       </c>
       <c r="J63" s="27"/>
       <c r="K63" s="27"/>
@@ -14648,25 +14652,24 @@
         <v>63</v>
       </c>
       <c r="C64" s="17"/>
-      <c r="D64" s="50" t="s">
-        <v>775</v>
-      </c>
-      <c r="E64" s="53">
-        <f>(2150/13)*2</f>
-        <v>330.76923076923077</v>
-      </c>
-      <c r="F64" s="17" t="s">
+      <c r="D64" s="19" t="s">
+        <v>785</v>
+      </c>
+      <c r="E64" s="18">
+        <v>4</v>
+      </c>
+      <c r="F64" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G64" s="54">
-        <v>220.5</v>
-      </c>
-      <c r="H64" s="54">
+      <c r="G64" s="25">
+        <v>290</v>
+      </c>
+      <c r="H64" s="25">
         <f t="shared" si="1"/>
-        <v>72934.61538461539</v>
-      </c>
-      <c r="I64" s="17" t="s">
-        <v>833</v>
+        <v>1160</v>
+      </c>
+      <c r="I64" s="18" t="s">
+        <v>576</v>
       </c>
       <c r="J64" s="27"/>
       <c r="K64" s="27"/>
@@ -14677,21 +14680,21 @@
       </c>
       <c r="C65" s="17"/>
       <c r="D65" s="50" t="s">
-        <v>758</v>
-      </c>
-      <c r="E65" s="17">
-        <f>2100/12</f>
-        <v>175</v>
+        <v>757</v>
+      </c>
+      <c r="E65" s="53">
+        <f>(2150*1.05)*0.15</f>
+        <v>338.625</v>
       </c>
       <c r="F65" s="17" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G65" s="54">
-        <v>56.2</v>
+        <v>670</v>
       </c>
       <c r="H65" s="54">
         <f t="shared" si="1"/>
-        <v>9835</v>
+        <v>226878.75</v>
       </c>
       <c r="I65" s="17" t="s">
         <v>833</v>
@@ -14705,20 +14708,21 @@
       </c>
       <c r="C66" s="17"/>
       <c r="D66" s="50" t="s">
-        <v>762</v>
-      </c>
-      <c r="E66" s="17">
-        <v>1000</v>
+        <v>775</v>
+      </c>
+      <c r="E66" s="53">
+        <f>(2150/13)*2</f>
+        <v>330.76923076923077</v>
       </c>
       <c r="F66" s="17" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="G66" s="54">
-        <v>7.3</v>
+        <v>220.5</v>
       </c>
       <c r="H66" s="54">
-        <f t="shared" ref="H66:H97" si="2">G66*E66</f>
-        <v>7300</v>
+        <f t="shared" si="1"/>
+        <v>72934.61538461539</v>
       </c>
       <c r="I66" s="17" t="s">
         <v>833</v>
@@ -14732,21 +14736,21 @@
       </c>
       <c r="C67" s="17"/>
       <c r="D67" s="50" t="s">
-        <v>792</v>
-      </c>
-      <c r="E67" s="53">
-        <f>E63</f>
-        <v>338.625</v>
+        <v>758</v>
+      </c>
+      <c r="E67" s="17">
+        <f>2100/12</f>
+        <v>175</v>
       </c>
       <c r="F67" s="17" t="s">
-        <v>766</v>
+        <v>760</v>
       </c>
       <c r="G67" s="54">
-        <v>50</v>
+        <v>56.2</v>
       </c>
       <c r="H67" s="54">
-        <f t="shared" si="2"/>
-        <v>16931.25</v>
+        <f t="shared" si="1"/>
+        <v>9835</v>
       </c>
       <c r="I67" s="17" t="s">
         <v>833</v>
@@ -14760,20 +14764,20 @@
       </c>
       <c r="C68" s="17"/>
       <c r="D68" s="50" t="s">
-        <v>826</v>
+        <v>762</v>
       </c>
       <c r="E68" s="17">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F68" s="17" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="G68" s="54">
-        <v>53550</v>
+        <v>7.3</v>
       </c>
       <c r="H68" s="54">
-        <f t="shared" si="2"/>
-        <v>53550</v>
+        <f t="shared" ref="H68:H99" si="2">G68*E68</f>
+        <v>7300</v>
       </c>
       <c r="I68" s="17" t="s">
         <v>833</v>
@@ -14785,25 +14789,26 @@
       <c r="B69" s="17">
         <v>68</v>
       </c>
-      <c r="C69" s="18"/>
-      <c r="D69" s="19" t="s">
-        <v>799</v>
-      </c>
-      <c r="E69" s="18">
-        <v>110</v>
-      </c>
-      <c r="F69" s="18" t="s">
-        <v>760</v>
-      </c>
-      <c r="G69" s="25">
-        <v>42.29</v>
-      </c>
-      <c r="H69" s="25">
+      <c r="C69" s="17"/>
+      <c r="D69" s="50" t="s">
+        <v>792</v>
+      </c>
+      <c r="E69" s="53">
+        <f>E65</f>
+        <v>338.625</v>
+      </c>
+      <c r="F69" s="17" t="s">
+        <v>766</v>
+      </c>
+      <c r="G69" s="54">
+        <v>50</v>
+      </c>
+      <c r="H69" s="54">
         <f t="shared" si="2"/>
-        <v>4651.8999999999996</v>
-      </c>
-      <c r="I69" s="18" t="s">
-        <v>831</v>
+        <v>16931.25</v>
+      </c>
+      <c r="I69" s="17" t="s">
+        <v>833</v>
       </c>
       <c r="J69" s="27"/>
       <c r="K69" s="27"/>
@@ -14812,25 +14817,25 @@
       <c r="B70" s="17">
         <v>69</v>
       </c>
-      <c r="C70" s="18"/>
-      <c r="D70" s="19" t="s">
-        <v>832</v>
-      </c>
-      <c r="E70" s="18">
-        <v>1</v>
-      </c>
-      <c r="F70" s="18" t="s">
+      <c r="C70" s="17"/>
+      <c r="D70" s="50" t="s">
+        <v>826</v>
+      </c>
+      <c r="E70" s="17">
+        <v>1</v>
+      </c>
+      <c r="F70" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G70" s="25">
-        <v>1400</v>
-      </c>
-      <c r="H70" s="25">
+      <c r="G70" s="54">
+        <v>53550</v>
+      </c>
+      <c r="H70" s="54">
         <f t="shared" si="2"/>
-        <v>1400</v>
-      </c>
-      <c r="I70" s="18" t="s">
-        <v>831</v>
+        <v>53550</v>
+      </c>
+      <c r="I70" s="17" t="s">
+        <v>833</v>
       </c>
       <c r="J70" s="27"/>
       <c r="K70" s="27"/>
@@ -14841,21 +14846,20 @@
       </c>
       <c r="C71" s="18"/>
       <c r="D71" s="19" t="s">
-        <v>757</v>
-      </c>
-      <c r="E71" s="52">
-        <f>((1260+960)*0.15)*1.1</f>
-        <v>366.3</v>
+        <v>799</v>
+      </c>
+      <c r="E71" s="18">
+        <v>110</v>
       </c>
       <c r="F71" s="18" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="G71" s="25">
-        <v>670</v>
+        <v>42.29</v>
       </c>
       <c r="H71" s="25">
         <f t="shared" si="2"/>
-        <v>245421</v>
+        <v>4651.8999999999996</v>
       </c>
       <c r="I71" s="18" t="s">
         <v>831</v>
@@ -14868,22 +14872,21 @@
         <v>71</v>
       </c>
       <c r="C72" s="18"/>
-      <c r="D72" s="50" t="s">
-        <v>775</v>
-      </c>
-      <c r="E72" s="52">
-        <f>(1260+960)/13*1.05</f>
-        <v>179.30769230769232</v>
+      <c r="D72" s="19" t="s">
+        <v>832</v>
+      </c>
+      <c r="E72" s="18">
+        <v>1</v>
       </c>
       <c r="F72" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G72" s="25">
-        <v>220.5</v>
+        <v>1400</v>
       </c>
       <c r="H72" s="25">
         <f t="shared" si="2"/>
-        <v>39537.346153846156</v>
+        <v>1400</v>
       </c>
       <c r="I72" s="18" t="s">
         <v>831</v>
@@ -14897,20 +14900,21 @@
       </c>
       <c r="C73" s="18"/>
       <c r="D73" s="19" t="s">
-        <v>834</v>
-      </c>
-      <c r="E73" s="18">
-        <v>1</v>
+        <v>757</v>
+      </c>
+      <c r="E73" s="52">
+        <f>((1260+960)*0.15)*1.1</f>
+        <v>366.3</v>
       </c>
       <c r="F73" s="18" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G73" s="25">
-        <v>62525</v>
+        <v>670</v>
       </c>
       <c r="H73" s="25">
         <f t="shared" si="2"/>
-        <v>62525</v>
+        <v>245421</v>
       </c>
       <c r="I73" s="18" t="s">
         <v>831</v>
@@ -14922,25 +14926,26 @@
       <c r="B74" s="17">
         <v>73</v>
       </c>
-      <c r="C74" s="17"/>
+      <c r="C74" s="18"/>
       <c r="D74" s="50" t="s">
-        <v>823</v>
-      </c>
-      <c r="E74" s="17">
-        <v>1</v>
-      </c>
-      <c r="F74" s="17" t="s">
+        <v>775</v>
+      </c>
+      <c r="E74" s="52">
+        <f>(1260+960)/13*1.05</f>
+        <v>179.30769230769232</v>
+      </c>
+      <c r="F74" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G74" s="44">
-        <v>24500</v>
-      </c>
-      <c r="H74" s="44">
+      <c r="G74" s="25">
+        <v>220.5</v>
+      </c>
+      <c r="H74" s="25">
         <f t="shared" si="2"/>
-        <v>24500</v>
-      </c>
-      <c r="I74" s="17" t="s">
-        <v>772</v>
+        <v>39537.346153846156</v>
+      </c>
+      <c r="I74" s="18" t="s">
+        <v>831</v>
       </c>
       <c r="J74" s="27"/>
       <c r="K74" s="27"/>
@@ -14949,25 +14954,25 @@
       <c r="B75" s="17">
         <v>74</v>
       </c>
-      <c r="C75" s="17"/>
-      <c r="D75" s="50" t="s">
-        <v>773</v>
-      </c>
-      <c r="E75" s="17">
-        <v>1</v>
-      </c>
-      <c r="F75" s="17" t="s">
+      <c r="C75" s="18"/>
+      <c r="D75" s="19" t="s">
+        <v>834</v>
+      </c>
+      <c r="E75" s="18">
+        <v>1</v>
+      </c>
+      <c r="F75" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G75" s="54">
-        <v>968004</v>
-      </c>
-      <c r="H75" s="54">
+      <c r="G75" s="25">
+        <v>62525</v>
+      </c>
+      <c r="H75" s="25">
         <f t="shared" si="2"/>
-        <v>968004</v>
-      </c>
-      <c r="I75" s="17" t="s">
-        <v>772</v>
+        <v>62525</v>
+      </c>
+      <c r="I75" s="18" t="s">
+        <v>831</v>
       </c>
       <c r="J75" s="27"/>
       <c r="K75" s="27"/>
@@ -14976,25 +14981,25 @@
       <c r="B76" s="17">
         <v>75</v>
       </c>
-      <c r="C76" s="18"/>
-      <c r="D76" s="19" t="s">
-        <v>904</v>
-      </c>
-      <c r="E76" s="18">
-        <v>1</v>
-      </c>
-      <c r="F76" s="18" t="s">
+      <c r="C76" s="17"/>
+      <c r="D76" s="50" t="s">
+        <v>823</v>
+      </c>
+      <c r="E76" s="17">
+        <v>1</v>
+      </c>
+      <c r="F76" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G76" s="25">
-        <v>32000</v>
-      </c>
-      <c r="H76" s="51">
+      <c r="G76" s="44">
+        <v>24500</v>
+      </c>
+      <c r="H76" s="44">
         <f t="shared" si="2"/>
-        <v>32000</v>
-      </c>
-      <c r="I76" s="18" t="s">
-        <v>859</v>
+        <v>24500</v>
+      </c>
+      <c r="I76" s="17" t="s">
+        <v>772</v>
       </c>
       <c r="J76" s="27"/>
       <c r="K76" s="27"/>
@@ -15003,25 +15008,25 @@
       <c r="B77" s="17">
         <v>76</v>
       </c>
-      <c r="C77" s="18"/>
-      <c r="D77" s="19" t="s">
-        <v>903</v>
-      </c>
-      <c r="E77" s="18">
-        <v>1</v>
-      </c>
-      <c r="F77" s="18" t="s">
+      <c r="C77" s="17"/>
+      <c r="D77" s="50" t="s">
+        <v>773</v>
+      </c>
+      <c r="E77" s="17">
+        <v>1</v>
+      </c>
+      <c r="F77" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G77" s="25">
-        <v>10000</v>
-      </c>
-      <c r="H77" s="51">
+      <c r="G77" s="54">
+        <v>968004</v>
+      </c>
+      <c r="H77" s="54">
         <f t="shared" si="2"/>
-        <v>10000</v>
-      </c>
-      <c r="I77" s="18" t="s">
-        <v>859</v>
+        <v>968004</v>
+      </c>
+      <c r="I77" s="17" t="s">
+        <v>772</v>
       </c>
       <c r="J77" s="27"/>
       <c r="K77" s="27"/>
@@ -15030,9 +15035,9 @@
       <c r="B78" s="17">
         <v>77</v>
       </c>
-      <c r="C78" s="17"/>
+      <c r="C78" s="18"/>
       <c r="D78" s="19" t="s">
-        <v>793</v>
+        <v>904</v>
       </c>
       <c r="E78" s="18">
         <v>1</v>
@@ -15041,27 +15046,25 @@
         <v>760</v>
       </c>
       <c r="G78" s="25">
-        <v>46600</v>
-      </c>
-      <c r="H78" s="25">
+        <v>32000</v>
+      </c>
+      <c r="H78" s="51">
         <f t="shared" si="2"/>
-        <v>46600</v>
+        <v>32000</v>
       </c>
       <c r="I78" s="18" t="s">
-        <v>837</v>
-      </c>
-      <c r="J78" s="42" t="s">
-        <v>922</v>
-      </c>
+        <v>859</v>
+      </c>
+      <c r="J78" s="27"/>
       <c r="K78" s="27"/>
     </row>
     <row r="79" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B79" s="17">
         <v>78</v>
       </c>
-      <c r="C79" s="17"/>
+      <c r="C79" s="18"/>
       <c r="D79" s="19" t="s">
-        <v>794</v>
+        <v>903</v>
       </c>
       <c r="E79" s="18">
         <v>1</v>
@@ -15070,18 +15073,16 @@
         <v>760</v>
       </c>
       <c r="G79" s="25">
-        <v>8100</v>
-      </c>
-      <c r="H79" s="25">
+        <v>10000</v>
+      </c>
+      <c r="H79" s="51">
         <f t="shared" si="2"/>
-        <v>8100</v>
+        <v>10000</v>
       </c>
       <c r="I79" s="18" t="s">
-        <v>837</v>
-      </c>
-      <c r="J79" s="42" t="s">
-        <v>922</v>
-      </c>
+        <v>859</v>
+      </c>
+      <c r="J79" s="27"/>
       <c r="K79" s="27"/>
     </row>
     <row r="80" spans="2:11" x14ac:dyDescent="0.25">
@@ -15090,7 +15091,7 @@
       </c>
       <c r="C80" s="17"/>
       <c r="D80" s="19" t="s">
-        <v>801</v>
+        <v>793</v>
       </c>
       <c r="E80" s="18">
         <v>1</v>
@@ -15099,11 +15100,11 @@
         <v>760</v>
       </c>
       <c r="G80" s="25">
-        <v>5000</v>
+        <v>46600</v>
       </c>
       <c r="H80" s="25">
         <f t="shared" si="2"/>
-        <v>5000</v>
+        <v>46600</v>
       </c>
       <c r="I80" s="18" t="s">
         <v>837</v>
@@ -15113,13 +15114,13 @@
       </c>
       <c r="K80" s="27"/>
     </row>
-    <row r="81" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B81" s="17">
         <v>80</v>
       </c>
       <c r="C81" s="17"/>
       <c r="D81" s="19" t="s">
-        <v>872</v>
+        <v>794</v>
       </c>
       <c r="E81" s="18">
         <v>1</v>
@@ -15128,40 +15129,40 @@
         <v>760</v>
       </c>
       <c r="G81" s="25">
-        <v>27000</v>
+        <v>8100</v>
       </c>
       <c r="H81" s="25">
         <f t="shared" si="2"/>
-        <v>27000</v>
+        <v>8100</v>
       </c>
       <c r="I81" s="18" t="s">
         <v>837</v>
       </c>
       <c r="J81" s="42" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="K81" s="27"/>
     </row>
-    <row r="82" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B82" s="17">
         <v>81</v>
       </c>
       <c r="C82" s="17"/>
       <c r="D82" s="19" t="s">
-        <v>893</v>
+        <v>801</v>
       </c>
       <c r="E82" s="18">
-        <v>320</v>
+        <v>1</v>
       </c>
       <c r="F82" s="18" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G82" s="25">
-        <v>16</v>
+        <v>5000</v>
       </c>
       <c r="H82" s="25">
         <f t="shared" si="2"/>
-        <v>5120</v>
+        <v>5000</v>
       </c>
       <c r="I82" s="18" t="s">
         <v>837</v>
@@ -15171,13 +15172,13 @@
       </c>
       <c r="K82" s="27"/>
     </row>
-    <row r="83" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B83" s="17">
         <v>82</v>
       </c>
       <c r="C83" s="17"/>
       <c r="D83" s="19" t="s">
-        <v>911</v>
+        <v>872</v>
       </c>
       <c r="E83" s="18">
         <v>1</v>
@@ -15186,40 +15187,40 @@
         <v>760</v>
       </c>
       <c r="G83" s="25">
-        <v>3400</v>
+        <v>27000</v>
       </c>
       <c r="H83" s="25">
         <f t="shared" si="2"/>
-        <v>3400</v>
+        <v>27000</v>
       </c>
       <c r="I83" s="18" t="s">
         <v>837</v>
       </c>
       <c r="J83" s="42" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="K83" s="27"/>
     </row>
-    <row r="84" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B84" s="17">
         <v>83</v>
       </c>
       <c r="C84" s="17"/>
       <c r="D84" s="19" t="s">
-        <v>912</v>
+        <v>893</v>
       </c>
       <c r="E84" s="18">
-        <v>1</v>
+        <v>320</v>
       </c>
       <c r="F84" s="18" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="G84" s="25">
-        <v>8000</v>
+        <v>16</v>
       </c>
       <c r="H84" s="25">
         <f t="shared" si="2"/>
-        <v>8000</v>
+        <v>5120</v>
       </c>
       <c r="I84" s="18" t="s">
         <v>837</v>
@@ -15229,13 +15230,13 @@
       </c>
       <c r="K84" s="27"/>
     </row>
-    <row r="85" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B85" s="17">
         <v>84</v>
       </c>
       <c r="C85" s="17"/>
       <c r="D85" s="19" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
       <c r="E85" s="18">
         <v>1</v>
@@ -15244,44 +15245,42 @@
         <v>760</v>
       </c>
       <c r="G85" s="25">
-        <v>2500</v>
+        <v>3400</v>
       </c>
       <c r="H85" s="25">
         <f t="shared" si="2"/>
-        <v>2500</v>
+        <v>3400</v>
       </c>
       <c r="I85" s="18" t="s">
         <v>837</v>
       </c>
       <c r="J85" s="42" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="K85" s="27"/>
     </row>
-    <row r="86" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B86" s="17">
         <v>85</v>
       </c>
-      <c r="C86" s="17" t="s">
-        <v>900</v>
-      </c>
-      <c r="D86" s="50" t="s">
-        <v>896</v>
-      </c>
-      <c r="E86" s="52">
-        <v>115</v>
+      <c r="C86" s="17"/>
+      <c r="D86" s="19" t="s">
+        <v>912</v>
+      </c>
+      <c r="E86" s="18">
+        <v>1</v>
       </c>
       <c r="F86" s="18" t="s">
         <v>760</v>
       </c>
       <c r="G86" s="25">
-        <v>102</v>
+        <v>8000</v>
       </c>
       <c r="H86" s="25">
         <f t="shared" si="2"/>
-        <v>11730</v>
-      </c>
-      <c r="I86" s="17" t="s">
+        <v>8000</v>
+      </c>
+      <c r="I86" s="18" t="s">
         <v>837</v>
       </c>
       <c r="J86" s="42" t="s">
@@ -15289,383 +15288,443 @@
       </c>
       <c r="K86" s="27"/>
     </row>
-    <row r="87" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B87" s="17">
+        <v>86</v>
+      </c>
+      <c r="C87" s="17"/>
+      <c r="D87" s="19" t="s">
+        <v>916</v>
+      </c>
+      <c r="E87" s="18">
+        <v>1</v>
+      </c>
+      <c r="F87" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G87" s="25">
+        <v>2500</v>
+      </c>
+      <c r="H87" s="25">
+        <f t="shared" si="2"/>
+        <v>2500</v>
+      </c>
+      <c r="I87" s="18" t="s">
+        <v>837</v>
+      </c>
+      <c r="J87" s="42" t="s">
+        <v>923</v>
+      </c>
+      <c r="K87" s="27"/>
+    </row>
+    <row r="88" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B88" s="17">
         <v>87</v>
       </c>
-      <c r="C87" s="17"/>
-      <c r="D87" s="50" t="s">
+      <c r="C88" s="17" t="s">
+        <v>900</v>
+      </c>
+      <c r="D88" s="50" t="s">
+        <v>896</v>
+      </c>
+      <c r="E88" s="52">
+        <v>115</v>
+      </c>
+      <c r="F88" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G88" s="25">
+        <v>102</v>
+      </c>
+      <c r="H88" s="25">
+        <f t="shared" si="2"/>
+        <v>11730</v>
+      </c>
+      <c r="I88" s="17" t="s">
+        <v>837</v>
+      </c>
+      <c r="J88" s="42" t="s">
+        <v>922</v>
+      </c>
+      <c r="K88" s="27"/>
+    </row>
+    <row r="89" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B89" s="17">
+        <v>88</v>
+      </c>
+      <c r="C89" s="17"/>
+      <c r="D89" s="50" t="s">
         <v>853</v>
       </c>
-      <c r="E87" s="17">
+      <c r="E89" s="17">
         <v>87</v>
       </c>
-      <c r="F87" s="17" t="s">
+      <c r="F89" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G87" s="44">
+      <c r="G89" s="44">
         <v>34.99</v>
       </c>
-      <c r="H87" s="44">
+      <c r="H89" s="44">
         <f t="shared" si="2"/>
         <v>3044.13</v>
       </c>
-      <c r="I87" s="17" t="s">
+      <c r="I89" s="17" t="s">
         <v>791</v>
       </c>
-      <c r="J87" s="27"/>
-      <c r="K87" s="27"/>
-    </row>
-    <row r="88" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B88" s="17">
-        <v>88</v>
-      </c>
-      <c r="C88" s="17"/>
-      <c r="D88" s="55" t="s">
+      <c r="J89" s="27"/>
+      <c r="K89" s="27"/>
+    </row>
+    <row r="90" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B90" s="17">
+        <v>89</v>
+      </c>
+      <c r="C90" s="17"/>
+      <c r="D90" s="55" t="s">
         <v>854</v>
       </c>
-      <c r="E88" s="17">
+      <c r="E90" s="17">
         <v>174</v>
       </c>
-      <c r="F88" s="17" t="s">
+      <c r="F90" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G88" s="44">
+      <c r="G90" s="44">
         <v>255.5</v>
       </c>
-      <c r="H88" s="44">
+      <c r="H90" s="44">
         <f t="shared" si="2"/>
         <v>44457</v>
       </c>
-      <c r="I88" s="17" t="s">
+      <c r="I90" s="17" t="s">
         <v>791</v>
       </c>
-      <c r="J88" s="27"/>
-      <c r="K88" s="27"/>
-    </row>
-    <row r="89" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B89" s="17">
-        <v>89</v>
-      </c>
-      <c r="C89" s="17"/>
-      <c r="D89" s="50" t="s">
+      <c r="J90" s="27"/>
+      <c r="K90" s="27"/>
+    </row>
+    <row r="91" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B91" s="17">
+        <v>90</v>
+      </c>
+      <c r="C91" s="17"/>
+      <c r="D91" s="50" t="s">
         <v>855</v>
       </c>
-      <c r="E89" s="17">
+      <c r="E91" s="17">
         <v>174</v>
       </c>
-      <c r="F89" s="17" t="s">
+      <c r="F91" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G89" s="44">
+      <c r="G91" s="44">
         <v>196</v>
       </c>
-      <c r="H89" s="44">
+      <c r="H91" s="44">
         <f t="shared" si="2"/>
         <v>34104</v>
       </c>
-      <c r="I89" s="17" t="s">
+      <c r="I91" s="17" t="s">
         <v>791</v>
       </c>
-      <c r="J89" s="27"/>
-      <c r="K89" s="27"/>
-    </row>
-    <row r="90" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B90" s="17">
-        <v>90</v>
-      </c>
-      <c r="C90" s="17"/>
-      <c r="D90" s="55" t="s">
+      <c r="J91" s="27"/>
+      <c r="K91" s="27"/>
+    </row>
+    <row r="92" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B92" s="17">
+        <v>91</v>
+      </c>
+      <c r="C92" s="17"/>
+      <c r="D92" s="55" t="s">
         <v>840</v>
       </c>
-      <c r="E90" s="17">
+      <c r="E92" s="17">
         <v>4700</v>
       </c>
-      <c r="F90" s="17" t="s">
+      <c r="F92" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G90" s="44">
+      <c r="G92" s="44">
         <v>0.5</v>
       </c>
-      <c r="H90" s="44">
+      <c r="H92" s="44">
         <f t="shared" si="2"/>
         <v>2350</v>
       </c>
-      <c r="I90" s="17" t="s">
+      <c r="I92" s="17" t="s">
         <v>791</v>
       </c>
-      <c r="J90" s="27"/>
-      <c r="K90" s="27"/>
-    </row>
-    <row r="91" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B91" s="17">
-        <v>91</v>
-      </c>
-      <c r="C91" s="17"/>
-      <c r="D91" s="50" t="s">
+      <c r="J92" s="27"/>
+      <c r="K92" s="27"/>
+    </row>
+    <row r="93" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B93" s="17">
+        <v>92</v>
+      </c>
+      <c r="C93" s="17"/>
+      <c r="D93" s="50" t="s">
         <v>841</v>
       </c>
-      <c r="E91" s="17">
+      <c r="E93" s="17">
         <v>3200</v>
       </c>
-      <c r="F91" s="17" t="s">
+      <c r="F93" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G91" s="44">
+      <c r="G93" s="44">
         <v>0.5</v>
       </c>
-      <c r="H91" s="44">
+      <c r="H93" s="44">
         <f t="shared" si="2"/>
         <v>1600</v>
       </c>
-      <c r="I91" s="17" t="s">
+      <c r="I93" s="17" t="s">
         <v>791</v>
       </c>
-      <c r="J91" s="27"/>
-      <c r="K91" s="27"/>
-    </row>
-    <row r="92" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B92" s="17">
-        <v>92</v>
-      </c>
-      <c r="C92" s="17"/>
-      <c r="D92" s="50" t="s">
+      <c r="J93" s="27"/>
+      <c r="K93" s="27"/>
+    </row>
+    <row r="94" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B94" s="17">
+        <v>93</v>
+      </c>
+      <c r="C94" s="17"/>
+      <c r="D94" s="50" t="s">
         <v>781</v>
       </c>
-      <c r="E92" s="17">
-        <v>1</v>
-      </c>
-      <c r="F92" s="17" t="s">
+      <c r="E94" s="17">
+        <v>1</v>
+      </c>
+      <c r="F94" s="17" t="s">
         <v>760</v>
       </c>
-      <c r="G92" s="44">
+      <c r="G94" s="44">
         <v>908615.35</v>
       </c>
-      <c r="H92" s="44">
+      <c r="H94" s="44">
         <f t="shared" si="2"/>
         <v>908615.35</v>
       </c>
-      <c r="I92" s="17" t="s">
+      <c r="I94" s="17" t="s">
         <v>780</v>
       </c>
-      <c r="J92" s="27"/>
-      <c r="K92" s="27"/>
-    </row>
-    <row r="93" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B93" s="17">
-        <v>93</v>
-      </c>
-      <c r="C93" s="17" t="s">
+      <c r="J94" s="27"/>
+      <c r="K94" s="27"/>
+    </row>
+    <row r="95" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B95" s="17">
+        <v>94</v>
+      </c>
+      <c r="C95" s="17" t="s">
         <v>900</v>
       </c>
-      <c r="D93" s="19" t="s">
+      <c r="D95" s="19" t="s">
         <v>894</v>
       </c>
-      <c r="E93" s="18">
+      <c r="E95" s="18">
         <v>750</v>
       </c>
-      <c r="F93" s="18" t="s">
+      <c r="F95" s="18" t="s">
         <v>761</v>
       </c>
-      <c r="G93" s="25">
+      <c r="G95" s="25">
         <v>124.25</v>
       </c>
-      <c r="H93" s="25">
+      <c r="H95" s="25">
         <f t="shared" si="2"/>
         <v>93187.5</v>
       </c>
-      <c r="I93" s="18" t="s">
+      <c r="I95" s="18" t="s">
         <v>836</v>
       </c>
-      <c r="J93" s="27"/>
-      <c r="K93" s="27"/>
-    </row>
-    <row r="94" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B94" s="17">
-        <v>94</v>
-      </c>
-      <c r="C94" s="17" t="s">
+      <c r="J95" s="27"/>
+      <c r="K95" s="27"/>
+    </row>
+    <row r="96" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B96" s="17">
+        <v>95</v>
+      </c>
+      <c r="C96" s="17" t="s">
         <v>900</v>
       </c>
-      <c r="D94" s="19" t="s">
+      <c r="D96" s="19" t="s">
         <v>895</v>
       </c>
-      <c r="E94" s="18">
+      <c r="E96" s="18">
         <v>250</v>
       </c>
-      <c r="F94" s="18" t="s">
+      <c r="F96" s="18" t="s">
         <v>761</v>
       </c>
-      <c r="G94" s="25">
+      <c r="G96" s="25">
         <v>55.57</v>
       </c>
-      <c r="H94" s="25">
+      <c r="H96" s="25">
         <f t="shared" si="2"/>
         <v>13892.5</v>
       </c>
-      <c r="I94" s="18" t="s">
+      <c r="I96" s="18" t="s">
         <v>836</v>
       </c>
-      <c r="J94" s="27"/>
-      <c r="K94" s="27"/>
-    </row>
-    <row r="95" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B95" s="17">
-        <v>95</v>
-      </c>
-      <c r="C95" s="17"/>
-      <c r="D95" s="19" t="s">
+      <c r="J96" s="27"/>
+      <c r="K96" s="27"/>
+    </row>
+    <row r="97" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B97" s="17">
+        <v>96</v>
+      </c>
+      <c r="C97" s="17"/>
+      <c r="D97" s="19" t="s">
         <v>897</v>
       </c>
-      <c r="E95" s="18">
-        <v>1</v>
-      </c>
-      <c r="F95" s="18" t="s">
+      <c r="E97" s="18">
+        <v>1</v>
+      </c>
+      <c r="F97" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G95" s="25">
+      <c r="G97" s="25">
         <v>4430</v>
       </c>
-      <c r="H95" s="25">
+      <c r="H97" s="25">
         <f t="shared" si="2"/>
         <v>4430</v>
       </c>
-      <c r="I95" s="18" t="s">
+      <c r="I97" s="18" t="s">
         <v>836</v>
       </c>
-      <c r="J95" s="27"/>
-      <c r="K95" s="27"/>
-    </row>
-    <row r="96" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B96" s="17">
-        <v>96</v>
-      </c>
-      <c r="C96" s="17"/>
-      <c r="D96" s="19" t="s">
+      <c r="J97" s="27"/>
+      <c r="K97" s="27"/>
+    </row>
+    <row r="98" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B98" s="17">
+        <v>97</v>
+      </c>
+      <c r="C98" s="17"/>
+      <c r="D98" s="19" t="s">
         <v>796</v>
       </c>
-      <c r="E96" s="18">
-        <v>1</v>
-      </c>
-      <c r="F96" s="18" t="s">
+      <c r="E98" s="18">
+        <v>1</v>
+      </c>
+      <c r="F98" s="18" t="s">
         <v>760</v>
       </c>
-      <c r="G96" s="25">
+      <c r="G98" s="25">
         <v>670000</v>
       </c>
-      <c r="H96" s="25">
+      <c r="H98" s="25">
         <f t="shared" si="2"/>
         <v>670000</v>
       </c>
-      <c r="I96" s="18" t="s">
+      <c r="I98" s="18" t="s">
         <v>836</v>
       </c>
-      <c r="J96" s="27"/>
-      <c r="K96" s="27"/>
-      <c r="L96" s="14"/>
-    </row>
-    <row r="97" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B97" s="17">
-        <v>97</v>
-      </c>
-      <c r="C97" s="17"/>
-      <c r="D97" s="19" t="s">
+      <c r="J98" s="27"/>
+      <c r="K98" s="27"/>
+      <c r="L98" s="14"/>
+    </row>
+    <row r="99" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B99" s="17">
+        <v>98</v>
+      </c>
+      <c r="C99" s="17"/>
+      <c r="D99" s="19" t="s">
         <v>827</v>
       </c>
-      <c r="E97" s="52">
+      <c r="E99" s="52">
         <f>8*4.2*0.35</f>
         <v>11.76</v>
       </c>
-      <c r="F97" s="18" t="s">
+      <c r="F99" s="18" t="s">
         <v>759</v>
       </c>
-      <c r="G97" s="25">
+      <c r="G99" s="25">
         <v>670</v>
       </c>
-      <c r="H97" s="25">
+      <c r="H99" s="25">
         <f t="shared" si="2"/>
         <v>7879.2</v>
       </c>
-      <c r="I97" s="18" t="s">
+      <c r="I99" s="18" t="s">
         <v>836</v>
       </c>
-      <c r="J97" s="27"/>
-      <c r="K97" s="27"/>
-    </row>
-    <row r="98" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B98" s="17">
-        <v>98</v>
-      </c>
-      <c r="C98" s="17"/>
-      <c r="D98" s="19" t="s">
-        <v>828</v>
-      </c>
-      <c r="E98" s="18">
-        <v>600</v>
-      </c>
-      <c r="F98" s="18" t="s">
-        <v>811</v>
-      </c>
-      <c r="G98" s="25">
-        <v>9.99</v>
-      </c>
-      <c r="H98" s="25">
-        <f t="shared" ref="H98" si="3">G98*E98</f>
-        <v>5994</v>
-      </c>
-      <c r="I98" s="18" t="s">
-        <v>836</v>
-      </c>
-      <c r="J98" s="27"/>
-      <c r="K98" s="27"/>
-      <c r="L98" s="14" t="s">
-        <v>812</v>
-      </c>
-    </row>
-    <row r="99" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B99" s="18"/>
-      <c r="C99" s="18"/>
-      <c r="D99" s="19"/>
-      <c r="E99" s="18"/>
-      <c r="F99" s="18"/>
-      <c r="G99" s="20"/>
-      <c r="H99" s="23"/>
-      <c r="I99" s="18"/>
       <c r="J99" s="27"/>
       <c r="K99" s="27"/>
     </row>
     <row r="100" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B100" s="18"/>
-      <c r="C100" s="18"/>
-      <c r="D100" s="19"/>
-      <c r="E100" s="18"/>
-      <c r="F100" s="18"/>
-      <c r="G100" s="20" t="s">
-        <v>925</v>
-      </c>
-      <c r="H100" s="23" t="s">
-        <v>926</v>
-      </c>
-      <c r="I100" s="18"/>
+      <c r="B100" s="17">
+        <v>99</v>
+      </c>
+      <c r="C100" s="17"/>
+      <c r="D100" s="19" t="s">
+        <v>828</v>
+      </c>
+      <c r="E100" s="18">
+        <v>600</v>
+      </c>
+      <c r="F100" s="18" t="s">
+        <v>811</v>
+      </c>
+      <c r="G100" s="25">
+        <v>9.99</v>
+      </c>
+      <c r="H100" s="25">
+        <f t="shared" ref="H100" si="3">G100*E100</f>
+        <v>5994</v>
+      </c>
+      <c r="I100" s="18" t="s">
+        <v>836</v>
+      </c>
       <c r="J100" s="27"/>
       <c r="K100" s="27"/>
+      <c r="L100" s="14" t="s">
+        <v>812</v>
+      </c>
     </row>
     <row r="101" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D101" s="21"/>
-      <c r="E101" s="22"/>
-      <c r="F101" s="22"/>
-      <c r="H101" s="16">
+      <c r="B101" s="18"/>
+      <c r="C101" s="18"/>
+      <c r="D101" s="19"/>
+      <c r="E101" s="18"/>
+      <c r="F101" s="18"/>
+      <c r="G101" s="20"/>
+      <c r="H101" s="23"/>
+      <c r="I101" s="18"/>
+      <c r="J101" s="27"/>
+      <c r="K101" s="27"/>
+    </row>
+    <row r="102" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B102" s="18"/>
+      <c r="C102" s="18"/>
+      <c r="D102" s="19"/>
+      <c r="E102" s="18"/>
+      <c r="F102" s="18"/>
+      <c r="G102" s="20" t="s">
+        <v>925</v>
+      </c>
+      <c r="H102" s="23" t="s">
+        <v>926</v>
+      </c>
+      <c r="I102" s="18"/>
+      <c r="J102" s="27"/>
+      <c r="K102" s="27"/>
+    </row>
+    <row r="103" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D103" s="21"/>
+      <c r="E103" s="22"/>
+      <c r="F103" s="22"/>
+      <c r="H103" s="16">
         <f>SUM(Tabela24[Preço Total])</f>
-        <v>5833096.2741069021</v>
-      </c>
-    </row>
-    <row r="102" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D102" s="28"/>
-      <c r="E102" s="29"/>
-      <c r="F102" s="29"/>
-    </row>
-    <row r="105" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="H105" s="26"/>
+        <v>7380849.444106902</v>
+      </c>
+    </row>
+    <row r="104" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D104" s="28"/>
+      <c r="E104" s="29"/>
+      <c r="F104" s="29"/>
+    </row>
+    <row r="107" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H107" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -15692,8 +15751,8 @@
         <v>910</v>
       </c>
       <c r="D2" s="37">
-        <f>'DPA IV'!H101</f>
-        <v>5833096.2741069021</v>
+        <f>'DPA IV'!H103</f>
+        <v>7380849.444106902</v>
       </c>
     </row>
     <row r="3" spans="3:7" x14ac:dyDescent="0.25">
@@ -15726,7 +15785,7 @@
       </c>
       <c r="E5" s="41">
         <f t="shared" ref="E5:E21" si="0">D5/$D$2</f>
-        <v>0.17015045755471625</v>
+        <v>0.13447015922976804</v>
       </c>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
@@ -15741,7 +15800,7 @@
       </c>
       <c r="E6" s="41">
         <f t="shared" si="0"/>
-        <v>0.15576896168049564</v>
+        <v>0.12310444168800469</v>
       </c>
       <c r="F6" s="14"/>
       <c r="G6" s="14"/>
@@ -15756,7 +15815,7 @@
       </c>
       <c r="E7" s="41">
         <f t="shared" si="0"/>
-        <v>0.15322925578876886</v>
+        <v>0.12109730835104345</v>
       </c>
       <c r="F7" s="38"/>
       <c r="G7" s="14"/>
@@ -15771,7 +15830,7 @@
       </c>
       <c r="E8" s="41">
         <f t="shared" si="0"/>
-        <v>0.13635694708669627</v>
+        <v>0.10776309773329118</v>
       </c>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
@@ -15801,7 +15860,7 @@
       </c>
       <c r="E10" s="41">
         <f t="shared" si="0"/>
-        <v>7.3537685620605739E-2</v>
+        <v>5.8116942128184024E-2</v>
       </c>
       <c r="F10" s="38"/>
       <c r="G10" s="14"/>
@@ -15816,7 +15875,7 @@
       </c>
       <c r="E11" s="41">
         <f t="shared" si="0"/>
-        <v>6.6419204686268316E-2</v>
+        <v>5.2491196076889381E-2</v>
       </c>
       <c r="F11" s="38"/>
       <c r="G11" s="14"/>
@@ -15831,7 +15890,7 @@
       </c>
       <c r="E12" s="41">
         <f t="shared" si="0"/>
-        <v>6.0608505250151296E-2</v>
+        <v>4.7898991685316056E-2</v>
       </c>
       <c r="F12" s="14"/>
       <c r="G12" s="14"/>
@@ -15846,7 +15905,7 @@
       </c>
       <c r="E13" s="41">
         <f t="shared" si="0"/>
-        <v>2.013510397922973E-2</v>
+        <v>1.5912802569597963E-2</v>
       </c>
       <c r="F13" s="14"/>
       <c r="G13" s="14"/>
@@ -15861,7 +15920,7 @@
       </c>
       <c r="E14" s="41">
         <f t="shared" si="0"/>
-        <v>1.7803457224079541E-2</v>
+        <v>1.4070098677180912E-2</v>
       </c>
       <c r="F14" s="38"/>
       <c r="G14" s="14"/>
@@ -15876,7 +15935,7 @@
       </c>
       <c r="E15" s="41">
         <f t="shared" si="0"/>
-        <v>1.7588760196574758E-2</v>
+        <v>1.3900423297580818E-2</v>
       </c>
       <c r="F15" s="38"/>
       <c r="G15" s="14"/>
@@ -15891,7 +15950,7 @@
       </c>
       <c r="E16" s="41">
         <f t="shared" si="0"/>
-        <v>1.466718977017043E-2</v>
+        <v>1.1591501851905387E-2</v>
       </c>
       <c r="F16" s="14"/>
       <c r="G16" s="14"/>
@@ -15906,7 +15965,7 @@
       </c>
       <c r="E17" s="41">
         <f t="shared" si="0"/>
-        <v>7.6704751424406222E-3</v>
+        <v>6.0619878935105351E-3</v>
       </c>
       <c r="F17" s="38"/>
       <c r="G17" s="14"/>
@@ -15921,7 +15980,7 @@
       </c>
       <c r="E18" s="41">
         <f t="shared" si="0"/>
-        <v>7.20029261070795E-3</v>
+        <v>5.6904019405969722E-3</v>
       </c>
       <c r="F18" s="14"/>
       <c r="G18" s="14"/>
@@ -15936,7 +15995,7 @@
       </c>
       <c r="E19" s="41">
         <f t="shared" si="0"/>
-        <v>1.3138733941389331E-2</v>
+        <v>1.0383560941104325E-2</v>
       </c>
       <c r="F19" s="38"/>
       <c r="G19" s="14"/>
@@ -15951,7 +16010,7 @@
       </c>
       <c r="E20" s="41">
         <f t="shared" si="0"/>
-        <v>9.1889448555701448E-4</v>
+        <v>7.2620367622856601E-4</v>
       </c>
       <c r="F20" s="38"/>
       <c r="G20" s="14"/>
@@ -15962,11 +16021,11 @@
       </c>
       <c r="D21" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Armazenamento",Tabela24[Preço Total])</f>
-        <v>0</v>
+        <v>1547753.1700000002</v>
       </c>
       <c r="E21" s="41">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.20969851528888372</v>
       </c>
       <c r="F21" s="14"/>
       <c r="G21" s="14"/>

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 15:32
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2378" uniqueCount="931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2364" uniqueCount="931">
   <si>
     <t>Código EAP</t>
   </si>
@@ -17574,156 +17574,108 @@
         <v>1220849.67</v>
       </c>
       <c r="E7" s="41">
-        <f t="shared" ref="E7:E20" si="0">D7/$D$2</f>
+        <f>D7/$D$2</f>
         <v>0.27915414542962674</v>
       </c>
-      <c r="F7" s="41">
-        <f>E7</f>
-        <v>0.27915414542962674</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>913</v>
-      </c>
+      <c r="F7" s="41"/>
     </row>
     <row r="8" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>779</v>
+        <v>798</v>
       </c>
       <c r="D8" s="40">
-        <f>SUMIF(Tabela2[Aplicação],"AVCB",Tabela2[Preço Total])</f>
-        <v>0</v>
+        <f>SUMIF(Tabela2[Aplicação],"Armazenamento",Tabela2[Preço Total])</f>
+        <v>1177977.5</v>
       </c>
       <c r="E8" s="41">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F8" s="41">
-        <f t="shared" ref="F8:F20" si="1">F7+E8</f>
-        <v>0.27915414542962674</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>913</v>
-      </c>
+        <f>D8/$D$2</f>
+        <v>0.26935118256437596</v>
+      </c>
+      <c r="F8" s="41"/>
     </row>
     <row r="9" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>419</v>
+        <v>635</v>
       </c>
       <c r="D9" s="40">
-        <f>SUMIF(Tabela2[Aplicação],"SPDA",Tabela2[Preço Total])</f>
-        <v>0</v>
+        <f>SUMIF(Tabela2[Aplicação],"Piso",Tabela2[Preço Total])</f>
+        <v>361131.5538461539</v>
       </c>
       <c r="E9" s="41">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F9" s="41">
-        <f t="shared" si="1"/>
-        <v>0.27915414542962674</v>
-      </c>
-      <c r="G9" s="14" t="s">
-        <v>913</v>
-      </c>
+        <f>D9/$D$2</f>
+        <v>8.2574761478697328E-2</v>
+      </c>
+      <c r="F9" s="41"/>
     </row>
     <row r="10" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>635</v>
+        <v>791</v>
       </c>
       <c r="D10" s="40">
-        <f>SUMIF(Tabela2[Aplicação],"Piso",Tabela2[Preço Total])</f>
-        <v>361131.5538461539</v>
+        <f>SUMIF(Tabela2[Aplicação],"Telhado",Tabela2[Preço Total])</f>
+        <v>216713.79700000002</v>
       </c>
       <c r="E10" s="41">
-        <f t="shared" si="0"/>
-        <v>8.2574761478697328E-2</v>
-      </c>
-      <c r="F10" s="41">
-        <f t="shared" si="1"/>
-        <v>0.36172890690832404</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>913</v>
-      </c>
+        <f>D10/$D$2</f>
+        <v>4.9552828895259984E-2</v>
+      </c>
+      <c r="F10" s="41"/>
     </row>
     <row r="11" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>791</v>
+        <v>780</v>
       </c>
       <c r="D11" s="40">
-        <f>SUMIF(Tabela2[Aplicação],"Telhado",Tabela2[Preço Total])</f>
-        <v>216713.79700000002</v>
+        <f>SUMIF(Tabela2[Aplicação],"Terraplanagem",Tabela2[Preço Total])</f>
+        <v>174417.38</v>
       </c>
       <c r="E11" s="41">
-        <f t="shared" si="0"/>
-        <v>4.9552828895259984E-2</v>
-      </c>
-      <c r="F11" s="41">
-        <f t="shared" si="1"/>
-        <v>0.41128173580358401</v>
-      </c>
-      <c r="G11" s="14" t="s">
-        <v>914</v>
-      </c>
+        <f>D11/$D$2</f>
+        <v>3.9881515192590811E-2</v>
+      </c>
+      <c r="F11" s="41"/>
     </row>
     <row r="12" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>780</v>
+        <v>771</v>
       </c>
       <c r="D12" s="40">
-        <f>SUMIF(Tabela2[Aplicação],"Terraplanagem",Tabela2[Preço Total])</f>
-        <v>174417.38</v>
+        <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
+        <v>164340</v>
       </c>
       <c r="E12" s="41">
-        <f t="shared" si="0"/>
-        <v>3.9881515192590811E-2</v>
-      </c>
-      <c r="F12" s="41">
-        <f t="shared" si="1"/>
-        <v>0.45116325099617482</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>914</v>
-      </c>
+        <f>D12/$D$2</f>
+        <v>3.7577265561209404E-2</v>
+      </c>
+      <c r="F12" s="41"/>
     </row>
     <row r="13" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="D13" s="40">
-        <f>SUMIF(Tabela2[Aplicação],"Fundação",Tabela2[Preço Total])</f>
-        <v>164340</v>
+        <f>SUMIF(Tabela2[Aplicação],"Fechamento Lateral",Tabela2[Preço Total])</f>
+        <v>79138.372999999992</v>
       </c>
       <c r="E13" s="41">
-        <f t="shared" si="0"/>
-        <v>3.7577265561209404E-2</v>
-      </c>
-      <c r="F13" s="41">
-        <f t="shared" si="1"/>
-        <v>0.48874051655738421</v>
-      </c>
-      <c r="G13" s="14" t="s">
-        <v>915</v>
-      </c>
+        <f>D13/$D$2</f>
+        <v>1.809543421140954E-2</v>
+      </c>
+      <c r="F13" s="41"/>
     </row>
     <row r="14" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>774</v>
+        <v>902</v>
       </c>
       <c r="D14" s="40">
-        <f>SUMIF(Tabela2[Aplicação],"Fechamento Lateral",Tabela2[Preço Total])</f>
-        <v>79138.372999999992</v>
+        <f>SUMIF(Tabela2[Aplicação],"Iluminação Galpão",Tabela2[Preço Total])</f>
+        <v>66919.5</v>
       </c>
       <c r="E14" s="41">
-        <f t="shared" si="0"/>
-        <v>1.809543421140954E-2</v>
-      </c>
-      <c r="F14" s="41">
-        <f t="shared" si="1"/>
-        <v>0.50683595076879373</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>915</v>
-      </c>
+        <f>D14/$D$2</f>
+        <v>1.5301520157742197E-2</v>
+      </c>
+      <c r="F14" s="41"/>
     </row>
     <row r="15" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
@@ -17734,16 +17686,10 @@
         <v>21626.68</v>
       </c>
       <c r="E15" s="41">
-        <f t="shared" si="0"/>
+        <f>D15/$D$2</f>
         <v>4.945062051644738E-3</v>
       </c>
-      <c r="F15" s="41">
-        <f t="shared" si="1"/>
-        <v>0.51178101282043842</v>
-      </c>
-      <c r="G15" s="14" t="s">
-        <v>915</v>
-      </c>
+      <c r="F15" s="41"/>
     </row>
     <row r="16" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
@@ -17754,133 +17700,103 @@
         <v>18517.59</v>
       </c>
       <c r="E16" s="41">
-        <f t="shared" si="0"/>
+        <f>D16/$D$2</f>
         <v>4.2341511317001077E-3</v>
       </c>
-      <c r="F16" s="41">
-        <f t="shared" si="1"/>
-        <v>0.51601516395213853</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>915</v>
-      </c>
-    </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="F16" s="41"/>
+    </row>
+    <row r="17" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
-        <v>902</v>
+        <v>576</v>
       </c>
       <c r="D17" s="40">
-        <f>SUMIF(Tabela2[Aplicação],"Iluminação Galpão",Tabela2[Preço Total])</f>
-        <v>66919.5</v>
-      </c>
-      <c r="E17" s="41">
-        <f t="shared" si="0"/>
-        <v>1.5301520157742197E-2</v>
-      </c>
-      <c r="F17" s="41">
-        <f t="shared" si="1"/>
-        <v>0.53131668410988075</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>915</v>
-      </c>
-    </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C18" t="s">
-        <v>576</v>
-      </c>
-      <c r="D18" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Pintura",Tabela2[Preço Total])</f>
         <v>5300</v>
       </c>
-      <c r="E18" s="41">
-        <f t="shared" si="0"/>
+      <c r="E17" s="41">
+        <f>D17/$D$2</f>
         <v>1.2118748172959099E-3</v>
       </c>
-      <c r="F18" s="41">
-        <f t="shared" si="1"/>
-        <v>0.53252855892717665</v>
-      </c>
-      <c r="G18" s="14" t="s">
-        <v>915</v>
-      </c>
-    </row>
-    <row r="19" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C19" t="s">
+      <c r="F17" s="41"/>
+    </row>
+    <row r="18" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
         <v>815</v>
       </c>
-      <c r="D19" s="40">
+      <c r="D18" s="40">
         <f>SUMIF(Tabela2[Aplicação],"Topografia",Tabela2[Preço Total])</f>
         <v>5000</v>
       </c>
+      <c r="E18" s="41">
+        <f>D18/$D$2</f>
+        <v>1.1432781295244432E-3</v>
+      </c>
+      <c r="F18" s="41"/>
+    </row>
+    <row r="19" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>779</v>
+      </c>
+      <c r="D19" s="40">
+        <f>SUMIF(Tabela2[Aplicação],"AVCB",Tabela2[Preço Total])</f>
+        <v>0</v>
+      </c>
       <c r="E19" s="41">
-        <f t="shared" si="0"/>
-        <v>1.1432781295244432E-3</v>
-      </c>
-      <c r="F19" s="41">
-        <f t="shared" si="1"/>
-        <v>0.53367183705670107</v>
-      </c>
-      <c r="G19" s="14" t="s">
-        <v>915</v>
-      </c>
-    </row>
-    <row r="20" spans="3:7" x14ac:dyDescent="0.25">
+        <f>D19/$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="41"/>
+    </row>
+    <row r="20" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>798</v>
+        <v>419</v>
       </c>
       <c r="D20" s="40">
-        <f>SUMIF(Tabela2[Aplicação],"Armazenamento",Tabela2[Preço Total])</f>
-        <v>1177977.5</v>
+        <f>SUMIF(Tabela2[Aplicação],"SPDA",Tabela2[Preço Total])</f>
+        <v>0</v>
       </c>
       <c r="E20" s="41">
-        <f t="shared" si="0"/>
-        <v>0.26935118256437596</v>
-      </c>
-      <c r="F20" s="41">
-        <f t="shared" si="1"/>
-        <v>0.80302301962107703</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>915</v>
-      </c>
-    </row>
-    <row r="21" spans="3:7" x14ac:dyDescent="0.25">
+        <f>D20/$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="41"/>
+    </row>
+    <row r="21" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D21" s="40"/>
       <c r="E21" s="38"/>
       <c r="F21" s="38"/>
     </row>
-    <row r="22" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D22" s="40"/>
       <c r="E22" s="38"/>
       <c r="F22" s="38"/>
     </row>
-    <row r="23" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D23" s="40"/>
       <c r="E23" s="38"/>
       <c r="F23" s="38"/>
     </row>
-    <row r="24" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D24" s="40"/>
       <c r="E24" s="38"/>
       <c r="F24" s="38"/>
     </row>
-    <row r="25" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D25" s="40"/>
       <c r="E25" s="38"/>
       <c r="F25" s="38"/>
     </row>
-    <row r="26" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D26" s="40"/>
       <c r="E26" s="38"/>
       <c r="F26" s="38"/>
     </row>
-    <row r="27" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D27" s="40"/>
       <c r="E27" s="38"/>
       <c r="F27" s="38"/>
     </row>
-    <row r="28" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:6" x14ac:dyDescent="0.25">
       <c r="D28" s="40"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 15:36
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2364" uniqueCount="931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2366" uniqueCount="932">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2822,6 +2822,9 @@
   </si>
   <si>
     <t>Frete</t>
+  </si>
+  <si>
+    <t>Prazo de Execução Depósito de produto acabado IV:</t>
   </si>
 </sst>
 </file>
@@ -17483,17 +17486,25 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:B2"/>
+  <dimension ref="A2:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="46.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
+        <v>931</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
         <v>927</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B3" s="20" t="s">
         <v>928</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 15:51
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Expansão DMP" sheetId="3" r:id="rId4"/>
     <sheet name="Prazo de Execução" sheetId="9" r:id="rId5"/>
     <sheet name="ABC DMP" sheetId="8" r:id="rId6"/>
+    <sheet name="DPA IV CARRO SHUTTLE" sheetId="10" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">' ABC DPA IV'!$C$4:$G$4</definedName>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2366" uniqueCount="932">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2709" uniqueCount="933">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2825,6 +2826,9 @@
   </si>
   <si>
     <t>Prazo de Execução Depósito de produto acabado IV:</t>
+  </si>
+  <si>
+    <t>Carro shuttle operação do drive in</t>
   </si>
 </sst>
 </file>
@@ -3087,7 +3091,170 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="32">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF404040"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF404040"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -3400,45 +3567,68 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B1:J100" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tabela24" displayName="Tabela24" ref="B1:J100" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
   <autoFilter ref="B1:J100"/>
   <sortState ref="B2:J100">
     <sortCondition ref="I1:I100"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" name="Item" dataDxfId="18" dataCellStyle="Normal"/>
-    <tableColumn id="8" name="Local" dataDxfId="17"/>
-    <tableColumn id="2" name="Insumo ou Serviço" dataDxfId="16" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="Quantidade" dataDxfId="15" dataCellStyle="Normal"/>
-    <tableColumn id="4" name="Unidade" dataDxfId="14" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Preço Unitário" dataDxfId="13" dataCellStyle="Moeda"/>
-    <tableColumn id="6" name="Preço Total" dataDxfId="12" dataCellStyle="Moeda">
+    <tableColumn id="1" name="Item" dataDxfId="29" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Local" dataDxfId="28"/>
+    <tableColumn id="2" name="Insumo ou Serviço" dataDxfId="27" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="26" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="25" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="24" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="23" dataCellStyle="Moeda">
       <calculatedColumnFormula>G2*E2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Aplicação" dataDxfId="11" dataCellStyle="Normal"/>
-    <tableColumn id="11" name="Grupo Serviço premilinar " dataDxfId="10"/>
+    <tableColumn id="7" name="Aplicação" dataDxfId="22" dataCellStyle="Normal"/>
+    <tableColumn id="11" name="Grupo Serviço premilinar " dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:I56" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela2" displayName="Tabela2" ref="B3:I56" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
   <autoFilter ref="B3:I56"/>
   <sortState ref="B4:I56">
     <sortCondition ref="H3:H56"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" name="Item" dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="2" name="Descrição" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="1" name="Item" dataDxfId="18" dataCellStyle="Normal"/>
+    <tableColumn id="2" name="Descrição" dataDxfId="17" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="Quantidade" dataDxfId="16" dataCellStyle="Normal"/>
+    <tableColumn id="4" name="Unidade" dataDxfId="15" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Preço Unitário" dataDxfId="14" dataCellStyle="Moeda"/>
+    <tableColumn id="6" name="Preço Total" dataDxfId="13" dataCellStyle="Moeda">
+      <calculatedColumnFormula>F4*D4</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" name="Aplicação" dataDxfId="12" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Grupo Serviço premilinar " dataDxfId="11" dataCellStyle="Normal"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela242" displayName="Tabela242" ref="B1:J101" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+  <autoFilter ref="B1:J101"/>
+  <sortState ref="B2:J100">
+    <sortCondition ref="I1:I100"/>
+  </sortState>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Item" dataDxfId="8" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Local" dataDxfId="7"/>
+    <tableColumn id="2" name="Insumo ou Serviço" dataDxfId="6" dataCellStyle="Normal"/>
     <tableColumn id="3" name="Quantidade" dataDxfId="5" dataCellStyle="Normal"/>
     <tableColumn id="4" name="Unidade" dataDxfId="4" dataCellStyle="Normal"/>
     <tableColumn id="5" name="Preço Unitário" dataDxfId="3" dataCellStyle="Moeda"/>
     <tableColumn id="6" name="Preço Total" dataDxfId="2" dataCellStyle="Moeda">
-      <calculatedColumnFormula>F4*D4</calculatedColumnFormula>
+      <calculatedColumnFormula>G2*E2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" name="Aplicação" dataDxfId="1" dataCellStyle="Normal"/>
-    <tableColumn id="8" name="Grupo Serviço premilinar " dataDxfId="0" dataCellStyle="Normal"/>
+    <tableColumn id="11" name="Grupo Serviço premilinar " dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -17818,4 +18008,3060 @@
   </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B1:O108"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.85546875" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="14"/>
+    <col min="3" max="3" width="27.7109375" style="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="92" customWidth="1"/>
+    <col min="5" max="5" width="16" style="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.42578125" style="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" style="15" customWidth="1"/>
+    <col min="9" max="9" width="23.85546875" style="14" customWidth="1"/>
+    <col min="10" max="10" width="43.7109375" style="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.28515625" style="14" customWidth="1"/>
+    <col min="12" max="12" width="55.5703125" style="24" customWidth="1"/>
+    <col min="13" max="13" width="54.42578125" style="14" customWidth="1"/>
+    <col min="14" max="15" width="16" style="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:12" s="15" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="15" t="s">
+        <v>753</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>795</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>858</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>755</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>756</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>764</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>765</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>767</v>
+      </c>
+      <c r="J1" s="15" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2" s="17">
+        <v>1</v>
+      </c>
+      <c r="C2" s="17"/>
+      <c r="D2" s="19" t="s">
+        <v>787</v>
+      </c>
+      <c r="E2" s="18">
+        <v>1</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G2" s="20">
+        <v>1983985.92</v>
+      </c>
+      <c r="H2" s="20">
+        <f>G2*E2</f>
+        <v>1983985.92</v>
+      </c>
+      <c r="I2" s="18" t="s">
+        <v>798</v>
+      </c>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="24" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B3" s="17">
+        <v>2</v>
+      </c>
+      <c r="C3" s="17"/>
+      <c r="D3" s="19" t="s">
+        <v>929</v>
+      </c>
+      <c r="E3" s="18">
+        <v>1</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G3" s="20">
+        <v>294700</v>
+      </c>
+      <c r="H3" s="20">
+        <f>G3*E3</f>
+        <v>294700</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>798</v>
+      </c>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+    </row>
+    <row r="4" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="17">
+        <v>3</v>
+      </c>
+      <c r="C4" s="17"/>
+      <c r="D4" s="19" t="s">
+        <v>930</v>
+      </c>
+      <c r="E4" s="18">
+        <v>1</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G4" s="20">
+        <v>88200</v>
+      </c>
+      <c r="H4" s="20">
+        <f>G4*E4</f>
+        <v>88200</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>798</v>
+      </c>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="24"/>
+    </row>
+    <row r="5" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="19" t="s">
+        <v>932</v>
+      </c>
+      <c r="E5" s="18">
+        <v>3</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G5" s="20">
+        <v>300000</v>
+      </c>
+      <c r="H5" s="20">
+        <f>G5*E5</f>
+        <v>900000</v>
+      </c>
+      <c r="I5" s="18" t="s">
+        <v>798</v>
+      </c>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="24"/>
+    </row>
+    <row r="6" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="17">
+        <v>4</v>
+      </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="50" t="s">
+        <v>819</v>
+      </c>
+      <c r="E6" s="17">
+        <v>1</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G6" s="44">
+        <v>486032</v>
+      </c>
+      <c r="H6" s="44">
+        <f>G6*E6</f>
+        <v>486032</v>
+      </c>
+      <c r="I6" s="31" t="s">
+        <v>920</v>
+      </c>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="24"/>
+    </row>
+    <row r="7" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="17">
+        <v>5</v>
+      </c>
+      <c r="C7" s="17"/>
+      <c r="D7" s="50" t="s">
+        <v>821</v>
+      </c>
+      <c r="E7" s="17">
+        <v>1</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G7" s="44">
+        <v>8650</v>
+      </c>
+      <c r="H7" s="44">
+        <f>G7*E7</f>
+        <v>8650</v>
+      </c>
+      <c r="I7" s="31" t="s">
+        <v>920</v>
+      </c>
+      <c r="J7" s="27"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="24"/>
+    </row>
+    <row r="8" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="17">
+        <v>6</v>
+      </c>
+      <c r="C8" s="17"/>
+      <c r="D8" s="50" t="s">
+        <v>820</v>
+      </c>
+      <c r="E8" s="17">
+        <v>6</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G8" s="44">
+        <v>21938</v>
+      </c>
+      <c r="H8" s="44">
+        <f>G8*E8</f>
+        <v>131628</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>835</v>
+      </c>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="24"/>
+    </row>
+    <row r="9" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="17">
+        <v>7</v>
+      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="50" t="s">
+        <v>899</v>
+      </c>
+      <c r="E9" s="17">
+        <v>1</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G9" s="44">
+        <v>11180</v>
+      </c>
+      <c r="H9" s="44">
+        <f>G9*E9</f>
+        <v>11180</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>835</v>
+      </c>
+      <c r="J9" s="27"/>
+      <c r="K9" s="27"/>
+      <c r="L9" s="24"/>
+    </row>
+    <row r="10" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="17">
+        <v>8</v>
+      </c>
+      <c r="C10" s="17"/>
+      <c r="D10" s="19" t="s">
+        <v>889</v>
+      </c>
+      <c r="E10" s="17">
+        <v>250</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>761</v>
+      </c>
+      <c r="G10" s="44">
+        <v>55.57</v>
+      </c>
+      <c r="H10" s="44">
+        <f>G10*E10</f>
+        <v>13892.5</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>835</v>
+      </c>
+      <c r="J10" s="27"/>
+      <c r="K10" s="27"/>
+      <c r="L10" s="24"/>
+    </row>
+    <row r="11" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="17">
+        <v>9</v>
+      </c>
+      <c r="C11" s="18"/>
+      <c r="D11" s="19" t="s">
+        <v>888</v>
+      </c>
+      <c r="E11" s="18">
+        <v>6</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G11" s="25">
+        <v>13855.22</v>
+      </c>
+      <c r="H11" s="51">
+        <f>G11*E11</f>
+        <v>83131.319999999992</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>835</v>
+      </c>
+      <c r="J11" s="27"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="24"/>
+    </row>
+    <row r="12" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="17">
+        <v>10</v>
+      </c>
+      <c r="C12" s="18"/>
+      <c r="D12" s="19" t="s">
+        <v>886</v>
+      </c>
+      <c r="E12" s="18">
+        <v>1</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G12" s="25">
+        <v>111260.98</v>
+      </c>
+      <c r="H12" s="51">
+        <f>G12*E12</f>
+        <v>111260.98</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>835</v>
+      </c>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="24"/>
+    </row>
+    <row r="13" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="17">
+        <v>11</v>
+      </c>
+      <c r="C13" s="18"/>
+      <c r="D13" s="19" t="s">
+        <v>887</v>
+      </c>
+      <c r="E13" s="18">
+        <v>300</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G13" s="25">
+        <v>55.57</v>
+      </c>
+      <c r="H13" s="51">
+        <f>G13*E13</f>
+        <v>16671</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>835</v>
+      </c>
+      <c r="J13" s="27"/>
+      <c r="K13" s="27"/>
+      <c r="L13" s="24"/>
+    </row>
+    <row r="14" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="17">
+        <v>12</v>
+      </c>
+      <c r="C14" s="18"/>
+      <c r="D14" s="19" t="s">
+        <v>838</v>
+      </c>
+      <c r="E14" s="18">
+        <v>1</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G14" s="25">
+        <v>27412.5</v>
+      </c>
+      <c r="H14" s="51">
+        <f>G14*E14</f>
+        <v>27412.5</v>
+      </c>
+      <c r="I14" s="17" t="s">
+        <v>835</v>
+      </c>
+      <c r="J14" s="27"/>
+      <c r="K14" s="27"/>
+      <c r="L14" s="24"/>
+    </row>
+    <row r="15" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="17">
+        <v>13</v>
+      </c>
+      <c r="C15" s="18"/>
+      <c r="D15" s="19" t="s">
+        <v>757</v>
+      </c>
+      <c r="E15" s="52">
+        <f>(1075*0.15)*1.1</f>
+        <v>177.37500000000003</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>759</v>
+      </c>
+      <c r="G15" s="25">
+        <v>670</v>
+      </c>
+      <c r="H15" s="25">
+        <f>G15*E15</f>
+        <v>118841.25000000001</v>
+      </c>
+      <c r="I15" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="24"/>
+    </row>
+    <row r="16" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="17">
+        <v>14</v>
+      </c>
+      <c r="C16" s="18"/>
+      <c r="D16" s="50" t="s">
+        <v>775</v>
+      </c>
+      <c r="E16" s="52">
+        <f>1075/13*2</f>
+        <v>165.38461538461539</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G16" s="25">
+        <v>220.5</v>
+      </c>
+      <c r="H16" s="25">
+        <f>G16*E16</f>
+        <v>36467.307692307695</v>
+      </c>
+      <c r="I16" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="24"/>
+    </row>
+    <row r="17" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="17">
+        <v>15</v>
+      </c>
+      <c r="C17" s="18"/>
+      <c r="D17" s="50" t="s">
+        <v>758</v>
+      </c>
+      <c r="E17" s="52">
+        <f>(20*53)/12</f>
+        <v>88.333333333333329</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G17" s="25">
+        <v>56.2</v>
+      </c>
+      <c r="H17" s="25">
+        <f>G17*E17</f>
+        <v>4964.333333333333</v>
+      </c>
+      <c r="I17" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
+      <c r="L17" s="24"/>
+    </row>
+    <row r="18" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="17">
+        <v>16</v>
+      </c>
+      <c r="C18" s="18"/>
+      <c r="D18" s="50" t="s">
+        <v>792</v>
+      </c>
+      <c r="E18" s="52">
+        <f>E15</f>
+        <v>177.37500000000003</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G18" s="25">
+        <v>50</v>
+      </c>
+      <c r="H18" s="25">
+        <f>G18*E18</f>
+        <v>8868.7500000000018</v>
+      </c>
+      <c r="I18" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="24"/>
+    </row>
+    <row r="19" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="17">
+        <v>17</v>
+      </c>
+      <c r="C19" s="17"/>
+      <c r="D19" s="19" t="s">
+        <v>839</v>
+      </c>
+      <c r="E19" s="18">
+        <v>1</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G19" s="25">
+        <v>67000</v>
+      </c>
+      <c r="H19" s="25">
+        <f>G19*E19</f>
+        <v>67000</v>
+      </c>
+      <c r="I19" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="24"/>
+    </row>
+    <row r="20" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="17">
+        <v>18</v>
+      </c>
+      <c r="C20" s="18"/>
+      <c r="D20" s="19" t="s">
+        <v>884</v>
+      </c>
+      <c r="E20" s="18">
+        <v>1</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G20" s="25">
+        <v>48600</v>
+      </c>
+      <c r="H20" s="51">
+        <f>G20*E20</f>
+        <v>48600</v>
+      </c>
+      <c r="I20" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="24"/>
+    </row>
+    <row r="21" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="17">
+        <v>19</v>
+      </c>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19" t="s">
+        <v>918</v>
+      </c>
+      <c r="E21" s="18">
+        <v>1</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G21" s="25">
+        <v>48600</v>
+      </c>
+      <c r="H21" s="51">
+        <f>G21*E21</f>
+        <v>48600</v>
+      </c>
+      <c r="I21" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="24"/>
+    </row>
+    <row r="22" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="17">
+        <v>20</v>
+      </c>
+      <c r="C22" s="18"/>
+      <c r="D22" s="19" t="s">
+        <v>885</v>
+      </c>
+      <c r="E22" s="18">
+        <v>50</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G22" s="25">
+        <v>243.39</v>
+      </c>
+      <c r="H22" s="51">
+        <f>G22*E22</f>
+        <v>12169.5</v>
+      </c>
+      <c r="I22" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
+      <c r="L22" s="24"/>
+    </row>
+    <row r="23" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="17">
+        <v>21</v>
+      </c>
+      <c r="C23" s="18"/>
+      <c r="D23" s="19" t="s">
+        <v>880</v>
+      </c>
+      <c r="E23" s="18">
+        <f>44*4</f>
+        <v>176</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G23" s="25">
+        <v>38.119999999999997</v>
+      </c>
+      <c r="H23" s="51">
+        <f>G23*E23</f>
+        <v>6709.12</v>
+      </c>
+      <c r="I23" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="24"/>
+    </row>
+    <row r="24" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="17">
+        <v>22</v>
+      </c>
+      <c r="C24" s="18"/>
+      <c r="D24" s="19" t="s">
+        <v>824</v>
+      </c>
+      <c r="E24" s="18">
+        <v>10</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G24" s="25">
+        <v>24</v>
+      </c>
+      <c r="H24" s="51">
+        <f>G24*E24</f>
+        <v>240</v>
+      </c>
+      <c r="I24" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="24" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="17">
+        <v>23</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>877</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>876</v>
+      </c>
+      <c r="E25" s="18">
+        <v>36</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G25" s="25">
+        <v>243.39</v>
+      </c>
+      <c r="H25" s="51">
+        <f>G25*E25</f>
+        <v>8762.0399999999991</v>
+      </c>
+      <c r="I25" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
+      <c r="L25" s="24"/>
+    </row>
+    <row r="26" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="17">
+        <v>24</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>877</v>
+      </c>
+      <c r="D26" s="19" t="s">
+        <v>856</v>
+      </c>
+      <c r="E26" s="18">
+        <v>72</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G26" s="25">
+        <v>38.119999999999997</v>
+      </c>
+      <c r="H26" s="51">
+        <f>G26*E26</f>
+        <v>2744.64</v>
+      </c>
+      <c r="I26" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J26" s="27"/>
+      <c r="K26" s="27"/>
+      <c r="L26" s="24"/>
+    </row>
+    <row r="27" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="17">
+        <v>25</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>877</v>
+      </c>
+      <c r="D27" s="19" t="s">
+        <v>778</v>
+      </c>
+      <c r="E27" s="18">
+        <v>36</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G27" s="25">
+        <v>32</v>
+      </c>
+      <c r="H27" s="51">
+        <f>G27*E27</f>
+        <v>1152</v>
+      </c>
+      <c r="I27" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
+      <c r="L27" s="24"/>
+    </row>
+    <row r="28" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="17">
+        <v>26</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>877</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>871</v>
+      </c>
+      <c r="E28" s="18">
+        <v>4</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G28" s="25">
+        <v>419</v>
+      </c>
+      <c r="H28" s="51">
+        <f>G28*E28</f>
+        <v>1676</v>
+      </c>
+      <c r="I28" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J28" s="27"/>
+      <c r="K28" s="27"/>
+      <c r="L28" s="24"/>
+    </row>
+    <row r="29" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="17">
+        <v>27</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>877</v>
+      </c>
+      <c r="D29" s="19" t="s">
+        <v>857</v>
+      </c>
+      <c r="E29" s="18">
+        <f>8*6</f>
+        <v>48</v>
+      </c>
+      <c r="F29" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G29" s="25">
+        <v>38.119999999999997</v>
+      </c>
+      <c r="H29" s="51">
+        <f>G29*E29</f>
+        <v>1829.7599999999998</v>
+      </c>
+      <c r="I29" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="24"/>
+    </row>
+    <row r="30" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="17">
+        <v>28</v>
+      </c>
+      <c r="C30" s="17"/>
+      <c r="D30" s="19" t="s">
+        <v>917</v>
+      </c>
+      <c r="E30" s="18">
+        <v>2</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G30" s="25">
+        <v>65000</v>
+      </c>
+      <c r="H30" s="25">
+        <f>G30*E30</f>
+        <v>130000</v>
+      </c>
+      <c r="I30" s="18" t="s">
+        <v>835</v>
+      </c>
+      <c r="J30" s="27"/>
+      <c r="K30" s="27"/>
+      <c r="L30" s="24"/>
+    </row>
+    <row r="31" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="17">
+        <v>29</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>878</v>
+      </c>
+      <c r="D31" s="50" t="s">
+        <v>861</v>
+      </c>
+      <c r="E31" s="17">
+        <v>58</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>881</v>
+      </c>
+      <c r="G31" s="44">
+        <v>198.72</v>
+      </c>
+      <c r="H31" s="44">
+        <f>G31*E31</f>
+        <v>11525.76</v>
+      </c>
+      <c r="I31" s="17" t="s">
+        <v>868</v>
+      </c>
+      <c r="J31" s="27"/>
+      <c r="K31" s="27"/>
+      <c r="L31" s="24"/>
+    </row>
+    <row r="32" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="17">
+        <v>30</v>
+      </c>
+      <c r="C32" s="17" t="s">
+        <v>879</v>
+      </c>
+      <c r="D32" s="50" t="s">
+        <v>864</v>
+      </c>
+      <c r="E32" s="17">
+        <v>31</v>
+      </c>
+      <c r="F32" s="17" t="s">
+        <v>881</v>
+      </c>
+      <c r="G32" s="44">
+        <v>484.24</v>
+      </c>
+      <c r="H32" s="44">
+        <f>G32*E32</f>
+        <v>15011.44</v>
+      </c>
+      <c r="I32" s="17" t="s">
+        <v>868</v>
+      </c>
+      <c r="J32" s="27"/>
+      <c r="K32" s="27"/>
+      <c r="L32" s="24"/>
+    </row>
+    <row r="33" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="17">
+        <v>31</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>879</v>
+      </c>
+      <c r="D33" s="50" t="s">
+        <v>867</v>
+      </c>
+      <c r="E33" s="17">
+        <v>28</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G33" s="44">
+        <v>703.93</v>
+      </c>
+      <c r="H33" s="44">
+        <f>G33*E33</f>
+        <v>19710.039999999997</v>
+      </c>
+      <c r="I33" s="17" t="s">
+        <v>868</v>
+      </c>
+      <c r="J33" s="27"/>
+      <c r="K33" s="27"/>
+      <c r="L33" s="24"/>
+    </row>
+    <row r="34" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="17">
+        <v>32</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>878</v>
+      </c>
+      <c r="D34" s="50" t="s">
+        <v>862</v>
+      </c>
+      <c r="E34" s="17">
+        <f>28*3</f>
+        <v>84</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G34" s="44">
+        <v>49.05</v>
+      </c>
+      <c r="H34" s="44">
+        <f>G34*E34</f>
+        <v>4120.2</v>
+      </c>
+      <c r="I34" s="17" t="s">
+        <v>868</v>
+      </c>
+      <c r="J34" s="27"/>
+      <c r="K34" s="27"/>
+      <c r="L34" s="24"/>
+    </row>
+    <row r="35" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="17">
+        <v>33</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>879</v>
+      </c>
+      <c r="D35" s="50" t="s">
+        <v>865</v>
+      </c>
+      <c r="E35" s="17">
+        <v>3</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G35" s="44">
+        <v>151.19999999999999</v>
+      </c>
+      <c r="H35" s="44">
+        <f>G35*E35</f>
+        <v>453.59999999999997</v>
+      </c>
+      <c r="I35" s="17" t="s">
+        <v>868</v>
+      </c>
+      <c r="J35" s="27"/>
+      <c r="K35" s="27"/>
+      <c r="L35" s="24"/>
+    </row>
+    <row r="36" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="17">
+        <v>34</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>879</v>
+      </c>
+      <c r="D36" s="50" t="s">
+        <v>866</v>
+      </c>
+      <c r="E36" s="17">
+        <v>2</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G36" s="44">
+        <v>48.38</v>
+      </c>
+      <c r="H36" s="44">
+        <f>G36*E36</f>
+        <v>96.76</v>
+      </c>
+      <c r="I36" s="17" t="s">
+        <v>868</v>
+      </c>
+      <c r="J36" s="27"/>
+      <c r="K36" s="27"/>
+      <c r="L36" s="24"/>
+    </row>
+    <row r="37" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="17">
+        <v>35</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>878</v>
+      </c>
+      <c r="D37" s="50" t="s">
+        <v>863</v>
+      </c>
+      <c r="E37" s="17">
+        <v>30</v>
+      </c>
+      <c r="F37" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G37" s="44">
+        <v>27.14</v>
+      </c>
+      <c r="H37" s="44">
+        <f>G37*E37</f>
+        <v>814.2</v>
+      </c>
+      <c r="I37" s="17" t="s">
+        <v>868</v>
+      </c>
+      <c r="J37" s="27"/>
+      <c r="K37" s="27"/>
+      <c r="L37" s="24"/>
+    </row>
+    <row r="38" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="17">
+        <v>36</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>882</v>
+      </c>
+      <c r="D38" s="50" t="s">
+        <v>869</v>
+      </c>
+      <c r="E38" s="17">
+        <v>12</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>881</v>
+      </c>
+      <c r="G38" s="44">
+        <v>703.93</v>
+      </c>
+      <c r="H38" s="44">
+        <f>G38*E38</f>
+        <v>8447.16</v>
+      </c>
+      <c r="I38" s="17" t="s">
+        <v>868</v>
+      </c>
+      <c r="J38" s="27"/>
+      <c r="K38" s="27"/>
+      <c r="L38" s="24"/>
+    </row>
+    <row r="39" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="17">
+        <v>37</v>
+      </c>
+      <c r="C39" s="17" t="s">
+        <v>882</v>
+      </c>
+      <c r="D39" s="50" t="s">
+        <v>870</v>
+      </c>
+      <c r="E39" s="17">
+        <f>78/6</f>
+        <v>13</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>881</v>
+      </c>
+      <c r="G39" s="44">
+        <v>484.24</v>
+      </c>
+      <c r="H39" s="44">
+        <f>G39*E39</f>
+        <v>6295.12</v>
+      </c>
+      <c r="I39" s="17" t="s">
+        <v>868</v>
+      </c>
+      <c r="J39" s="27"/>
+      <c r="K39" s="27"/>
+      <c r="L39" s="24"/>
+    </row>
+    <row r="40" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="17">
+        <v>38</v>
+      </c>
+      <c r="C40" s="18"/>
+      <c r="D40" s="19" t="s">
+        <v>883</v>
+      </c>
+      <c r="E40" s="18">
+        <v>1</v>
+      </c>
+      <c r="F40" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G40" s="25">
+        <v>37375</v>
+      </c>
+      <c r="H40" s="51">
+        <f>G40*E40</f>
+        <v>37375</v>
+      </c>
+      <c r="I40" s="18" t="s">
+        <v>868</v>
+      </c>
+      <c r="J40" s="27"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="24"/>
+    </row>
+    <row r="41" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="17">
+        <v>39</v>
+      </c>
+      <c r="C41" s="17"/>
+      <c r="D41" s="50" t="s">
+        <v>805</v>
+      </c>
+      <c r="E41" s="17">
+        <f>54*2</f>
+        <v>108</v>
+      </c>
+      <c r="F41" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G41" s="44">
+        <v>243.39</v>
+      </c>
+      <c r="H41" s="44">
+        <f>G41*E41</f>
+        <v>26286.12</v>
+      </c>
+      <c r="I41" s="17" t="s">
+        <v>806</v>
+      </c>
+      <c r="J41" s="27"/>
+      <c r="K41" s="27"/>
+    </row>
+    <row r="42" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="17">
+        <v>40</v>
+      </c>
+      <c r="C42" s="17"/>
+      <c r="D42" s="50" t="s">
+        <v>807</v>
+      </c>
+      <c r="E42" s="17">
+        <v>30</v>
+      </c>
+      <c r="F42" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G42" s="44">
+        <v>119.7</v>
+      </c>
+      <c r="H42" s="44">
+        <f>G42*E42</f>
+        <v>3591</v>
+      </c>
+      <c r="I42" s="17" t="s">
+        <v>806</v>
+      </c>
+      <c r="J42" s="27"/>
+      <c r="K42" s="27"/>
+      <c r="L42" s="24"/>
+    </row>
+    <row r="43" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="17">
+        <v>41</v>
+      </c>
+      <c r="C43" s="17"/>
+      <c r="D43" s="50" t="s">
+        <v>804</v>
+      </c>
+      <c r="E43" s="18">
+        <v>390</v>
+      </c>
+      <c r="F43" s="17" t="s">
+        <v>761</v>
+      </c>
+      <c r="G43" s="44">
+        <v>38.116666600000002</v>
+      </c>
+      <c r="H43" s="44">
+        <f>G43*E43</f>
+        <v>14865.499974</v>
+      </c>
+      <c r="I43" s="17" t="s">
+        <v>806</v>
+      </c>
+      <c r="J43" s="27"/>
+      <c r="K43" s="27"/>
+      <c r="L43" s="24"/>
+    </row>
+    <row r="44" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="17">
+        <v>42</v>
+      </c>
+      <c r="C44" s="17"/>
+      <c r="D44" s="50" t="s">
+        <v>805</v>
+      </c>
+      <c r="E44" s="53">
+        <f>(84*1.02)*2*1.02</f>
+        <v>174.78720000000001</v>
+      </c>
+      <c r="F44" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G44" s="44">
+        <v>243.39</v>
+      </c>
+      <c r="H44" s="44">
+        <f>G44*E44</f>
+        <v>42541.456608</v>
+      </c>
+      <c r="I44" s="17" t="s">
+        <v>774</v>
+      </c>
+      <c r="J44" s="27"/>
+      <c r="K44" s="27"/>
+    </row>
+    <row r="45" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="17">
+        <v>43</v>
+      </c>
+      <c r="C45" s="17"/>
+      <c r="D45" s="50" t="s">
+        <v>804</v>
+      </c>
+      <c r="E45" s="17">
+        <f>84*7</f>
+        <v>588</v>
+      </c>
+      <c r="F45" s="17" t="s">
+        <v>761</v>
+      </c>
+      <c r="G45" s="44">
+        <v>38.116666600000002</v>
+      </c>
+      <c r="H45" s="44">
+        <f>G45*E45</f>
+        <v>22412.599960800002</v>
+      </c>
+      <c r="I45" s="17" t="s">
+        <v>774</v>
+      </c>
+      <c r="J45" s="27"/>
+      <c r="K45" s="27"/>
+      <c r="L45" s="24"/>
+    </row>
+    <row r="46" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="17">
+        <v>44</v>
+      </c>
+      <c r="C46" s="17"/>
+      <c r="D46" s="50" t="s">
+        <v>824</v>
+      </c>
+      <c r="E46" s="17">
+        <v>30</v>
+      </c>
+      <c r="F46" s="17" t="s">
+        <v>818</v>
+      </c>
+      <c r="G46" s="44">
+        <v>24</v>
+      </c>
+      <c r="H46" s="44">
+        <f>G46*E46</f>
+        <v>720</v>
+      </c>
+      <c r="I46" s="17" t="s">
+        <v>774</v>
+      </c>
+      <c r="J46" s="27"/>
+      <c r="K46" s="27"/>
+      <c r="L46" s="24"/>
+    </row>
+    <row r="47" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="17">
+        <v>45</v>
+      </c>
+      <c r="C47" s="17"/>
+      <c r="D47" s="50" t="s">
+        <v>825</v>
+      </c>
+      <c r="E47" s="17">
+        <v>1</v>
+      </c>
+      <c r="F47" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G47" s="44">
+        <v>860</v>
+      </c>
+      <c r="H47" s="44">
+        <f>G47*E47</f>
+        <v>860</v>
+      </c>
+      <c r="I47" s="17" t="s">
+        <v>774</v>
+      </c>
+      <c r="J47" s="27"/>
+      <c r="K47" s="27"/>
+      <c r="L47" s="24"/>
+    </row>
+    <row r="48" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="17">
+        <v>46</v>
+      </c>
+      <c r="C48" s="17"/>
+      <c r="D48" s="19" t="s">
+        <v>873</v>
+      </c>
+      <c r="E48" s="18">
+        <v>140</v>
+      </c>
+      <c r="F48" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G48" s="25">
+        <v>23.90625</v>
+      </c>
+      <c r="H48" s="25">
+        <f>G48*E48</f>
+        <v>3346.875</v>
+      </c>
+      <c r="I48" s="18" t="s">
+        <v>774</v>
+      </c>
+      <c r="J48" s="27"/>
+      <c r="K48" s="27"/>
+      <c r="L48" s="24"/>
+    </row>
+    <row r="49" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="17">
+        <v>47</v>
+      </c>
+      <c r="C49" s="17"/>
+      <c r="D49" s="19" t="s">
+        <v>778</v>
+      </c>
+      <c r="E49" s="18">
+        <v>66</v>
+      </c>
+      <c r="F49" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G49" s="25">
+        <v>26</v>
+      </c>
+      <c r="H49" s="25">
+        <f>G49*E49</f>
+        <v>1716</v>
+      </c>
+      <c r="I49" s="18" t="s">
+        <v>774</v>
+      </c>
+      <c r="J49" s="27"/>
+      <c r="K49" s="27"/>
+      <c r="L49" s="24"/>
+    </row>
+    <row r="50" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="17">
+        <v>48</v>
+      </c>
+      <c r="C50" s="17"/>
+      <c r="D50" s="19" t="s">
+        <v>800</v>
+      </c>
+      <c r="E50" s="18">
+        <v>1</v>
+      </c>
+      <c r="F50" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G50" s="25">
+        <f>7500+7000+6500+10000</f>
+        <v>31000</v>
+      </c>
+      <c r="H50" s="25">
+        <f>G50*E50</f>
+        <v>31000</v>
+      </c>
+      <c r="I50" s="18" t="s">
+        <v>774</v>
+      </c>
+      <c r="J50" s="27"/>
+      <c r="K50" s="27"/>
+      <c r="L50" s="24"/>
+    </row>
+    <row r="51" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="17">
+        <v>49</v>
+      </c>
+      <c r="C51" s="17"/>
+      <c r="D51" s="50" t="s">
+        <v>788</v>
+      </c>
+      <c r="E51" s="17">
+        <v>1</v>
+      </c>
+      <c r="F51" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G51" s="54">
+        <v>6000</v>
+      </c>
+      <c r="H51" s="54">
+        <f>G51*E51</f>
+        <v>6000</v>
+      </c>
+      <c r="I51" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="J51" s="27"/>
+      <c r="K51" s="27"/>
+      <c r="L51" s="24"/>
+    </row>
+    <row r="52" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="17">
+        <v>50</v>
+      </c>
+      <c r="C52" s="17"/>
+      <c r="D52" s="50" t="s">
+        <v>769</v>
+      </c>
+      <c r="E52" s="17">
+        <v>4100</v>
+      </c>
+      <c r="F52" s="17" t="s">
+        <v>811</v>
+      </c>
+      <c r="G52" s="54">
+        <v>9.65</v>
+      </c>
+      <c r="H52" s="54">
+        <f>G52*E52</f>
+        <v>39565</v>
+      </c>
+      <c r="I52" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="J52" s="27"/>
+      <c r="K52" s="27"/>
+      <c r="L52" s="24"/>
+    </row>
+    <row r="53" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="17">
+        <v>51</v>
+      </c>
+      <c r="C53" s="17"/>
+      <c r="D53" s="50" t="s">
+        <v>770</v>
+      </c>
+      <c r="E53" s="17">
+        <v>4000</v>
+      </c>
+      <c r="F53" s="17" t="s">
+        <v>811</v>
+      </c>
+      <c r="G53" s="54">
+        <v>9.65</v>
+      </c>
+      <c r="H53" s="54">
+        <f>G53*E53</f>
+        <v>38600</v>
+      </c>
+      <c r="I53" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="J53" s="27"/>
+      <c r="K53" s="27"/>
+      <c r="L53" s="14" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="54" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="17">
+        <v>52</v>
+      </c>
+      <c r="C54" s="17"/>
+      <c r="D54" s="50" t="s">
+        <v>803</v>
+      </c>
+      <c r="E54" s="17">
+        <v>1</v>
+      </c>
+      <c r="F54" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G54" s="54">
+        <v>164000</v>
+      </c>
+      <c r="H54" s="54">
+        <f>G54*E54</f>
+        <v>164000</v>
+      </c>
+      <c r="I54" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="J54" s="27"/>
+      <c r="K54" s="27"/>
+      <c r="L54" s="14" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="55" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="17">
+        <v>53</v>
+      </c>
+      <c r="C55" s="17"/>
+      <c r="D55" s="50" t="s">
+        <v>830</v>
+      </c>
+      <c r="E55" s="53">
+        <v>99.22</v>
+      </c>
+      <c r="F55" s="17" t="s">
+        <v>759</v>
+      </c>
+      <c r="G55" s="54">
+        <v>670</v>
+      </c>
+      <c r="H55" s="54">
+        <f>G55*E55</f>
+        <v>66477.399999999994</v>
+      </c>
+      <c r="I55" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="J55" s="27"/>
+      <c r="K55" s="27"/>
+      <c r="L55" s="24"/>
+    </row>
+    <row r="56" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="17">
+        <v>54</v>
+      </c>
+      <c r="C56" s="17"/>
+      <c r="D56" s="50" t="s">
+        <v>829</v>
+      </c>
+      <c r="E56" s="17">
+        <v>68</v>
+      </c>
+      <c r="F56" s="17" t="s">
+        <v>759</v>
+      </c>
+      <c r="G56" s="54">
+        <v>670</v>
+      </c>
+      <c r="H56" s="54">
+        <f>G56*E56</f>
+        <v>45560</v>
+      </c>
+      <c r="I56" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="J56" s="27"/>
+      <c r="K56" s="27"/>
+      <c r="L56" s="24"/>
+    </row>
+    <row r="57" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="17">
+        <v>55</v>
+      </c>
+      <c r="C57" s="17"/>
+      <c r="D57" s="50" t="s">
+        <v>808</v>
+      </c>
+      <c r="E57" s="17">
+        <v>1</v>
+      </c>
+      <c r="F57" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G57" s="54">
+        <v>56500</v>
+      </c>
+      <c r="H57" s="54">
+        <f>G57*E57</f>
+        <v>56500</v>
+      </c>
+      <c r="I57" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="J57" s="27"/>
+      <c r="K57" s="27"/>
+      <c r="L57" s="24"/>
+    </row>
+    <row r="58" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="17">
+        <v>56</v>
+      </c>
+      <c r="C58" s="17"/>
+      <c r="D58" s="50" t="s">
+        <v>777</v>
+      </c>
+      <c r="E58" s="17">
+        <v>50</v>
+      </c>
+      <c r="F58" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G58" s="44">
+        <v>125</v>
+      </c>
+      <c r="H58" s="44">
+        <f>G58*E58</f>
+        <v>6250</v>
+      </c>
+      <c r="I58" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="J58" s="27"/>
+      <c r="K58" s="27"/>
+      <c r="L58" s="24"/>
+    </row>
+    <row r="59" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B59" s="17">
+        <v>57</v>
+      </c>
+      <c r="C59" s="17"/>
+      <c r="D59" s="50" t="s">
+        <v>842</v>
+      </c>
+      <c r="E59" s="17">
+        <v>4</v>
+      </c>
+      <c r="F59" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G59" s="44">
+        <v>1500</v>
+      </c>
+      <c r="H59" s="44">
+        <f>G59*E59</f>
+        <v>6000</v>
+      </c>
+      <c r="I59" s="17" t="s">
+        <v>771</v>
+      </c>
+      <c r="J59" s="27"/>
+      <c r="K59" s="27"/>
+      <c r="L59" s="24"/>
+    </row>
+    <row r="60" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B60" s="17">
+        <v>58</v>
+      </c>
+      <c r="C60" s="17"/>
+      <c r="D60" s="19" t="s">
+        <v>850</v>
+      </c>
+      <c r="E60" s="18">
+        <v>26</v>
+      </c>
+      <c r="F60" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G60" s="25">
+        <v>420</v>
+      </c>
+      <c r="H60" s="25">
+        <f>G60*E60</f>
+        <v>10920</v>
+      </c>
+      <c r="I60" s="17" t="s">
+        <v>901</v>
+      </c>
+      <c r="J60" s="27"/>
+      <c r="K60" s="27"/>
+      <c r="L60" s="24" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="61" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="17">
+        <v>59</v>
+      </c>
+      <c r="C61" s="17"/>
+      <c r="D61" s="50" t="s">
+        <v>898</v>
+      </c>
+      <c r="E61" s="18">
+        <v>400</v>
+      </c>
+      <c r="F61" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G61" s="25">
+        <v>15</v>
+      </c>
+      <c r="H61" s="25">
+        <f>G61*E61</f>
+        <v>6000</v>
+      </c>
+      <c r="I61" s="17" t="s">
+        <v>901</v>
+      </c>
+      <c r="J61" s="27"/>
+      <c r="K61" s="27"/>
+      <c r="L61" s="24"/>
+    </row>
+    <row r="62" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="17">
+        <v>60</v>
+      </c>
+      <c r="C62" s="17"/>
+      <c r="D62" s="19" t="s">
+        <v>851</v>
+      </c>
+      <c r="E62" s="18">
+        <v>1</v>
+      </c>
+      <c r="F62" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G62" s="25">
+        <f>119439/2</f>
+        <v>59719.5</v>
+      </c>
+      <c r="H62" s="25">
+        <f>G62*E62</f>
+        <v>59719.5</v>
+      </c>
+      <c r="I62" s="17" t="s">
+        <v>901</v>
+      </c>
+      <c r="J62" s="27"/>
+      <c r="K62" s="27"/>
+      <c r="L62" s="24"/>
+    </row>
+    <row r="63" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B63" s="17">
+        <v>61</v>
+      </c>
+      <c r="C63" s="17"/>
+      <c r="D63" s="19" t="s">
+        <v>783</v>
+      </c>
+      <c r="E63" s="18">
+        <v>8</v>
+      </c>
+      <c r="F63" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G63" s="25">
+        <v>380</v>
+      </c>
+      <c r="H63" s="25">
+        <f>G63*E63</f>
+        <v>3040</v>
+      </c>
+      <c r="I63" s="18" t="s">
+        <v>576</v>
+      </c>
+      <c r="J63" s="27"/>
+      <c r="K63" s="27"/>
+      <c r="L63" s="24"/>
+    </row>
+    <row r="64" spans="2:12" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B64" s="17">
+        <v>62</v>
+      </c>
+      <c r="C64" s="17"/>
+      <c r="D64" s="19" t="s">
+        <v>784</v>
+      </c>
+      <c r="E64" s="18">
+        <v>4</v>
+      </c>
+      <c r="F64" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G64" s="25">
+        <v>290</v>
+      </c>
+      <c r="H64" s="25">
+        <f>G64*E64</f>
+        <v>1160</v>
+      </c>
+      <c r="I64" s="18" t="s">
+        <v>576</v>
+      </c>
+      <c r="J64" s="27"/>
+      <c r="K64" s="27"/>
+      <c r="L64" s="24"/>
+    </row>
+    <row r="65" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="17">
+        <v>63</v>
+      </c>
+      <c r="C65" s="17"/>
+      <c r="D65" s="19" t="s">
+        <v>785</v>
+      </c>
+      <c r="E65" s="18">
+        <v>4</v>
+      </c>
+      <c r="F65" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G65" s="25">
+        <v>290</v>
+      </c>
+      <c r="H65" s="25">
+        <f>G65*E65</f>
+        <v>1160</v>
+      </c>
+      <c r="I65" s="18" t="s">
+        <v>576</v>
+      </c>
+      <c r="J65" s="27"/>
+      <c r="K65" s="27"/>
+      <c r="L65" s="24"/>
+    </row>
+    <row r="66" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="17">
+        <v>64</v>
+      </c>
+      <c r="C66" s="17"/>
+      <c r="D66" s="50" t="s">
+        <v>757</v>
+      </c>
+      <c r="E66" s="53">
+        <f>(2150*1.05)*0.15</f>
+        <v>338.625</v>
+      </c>
+      <c r="F66" s="17" t="s">
+        <v>759</v>
+      </c>
+      <c r="G66" s="54">
+        <v>670</v>
+      </c>
+      <c r="H66" s="54">
+        <f>G66*E66</f>
+        <v>226878.75</v>
+      </c>
+      <c r="I66" s="17" t="s">
+        <v>833</v>
+      </c>
+      <c r="J66" s="27"/>
+      <c r="K66" s="27"/>
+      <c r="M66" s="14"/>
+      <c r="N66" s="14"/>
+      <c r="O66" s="14"/>
+    </row>
+    <row r="67" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B67" s="17">
+        <v>65</v>
+      </c>
+      <c r="C67" s="17"/>
+      <c r="D67" s="50" t="s">
+        <v>775</v>
+      </c>
+      <c r="E67" s="53">
+        <f>(2150/13)*2</f>
+        <v>330.76923076923077</v>
+      </c>
+      <c r="F67" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G67" s="54">
+        <v>220.5</v>
+      </c>
+      <c r="H67" s="54">
+        <f>G67*E67</f>
+        <v>72934.61538461539</v>
+      </c>
+      <c r="I67" s="17" t="s">
+        <v>833</v>
+      </c>
+      <c r="J67" s="27"/>
+      <c r="K67" s="27"/>
+      <c r="M67" s="14"/>
+      <c r="N67" s="14"/>
+      <c r="O67" s="14"/>
+    </row>
+    <row r="68" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B68" s="17">
+        <v>66</v>
+      </c>
+      <c r="C68" s="17"/>
+      <c r="D68" s="50" t="s">
+        <v>758</v>
+      </c>
+      <c r="E68" s="17">
+        <f>2100/12</f>
+        <v>175</v>
+      </c>
+      <c r="F68" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G68" s="54">
+        <v>56.2</v>
+      </c>
+      <c r="H68" s="54">
+        <f>G68*E68</f>
+        <v>9835</v>
+      </c>
+      <c r="I68" s="17" t="s">
+        <v>833</v>
+      </c>
+      <c r="J68" s="27"/>
+      <c r="K68" s="27"/>
+      <c r="M68" s="14"/>
+      <c r="N68" s="14"/>
+      <c r="O68" s="14"/>
+    </row>
+    <row r="69" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B69" s="17">
+        <v>67</v>
+      </c>
+      <c r="C69" s="17"/>
+      <c r="D69" s="50" t="s">
+        <v>762</v>
+      </c>
+      <c r="E69" s="17">
+        <v>1000</v>
+      </c>
+      <c r="F69" s="17" t="s">
+        <v>763</v>
+      </c>
+      <c r="G69" s="54">
+        <v>7.3</v>
+      </c>
+      <c r="H69" s="54">
+        <f>G69*E69</f>
+        <v>7300</v>
+      </c>
+      <c r="I69" s="17" t="s">
+        <v>833</v>
+      </c>
+      <c r="J69" s="27"/>
+      <c r="K69" s="27"/>
+      <c r="M69" s="14"/>
+      <c r="N69" s="14"/>
+      <c r="O69" s="14"/>
+    </row>
+    <row r="70" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B70" s="17">
+        <v>68</v>
+      </c>
+      <c r="C70" s="17"/>
+      <c r="D70" s="50" t="s">
+        <v>792</v>
+      </c>
+      <c r="E70" s="53">
+        <f>E66</f>
+        <v>338.625</v>
+      </c>
+      <c r="F70" s="17" t="s">
+        <v>766</v>
+      </c>
+      <c r="G70" s="54">
+        <v>50</v>
+      </c>
+      <c r="H70" s="54">
+        <f>G70*E70</f>
+        <v>16931.25</v>
+      </c>
+      <c r="I70" s="17" t="s">
+        <v>833</v>
+      </c>
+      <c r="J70" s="27"/>
+      <c r="K70" s="27"/>
+      <c r="M70" s="14"/>
+      <c r="N70" s="14"/>
+      <c r="O70" s="14"/>
+    </row>
+    <row r="71" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B71" s="17">
+        <v>69</v>
+      </c>
+      <c r="C71" s="17"/>
+      <c r="D71" s="50" t="s">
+        <v>826</v>
+      </c>
+      <c r="E71" s="17">
+        <v>1</v>
+      </c>
+      <c r="F71" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G71" s="54">
+        <v>53550</v>
+      </c>
+      <c r="H71" s="54">
+        <f>G71*E71</f>
+        <v>53550</v>
+      </c>
+      <c r="I71" s="17" t="s">
+        <v>833</v>
+      </c>
+      <c r="J71" s="27"/>
+      <c r="K71" s="27"/>
+      <c r="M71" s="14"/>
+      <c r="N71" s="14"/>
+      <c r="O71" s="14"/>
+    </row>
+    <row r="72" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B72" s="17">
+        <v>70</v>
+      </c>
+      <c r="C72" s="18"/>
+      <c r="D72" s="19" t="s">
+        <v>799</v>
+      </c>
+      <c r="E72" s="18">
+        <v>110</v>
+      </c>
+      <c r="F72" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G72" s="25">
+        <v>42.29</v>
+      </c>
+      <c r="H72" s="25">
+        <f>G72*E72</f>
+        <v>4651.8999999999996</v>
+      </c>
+      <c r="I72" s="18" t="s">
+        <v>831</v>
+      </c>
+      <c r="J72" s="27"/>
+      <c r="K72" s="27"/>
+      <c r="M72" s="14"/>
+      <c r="N72" s="14"/>
+      <c r="O72" s="14"/>
+    </row>
+    <row r="73" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B73" s="17">
+        <v>71</v>
+      </c>
+      <c r="C73" s="18"/>
+      <c r="D73" s="19" t="s">
+        <v>832</v>
+      </c>
+      <c r="E73" s="18">
+        <v>1</v>
+      </c>
+      <c r="F73" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G73" s="25">
+        <v>1400</v>
+      </c>
+      <c r="H73" s="25">
+        <f>G73*E73</f>
+        <v>1400</v>
+      </c>
+      <c r="I73" s="18" t="s">
+        <v>831</v>
+      </c>
+      <c r="J73" s="27"/>
+      <c r="K73" s="27"/>
+      <c r="M73" s="14"/>
+      <c r="N73" s="14"/>
+      <c r="O73" s="14"/>
+    </row>
+    <row r="74" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B74" s="17">
+        <v>72</v>
+      </c>
+      <c r="C74" s="18"/>
+      <c r="D74" s="19" t="s">
+        <v>757</v>
+      </c>
+      <c r="E74" s="52">
+        <f>((1260+960)*0.15)*1.1</f>
+        <v>366.3</v>
+      </c>
+      <c r="F74" s="18" t="s">
+        <v>759</v>
+      </c>
+      <c r="G74" s="25">
+        <v>670</v>
+      </c>
+      <c r="H74" s="25">
+        <f>G74*E74</f>
+        <v>245421</v>
+      </c>
+      <c r="I74" s="18" t="s">
+        <v>831</v>
+      </c>
+      <c r="J74" s="27"/>
+      <c r="K74" s="27"/>
+      <c r="M74" s="14"/>
+      <c r="N74" s="14"/>
+      <c r="O74" s="14"/>
+    </row>
+    <row r="75" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B75" s="17">
+        <v>73</v>
+      </c>
+      <c r="C75" s="18"/>
+      <c r="D75" s="50" t="s">
+        <v>775</v>
+      </c>
+      <c r="E75" s="52">
+        <f>(1260+960)/13*1.05</f>
+        <v>179.30769230769232</v>
+      </c>
+      <c r="F75" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G75" s="25">
+        <v>220.5</v>
+      </c>
+      <c r="H75" s="25">
+        <f>G75*E75</f>
+        <v>39537.346153846156</v>
+      </c>
+      <c r="I75" s="18" t="s">
+        <v>831</v>
+      </c>
+      <c r="J75" s="27"/>
+      <c r="K75" s="27"/>
+      <c r="M75" s="14"/>
+      <c r="N75" s="14"/>
+      <c r="O75" s="14"/>
+    </row>
+    <row r="76" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B76" s="17">
+        <v>74</v>
+      </c>
+      <c r="C76" s="18"/>
+      <c r="D76" s="19" t="s">
+        <v>834</v>
+      </c>
+      <c r="E76" s="18">
+        <v>1</v>
+      </c>
+      <c r="F76" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G76" s="25">
+        <v>62525</v>
+      </c>
+      <c r="H76" s="25">
+        <f>G76*E76</f>
+        <v>62525</v>
+      </c>
+      <c r="I76" s="18" t="s">
+        <v>831</v>
+      </c>
+      <c r="J76" s="27"/>
+      <c r="K76" s="27"/>
+      <c r="M76" s="14"/>
+      <c r="N76" s="14"/>
+      <c r="O76" s="14"/>
+    </row>
+    <row r="77" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B77" s="17">
+        <v>75</v>
+      </c>
+      <c r="C77" s="17"/>
+      <c r="D77" s="50" t="s">
+        <v>823</v>
+      </c>
+      <c r="E77" s="17">
+        <v>1</v>
+      </c>
+      <c r="F77" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G77" s="44">
+        <v>24500</v>
+      </c>
+      <c r="H77" s="44">
+        <f>G77*E77</f>
+        <v>24500</v>
+      </c>
+      <c r="I77" s="17" t="s">
+        <v>772</v>
+      </c>
+      <c r="J77" s="27"/>
+      <c r="K77" s="27"/>
+      <c r="M77" s="14"/>
+      <c r="N77" s="14"/>
+      <c r="O77" s="14"/>
+    </row>
+    <row r="78" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B78" s="17">
+        <v>76</v>
+      </c>
+      <c r="C78" s="17"/>
+      <c r="D78" s="50" t="s">
+        <v>773</v>
+      </c>
+      <c r="E78" s="17">
+        <v>1</v>
+      </c>
+      <c r="F78" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G78" s="54">
+        <v>968004</v>
+      </c>
+      <c r="H78" s="54">
+        <f>G78*E78</f>
+        <v>968004</v>
+      </c>
+      <c r="I78" s="17" t="s">
+        <v>772</v>
+      </c>
+      <c r="J78" s="27"/>
+      <c r="K78" s="27"/>
+      <c r="M78" s="14"/>
+      <c r="N78" s="14"/>
+      <c r="O78" s="14"/>
+    </row>
+    <row r="79" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B79" s="17">
+        <v>77</v>
+      </c>
+      <c r="C79" s="18"/>
+      <c r="D79" s="19" t="s">
+        <v>904</v>
+      </c>
+      <c r="E79" s="18">
+        <v>1</v>
+      </c>
+      <c r="F79" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G79" s="25">
+        <v>32000</v>
+      </c>
+      <c r="H79" s="51">
+        <f>G79*E79</f>
+        <v>32000</v>
+      </c>
+      <c r="I79" s="18" t="s">
+        <v>859</v>
+      </c>
+      <c r="J79" s="27"/>
+      <c r="K79" s="27"/>
+      <c r="M79" s="14"/>
+      <c r="N79" s="14"/>
+      <c r="O79" s="14"/>
+    </row>
+    <row r="80" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B80" s="17">
+        <v>78</v>
+      </c>
+      <c r="C80" s="18"/>
+      <c r="D80" s="19" t="s">
+        <v>903</v>
+      </c>
+      <c r="E80" s="18">
+        <v>1</v>
+      </c>
+      <c r="F80" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G80" s="25">
+        <v>10000</v>
+      </c>
+      <c r="H80" s="51">
+        <f>G80*E80</f>
+        <v>10000</v>
+      </c>
+      <c r="I80" s="18" t="s">
+        <v>859</v>
+      </c>
+      <c r="J80" s="27"/>
+      <c r="K80" s="27"/>
+      <c r="M80" s="14"/>
+      <c r="N80" s="14"/>
+      <c r="O80" s="14"/>
+    </row>
+    <row r="81" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B81" s="17">
+        <v>79</v>
+      </c>
+      <c r="C81" s="17"/>
+      <c r="D81" s="19" t="s">
+        <v>793</v>
+      </c>
+      <c r="E81" s="18">
+        <v>1</v>
+      </c>
+      <c r="F81" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G81" s="25">
+        <v>46600</v>
+      </c>
+      <c r="H81" s="25">
+        <f>G81*E81</f>
+        <v>46600</v>
+      </c>
+      <c r="I81" s="18" t="s">
+        <v>837</v>
+      </c>
+      <c r="J81" s="42" t="s">
+        <v>922</v>
+      </c>
+      <c r="K81" s="27"/>
+      <c r="M81" s="14"/>
+      <c r="N81" s="14"/>
+      <c r="O81" s="14"/>
+    </row>
+    <row r="82" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B82" s="17">
+        <v>80</v>
+      </c>
+      <c r="C82" s="17"/>
+      <c r="D82" s="19" t="s">
+        <v>794</v>
+      </c>
+      <c r="E82" s="18">
+        <v>1</v>
+      </c>
+      <c r="F82" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G82" s="25">
+        <v>8100</v>
+      </c>
+      <c r="H82" s="25">
+        <f>G82*E82</f>
+        <v>8100</v>
+      </c>
+      <c r="I82" s="18" t="s">
+        <v>837</v>
+      </c>
+      <c r="J82" s="42" t="s">
+        <v>922</v>
+      </c>
+      <c r="K82" s="27"/>
+      <c r="M82" s="14"/>
+      <c r="N82" s="14"/>
+      <c r="O82" s="14"/>
+    </row>
+    <row r="83" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B83" s="17">
+        <v>81</v>
+      </c>
+      <c r="C83" s="17"/>
+      <c r="D83" s="19" t="s">
+        <v>801</v>
+      </c>
+      <c r="E83" s="18">
+        <v>1</v>
+      </c>
+      <c r="F83" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G83" s="25">
+        <v>5000</v>
+      </c>
+      <c r="H83" s="25">
+        <f>G83*E83</f>
+        <v>5000</v>
+      </c>
+      <c r="I83" s="18" t="s">
+        <v>837</v>
+      </c>
+      <c r="J83" s="42" t="s">
+        <v>922</v>
+      </c>
+      <c r="K83" s="27"/>
+      <c r="M83" s="14"/>
+      <c r="N83" s="14"/>
+      <c r="O83" s="14"/>
+    </row>
+    <row r="84" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B84" s="17">
+        <v>82</v>
+      </c>
+      <c r="C84" s="17"/>
+      <c r="D84" s="19" t="s">
+        <v>872</v>
+      </c>
+      <c r="E84" s="18">
+        <v>1</v>
+      </c>
+      <c r="F84" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G84" s="25">
+        <v>27000</v>
+      </c>
+      <c r="H84" s="25">
+        <f>G84*E84</f>
+        <v>27000</v>
+      </c>
+      <c r="I84" s="18" t="s">
+        <v>837</v>
+      </c>
+      <c r="J84" s="42" t="s">
+        <v>923</v>
+      </c>
+      <c r="K84" s="27"/>
+      <c r="M84" s="14"/>
+      <c r="N84" s="14"/>
+      <c r="O84" s="14"/>
+    </row>
+    <row r="85" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B85" s="17">
+        <v>83</v>
+      </c>
+      <c r="C85" s="17"/>
+      <c r="D85" s="19" t="s">
+        <v>893</v>
+      </c>
+      <c r="E85" s="18">
+        <v>320</v>
+      </c>
+      <c r="F85" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G85" s="25">
+        <v>16</v>
+      </c>
+      <c r="H85" s="25">
+        <f>G85*E85</f>
+        <v>5120</v>
+      </c>
+      <c r="I85" s="18" t="s">
+        <v>837</v>
+      </c>
+      <c r="J85" s="42" t="s">
+        <v>922</v>
+      </c>
+      <c r="K85" s="27"/>
+      <c r="M85" s="14"/>
+      <c r="N85" s="14"/>
+      <c r="O85" s="14"/>
+    </row>
+    <row r="86" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B86" s="17">
+        <v>84</v>
+      </c>
+      <c r="C86" s="17"/>
+      <c r="D86" s="19" t="s">
+        <v>911</v>
+      </c>
+      <c r="E86" s="18">
+        <v>1</v>
+      </c>
+      <c r="F86" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G86" s="25">
+        <v>3400</v>
+      </c>
+      <c r="H86" s="25">
+        <f>G86*E86</f>
+        <v>3400</v>
+      </c>
+      <c r="I86" s="18" t="s">
+        <v>837</v>
+      </c>
+      <c r="J86" s="42" t="s">
+        <v>922</v>
+      </c>
+      <c r="K86" s="27"/>
+      <c r="M86" s="14"/>
+      <c r="N86" s="14"/>
+      <c r="O86" s="14"/>
+    </row>
+    <row r="87" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B87" s="17">
+        <v>85</v>
+      </c>
+      <c r="C87" s="17"/>
+      <c r="D87" s="19" t="s">
+        <v>912</v>
+      </c>
+      <c r="E87" s="18">
+        <v>1</v>
+      </c>
+      <c r="F87" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G87" s="25">
+        <v>8000</v>
+      </c>
+      <c r="H87" s="25">
+        <f>G87*E87</f>
+        <v>8000</v>
+      </c>
+      <c r="I87" s="18" t="s">
+        <v>837</v>
+      </c>
+      <c r="J87" s="42" t="s">
+        <v>922</v>
+      </c>
+      <c r="K87" s="27"/>
+      <c r="M87" s="14"/>
+      <c r="N87" s="14"/>
+      <c r="O87" s="14"/>
+    </row>
+    <row r="88" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B88" s="17">
+        <v>86</v>
+      </c>
+      <c r="C88" s="17"/>
+      <c r="D88" s="19" t="s">
+        <v>916</v>
+      </c>
+      <c r="E88" s="18">
+        <v>1</v>
+      </c>
+      <c r="F88" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G88" s="25">
+        <v>2500</v>
+      </c>
+      <c r="H88" s="25">
+        <f>G88*E88</f>
+        <v>2500</v>
+      </c>
+      <c r="I88" s="18" t="s">
+        <v>837</v>
+      </c>
+      <c r="J88" s="42" t="s">
+        <v>923</v>
+      </c>
+      <c r="K88" s="27"/>
+      <c r="M88" s="14"/>
+      <c r="N88" s="14"/>
+      <c r="O88" s="14"/>
+    </row>
+    <row r="89" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B89" s="17">
+        <v>87</v>
+      </c>
+      <c r="C89" s="17" t="s">
+        <v>900</v>
+      </c>
+      <c r="D89" s="50" t="s">
+        <v>896</v>
+      </c>
+      <c r="E89" s="52">
+        <v>115</v>
+      </c>
+      <c r="F89" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G89" s="25">
+        <v>102</v>
+      </c>
+      <c r="H89" s="25">
+        <f>G89*E89</f>
+        <v>11730</v>
+      </c>
+      <c r="I89" s="17" t="s">
+        <v>837</v>
+      </c>
+      <c r="J89" s="42" t="s">
+        <v>922</v>
+      </c>
+      <c r="K89" s="27"/>
+      <c r="M89" s="14"/>
+      <c r="N89" s="14"/>
+      <c r="O89" s="14"/>
+    </row>
+    <row r="90" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B90" s="17">
+        <v>88</v>
+      </c>
+      <c r="C90" s="17"/>
+      <c r="D90" s="50" t="s">
+        <v>853</v>
+      </c>
+      <c r="E90" s="17">
+        <v>87</v>
+      </c>
+      <c r="F90" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G90" s="44">
+        <v>34.99</v>
+      </c>
+      <c r="H90" s="44">
+        <f>G90*E90</f>
+        <v>3044.13</v>
+      </c>
+      <c r="I90" s="17" t="s">
+        <v>791</v>
+      </c>
+      <c r="J90" s="27"/>
+      <c r="K90" s="27"/>
+      <c r="M90" s="14"/>
+      <c r="N90" s="14"/>
+      <c r="O90" s="14"/>
+    </row>
+    <row r="91" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B91" s="17">
+        <v>89</v>
+      </c>
+      <c r="C91" s="17"/>
+      <c r="D91" s="55" t="s">
+        <v>854</v>
+      </c>
+      <c r="E91" s="17">
+        <v>174</v>
+      </c>
+      <c r="F91" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G91" s="44">
+        <v>255.5</v>
+      </c>
+      <c r="H91" s="44">
+        <f>G91*E91</f>
+        <v>44457</v>
+      </c>
+      <c r="I91" s="17" t="s">
+        <v>791</v>
+      </c>
+      <c r="J91" s="27"/>
+      <c r="K91" s="27"/>
+      <c r="M91" s="14"/>
+      <c r="N91" s="14"/>
+      <c r="O91" s="14"/>
+    </row>
+    <row r="92" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B92" s="17">
+        <v>90</v>
+      </c>
+      <c r="C92" s="17"/>
+      <c r="D92" s="50" t="s">
+        <v>855</v>
+      </c>
+      <c r="E92" s="17">
+        <v>174</v>
+      </c>
+      <c r="F92" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G92" s="44">
+        <v>196</v>
+      </c>
+      <c r="H92" s="44">
+        <f>G92*E92</f>
+        <v>34104</v>
+      </c>
+      <c r="I92" s="17" t="s">
+        <v>791</v>
+      </c>
+      <c r="J92" s="27"/>
+      <c r="K92" s="27"/>
+      <c r="M92" s="14"/>
+      <c r="N92" s="14"/>
+      <c r="O92" s="14"/>
+    </row>
+    <row r="93" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B93" s="17">
+        <v>91</v>
+      </c>
+      <c r="C93" s="17"/>
+      <c r="D93" s="55" t="s">
+        <v>840</v>
+      </c>
+      <c r="E93" s="17">
+        <v>4700</v>
+      </c>
+      <c r="F93" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G93" s="44">
+        <v>0.5</v>
+      </c>
+      <c r="H93" s="44">
+        <f>G93*E93</f>
+        <v>2350</v>
+      </c>
+      <c r="I93" s="17" t="s">
+        <v>791</v>
+      </c>
+      <c r="J93" s="27"/>
+      <c r="K93" s="27"/>
+      <c r="M93" s="14"/>
+      <c r="N93" s="14"/>
+      <c r="O93" s="14"/>
+    </row>
+    <row r="94" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B94" s="17">
+        <v>92</v>
+      </c>
+      <c r="C94" s="17"/>
+      <c r="D94" s="50" t="s">
+        <v>841</v>
+      </c>
+      <c r="E94" s="17">
+        <v>3200</v>
+      </c>
+      <c r="F94" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G94" s="44">
+        <v>0.5</v>
+      </c>
+      <c r="H94" s="44">
+        <f>G94*E94</f>
+        <v>1600</v>
+      </c>
+      <c r="I94" s="17" t="s">
+        <v>791</v>
+      </c>
+      <c r="J94" s="27"/>
+      <c r="K94" s="27"/>
+      <c r="M94" s="14"/>
+      <c r="N94" s="14"/>
+      <c r="O94" s="14"/>
+    </row>
+    <row r="95" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B95" s="17">
+        <v>93</v>
+      </c>
+      <c r="C95" s="17"/>
+      <c r="D95" s="50" t="s">
+        <v>781</v>
+      </c>
+      <c r="E95" s="17">
+        <v>1</v>
+      </c>
+      <c r="F95" s="17" t="s">
+        <v>760</v>
+      </c>
+      <c r="G95" s="44">
+        <v>908615.35</v>
+      </c>
+      <c r="H95" s="44">
+        <f>G95*E95</f>
+        <v>908615.35</v>
+      </c>
+      <c r="I95" s="17" t="s">
+        <v>780</v>
+      </c>
+      <c r="J95" s="27"/>
+      <c r="K95" s="27"/>
+      <c r="M95" s="14"/>
+      <c r="N95" s="14"/>
+      <c r="O95" s="14"/>
+    </row>
+    <row r="96" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B96" s="17">
+        <v>94</v>
+      </c>
+      <c r="C96" s="17" t="s">
+        <v>900</v>
+      </c>
+      <c r="D96" s="19" t="s">
+        <v>894</v>
+      </c>
+      <c r="E96" s="18">
+        <v>750</v>
+      </c>
+      <c r="F96" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G96" s="25">
+        <v>124.25</v>
+      </c>
+      <c r="H96" s="25">
+        <f>G96*E96</f>
+        <v>93187.5</v>
+      </c>
+      <c r="I96" s="18" t="s">
+        <v>836</v>
+      </c>
+      <c r="J96" s="27"/>
+      <c r="K96" s="27"/>
+      <c r="M96" s="14"/>
+      <c r="N96" s="14"/>
+      <c r="O96" s="14"/>
+    </row>
+    <row r="97" spans="2:15" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B97" s="17">
+        <v>95</v>
+      </c>
+      <c r="C97" s="17" t="s">
+        <v>900</v>
+      </c>
+      <c r="D97" s="19" t="s">
+        <v>895</v>
+      </c>
+      <c r="E97" s="18">
+        <v>250</v>
+      </c>
+      <c r="F97" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="G97" s="25">
+        <v>55.57</v>
+      </c>
+      <c r="H97" s="25">
+        <f>G97*E97</f>
+        <v>13892.5</v>
+      </c>
+      <c r="I97" s="18" t="s">
+        <v>836</v>
+      </c>
+      <c r="J97" s="27"/>
+      <c r="K97" s="27"/>
+      <c r="M97" s="14"/>
+      <c r="N97" s="14"/>
+      <c r="O97" s="14"/>
+    </row>
+    <row r="98" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B98" s="17">
+        <v>96</v>
+      </c>
+      <c r="C98" s="17"/>
+      <c r="D98" s="19" t="s">
+        <v>897</v>
+      </c>
+      <c r="E98" s="18">
+        <v>1</v>
+      </c>
+      <c r="F98" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G98" s="25">
+        <v>4430</v>
+      </c>
+      <c r="H98" s="25">
+        <f>G98*E98</f>
+        <v>4430</v>
+      </c>
+      <c r="I98" s="18" t="s">
+        <v>836</v>
+      </c>
+      <c r="J98" s="27"/>
+      <c r="K98" s="27"/>
+      <c r="L98" s="24"/>
+    </row>
+    <row r="99" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B99" s="17">
+        <v>97</v>
+      </c>
+      <c r="C99" s="17"/>
+      <c r="D99" s="19" t="s">
+        <v>796</v>
+      </c>
+      <c r="E99" s="18">
+        <v>1</v>
+      </c>
+      <c r="F99" s="18" t="s">
+        <v>760</v>
+      </c>
+      <c r="G99" s="25">
+        <v>670000</v>
+      </c>
+      <c r="H99" s="25">
+        <f>G99*E99</f>
+        <v>670000</v>
+      </c>
+      <c r="I99" s="18" t="s">
+        <v>836</v>
+      </c>
+      <c r="J99" s="27"/>
+      <c r="K99" s="27"/>
+    </row>
+    <row r="100" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B100" s="17">
+        <v>98</v>
+      </c>
+      <c r="C100" s="17"/>
+      <c r="D100" s="19" t="s">
+        <v>827</v>
+      </c>
+      <c r="E100" s="52">
+        <f>8*4.2*0.35</f>
+        <v>11.76</v>
+      </c>
+      <c r="F100" s="18" t="s">
+        <v>759</v>
+      </c>
+      <c r="G100" s="25">
+        <v>670</v>
+      </c>
+      <c r="H100" s="25">
+        <f>G100*E100</f>
+        <v>7879.2</v>
+      </c>
+      <c r="I100" s="18" t="s">
+        <v>836</v>
+      </c>
+      <c r="J100" s="27"/>
+      <c r="K100" s="27"/>
+      <c r="L100" s="24"/>
+    </row>
+    <row r="101" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B101" s="17">
+        <v>99</v>
+      </c>
+      <c r="C101" s="17"/>
+      <c r="D101" s="19" t="s">
+        <v>828</v>
+      </c>
+      <c r="E101" s="18">
+        <v>600</v>
+      </c>
+      <c r="F101" s="18" t="s">
+        <v>811</v>
+      </c>
+      <c r="G101" s="25">
+        <v>9.99</v>
+      </c>
+      <c r="H101" s="25">
+        <f>G101*E101</f>
+        <v>5994</v>
+      </c>
+      <c r="I101" s="18" t="s">
+        <v>836</v>
+      </c>
+      <c r="J101" s="27"/>
+      <c r="K101" s="27"/>
+      <c r="L101" s="14" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="102" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B102" s="18"/>
+      <c r="C102" s="18"/>
+      <c r="D102" s="19"/>
+      <c r="E102" s="18"/>
+      <c r="F102" s="18"/>
+      <c r="G102" s="20"/>
+      <c r="H102" s="23"/>
+      <c r="I102" s="18"/>
+      <c r="J102" s="27"/>
+      <c r="K102" s="27"/>
+      <c r="L102" s="24"/>
+    </row>
+    <row r="103" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B103" s="18"/>
+      <c r="C103" s="18"/>
+      <c r="D103" s="19"/>
+      <c r="E103" s="18"/>
+      <c r="F103" s="18"/>
+      <c r="G103" s="20" t="s">
+        <v>925</v>
+      </c>
+      <c r="H103" s="23" t="s">
+        <v>926</v>
+      </c>
+      <c r="I103" s="18"/>
+      <c r="J103" s="27"/>
+      <c r="K103" s="27"/>
+      <c r="L103" s="24"/>
+    </row>
+    <row r="104" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D104" s="21"/>
+      <c r="E104" s="22"/>
+      <c r="F104" s="22"/>
+      <c r="G104" s="15"/>
+      <c r="H104" s="16">
+        <f>SUM(Tabela242[Preço Total])</f>
+        <v>9099982.1941069029</v>
+      </c>
+      <c r="L104" s="24"/>
+    </row>
+    <row r="105" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D105" s="28"/>
+      <c r="E105" s="29"/>
+      <c r="F105" s="29"/>
+      <c r="G105" s="15"/>
+      <c r="H105" s="15"/>
+      <c r="L105" s="24"/>
+    </row>
+    <row r="108" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D108"/>
+      <c r="G108" s="15"/>
+      <c r="H108" s="26"/>
+      <c r="L108" s="24"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza planilha 22/10/2026 16:29
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="6"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_Cronograma" sheetId="1" r:id="rId1"/>
@@ -13059,7 +13059,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:O107"/>
+  <dimension ref="B1:O111"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" customWidth="1"/>
@@ -13067,7 +13067,7 @@
     <col min="3" max="3" width="27.7109375" style="14" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="92" customWidth="1"/>
     <col min="5" max="5" width="16" style="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17" style="14" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.42578125" style="15" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.42578125" style="15" customWidth="1"/>
     <col min="9" max="9" width="23.85546875" style="14" customWidth="1"/>
@@ -15918,6 +15918,18 @@
     </row>
     <row r="107" spans="2:12" x14ac:dyDescent="0.25">
       <c r="H107" s="26"/>
+    </row>
+    <row r="108" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="F108" s="39"/>
+    </row>
+    <row r="109" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="F109" s="39">
+        <f>H103+'Expansão DMP'!G59</f>
+        <v>11754238.447953057</v>
+      </c>
+    </row>
+    <row r="111" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="F111" s="39"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Atualiza planilha 23/10/2026 11:39
</commit_message>
<xml_diff>
--- a/dados/planilha.xlsx
+++ b/dados/planilha.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2709" uniqueCount="933">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2715" uniqueCount="934">
   <si>
     <t>Código EAP</t>
   </si>
@@ -2829,6 +2829,9 @@
   </si>
   <si>
     <t>Carro shuttle operação do drive in</t>
+  </si>
+  <si>
+    <t>Tratamento de esgoto</t>
   </si>
 </sst>
 </file>
@@ -2851,6 +2854,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2870,12 +2874,14 @@
       <sz val="11"/>
       <color theme="1" tint="0.249977111117893"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF404040"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -13126,7 +13132,7 @@
         <v>1273653.1700000002</v>
       </c>
       <c r="H2" s="20">
-        <f>G2*E2</f>
+        <f t="shared" ref="H2:H33" si="0">G2*E2</f>
         <v>1273653.1700000002</v>
       </c>
       <c r="I2" s="18" t="s">
@@ -13156,7 +13162,7 @@
         <v>185900</v>
       </c>
       <c r="H3" s="20">
-        <f>G3*E3</f>
+        <f t="shared" si="0"/>
         <v>185900</v>
       </c>
       <c r="I3" s="18" t="s">
@@ -13183,7 +13189,7 @@
         <v>88200</v>
       </c>
       <c r="H4" s="20">
-        <f>G4*E4</f>
+        <f t="shared" si="0"/>
         <v>88200</v>
       </c>
       <c r="I4" s="18" t="s">
@@ -13210,7 +13216,7 @@
         <v>486032</v>
       </c>
       <c r="H5" s="44">
-        <f>G5*E5</f>
+        <f t="shared" si="0"/>
         <v>486032</v>
       </c>
       <c r="I5" s="31" t="s">
@@ -13237,7 +13243,7 @@
         <v>8650</v>
       </c>
       <c r="H6" s="44">
-        <f>G6*E6</f>
+        <f t="shared" si="0"/>
         <v>8650</v>
       </c>
       <c r="I6" s="31" t="s">
@@ -13264,7 +13270,7 @@
         <v>21938</v>
       </c>
       <c r="H7" s="44">
-        <f>G7*E7</f>
+        <f t="shared" si="0"/>
         <v>131628</v>
       </c>
       <c r="I7" s="17" t="s">
@@ -13291,7 +13297,7 @@
         <v>11180</v>
       </c>
       <c r="H8" s="44">
-        <f>G8*E8</f>
+        <f t="shared" si="0"/>
         <v>11180</v>
       </c>
       <c r="I8" s="17" t="s">
@@ -13318,7 +13324,7 @@
         <v>55.57</v>
       </c>
       <c r="H9" s="44">
-        <f>G9*E9</f>
+        <f t="shared" si="0"/>
         <v>13892.5</v>
       </c>
       <c r="I9" s="17" t="s">
@@ -13345,7 +13351,7 @@
         <v>13855.22</v>
       </c>
       <c r="H10" s="51">
-        <f>G10*E10</f>
+        <f t="shared" si="0"/>
         <v>83131.319999999992</v>
       </c>
       <c r="I10" s="17" t="s">
@@ -13372,7 +13378,7 @@
         <v>111260.98</v>
       </c>
       <c r="H11" s="51">
-        <f>G11*E11</f>
+        <f t="shared" si="0"/>
         <v>111260.98</v>
       </c>
       <c r="I11" s="17" t="s">
@@ -13399,7 +13405,7 @@
         <v>55.57</v>
       </c>
       <c r="H12" s="51">
-        <f>G12*E12</f>
+        <f t="shared" si="0"/>
         <v>16671</v>
       </c>
       <c r="I12" s="17" t="s">
@@ -13426,7 +13432,7 @@
         <v>27412.5</v>
       </c>
       <c r="H13" s="51">
-        <f>G13*E13</f>
+        <f t="shared" si="0"/>
         <v>27412.5</v>
       </c>
       <c r="I13" s="17" t="s">
@@ -13454,7 +13460,7 @@
         <v>670</v>
       </c>
       <c r="H14" s="25">
-        <f>G14*E14</f>
+        <f t="shared" si="0"/>
         <v>118841.25000000001</v>
       </c>
       <c r="I14" s="18" t="s">
@@ -13482,7 +13488,7 @@
         <v>220.5</v>
       </c>
       <c r="H15" s="25">
-        <f>G15*E15</f>
+        <f t="shared" si="0"/>
         <v>36467.307692307695</v>
       </c>
       <c r="I15" s="18" t="s">
@@ -13510,7 +13516,7 @@
         <v>56.2</v>
       </c>
       <c r="H16" s="25">
-        <f>G16*E16</f>
+        <f t="shared" si="0"/>
         <v>4964.333333333333</v>
       </c>
       <c r="I16" s="18" t="s">
@@ -13538,7 +13544,7 @@
         <v>50</v>
       </c>
       <c r="H17" s="25">
-        <f>G17*E17</f>
+        <f t="shared" si="0"/>
         <v>8868.7500000000018</v>
       </c>
       <c r="I17" s="18" t="s">
@@ -13565,7 +13571,7 @@
         <v>67000</v>
       </c>
       <c r="H18" s="25">
-        <f>G18*E18</f>
+        <f t="shared" si="0"/>
         <v>67000</v>
       </c>
       <c r="I18" s="18" t="s">
@@ -13592,7 +13598,7 @@
         <v>48600</v>
       </c>
       <c r="H19" s="51">
-        <f>G19*E19</f>
+        <f t="shared" si="0"/>
         <v>48600</v>
       </c>
       <c r="I19" s="18" t="s">
@@ -13619,7 +13625,7 @@
         <v>48600</v>
       </c>
       <c r="H20" s="51">
-        <f>G20*E20</f>
+        <f t="shared" si="0"/>
         <v>48600</v>
       </c>
       <c r="I20" s="18" t="s">
@@ -13646,7 +13652,7 @@
         <v>243.39</v>
       </c>
       <c r="H21" s="51">
-        <f>G21*E21</f>
+        <f t="shared" si="0"/>
         <v>12169.5</v>
       </c>
       <c r="I21" s="18" t="s">
@@ -13674,7 +13680,7 @@
         <v>38.119999999999997</v>
       </c>
       <c r="H22" s="51">
-        <f>G22*E22</f>
+        <f t="shared" si="0"/>
         <v>6709.12</v>
       </c>
       <c r="I22" s="18" t="s">
@@ -13701,7 +13707,7 @@
         <v>24</v>
       </c>
       <c r="H23" s="51">
-        <f>G23*E23</f>
+        <f t="shared" si="0"/>
         <v>240</v>
       </c>
       <c r="I23" s="18" t="s">
@@ -13733,7 +13739,7 @@
         <v>243.39</v>
       </c>
       <c r="H24" s="51">
-        <f>G24*E24</f>
+        <f t="shared" si="0"/>
         <v>8762.0399999999991</v>
       </c>
       <c r="I24" s="18" t="s">
@@ -13762,7 +13768,7 @@
         <v>38.119999999999997</v>
       </c>
       <c r="H25" s="51">
-        <f>G25*E25</f>
+        <f t="shared" si="0"/>
         <v>2744.64</v>
       </c>
       <c r="I25" s="18" t="s">
@@ -13791,7 +13797,7 @@
         <v>32</v>
       </c>
       <c r="H26" s="51">
-        <f>G26*E26</f>
+        <f t="shared" si="0"/>
         <v>1152</v>
       </c>
       <c r="I26" s="18" t="s">
@@ -13820,7 +13826,7 @@
         <v>419</v>
       </c>
       <c r="H27" s="51">
-        <f>G27*E27</f>
+        <f t="shared" si="0"/>
         <v>1676</v>
       </c>
       <c r="I27" s="18" t="s">
@@ -13850,7 +13856,7 @@
         <v>38.119999999999997</v>
       </c>
       <c r="H28" s="51">
-        <f>G28*E28</f>
+        <f t="shared" si="0"/>
         <v>1829.7599999999998</v>
       </c>
       <c r="I28" s="18" t="s">
@@ -13877,7 +13883,7 @@
         <v>65000</v>
       </c>
       <c r="H29" s="25">
-        <f>G29*E29</f>
+        <f t="shared" si="0"/>
         <v>130000</v>
       </c>
       <c r="I29" s="18" t="s">
@@ -13906,7 +13912,7 @@
         <v>198.72</v>
       </c>
       <c r="H30" s="44">
-        <f>G30*E30</f>
+        <f t="shared" si="0"/>
         <v>11525.76</v>
       </c>
       <c r="I30" s="17" t="s">
@@ -13935,7 +13941,7 @@
         <v>484.24</v>
       </c>
       <c r="H31" s="44">
-        <f>G31*E31</f>
+        <f t="shared" si="0"/>
         <v>15011.44</v>
       </c>
       <c r="I31" s="17" t="s">
@@ -13964,7 +13970,7 @@
         <v>703.93</v>
       </c>
       <c r="H32" s="44">
-        <f>G32*E32</f>
+        <f t="shared" si="0"/>
         <v>19710.039999999997</v>
       </c>
       <c r="I32" s="17" t="s">
@@ -13994,7 +14000,7 @@
         <v>49.05</v>
       </c>
       <c r="H33" s="44">
-        <f>G33*E33</f>
+        <f t="shared" si="0"/>
         <v>4120.2</v>
       </c>
       <c r="I33" s="17" t="s">
@@ -14023,7 +14029,7 @@
         <v>151.19999999999999</v>
       </c>
       <c r="H34" s="44">
-        <f>G34*E34</f>
+        <f t="shared" ref="H34:H65" si="1">G34*E34</f>
         <v>453.59999999999997</v>
       </c>
       <c r="I34" s="17" t="s">
@@ -14052,7 +14058,7 @@
         <v>48.38</v>
       </c>
       <c r="H35" s="44">
-        <f>G35*E35</f>
+        <f t="shared" si="1"/>
         <v>96.76</v>
       </c>
       <c r="I35" s="17" t="s">
@@ -14081,7 +14087,7 @@
         <v>27.14</v>
       </c>
       <c r="H36" s="44">
-        <f>G36*E36</f>
+        <f t="shared" si="1"/>
         <v>814.2</v>
       </c>
       <c r="I36" s="17" t="s">
@@ -14110,7 +14116,7 @@
         <v>703.93</v>
       </c>
       <c r="H37" s="44">
-        <f>G37*E37</f>
+        <f t="shared" si="1"/>
         <v>8447.16</v>
       </c>
       <c r="I37" s="17" t="s">
@@ -14140,7 +14146,7 @@
         <v>484.24</v>
       </c>
       <c r="H38" s="44">
-        <f>G38*E38</f>
+        <f t="shared" si="1"/>
         <v>6295.12</v>
       </c>
       <c r="I38" s="17" t="s">
@@ -14167,7 +14173,7 @@
         <v>37375</v>
       </c>
       <c r="H39" s="51">
-        <f>G39*E39</f>
+        <f t="shared" si="1"/>
         <v>37375</v>
       </c>
       <c r="I39" s="18" t="s">
@@ -14195,7 +14201,7 @@
         <v>243.39</v>
       </c>
       <c r="H40" s="44">
-        <f>G40*E40</f>
+        <f t="shared" si="1"/>
         <v>26286.12</v>
       </c>
       <c r="I40" s="17" t="s">
@@ -14223,7 +14229,7 @@
         <v>119.7</v>
       </c>
       <c r="H41" s="44">
-        <f>G41*E41</f>
+        <f t="shared" si="1"/>
         <v>3591</v>
       </c>
       <c r="I41" s="17" t="s">
@@ -14250,7 +14256,7 @@
         <v>38.116666600000002</v>
       </c>
       <c r="H42" s="44">
-        <f>G42*E42</f>
+        <f t="shared" si="1"/>
         <v>14865.499974</v>
       </c>
       <c r="I42" s="17" t="s">
@@ -14278,7 +14284,7 @@
         <v>243.39</v>
       </c>
       <c r="H43" s="44">
-        <f>G43*E43</f>
+        <f t="shared" si="1"/>
         <v>42541.456608</v>
       </c>
       <c r="I43" s="17" t="s">
@@ -14307,7 +14313,7 @@
         <v>38.116666600000002</v>
       </c>
       <c r="H44" s="44">
-        <f>G44*E44</f>
+        <f t="shared" si="1"/>
         <v>22412.599960800002</v>
       </c>
       <c r="I44" s="17" t="s">
@@ -14334,7 +14340,7 @@
         <v>24</v>
       </c>
       <c r="H45" s="44">
-        <f>G45*E45</f>
+        <f t="shared" si="1"/>
         <v>720</v>
       </c>
       <c r="I45" s="17" t="s">
@@ -14361,7 +14367,7 @@
         <v>860</v>
       </c>
       <c r="H46" s="44">
-        <f>G46*E46</f>
+        <f t="shared" si="1"/>
         <v>860</v>
       </c>
       <c r="I46" s="17" t="s">
@@ -14388,7 +14394,7 @@
         <v>23.90625</v>
       </c>
       <c r="H47" s="25">
-        <f>G47*E47</f>
+        <f t="shared" si="1"/>
         <v>3346.875</v>
       </c>
       <c r="I47" s="18" t="s">
@@ -14415,7 +14421,7 @@
         <v>26</v>
       </c>
       <c r="H48" s="25">
-        <f>G48*E48</f>
+        <f t="shared" si="1"/>
         <v>1716</v>
       </c>
       <c r="I48" s="18" t="s">
@@ -14443,7 +14449,7 @@
         <v>31000</v>
       </c>
       <c r="H49" s="25">
-        <f>G49*E49</f>
+        <f t="shared" si="1"/>
         <v>31000</v>
       </c>
       <c r="I49" s="18" t="s">
@@ -14470,7 +14476,7 @@
         <v>6000</v>
       </c>
       <c r="H50" s="54">
-        <f>G50*E50</f>
+        <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="I50" s="17" t="s">
@@ -14497,7 +14503,7 @@
         <v>9.65</v>
       </c>
       <c r="H51" s="54">
-        <f>G51*E51</f>
+        <f t="shared" si="1"/>
         <v>39565</v>
       </c>
       <c r="I51" s="17" t="s">
@@ -14524,7 +14530,7 @@
         <v>9.65</v>
       </c>
       <c r="H52" s="54">
-        <f>G52*E52</f>
+        <f t="shared" si="1"/>
         <v>38600</v>
       </c>
       <c r="I52" s="17" t="s">
@@ -14554,7 +14560,7 @@
         <v>164000</v>
       </c>
       <c r="H53" s="54">
-        <f>G53*E53</f>
+        <f t="shared" si="1"/>
         <v>164000</v>
       </c>
       <c r="I53" s="17" t="s">
@@ -14584,7 +14590,7 @@
         <v>670</v>
       </c>
       <c r="H54" s="54">
-        <f>G54*E54</f>
+        <f t="shared" si="1"/>
         <v>66477.399999999994</v>
       </c>
       <c r="I54" s="17" t="s">
@@ -14611,7 +14617,7 @@
         <v>670</v>
       </c>
       <c r="H55" s="54">
-        <f>G55*E55</f>
+        <f t="shared" si="1"/>
         <v>45560</v>
       </c>
       <c r="I55" s="17" t="s">
@@ -14638,7 +14644,7 @@
         <v>56500</v>
       </c>
       <c r="H56" s="54">
-        <f>G56*E56</f>
+        <f t="shared" si="1"/>
         <v>56500</v>
       </c>
       <c r="I56" s="17" t="s">
@@ -14665,7 +14671,7 @@
         <v>125</v>
       </c>
       <c r="H57" s="44">
-        <f>G57*E57</f>
+        <f t="shared" si="1"/>
         <v>6250</v>
       </c>
       <c r="I57" s="17" t="s">
@@ -14692,7 +14698,7 @@
         <v>1500</v>
       </c>
       <c r="H58" s="44">
-        <f>G58*E58</f>
+        <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="I58" s="17" t="s">
@@ -14719,7 +14725,7 @@
         <v>420</v>
       </c>
       <c r="H59" s="25">
-        <f>G59*E59</f>
+        <f t="shared" si="1"/>
         <v>10920</v>
       </c>
       <c r="I59" s="17" t="s">
@@ -14749,7 +14755,7 @@
         <v>15</v>
       </c>
       <c r="H60" s="25">
-        <f>G60*E60</f>
+        <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="I60" s="17" t="s">
@@ -14777,7 +14783,7 @@
         <v>59719.5</v>
       </c>
       <c r="H61" s="25">
-        <f>G61*E61</f>
+        <f t="shared" si="1"/>
         <v>59719.5</v>
       </c>
       <c r="I61" s="17" t="s">
@@ -14804,7 +14810,7 @@
         <v>380</v>
       </c>
       <c r="H62" s="25">
-        <f>G62*E62</f>
+        <f t="shared" si="1"/>
         <v>3040</v>
       </c>
       <c r="I62" s="18" t="s">
@@ -14831,7 +14837,7 @@
         <v>290</v>
       </c>
       <c r="H63" s="25">
-        <f>G63*E63</f>
+        <f t="shared" si="1"/>
         <v>1160</v>
       </c>
       <c r="I63" s="18" t="s">
@@ -14858,7 +14864,7 @@
         <v>290</v>
       </c>
       <c r="H64" s="25">
-        <f>G64*E64</f>
+        <f t="shared" si="1"/>
         <v>1160</v>
       </c>
       <c r="I64" s="18" t="s">
@@ -14886,7 +14892,7 @@
         <v>670</v>
       </c>
       <c r="H65" s="54">
-        <f>G65*E65</f>
+        <f t="shared" si="1"/>
         <v>226878.75</v>
       </c>
       <c r="I65" s="17" t="s">
@@ -14914,7 +14920,7 @@
         <v>220.5</v>
       </c>
       <c r="H66" s="54">
-        <f>G66*E66</f>
+        <f t="shared" ref="H66:H97" si="2">G66*E66</f>
         <v>72934.61538461539</v>
       </c>
       <c r="I66" s="17" t="s">
@@ -14942,7 +14948,7 @@
         <v>56.2</v>
       </c>
       <c r="H67" s="54">
-        <f>G67*E67</f>
+        <f t="shared" si="2"/>
         <v>9835</v>
       </c>
       <c r="I67" s="17" t="s">
@@ -14969,7 +14975,7 @@
         <v>7.3</v>
       </c>
       <c r="H68" s="54">
-        <f>G68*E68</f>
+        <f t="shared" si="2"/>
         <v>7300</v>
       </c>
       <c r="I68" s="17" t="s">
@@ -14997,7 +15003,7 @@
         <v>50</v>
       </c>
       <c r="H69" s="54">
-        <f>G69*E69</f>
+        <f t="shared" si="2"/>
         <v>16931.25</v>
       </c>
       <c r="I69" s="17" t="s">
@@ -15024,7 +15030,7 @@
         <v>53550</v>
       </c>
       <c r="H70" s="54">
-        <f>G70*E70</f>
+        <f t="shared" si="2"/>
         <v>53550</v>
       </c>
       <c r="I70" s="17" t="s">
@@ -15051,7 +15057,7 @@
         <v>42.29</v>
       </c>
       <c r="H71" s="25">
-        <f>G71*E71</f>
+        <f t="shared" si="2"/>
         <v>4651.8999999999996</v>
       </c>
       <c r="I71" s="18" t="s">
@@ -15078,7 +15084,7 @@
         <v>1400</v>
       </c>
       <c r="H72" s="25">
-        <f>G72*E72</f>
+        <f t="shared" si="2"/>
         <v>1400</v>
       </c>
       <c r="I72" s="18" t="s">
@@ -15106,7 +15112,7 @@
         <v>670</v>
       </c>
       <c r="H73" s="25">
-        <f>G73*E73</f>
+        <f t="shared" si="2"/>
         <v>245421</v>
       </c>
       <c r="I73" s="18" t="s">
@@ -15134,7 +15140,7 @@
         <v>220.5</v>
       </c>
       <c r="H74" s="25">
-        <f>G74*E74</f>
+        <f t="shared" si="2"/>
         <v>39537.346153846156</v>
       </c>
       <c r="I74" s="18" t="s">
@@ -15161,7 +15167,7 @@
         <v>62525</v>
       </c>
       <c r="H75" s="25">
-        <f>G75*E75</f>
+        <f t="shared" si="2"/>
         <v>62525</v>
       </c>
       <c r="I75" s="18" t="s">
@@ -15188,7 +15194,7 @@
         <v>24500</v>
       </c>
       <c r="H76" s="44">
-        <f>G76*E76</f>
+        <f t="shared" si="2"/>
         <v>24500</v>
       </c>
       <c r="I76" s="17" t="s">
@@ -15215,7 +15221,7 @@
         <v>968004</v>
       </c>
       <c r="H77" s="54">
-        <f>G77*E77</f>
+        <f t="shared" si="2"/>
         <v>968004</v>
       </c>
       <c r="I77" s="17" t="s">
@@ -15242,7 +15248,7 @@
         <v>32000</v>
       </c>
       <c r="H78" s="51">
-        <f>G78*E78</f>
+        <f t="shared" si="2"/>
         <v>32000</v>
       </c>
       <c r="I78" s="18" t="s">
@@ -15269,7 +15275,7 @@
         <v>10000</v>
       </c>
       <c r="H79" s="51">
-        <f>G79*E79</f>
+        <f t="shared" si="2"/>
         <v>10000</v>
       </c>
       <c r="I79" s="18" t="s">
@@ -15296,7 +15302,7 @@
         <v>46600</v>
       </c>
       <c r="H80" s="25">
-        <f>G80*E80</f>
+        <f t="shared" si="2"/>
         <v>46600</v>
       </c>
       <c r="I80" s="18" t="s">
@@ -15325,7 +15331,7 @@
         <v>8100</v>
       </c>
       <c r="H81" s="25">
-        <f>G81*E81</f>
+        <f t="shared" si="2"/>
         <v>8100</v>
       </c>
       <c r="I81" s="18" t="s">
@@ -15354,7 +15360,7 @@
         <v>5000</v>
       </c>
       <c r="H82" s="25">
-        <f>G82*E82</f>
+        <f t="shared" si="2"/>
         <v>5000</v>
       </c>
       <c r="I82" s="18" t="s">
@@ -15383,7 +15389,7 @@
         <v>27000</v>
       </c>
       <c r="H83" s="25">
-        <f>G83*E83</f>
+        <f t="shared" si="2"/>
         <v>27000</v>
       </c>
       <c r="I83" s="18" t="s">
@@ -15412,7 +15418,7 @@
         <v>16</v>
       </c>
       <c r="H84" s="25">
-        <f>G84*E84</f>
+        <f t="shared" si="2"/>
         <v>5120</v>
       </c>
       <c r="I84" s="18" t="s">
@@ -15441,7 +15447,7 @@
         <v>3400</v>
       </c>
       <c r="H85" s="25">
-        <f>G85*E85</f>
+        <f t="shared" si="2"/>
         <v>3400</v>
       </c>
       <c r="I85" s="18" t="s">
@@ -15470,7 +15476,7 @@
         <v>8000</v>
       </c>
       <c r="H86" s="25">
-        <f>G86*E86</f>
+        <f t="shared" si="2"/>
         <v>8000</v>
       </c>
       <c r="I86" s="18" t="s">
@@ -15499,7 +15505,7 @@
         <v>2500</v>
       </c>
       <c r="H87" s="25">
-        <f>G87*E87</f>
+        <f t="shared" si="2"/>
         <v>2500</v>
       </c>
       <c r="I87" s="18" t="s">
@@ -15530,7 +15536,7 @@
         <v>102</v>
       </c>
       <c r="H88" s="25">
-        <f>G88*E88</f>
+        <f t="shared" si="2"/>
         <v>11730</v>
       </c>
       <c r="I88" s="17" t="s">
@@ -15559,7 +15565,7 @@
         <v>34.99</v>
       </c>
       <c r="H89" s="44">
-        <f>G89*E89</f>
+        <f t="shared" si="2"/>
         <v>3044.13</v>
       </c>
       <c r="I89" s="17" t="s">
@@ -15586,7 +15592,7 @@
         <v>255.5</v>
       </c>
       <c r="H90" s="44">
-        <f>G90*E90</f>
+        <f t="shared" si="2"/>
         <v>44457</v>
       </c>
       <c r="I90" s="17" t="s">
@@ -15613,7 +15619,7 @@
         <v>196</v>
       </c>
       <c r="H91" s="44">
-        <f>G91*E91</f>
+        <f t="shared" si="2"/>
         <v>34104</v>
       </c>
       <c r="I91" s="17" t="s">
@@ -15640,7 +15646,7 @@
         <v>0.5</v>
       </c>
       <c r="H92" s="44">
-        <f>G92*E92</f>
+        <f t="shared" si="2"/>
         <v>2350</v>
       </c>
       <c r="I92" s="17" t="s">
@@ -15667,7 +15673,7 @@
         <v>0.5</v>
       </c>
       <c r="H93" s="44">
-        <f>G93*E93</f>
+        <f t="shared" si="2"/>
         <v>1600</v>
       </c>
       <c r="I93" s="17" t="s">
@@ -15694,7 +15700,7 @@
         <v>908615.35</v>
       </c>
       <c r="H94" s="44">
-        <f>G94*E94</f>
+        <f t="shared" si="2"/>
         <v>908615.35</v>
       </c>
       <c r="I94" s="17" t="s">
@@ -15723,13 +15729,15 @@
         <v>124.25</v>
       </c>
       <c r="H95" s="25">
-        <f>G95*E95</f>
+        <f t="shared" si="2"/>
         <v>93187.5</v>
       </c>
-      <c r="I95" s="18" t="s">
-        <v>836</v>
-      </c>
-      <c r="J95" s="27"/>
+      <c r="I95" s="17" t="s">
+        <v>837</v>
+      </c>
+      <c r="J95" s="27" t="s">
+        <v>933</v>
+      </c>
       <c r="K95" s="27"/>
     </row>
     <row r="96" spans="2:11" x14ac:dyDescent="0.25">
@@ -15752,13 +15760,15 @@
         <v>55.57</v>
       </c>
       <c r="H96" s="25">
-        <f>G96*E96</f>
+        <f t="shared" si="2"/>
         <v>13892.5</v>
       </c>
-      <c r="I96" s="18" t="s">
-        <v>836</v>
-      </c>
-      <c r="J96" s="27"/>
+      <c r="I96" s="17" t="s">
+        <v>837</v>
+      </c>
+      <c r="J96" s="27" t="s">
+        <v>933</v>
+      </c>
       <c r="K96" s="27"/>
     </row>
     <row r="97" spans="2:12" x14ac:dyDescent="0.25">
@@ -15779,13 +15789,15 @@
         <v>4430</v>
       </c>
       <c r="H97" s="25">
-        <f>G97*E97</f>
+        <f t="shared" si="2"/>
         <v>4430</v>
       </c>
-      <c r="I97" s="18" t="s">
-        <v>836</v>
-      </c>
-      <c r="J97" s="27"/>
+      <c r="I97" s="17" t="s">
+        <v>837</v>
+      </c>
+      <c r="J97" s="27" t="s">
+        <v>933</v>
+      </c>
       <c r="K97" s="27"/>
     </row>
     <row r="98" spans="2:12" x14ac:dyDescent="0.25">
@@ -15806,13 +15818,15 @@
         <v>670000</v>
       </c>
       <c r="H98" s="25">
-        <f>G98*E98</f>
+        <f t="shared" ref="H98:H129" si="3">G98*E98</f>
         <v>670000</v>
       </c>
-      <c r="I98" s="18" t="s">
-        <v>836</v>
-      </c>
-      <c r="J98" s="27"/>
+      <c r="I98" s="17" t="s">
+        <v>837</v>
+      </c>
+      <c r="J98" s="27" t="s">
+        <v>933</v>
+      </c>
       <c r="K98" s="27"/>
       <c r="L98" s="14"/>
     </row>
@@ -15835,13 +15849,15 @@
         <v>670</v>
       </c>
       <c r="H99" s="25">
-        <f>G99*E99</f>
+        <f t="shared" si="3"/>
         <v>7879.2</v>
       </c>
-      <c r="I99" s="18" t="s">
-        <v>836</v>
-      </c>
-      <c r="J99" s="27"/>
+      <c r="I99" s="17" t="s">
+        <v>837</v>
+      </c>
+      <c r="J99" s="27" t="s">
+        <v>933</v>
+      </c>
       <c r="K99" s="27"/>
     </row>
     <row r="100" spans="2:12" x14ac:dyDescent="0.25">
@@ -15862,13 +15878,15 @@
         <v>9.99</v>
       </c>
       <c r="H100" s="25">
-        <f>G100*E100</f>
+        <f t="shared" si="3"/>
         <v>5994</v>
       </c>
-      <c r="I100" s="18" t="s">
-        <v>836</v>
-      </c>
-      <c r="J100" s="27"/>
+      <c r="I100" s="17" t="s">
+        <v>837</v>
+      </c>
+      <c r="J100" s="27" t="s">
+        <v>933</v>
+      </c>
       <c r="K100" s="27"/>
       <c r="L100" s="14" t="s">
         <v>812</v>
@@ -15989,7 +16007,7 @@
         <v>1547753.1700000002</v>
       </c>
       <c r="E5" s="41">
-        <f>D5/$D$2</f>
+        <f t="shared" ref="E5:E21" si="0">D5/$D$2</f>
         <v>0.20969851528888372</v>
       </c>
       <c r="F5" s="14"/>
@@ -16004,7 +16022,7 @@
         <v>992504</v>
       </c>
       <c r="E6" s="41">
-        <f>D6/$D$2</f>
+        <f t="shared" si="0"/>
         <v>0.13447015922976804</v>
       </c>
       <c r="F6" s="14"/>
@@ -16019,7 +16037,7 @@
         <v>908615.35</v>
       </c>
       <c r="E7" s="41">
-        <f>D7/$D$2</f>
+        <f t="shared" si="0"/>
         <v>0.12310444168800469</v>
       </c>
       <c r="F7" s="14"/>
@@ -16034,7 +16052,7 @@
         <v>893801.0010256411</v>
       </c>
       <c r="E8" s="41">
-        <f>D8/$D$2</f>
+        <f t="shared" si="0"/>
         <v>0.12109730835104345</v>
       </c>
       <c r="F8" s="38"/>
@@ -16046,11 +16064,11 @@
       </c>
       <c r="D9" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Tratamento de Esgoto",Tabela24[Preço Total])</f>
-        <v>795383.2</v>
+        <v>0</v>
       </c>
       <c r="E9" s="41">
-        <f>D9/$D$2</f>
-        <v>0.10776309773329118</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
@@ -16064,7 +16082,7 @@
         <v>428952.4</v>
       </c>
       <c r="E10" s="41">
-        <f>D10/$D$2</f>
+        <f t="shared" si="0"/>
         <v>5.8116942128184024E-2</v>
       </c>
       <c r="F10" s="38"/>
@@ -16079,7 +16097,7 @@
         <v>387429.61538461538</v>
       </c>
       <c r="E11" s="41">
-        <f>D11/$D$2</f>
+        <f t="shared" si="0"/>
         <v>5.2491196076889381E-2</v>
       </c>
       <c r="F11" s="38"/>
@@ -16094,7 +16112,7 @@
         <v>353535.24615384615</v>
       </c>
       <c r="E12" s="41">
-        <f>D12/$D$2</f>
+        <f t="shared" si="0"/>
         <v>4.7898991685316056E-2</v>
       </c>
       <c r="F12" s="14"/>
@@ -16106,11 +16124,11 @@
       </c>
       <c r="D13" s="35">
         <f>SUMIF(Tabela24[Aplicação],"Serviço Preliminar",Tabela24[Preço Total])</f>
-        <v>117450</v>
+        <v>912833.2</v>
       </c>
       <c r="E13" s="41">
-        <f>D13/$D$2</f>
-        <v>1.5912802569597963E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.12367590030288914</v>
       </c>
       <c r="F13" s="14"/>
       <c r="G13" s="14"/>
@@ -16124,7 +16142,7 @@
         <v>103849.27999999998</v>
       </c>
       <c r="E14" s="41">
-        <f>D14/$D$2</f>
+        <f t="shared" si="0"/>
         <v>1.4070098677180912E-2</v>
       </c>
       <c r="F14" s="38"/>
@@ -16139,7 +16157,7 @@
         <v>102596.93156880001</v>
       </c>
       <c r="E15" s="41">
-        <f>D15/$D$2</f>
+        <f t="shared" si="0"/>
         <v>1.3900423297580818E-2</v>
       </c>
       <c r="F15" s="38"/>
@@ -16154,7 +16172,7 @@
         <v>85555.13</v>
       </c>
       <c r="E16" s="41">
-        <f>D16/$D$2</f>
+        <f t="shared" si="0"/>
         <v>1.1591501851905387E-2</v>
       </c>
       <c r="F16" s="14"/>
@@ -16169,7 +16187,7 @@
         <v>76639.5</v>
       </c>
       <c r="E17" s="41">
-        <f>D17/$D$2</f>
+        <f t="shared" si="0"/>
         <v>1.0383560941104325E-2</v>
       </c>
       <c r="F17" s="38"/>
@@ -16184,7 +16202,7 @@
         <v>44742.619974000001</v>
       </c>
       <c r="E18" s="41">
-        <f>D18/$D$2</f>
+        <f t="shared" si="0"/>
         <v>6.0619878935105351E-3</v>
       </c>
       <c r="F18" s="38"/>
@@ -16199,7 +16217,7 @@
         <v>42000</v>
       </c>
       <c r="E19" s="41">
-        <f>D19/$D$2</f>
+        <f t="shared" si="0"/>
         <v>5.6904019405969722E-3</v>
       </c>
       <c r="F19" s="14"/>
@@ -16214,7 +16232,7 @@
         <v>5360</v>
       </c>
       <c r="E20" s="41">
-        <f>D20/$D$2</f>
+        <f t="shared" si="0"/>
         <v>7.2620367622856601E-4</v>
       </c>
       <c r="F20" s="38"/>
@@ -16229,7 +16247,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="41">
-        <f>D21/$D$2</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F21" s="38"/>
@@ -16311,7 +16329,7 @@
         <v>1019077.5</v>
       </c>
       <c r="G4" s="20">
-        <f>F4*D4</f>
+        <f t="shared" ref="G4:G20" si="0">F4*D4</f>
         <v>1019077.5</v>
       </c>
       <c r="H4" s="33" t="s">
@@ -16339,7 +16357,7 @@
         <v>70700</v>
       </c>
       <c r="G5" s="20">
-        <f>F5*D5</f>
+        <f t="shared" si="0"/>
         <v>70700</v>
       </c>
       <c r="H5" s="33" t="s">
@@ -16365,7 +16383,7 @@
         <v>88200</v>
       </c>
       <c r="G6" s="20">
-        <f>F6*D6</f>
+        <f t="shared" si="0"/>
         <v>88200</v>
       </c>
       <c r="H6" s="33" t="s">
@@ -16392,7 +16410,7 @@
         <v>421112</v>
       </c>
       <c r="G7" s="44">
-        <f>F7*D7</f>
+        <f t="shared" si="0"/>
         <v>421112</v>
       </c>
       <c r="H7" s="31" t="s">
@@ -16417,7 +16435,7 @@
         <v>6650</v>
       </c>
       <c r="G8" s="44">
-        <f>F8*D8</f>
+        <f t="shared" si="0"/>
         <v>6650</v>
       </c>
       <c r="H8" s="31" t="s">
@@ -16442,7 +16460,7 @@
         <v>198.72</v>
       </c>
       <c r="G9" s="44">
-        <f>F9*D9</f>
+        <f t="shared" si="0"/>
         <v>1987.2</v>
       </c>
       <c r="H9" s="31" t="s">
@@ -16467,7 +16485,7 @@
         <v>484.24</v>
       </c>
       <c r="G10" s="44">
-        <f>F10*D10</f>
+        <f t="shared" si="0"/>
         <v>12106</v>
       </c>
       <c r="H10" s="31" t="s">
@@ -16492,7 +16510,7 @@
         <v>703.93</v>
       </c>
       <c r="G11" s="44">
-        <f>F11*D11</f>
+        <f t="shared" si="0"/>
         <v>5631.44</v>
       </c>
       <c r="H11" s="31" t="s">
@@ -16517,7 +16535,7 @@
         <v>49.05</v>
       </c>
       <c r="G12" s="44">
-        <f>F12*D12</f>
+        <f t="shared" si="0"/>
         <v>1177.1999999999998</v>
       </c>
       <c r="H12" s="31" t="s">
@@ -16542,7 +16560,7 @@
         <v>151.19999999999999</v>
       </c>
       <c r="G13" s="44">
-        <f>F13*D13</f>
+        <f t="shared" si="0"/>
         <v>302.39999999999998</v>
       </c>
       <c r="H13" s="31" t="s">
@@ -16567,7 +16585,7 @@
         <v>48.38</v>
       </c>
       <c r="G14" s="44">
-        <f>F14*D14</f>
+        <f t="shared" si="0"/>
         <v>96.76</v>
       </c>
       <c r="H14" s="31" t="s">
@@ -16592,7 +16610,7 @@
         <v>27.14</v>
       </c>
       <c r="G15" s="44">
-        <f>F15*D15</f>
+        <f t="shared" si="0"/>
         <v>325.68</v>
       </c>
       <c r="H15" s="31" t="s">
@@ -16617,7 +16635,7 @@
         <v>1056959.67</v>
       </c>
       <c r="G16" s="44">
-        <f>F16*D16</f>
+        <f t="shared" si="0"/>
         <v>1056959.67</v>
       </c>
       <c r="H16" s="31" t="s">
@@ -16642,7 +16660,7 @@
         <v>163890</v>
       </c>
       <c r="G17" s="44">
-        <f>F17*D17</f>
+        <f t="shared" si="0"/>
         <v>163890</v>
       </c>
       <c r="H17" s="31" t="s">
@@ -16668,7 +16686,7 @@
         <v>243.39</v>
       </c>
       <c r="G18" s="44">
-        <f>F18*D18</f>
+        <f t="shared" si="0"/>
         <v>12412.89</v>
       </c>
       <c r="H18" s="31" t="s">
@@ -16696,7 +16714,7 @@
         <v>119.7</v>
       </c>
       <c r="G19" s="44">
-        <f>F19*D19</f>
+        <f t="shared" si="0"/>
         <v>6104.7</v>
       </c>
       <c r="H19" s="31" t="s">
@@ -16722,7 +16740,7 @@
         <v>243.39</v>
       </c>
       <c r="G20" s="44">
-        <f>F20*D20</f>
+        <f t="shared" si="0"/>
         <v>39721.247999999992</v>
       </c>
       <c r="H20" s="31" t="s">
@@ -16873,7 +16891,7 @@
         <v>4500</v>
       </c>
       <c r="G26" s="44">
-        <f>F26*D26</f>
+        <f t="shared" ref="G26:G56" si="1">F26*D26</f>
         <v>4500</v>
       </c>
       <c r="H26" s="31" t="s">
@@ -16898,7 +16916,7 @@
         <v>9.65</v>
       </c>
       <c r="G27" s="44">
-        <f>F27*D27</f>
+        <f t="shared" si="1"/>
         <v>20265</v>
       </c>
       <c r="H27" s="31" t="s">
@@ -16923,7 +16941,7 @@
         <v>9.65</v>
       </c>
       <c r="G28" s="44">
-        <f>F28*D28</f>
+        <f t="shared" si="1"/>
         <v>22195</v>
       </c>
       <c r="H28" s="31" t="s">
@@ -16948,7 +16966,7 @@
         <v>51500</v>
       </c>
       <c r="G29" s="44">
-        <f>F29*D29</f>
+        <f t="shared" si="1"/>
         <v>51500</v>
       </c>
       <c r="H29" s="31" t="s">
@@ -16973,7 +16991,7 @@
         <v>670</v>
       </c>
       <c r="G30" s="44">
-        <f>F30*D30</f>
+        <f t="shared" si="1"/>
         <v>31355.999999999996</v>
       </c>
       <c r="H30" s="31" t="s">
@@ -17001,7 +17019,7 @@
         <v>670</v>
       </c>
       <c r="G31" s="44">
-        <f>F31*D31</f>
+        <f t="shared" si="1"/>
         <v>24924.000000000004</v>
       </c>
       <c r="H31" s="31" t="s">
@@ -17029,7 +17047,7 @@
         <v>120</v>
       </c>
       <c r="G32" s="44">
-        <f>F32*D32</f>
+        <f t="shared" si="1"/>
         <v>3600</v>
       </c>
       <c r="H32" s="31" t="s">
@@ -17054,7 +17072,7 @@
         <v>420</v>
       </c>
       <c r="G33" s="25">
-        <f>F33*D33</f>
+        <f t="shared" si="1"/>
         <v>4200</v>
       </c>
       <c r="H33" s="31" t="s">
@@ -17079,7 +17097,7 @@
         <v>15</v>
       </c>
       <c r="G34" s="25">
-        <f>F34*D34</f>
+        <f t="shared" si="1"/>
         <v>3000</v>
       </c>
       <c r="H34" s="31" t="s">
@@ -17105,7 +17123,7 @@
         <v>59719.5</v>
       </c>
       <c r="G35" s="25">
-        <f>F35*D35</f>
+        <f t="shared" si="1"/>
         <v>59719.5</v>
       </c>
       <c r="H35" s="31" t="s">
@@ -17130,7 +17148,7 @@
         <v>280</v>
       </c>
       <c r="G36" s="25">
-        <f>F36*D36</f>
+        <f t="shared" si="1"/>
         <v>2240</v>
       </c>
       <c r="H36" s="33" t="s">
@@ -17155,7 +17173,7 @@
         <v>380</v>
       </c>
       <c r="G37" s="25">
-        <f>F37*D37</f>
+        <f t="shared" si="1"/>
         <v>1900</v>
       </c>
       <c r="H37" s="33" t="s">
@@ -17180,7 +17198,7 @@
         <v>290</v>
       </c>
       <c r="G38" s="25">
-        <f>F38*D38</f>
+        <f t="shared" si="1"/>
         <v>580</v>
       </c>
       <c r="H38" s="33" t="s">
@@ -17205,7 +17223,7 @@
         <v>290</v>
       </c>
       <c r="G39" s="25">
-        <f>F39*D39</f>
+        <f t="shared" si="1"/>
         <v>580</v>
       </c>
       <c r="H39" s="33" t="s">
@@ -17231,7 +17249,7 @@
         <v>670</v>
       </c>
       <c r="G40" s="44">
-        <f>F40*D40</f>
+        <f t="shared" si="1"/>
         <v>211050</v>
       </c>
       <c r="H40" s="31" t="s">
@@ -17257,7 +17275,7 @@
         <v>220.5</v>
       </c>
       <c r="G41" s="44">
-        <f>F41*D41</f>
+        <f t="shared" si="1"/>
         <v>67846.153846153844</v>
       </c>
       <c r="H41" s="31" t="s">
@@ -17282,7 +17300,7 @@
         <v>56.2</v>
       </c>
       <c r="G42" s="44">
-        <f>F42*D42</f>
+        <f t="shared" si="1"/>
         <v>9385.4</v>
       </c>
       <c r="H42" s="31" t="s">
@@ -17307,7 +17325,7 @@
         <v>7.3</v>
       </c>
       <c r="G43" s="44">
-        <f>F43*D43</f>
+        <f t="shared" si="1"/>
         <v>7300</v>
       </c>
       <c r="H43" s="31" t="s">
@@ -17332,7 +17350,7 @@
         <v>50</v>
       </c>
       <c r="G44" s="44">
-        <f>F44*D44</f>
+        <f t="shared" si="1"/>
         <v>15750</v>
       </c>
       <c r="H44" s="31" t="s">
@@ -17357,7 +17375,7 @@
         <v>49800</v>
       </c>
       <c r="G45" s="44">
-        <f>F45*D45</f>
+        <f t="shared" si="1"/>
         <v>49800</v>
       </c>
       <c r="H45" s="31" t="s">
@@ -17382,7 +17400,7 @@
         <v>15000</v>
       </c>
       <c r="G46" s="44">
-        <f>F46*D46</f>
+        <f t="shared" si="1"/>
         <v>15000</v>
       </c>
       <c r="H46" s="31" t="s">
@@ -17409,7 +17427,7 @@
         <v>404191.96</v>
       </c>
       <c r="G47" s="44">
-        <f>F47*D47</f>
+        <f t="shared" si="1"/>
         <v>404191.96</v>
       </c>
       <c r="H47" s="31" t="s">
@@ -17436,7 +17454,7 @@
         <v>14503</v>
       </c>
       <c r="G48" s="44">
-        <f>F48*D48</f>
+        <f t="shared" si="1"/>
         <v>14503</v>
       </c>
       <c r="H48" s="31" t="s">
@@ -17463,7 +17481,7 @@
         <v>95.9</v>
       </c>
       <c r="G49" s="44">
-        <f>F49*D49</f>
+        <f t="shared" si="1"/>
         <v>139619.85100000002</v>
       </c>
       <c r="H49" s="31" t="s">
@@ -17488,7 +17506,7 @@
         <v>95.9</v>
       </c>
       <c r="G50" s="44">
-        <f>F50*D50</f>
+        <f t="shared" si="1"/>
         <v>67795.546000000002</v>
       </c>
       <c r="H50" s="31" t="s">
@@ -17513,7 +17531,7 @@
         <v>95</v>
       </c>
       <c r="G51" s="44">
-        <f>F51*D51</f>
+        <f t="shared" si="1"/>
         <v>4180</v>
       </c>
       <c r="H51" s="31" t="s">
@@ -17538,7 +17556,7 @@
         <v>35</v>
       </c>
       <c r="G52" s="44">
-        <f>F52*D52</f>
+        <f t="shared" si="1"/>
         <v>105</v>
       </c>
       <c r="H52" s="31" t="s">
@@ -17563,7 +17581,7 @@
         <v>25.9</v>
       </c>
       <c r="G53" s="44">
-        <f>F53*D53</f>
+        <f t="shared" si="1"/>
         <v>3263.3999999999996</v>
       </c>
       <c r="H53" s="31" t="s">
@@ -17588,7 +17606,7 @@
         <v>1750</v>
       </c>
       <c r="G54" s="44">
-        <f>F54*D54</f>
+        <f t="shared" si="1"/>
         <v>1750</v>
       </c>
       <c r="H54" s="31" t="s">
@@ -17613,7 +17631,7 @@
         <v>174417.38</v>
       </c>
       <c r="G55" s="44">
-        <f>F55*D55</f>
+        <f t="shared" si="1"/>
         <v>174417.38</v>
       </c>
       <c r="H55" s="31" t="s">
@@ -17638,7 +17656,7 @@
         <v>5000</v>
       </c>
       <c r="G56" s="25">
-        <f>F56*D56</f>
+        <f t="shared" si="1"/>
         <v>5000</v>
       </c>
       <c r="H56" s="33" t="s">
@@ -17787,7 +17805,7 @@
         <v>1220849.67</v>
       </c>
       <c r="E7" s="41">
-        <f>D7/$D$2</f>
+        <f t="shared" ref="E7:E20" si="0">D7/$D$2</f>
         <v>0.27915414542962674</v>
       </c>
       <c r="F7" s="41"/>
@@ -17801,7 +17819,7 @@
         <v>1177977.5</v>
       </c>
       <c r="E8" s="41">
-        <f>D8/$D$2</f>
+        <f t="shared" si="0"/>
         <v>0.26935118256437596</v>
       </c>
       <c r="F8" s="41"/>
@@ -17815,7 +17833,7 @@
         <v>361131.5538461539</v>
       </c>
       <c r="E9" s="41">
-        <f>D9/$D$2</f>
+        <f t="shared" si="0"/>
         <v>8.2574761478697328E-2</v>
       </c>
       <c r="F9" s="41"/>
@@ -17829,7 +17847,7 @@
         <v>216713.79700000002</v>
       </c>
       <c r="E10" s="41">
-        <f>D10/$D$2</f>
+        <f t="shared" si="0"/>
         <v>4.9552828895259984E-2</v>
       </c>
       <c r="F10" s="41"/>
@@ -17843,7 +17861,7 @@
         <v>174417.38</v>
       </c>
       <c r="E11" s="41">
-        <f>D11/$D$2</f>
+        <f t="shared" si="0"/>
         <v>3.9881515192590811E-2</v>
       </c>
       <c r="F11" s="41"/>
@@ -17857,7 +17875,7 @@
         <v>164340</v>
       </c>
       <c r="E12" s="41">
-        <f>D12/$D$2</f>
+        <f t="shared" si="0"/>
         <v>3.7577265561209404E-2</v>
       </c>
       <c r="F12" s="41"/>
@@ -17871,7 +17889,7 @@
         <v>79138.372999999992</v>
       </c>
       <c r="E13" s="41">
-        <f>D13/$D$2</f>
+        <f t="shared" si="0"/>
         <v>1.809543421140954E-2</v>
       </c>
       <c r="F13" s="41"/>
@@ -17885,7 +17903,7 @@
         <v>66919.5</v>
       </c>
       <c r="E14" s="41">
-        <f>D14/$D$2</f>
+        <f t="shared" si="0"/>
         <v>1.5301520157742197E-2</v>
       </c>
       <c r="F14" s="41"/>
@@ -17899,7 +17917,7 @@
         <v>21626.68</v>
       </c>
       <c r="E15" s="41">
-        <f>D15/$D$2</f>
+        <f t="shared" si="0"/>
         <v>4.945062051644738E-3</v>
       </c>
       <c r="F15" s="41"/>
@@ -17913,7 +17931,7 @@
         <v>18517.59</v>
       </c>
       <c r="E16" s="41">
-        <f>D16/$D$2</f>
+        <f t="shared" si="0"/>
         <v>4.2341511317001077E-3</v>
       </c>
       <c r="F16" s="41"/>
@@ -17927,7 +17945,7 @@
         <v>5300</v>
       </c>
       <c r="E17" s="41">
-        <f>D17/$D$2</f>
+        <f t="shared" si="0"/>
         <v>1.2118748172959099E-3</v>
       </c>
       <c r="F17" s="41"/>
@@ -17941,7 +17959,7 @@
         <v>5000</v>
       </c>
       <c r="E18" s="41">
-        <f>D18/$D$2</f>
+        <f t="shared" si="0"/>
         <v>1.1432781295244432E-3</v>
       </c>
       <c r="F18" s="41"/>
@@ -17955,7 +17973,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="41">
-        <f>D19/$D$2</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F19" s="41"/>
@@ -17969,7 +17987,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="41">
-        <f>D20/$D$2</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F20" s="41"/>
@@ -18090,7 +18108,7 @@
         <v>1983985.92</v>
       </c>
       <c r="H2" s="20">
-        <f>G2*E2</f>
+        <f t="shared" ref="H2:H33" si="0">G2*E2</f>
         <v>1983985.92</v>
       </c>
       <c r="I2" s="18" t="s">
@@ -18120,7 +18138,7 @@
         <v>294700</v>
       </c>
       <c r="H3" s="20">
-        <f>G3*E3</f>
+        <f t="shared" si="0"/>
         <v>294700</v>
       </c>
       <c r="I3" s="18" t="s">
@@ -18147,7 +18165,7 @@
         <v>88200</v>
       </c>
       <c r="H4" s="20">
-        <f>G4*E4</f>
+        <f t="shared" si="0"/>
         <v>88200</v>
       </c>
       <c r="I4" s="18" t="s">
@@ -18173,7 +18191,7 @@
         <v>300000</v>
       </c>
       <c r="H5" s="20">
-        <f>G5*E5</f>
+        <f t="shared" si="0"/>
         <v>900000</v>
       </c>
       <c r="I5" s="18" t="s">
@@ -18201,7 +18219,7 @@
         <v>486032</v>
       </c>
       <c r="H6" s="44">
-        <f>G6*E6</f>
+        <f t="shared" si="0"/>
         <v>486032</v>
       </c>
       <c r="I6" s="31" t="s">
@@ -18229,7 +18247,7 @@
         <v>8650</v>
       </c>
       <c r="H7" s="44">
-        <f>G7*E7</f>
+        <f t="shared" si="0"/>
         <v>8650</v>
       </c>
       <c r="I7" s="31" t="s">
@@ -18257,7 +18275,7 @@
         <v>21938</v>
       </c>
       <c r="H8" s="44">
-        <f>G8*E8</f>
+        <f t="shared" si="0"/>
         <v>131628</v>
       </c>
       <c r="I8" s="17" t="s">
@@ -18285,7 +18303,7 @@
         <v>11180</v>
       </c>
       <c r="H9" s="44">
-        <f>G9*E9</f>
+        <f t="shared" si="0"/>
         <v>11180</v>
       </c>
       <c r="I9" s="17" t="s">
@@ -18313,7 +18331,7 @@
         <v>55.57</v>
       </c>
       <c r="H10" s="44">
-        <f>G10*E10</f>
+        <f t="shared" si="0"/>
         <v>13892.5</v>
       </c>
       <c r="I10" s="17" t="s">
@@ -18341,7 +18359,7 @@
         <v>13855.22</v>
       </c>
       <c r="H11" s="51">
-        <f>G11*E11</f>
+        <f t="shared" si="0"/>
         <v>83131.319999999992</v>
       </c>
       <c r="I11" s="17" t="s">
@@ -18369,7 +18387,7 @@
         <v>111260.98</v>
       </c>
       <c r="H12" s="51">
-        <f>G12*E12</f>
+        <f t="shared" si="0"/>
         <v>111260.98</v>
       </c>
       <c r="I12" s="17" t="s">
@@ -18397,7 +18415,7 @@
         <v>55.57</v>
       </c>
       <c r="H13" s="51">
-        <f>G13*E13</f>
+        <f t="shared" si="0"/>
         <v>16671</v>
       </c>
       <c r="I13" s="17" t="s">
@@ -18425,7 +18443,7 @@
         <v>27412.5</v>
       </c>
       <c r="H14" s="51">
-        <f>G14*E14</f>
+        <f t="shared" si="0"/>
         <v>27412.5</v>
       </c>
       <c r="I14" s="17" t="s">
@@ -18454,7 +18472,7 @@
         <v>670</v>
       </c>
       <c r="H15" s="25">
-        <f>G15*E15</f>
+        <f t="shared" si="0"/>
         <v>118841.25000000001</v>
       </c>
       <c r="I15" s="18" t="s">
@@ -18483,7 +18501,7 @@
         <v>220.5</v>
       </c>
       <c r="H16" s="25">
-        <f>G16*E16</f>
+        <f t="shared" si="0"/>
         <v>36467.307692307695</v>
       </c>
       <c r="I16" s="18" t="s">
@@ -18512,7 +18530,7 @@
         <v>56.2</v>
       </c>
       <c r="H17" s="25">
-        <f>G17*E17</f>
+        <f t="shared" si="0"/>
         <v>4964.333333333333</v>
       </c>
       <c r="I17" s="18" t="s">
@@ -18541,7 +18559,7 @@
         <v>50</v>
       </c>
       <c r="H18" s="25">
-        <f>G18*E18</f>
+        <f t="shared" si="0"/>
         <v>8868.7500000000018</v>
       </c>
       <c r="I18" s="18" t="s">
@@ -18569,7 +18587,7 @@
         <v>67000</v>
       </c>
       <c r="H19" s="25">
-        <f>G19*E19</f>
+        <f t="shared" si="0"/>
         <v>67000</v>
       </c>
       <c r="I19" s="18" t="s">
@@ -18597,7 +18615,7 @@
         <v>48600</v>
       </c>
       <c r="H20" s="51">
-        <f>G20*E20</f>
+        <f t="shared" si="0"/>
         <v>48600</v>
       </c>
       <c r="I20" s="18" t="s">
@@ -18625,7 +18643,7 @@
         <v>48600</v>
       </c>
       <c r="H21" s="51">
-        <f>G21*E21</f>
+        <f t="shared" si="0"/>
         <v>48600</v>
       </c>
       <c r="I21" s="18" t="s">
@@ -18653,7 +18671,7 @@
         <v>243.39</v>
       </c>
       <c r="H22" s="51">
-        <f>G22*E22</f>
+        <f t="shared" si="0"/>
         <v>12169.5</v>
       </c>
       <c r="I22" s="18" t="s">
@@ -18682,7 +18700,7 @@
         <v>38.119999999999997</v>
       </c>
       <c r="H23" s="51">
-        <f>G23*E23</f>
+        <f t="shared" si="0"/>
         <v>6709.12</v>
       </c>
       <c r="I23" s="18" t="s">
@@ -18710,7 +18728,7 @@
         <v>24</v>
       </c>
       <c r="H24" s="51">
-        <f>G24*E24</f>
+        <f t="shared" si="0"/>
         <v>240</v>
       </c>
       <c r="I24" s="18" t="s">
@@ -18742,7 +18760,7 @@
         <v>243.39</v>
       </c>
       <c r="H25" s="51">
-        <f>G25*E25</f>
+        <f t="shared" si="0"/>
         <v>8762.0399999999991</v>
       </c>
       <c r="I25" s="18" t="s">
@@ -18772,7 +18790,7 @@
         <v>38.119999999999997</v>
       </c>
       <c r="H26" s="51">
-        <f>G26*E26</f>
+        <f t="shared" si="0"/>
         <v>2744.64</v>
       </c>
       <c r="I26" s="18" t="s">
@@ -18802,7 +18820,7 @@
         <v>32</v>
       </c>
       <c r="H27" s="51">
-        <f>G27*E27</f>
+        <f t="shared" si="0"/>
         <v>1152</v>
       </c>
       <c r="I27" s="18" t="s">
@@ -18832,7 +18850,7 @@
         <v>419</v>
       </c>
       <c r="H28" s="51">
-        <f>G28*E28</f>
+        <f t="shared" si="0"/>
         <v>1676</v>
       </c>
       <c r="I28" s="18" t="s">
@@ -18863,7 +18881,7 @@
         <v>38.119999999999997</v>
       </c>
       <c r="H29" s="51">
-        <f>G29*E29</f>
+        <f t="shared" si="0"/>
         <v>1829.7599999999998</v>
       </c>
       <c r="I29" s="18" t="s">
@@ -18891,7 +18909,7 @@
         <v>65000</v>
       </c>
       <c r="H30" s="25">
-        <f>G30*E30</f>
+        <f t="shared" si="0"/>
         <v>130000</v>
       </c>
       <c r="I30" s="18" t="s">
@@ -18921,7 +18939,7 @@
         <v>198.72</v>
       </c>
       <c r="H31" s="44">
-        <f>G31*E31</f>
+        <f t="shared" si="0"/>
         <v>11525.76</v>
       </c>
       <c r="I31" s="17" t="s">
@@ -18951,7 +18969,7 @@
         <v>484.24</v>
       </c>
       <c r="H32" s="44">
-        <f>G32*E32</f>
+        <f t="shared" si="0"/>
         <v>15011.44</v>
       </c>
       <c r="I32" s="17" t="s">
@@ -18981,7 +18999,7 @@
         <v>703.93</v>
       </c>
       <c r="H33" s="44">
-        <f>G33*E33</f>
+        <f t="shared" si="0"/>
         <v>19710.039999999997</v>
       </c>
       <c r="I33" s="17" t="s">
@@ -19012,7 +19030,7 @@
         <v>49.05</v>
       </c>
       <c r="H34" s="44">
-        <f>G34*E34</f>
+        <f t="shared" ref="H34:H65" si="1">G34*E34</f>
         <v>4120.2</v>
       </c>
       <c r="I34" s="17" t="s">
@@ -19042,7 +19060,7 @@
         <v>151.19999999999999</v>
       </c>
       <c r="H35" s="44">
-        <f>G35*E35</f>
+        <f t="shared" si="1"/>
         <v>453.59999999999997</v>
       </c>
       <c r="I35" s="17" t="s">
@@ -19072,7 +19090,7 @@
         <v>48.38</v>
       </c>
       <c r="H36" s="44">
-        <f>G36*E36</f>
+        <f t="shared" si="1"/>
         <v>96.76</v>
       </c>
       <c r="I36" s="17" t="s">
@@ -19102,7 +19120,7 @@
         <v>27.14</v>
       </c>
       <c r="H37" s="44">
-        <f>G37*E37</f>
+        <f t="shared" si="1"/>
         <v>814.2</v>
       </c>
       <c r="I37" s="17" t="s">
@@ -19132,7 +19150,7 @@
         <v>703.93</v>
       </c>
       <c r="H38" s="44">
-        <f>G38*E38</f>
+        <f t="shared" si="1"/>
         <v>8447.16</v>
       </c>
       <c r="I38" s="17" t="s">
@@ -19163,7 +19181,7 @@
         <v>484.24</v>
       </c>
       <c r="H39" s="44">
-        <f>G39*E39</f>
+        <f t="shared" si="1"/>
         <v>6295.12</v>
       </c>
       <c r="I39" s="17" t="s">
@@ -19191,7 +19209,7 @@
         <v>37375</v>
       </c>
       <c r="H40" s="51">
-        <f>G40*E40</f>
+        <f t="shared" si="1"/>
         <v>37375</v>
       </c>
       <c r="I40" s="18" t="s">
@@ -19220,7 +19238,7 @@
         <v>243.39</v>
       </c>
       <c r="H41" s="44">
-        <f>G41*E41</f>
+        <f t="shared" si="1"/>
         <v>26286.12</v>
       </c>
       <c r="I41" s="17" t="s">
@@ -19247,7 +19265,7 @@
         <v>119.7</v>
       </c>
       <c r="H42" s="44">
-        <f>G42*E42</f>
+        <f t="shared" si="1"/>
         <v>3591</v>
       </c>
       <c r="I42" s="17" t="s">
@@ -19275,7 +19293,7 @@
         <v>38.116666600000002</v>
       </c>
       <c r="H43" s="44">
-        <f>G43*E43</f>
+        <f t="shared" si="1"/>
         <v>14865.499974</v>
       </c>
       <c r="I43" s="17" t="s">
@@ -19304,7 +19322,7 @@
         <v>243.39</v>
       </c>
       <c r="H44" s="44">
-        <f>G44*E44</f>
+        <f t="shared" si="1"/>
         <v>42541.456608</v>
       </c>
       <c r="I44" s="17" t="s">
@@ -19332,7 +19350,7 @@
         <v>38.116666600000002</v>
       </c>
       <c r="H45" s="44">
-        <f>G45*E45</f>
+        <f t="shared" si="1"/>
         <v>22412.599960800002</v>
       </c>
       <c r="I45" s="17" t="s">
@@ -19360,7 +19378,7 @@
         <v>24</v>
       </c>
       <c r="H46" s="44">
-        <f>G46*E46</f>
+        <f t="shared" si="1"/>
         <v>720</v>
       </c>
       <c r="I46" s="17" t="s">
@@ -19388,7 +19406,7 @@
         <v>860</v>
       </c>
       <c r="H47" s="44">
-        <f>G47*E47</f>
+        <f t="shared" si="1"/>
         <v>860</v>
       </c>
       <c r="I47" s="17" t="s">
@@ -19416,7 +19434,7 @@
         <v>23.90625</v>
       </c>
       <c r="H48" s="25">
-        <f>G48*E48</f>
+        <f t="shared" si="1"/>
         <v>3346.875</v>
       </c>
       <c r="I48" s="18" t="s">
@@ -19444,7 +19462,7 @@
         <v>26</v>
       </c>
       <c r="H49" s="25">
-        <f>G49*E49</f>
+        <f t="shared" si="1"/>
         <v>1716</v>
       </c>
       <c r="I49" s="18" t="s">
@@ -19473,7 +19491,7 @@
         <v>31000</v>
       </c>
       <c r="H50" s="25">
-        <f>G50*E50</f>
+        <f t="shared" si="1"/>
         <v>31000</v>
       </c>
       <c r="I50" s="18" t="s">
@@ -19501,7 +19519,7 @@
         <v>6000</v>
       </c>
       <c r="H51" s="54">
-        <f>G51*E51</f>
+        <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="I51" s="17" t="s">
@@ -19529,7 +19547,7 @@
         <v>9.65</v>
       </c>
       <c r="H52" s="54">
-        <f>G52*E52</f>
+        <f t="shared" si="1"/>
         <v>39565</v>
       </c>
       <c r="I52" s="17" t="s">
@@ -19557,7 +19575,7 @@
         <v>9.65</v>
       </c>
       <c r="H53" s="54">
-        <f>G53*E53</f>
+        <f t="shared" si="1"/>
         <v>38600</v>
       </c>
       <c r="I53" s="17" t="s">
@@ -19587,7 +19605,7 @@
         <v>164000</v>
       </c>
       <c r="H54" s="54">
-        <f>G54*E54</f>
+        <f t="shared" si="1"/>
         <v>164000</v>
       </c>
       <c r="I54" s="17" t="s">
@@ -19617,7 +19635,7 @@
         <v>670</v>
       </c>
       <c r="H55" s="54">
-        <f>G55*E55</f>
+        <f t="shared" si="1"/>
         <v>66477.399999999994</v>
       </c>
       <c r="I55" s="17" t="s">
@@ -19645,7 +19663,7 @@
         <v>670</v>
       </c>
       <c r="H56" s="54">
-        <f>G56*E56</f>
+        <f t="shared" si="1"/>
         <v>45560</v>
       </c>
       <c r="I56" s="17" t="s">
@@ -19673,7 +19691,7 @@
         <v>56500</v>
       </c>
       <c r="H57" s="54">
-        <f>G57*E57</f>
+        <f t="shared" si="1"/>
         <v>56500</v>
       </c>
       <c r="I57" s="17" t="s">
@@ -19701,7 +19719,7 @@
         <v>125</v>
       </c>
       <c r="H58" s="44">
-        <f>G58*E58</f>
+        <f t="shared" si="1"/>
         <v>6250</v>
       </c>
       <c r="I58" s="17" t="s">
@@ -19729,7 +19747,7 @@
         <v>1500</v>
       </c>
       <c r="H59" s="44">
-        <f>G59*E59</f>
+        <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="I59" s="17" t="s">
@@ -19757,7 +19775,7 @@
         <v>420</v>
       </c>
       <c r="H60" s="25">
-        <f>G60*E60</f>
+        <f t="shared" si="1"/>
         <v>10920</v>
       </c>
       <c r="I60" s="17" t="s">
@@ -19787,7 +19805,7 @@
         <v>15</v>
       </c>
       <c r="H61" s="25">
-        <f>G61*E61</f>
+        <f t="shared" si="1"/>
         <v>6000</v>
       </c>
       <c r="I61" s="17" t="s">
@@ -19816,7 +19834,7 @@
         <v>59719.5</v>
       </c>
       <c r="H62" s="25">
-        <f>G62*E62</f>
+        <f t="shared" si="1"/>
         <v>59719.5</v>
       </c>
       <c r="I62" s="17" t="s">
@@ -19844,7 +19862,7 @@
         <v>380</v>
       </c>
       <c r="H63" s="25">
-        <f>G63*E63</f>
+        <f t="shared" si="1"/>
         <v>3040</v>
       </c>
       <c r="I63" s="18" t="s">
@@ -19872,7 +19890,7 @@
         <v>290</v>
       </c>
       <c r="H64" s="25">
-        <f>G64*E64</f>
+        <f t="shared" si="1"/>
         <v>1160</v>
       </c>
       <c r="I64" s="18" t="s">
@@ -19900,7 +19918,7 @@
         <v>290</v>
       </c>
       <c r="H65" s="25">
-        <f>G65*E65</f>
+        <f t="shared" si="1"/>
         <v>1160</v>
       </c>
       <c r="I65" s="18" t="s">
@@ -19929,7 +19947,7 @@
         <v>670</v>
       </c>
       <c r="H66" s="54">
-        <f>G66*E66</f>
+        <f t="shared" ref="H66:H97" si="2">G66*E66</f>
         <v>226878.75</v>
       </c>
       <c r="I66" s="17" t="s">
@@ -19960,7 +19978,7 @@
         <v>220.5</v>
       </c>
       <c r="H67" s="54">
-        <f>G67*E67</f>
+        <f t="shared" si="2"/>
         <v>72934.61538461539</v>
       </c>
       <c r="I67" s="17" t="s">
@@ -19991,7 +20009,7 @@
         <v>56.2</v>
       </c>
       <c r="H68" s="54">
-        <f>G68*E68</f>
+        <f t="shared" si="2"/>
         <v>9835</v>
       </c>
       <c r="I68" s="17" t="s">
@@ -20021,7 +20039,7 @@
         <v>7.3</v>
       </c>
       <c r="H69" s="54">
-        <f>G69*E69</f>
+        <f t="shared" si="2"/>
         <v>7300</v>
       </c>
       <c r="I69" s="17" t="s">
@@ -20052,7 +20070,7 @@
         <v>50</v>
       </c>
       <c r="H70" s="54">
-        <f>G70*E70</f>
+        <f t="shared" si="2"/>
         <v>16931.25</v>
       </c>
       <c r="I70" s="17" t="s">
@@ -20082,7 +20100,7 @@
         <v>53550</v>
       </c>
       <c r="H71" s="54">
-        <f>G71*E71</f>
+        <f t="shared" si="2"/>
         <v>53550</v>
       </c>
       <c r="I71" s="17" t="s">
@@ -20112,7 +20130,7 @@
         <v>42.29</v>
       </c>
       <c r="H72" s="25">
-        <f>G72*E72</f>
+        <f t="shared" si="2"/>
         <v>4651.8999999999996</v>
       </c>
       <c r="I72" s="18" t="s">
@@ -20142,7 +20160,7 @@
         <v>1400</v>
       </c>
       <c r="H73" s="25">
-        <f>G73*E73</f>
+        <f t="shared" si="2"/>
         <v>1400</v>
       </c>
       <c r="I73" s="18" t="s">
@@ -20173,7 +20191,7 @@
         <v>670</v>
       </c>
       <c r="H74" s="25">
-        <f>G74*E74</f>
+        <f t="shared" si="2"/>
         <v>245421</v>
       </c>
       <c r="I74" s="18" t="s">
@@ -20204,7 +20222,7 @@
         <v>220.5</v>
       </c>
       <c r="H75" s="25">
-        <f>G75*E75</f>
+        <f t="shared" si="2"/>
         <v>39537.346153846156</v>
       </c>
       <c r="I75" s="18" t="s">
@@ -20234,7 +20252,7 @@
         <v>62525</v>
       </c>
       <c r="H76" s="25">
-        <f>G76*E76</f>
+        <f t="shared" si="2"/>
         <v>62525</v>
       </c>
       <c r="I76" s="18" t="s">
@@ -20264,7 +20282,7 @@
         <v>24500</v>
       </c>
       <c r="H77" s="44">
-        <f>G77*E77</f>
+        <f t="shared" si="2"/>
         <v>24500</v>
       </c>
       <c r="I77" s="17" t="s">
@@ -20294,7 +20312,7 @@
         <v>968004</v>
       </c>
       <c r="H78" s="54">
-        <f>G78*E78</f>
+        <f t="shared" si="2"/>
         <v>968004</v>
       </c>
       <c r="I78" s="17" t="s">
@@ -20324,7 +20342,7 @@
         <v>32000</v>
       </c>
       <c r="H79" s="51">
-        <f>G79*E79</f>
+        <f t="shared" si="2"/>
         <v>32000</v>
       </c>
       <c r="I79" s="18" t="s">
@@ -20354,7 +20372,7 @@
         <v>10000</v>
       </c>
       <c r="H80" s="51">
-        <f>G80*E80</f>
+        <f t="shared" si="2"/>
         <v>10000</v>
       </c>
       <c r="I80" s="18" t="s">
@@ -20384,7 +20402,7 @@
         <v>46600</v>
       </c>
       <c r="H81" s="25">
-        <f>G81*E81</f>
+        <f t="shared" si="2"/>
         <v>46600</v>
       </c>
       <c r="I81" s="18" t="s">
@@ -20416,7 +20434,7 @@
         <v>8100</v>
       </c>
       <c r="H82" s="25">
-        <f>G82*E82</f>
+        <f t="shared" si="2"/>
         <v>8100</v>
       </c>
       <c r="I82" s="18" t="s">
@@ -20448,7 +20466,7 @@
         <v>5000</v>
       </c>
       <c r="H83" s="25">
-        <f>G83*E83</f>
+        <f t="shared" si="2"/>
         <v>5000</v>
       </c>
       <c r="I83" s="18" t="s">
@@ -20480,7 +20498,7 @@
         <v>27000</v>
       </c>
       <c r="H84" s="25">
-        <f>G84*E84</f>
+        <f t="shared" si="2"/>
         <v>27000</v>
       </c>
       <c r="I84" s="18" t="s">
@@ -20512,7 +20530,7 @@
         <v>16</v>
       </c>
       <c r="H85" s="25">
-        <f>G85*E85</f>
+        <f t="shared" si="2"/>
         <v>5120</v>
       </c>
       <c r="I85" s="18" t="s">
@@ -20544,7 +20562,7 @@
         <v>3400</v>
       </c>
       <c r="H86" s="25">
-        <f>G86*E86</f>
+        <f t="shared" si="2"/>
         <v>3400</v>
       </c>
       <c r="I86" s="18" t="s">
@@ -20576,7 +20594,7 @@
         <v>8000</v>
       </c>
       <c r="H87" s="25">
-        <f>G87*E87</f>
+        <f t="shared" si="2"/>
         <v>8000</v>
       </c>
       <c r="I87" s="18" t="s">
@@ -20608,7 +20626,7 @@
         <v>2500</v>
       </c>
       <c r="H88" s="25">
-        <f>G88*E88</f>
+        <f t="shared" si="2"/>
         <v>2500</v>
       </c>
       <c r="I88" s="18" t="s">
@@ -20642,7 +20660,7 @@
         <v>102</v>
       </c>
       <c r="H89" s="25">
-        <f>G89*E89</f>
+        <f t="shared" si="2"/>
         <v>11730</v>
       </c>
       <c r="I89" s="17" t="s">
@@ -20674,7 +20692,7 @@
         <v>34.99</v>
       </c>
       <c r="H90" s="44">
-        <f>G90*E90</f>
+        <f t="shared" si="2"/>
         <v>3044.13</v>
       </c>
       <c r="I90" s="17" t="s">
@@ -20704,7 +20722,7 @@
         <v>255.5</v>
       </c>
       <c r="H91" s="44">
-        <f>G91*E91</f>
+        <f t="shared" si="2"/>
         <v>44457</v>
       </c>
       <c r="I91" s="17" t="s">
@@ -20734,7 +20752,7 @@
         <v>196</v>
       </c>
       <c r="H92" s="44">
-        <f>G92*E92</f>
+        <f t="shared" si="2"/>
         <v>34104</v>
       </c>
       <c r="I92" s="17" t="s">
@@ -20764,7 +20782,7 @@
         <v>0.5</v>
       </c>
       <c r="H93" s="44">
-        <f>G93*E93</f>
+        <f t="shared" si="2"/>
         <v>2350</v>
       </c>
       <c r="I93" s="17" t="s">
@@ -20794,7 +20812,7 @@
         <v>0.5</v>
       </c>
       <c r="H94" s="44">
-        <f>G94*E94</f>
+        <f t="shared" si="2"/>
         <v>1600</v>
       </c>
       <c r="I94" s="17" t="s">
@@ -20824,7 +20842,7 @@
         <v>908615.35</v>
       </c>
       <c r="H95" s="44">
-        <f>G95*E95</f>
+        <f t="shared" si="2"/>
         <v>908615.35</v>
       </c>
       <c r="I95" s="17" t="s">
@@ -20856,7 +20874,7 @@
         <v>124.25</v>
       </c>
       <c r="H96" s="25">
-        <f>G96*E96</f>
+        <f t="shared" si="2"/>
         <v>93187.5</v>
       </c>
       <c r="I96" s="18" t="s">
@@ -20888,7 +20906,7 @@
         <v>55.57</v>
       </c>
       <c r="H97" s="25">
-        <f>G97*E97</f>
+        <f t="shared" si="2"/>
         <v>13892.5</v>
       </c>
       <c r="I97" s="18" t="s">
@@ -20918,7 +20936,7 @@
         <v>4430</v>
       </c>
       <c r="H98" s="25">
-        <f>G98*E98</f>
+        <f t="shared" ref="H98:H129" si="3">G98*E98</f>
         <v>4430</v>
       </c>
       <c r="I98" s="18" t="s">
@@ -20946,7 +20964,7 @@
         <v>670000</v>
       </c>
       <c r="H99" s="25">
-        <f>G99*E99</f>
+        <f t="shared" si="3"/>
         <v>670000</v>
       </c>
       <c r="I99" s="18" t="s">
@@ -20974,7 +20992,7 @@
         <v>670</v>
       </c>
       <c r="H100" s="25">
-        <f>G100*E100</f>
+        <f t="shared" si="3"/>
         <v>7879.2</v>
       </c>
       <c r="I100" s="18" t="s">
@@ -21002,7 +21020,7 @@
         <v>9.99</v>
       </c>
       <c r="H101" s="25">
-        <f>G101*E101</f>
+        <f t="shared" si="3"/>
         <v>5994</v>
       </c>
       <c r="I101" s="18" t="s">

</xml_diff>